<commit_message>
Standardize dashboard and workbook headers
</commit_message>
<xml_diff>
--- a/site/matches-positive.xlsx
+++ b/site/matches-positive.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,7 +444,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>省级行政区</t>
+          <t>省份</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -454,45 +454,40 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>县级市</t>
+          <t>城市</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>次级行政区</t>
+          <t>项目内容</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>项目内容</t>
+          <t>合计金额（元）</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>资金情况</t>
+          <t>产品种类</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>产品种类</t>
+          <t>项目详细内容</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>项目详细内容</t>
+          <t>产品用量</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>产品用量</t>
+          <t>匹配程度</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
-        <is>
-          <t>匹配程度</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
         <is>
           <t>匹配关键词</t>
         </is>
@@ -537,34 +532,29 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>璧山区</t>
+          <t>本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。</t>
+          <t>项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。</t>
+          <t>钢筋混凝土管及管件</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>钢筋混凝土管及管件</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
           <t>璧山项目钢筋混凝土管询价公告 本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用 地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行 建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉 泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含 市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范 围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期 实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。 网 登录地 mhem&amp;cNh6e0&amp;ce2C2m3s1e71=a64so0d9FAe=0903%e08005206E%6772dm6=%82he29&amp;=cI8p9eeyAs%7t?E%5lB%1iB%a1DetE%c9eweNAi%1iotvB%n/9cE%7.cBe9%ccAiE%p.E%s9%/29址/A%2:：psE%7tAhtD%B8%E%6B%7B%7E%5%78D9%E%5C9%F%9E%7AE%A%1E%9%78%78E%8B%4AD%N&amp;8E%6m657optUa3%6=6290%e3ni51B%5917E%443d6=E%862B%I8eAc%A1iD&amp;88no%tE%4BA%A%4E%7AC%AC%E%4BA%C8%E%8%88AA%E%5A8%A%1E%5B%7A%5E%7A%8B8%E%5B%1%08E%6C9%%98E%9%99%09E%5%58AC%E%5F%8B%8E%8A%5BF%E%9%38A%8EF%BC%%88E%5B9%BD%E%9%99%58EF%BC%%98E%6%59B%0E%5AD%%79E%7BB%F%8E%6B%5E8%E%4BA%A%7E%4B%8A9%E%5B9%AD%E%5C8%BA%E%9%58D8%E%5A%5%79E%9A%1B%9E%7B9%AE%EF%BC%%88E%8A%5BF%E%7%98%78E%5C8%BA%EF%BC%%98E%9A%1B%9E%7B9%AE%E%7=BgB&amp;upC%a=sod&amp;euF%pN=8Flk&amp;cmsusheaE%c7=te%0a9m%6he=8tT&amp;cpS7eeyeE%s9sha%&amp;3c2845d5=pur5A6I&amp;8optUni 信息来源:https://www.chinapipe.net/project/d3077008.html 务 cqdingjiu 2026.08.21 10:06:40 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="n">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="n">
         <v>70</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -609,34 +599,29 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>忠县</t>
+          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。</t>
+          <t>本项目工程总投资金额：约3140万元；本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>本项目工程总投资金额：约3140万元；本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。</t>
+          <t>高标准农田建设工程</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>高标准农田建设工程</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 务 2.1 建设地点： 忠县花桥镇、新立镇、石宝镇、兴峰乡。 商 2.2 项目概况与建设规模①忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）：田块整治 工程：旱地区域撂荒地整治278.95亩；灌溉与排水工程：新建200m蓄水池6座、PE75管道967m、新建1.2*1.2m箱 涵16m、新建2*2m箱涵8m；田间道路工程：新建2.5m混凝土生产路15114m、改建2.5m混凝土生产路1078m、新 建2.5m泥结碎石生产路910m、改建2.5m泥结碎道石生产路279m、新建3.0m混凝土生产路601m、改建3.5m混凝土机 耕路4587m；地力提升工程：施有机肥278.95亩；其他工程：工号牌124块。 管 ②忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）：田块整治工程：旱地区域撂荒地 整治195.54亩；灌溉与排水工程：新建100m蓄水池4座、新建200m蓄水池6座、PE75管道5258m、PE90管 道1375m、PE110管道2156m、改建0.5*0.6m混凝土排水沟740m、改建0.6*0.8m混凝土排水沟109m、改建0.8*1.0m混 凝土排水沟296m、改建1*1.5m混凝土排水沟262m、新建3*2m盖板涵1座；田间道路工程：新建2.5m混凝土生产 路11359m、改建2.5m混国凝土生产路3430m、新建2.5m泥结碎石生产路1834m、新建3.0m混凝土生产路350m；农田 防护工程：新建1.0m高挡土墙39m；地力提升工程：施有机肥195.54亩；其他工程：工号牌142块。 中 2.3 本项目工程总投资金额：约3140万元； 本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： 标段划分情况、建设规模及标段合同估算金额等内容如下： 合同估算金额 序号 项目名称 建设地点 （万元） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二 1 花桥镇、新立镇 1022 标段） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三 2 石宝镇、兴峰乡 735 标段） 网 本项目共分为2个标段，每家投标单位仅对2个标段中的任意1个标段进行投标，若同时参与2个及以上标段投标的， 其投标文件无效。 务 2.7 其他： / 商 3.政府采购工程 道 3.1 是否属于政府采购工程：是 □否 管 3.2 是否专门面向中小企业预留：是 国 专门面向中小企业预留的实施方式： 中 方式一：本项目整体面向中小企业。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字 证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责 任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要网提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-10-12 09:30，投标人应当在投标截止时间前，通过互 务 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 商 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 道 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 管 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 国 开户银行: 开户银行: 账 号: 账 号: 中 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段） 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005499 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421353 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891814619 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082001038 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00385 信息来源:https://www.chinapipe.net/project/d3076880.html cqdingjiu 2026.08.21 10:06:45</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="n">
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="n">
         <v>90</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>重庆, 高标准农田建设工程, 资金情况, 产品种类</t>
         </is>
@@ -681,34 +666,29 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>忠县</t>
+          <t>田块整治工程、灌溉与排水工程、田间道路工程、地力提升工程、其他工程</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>田块整治工程、灌溉与排水工程、田间道路工程、地力提升工程、其他工程</t>
+          <t>项目总投资金额约3140万元，本次招标项目合同估算金额一标段1167万元</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>项目总投资金额约3140万元，本次招标项目合同估算金额一标段1167万元</t>
+          <t>高标准农田建设工程</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>高标准农田建设工程</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(一标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）已由 忠县发展和改革委 员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来 自 业主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具 备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 务 2.项目概况与招标范围 商 2.1 建设地点： 忠县马灌镇、三汇镇、永丰镇。 道 2.2 项目概况与建设规模：忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）：田块整治 工程：水田整治50.67亩、水田区域撂荒地整治79亩、旱地区域撂荒地整治62.83亩；灌溉与排水工程：新 建200m蓄水池5座、新建500m蓄水池1座、泵站1座；田间道路工程：新建2.5m混凝土生产路12325m、改 建2.5m混凝土生产路8549m、新建2.5m泥结碎石生产路1223m、新建3.0m混凝土生产路576m、改建3.0m混凝土生 管 产路648m、改建3.0m混凝土生产路（拆除原1.5m宽路）266m、改建3.5m混凝土机耕路1662m；地力提升工程：施 有机肥136.48亩；其他工程：公示牌1座、工号牌213块。 国 2.3 本项目工程总投资金额：约3140万元； 中 本次招标项目合同估算金额：一标段1167万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 网 方式一：本项目整体面向中小企业。 务 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 商 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 道 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 管 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 国 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 中 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及CA数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-10 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 网 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 务 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段） 商 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082000104 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005469 道 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421379 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00387 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891884496 管 信息来源:https://www.chinapipe.net/project/d3076876.html cqdingjiu 2026.08.21 10:06:46 国 中</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="n">
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="n">
         <v>95</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>重庆, 高标准农田建设工程, 投资金额, 产品种类</t>
         </is>
@@ -753,34 +733,29 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>永川区</t>
+          <t>农村供水管网巩固提升改造工程</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>农村供水管网巩固提升改造工程</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>供水管网</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>供水管网</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
           <t>永川区农村供水管网巩固提升改造工程(东部片区)答疑补遗文件 永川区农村供水管网巩固提升改造工程（东部片区） 补遗文件（01） 各潜在投标人： 现将“永川区农村供水管网巩固提升改造工程（东部片区）”招标文件补遗通知如下，本次发布的补遗文件中 的所有内容与招标文件具有同等法律效力，如与招标文件、答疑补遗文件（01）网不一致时，以本补遗文件为准。 请各潜在投标人自行下载本补遗文件，不管下载与否，都视为全部知晓其全部内容。 一、本招标项目招标文件第二章投标人须知前附表第1.4.1项第1条第（3）款中“具备建设行政主管部门颁发的有 效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由建设行政主管部门颁发的有效的安全生产 务 考核合格证书。”修改为： “（3）具备建设行政主管部门颁发的有效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由水 行政主管部门颁发的有效的安全生产考核合格证书”。 商 二、本招标项目招标文件第二章投标人须知前附表第1.4.1项中第3条“业绩要求”修改为： “投标人自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成过1个单项合同 输配水管网长度不少于100km的水利工程施工道业绩。 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 管 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 三、本招标项目招标文国件第二章投标人须知前附表第1.4.1项中第5条中的“5.3项目经理业绩要求”修改为： “投标人拟派的项目经理自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成 过1个单项合同输配水管网长度不少于100km的水利工程施工业绩，并在该业绩中担任项目经理。 中 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 四、本招标项目的投标文件递交的截止时间（投标截止时间）调整为2026年9月4日9时30分（北京时间），开标 时间及投标保证金递交截止时间相应顺延。 招标人：重庆市永川区惠永水务有限公司 招标代理机构：重庆永川政鑫综合能源有限公司 2026年8月20日 信息来源:https://www.chinapipe.net/project/d3076870.html cqdingjiu 2026.08.21 10:06:46</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="n">
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="n">
         <v>80</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>重庆, 农村供水管网, 巩固提升改造, 东部片区, 管材招标</t>
         </is>
@@ -825,34 +800,29 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>万州区</t>
+          <t>渝万高铁站前1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~D1K47+550.4，正线长度33.01km，中标造价31.73亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁301孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负责DK0+000~DK57+136段小型构件预制。</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>渝万高铁站前1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~D1K47+550.4，正线长度33.01km，中标造价31.73亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁301孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负责DK0+000~DK57+136段小型构件预制。</t>
+          <t>中标造价31.73亿元</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>中标造价31.73亿元</t>
+          <t>刺丝滚笼,塑钢模板,泄水管</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>刺丝滚笼,塑钢模板,泄水管</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
           <t>中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部刺丝滚笼、塑钢模板、泄水管询价采购公告 中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 刺丝滚笼、塑钢模板、泄水管询价采购公告 询价编号： ZT1105-XJ-2026-590 尊敬的 各潜 在供应商 : 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与 中铁十一局集团有限公司重庆至万州高铁站 前 1标项目经理部 ZT1105-XJ-2026-590， 刺丝滚笼、塑钢模板、泄水管 的报价。 一、 项目概况 务 渝万高铁站前 1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~ D1K47+550.4，正线长度 33.01km，中标造 价 31.73 亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁 301 孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负 责DK0+000~DK57+136段小型构件预制。合同工期54.7月商，开工日期为2022年11月01日，竣工日期为2027 年04 月30日。 二、 询价内容 道 本次 计划对刺丝滚笼、塑钢模板、泄水管 进行询价，询价内容如下： 询价物资一览表 管 计 序 物资 量 包件号 规格型号 数量 备注 号 名称 单 位 国 刺丝 1 GL-01 2.5mm 6m0.5m 米 6500 半径 ≥225mm，包括刀片刺绳、挂丝、连接卡、支架 滚笼 防护 中 栅栏 2 GL-01 用立 50X30X765X2.5mm 套 500 含抱箍、螺栓等配件 柱支 架 平 塑钢 3 MB-01 350X300mm 方 19.2 400*400,1个挡水沿，配固定手柄 模板 米 平 塑钢 4 MB-01 350X300mm 方 19.2 400*400,2个挡水沿，配固定手柄 模板 米 平 塑钢 5 MB-01 300X300mm 方 75.6 2个挡水沿，配固定手柄 模板 米 平 塑钢 6 MB-01 300X300mm 方 75.6 1个挡水沿，配固定手柄 模板 米 7 SSG-01 管篦 PVC250X200x10mm 个 220 材质硬聚氯乙烯 PVC，详见附图 PVC 8 SSG-01 泄水 135X38mm 块 220 材质硬聚氯乙烯 PVC，详见附图 管盖 U型 9 SSG-01 125mm 个 900 详见附图 管卡 UPV 材质硬聚氯乙烯 PVC，两端接头采用阴阳螺纹连接详见 10 SSG-01 C排 125X8mm螺纹 米 2870 附图 水管 UPV 11 SSG-01 C弯 DN125X8mm90° 个 240 材质硬聚氯乙烯 PVC，详见附图 管 UPV 网 125X125X110mm弹性密 12 SSG-01 C三 个 120 材质硬聚氯乙烯 PVC，详见附图 封圈异径斜三通 通 无压 埋地 务 排污 排水 用硬 13 SSG-01 DN125 个 150 材质硬聚氯乙烯 PVC，详见附图 聚氯 商 乙烯 管 T 型接 头 道 合 计 管 说明： 1. 表中数量为计划数量，实际 采购 过程中可能有所调整，最终结算按照实际 采购 数量结算。 2.收货地点：中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部 三、 技术质量 及报价国 要求 1. 此次 询价物资 各项技术性能要 符合 甲方 的要求，质量满足甲方项目部正常使用的要求，保证 产品 的质量合 格。 具体要求或图纸见询价文件技术规格书。 。 中 2 .报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、 结算及付款方式 每个月 15 日为双方价款结算日期（即上月 16 日至当月 15 日内），结算前双方要在对帐确认单上签字认可，乙 方按双方确认的金额开具增值税专用发票，并自发票开具之日起 7日内传递给甲方。甲乙双方在增值税专用发票 传递过程中必须留取相应的交接签证手续。自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发 票认证完成之日起第6个月，支付至本次结算金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内， 累计支付总额不超结算总金额的75%，剩余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理 末次结算后第二年，支付金额应大于等于尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总 额的15%；办理末次结算后第四年，全部付清）。 五、 报价 人资格要求 1.营业范围要求：在中华人民共和国境内依法注册，具有询价物资生产或供应经验的生产商或代理商，并且具有 合法有效的营业执照。 2.生产能力要求： 生产商须具备 询价 物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定 。 代理商需出具制造厂出具签字盖章的授权函。 3.财务能力要求：报价人为增值税一般纳税人或小规模纳税人，有依法纳税的良好记录。 4.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8月至今） 国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；每种物资全指标技术参数性能满足 国家和行业最新标准的各项规定。 5.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年8月至今）企业或企业法定代表人有人民法院生效判决、裁定 认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接受 通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合作 方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 6.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★7 .下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、 报价人需要提供的资料 1. 营业执照复印件、 法人身份证复印件、 开户许可证、商授权委托书 、 报价表 和报价人资格要求中所需的证明资 料， 所有资料需加盖公司鲜章。 2. 产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、 询价 报名截止 时间 管 有意参加本次询价采购的报价人 须在铁建云链平台 （ https:// www.crccep. cn） 完成供应商注册，并 于 202 6 年 8 月 20 日 9时 00 分 至 202 6 年 8 月 24 日 9时 00 分在网上 完成报名工作。 八、 询价 截止 时间 国 凡有意参加本次询价采购的报价人，请于 202 6 年 8 月 24 日 14 时 00分 前 提交报价。截止时间前未完成 报价 文 件传输的，视为放弃 报价 。 供应商报价必须严格按照《 报价表 》格式进行报价。 中 九、 联系方式 采购 组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村 71号 联系人：胡先生 联系电话： 13983336494 （提供平台服务支持） 采购人名称：中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 地址： 重庆市万州区双河口街道檬兴路万州现代综合物流中心信息交易大厅（中铁十一局） 联系人： 唐大伟 联系电话： 18323391938（提供采购服务支持、保证金退还） 中铁十一局集团有限公司物资设备集中采购管理中心 第五分中心 2026 年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076805.html cqdingjiu 2026.08.21 10:06:47 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="n">
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
         <v>85</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>重庆, 万州, 高铁站前, 刺丝滚笼, 塑钢模板, 泄水管, 询价采购</t>
         </is>
@@ -897,34 +867,29 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>垫江县</t>
+          <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目，主要内容包括河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m，化粪池2座；产业基地水肥一体化改造45亩等。</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目，主要内容包括河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m，化粪池2座；产业基地水肥一体化改造45亩等。</t>
+          <t>项目总投资金额为642.89万元，本次招标项目合同估算金额约为5014864.52元。</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>项目总投资金额为642.89万元，本次招标项目合同估算金额约为5014864.52元。</t>
+          <t>水利水电工程施工</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>水利水电工程施工</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
           <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 1.招标条件 本招标项目 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 已由 垫江县发展和 改革委员会 以 垫江发改委发〔2026〕20号 文批准建设，项目业主为 垫江县太平镇人民政府，建设资金来 自 大中型后扶资金及自筹资金 ，项目出资比例为 100% ，招标人为垫江县太平镇人民政府。项目已具备招 标条件，现对本项目施工进行公开招标，评标办法采用经评审的最低投标价法。网 务 2.项目概况与招标范围 商 2.1 建设地点：垫江县太平镇桂花村 道 2.2 项目概况与建设规模：主要为河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m， 化粪池2座；产业基地水肥一体化改造45亩等。 管 2.3 本项目工程总投资金额：642.89万元 国 本次招标项目合同估算金额：约5014864.52元 中 2.4 招标范围：本工程施工图纸所含全部的施工内容，具体以招标人发布的工程量清单为准。 2.5 工期要求：工期为360日历天 ，缺陷责任期为24个月。 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：□是 否，因专门面向中小企业预留无法确保充分供应、充分竞争，根据 《政府采购促进中小企业发展管理办法》第六条第(三)“按本办法规定预留采购份额无法确保充分供应、充分竞 争，或者存在可能影响政府采购目标实现的情形”的规定，本项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 网 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的水利水电工程施工总承包三级 务 及以上资质。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相商应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 道 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 管 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com国/dianjiangweb/)、重庆市公共资源交易监督网下载招标文件、工程量清单、电子图纸等资 料。参与投标的投标人需在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共 资源交易监督网完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督网导航栏“主体信息”页面中“市场主体信息 登记”、“中CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流 程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督 网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-24 17:00:00前。 5.3招标人应于2026-08-28 17:00:00前在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重 庆市公共资源交易监督网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交 易监督网发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 垫江县太平镇人民政府 代理机构: 重庆皓辰建设工程咨询有限公司 重庆市渝北区金开大道1228号大雅金开国际1 地 址: 重庆市垫江县太平镇牡丹路191号 地 址: 栋9-2 邮 编: 邮 编: 项目负责人: 余老师 项目负责人: 雷雨得 电 话: 13996889839 电 话: 023-86018770 18580880860 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 网 2026年08月19日 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 务 户名 开户行 投标保证金账号 垫江县公共资源交易中心 中国农业银行重庆垫江支行 316301010400077950000005966 垫江县公共资源交易中心 中国银行重庆垫江支行 111616885778VA00139 商 垫江县公共资源交易中心 重庆农村商业银行垫江支行 2501010120010009065000128 垫江县公共资源交易中心 工商银行重庆垫江支行营业部 9558853100016843371 垫江县公共资源交易中心 重庆银行垫江支行 820101040000584-101195 道 附件：垫江县2026年度大中型水库移民后期扶持项目-.zip https://www.cqggzy.com/trade/014001/dac54522-3264-4eac-ae47-f434567ce374?categoryNum=014001001007 信息来源:https://www.chinapipe.net管/project/d3076788.html cqdingjiu 2026.08.21 10:06:47 国 中</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="n">
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="n">
         <v>85</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 水利, 移民, 后期扶持</t>
         </is>
@@ -969,34 +934,29 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>万州区</t>
+          <t>新建水厂1座（新建2000m³茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管径DN20~DN250，管材为涂塑钢管。</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>新建水厂1座（新建2000m³茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管径DN20~DN250，管材为涂塑钢管。</t>
+          <t>合同预估金额：5000万元</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>合同预估金额：5000万元</t>
+          <t>涂塑钢管</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>涂塑钢管</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
           <t>万州区新田等6个镇乡农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区新田等6个镇乡农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建水厂1座（新建2000m3茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管 主要建设内容 径DN20~DN250，管材为涂塑钢管。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 备注 称 式 发布时间 所 额(万元) 商 万州区新田 万州区新田 重庆市万 招标项目 等6个镇乡农 等6个镇乡农 公开招 州区公共 1 村饮水质量提 2026-08 5000.00 村饮水质量 标 资源交易 升项目道施工总 提升项目 中心 承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076721.html 管 cqdingjiu 2026.08.21 10:06:48 国 中</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="n">
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="n">
         <v>80</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 商机</t>
         </is>
@@ -1041,34 +1001,29 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>万州区</t>
+          <t>新建50m³蓄水池4口、取水池2座；新建50m³/d-100m³/d水厂2座；改造100m³/d-300m³/d水厂5座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设施。</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>新建50m³蓄水池4口、取水池2座；新建50m³/d-100m³/d水厂2座；改造100m³/d-300m³/d水厂5座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设施。</t>
+          <t>合同预估金额：3000万元</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>合同预估金额：3000万元</t>
+          <t>DN25-DN250涂塑钢管</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>DN25-DN250涂塑钢管</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
           <t>万州区大周等4个镇乡街道农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区大周等4个镇乡街道农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建50m3蓄水池4口、取水池2座；新建50m3/d-100m3/d水厂2座；改造100m3/d-300m3/d水厂5 主要建设内容 座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设 施。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 商 备注 称 式 发布时间 所 额(万元) 万州区大周 万州区大周 重庆市万 招标项目 等4个镇乡街 等4个镇乡街 公开招 州区公共 1 道农村饮水 道农村饮道水质 2026-08 3000.00 标 资源交易 质量提升项 量提升项目施 中心 目 工总承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3076720.html cqdingjiu 2026.08.21 10:06:49 国 中</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="n">
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
         <v>80</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>重庆, 农村饮水质量提升项目, 管材招标, 合同预估金额</t>
         </is>
@@ -1107,32 +1062,31 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。</t>
+          <t>采购项目资金为企业自筹。</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>采购项目资金为企业自筹。</t>
+          <t>纤维编绕拉挤电缆保护套管(BWFRP100/2.0，79158米)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>纤维编绕拉挤电缆保护套管(BWFRP100/2.0，79158米)</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
           <t>二航科工新燕尾山项目纤维编绕拉挤电缆保护套管采购询价通知公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目询比采购 公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目已具备采 购条件，现公开邀请供应商参加询比采购活动。 网 1. 采购项目简介 1.1 采购项目名称：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机 电工程项目。 务 1.2采购方案编号：FA00000674478。 1.3 采购人：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程 项目经理部。 商 1.4 采购代理机构：中交二航局科工（武汉）有限公司。 1.5 采购项目资金：企业自筹。 道 1.6 采购项目概况：新燕尾山隧道工程位于重庆市内环吉庆隧道北侧，四横线分流道鹿角隧道南侧，西接白居 寺大桥，东接内环快速路，并向东延伸接渝黔复线高速，其所在的道路系统呈东西布置，为主城区南部片区重 要干道。本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目 管 全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程 包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。 2.采购范围及相关要求 国 2.1 采购范围：纤维编绕拉挤电缆保护套管（BWFRP100/2.0，79158米）。 2.2 交货期：以甲方实际订单要求为准。 中 2.3 交货地点：重庆市巴南区新燕尾山项目甲方指定位置。 2.4 物资质量标准：满足国家法律法规、标准、规范、设计参数及技术规格书要求。 3.供应商资格要求 3.1 供应商应依法设立且满足如下要求： （1）资质要求：在中华人民共和国境内依法注册，具有独立法人资格、具有采购物资生产或供应经验的企业， 并且具有合法、有效的“三证合一”的营业执照,代理商需提供制造商授权委托书。 （2）财务要求：必须是经税务部门注册登记核准的一般纳税人，有依法纳税的良好记录，提供近三年的财务报 告。 （3）业绩要求：同类产品销售业绩不少于2个，并具备与本招标项目需求相适应的供货能力。 （4）信誉要求：本项目投标截止期前未被“信用中国”、“中国政府采购网”、中国交建物资采购管理信息系 统网站列入失信被执行人、违法案件当事人、违法失信行为记录名单。 （5）其他要求：提供运输方案及生产周期。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他： / 。 4.供应商报名 4.1有意参加询比采购活动的单位，请于2026年 8 月 20 日 11 时 00 分至2026 网 年 8 月 25 日 11 时 00 分（北京时间、下同），登录“中交招采网”（网 址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 务 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 商 5. 供应商报价 5.1 报价结束（递交响应文件截止）时间：2026年 8 月 25 日 11 时 00 分。 道 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的 电子响应文件，采购人将拒收。 5.3电子采购的供应商报价文件由线上电子报价表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 管 子报价表的数据为准。 6. 开标 6.1开标时间：与报价结国束时间相同。 6.2开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标，现场开标地点/。 7. 发布公告的媒介 中 本询比采购公告在中交招采网上发布。 8. 评审办法 本项目评审办法采用 经评审的最低价法 。 9. 合同主要条款 9.1 付款条件：无预付款，到货后办理结算，双方办理完结算手续、卖方提供符合合同要求的正式发票给买方 后60天，买方支付该批材料价值80%的货款，完工结算后支付至97%，剩余3%为质保金，质保期2年，两年后供 应方申请返还3%（无息）；银行转账、承兑、18个月供应链金融混合支付方式。 9.2履约保证金的递交： （1）□不要求递交 （2）要求递交 保证金金额：2万元 ； 保证金形式：银行转账、银行保函等电子保函；其他形式：无 。 10. 成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”（网址：https://zjzcw.iccec.cn）发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联 系4006765885中标服务费请按7咨询。 10.1收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； 务 （3）在1000万元（含）至3000万元之间的，每次收取1000元； （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 10.2支付流程 （1）通知推送：中标结果发布后，系统自动道推送缴费通知（含应缴金额及支付链接）； （2）费用查询：供应商登录“中交招采网-服务管理”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网- 服务管理－发票下载”模块获取。 11.监督机构 国 监督机构名称：中交二航局科工（武汉）有限公司纪委监察部 举报电话：中027-82796466 举报邮箱：sneb_kggs@ccccltd.cn 12.其他 投标保证金采用银行转账形式的需转至中交二航局科工（武汉）有限公司账户（账 号：42001186108053006379-0006开户行：建行武汉长江支行，行号：105521000053），并备注二航科工燕尾山机 电照明项目纤维编绕管投标保证金。 13.联系方式 采购 人：中交二航局科工（武汉）有限公司 采购代理机构：中交二航局科工（武汉）有限公司 地 址：武汉市新洲区双柳街星谷大道158号地 址：武汉市新洲区双柳街星谷大道158号 邮政编码：430400 邮政编 码：430400 联系人：李鑫 联系人：毕明 月 电 话：18186145302 电 话：17853118573 电子邮件：18186145302@ccccltd.cn 电子邮件：bimingyue@ccccltd.cn 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076715.html cqdingjiu 2026.08.21 10:06:50 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="n">
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
         <v>90</v>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 光纤电缆保护套管</t>
         </is>
@@ -1177,34 +1131,29 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>巴南区</t>
+          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>天然气表后管道安装工程</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>天然气表后管道安装工程</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告 重庆巴南天然气有限责任公司 重庆国际生物城配套公寓项目天然气表后管道安装工程 变更公 告 公告编号： RQBGGG202608200006 本公司于2026年08月19日发布的重庆国际生物城配套公寓项目天然气表后管道安装工程公告（编 号：RQCGXY202608170010），现做出如下变更： 网 1、对采购文件第一卷“采购需求“中墙体管道暗埋的具体内容进行明确。墙体管道暗埋应包含墙体开槽，输送 用不锈钢波纹管及钢制槽板的安装，墙体恢复，暗埋管道视频记录。 2、对由响应供应商提供的钢制槽板的规格进行明确。钢制槽板为U型开口槽，采用热镀锌Q235B钢板，钢板厚度 务 不得小于1.2mm，尺寸不得小于U40*30*1.2（宽40mm,高30mm,壁厚1.2mm热镀锌） 3、对由响应供应商提供的F型不锈钢三通，材质可以选用黄铜进行替代。 4、采购文件第二卷“技术规范及要求“中增加T/CECS633-2019 《燃气用户工程不锈钢波纹软管技术规程》。 以上内容在合同中也同步进行调整。 商 除上述变更外，原公告其余内容仍有效。 道 重庆巴南天然气有限责任公司 管 2026-08-20 信息来源:https://www.chinapipe.net/project/d3076704.html cqdingjiu 2026.08.21 10:国06:50 中</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="n">
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
         <v>80</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>重庆, 天然气表后管道安装工程, 变更公告</t>
         </is>
@@ -1249,34 +1198,29 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>合川区</t>
+          <t>主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米，螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清淤2627米。</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米，螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清淤2627米。</t>
+          <t>合同预估金额为1708.44万元</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>合同预估金额为1708.44万元</t>
+          <t>排水管道、检查井、紫外线修复设备、螺旋缠绕修复材料、树脂修复材料、不锈钢快速锁修复设备</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>排水管道、检查井、紫外线修复设备、螺旋缠绕修复材料、树脂修复材料、不锈钢快速锁修复设备</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
           <t>合川区中南片区污水管网工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 合川区中南片区污水管网工程（一期） 名称 招标 网 法人 或招 标人 重庆市合川区住房和城乡建设委员会 名称 （盖 务 章） 项目 批准 文件 合川发改投〔2025〕19 号 商 及文 号 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新 主要 建D300排水管道38米；紫外光修复 D300-D道800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 建设 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42 内容 米；完成 D300-D1000管道清障189米、清淤2627米。 拟 招 招标文 合同预 招标 管 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 国 重 庆 市 合川 合 招标 区中 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300- 川 项目 中 南片 D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 公 区 区污 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 开 公 1 2026-09 1708.44 水管 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米， 招 共 网工程 不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清 标 资 （一 淤2627米。 源 期） 交 易 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076543.html cqdingjiu 2026.08.21 10:06:50</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="n">
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
         <v>90</v>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>重庆, 污水管网工程, 管网修复, 新建工程, 排水管道, 检查井, 紫外线修复, 螺旋缠绕修复, 树脂修复, 不锈钢快速锁修复</t>
         </is>
@@ -1315,32 +1259,31 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>本次采购项目涉及球墨铸铁管及管件的供应，具体包括样品的规格和数量要求。</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>本次采购项目涉及球墨铸铁管及管件的供应，具体包括样品的规格和数量要求。</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>球墨铸铁管及管件</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>球墨铸铁管及管件</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
           <t>重庆市自来水有限公司球墨铸铁管及管件2026-2027(2年)采购项目(第二次)答疑补遗文件 重庆市自来水有限公司球墨铸铁管及管件2026-2027（2年）采购项目（第二次）答疑 提问1：样品20CM长含承口吗？如果含承口20CM那就太短，标识LOGO无法体现完整建议≥20CM 答1：球墨铸铁管样品含承口，样品长度≥20CM 网 务 招标人：重庆市自来水有限公司 招标代理机构：重庆水务集团公用工程咨询有限公司 商 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d30道76446.html cqdingjiu 2026.08.21 10:06:50 管 国 中</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="n">
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
         <v>80</v>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>重庆, 球墨铸铁管, 管件, 采购项目</t>
         </is>
@@ -1385,12 +1328,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>大足区</t>
+          <t>大足区中心城区和龙水镇市政公共排水设施的运维(材料)。</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>大足区中心城区和龙水镇市政公共排水设施的运维(材料)。</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1400,19 +1343,14 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
           <t>大足区中心城区和龙水镇市政公共排水设施运维(材料)更正一号公告 一、更正项 更正项 更正子项 更正前内容 更正后内容 网上投标 网上投标截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 递交投标响应文件 线下递交投标（响应）文件开始时间 2026-08-20 14:30:00 2026-08-25 14:30:00 递交投标响应文件 线下递交投标（响应）文件截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 网 开标 开标时间 2026-08-20 15:00:00 2026-08-25 15:00:00 招标采购（附件） 附件 务 二、补遗更正说明 清单限价重新做调整，开标时间已更正，详见更正文件内容 商 三、联系方式 采购执行方： 道 单位名称：重庆誉双项目管理有限公司 联系人：陈老师 联系电话：13996336872 采购需求方： 管 单位名称：重庆市大足区茂泰市政工程有限公司 联系人：谢老师 联系电话：18523539371 信息来源:https://www.chinapipe.net/project/d3076319.html 国 cqdingjiu 2026.08.21 10:06:50 中</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="n">
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
         <v>80</v>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>重庆, 管材招标</t>
         </is>
@@ -1457,34 +1395,29 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>璧山区</t>
+          <t>项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6.都市农文旅配套建设1000平方米。</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6.都市农文旅配套建设1000平方米。</t>
+          <t>合同预估金额为9182.25万元</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>合同预估金额为9182.25万元</t>
+          <t>温度调控系统、水肥一体化设备、人工补光系统、二氧化碳补施系统、智能环境控制系统、作业物流装备</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>温度调控系统、水肥一体化设备、人工补光系统、二氧化碳补施系统、智能环境控制系统、作业物流装备</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
           <t>璧山区2026年大路街道三台村智慧设施农业建设项目招标计划表 重庆市工程建设项目招标计划表 项目 璧山区2026年大路街道三台村智慧设施农业建设项目 名称 招标 法人 或招 网 标人 中农良品（重庆）生态农业有限公司 名称 （盖 章） 项目 批准 务 文件 及文 号 主要 1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流 建设 装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6. 内容 都市农文旅配套建设1000平方米。 商 招 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 道 璧 山 区2026 重 年 庆 大 市 路 公 招标 街 管 共 项目 道 资 三 公 源 台 项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米； 2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、 开 交 1 村 二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套； 3.项目后勤及仓储配套（含装修）5000平方米； 4.土方回填及场地平整53000平 2026-09 9182.25 招 易 智 方米； 5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米； 6.都市农文旅配套建设1000平方米。 标 中 慧 心 设 国 璧 施 山 农 分 业 中 建 心 设 项 目 中 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076777.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="n">
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
         <v>80</v>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>重庆, 智慧设施农业, 招标计划, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -1529,34 +1462,29 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>长寿区</t>
+          <t>本项目包括但不限于新建混凝池-三沉池，还建格栅池，厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统，原斜管沉淀池改造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰），拆除原有污泥池，新增临时污泥储罐务并还建污泥池，污泥堆场临时改建及恢复，实施技改期间的临时排放工程，进行基础的自控改造。</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>本项目包括但不限于新建混凝池-三沉池，还建格栅池，厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统，原斜管沉淀池改造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰），拆除原有污泥池，新增临时污泥储罐务并还建污泥池，污泥堆场临时改建及恢复，实施技改期间的临时排放工程，进行基础的自控改造。</t>
+          <t>企业自筹，出资比例为100%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>企业自筹，出资比例为100%</t>
+          <t>污水处理设备</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>污水处理设备</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
           <t>长寿区江南街道污水处理厂更新改造工程项目公告 长寿区江南街道污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目长寿区江南街道污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源为企业 自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：长寿区江南街道污水处理厂更新改造工程包括但不限于以下内容新建混凝池-三沉池；还建格栅池； 厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统；原斜管沉淀池改 造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰）。拆除原有污泥池，新增临时污泥储罐 务 并还建污泥池；污泥堆场临时改建及恢复；实施技改期间的临时排放工程；进行基础的自控改造。 2.2 比选范围：长寿区江南街道污水处理厂更新改造工程施工图范围中的所有工作内容，包括但不限于土建工 程、设备及安装工程、工艺管道工程、电气工程、临排工程等内容，具体以比选人提供的图纸、技术规范、设 备需求清单、答疑资料、澄清资料、其他补遗资料等相关商内容为准。 2.3 建设地点：重庆市长寿区江南街道。 2.4 工期：110日历天（实际开工日期以监理工道程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 3. 参选人资格要求 管 3.1 本次比选要求参选人具备以下条件： （1）独立法人资格； （2）建设行政主管部国门颁发的有效的市政公用工程施工总承包二级及以上资质； 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 中 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月 27 日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务 大厦5楼。 5.2 比选截止时间：2026年8月 27 日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 网 联系人：曹老师 电话：023-71618725 务 代理机构：重庆招标采购（集团）有限责任公司 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 商 联系人：高老师 电话：023-67706841 道 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 管 信息来源:https://www.chinapipe.net/project/d3076456.html cqdingjiu 2026.08.21 10:06:51 国 中</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="n">
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
         <v>90</v>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 污水处理厂</t>
         </is>
@@ -1601,34 +1529,29 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>潼南区</t>
+          <t>本项目包括两个子项目：一是潼南区新胜镇污水处理厂的更新改造，主要内容是新增一体化污水处理设备基础，更新现有污水处理系统设备，升级处理系统，新建风机房-配电室防尘防渗地坪；二是潼南区双江镇污水处理厂的更新改造，内容包括将原有斜管沉淀池改建为好氧池，新建竖流沉淀池，更新老旧及故障设备，新建储药加药区和一体化危废储存间，完善污水处理配套设施。</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>本项目包括两个子项目：一是潼南区新胜镇污水处理厂的更新改造，主要内容是新增一体化污水处理设备基础，更新现有污水处理系统设备，升级处理系统，新建风机房-配电室防尘防渗地坪；二是潼南区双江镇污水处理厂的更新改造，内容包括将原有斜管沉淀池改建为好氧池，新建竖流沉淀池，更新老旧及故障设备，新建储药加药区和一体化危废储存间，完善污水处理配套设施。</t>
+          <t>本项目资金来源为企业自筹，出资比例为100%。</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>本项目资金来源为企业自筹，出资比例为100%。</t>
+          <t>污水处理设备、一体化设备、沉淀池、好氧池、竖流沉淀池、储药加药区、一体化危废储存间、污水处理配套设施</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>污水处理设备、一体化设备、沉淀池、好氧池、竖流沉淀池、储药加药区、一体化危废储存间、污水处理配套设施</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
           <t>潼南区新胜镇、双江镇污水处理厂更新改造工程项目项目公告 潼南区新胜镇、双江镇污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目潼南区新胜镇、双江镇污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源 为企业自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：潼南区新胜镇污水处理厂更新改造工程，主要建设内容为新增200m?/d一体化污水处理设备基础； 更新现有污水处理系统设备，提高现有沉淀池二沉池、三沉池液位；升级处理系统（干化池改建为污泥池，新 增叠螺脱水机，改建污泥堆场及雨棚）；新建风机房－配电室防尘防渗地坪。潼南区双江镇污水处理厂更新改 务 造工程，主要建设内容为将原有斜管沉淀池改建为好氧池，新建3座竖流沉淀池，配套安装相关设备；更新污水 处理系统中老旧及故障设备；新建储药加药区与一体化危废储存间，完善污水处理配套设施。 2.2 比选范围：潼南区新胜镇、双江镇污水处理厂更新改造工程施工图范围中的工作内容（一体化设备采购及 相关安装工作除外），包括但不限于土建工程、附属工程商（包括但不限于绿化工程、工艺管线工程、电气及自 控工程、临排清淤工程等）、一体化污水处理设备基础、标准化建设、配套设备材料采购及安装工程等内容， 其中一体化设备采购及相关安装工作不在本次比选范围内；具体以比选人提供的图纸、技术规范、工程量清单、 答疑资料、澄清资料、其他补遗资料等相关内容为准。 道 2.3 建设地点：潼南区新胜镇、双江镇。 2.4 工期：120日历天（实际开工日期以监理工程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 管 3. 参选人资格要求 3.1 本次比选要求参选人具备以下条件： 国 （1）独立法人资格； （2）建设行政主管部门颁发的有效的市政公用工程施工总承包二级及以上资质； 中 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月27日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务大厦5 楼。 5.2 比选截止时间：2026年8月27日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 网 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 务 联系人：陈老师 电话：023-42756696 商 代理机构：重庆招标采购（集团）有限责任公司 道 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 联系人：高老师 管 电话：023-67706841 重庆水务电子商务平台国咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3076454.html cqdingjiu 2026.08.21 10:06:51 中</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="n">
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
         <v>90</v>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 污水处理厂更新改造</t>
         </is>
@@ -1667,32 +1590,31 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源</t>
+          <t>采购预算 409674.71元</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>采购预算 409674.71元</t>
+          <t>市政水源</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>市政水源</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
           <t>重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 采购需求单位(全称) 重庆医科大学附属第二医院总务科 项目名称 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程 项目内容 给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源 采购预算 409674.71元 网 拟采购供应商全称 东部自来水分公司 配套业务用房第二市政水源从重庆水资源产业股份有限公司东部自来水分公司管辖范围 单一来源采购理由 的管网具体接入，属于市政管网施工，具有特殊要求。 务 公示时间 2026年8月19日-2026年8月25日 联系人及联系电话 刘老师 023-63693215 注：1.以上陈述是否真实，欢迎社会各界监督，公示时间商至少5个工作日； 2.公示期内无异议的，采购管理处将进行该项目采购；有异议请将意见反映采购人。 信息来源:https://www.chinapipe.net/project/d30道76334.html cqdingjiu 2026.08.21 10:06:51 管 国 中</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="n">
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
         <v>80</v>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -1737,34 +1659,29 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>黔江区</t>
+          <t>本项目服务内容为G319黔江区正阳至城西段改建工程管线探测工作。</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>本项目服务内容为G319黔江区正阳至城西段改建工程管线探测工作。</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>管线探测工作</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>管线探测工作</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
           <t>中铁二院工程集团有限责任公司G319黔江区正阳至城西段改建工程管线探测工作线上询价采购公告 中铁二院工程集团有限责任公司G319黔江区正阳至城西 段改建工程管线探测工作线上询价采购 ZTEYCQ-XJ-2026-019 网 采购单位: 中铁二院工程集团有限责任公司 发布时间: 2026-08-19 16:10 报价截止时间: 务 2026-08-21 17:00 招标方联系人: 杨先生 招标方联系电话: 商 13883021521 招标方邮箱: 监督方联系人: 李先生 道 监督方联系电话: 15823237919 监督方邮箱: 保证金: 0元 管 结算与发票信息: 详情 交货信息: 详情 国 其他说明事项: 标的明细 流水号：询2026081900304 中 计量单 技术标准及要 序号 标的名称 数量 交货期 送货地址 位 求 G319黔江区正阳至城西段 合同签订后5天内完成 西南区-重庆市-市辖 1 1 项 详见询价文件 改建工程管线探测工作 本项目服务内容。 区-黔江区-项目地点 信息来源:https://www.chinapipe.net/project/d3076309.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="n">
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
         <v>80</v>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类, 匹配程度, 匹配关键词</t>
         </is>
@@ -1809,34 +1726,29 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>本项目主要涉及室外蒸汽管道φ219x6mm的安装，管道材质为20#，地上敷设，蒸汽管道运行压力1.08MPa，管道设计压力1.2MPa。蒸汽管道系统包括从锅炉房分汽缸到6#和8#车间分汽缸的所有蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温工作。还包括钢结构桁架工程的采购、运输、制作、安装、防腐工作，以及管道附件及控制系统的采购、运输、安装、接线等工作。此外，还需要进行调试与验收，确保蒸汽管道系统能够正常使用并备案。</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>本项目主要涉及室外蒸汽管道φ219x6mm的安装，管道材质为20#，地上敷设，蒸汽管道运行压力1.08MPa，管道设计压力1.2MPa。蒸汽管道系统包括从锅炉房分汽缸到6#和8#车间分汽缸的所有蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温工作。还包括钢结构桁架工程的采购、运输、制作、安装、防腐工作，以及管道附件及控制系统的采购、运输、安装、接线等工作。此外，还需要进行调试与验收，确保蒸汽管道系统能够正常使用并备案。</t>
+          <t>项目总投资额为580.643717万元，全部为企业自筹资金。</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>项目总投资额为580.643717万元，全部为企业自筹资金。</t>
+          <t>蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸、钢结构桁架、阀门、压力表、温度表、流量计、电动/气动执行机构、配套仪表电缆、桥架、保护管</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸、钢结构桁架、阀门、压力表、温度表、流量计、电动/气动执行机构、配套仪表电缆、桥架、保护管</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
           <t>乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 1.招标条件 本招标项目乌江涪陵榨菜绿色智能化生产基地(一期)已由重庆市涪陵区发展和改革委员会以重庆市企业投资项目 备案证2020-500102-13-03-000003 批准建设，项目业主为重庆市涪陵榨菜集团股份有限公司，建设资金来自企业 自筹，项目出资比例为100% ，招标人为重庆市涪陵榨菜集团股份有限公司。项目已具备招标条件，现对乌江 涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 2.1 建设地点： 重庆市涪陵区马鞍街道人和社区 。 网 2.2 项目概况与建设规模：建筑面积约369384.27㎡。本项目蒸汽管道主要为室外蒸汽管道φ219x6mm，管道材质： 20#地上敷设，由14#锅炉房分汽缸分别接至6#和8#智能化车间分汽缸，蒸汽管道运行压力1.08MPa，管道设计压 力1.2MPa。 务 2.3 本次招标项目合同估算金额：580.643717万元。 2.4 招标范围： 商 （1）蒸汽管道系统本体：从锅炉房分汽缸后（含分气缸阀门）至6#车间、8#车间分气缸处，所有蒸汽管道、管 件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温（含保温层及保 护层）工作。 道 （2）钢结构桁架工程：负责本项目范围内所有钢结构架空桁架（管廊）的采购、运输、制作、安装、防腐工作。 （3）管道附件及控制系统：负责本工程范围内所有阀门、压力表、温度表、流量计、电动/气动执行机构以及配 套仪表电缆、桥架、保护管的采购、运输、安装、接线。负责与DCS/PLC系统接口的接线与联动调试。 管 （4）调试与验收：组织并确保整个蒸汽管道系统（含分气缸后段末端管道、桁架及其安全附件）通过项目所在 地特种设备安全监察管理部门实施的安装监督检验。负责报检、配合现场检验、整改、出具深化图纸并由设计 单位审核盖章、特种设备法定报检取证的全部费用，包括但不限于：施工前办理安装告知，设计院盖章审核， 施工中接受并通过安装国监督检验，最终负责取得《压力管道安装监督检验证书》与《特种设备使用登记证》， 确保蒸汽管道投入使用并备案，提交全套法定检验报告。 （5）土建工作部分 中 1）管架和桁架基础的施工，包括但不限于钢结构桁架的混凝土独立基础的土方开挖、浇筑、养护及回填恢复。 2）管道穿墙/板孔洞的开挖、封堵与修复。 3）室内外地面的开挖（包括但不限于疏水井、沟槽开挖、通行地沟、设备基础开挖）与恢复（包括但不限于土 方回填、渣土弃运、地面硬化）。 4）桁架及设备接地线的施工，包括但不限于接地极制作、接地干线敷设，并与厂区主接地网可靠连接，接地电 阻测试合格。 具体详见施工图、招标文件、工程量清单、答疑补遗等资料。 2.5 工期要求： 60 日历天 缺陷责任期要求： 24 个月 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：投标人应同时具备以下(1)、(2)项资质： （1）具备建设行政主管部门颁发的有效的建筑工程施工总承包二级及以上资质； （2）具备有效的《中华人民共和国特种设备生产许可证》（许可子项目：工业管道安装GC2级及以上）。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 网 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 务 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（涪陵区） （https://www.cqggzy.com/fulingweb/）下载招标文件、工程商量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网（涪陵区道）（https://www.cqggzy.com/fulingweb/）本项目招标公告网页下 方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-23 17:00:00前。 4.3招标人应于2026-08-24 18:00:00前在重庆市公共资源交易网（涪陵区）（https://www.cqggzy.com/fulingweb/）发 布澄清。 5.投标文件递交的内容 管 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-09 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 国 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（涪陵区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 中重庆市涪陵榨菜集团股份有限公司 代理机构: 中招国际招标有限公司 重庆两江新区黄山大道中段53号5-1（双 地 址: 重庆市涪陵区江北街道办事处二渡村一组 地 址: 鱼座A栋5楼） 邮 编: 408000 邮 编: 项目负责人: 徐老师 项目负责人: 寿云凤 电 话: 13212467016 电 话: 023-68881331-9032 传 真: 传 真: 电子邮箱: bsd2me@126.com 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市涪陵区发展和改革委员会 电 话: 023-72203687 2026年08月19日 乌江 涪陵 榨菜 绿色 智能 化生 产基地 (一 期)6#、 8#车 网 间蒸 汽管 道安 装工 务 程 中 中 国 国 重 银 重 商民 重 庆 行 庆 生 庆 涪 股 涪 银 涪 陵 份 陵 行 陵 重 投 公 有 道公 股 公 庆 标 共 限 共 份 共 银 开 保 户 资 公 资 有 资 行 户 证 110292140553VA00154 9902001860445897 430102029007791845-275 名 源 司 源 限 源 涪 行 金 交 重 交 公 交 陵 账 管 易 庆 易 司 易 支 号 有 涪 有 重 有 行 限 陵 限 庆 限 公 马 公 涪 公 国 司 鞍 司 陵 司 支 支 行 行 中 信息来源:https://www.chinapipe.net/project/d3076300.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="n">
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
         <v>95</v>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>重庆, 蒸汽管道, 安装工程, 资金情况, 产品种类</t>
         </is>
@@ -1881,34 +1793,29 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>巴南区</t>
+          <t>完成重庆国际生物城配套公寓项目（民用1020户）天然气表后管道定制化服务。（含安装燃气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个，其它配套管件及辅材，墙体管道暗埋等）</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>完成重庆国际生物城配套公寓项目（民用1020户）天然气表后管道定制化服务。（含安装燃气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个，其它配套管件及辅材，墙体管道暗埋等）</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>天然气表后管道定制化服务</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>天然气表后管道定制化服务</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程询比采购公告 采购公告 公告编号： RQXYGG202608190057 一、采购项目基本情况 采购人：重庆巴南天然气有限责任公司 网 采购项目编号：RQCGXY202608170010 采购项目名称：重庆国际生物城配套公寓项目天然气表后管道安装工程 务 采购内容和范围：完成重庆国际生物城配套公寓项目 （民用1020户）天然气表后管道定制化服务。（含安装燃 气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个， 其它配套管件及辅材，墙体管道暗埋等） 二、供应商资格要求 商 1. 资质要求:资质要求： 1.响应供应商为中华人民共和国境内合法注册的独立法人或其他组织，具有独立承担民事责任能力，具有独立订 立合同的权利。 道 2.响应供应商应具备市政公用工程施工总承包三级及以上资质、具备有效的安全生产许可证。 3.响应供应商应为本项目配备项目负责人一名，持有市政公用工程或机电工程专业二级建造师及以上资质，且为 本单位在职人员并提供社保证明。 4.响应供应商应为本项目配备专职安全员一名，持有安全生产考核合格C证，且为本单位在职人员并提供社保证 管 明。 5.项目负责人及专职安全员社保证明期限须包含2026年5月至2026年7月。提供的社保证明，须体现上述人员的姓 名、身份证号（或社保号）、单位名称、本单位参保时间（或起始参保时间），并带有社保部门公章或社保部 门的有效电子印章。 2. 信用要求:6.信用要求国： （1）响应供应商（含联合体响应的成员单位）未被“国家企业信用信息公示系统” 网站（www.gsxt.gov.cn）列 入严重违法失信企业名单（如：提供网站查询界面截图）； （2）响应供应商（含联合体响应的成员单位）未被 “信用中国”网站（www.creditchina.gov.cn）列入严重失信 主体名单（中如：提供网站查询界面截图）。 三、采购文件的获取 采购文件在 华润守正采购交易平台 发布，不再另行线下提供纸质采购文件，凡有意参与者请自行登录守正平台 查看和下载采购文件。 四、响应文件的提交 响应文件提交 / 报价截止时间： 2026-08-25 08:00:00 （北京时间，若有变化另行通知）。 响应文件提交 / 报价方式：在响应文件提交 / 报价截止时间前，通过 华润守正采购交易平台 提交电子响应文件或 报价，逾期提交将被拒收。 五、采购人联系方式 联系人：何俊 电话：15178855716 邮箱：1460553040@qq.com 六、采购明细 行号 采购内容 需求数量 单位 补充说明 1 重庆国际生物城配套公寓项目天然气表后管道定制化服务 1 元/次 具体内容详见采购文件 七、答疑澄清、通知 答疑澄清、通知等文件一经在 华润守正采购交易平台 发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注 华润守正采购交易平台 发布的相关信息，并及时查阅和处理。 八、服务费交纳 网 本项目向成交人收取服务费,供应商收到预成交通知书和服务费交款通知书10日内,向平台运营方(华润守正招标有 限公司)支付服务费,经确认无误后由采购人发送成交通知书。平台运营方在收到服务费后向成交人开具服务费发 票。 收费标准：项目总成交金额＜50万元的采购项目，免收服务费。项目总成交金额≥50万元的采购项目，按成交金 务 额的0.15%向成交人收取（金额四舍五入，精确到分）。单项目总收费封顶100000元。其他说明：（1）总价采购， 收费基数为成交金额；单价、费率采购，收费基数为预算金额。（2）单项目存在多个成交人情形的，按总成交 金额计算收费总额，各成交人按成交比例分摊；项目总成交金额50万以上，但单个成交人成交金额少于50万仍按 比例收取服务费。 商 退款说明：成交通知书发布后,平台提供相关服务已完成,成交人已交纳服务费不予退还。 多成交人服务费收取示例： 以某项目总成交金额100万为例,A、B、C多成交人情形,总服务费为0.15万, 供应商A成交金额为50万,A服务费为0.075万; 供应商B成交金额为30万,B服务费为0.045万; 道 供应商C成交金额为20万,C服务费为0.03万。 九、其它事项 管 1.本公告在 华润守正采购交易平台 ( https://www.szecp.com.cn/ )上公开发布。 2.本项目采购通过守正平台线上进行，供应商需注册 华润守正采购交易平台 ，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 国 3.如对采购项目有异议，请登录 华润守正采购交易平台 ,通过异议菜单提出。 2026年08月19日 中 信息来源:https://www.chinapipe.net/project/d3076125.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="n">
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
         <v>80</v>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>重庆, 天然气表后管道安装工程, 管材招标</t>
         </is>
@@ -1947,32 +1854,31 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)建设。</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)建设。</t>
+          <t>项目资金来自业主自筹，项目出资比例为100%。本次招标项目货物采购估算金额约为330万元。</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>项目资金来自业主自筹，项目出资比例为100%。本次招标项目货物采购估算金额约为330万元。</t>
+          <t>非金属管道管件阀门</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>非金属管道管件阀门</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)非金属管道管件阀门采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）非金属管道管件阀门采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约 330 万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采 购”包括不限于非金属管道管件阀门所含设计、制造、试验、出厂检验、防腐、运输（含保护、包装及运输、 货到现场车板交货）、保险（交货验收前）、指导安装、调试、备件及专用工具、税费、技术资料和图纸及质 保期内的各种备品、备件的供应及相关的技术服务、产品质量证明书及原材料检测报告等。（详见“第五章货 物需求一览中表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 2.6 交货期： 2.6.1合同签订后3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向买方提交完整的技术资料，以供设计院开展相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）投标人具备有效的《中华人民共和国特种设备生产许可证》压力管道管子-B级及以上资质、压力管道管 件B2级及以上资质； （3）投标人具备塑料管道管子、管件的型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4. 招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年 8 月19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 网 5.投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月10 日上午09时30分，地点在重庆市公共资源交易中心开标厅（地 址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见一、二楼大厅显示屏。 务 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 商 本次招标公告在中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 道 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 管 联 系 人：张先生 电 话：023-40717888 国 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区五里店五简路2号重庆咨询大厦A栋20楼2001室 中 项目负责人：彭文婷 电 话： 023-67703002 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购 户名 开户行 投标保证金账号 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000631258 支行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051303372 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630010400 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000002549 贸易试验区分行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835014652 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146619529 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764260665 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020038958 信息来源:https://www.chinapipe.net/project/d3076119.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="n">
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
         <v>85</v>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 资金, 产品</t>
         </is>
@@ -2011,32 +1917,31 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)，包括衬氟管道及管件的采购。</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)，包括衬氟管道及管件的采购。</t>
+          <t>项目资金来自业主自筹，项目出资比例为100%。货物采购估算金额约为225万元。</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>项目资金来自业主自筹，项目出资比例为100%。货物采购估算金额约为225万元。</t>
+          <t>衬氟管道及管件</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>衬氟管道及管件</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)衬氟管道及管件采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）衬氟管道及管件采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约225万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）衬氟管道及管件采购一批” 包括但不限于制造、涂漆、包装、运输、配合验收工作、检验检测、产品质量证明书等。（详见“第五章货物 （材料）需求一览表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 中 2.6 交货期： 2.6.1合同签订后 3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向招标方提交完整的技术资料，以供设计院开展设备相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）具备有效的《中华人民共和国特种设备生产许可证》-压力管道元件制造-元件组合装置。 （3）具有防腐管道元件特种设备型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4、招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年8 月 19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 5、投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月 10 日上午09时30分，地点在重庆市公共资源交易中心开标厅 （地址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见网一、二楼大厅显示屏。 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 务 本次招标公告在 中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 商 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 道 联 系 人：张先生 电 话：023-40717888 管 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区国五里店五简路2号重庆咨询大厦A栋20楼2001室 项目负责人：彭文婷 电 话： 023-67703002 中 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630011190 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835003139 坝支行 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000000834 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146638621 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051302432 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000620855 支行 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020013554 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764235261 信息来源:https://www.chinapipe.net/project/d3076111.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="n">
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
         <v>85</v>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>重庆, 废盐综合利用, 离子膜烧碱, 衬氟管道, 管件采购</t>
         </is>
@@ -2081,34 +1986,29 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>永川区</t>
+          <t>蒸汽管道改造</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>蒸汽管道改造</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>蒸汽管道</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>蒸汽管道</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
           <t>重庆市益康环保工程有限公司永川分公司蒸汽管道改造项目询价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3076108.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="n">
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
         <v>60</v>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>重庆, 蒸汽管道, 改造项目, 询价采购</t>
         </is>
@@ -2153,34 +2053,29 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>南岸区</t>
+          <t>包括改造市政混接点194个，改造管网8582米，缺陷管网开挖修复1355米，非开挖修复8679米。</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>包括改造市政混接点194个，改造管网8582米，缺陷管网开挖修复1355米，非开挖修复8679米。</t>
+          <t>总投资概算未明确具体金额，但合同预估金额为6600万元。</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>总投资概算未明确具体金额，但合同预估金额为6600万元。</t>
+          <t>排水管网改造</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>排水管网改造</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
           <t>南岸区融侨大道、江南大道片区2023年排水管网改造项目(三标段)招标计划表 重庆市工程建设项目招标计划表 项目名 南岸区融侨大道、江南大道片区 2023年排水管网改造项目（三标段） 称 网 招标法 人或招 重庆市南岸区城市建设发展（集团）有限公司 标人名称 （盖章） 务 项目批 准文件 南岸发改〔2024〕304《南岸区融侨大道、江南大道片区2023年排水管网改造项目总投资概算的批复》 及文号 主要建 包括改造市政混接点194个，改造管网8582米，商管径d300~d1500;缺陷管网开挖修复1355米，管 设内容 径d300~d600;非开挖修复8679米，管径d300~d1200。 招标文件 拟交 合同预估 招标内 招标 序号 招标项目名称 计划发布 易场 金额(万 备注 道容 方式 时间 所 元) 51处雨 污混错 重庆 招标项 接点位 管 市公 目 改 南岸区融侨大道、江南大道片区 2023年排 公开 共资 1 造，1082 2026-08 6600.00 水管网改造项目（三标段） 招标 源交 个管网 易中 三四级 国 心 缺陷修 复。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 中 信息来源:https://www.chinapipe.net/project/d3076097.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="n">
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
         <v>80</v>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>重庆, 排水管网改造, 资金情况, 产品种类</t>
         </is>
@@ -2225,34 +2120,29 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>永川区</t>
+          <t>项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、综合楼、生产建（构）筑物以及附属建筑物等。</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、综合楼、生产建（构）筑物以及附属建筑物等。</t>
+          <t>项目合同额1.7亿元</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>项目合同额1.7亿元</t>
+          <t>钢筋混凝土排水管</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>钢筋混凝土排水管</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
           <t>中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购公告 永川三教水厂项目 已具备采购条件，现公开邀请供应商参加询比采购活动。 1.采购项目简介 1.1 采购项目名称：中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购。 1.2 采购方案编号：FA00000663117。 网 1.3 采购人：中交一公局重庆工程有限公司。 1.4 采购代理机构：/。 务 1.5 采购项目资金：已落实 1.6 采购项目概况： 商 永川三教水厂项目：项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建 净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、 综合楼、生产建（构）筑物以及附属建筑物等。项目合同额1.7亿元，工期450天。 道 项目地址：重庆市永川区。 2.采购范围及相关要求 管 2.1 采购范围：钢筋混凝土排水管。 2.2 交货期：2026年9月-2026年12月。 2.3 交货地点：重庆市永国川区项目指定地点。 2.4 物资质量标准：满足《混凝土和钢筋混凝土排水管》（GB/T 11836-2023）的相关要求。 3.供应商资格要求 中 3.1 供应商应依法设立且满足如下要求： （1）资质要求：本次询比采购要求供应商须是在中华人民共和国境内依法注册，具有合法有效的营业执照、税 务登记、组织机构代码等证件，具有独立法人资格、具有采购物资生产经营范围的生产商或代理商（销售商）。 （2）财务要求：供应商必须是经税务部门注册登记核准的纳税人，有依法纳税的良好记录。 （3）业绩要求：无。 （4）信誉要求：无不良履约记录、未列入工程所在地质量监督部门和中国交建、中交一公局集团企业黑名单。 因质量原因被交通部质监站通报，正在进行整改的生产厂家和产品不得参与投标。生产商或代理商（销售商） 具有良好的社会信誉，近3年内没有与骗取合同有关的犯罪或严重违法行为而引起的诉讼和仲裁；近3年不曾在合 同中严重违约或被逐；财产未被接管或冻结，企业未处于禁止或取消投标状态；在最高人民法院、信用中国 （www.creditchina.gov.cn）或各级信用信息共享平台查询拟入库单位无不良行为记录。 （5）其他要求：无。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他：无。 4.供应商报名 4.1 有意参加询比采购活动的单位，请于2026年8月19日15时00分至2026年8月26日17时00分（北京时间，下同，法 定公休日、节假日不休），登录“中交招采网”（网址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 网 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 务 5.供应商报价 5.1 报价结束（递交响应文件截止）时间为2026年8月26日17时00分。 商 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的电 子响应文件，采购人将拒收。 5.3电子采购的供应商响应文件由线上电子报价道表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 子报价表的数据为准。 6.开标 管 6.1 开标时间：与报价结束时间相同。 6.2 开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标。 国 7.发布公告的媒介 本询比采购公告在 “中交招采网” 上发布。 中 8.评审办法 本项目评审办法采用 经评审的最低价法 。 9.合同主要条款 9.1 付款条件：按月结算，上月11日至本月10日为一个结算对账期，乙方必须按照甲方要求开具合规的增值税专 用发票，无发票不予付款。结算完成后1个月内支付已结算金额的70%，剩余30%货款在结算完成后3个月内支付。 付款方式为银行转账，甲方有权采用票据支付或者供应链支付的方式支付货款，因此产生的费用包含在综合单 价中，乙方不得因此调价和索赔。如遇业主支付不及时，乙方应予理解。 9.2 履约保证金的递交： （1）R不要求递交 （2）要求递交，保证金金额：/，保证金形式：/，其他形式：/ 。 10.监督机构 监督机构名称： 中交一公局重庆工程有限公司审计部 11.成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联系400-676-5885，中标服务费请按7咨询。 11.1 收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； （3）在1000万元（含）至3000万元之间的，每次收取1000元； 务 （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 11.2 支付流程 （1）通知推送：中标结果发布后，系统自动推送缴费通知（含应缴金额及支付链接）； 道 （2）费用查询：供应商登录“中交招采网—供应商协同—服务费”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网— 供应商协同—服务费—发票查询”模块获取。 12.其他 国 / 。 13.联系方式 中 采 购 人：中交一公局重庆工程有限公司 地 址：重庆市江北区创富路5号 邮 编：361021 联 系 人：汪仁宽 电 话：13527572392 电子邮件：1176245792@qq.com 项目联系人及电话： 序号 项目名称 联系人 联系电话 1 永川三教水厂项目 高博 17788661005 中交一公局重庆工程有限公司 2026年8月19日 物资信息 序号 设备物资名称 设备物资说明 税率 单位 网 1 钢筋混凝土排水管 2000mm Ⅲ级 承插口 13% 米 信息来源:https://www.chinapipe.net/project/d3076078.html 务 cqdingjiu 2026.08.21 10:06:52 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="n">
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="n">
         <v>90</v>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 钢筋混泥土排水管, 永川三教水厂项目</t>
         </is>
@@ -2297,34 +2187,29 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>云阳县</t>
+          <t>新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。</t>
+          <t>合同预估金额：9100.00万元</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>合同预估金额：9100.00万元</t>
+          <t>污水管网</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>污水管网</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
           <t>长江流域云阳青龙段污水管网一体化建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 长江流域云阳青龙段污水管网一体化建设项目 招标法人或 招标人名称 云阳县青江环境综合整治有限公司 网 （盖章） 项目批准文 云阳发改资环【2025】55号 件及文号 务 主要建设内 新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。 容 招标方 招标文件计 拟交易场 合同预估金额 序号 招标项目名称 招标内容 备注 式 划发布时间 所 (万元) 商 长江流域云阳 新建污水管网55.5千米， 重庆市公 青龙段污水管 其中DN200管网12千 公开招 共资源交 1 网一体化建设 米、DN300管网24千 2026-08 9100.00 标 易中心云 项目EPC总承 米、DN40道0管网19.5千 招标项目 阳分中心 包 米等。 新建污水管网55.5千米， 长江流域云阳 重庆市公 其中DN200管网12千 青龙段污水管 公开招 共资源交 2 管米、DN300管网24千 2026-08 140.00 网一体化建设 标 易中心云 米、DN400管网19.5千 项目监理 阳分中心 米等监理。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 国 信息来源:https://www.chinapipe.net/project/d3075867.html cqdingjiu 2026.08.21 10:06:53 中</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="n">
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
         <v>80</v>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 污水管网, 资金情况, 产品种类</t>
         </is>
@@ -2363,32 +2248,31 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3站5区间的土建）：高龙大道站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子站区间、石家院子站～终点区间、7/17号线联络线区间。采购范围为雨污水排水迁改工程。</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3站5区间的土建）：高龙大道站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子站区间、石家院子站～终点区间、7/17号线联络线区间。采购范围为雨污水排水迁改工程。</t>
+          <t>建设资金来源已落实，但具体资金数额未明确。</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>建设资金来源已落实，但具体资金数额未明确。</t>
+          <t>雨污水排水迁改工程</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>雨污水排水迁改工程</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
           <t>中国电建水电四局华中公司重庆轨道交通17号线一期5标项目雨污水排水迁改工程施工劳务分包采购项目公开询 比采购公告 询比采购公告 采购编号： PC-0104-26J6-FP0895 一、采购条件 受中国水利水电第四工程局有限公司重庆轨道交通17号线一期5标项目委托，中水电四局华中（武汉）工程有限 公司以公开询比方式采购重庆轨道交通17号线一期5标雨污水排水迁改工程项目网，建设资金来源已落实。目前项 目已具备采购条件，现进行公开询比采购。 二、项目概况、采购范围 务 1、项目概况：重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3 站5 区间的土建）：高龙大道 站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子 站区间、石家院子站～终点区间、7/17号线联络线区间。 2、采购范围： 商 （1）雨污水排水迁改工程 （2）工程招标范围工作内容：17号线一期5标道中高龙大道站、斑竹林站及高斑竖井位于城市既有道路下方，设计 采用明挖法施工。为保证市政排水管网的正常使用，在明挖施工前需对既有管网进行临时迁改，车站结构施工 后进行恢复。施工PE钢带管长度2387米、B型排水管长度2799m、钢筋混凝土管127米，检查井239座劳务部分。 （3）施工内容详见工程量清单，以及为完成此项工程而做的一切工作。 管 3、计划工期:计划开工日期：2026年9月25日（具体时间以采购人通知为准），计划完工日期：2027年 12 月25 日； 合同工期总日历天数为457天。 4、质量要求：符合《国给水排水管道工程施工及验收规范》（GB 50268）、《混凝土结构工程施工质量验收规范》 （GB 50204）、《城镇道路工程施工与质量验收规范》（CJJ 1-2008）以及项目所在地最新的相关法规、标准和 图集。工程质量全面达到设计要求和标准，其中：验收合格率 100%，优良率达 90%以上，工程综合验收质量评 定达优良标准。 中 5、付款方式：采用银行转账/支票支付工程价款，月度结算完成具备付款条件后30天内工程进度款支付比例约定 为扣除各项保证金及费用后应付价款不低于65%；清算完成并签订《退场协议》后30天内工程进度款支付比例约 定为扣除各项保证金及费用后应付价款不低于80%；清算完成并签订《退场协议》后一年内工程进度款支付比例 约定为扣除响应人缺陷责任等相关费用后应付价款不低于90%；清算完成并签订《退场协议》，办理完成保证金 退还手续后两年内，工程进度款支付比例约定为扣除响应人缺陷责任等相关费用后应付价款的100%。 6、其他：无。 三、响应人资格要求 响应人必须满足以下全部资格要求： （1）资质要求：施工劳务不分等级 （2）主要人员要求:授权委托人（如有）及项目经理、专职安全员应提供社保和劳动合同。其中劳动合同至少提 供首、末两页，并且包含有关人员的详细信息;社保证明应提供响应截止时间前三个月的社保缴纳记录。 （3）安全三类人员要求:应提供企业主要负责人安全A证、项目经理B证、专职安全员C证。 （4）响应人具有良好的银行资信和商业信誉，没有处于被责令停业，财产被接管、冻结、破产状态。 （5）响应人应具有 雨污水排水迁改 工程的施工业绩，在近 5年内(2021年7月-2026年7月内签订)的施工合同不少 于 1 个，且签订单项合同金额均在 100 万元以上（应附成交通知书和（或）合同扫描件）。 （6）其它要求:无。 （7）本次采购不接受联合体响应。 四、采购文件的获取 凡满足本公告规定资格要求并有意参加的响应人，请于2026年8月22日10时00分前在中国电建采购招标数智化平台 （https://bid.powerchina.cn/bidweb/#/login，以下简称“数智化平台”）获取采购文件，采购文件免费提供。 五、响应文件的递交 1、响应文件递交的截止时间（响应截止时间，下同）为2026年8月26日10时30分网（北京时间），响应人应在截止 时间前通过数智化平台递交电子响应文件。 2、本次采购将通过数智化平台全程在线开展，电子响应文件的加密、提交等流程须响应人在线进行操作。响应 人须提前办理数字证书用于在线递交响应文件，办理方式详见数智化平台首页，并严格按照要求进行在线操作， 务 因操作流程失误造成的递交失败将由响应人自行承担后果。 3、开启由“数智化平台”在响应截止时间后自动对响应文件进行解密，响应人及时关注开启结果。 4、响应截止时间如有变动，采购人将及时通知已获取采商购文件的响应人。 六、发布公告的媒介 本次询比采购公告同时在中国电建阳光采购网道（https://bid-zb.powerchina.cn）上发布。 七、评审办法 采用综合评估法。 管 八、联系方式 采 购 人： 中水电四局华中（武汉）工程有限公司 国 地 址： 湖北省武汉市江岸区塔子湖东路健美街30号立城中心商务楼13、14层 邮 编： 430014 中 联 系 人： 王飞 电 话： 15827222587 电子邮箱： 107830343@qq.com 九、提出异议的渠道和方式 单位名称： 中水电四局华中（武汉）工程有限公司 电 话： 17708178186 电子邮箱： sjhzgsjw@163.com 十、纪检监督机构 响应人或者其他利害关系人认为本次采购活动存在违规违纪行为的，可以书面形式向中国水利水电第四工程局 有限公司中水电四局华中（武汉）工程有限公司纪委办公室（联系方式：17708178186）提出投诉。 2026年8月 19 日 报价网址:https://bid.powerchina.cn/notice/detail?id=2409510708 信息来源:https://www.chinapipe.net/project/d3075750.html cqdingjiu 2026.08.21 10:06:53 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="n">
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
         <v>85</v>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>重庆, 轨道交通, 雨污水排水迁改, 施工劳务分包</t>
         </is>
@@ -2433,34 +2317,29 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>万州区</t>
+          <t>本项目涉及预制钢筋砼管、成品混凝土仿木栏杆等材料的采购。</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>本项目涉及预制钢筋砼管、成品混凝土仿木栏杆等材料的采购。</t>
+          <t>建设资金为国债资金，项目出资比例为100%。具体预算金额未在文本中明确列出。</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>建设资金为国债资金，项目出资比例为100%。具体预算金额未在文本中明确列出。</t>
+          <t>预制钢筋砼管,成品混凝土仿木栏杆</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>预制钢筋砼管,成品混凝土仿木栏杆</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
           <t>万州区2026年超长期特别国债高标准农田建设项目拟进行预制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜的 信息公告 1.采购条件 1.1本项目万州区2026年超长期特别国债高标准农田建设项目工程已由 重庆市万州路桥建设有限公司承建，项目 业主为重庆市万州区农业技术与机械推广中心，代建业主为重庆市万州区农业发展有限公司，建设资金为国债 资金，项目出资比例为 100% ，承包人为重庆市万州路桥建设有限公司。项目已具备施工条件，现对该项目的预 制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜发布信息公告。 网 2.项目概况与采购范围 2.1建设地点：重庆市万州区走马镇、瀼渡镇、罗田镇、余家镇、高梁镇、分水镇、柱山乡等7个镇乡。 务 2.2本项目材料采购拟进行比选情况如下： 罗田镇谷山片区材料采购费暂定金额约： 17.5万元； 余家镇桥亭片区材料采购费暂定金额约： 17.99万元； 商 柱山乡山田片区材料采购费暂定金额约： 26.32 万元； 走马镇凉风片区材料采购费暂定金额约： 15.道66万元； 瀼渡镇高村片区材料采购费暂定金额约： 17.72 万元； 分水镇大冲片区材料采购费暂定金额约： 47.12 万元； 管 高梁镇茨坪片区材料采购费暂定金额约： 10.7万元； （以上片区片区金额为暂定金额，最终比选限价金额以比选文件为准）。 国 2.3计划采购周期： 以合同签订为准 日历天。 2.4采购范围：本项目各片区所包含的预制钢筋砼管、成品混凝土仿木栏杆等材料。 中 3.供应商资格要求 3.1本次材料采购要求供应商具备独立企业法人，具有本次所需材料生产能力的厂家或经销商等，其经营范围和 权限应满足本次所需材料的要求，并依法取得国家行政主管部门颁发的有效工商营业执照(建筑材料销售或水泥 制品制造、水泥制品销售等相关营业资格），所提供产品必须满足各项检测要求，达到国家现行标准规定的合 格标准。具有良好的商业信誉和充分的供应保障能力，具备相应售后服务能力。要求竞选人为一般纳税人，可 开具13%税率增值税专用发票，提供一般纳税人认定证明。 3.2本次供应商单位优先选择万州本地企业。 3.3本次 不接受 联合体竞选。 4. 报名要求 4.1报名时间：2026年8月 19日9:00起至 8月21日17:00止。 4.2报名地点：重庆市万州路桥建设有限公司经营部（重庆市万州区天城东路278号）。 4.3报名时，须提交有效的营业执照(有效工商营业执照((建筑材料销售或水泥制品制造、水泥制品销售等相关营 业资格）)，前述证书均为复印件并加盖单位公章。法定代表人参加报名的不需要授权委托书，只需要提供法定 代表人身份证明；非法定代表人参加报名的除提供法定代表人身份证明外还须提供授权委托书、委托代理人身 份证明。 4.4 本项目材料采购需提前报名。经资格预审合格后，通知资格预审合格的供应商，到承包人单位领取相关文件。 4.5本项目材料采购设七个片区进行比选，为保证比选公平、公正、有效，规定同一参选单位报名片区上限为2个， 且最终仅限中选一个片区。 5.联系方式 承包人：重庆市万州路桥建设有限公司 地 址：重庆市万州区天城东路278号 网 联系人： 张红娟 电 话：15923491915 务 邮 箱： 商 重庆市万州路桥建设有限公司 2026年8月19日 道 信息来源:https://www.chinapipe.net/project/d3075512.html cqdingjiu 2026.08.21 10:06:53 管 国 中</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="n">
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="n">
         <v>80</v>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>重庆, 预制钢筋砼管, 成品混凝土仿木栏杆, 国债资金, 高标准农田建设</t>
         </is>
@@ -2505,34 +2384,29 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>酉阳土家族苗族自治县</t>
+          <t>酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水管道)公开招标采购。</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水管道)公开招标采购。</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>污水管道</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>污水管道</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
           <t>中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水 管道)招标采购流标公告 发布单位：中国铁建/中铁十一局/六公司 发布时间：2026-08-19 10:40:49 投标截至时间：2026-08-18 10:00:00 内容： 各投标人： 网 中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资（污水 管道）公开招标采购（采购编号： CR1106-JC-2026-26-02）评标工作，已于北京时间2026年08月18日10:00整，在 铁建云链（https://www.crccep.com）线上平台公开开标。评审委员会根据招标文件载明的评审办法完成评审工作， 现将评审结果公示如下： 务 一、招标公告发布日期及媒体 招标公告发布日期：2026年07月27日至2026年08月01日 商 招标公告媒体：铁建云链（https://www.crccep.com） 二、拟中标信息 道 公开招标采购编号：CR1106-JC-2026-26-02 包件号：WSGD-01 序号 供应商名称 推荐排序 管 1 无 1 国 以上包件有效投标不足三家，本次招标做流标处理。 三、公示时间 中 自2026年08月19日始，至2026年08月22日止。在公示期间，所有竞标人和其他利害关系人如对公示的评审结果有 异议，可以向相关监督部门举报，逾期将不再受理。举报人必须由其法定代表人或者授权代表签字并盖章，其 他组织或者个人举报的，必须由其主要负责人或者本人签字，并附有效身份证明复印件。举报人如实反映情况 受法律保护。 公示期满，如无异议，即时生效。 监督竞诉受理部门： 中铁十一局集团第六工程有限公司招采中心 联系电话：18671041790 信息来源:https://www.chinapipe.net/project/d3075461.html cqdingjiu 2026.08.21 10:06:53</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="n">
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="n">
         <v>80</v>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 酉阳县, 污水管网, 新建改造工程</t>
         </is>
@@ -2571,32 +2445,31 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>详见附件。</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>详见附件。</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>镀锌管件</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>镀锌管件</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
           <t>协同创新区-四期房建三标段镀锌管件物资竞价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3075420.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="n">
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="n">
         <v>60</v>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 商机</t>
         </is>
@@ -2641,34 +2514,29 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>新建一体化提升泵站及管道约5000m，投资约800万元。</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>新建一体化提升泵站及管道约5000m，投资约800万元。</t>
+          <t>投资约800万元</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>投资约800万元</t>
+          <t>施工</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>施工</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
           <t>中化重庆涪陵化工搬迁后污水处理厂建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 中化重庆涪陵化工搬迁后污水处理厂建设项目 招标法人或 招标人名称 重庆市涪陵交通旅游建设投资集团有限公司 网 （盖章） 项目批准文 涪发改委发[2019] 505号 件及文号 务 主要建设内 新建一体化提升泵站及管道约5000m，投资约800万元。 容 招标 招标 招标文件计 拟交易 合同预估 序号 招标项目名称 备注 内容 方式 划发布时间 场所 金额(万元) 商 本招标计划与2026年5 月25日发布的招标项目 中化重庆涪陵 重庆市 名称为“中化重庆涪陵 招标项目 化工搬迁后污 涪陵区 公道开 化工搬迁后污水处理厂 1 水处理厂建设 施工 2026-09 公共资 800.00 招标 建设项目（场外连接管 项目（场外干 源交易 网）”的招标计划，除 管部分） 中心 招标项目名称调整外， 其余内容完全一致。 管 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075591.html cqdingjiu 2026.08.21 10:国06:54 中</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="n">
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="n">
         <v>80</v>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 商机</t>
         </is>
@@ -2713,34 +2581,29 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>綦江区</t>
+          <t>对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造，包括配电柜、风机、污水提升泵、在线监测等设备的更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造，包括配电柜、风机、污水提升泵、在线监测等设备的更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。</t>
+          <t>上级补助和业主自筹，项目出资比例为100%，本项目工程总投资金额约1327.40万元</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>上级补助和业主自筹，项目出资比例为100%，本项目工程总投资金额约1327.40万元</t>
+          <t>污水处理设施设备</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>污水处理设施设备</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
           <t>綦江区污水处理厂设施设备更新改造工程(二期)招标公告 1.招标条件 本招标项目 綦江区污水处理厂设施设备更新改造工程（二期） 已由 重庆市綦江区发展和改革委员会 以 重庆市企业投资备案证（项目代码：2502-500110-04-01-844057） 批准建设，项目业主为 重庆南州城市管 理服务有限公司 ，建设资金来自 上级补助和业主自筹 ，项目出资比例为 100% ，招标人为 重庆南州 城市管理服务有限公司。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用经评审的最低 投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 綦江区 2.2 项目概况与建设规模：对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造， 务 包括配电柜、风机、污水提升泵、在线监测等设备更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污 水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。 2.3 本项目工程总投资金额： 约1327.40万元 商 2.4 招标范围： 本项目设计施工图和招标文件、答疑、补遗、工程量清单等资料所涉及的全部内容。 2.5 工期要求： 180日历天 道 缺陷责任期要求： 24个月 2.6 标段划分（如有）： / 管 2.7 其他： / 3.政府采购工程 国 3.1 是否属于政府采购工程：否 4.投标人资格要求 中 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（綦江区） （https://www.cqggzy.com/qijiangweb/）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网（綦江区）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间 从本公告发布至2026-08-22 18:00:00前。 5.3招标人应于2026-09-11 18:00:00前在重庆市公共资源交易网（綦江区）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（綦江区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆南州城市管理服务有限公司 代理机构: 永卓国际工程技术有限公司 地 址: 重庆市綦江区红星美凯龙生活广场3幢19-3 地 址: 两江新区网泰山大道东段98号2幢10-12号 邮 编: 邮 编: 项目负责人: 赵老师 项目负责人: 廖淼 电 话: 023-48690537 电 话: 务023-60391733 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 商开户银行: 账 号: 账 号: 监督部门: 道 电 话: 2026年08月18日 綦江区污水处理厂设施设备更新改造工程（二期） 管 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051287453 中国农业银行股份有限公司重庆自由贸 重庆联合产权交易所集国团股份有限公司 312601010400083780000031123 易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146631326 信息来源:https://www.chinapipe.net/project/d3075589.html 中 cqdingjiu 2026.08.21 10:06:54</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="n">
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="n">
         <v>90</v>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>重庆, 綦江区, 污水处理厂, 设施设备更新改造, 管材招标</t>
         </is>
@@ -2785,34 +2648,29 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>南岸区</t>
+          <t>本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统，对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平台。</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统，对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平台。</t>
+          <t>概算批复工程建安费2975.27万元。</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>概算批复工程建安费2975.27万元。</t>
+          <t>农村供水管网、智慧加压泵站、水厂升级改造、智能控制系统、加药系统、金属防腐工程、入户管道、入户水表、监测计量基础设施。</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>农村供水管网、智慧加压泵站、水厂升级改造、智能控制系统、加药系统、金属防腐工程、入户管道、入户水表、监测计量基础设施。</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
           <t>南岸区峡口、迎龙片区农村供水保障提升工程招标计划表 重庆市工程建设项目招标计划表 项目 南岸区峡口、迎龙片区农村供水保障提升工程 名称 招标 网 法人 或招 标人 重庆市江南城市建设发展（集团）有限公司 名称 务 （盖 章） 项目 批准 商 文件 南岸发改﹝2026﹞156号 及文 号 本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体 主要 化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统， 建设 对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平 内容 台。概算批复工程建安费2975.27万元。 管 拟 招 招标文 合同预 招标 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 国 所 南岸 重 区峡 庆 口、 中 市 迎龙 朱家岩水厂升级改造工程：对全厂老旧设备进行设备更新；对全 公 片区 公 厂进行智慧化改造，增加高级工艺控制系统；对厂区建筑和构筑 共 农村 开 1 物修缮；优化加药系统投加模式，增加精确加药系统；对全厂部 2026-08 资 1600.00 供水 招 分老旧管道进行更换；金属防腐工程，对金属设备和管道的防锈 源 保障 标 刷漆工作。 交 提升 招标 易 工程 项目 中 （一 心 标段） 南岸 重 区峡 庆 口、 市 迎龙 公 片区 管网工程：延伸、改造峡口镇、迎龙镇等4个乡镇 46 公里 公 共 农村 DN40~DN300 配水主支管，36公里 DN20入户管道，新建3座一体 开 2 2026-08 资 1300.00 供水 化智慧加压泵房，入户水表改造 1752 户，并配套建设监测计量 招 源 保障 基础设施。 标 交 提升 易 工程 中 （二 心 标段） 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075572.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="n">
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="n">
         <v>90</v>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>重庆, 农村供水保障提升工程, 管材招标, 资金情况, 产品种类</t>
         </is>
@@ -2857,34 +2715,29 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>北碚区</t>
+          <t>工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水主要建设内容管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网附属设施。</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水主要建设内容管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网附属设施。</t>
+          <t>合同预估金额为8457万元</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>合同预估金额为8457万元</t>
+          <t>供水管网</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>供水管网</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
           <t>北碚区东阳天府片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区东阳天府片区农村供水提升工程 招标法人或招 标人名称（盖 重庆北碚文旅产业发展有限公司 网 章） 项目批准文件 及文号 务 工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水 主要建设内容 管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网 附属设施。 招标项目名 招标内 招标方 招标文件计划 拟交易场 合同预估金 序号 商 备注 称 容 式 发布时间 所 额(万元) 北碚区东阳 招标项目 重庆市公 天府片区农 施工招 公开招 1 2026-08 共资源交 8457.00 村供水提升 标 道标 易中心 工程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075569.html 管 cqdingjiu 2026.08.21 10:06:55 国 中</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="n">
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="n">
         <v>80</v>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 农村供水提升工程, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -2929,34 +2782,29 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>北碚区</t>
+          <t>改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供水管网68.5km及其附属设施。</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供水管网68.5km及其附属设施。</t>
+          <t>合同预估金额：8741.00万元</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>合同预估金额：8741.00万元</t>
+          <t>供水管网及相关附属设施</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>供水管网及相关附属设施</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
           <t>北碚区澄江片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区澄江片区农村供水提升工程 招标法人或招标 重庆北碚文旅产业发展有限公司 人名称（盖章） 网 项目批准文件及 文号 改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供 主要建设内容 务 水管网68.5km及其附属设施。 招标项目名 招标文件计划 合同预估金 序号 招标内容 招标方式 拟交易场所 备注 称 发布时间 额(万元) 招标项目 北碚区澄江 商重庆市公共 1 片区农村供 施工招标 公开招标 2026-08 资源交易中 8741.00 水提升工程 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 道 信息来源:https://www.chinapipe.net/project/d3075568.html cqdingjiu 2026.08.21 10:06:55 管 国 中</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="n">
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="n">
         <v>80</v>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 商机</t>
         </is>
@@ -3001,34 +2849,29 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>主要改造及延伸配水管188.2千米，新建加压泵站4座，新建计量监测设施建设以及配套电气工程。</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>主要改造及延伸配水管188.2千米，新建加压泵站4座，新建计量监测设施建设以及配套电气工程。</t>
+          <t>预算金额为3137.22万元</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>预算金额为3137.22万元</t>
+          <t>管道、加压泵站、计量监测设施、电气设备</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>管道、加压泵站、计量监测设施、电气设备</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
           <t>涪陵区江东街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区江东街道农村供水保障能力提升工程（二期） 名称 招标 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 项目 网 批准 文件 涪陵发改〔2026〕471号 及文 号 主要 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 建设 以及配套电气工程。 务 内容 招 标 合 文 同 招 件 预 招标 标 招标方 计 拟交易 备 序号 招标项目名商称 估 项目 内 式 划 场所 注 金额 容 发 (万 布 元) 时 间 重 道 庆 市 涪 陵 公 区 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 开 公 1 涪陵区江东街道农村供水保障能力提升工程（二期） 2026-09 3137.22 管以及配套电气工程。 招 共 标 资 源 交 易 中 心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075558.html cqdingjiu 2026.08.21 10:06:55 中</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="n">
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="n">
         <v>80</v>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -3073,34 +2916,29 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>改造荣桂水厂老化、破损、生锈的输水管道7.36公里。马武水厂增设废水回收及污泥浓缩系统1套。荣桂水厂增设废水回收及污泥浓缩系统1套。新建配水管道总长0.74公里；改造配水管道总长139.42公里。新建1座微型集成泵房及改造1座泵站(原牌坊泵站)。新增管网监测设施40套。</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>改造荣桂水厂老化、破损、生锈的输水管道7.36公里。马武水厂增设废水回收及污泥浓缩系统1套。荣桂水厂增设废水回收及污泥浓缩系统1套。新建配水管道总长0.74公里；改造配水管道总长139.42公里。新建1座微型集成泵房及改造1座泵站(原牌坊泵站)。新增管网监测设施40套。</t>
+          <t>预估合同金额为3236.36万元人民币</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>预估合同金额为3236.36万元人民币</t>
+          <t>输水管道、废水回收及污泥浓缩系统、配水管道、微型集成泵房、泵站、管网监测设施</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>输水管道、废水回收及污泥浓缩系统、配水管道、微型集成泵房、泵站、管网监测设施</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
           <t>涪陵区龙桥街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 涪陵区龙桥街道农村供水保障能力 项目名称 提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水 名称（盖 有限公司 章） 网 项目批准 文件及文 涪陵发改〔2026〕466号 号 改造荣桂水厂老化、破损、生锈的 务 输水管道7.36公里。马武水厂增设 废水回收及污泥浓缩系统1套。荣 桂水厂增设废水回收及污泥浓缩系 主要建设 统1套。新建配水管道总长0.74公里； 商 内容 改造配水管道总长139.42公里。新 建1座微型集成泵房及改造1座泵 站(原牌坊泵站)。新增管网监测设 施40套。 道 招标 合同 招 文件 预估 标 招标方 拟交易 备 招标项目 序号 招标项目名称 计划 金 内 式 场所 注 管 发布 额(万 容 时间 元) 改造荣桂水厂老化、 破损、生锈的输水管 国 道7.36公里。马武水厂 增设废水回收及污泥 重庆 浓缩系统1套。荣桂水 市涪 厂增设废水回收及污 公 陵区 中 涪陵区龙桥街道农村供水保障能力 泥浓缩系统1套。新建 开 1 2026-09 公共 3236.36 提升工程 配水管道总长0.74公里； 招 资源 改造配水管道总 标 交易 长139.42公里。新建1 中心 座微型集成泵房及改 造1座泵站(原牌坊泵 站)。新增管网监测设 施40套。 本计划表所列招标项目信息均为暂 备注 定，最终以实际招标时的信 信息来源:https://www.chinapipe.net/project/d3075556.html cqdingjiu 2026.08.21 10:06:55</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="n">
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="n">
         <v>90</v>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>涪陵区龙桥街道, 农村供水保障能力提升工程, 输水管道, 废水回收及污泥浓缩系统, 配水管道, 微型集成泵房, 泵站, 管网监测设施</t>
         </is>
@@ -3145,34 +2983,29 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>整治De315原水管长1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>整治De315原水管长1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。</t>
+          <t>合同金额1489.90万元</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>合同金额1489.90万元</t>
+          <t>管材、水泵、加压泵站、废水处理系统、电气工程</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>管材、水泵、加压泵站、废水处理系统、电气工程</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
           <t>涪陵区百胜镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区百胜镇农村供水保障能力提升工程 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕465号 及文 号 务 主要 建设整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。 内容 招 拟 标 招招标文 合同预 交 序项 标件计划 估金 备 招标内容 易 号目 方发布时 额(万 注 场 名 商 式间 所 元) 称 涪 陵 区 重 百 庆 胜 市 招标 镇 涪 项目 农 道 陵 村 公 区 供整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1开 公 1 2026-09 1489.90 水套及配套电气工程。 招 共 保 标 资 障 源 能 交 力 易 提 中 管 升 心 工 程 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075553.html 国 cqdingjiu 2026.08.21 10:06:55 中</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="n">
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="n">
         <v>80</v>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>涪陵区百胜镇, 农村供水保障能力提升工程, 管材招标, 重庆</t>
         </is>
@@ -3217,34 +3050,29 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>对清溪水厂原取水口进行改造。改造清溪厂输水管道长6.38公里。清溪水厂新建3000m³/d集成水厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04公里。四合村泵站增加1套备用加压泵。新增管网监测设施35套。</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>对清溪水厂原取水口进行改造。改造清溪厂输水管道长6.38公里。清溪水厂新建3000m³/d集成水厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04公里。四合村泵站增加1套备用加压泵。新增管网监测设施35套。</t>
+          <t>合同预估金额：2888.89万元</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>合同预估金额：2888.89万元</t>
+          <t>集成水厂、输水管道、配水管道、加压泵、管网监测设施</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>集成水厂、输水管道、配水管道、加压泵、管网监测设施</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
           <t>涪陵区清溪镇农村供水保障能力提升工程招标计划 重庆市工程建设项目招标计划表 项目名称 涪陵区清溪镇农村供水保障能力提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕467号 务 号 对清溪水厂原取水口进行改造。改造清溪水厂输水管道长6.38公里。清溪水厂新建3000m3/d集成水 主要建设 厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04 内容 公里。四合村泵站增加1套备用加压泵。新商增管网监测设施35套。 招标项目 招标方 招标文件计 拟交易场 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 所 (万元) 对清溪水厂原道取水口进行 改造。改造清溪水厂输水 管道长6.38公里。清溪水厂 涪陵区清 新建3000m3/d集成水厂1套， 重庆市涪 招标项目 溪镇农村 增设废水回收及污泥浓缩 公开招 陵区公共 管 1 供水保障 2026-09 2888.89 系统1套。新建配水管道总 标 资源交易 能力提升 长2.46公里。改造配水管道 中心 工程 总长145.04公里。四合村泵 站增加1套备用加压泵。新 国 增管网监测设施35套。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075552.html 中 cqdingjiu 2026.08.21 10:06:55</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="n">
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="n">
         <v>80</v>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -3289,34 +3117,29 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>改造11000m³/d(旺水垭6000m³/d和二水厂5000m³/d)原水处理系统及辅助设施，主要包括加氯系统、加药系统、清水池、絮凝池、重力无阀滤池、污水处理回收池、二水厂泵房设备等及其他辅助设施。更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km，新建应急泵站至百汇大桥配水管9km；百汇至观将泵站4.5km；共计37.3km。</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>改造11000m³/d(旺水垭6000m³/d和二水厂5000m³/d)原水处理系统及辅助设施，主要包括加氯系统、加药系统、清水池、絮凝池、重力无阀滤池、污水处理回收池、二水厂泵房设备等及其他辅助设施。更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km，新建应急泵站至百汇大桥配水管9km；百汇至观将泵站4.5km；共计37.3km。</t>
+          <t>合同预估金额3427.27万元</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>合同预估金额3427.27万元</t>
+          <t>管材</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>管材</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
           <t>涪陵区珍溪镇农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区珍溪镇农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕476号 及文号 (一)改造11000m3/d(旺水垭6000m3/d和二水厂5000m3/d)原水处理系统及辅助设施，主要有加氯系统、 加药系统、清水池、絮凝池、重力无阀滤池、商污水处理回收池、二水厂泵房设备等及其他辅助设施。 主要建 (二)更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪 设内容 湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km， 新建应急泵站至百汇大桥配水管9km：百汇至观将泵站4.5km；共计37.3km。 道 招标项目 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 场所 (万元) (一)改造11000m3/d(旺水 垭6000m3/d和二水厂5000m3/d) 管 原水处理系统及辅助设施，主 要有加氯系统、加药系统、清 水池、絮凝池、重力无阀滤池、 污水处理回收池、二水厂泵房 涪陵国区珍 设备等及其他辅助设施。(二) 重庆市 招标项 溪镇农村 更换旺水垭水厂至张家塘配水 涪陵区 目 供水保障 公开招 1 管13.5km，张家塘至滴水配水 2026-09 公共资 3427.27 能力提升 标 管长3.3km，全长16.8km；滴水 源交易 中工程（一 至洪湖配水管长0.3km；更换八 中心 期） 一水库至旺水垭水厂引水 管1.7km，更换珍溪二水厂至珍 溪大桥配水管5km，新建应急 泵站至百汇大桥配水管9km： 百汇至观将泵站4.5km；共 计37.3km。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075551.html cqdingjiu 2026.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="n">
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="n">
         <v>80</v>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 供水, 改造</t>
         </is>
@@ -3361,34 +3184,29 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>新建及整治输配水管网总长124.26千米，新建加压泵站5座，新建高位水箱4座（总容积354立方米），武陵山水厂新建废水处理系统1套及配套电气工程等。</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>新建及整治输配水管网总长124.26千米，新建加压泵站5座，新建高位水箱4座（总容积354立方米），武陵山水厂新建废水处理系统1套及配套电气工程等。</t>
+          <t>合同预估金额1861.77万元</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>合同预估金额1861.77万元</t>
+          <t>输配水管网、加压泵站、高位水箱、废水处理系统、电气工程</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>输配水管网、加压泵站、高位水箱、废水处理系统、电气工程</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
           <t>涪陵区武陵山镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区武陵山镇农村供水保障能力提升工程 名称 招标 网 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 务 （盖 章） 项目 批准 商 文件 涪陵发改〔2026〕468号 及文 号 主要 道 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高位水箱4座（总容积 354立方米），武 建设 陵山水厂新建废水处理系统1套及配套电气工程等。 内容 招 管 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 国 称 涪 陵 区 中 重 武 庆 陵 市 山 招标 涪 镇 项目 陵 农 公 区 村 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高 开 公 1 供 位水箱4座（总容积 354立方米），武陵山水厂新建废水处理系统1套 2026-09 1861.77 招 共 水 及配套电气工程等。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075549.html cqdingjiu 2026.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="n">
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="n">
         <v>80</v>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>涪陵区武陵山镇, 农村供水保障能力提升工程, 重庆, 输配水管网, 加压泵站, 高位水箱, 废水处理系统, 电气工程</t>
         </is>
@@ -3433,34 +3251,29 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>建设配水管网总长34.80km，新建加压泵站2座、改造已成泵站2座、新建加氯加药间1座、新建高位水箱7座、新建计量监测设施以及配套电气工程。</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>建设配水管网总长34.80km，新建加压泵站2座、改造已成泵站2座、新建加氯加药间1座、新建高位水箱7座、新建计量监测设施以及配套电气工程。</t>
+          <t>合同预估金额3503.77万元</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>合同预估金额3503.77万元</t>
+          <t>配水管网、加压泵站、加氯加药间、高位水箱、计量监测设施、电气工程</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>配水管网、加压泵站、加氯加药间、高位水箱、计量监测设施、电气工程</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
           <t>涪陵区江东街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区江东街道农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕470 号 及文号 主要建 建设配水管网总长 34.80km，新建加压泵站 2 座、改造已成泵站 2 座、新建加氯加药间 1 座、新建高位 设内容 水箱 7 座、新建计量监测设施以及配套电气工程商。 招 招标文件 拟交 合同预估 序 招标项 标 备 招标内容 计划发布 易场 金额(万 号 目名称 方 注 道 时间 所 元) 式 涪陵区 重庆 招标项 江东街 市涪 目 建设配水管网总长 34.80km，新建加压泵站 2 座、 公 道农村 陵区 管 改造已成泵站 2 座、新建加氯加药间 1 座、新建高 开 1 供水保 2026-09 公共 3503.77 位水箱 7 座、新建计量监测设施以及配套电气工 招 障能力 资源 程。 标 提升工程 交易 （一期） 中心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075548.html cqdingjiu 20中26.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="n">
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="n">
         <v>90</v>
       </c>
-      <c r="P43" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>重庆, 农村供水保障能力提升工程, 配水管网, 加压泵站, 加氯加药间, 高位水箱, 计量监测设施, 电气工程</t>
         </is>
@@ -3499,32 +3312,31 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>详见附件。</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>详见附件。</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>内外涂环氧消防复合钢管管件</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>内外涂环氧消防复合钢管管件</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
           <t>中国电建水电五局二公司重庆轨道交通17号线一期7标内外涂环氧消防复合钢管管件采购项目公开竞价采购(二次 挂网)变更公告(一) 详见附件。 信息来源:https://www.chinapipe.net/project/d3075376.html cqdingjiu 2026.08.21 10:06:56 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="n">
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="n">
         <v>60</v>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="O44" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -3569,34 +3381,29 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>新建、更换配水管网396.72km（dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>新建、更换配水管网396.72km（dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。</t>
+          <t>合同金额：3611.91万元</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>合同金额：3611.91万元</t>
+          <t>dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
           <t>涪陵区蔺市街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（一期） 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕474号 及文 号 主要 务 建设新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。 内容 拟 招招标文 合同预 招标 交 序 标件计划 估金 备 项目招标内容 易 号 方发布时 额(万 注 名称 场 式间 元) 所 商 重 庆 涪陵 市 区蔺 招标 市街 涪 项目 道农 陵 公 区 村供 新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收 开 公 1 水保 2026-09 3611.91 及污泥浓缩处理系统。 招 共 障能 道 标 资 力提 源 升工程 交 （一 易 期） 中 心 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075278.html 管 cqdingjiu 2026.08.21 10:06:57 国 中</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="n">
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="n">
         <v>80</v>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 商机</t>
         </is>
@@ -3641,34 +3448,29 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>改造李渡街道15个村（社区）配水主支管道，更换配水主管网193.71千米（DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治3座，新建测控井78座。</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>改造李渡街道15个村（社区）配水主支管道，更换配水主管网193.71千米（DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治3座，新建测控井78座。</t>
+          <t>项目批准文件：涪陵发改[2026]469号</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>项目批准文件：涪陵发改[2026]469号</t>
+          <t>DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
           <t>涪陵区李渡街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区李渡街道农村供水保障能力提升工程 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕469号 及文 号 商 主要 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套 建设 附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建测控井78座。 内容 招 拟 标 道 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 管 涪 陵 区 重 李 庆 渡 市 街 国 招标 涪 道 项目 陵 农 公 区 村 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂 开 公 1 供 塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建 2026-09 2372.74 招 共 水中测控井78座。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075277.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="n">
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="n">
         <v>80</v>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="O46" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 改造, 配水主支管道, 更换配水主管网, 抗菌耐磨涂塑钢管, 泵站改造, 集成泵站, 蓄水池整治, 测控井</t>
         </is>
@@ -3713,34 +3515,29 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管主要建设有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管主要建设有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。</t>
+          <t>合同预估金额为2182.77万元</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>合同预估金额为2182.77万元</t>
+          <t>PE管、衬塑钢管、水泵、不锈钢水箱、减压阀、排污阀</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>PE管、衬塑钢管、水泵、不锈钢水箱、减压阀、排污阀</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
           <t>涪陵区珍溪镇农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目名称 涪陵区珍溪镇农村供水保障能力提升工程（二期） 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕477号 务 号 (一)本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管 主要建设 有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵 内容 站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水 箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。 招标项目名 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 称 式 划发布时间 场所 (万元) 道 (一)本项目对珍溪镇23个 村(社区)安装配水管网660km 及配套附属设施，其 中：1.De160~De40的PE管 管 有232km；2.连接各村社 涪陵区珍溪 重庆市 的De32~De20的PE管有381km； 招标项目 镇农村供水 涪陵区 3.219~32的衬塑钢 公开招 1 保障能力提 2026-09 公共资 2182.77 管47km。(二)购置安装泵 标 升工国程（二 源交易 站14座(一用一备共计28台水 期） 中心 泵)，其中新建泵站10座、更 换泵站4座及配套电力设施; 新建不锈钢水箱2座等。(三) 中 购置安装(0~25kg)减压阀61 个;排污阀(25kg）3个。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075275.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="n">
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="n">
         <v>90</v>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="O47" t="inlineStr">
         <is>
           <t>涪陵区, 珍溪镇, 农村供水, 提升工程, 衬塑钢管, 水泵, 不锈钢水箱, 减压阀, 排污阀</t>
         </is>
@@ -3785,34 +3582,29 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长105.307km（dn20-dn40PE管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建1座改造3座；新建测控井52座。</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长105.307km（dn20-dn40PE管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建1座改造3座；新建测控井52座。</t>
+          <t>合同预估金额：2652.89万元</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>合同预估金额：2652.89万元</t>
+          <t>净水设备、PE管、抗菌耐磨涂塑钢管</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>净水设备、PE管、抗菌耐磨涂塑钢管</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
           <t>涪陵区蔺市街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（二期） 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕475号 及文 号 商 主要 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 105.307km（dn20-dn40PE 建设 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座；新建测控井 52座。 内容 拟 招 招标文 合同预 招标 交 序 道 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 重 庆 涪陵 管 市 区蔺 涪 招标 市街 陵 项目 道农 公 区 村供 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 开 公 1 水保 105.307km（dn20-dn40PE 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座； 2026-09 2652.89 国 招 共 障能 新建测控井 52座。 标 资 力提 源 升工程 交 （二 易 期） 中 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075274.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="n">
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="n">
         <v>80</v>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="O48" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -3851,32 +3643,31 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1，该管道为自流管道，位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水厂的正常收水及运行，需对该段管道进行改造。</t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1，该管道为自流管道，位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水厂的正常收水及运行，需对该段管道进行改造。</t>
+          <t>项目资金来自企业自筹</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>项目资金来自企业自筹</t>
+          <t>DN600混凝土管，检查井</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>DN600混凝土管，检查井</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
           <t>重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目项目公告 重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称）比选公告 1.比选条件 本比选项目重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称），比选人为重庆市排 网 水有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。中标后合同与重庆市豪洋水务 建设管理有限公司签订。现对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 2.项目概况与比选范围 务 2.1 建设地点：重庆市巴南区 2.2 项目概况：本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1,该管道为自流管道， 位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道 为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现 象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水 厂的正常收水及运行，需对该段管道进行改造。 道 2.3 比选范围：拆除现状管道为DN600混凝土管，同时需拆除并新建9座检查井。 2.4 工期要求：30日历天，以甲方通知进场时间为准。 管 2.5缺陷责任期要求：24个月 3.投标人资格要求 国 3.1 本次比选要求投标人须具备以下条件： 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质。 中 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 项内容。 3.2 本次比选接受不联合体投标。 4.比选文件的获取 4.1 投标人于2026年8月 18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子 版，以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都 视为投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的 一切后果由投标人自行负责。各投标单位应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行供应商注册，填写相关信息，审批过后成为 平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价、递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，将被否决投标。 4.4 比选文件每份售价800元，售后不退。投标单位在递交纸质投标文件时扫描支付，否则比选人拒绝接收其投标 文件。 5.投标文件的递交 5.1 电子投标文件递交时间：2026年8月24日14时30分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年8月24日14时00分至14时30分（北京时间），地点：重庆水务招标采购中心 （重庆市两江新区嘉华路36号重庆水务大厦5楼）。 5.3 投标截止时间：2026年 8月24日14时30分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆市排水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝中区长江滨江路126号 地 址：重庆市两江新区嘉华路36号重庆水务大厦 道 联 系 人： 黄老师 联 系 人： 黄晓华 电 话： 023-67767416 电 话： 18523396416 管 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3075272.html 国 cqdingjiu 2026.08.21 10:06:57 中</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="n">
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="n">
         <v>90</v>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="O49" t="inlineStr">
         <is>
           <t>重庆, 排水公司, 污水处理厂, 管网改造, DN600混凝土管, 检查井</t>
         </is>
@@ -3921,34 +3712,29 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>潼南区</t>
+          <t>改建潼南城区输水主管网约39.63km及配套相应阀门阀件等，对城区供水管网上商老旧阀门阀件、设施设备进行更换，合理增设部分计量及压力监控、水质监控等。</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>改建潼南城区输水主管网约39.63km及配套相应阀门阀件等，对城区供水管网上商老旧阀门阀件、设施设备进行更换，合理增设部分计量及压力监控、水质监控等。</t>
+          <t>合同预估金额：918.00万元</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>合同预估金额：918.00万元</t>
+          <t>城区配套阀门阀件改造工程</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>城区配套阀门阀件改造工程</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
           <t>重庆市潼南城区老旧供水管网改造工程招标计划 重庆市工程建设项目招标计划表 项目名称 重庆市潼南城区老旧供水管网改造工程 招标法人或招 标人名称（盖 重庆市潼南自来水有限公司 网 章） 项目批准文件 及文号 务 主要建设内容 改建潼南城区输水主管网约39.63km及配套相应阀门阀件等 招标方 招标文件计 拟交易场 合同预估 序号 招标项目名称 招标内容 备注 式 划发布时间 所 金额(万元) 对城区供水管网上商 重庆市潼南城 老旧阀门阀件、设 区老旧供水管 重庆市潼 招标项目 施设备进行更换， 网改造工程 公开招 南区公共 1 保障供水管网稳定 2026-09 918.00 （城区配套阀 标 资源交易 运行合道理增设部分 门阀件改造工 中心 计量及压力监控、 程） 水质监控等。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3075266.html cqdingjiu 2026.08.21 10:06:58 国 中</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="n">
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="n">
         <v>80</v>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -3993,34 +3779,29 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>开州区</t>
+          <t>该项目涉及硬化生产便道、建设防旱池和蓄水池、建造育苗大棚和小棚、安装水源处理和水肥一体化设施、新建设备管理房以及完善蔬菜基地配套设施等内容。</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>该项目涉及硬化生产便道、建设防旱池和蓄水池、建造育苗大棚和小棚、安装水源处理和水肥一体化设施、新建设备管理房以及完善蔬菜基地配套设施等内容。</t>
+          <t>工程总投资335万元。</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>工程总投资335万元。</t>
+          <t>工程设计服务</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>工程设计服务</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
           <t>关于为【重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购】公开选取【工程设计】 机构的公告 我单位在重庆市网上中介超市公开选取工程设计中介服务机构，现将相关事项公告如下： 该项目为直接选取项目，由采购人从报名的中介服务机构中直接选定一家中介服务机构进行项目服务。 项目 重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购 名称 网 采购 重庆市开州区河堰镇人民政府 人 投资 审批 否 务 项目 是否 破产 商 业务 否 服务 项目 采购 道 所需 中介 其他 服务 事项 管 所需 服务 工程设计 类型 项目实施地点为国河堰镇清泉社区，项目建设内容为：硬化2米宽生产便道5.5千米，100方防旱池1口，50方 服务 蓄水池1口，标准自动化育苗大棚1个，蔬菜小棚20个，水源处理设施1套，水肥一体化配套设施1套，新 内容 建50平方米设备管理房，完善蔬菜基地配套设施等。工程总投资335万元。选取此项目设计单位（含预算 编制服务）。 中 中介 机构 资质（资格）要求 要求 资质 （资 1、报名单位提供有效的营业执照，资质证书（资质丙级或丙级以上），具备从事项目设计服务工作； 2、 格） 具有独立承担民事责任的能力； 3、具有良好的商业信誉和健全的财务会计制度； 4、具有履行合同所必 要求 需的专业技术能力； 5、有依法缴纳税收和社会保障资金的良好记录。 说明 其他 要求 无 说明 服务 时限 无要求，按照合同双方自行约定 说明 服务 3.1%费率 金额 金额 按文件要求执行 说明 选取 直接选取 方式 需规 避机 构 规避 原因 选取 2026-08-20 16:00:00 （选取时间到达后不接受报名，建议中介机构至少在选取开始半小时前完成报名。） 时间 采购 人业 网 务咨 重庆市开州区河堰镇人民政府（18716685679） 询电 话 采购 务 需求 26清泉社区项目设计服务采购说明.pdf 书下 载 商 2026-08-18 信息来源:https://www.chinapipe.net/project/d3075198.html 道 cqdingjiu 2026.08.21 10:06:58 管 国 中</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="n">
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="n">
         <v>90</v>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="O51" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -4065,34 +3846,29 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>开州区</t>
+          <t>1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米，务周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米，务周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。</t>
+          <t>项目总投资金额：500万元，本次招标项目合同估算金额：446.278921万元</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>项目总投资金额：500万元，本次招标项目合同估算金额：446.278921万元</t>
+          <t>柑橘基地改造提升项目</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>柑橘基地改造提升项目</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
           <t>重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目招标公告 1.招标条件 本招标项目重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目已由重庆市开州区发展和改革委员会以开州 发改审〔2026〕357号批准建设，项目业主为重庆市开州区长沙镇人民政府，建设资金来自开州区2026年中央和 市级提前批财政衔接推进乡村振兴补助资金，项目出资比例为 100% ，招标人为重庆市开州区长沙镇人民 政府。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：开州区长沙镇桔香村 2.2 项目概况与建设规模：1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输 线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米， 务 周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。 2.3 本项目工程总投资金额： 500万元 本次招标项目合同估算金额： 446.278921万元 商 2.4 招标范围：招标人发布的由重庆中煜华资工程技术有限公司设计的《重庆市开州区2026年长沙镇桔香村柑橘 基地改造提升项目》施工图及图纸说明、招标文件(含补遗)及工程量清单、答疑资料、澄清资料范围内所涉及的 工作内容，具体以招标人发布的工程量清单及道施工图为准。 2.5 工期要求： 150日历天 缺陷责任期要求： 12个月 管 2.6 标段划分（如有）： / 2.7 其他： / 国 3.政府采购工程 3.1 是否属于政府采购工程：是 中 3.2 是否专门面向中小企业预留：否，按照《政府采购促进中小企业发展管理办法》第六条第(三)“按照本办法 规定预留采购份额 无法确保充分供应、充分竞争，或者存在可能影响政府采购目标实现的情形”的规定，故本 项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的建筑工程施工总承包叁级及以 上资质或市政公用工程施工总承包叁级及以上资质或水利水电工程施工总承包叁级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）下载招 标文件、工程量清单、电子图纸等资料。参与投标的投标人需在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）完成市 场主体信息登记以及CA数字证书办理，办理方式请参见 重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、 重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）导航栏“主体信息”页面中“市场主 体信息登记”、“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完 成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告 发布至2026-08-21 17:00:00前。 5.3招标人应于2026-08-25 23:59:59前在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源 交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）发布澄清。 6.投标文件递交的内容 网 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-21 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 务 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交 易监督网上发布。] 商 8.联系方式 招 标 人: 重庆市开州区长沙镇人民政府 代理机构: 重庆毅仁建设项目管理有限公司 重庆市开州区文峰街道天鹅湖社区富厚街158号附10 地 址: 重庆市开州区长沙镇山花街1号 地 址: 道号 邮 编: 邮 编: 项目负责人: 丁敬余 项目负责人: 谭毅 电 话: 15826368887 管电 话: 13452653126 传 真: 传 真: 电子邮箱: 1415705480@qq.com 电子邮箱: 开户银行: 国 开户银行: 账 号: 账 号: 监督部门:中重庆市开州区公共资源交易管理局 电 话: 023-52218977 2026年08月17日 重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目 户名 开户行 投标保证金账号 重庆市开州区公共资源交易中心 重庆农村商业银行股份有限公司开州支行 3401010120010012772000200 中国农业银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 314401010400104500000006031 业部 中国工商银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 9558853100005824176 业部 重庆市开州区公共资源交易中心 重庆银行股份有限公司开州支行 680101040007547-100984 重庆市开州区公共资源交易中心 中国银行股份有限公司重庆开州支行 108865555576VA00149 信息来源:https://www.chinapipe.net/project/d3075199.html cqdingjiu 2026.08.21 10:06:58</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="n">
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="n">
         <v>90</v>
       </c>
-      <c r="P52" t="inlineStr">
+      <c r="O52" t="inlineStr">
         <is>
           <t>重庆, 柑橘基地改造, 水肥一体化系统, 运输线, 排灌站, 生产便道, 无人机, 小型挖机, 智慧平台</t>
         </is>
@@ -4137,34 +3913,29 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>万盛区</t>
+          <t>万盛城区老旧供水管网更新改造工程答疑及补遗。</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程答疑及补遗。</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>供水管网</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>供水管网</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
           <t>万盛城区老旧供水管网更新改造工程答疑及补遗(一) 万盛城区老旧供水管网更新改造工程 答疑及补遗（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程答疑及补遗（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。? 问题2：本项目是否采用异地评标方式？ 答：是 。 商 问题3：本项目是否有业主代表，如有，请明确业主代表数量。 答：是，本项目评标委员会共7人，其中在重道庆市综合评标专家库随机抽取5人，招标人代表2人 。 问题4：投标函中的缺陷责任期可以填“达到招标文件的要求”吗？ 答：可以。 管 问题5：污水处理厂提标改造及附属管道施工业绩满足吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 国 问题6：投标文件格式中下划线上、空格处、表格中无需要填写或无法填写内容的，是填“/”或“无”还是可以 不填(空白)，对此有无要求？ 答：无要求。? 中 问题7：我公司业绩为epc业绩，我公司与设计单位组成联合体承接，竣工验收报告中施工单位盖章由我公司盖章， 请问需要提供联合体协议书吗？ 。 答： 根据招标文件第二章“投标人须知前附表”1.4.1 第3条业绩要求中：“注：（2）投标人提供的业绩为联 合体业绩的，其在该业绩中的工作分工应与本项目承担的工作一致。”要求，故需要提供联合体协议书。 问题8：投标函附录中，工期、分包和工程质量要求对应的约定内容，可以统一填写“达到招标文件要求”吗？ 答：填写“达到招标文件的要求”或按照招标文件相关条款填写具体内容均可 。 问题9：招标人提供的工程量清单单项最高限价中金额为零的，清单综合单价报价可以为0吗？ 答：投标人的工程量清单单项报价不得为零报价(招标人提供的工程量清单单项最高限价中金额为零的除外)或者 负数报价，否则由评标委员会作否决投标处理。 问题10：招标人应当在法定时间内确定中标人。招标人或者招标投标交易场所运行服务机构应当在中标通知书发 出后 5 日内，向除中标人以外的其他投标人退还纸质投标保函正本，并书面通知相关金融机构本项目准予提前注 销纸质投标保函。具体注销事宜由投标人与金融机构协商。保函原件上需要加盖正本吗？ 答：需要。但不将加盖正本作为评审因素。 问题11：我公司业绩为三个项目合并招标，三个项目合起来满足业绩要求，但分别签了三个合同和分别验收，请 问我公司业绩满足业绩要求吗？ 答：不满足。? 问题12：财务报告可以只提供审计报告、现金流量表、资产负债表、利润表吗？ 答：可以 。 问题13：业绩要求的竣工时间是指竣工验收时间吗？ 答：是的。 网 问题14：重庆市电子招投标系统投标文件-报价部分“己标价工程量清单”-“投标总价”页面招标人名称需要填 写吗？ 务 答：由投标人自行决定是否填写，是否填写不作为评审因素。 问题15：请问招标人是否委派业主专家参与评标吗？ 答：是，本项目评标委员会共7人，其中在重庆市综合评商标专家库随机抽取5人，招标人代表2人。 问题16：自来水厂或者净水厂含管道施工业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需道满足招标文件要求。? 问题17：有没有人行贿专家，有的话我们就不参加了。 答：本项目评标委员会由招标人按法律法规及相关规定依法组建。 管 问题18：招标文件第八章投标文件格式中（二）承诺部分是否包含招标文件要求的所有承诺，投标人是否还需要 提供其他格式之外的其他承诺？ 答：请各潜在投标人仔国细阅读招标文件，并按招标文件要求提供相应承诺。 问题19：财务报告可以不提供财务报表附注吗？ 答：可以。 中 问题20：乡、镇供水厂及供水管道业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题21：在职的已退休的注册人员，其社保局出具的养老证明已无法提供，该类人员是否可以用退休证、注册证 及在本单位注册的证明文件替代？ 答：退休证等材料不能替代养老保险证明，按招标文件执行。? 问题22：本项目是异地评标吗？ 答：是。 问题23：现在除了没有警戒线和技术方案的低价项目评标专家不被围猎，哪个项目不围猎评标专家，请问招标人 如何保证公平？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题24：没有低价警戒线怎么保证中高价呢？ 答：本项目未设置低价警戒线，通过综合评估法对各潜在投标人进行评审。分值由技术、商务、报价组成，综 合实力优良的投标人合理中高价可依靠综合得分优势参与竞争，同时招标文件履约追责条款约束投标人理性报 价，保障合理报价竞争环境。 问题25：现场递交纸质保函原件是否需要本项目投标人须知前附表中要求的委托代理人持授权委托书和养老保险 证明材料复印件递交吗？ 答：现场递交纸质保函原件的人员不作要求 。 问题26：请问投标文件制作系统软件导出的电子投标文件格式与加盖公章的招标文件PDF文件中的投标文件格式 不一致的以哪个为准？ 网 答：电子投标系统中锁定不可修改的格式（如封面、投标函）直接填空即可，其他投标文件格式以加盖公章的 招标文件PDF文件为准。? 问题27：专业分包业绩满足业绩要求吗？ 务 答：不满足。 问题28： 市政道路包含给水管网施工业绩满足业绩要求吗？ 商 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题29：技术负责人在资格审查部分中提供了工程类高级及以上职称证后，在商务部分中再提供工程类高级及以 上职称证可以加分吗？ 道 答：可以。 问题30：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 管 全是万盛的公司中的！业主、专家全是你们自己人吧？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 国 二、补遗 1、本次重新发布本项目的工程量清单，在《重庆市公共资源交易网》(綦江区) （https://www.cqggzy.com/qijiangweb/）网上发布，请投标人自行下载。 中 招 标 人：重庆市万盛经济技术开发区城市管理局 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 信息来源:https://www.chinapipe.net/project/d3074975.html cqdingjiu 2026.08.21 10:06:58</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="n">
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="n">
         <v>80</v>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="O53" t="inlineStr">
         <is>
           <t>重庆, 供水管网, 更新改造</t>
         </is>
@@ -4209,34 +3980,29 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>巴南区</t>
+          <t>为解决片区内涝问题，在李家沱街道、花溪街道改建d400-d800雨水管网9665m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管；改建d1000-d1400雨水管网664m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管；改建d1500-d2000雨水管网426m，管材采用III级钢筋混凝土管；改建d2100-d2600雨水管网1000m，管材采用III级钢筋混凝土管；修复雨水管网5345m，增加智能感知设备6套。</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>为解决片区内涝问题，在李家沱街道、花溪街道改建d400-d800雨水管网9665m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管；改建d1000-d1400雨水管网664m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管；改建d1500-d2000雨水管网426m，管材采用III级钢筋混凝土管；改建d2100-d2600雨水管网1000m，管材采用III级钢筋混凝土管；修复雨水管网5345m，增加智能感知设备6套。</t>
+          <t>本次招标项目工程费估算金额：11061.83万元，勘察设计合同估算金额：334.544万元。</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>本次招标项目工程费估算金额：11061.83万元，勘察设计合同估算金额：334.544万元。</t>
+          <t>雨水管网、高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管、智能感知设备</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>雨水管网、高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管、智能感知设备</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
           <t>重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 1.招标条件 本招标项目 重庆市巴南区土桥片区内涝积水整治工程已由重庆市巴南区发展和改革委员会以巴南发改审 发[2025]33号文批准建设，项目业主为重庆市巴南区住房和城乡建设委员会，代建业主为重庆市巴南公路建设有 限公司，建设资金来自区级财政资金统筹，项目出资比例为 100%，招标人为重庆市巴南公路建设有限公司。 项目已具备招标条件，现对该工程的勘察设计进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 2.1 建设地点：重庆市巴南区花溪街道、李家沱街道 务 2.2 项目概况与建设规模：为解决片区内涝问题，在李家沱街道、花溪街道改建 d400-d800 雨水管网 9665m，管材 采用高密度聚乙烯(HDPE)缠绕结构壁管 B型管；改建 d1商000-d1400雨水管网 664m，管材采用高密度聚乙 烯(HDPE)缠绕结构壁管 B 型管、III 级钢筋混凝土管；改建 d1500-d2000 雨水管网 426m，管材采用III 级钢筋混凝 土管;改建 d2100-d2600 雨水管网 1000m，管材采用 III 级钢筋混凝土管；修复雨水管网 5345m，增加智能感知设 备6 套。 道 2.3 本项目工程总投资金额：13477.10万元 管 本次招标项目工程费估算金额：11061.83万元 国 本次招标项目勘察设计合同估算金额：334.544万元 中 2.4 招标范围：主要包括勘察、施工图设计（包含高边坡、深基坑）和相应阶段的勘察工作，以及提供施工现场 全过程技术服务，并配合业主办理相关手续等，具体范围为： （1）勘察部分：完成本项目范围内的勘察工作，包括但不限于排水管网排查、1:500地形图测量、地质钻勘、管 线内窥、物探、综合管线测量，市政管网错混接点测量及调查等工作，解决区域地下空间臭气问题，勘察成果 需达到重庆市城市建成区排水管网排查技术导则的要求，并配合业主完成对应的成果审查等事宜。 （2）设计部分：包括不限于完成本项目的施工图设计、施工期间交通组织设计、桥梁（涉轨）安全论证方案及 施工期间至竣工验收阶段，质量保修阶段的设计配合服务，配合办理施工图审查相关手续及竣工验收阶段、质 量保修阶段的设计服务等工作以及协助招标人完成各项审批手续办理等工作。 2.5 勘察设计服务期限：30日历天 2.6 标段划分（如有）：/ 2.7 其他：/ 3.政府采购工程 3.投标人资格要求 3.1 本次招标要求投标人须具备以下条件： 网 3.1.1 本次招标要求投标人具备的资质条件： 务 投标人应同时具有建设行政主管部门颁发的下列勘察和设计两类资质： 商 I、投标人应具备下列勘察资质之一： 道 ①工程勘察综合甲级资质。 管 ②工程勘察专业类（岩土工程）专业甲级资质和工程勘察专业类（工程测量）甲级资质； 国 II、投标人应具备下列设计资质之一： 中 ①工程设计综合甲级资质； ②工程设计市政行业甲级资质； ③工程设计市政行业(燃气工程、轨道交通工程除外)甲级资质； ④工程设计市政行业(排水工程)甲级资质。 3.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的勘察设计能力，详见招标文件第二章投标人须知 前附表第1.4.1项内容。 3.2 本次招标接受联合体投标。联合体投标的，应满足下列要求：联合体组成单位数量不超过2家，由负责设计 任务的单位作为联合体牵头人。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件及其附件、澄 清、修改、补充通知、最高限价通知等资料。参与投标的投标人需在重庆市公共网资源交易网完成市场主体信息 登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息 登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程 电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 务 布至2026-08-23 12:00:00前。 4.3招标人应于2026-08-26 17:00:00前在重庆市公共资源交易网发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-24 09:30，投标人应当在投标截止时间前，通过互 商 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督道网、重庆市公共资源交易网、重庆市公共资源交易网（巴南区） 发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 重庆市巴南公路建设有限公司 代理机构: 重庆云远项目管理有限公司 管 地 址: 重庆市巴南区龙洲大道265号 地 址: 重庆市九龙坡区渝隆大厦28楼 邮 编: 邮 编: 项目负责人: 牟老师 项目负责人: 李强 国 电 话: 023-66238079 电 话: 023-68434996 传 真: 传 真: 电子邮箱: 电子邮箱: 中 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市巴南区发展和改革委员会 电 话: 023-66221670 2026年08月18日 重庆市巴南区土桥片区内涝积水整治工程勘察设计 户名 开户行 投标保证金账号 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000001675 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051304894 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020041267 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764210157 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000682897 支行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835000509 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146639123 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630018252 信息来源:https://www.chinapipe.net/project/d3074953.html cqdingjiu 2026.08.21 10:06:58 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="n">
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="n">
         <v>95</v>
       </c>
-      <c r="P54" t="inlineStr">
+      <c r="O54" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 雨水管网, 高密度聚乙烯, 钢筋混凝土管</t>
         </is>
@@ -4281,34 +4047,29 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>大渡口区</t>
+          <t>安装部分包括材料验收、运输及履带式挖掘机及人工布管、管道管件安装、新旧管道的碰口、安装DN400直埋球阀1座、管道和商焊口的除锈及防腐、管道下沟后15KV电火花检测、管道的清管、强度及严密性试验、警示带敷设和线路标志桩（砖）安装、监检手续等。土建部分包括清表、扫线、平整场地、沟槽、基坑、阀井砌筑、回填土方、余方弃置、人工开挖人行道（花台）、公路及路面恢复、其他线缆穿跨越工道程施工、交通组织、水工保护等。</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>安装部分包括材料验收、运输及履带式挖掘机及人工布管、管道管件安装、新旧管道的碰口、安装DN400直埋球阀1座、管道和商焊口的除锈及防腐、管道下沟后15KV电火花检测、管道的清管、强度及严密性试验、警示带敷设和线路标志桩（砖）安装、监检手续等。土建部分包括清表、扫线、平整场地、沟槽、基坑、阀井砌筑、回填土方、余方弃置、人工开挖人行道（花台）、公路及路面恢复、其他线缆穿跨越工道程施工、交通组织、水工保护等。</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>燃气管线工程</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>燃气管线工程</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
           <t>重庆燃气集团股份有限公司输配分公司大渡口调压站至二郎调压站次高压燃气管线工程(大渡口段)公告 采购 公告 公告编号： RQXYGG202608130064 一、采购项目基本情况 网 采购人：重庆燃气集团股份有限公司输配分公司 采购项目编号：RQCGXY202608130040 务 采购项目名称：大渡口调压站至二郎调压站次高压燃气管线工程（大渡口段） 采购内容或范围：安装部分： ①材料验收（甲供材料：阀门、管材、弯头、标志桩等）、运输及履带式挖掘机及人工布管； ②管道管件安装， 新旧管道的碰口；③安装DN400直埋球阀1座； ④管道和商焊口的除锈及防腐； ⑤管道下沟后15KV电火花检测； ⑥管道的清管，强度及严密性试验；⑦警示带敷设和线路标志桩（砖）安装； ⑧监检手续等。 土建部分： ①清表； ②扫线、平整场地； ③沟槽、基坑、阀井砌筑； ④回填土方； ⑤余方弃置； ⑥人工开挖人行道（花 台），公路及路面恢复； ⑦其他线缆穿跨越工道程施工，交通组织； ⑧水工保护等。 （具体内容详见施工图纸和 工程量清单） 公告发布时间 ：2026-08-18 14:39:10 管 二、采购人联系方式 联系人：王瑶 电话：023-67502265 国 邮箱：wangyao232@crcgas.com 三、采购明细 中 行号 采购内容 需求数量 单位 补充说明 拟邀请单位 大渡口调压站至二郎调压站次高压燃气管线 重庆燃气安装工程有限责任公 1 1 项目 无 工程(大渡口段) 司 四、服务费交纳 本项目不收取服务费。 五、 其他 事项 1.本公告在华润守正 采购交易 平 台（ https://www.szecp.com.cn/ ）上公开 发布。 2. 本项目采购通过守正平台线上进行，供应商需注册华润守正 采购交易 平台，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 3 .答疑澄清、通知等文件一经在华润守正 采购交易 平台发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注华润守正 采购交易 平台发布的相关信息，并及时查阅和处理。 4 .若有参与意向 ， 请于 2026-08-22 00:00:00前联系采购人 （联系方式见公示内容）反馈。 5 .若有异议 ， 请于 2026-08-22 00:00:00前提出异议 。 信息来源:https://www.chinapipe.net/project/d3074793.html cqdingjiu 2026.08.21 10:06:59 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="n">
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="n">
         <v>80</v>
       </c>
-      <c r="P55" t="inlineStr">
+      <c r="O55" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -4353,34 +4114,29 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>石柱土家族自治县</t>
+          <t>2026-2027年度用户供水管道安装及管网抢（维）修服务</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-2027年度用户供水管道安装及管网抢（维）修服务</t>
+          <t>项目资金来自企业自筹，合同估算金额约280万元</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>项目资金来自企业自筹，合同估算金额约280万元</t>
+          <t>供水管道安装及管网抢（维）修服务</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>供水管道安装及管网抢（维）修服务</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
           <t>石柱公司2026-2027年度用户供水管道安装及管网抢(维)修工程(第二次)项目公告 石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（比选公告 1.比选条件 本比选项目石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（项目名称），比选人 为重庆石柱水利水电实业开发有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。现 对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 网 2.项目概况与比选范围 2.1 建设地点：比选人指定地点 务 2.2 项目概况与建设规模：2026-2027年度用户供水管道安装及管网抢（维）修服务 2.3 本次比选项目合同估算金额：约280万元 商 2.4 比选范围：完成石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程包括公司供水范围内用户 各类管道及管件安装、水表安装及更换、阀门安装等、并完成配套土建工程、零星签证等工程量清单所列项目、 管网抢维修和公司所属生产单元零星项目，具体内容详见第五章 工程量清单。 道 2.5 工期要求：1年 缺陷责任期要求：24个月 管 3.投标人资格要求 3.1 本次比选要求投标人须具备以下条件： 国 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质； 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 中 项内容。 3.2 本次比选不接受联合体投标。 4.比选文件的获取 4.1 投标人于2026年08月18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子版， 以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都视为 投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的一切 后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价，递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，被视为无效。 4.4比选文件每份售价1000 元，售后不退。投标人在递交纸质投标文件时支付，否则比选人拒绝接收其投标文 件。 5.投标文件的递交 5.1电子投标文件递交时间：2026年08月24日10时00分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年08月24日09时30分至10时00分，地点：水务集团招标采购中心（重庆市两江新 区嘉华路36号重庆水务大厦五楼）。 5.3 投标截止时间：2026年08月24日10时00分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆石柱水利水电实业开发有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市石柱土家族自治县都督大道11号 地 址：重庆市两江新区嘉华路36号重庆水务大厦1018 联 系 人：王老师 联 系 人：颜老师 道 电 话：13658292968 电 话：023-67901915 重庆水务电子商务平台咨询电话：管023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3074720.html cqdingjiu 2026.08.21 10:06:59 国 中</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="n">
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="n">
         <v>90</v>
       </c>
-      <c r="P56" t="inlineStr">
+      <c r="O56" t="inlineStr">
         <is>
           <t>重庆, 供水管道安装, 管网抢修, 企业自筹, 280万元</t>
         </is>
@@ -4419,32 +4175,31 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>万盛城区老旧供水管网更新改造工程涉及3PE防腐钢管的采购，其管道部分壁厚需符合国标标准并达到设计要求。</t>
+        </is>
+      </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程涉及3PE防腐钢管的采购，其管道部分壁厚需符合国标标准并达到设计要求。</t>
+          <t>项目详情中未提及具体资金情况。</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>项目详情中未提及具体资金情况。</t>
+          <t>3PE防腐钢管</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>3PE防腐钢管</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
           <t>万盛城区老旧供水管网更新改造工程(甲供材料)答疑(一) 万盛城区老旧供水管网更新改造工程（甲供材料） 答疑（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程（甲供材料）答疑（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。 问题2：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 全是万盛的公司中的！业主、专家全是你们自己人吧？ 商 答：本项目招标文件严格按照《重庆市工程建设项目货物采购招标文件示范文本（2026年版）》编制，且本项目 评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题3：3PE管道部分壁厚是多少呢？ 道 答：本项目采购的3PE防腐钢管的管道部分壁厚须符合国标标准并达到设计要求。 招 标 人：重庆市万盛经济技术开发区城市管理局 管 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 国 信息来源:https://www.chinapipe.net/project/d3074712.html cqdingjiu 2026.08.21 10:06:59 中</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="n">
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="n">
         <v>80</v>
       </c>
-      <c r="P57" t="inlineStr">
+      <c r="O57" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 3PE防腐钢管, 资金情况, 产品种类</t>
         </is>
@@ -4489,34 +4244,29 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>南岸区</t>
+          <t>本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展水土保持监管测工作。</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展水土保持监管测工作。</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>供水管网</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>供水管网</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
           <t>南岸区茶园片区乡镇老旧供水管网更新改造工程更正公告 南岸区茶园片区乡镇老旧供水管网更新改造工程更正公 告 发布日期： 2026年8月18日 网 首次公示日期： 2026年8月14日 更正日期： 2026年8月18日 采购人名称： 重庆市江南城市建设发展（集团）有限公司务 采购人地址： 重庆市南岸区米兰路51号电子信息标准化厂房2号楼 联系人： 赵老师 商 电话： 023-62820331 采购代理机构名称： 重庆多杰数字科技咨询服务有限公司 采购代理机构地址： 重庆市重庆市经开区重庆市经开区长生桥镇江峡路8号13-1幢1楼 道 经办人名称： 李佩奇、戴沛轩、李倩 联系电话： 023-67648437 本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展 更正事项： 水土保持监管测工作。 https://www.gec123.com/notices/detail/1665701682723590144 信息来源:https://www.c国hinapipe.net/project/d3074669.html cqdingjiu 2026.08.21 10:07:01 中</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="n">
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="n">
         <v>80</v>
       </c>
-      <c r="P58" t="inlineStr">
+      <c r="O58" t="inlineStr">
         <is>
           <t>重庆, 管材招标, 商机</t>
         </is>
@@ -4555,32 +4305,31 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治县。合同金额28.01亿元，合同工期73个月，主要工程包括新方斗山隧道、石板坡隧道、城北隧道、刘家坪隧道、刘家店子1号大桥工程、刘家店子2号大桥、城北大桥、冉家湾大桥，采用移动模架和支商架法现浇施工，正线铺无砟道床43.808Km。</t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治县。合同金额28.01亿元，合同工期73个月，主要工程包括新方斗山隧道、石板坡隧道、城北隧道、刘家坪隧道、刘家店子1号大桥工程、刘家店子2号大桥、城北大桥、冉家湾大桥，采用移动模架和支商架法现浇施工，正线铺无砟道床43.808Km。</t>
+          <t>合同金额28.01亿元</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>合同金额28.01亿元</t>
+          <t>排水钢管Φ200*6m</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>排水钢管Φ200*6m</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
           <t>中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部排水钢管询价采购公告 中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 排水钢管询价采购公告 询价编号：ZT1105-XJ-2026-561-1 尊敬的各潜在供应商: 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与中铁十一局集团有限公司宜涪高铁重庆段站 前3标项目经理ZT1105-XJ-2026-561-1，排水钢管材料的报价。 一、项目概况 务 中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治（县）。合同金额28.01亿元，合同工期73个月， 开工日期：2024年12月，竣工日期：2030年12月。主要工程：新方斗山隧道(10660m)、石板坡隧道(4148m)、城北 隧道(3228m)、刘家坪隧道(2077m);刘家店子1号大桥工程(224.096m)、刘家店子2号大桥(232.099m)、城北大 桥(330.241m)、冉家湾大桥(355.245m),采用移动模架和支商架法现浇施工，其中24米移动模架施工6孔；32米支架法 施工5孔，移动模架施工28孔;正线铺无砟道床43.808Km。 二、询价内容 道 本次计划对排水钢管、GG-01材料进行询价，询价内容如下： 询价物资一览表 管 序号 包件号 物资名称 规格型号 计量单位 数量 备注 1 GG-01 排水钢管 Φ200*6m 米 3000 Q235B，壁厚6mm 合计 3000 国 说明：1.表中数量为计划数量，实际采购过程中可能有所调整，最终结算按照实际采购数量结算。 2.收货地点：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 中 三、技术质量及报价要求 1. 此次排水钢管、GG-01各项技术性能：Q235B 碳素结构钢无缝钢管，符合 GB/T8163 标准。质量需满足甲方项 目部正常使用的要求，保证产品的质量合格，满足试验室检测所有要求，详见技术规格书。 2.报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、结算及付款方式 自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发票认证完成之日起第6个月，支付至本次结算 金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内，累计支付总额不超结算总金额的75%，剩 余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理末次结算后第二年，支付金额应大于等于 尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总额的15%；办理末次结算后第四年，全部 付清）。 五、报价人资格要求 1.营业范围要求：在中华人民共和国境内依法注册、符合项目经营范围，具有询价物资生产或供应经验 的生产商或代理商，并且具有合法有效的营业执照。 2.生产能力要求：生产商须具备询价物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定。代 理商需出具制造厂出具签字盖章的授权函。 3.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8 月至今）国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；需满足排水钢管的相关所 有要求。 4.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年12月至今）企业或企业法定代表人有人民法院生效判决、裁 定认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接 受通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合 作方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 5.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★6.下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、报价人需要提供的资料 1.营业执照复印件、法人身份证复印件、开户许可证、授商权委托书、报价表和报价人资格要求中所需的证明资料， 所有资料需加盖公司鲜章。 2.生产厂家资质，产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、询价报名截止时间 管 有意参加本次询价采购的报价人须在铁建云链平台（https://www.crccep.cn）完成供应商注册，并于2026年8月18 日9时00分至2026年8月21日9时00分在网上完成报名工作。 八、询价截止时间 国 凡有意参加本次询价采购的报价人，请于 2026年8月21日14时00分 前提交报价。截止时间前未完成报价文件传 输的，视为放弃报价。 供应商报价必须严格按照《报价表》格式进行报价。 中 九、联系方式 采购组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村71号 采购人名称：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 地址：重庆市石柱土家族自治县金彰工业园区C区中铁十一局项目部 联系人：罗先生 联系电话：18580400001（提供采购服务支持） 中铁十一局集团有限公司 物资设备集中采购管理中心第五分中心 2026年8月18日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3074654.html cqdingjiu 2026.08.21 10:07:01 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="n">
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="n">
         <v>90</v>
       </c>
-      <c r="P59" t="inlineStr">
+      <c r="O59" t="inlineStr">
         <is>
           <t>重庆, 排水钢管, 询价采购</t>
         </is>
@@ -4619,32 +4368,31 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热交换机组采购。</t>
+        </is>
+      </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热交换机组采购。</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>冷却塔、分集水器、水板式热交换机组</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>冷却塔、分集水器、水板式热交换机组</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
           <t>中铁建设集团(重庆)建设有限公司重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热 交换机组采购竞价补遗公告二 各 投标单位 ： 根据参加报名的潜在投标单位数量不满足招标方充分竞价要求的情况，此次重庆协同创新区供冷供热能源站及 配套系统工程冷却塔、分集水器、水板式热交换机组采购竞价资格预审报名截止日期将延期至 8月19日（周三） 上午9:00。 特此说明。 网 中铁建设集团（重庆）建设有限公司 2026年8月17日 务 信息来源:https://www.chinapipe.net/project/d3074650.html cqdingjiu 2026.08.21 10:07:01 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="n">
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="n">
         <v>80</v>
       </c>
-      <c r="P60" t="inlineStr">
+      <c r="O60" t="inlineStr">
         <is>
           <t>重庆协同创新区, 供冷供热能源站, 冷却塔, 分集水器, 水板式热交换机组, 采购竞价</t>
         </is>
@@ -4689,34 +4437,29 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>城口县</t>
+          <t>在城口县东安镇新建一座污水处理站，铺设不同直径的污水管道共计29.3公里，包括dn110、dn160、dn200、DN300、DN400等规格的污水管道，以及DN200压力管道7.4公里，建设配套泵站2座和化粪池56座、隔油池32座。</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>在城口县东安镇新建一座污水处理站，铺设不同直径的污水管道共计29.3公里，包括dn110、dn160、dn200、DN300、DN400等规格的污水管道，以及DN200压力管道7.4公里，建设配套泵站2座和化粪池56座、隔油池32座。</t>
+          <t>合同预估金额为3400万元人民币。</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>合同预估金额为3400万元人民币。</t>
+          <t>污水管网、泵站、化粪池、隔油池</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>污水管网、泵站、化粪池、隔油池</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
           <t>城口县东安及河鱼片区污水管网建设项目(一期)招标计划表 重庆市工程建设项目招标计划表 项 名 目 称城口县东安及河鱼片区污水管网建设项目（一期） 招标 法人 或招 标人城口县生态环境局 名称 （盖 网 章） 项目 批准 文件 及文 号 主 建 内 要 设 容 在 污 城 水 口 处 县 理 东 站 安 1座 镇 ， 等 改 片 建 区 后 新 设 建 计 污 规 水 模 管 20 网 0m 29 3 . / 0 d 0 。 km，其中新建dn110污水管5.80km，dn160污水管2.75km，dn200污水管0.57km，DN300污水干管4.36km，D 务 N400污水干管8.12km，DN200压力管7.4km,以及建设配套泵站2座,化粪池56座，隔油池32座。改扩建 序号 招标项目名称 招标内容 招标方式 招标文件计划发布时间 拟交易场所 合同预估金额(万元) 备注 招 项 标 目1 城 建 口 设 县 项 东 目 安 （ 及 一 河 期 鱼 ） 片区污水管网 工程施工 公开招标 2026-09 城 易 口 中 县 心 公共资源交 3400.00 本 暂 为 计 定 准 划 ， 。 表 最 所 终 列 以 招 实 标 际 项 招 目 标 信 时 息 的 均 信 为 息 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3074602.html 商 cqdingjiu 2026.08.21 10:07:01 道 管 国 中</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="n">
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="n">
         <v>90</v>
       </c>
-      <c r="P61" t="inlineStr">
+      <c r="O61" t="inlineStr">
         <is>
           <t>重庆, 管材, 招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
@@ -4755,32 +4498,31 @@
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路长4000米，包括道路、综合管网等基础配套设施等。</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路长4000米，包括道路、综合管网等基础配套设施等。</t>
+          <t>本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元</t>
+          <t>土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
           <t>阀门产业园(管网改造)项目招标公告 阀门产业园（管网改造）项目招标公告 1.招标条件 本招标项目 阀门产业园（管网改造）项目已由垫江县发展和改革委员会以垫江发改委发【2022】459 号（批文 名称及编号）批准建设，项目业主为 垫江县丹香建设有限公司，建设资金来自 自筹资金 （资金来源）， 项目出资比例为 100% ，招标人为 垫江县丹香建设有限公司。项目已具备招标条件，现对该项目的施工进 行公开招标，评标办法采用经评审的最低投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 重庆市垫江县高新区县城组团 2.2 项目概况与建设规模： 场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路 务 长4000米，包括道路、综合管网等基础配套设施等。 2.3 本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元 商 2.4 招标范围： 包括土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等。具体详见施工图和 工程量清单。 道 2.5 工期要求：建设工期180日历天 缺陷责任期要求：24个月 管 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 国 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 中 4.1.1 本次招标要求投标人具备的资质条件： 具备建设行政主管部门颁发的有效的市政公用工程施工总承包叁 级及以上资质 ； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标 不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易监督网、重庆市公共资源交易网 （垫江县）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易监督网、 重庆市公共资源交易网（垫江县）完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资 源交易监督网、重庆市公共资源交易网（垫江县）导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 4.2投标人可在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）本项目招标公告网页下方“我要 提问”栏提出疑问，提问时间从本公告发布至2026-08-24 09:00:00前。 4.3招标人应于2026-08-24 23:59:59前在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-18 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 垫江县丹香建设有限公司 代理机构: 重庆博钰大数据科技有限公司 地 址: 地 址: 重庆市垫江县桂溪街道南内街88号 网 邮 编: 邮 编: 项目负责人: 熊老师 项目负责人: 郭威 电 话: 023-74630098 电 话: 023-74692498 务 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 商 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 道 2026年08月18日 信息来源:https://www.chinapipe.net/project/d3074578.html cqdingjiu 2026.08.21 10:07:02 管 国 中</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="n">
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="n">
         <v>90</v>
       </c>
-      <c r="P62" t="inlineStr">
+      <c r="O62" t="inlineStr">
         <is>
           <t>重庆, 管网改造, 投资金额, 产品种类</t>
         </is>

</xml_diff>

<commit_message>
Populate product usage in workbook exports
</commit_message>
<xml_diff>
--- a/site/matches-positive.xlsx
+++ b/site/matches-positive.xlsx
@@ -550,7 +550,11 @@
           <t>璧山项目钢筋混凝土管询价公告 本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用 地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行 建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉 泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含 市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范 围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期 实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。 网 登录地 mhem&amp;cNh6e0&amp;ce2C2m3s1e71=a64so0d9FAe=0903%e08005206E%6772dm6=%82he29&amp;=cI8p9eeyAs%7t?E%5lB%1iB%a1DetE%c9eweNAi%1iotvB%n/9cE%7.cBe9%ccAiE%p.E%s9%/29址/A%2:：psE%7tAhtD%B8%E%6B%7B%7E%5%78D9%E%5C9%F%9E%7AE%A%1E%9%78%78E%8B%4AD%N&amp;8E%6m657optUa3%6=6290%e3ni51B%5917E%443d6=E%862B%I8eAc%A1iD&amp;88no%tE%4BA%A%4E%7AC%AC%E%4BA%C8%E%8%88AA%E%5A8%A%1E%5B%7A%5E%7A%8B8%E%5B%1%08E%6C9%%98E%9%99%09E%5%58AC%E%5F%8B%8E%8A%5BF%E%9%38A%8EF%BC%%88E%5B9%BD%E%9%99%58EF%BC%%98E%6%59B%0E%5AD%%79E%7BB%F%8E%6B%5E8%E%4BA%A%7E%4B%8A9%E%5B9%AD%E%5C8%BA%E%9%58D8%E%5A%5%79E%9A%1B%9E%7B9%AE%EF%BC%%88E%8A%5BF%E%7%98%78E%5C8%BA%EF%BC%%98E%9A%1B%9E%7B9%AE%E%7=BgB&amp;upC%a=sod&amp;euF%pN=8Flk&amp;cmsusheaE%c7=te%0a9m%6he=8tT&amp;cpS7eeyeE%s9sha%&amp;3c2845d5=pur5A6I&amp;8optUni 信息来源:https://www.chinapipe.net/project/d3077008.html 务 cqdingjiu 2026.08.21 10:06:40 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N2" t="n">
         <v>70</v>
       </c>
@@ -617,7 +621,11 @@
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 务 2.1 建设地点： 忠县花桥镇、新立镇、石宝镇、兴峰乡。 商 2.2 项目概况与建设规模①忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）：田块整治 工程：旱地区域撂荒地整治278.95亩；灌溉与排水工程：新建200m蓄水池6座、PE75管道967m、新建1.2*1.2m箱 涵16m、新建2*2m箱涵8m；田间道路工程：新建2.5m混凝土生产路15114m、改建2.5m混凝土生产路1078m、新 建2.5m泥结碎石生产路910m、改建2.5m泥结碎道石生产路279m、新建3.0m混凝土生产路601m、改建3.5m混凝土机 耕路4587m；地力提升工程：施有机肥278.95亩；其他工程：工号牌124块。 管 ②忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）：田块整治工程：旱地区域撂荒地 整治195.54亩；灌溉与排水工程：新建100m蓄水池4座、新建200m蓄水池6座、PE75管道5258m、PE90管 道1375m、PE110管道2156m、改建0.5*0.6m混凝土排水沟740m、改建0.6*0.8m混凝土排水沟109m、改建0.8*1.0m混 凝土排水沟296m、改建1*1.5m混凝土排水沟262m、新建3*2m盖板涵1座；田间道路工程：新建2.5m混凝土生产 路11359m、改建2.5m混国凝土生产路3430m、新建2.5m泥结碎石生产路1834m、新建3.0m混凝土生产路350m；农田 防护工程：新建1.0m高挡土墙39m；地力提升工程：施有机肥195.54亩；其他工程：工号牌142块。 中 2.3 本项目工程总投资金额：约3140万元； 本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： 标段划分情况、建设规模及标段合同估算金额等内容如下： 合同估算金额 序号 项目名称 建设地点 （万元） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二 1 花桥镇、新立镇 1022 标段） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三 2 石宝镇、兴峰乡 735 标段） 网 本项目共分为2个标段，每家投标单位仅对2个标段中的任意1个标段进行投标，若同时参与2个及以上标段投标的， 其投标文件无效。 务 2.7 其他： / 商 3.政府采购工程 道 3.1 是否属于政府采购工程：是 □否 管 3.2 是否专门面向中小企业预留：是 国 专门面向中小企业预留的实施方式： 中 方式一：本项目整体面向中小企业。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字 证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责 任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要网提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-10-12 09:30，投标人应当在投标截止时间前，通过互 务 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 商 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 道 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 管 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 国 开户银行: 开户银行: 账 号: 账 号: 中 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段） 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005499 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421353 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891814619 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082001038 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00385 信息来源:https://www.chinapipe.net/project/d3076880.html cqdingjiu 2026.08.21 10:06:45</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>管道：967m；管道：5258m；管道：2156m</t>
+        </is>
+      </c>
       <c r="N3" t="n">
         <v>90</v>
       </c>
@@ -684,7 +692,11 @@
           <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(一标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）已由 忠县发展和改革委 员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来 自 业主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具 备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 务 2.项目概况与招标范围 商 2.1 建设地点： 忠县马灌镇、三汇镇、永丰镇。 道 2.2 项目概况与建设规模：忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）：田块整治 工程：水田整治50.67亩、水田区域撂荒地整治79亩、旱地区域撂荒地整治62.83亩；灌溉与排水工程：新 建200m蓄水池5座、新建500m蓄水池1座、泵站1座；田间道路工程：新建2.5m混凝土生产路12325m、改 建2.5m混凝土生产路8549m、新建2.5m泥结碎石生产路1223m、新建3.0m混凝土生产路576m、改建3.0m混凝土生 管 产路648m、改建3.0m混凝土生产路（拆除原1.5m宽路）266m、改建3.5m混凝土机耕路1662m；地力提升工程：施 有机肥136.48亩；其他工程：公示牌1座、工号牌213块。 国 2.3 本项目工程总投资金额：约3140万元； 中 本次招标项目合同估算金额：一标段1167万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 网 方式一：本项目整体面向中小企业。 务 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 商 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 道 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 管 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 国 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 中 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及CA数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-10 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 网 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 务 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段） 商 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082000104 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005469 道 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421379 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00387 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891884496 管 信息来源:https://www.chinapipe.net/project/d3076876.html cqdingjiu 2026.08.21 10:06:46 国 中</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>泵站：1座</t>
+        </is>
+      </c>
       <c r="N4" t="n">
         <v>95</v>
       </c>
@@ -751,7 +763,11 @@
           <t>永川区农村供水管网巩固提升改造工程(东部片区)答疑补遗文件 永川区农村供水管网巩固提升改造工程（东部片区） 补遗文件（01） 各潜在投标人： 现将“永川区农村供水管网巩固提升改造工程（东部片区）”招标文件补遗通知如下，本次发布的补遗文件中 的所有内容与招标文件具有同等法律效力，如与招标文件、答疑补遗文件（01）网不一致时，以本补遗文件为准。 请各潜在投标人自行下载本补遗文件，不管下载与否，都视为全部知晓其全部内容。 一、本招标项目招标文件第二章投标人须知前附表第1.4.1项第1条第（3）款中“具备建设行政主管部门颁发的有 效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由建设行政主管部门颁发的有效的安全生产 务 考核合格证书。”修改为： “（3）具备建设行政主管部门颁发的有效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由水 行政主管部门颁发的有效的安全生产考核合格证书”。 商 二、本招标项目招标文件第二章投标人须知前附表第1.4.1项中第3条“业绩要求”修改为： “投标人自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成过1个单项合同 输配水管网长度不少于100km的水利工程施工道业绩。 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 管 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 三、本招标项目招标文国件第二章投标人须知前附表第1.4.1项中第5条中的“5.3项目经理业绩要求”修改为： “投标人拟派的项目经理自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成 过1个单项合同输配水管网长度不少于100km的水利工程施工业绩，并在该业绩中担任项目经理。 中 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 四、本招标项目的投标文件递交的截止时间（投标截止时间）调整为2026年9月4日9时30分（北京时间），开标 时间及投标保证金递交截止时间相应顺延。 招标人：重庆市永川区惠永水务有限公司 招标代理机构：重庆永川政鑫综合能源有限公司 2026年8月20日 信息来源:https://www.chinapipe.net/project/d3076870.html cqdingjiu 2026.08.21 10:06:46</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>输配水管网：100km</t>
+        </is>
+      </c>
       <c r="N5" t="n">
         <v>80</v>
       </c>
@@ -818,7 +834,11 @@
           <t>中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部刺丝滚笼、塑钢模板、泄水管询价采购公告 中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 刺丝滚笼、塑钢模板、泄水管询价采购公告 询价编号： ZT1105-XJ-2026-590 尊敬的 各潜 在供应商 : 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与 中铁十一局集团有限公司重庆至万州高铁站 前 1标项目经理部 ZT1105-XJ-2026-590， 刺丝滚笼、塑钢模板、泄水管 的报价。 一、 项目概况 务 渝万高铁站前 1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~ D1K47+550.4，正线长度 33.01km，中标造 价 31.73 亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁 301 孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负 责DK0+000~DK57+136段小型构件预制。合同工期54.7月商，开工日期为2022年11月01日，竣工日期为2027 年04 月30日。 二、 询价内容 道 本次 计划对刺丝滚笼、塑钢模板、泄水管 进行询价，询价内容如下： 询价物资一览表 管 计 序 物资 量 包件号 规格型号 数量 备注 号 名称 单 位 国 刺丝 1 GL-01 2.5mm 6m0.5m 米 6500 半径 ≥225mm，包括刀片刺绳、挂丝、连接卡、支架 滚笼 防护 中 栅栏 2 GL-01 用立 50X30X765X2.5mm 套 500 含抱箍、螺栓等配件 柱支 架 平 塑钢 3 MB-01 350X300mm 方 19.2 400*400,1个挡水沿，配固定手柄 模板 米 平 塑钢 4 MB-01 350X300mm 方 19.2 400*400,2个挡水沿，配固定手柄 模板 米 平 塑钢 5 MB-01 300X300mm 方 75.6 2个挡水沿，配固定手柄 模板 米 平 塑钢 6 MB-01 300X300mm 方 75.6 1个挡水沿，配固定手柄 模板 米 7 SSG-01 管篦 PVC250X200x10mm 个 220 材质硬聚氯乙烯 PVC，详见附图 PVC 8 SSG-01 泄水 135X38mm 块 220 材质硬聚氯乙烯 PVC，详见附图 管盖 U型 9 SSG-01 125mm 个 900 详见附图 管卡 UPV 材质硬聚氯乙烯 PVC，两端接头采用阴阳螺纹连接详见 10 SSG-01 C排 125X8mm螺纹 米 2870 附图 水管 UPV 11 SSG-01 C弯 DN125X8mm90° 个 240 材质硬聚氯乙烯 PVC，详见附图 管 UPV 网 125X125X110mm弹性密 12 SSG-01 C三 个 120 材质硬聚氯乙烯 PVC，详见附图 封圈异径斜三通 通 无压 埋地 务 排污 排水 用硬 13 SSG-01 DN125 个 150 材质硬聚氯乙烯 PVC，详见附图 聚氯 商 乙烯 管 T 型接 头 道 合 计 管 说明： 1. 表中数量为计划数量，实际 采购 过程中可能有所调整，最终结算按照实际 采购 数量结算。 2.收货地点：中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部 三、 技术质量 及报价国 要求 1. 此次 询价物资 各项技术性能要 符合 甲方 的要求，质量满足甲方项目部正常使用的要求，保证 产品 的质量合 格。 具体要求或图纸见询价文件技术规格书。 。 中 2 .报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、 结算及付款方式 每个月 15 日为双方价款结算日期（即上月 16 日至当月 15 日内），结算前双方要在对帐确认单上签字认可，乙 方按双方确认的金额开具增值税专用发票，并自发票开具之日起 7日内传递给甲方。甲乙双方在增值税专用发票 传递过程中必须留取相应的交接签证手续。自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发 票认证完成之日起第6个月，支付至本次结算金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内， 累计支付总额不超结算总金额的75%，剩余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理 末次结算后第二年，支付金额应大于等于尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总 额的15%；办理末次结算后第四年，全部付清）。 五、 报价 人资格要求 1.营业范围要求：在中华人民共和国境内依法注册，具有询价物资生产或供应经验的生产商或代理商，并且具有 合法有效的营业执照。 2.生产能力要求： 生产商须具备 询价 物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定 。 代理商需出具制造厂出具签字盖章的授权函。 3.财务能力要求：报价人为增值税一般纳税人或小规模纳税人，有依法纳税的良好记录。 4.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8月至今） 国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；每种物资全指标技术参数性能满足 国家和行业最新标准的各项规定。 5.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年8月至今）企业或企业法定代表人有人民法院生效判决、裁定 认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接受 通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合作 方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 6.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★7 .下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、 报价人需要提供的资料 1. 营业执照复印件、 法人身份证复印件、 开户许可证、商授权委托书 、 报价表 和报价人资格要求中所需的证明资 料， 所有资料需加盖公司鲜章。 2. 产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、 询价 报名截止 时间 管 有意参加本次询价采购的报价人 须在铁建云链平台 （ https:// www.crccep. cn） 完成供应商注册，并 于 202 6 年 8 月 20 日 9时 00 分 至 202 6 年 8 月 24 日 9时 00 分在网上 完成报名工作。 八、 询价 截止 时间 国 凡有意参加本次询价采购的报价人，请于 202 6 年 8 月 24 日 14 时 00分 前 提交报价。截止时间前未完成 报价 文 件传输的，视为放弃 报价 。 供应商报价必须严格按照《 报价表 》格式进行报价。 中 九、 联系方式 采购 组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村 71号 联系人：胡先生 联系电话： 13983336494 （提供平台服务支持） 采购人名称：中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 地址： 重庆市万州区双河口街道檬兴路万州现代综合物流中心信息交易大厅（中铁十一局） 联系人： 唐大伟 联系电话： 18323391938（提供采购服务支持、保证金退还） 中铁十一局集团有限公司物资设备集中采购管理中心 第五分中心 2026 年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076805.html cqdingjiu 2026.08.21 10:06:47 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N6" t="n">
         <v>85</v>
       </c>
@@ -885,7 +905,11 @@
           <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 1.招标条件 本招标项目 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 已由 垫江县发展和 改革委员会 以 垫江发改委发〔2026〕20号 文批准建设，项目业主为 垫江县太平镇人民政府，建设资金来 自 大中型后扶资金及自筹资金 ，项目出资比例为 100% ，招标人为垫江县太平镇人民政府。项目已具备招 标条件，现对本项目施工进行公开招标，评标办法采用经评审的最低投标价法。网 务 2.项目概况与招标范围 商 2.1 建设地点：垫江县太平镇桂花村 道 2.2 项目概况与建设规模：主要为河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m， 化粪池2座；产业基地水肥一体化改造45亩等。 管 2.3 本项目工程总投资金额：642.89万元 国 本次招标项目合同估算金额：约5014864.52元 中 2.4 招标范围：本工程施工图纸所含全部的施工内容，具体以招标人发布的工程量清单为准。 2.5 工期要求：工期为360日历天 ，缺陷责任期为24个月。 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：□是 否，因专门面向中小企业预留无法确保充分供应、充分竞争，根据 《政府采购促进中小企业发展管理办法》第六条第(三)“按本办法规定预留采购份额无法确保充分供应、充分竞 争，或者存在可能影响政府采购目标实现的情形”的规定，本项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 网 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的水利水电工程施工总承包三级 务 及以上资质。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相商应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 道 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 管 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com国/dianjiangweb/)、重庆市公共资源交易监督网下载招标文件、工程量清单、电子图纸等资 料。参与投标的投标人需在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共 资源交易监督网完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督网导航栏“主体信息”页面中“市场主体信息 登记”、“中CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流 程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督 网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-24 17:00:00前。 5.3招标人应于2026-08-28 17:00:00前在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重 庆市公共资源交易监督网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交 易监督网发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 垫江县太平镇人民政府 代理机构: 重庆皓辰建设工程咨询有限公司 重庆市渝北区金开大道1228号大雅金开国际1 地 址: 重庆市垫江县太平镇牡丹路191号 地 址: 栋9-2 邮 编: 邮 编: 项目负责人: 余老师 项目负责人: 雷雨得 电 话: 13996889839 电 话: 023-86018770 18580880860 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 网 2026年08月19日 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 务 户名 开户行 投标保证金账号 垫江县公共资源交易中心 中国农业银行重庆垫江支行 316301010400077950000005966 垫江县公共资源交易中心 中国银行重庆垫江支行 111616885778VA00139 商 垫江县公共资源交易中心 重庆农村商业银行垫江支行 2501010120010009065000128 垫江县公共资源交易中心 工商银行重庆垫江支行营业部 9558853100016843371 垫江县公共资源交易中心 重庆银行垫江支行 820101040000584-101195 道 附件：垫江县2026年度大中型水库移民后期扶持项目-.zip https://www.cqggzy.com/trade/014001/dac54522-3264-4eac-ae47-f434567ce374?categoryNum=014001001007 信息来源:https://www.chinapipe.net管/project/d3076788.html cqdingjiu 2026.08.21 10:06:47 国 中</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>污水管网：450m</t>
+        </is>
+      </c>
       <c r="N7" t="n">
         <v>85</v>
       </c>
@@ -952,7 +976,11 @@
           <t>万州区新田等6个镇乡农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区新田等6个镇乡农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建水厂1座（新建2000m3茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管 主要建设内容 径DN20~DN250，管材为涂塑钢管。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 备注 称 式 发布时间 所 额(万元) 商 万州区新田 万州区新田 重庆市万 招标项目 等6个镇乡农 等6个镇乡农 公开招 州区公共 1 村饮水质量提 2026-08 5000.00 村饮水质量 标 资源交易 升项目道施工总 提升项目 中心 承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076721.html 管 cqdingjiu 2026.08.21 10:06:48 国 中</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>管道：226.127km</t>
+        </is>
+      </c>
       <c r="N8" t="n">
         <v>80</v>
       </c>
@@ -1019,7 +1047,11 @@
           <t>万州区大周等4个镇乡街道农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区大周等4个镇乡街道农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建50m3蓄水池4口、取水池2座；新建50m3/d-100m3/d水厂2座；改造100m3/d-300m3/d水厂5 主要建设内容 座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设 施。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 商 备注 称 式 发布时间 所 额(万元) 万州区大周 万州区大周 重庆市万 招标项目 等4个镇乡街 等4个镇乡街 公开招 州区公共 1 道农村饮水 道农村饮道水质 2026-08 3000.00 标 资源交易 质量提升项 量提升项目施 中心 目 工总承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3076720.html cqdingjiu 2026.08.21 10:06:49 国 中</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>涂塑钢管：86km；提水泵站：8座</t>
+        </is>
+      </c>
       <c r="N9" t="n">
         <v>80</v>
       </c>
@@ -1082,7 +1114,11 @@
           <t>二航科工新燕尾山项目纤维编绕拉挤电缆保护套管采购询价通知公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目询比采购 公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目已具备采 购条件，现公开邀请供应商参加询比采购活动。 网 1. 采购项目简介 1.1 采购项目名称：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机 电工程项目。 务 1.2采购方案编号：FA00000674478。 1.3 采购人：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程 项目经理部。 商 1.4 采购代理机构：中交二航局科工（武汉）有限公司。 1.5 采购项目资金：企业自筹。 道 1.6 采购项目概况：新燕尾山隧道工程位于重庆市内环吉庆隧道北侧，四横线分流道鹿角隧道南侧，西接白居 寺大桥，东接内环快速路，并向东延伸接渝黔复线高速，其所在的道路系统呈东西布置，为主城区南部片区重 要干道。本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目 管 全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程 包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。 2.采购范围及相关要求 国 2.1 采购范围：纤维编绕拉挤电缆保护套管（BWFRP100/2.0，79158米）。 2.2 交货期：以甲方实际订单要求为准。 中 2.3 交货地点：重庆市巴南区新燕尾山项目甲方指定位置。 2.4 物资质量标准：满足国家法律法规、标准、规范、设计参数及技术规格书要求。 3.供应商资格要求 3.1 供应商应依法设立且满足如下要求： （1）资质要求：在中华人民共和国境内依法注册，具有独立法人资格、具有采购物资生产或供应经验的企业， 并且具有合法、有效的“三证合一”的营业执照,代理商需提供制造商授权委托书。 （2）财务要求：必须是经税务部门注册登记核准的一般纳税人，有依法纳税的良好记录，提供近三年的财务报 告。 （3）业绩要求：同类产品销售业绩不少于2个，并具备与本招标项目需求相适应的供货能力。 （4）信誉要求：本项目投标截止期前未被“信用中国”、“中国政府采购网”、中国交建物资采购管理信息系 统网站列入失信被执行人、违法案件当事人、违法失信行为记录名单。 （5）其他要求：提供运输方案及生产周期。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他： / 。 4.供应商报名 4.1有意参加询比采购活动的单位，请于2026年 8 月 20 日 11 时 00 分至2026 网 年 8 月 25 日 11 时 00 分（北京时间、下同），登录“中交招采网”（网 址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 务 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 商 5. 供应商报价 5.1 报价结束（递交响应文件截止）时间：2026年 8 月 25 日 11 时 00 分。 道 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的 电子响应文件，采购人将拒收。 5.3电子采购的供应商报价文件由线上电子报价表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 管 子报价表的数据为准。 6. 开标 6.1开标时间：与报价结国束时间相同。 6.2开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标，现场开标地点/。 7. 发布公告的媒介 中 本询比采购公告在中交招采网上发布。 8. 评审办法 本项目评审办法采用 经评审的最低价法 。 9. 合同主要条款 9.1 付款条件：无预付款，到货后办理结算，双方办理完结算手续、卖方提供符合合同要求的正式发票给买方 后60天，买方支付该批材料价值80%的货款，完工结算后支付至97%，剩余3%为质保金，质保期2年，两年后供 应方申请返还3%（无息）；银行转账、承兑、18个月供应链金融混合支付方式。 9.2履约保证金的递交： （1）□不要求递交 （2）要求递交 保证金金额：2万元 ； 保证金形式：银行转账、银行保函等电子保函；其他形式：无 。 10. 成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”（网址：https://zjzcw.iccec.cn）发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联 系4006765885中标服务费请按7咨询。 10.1收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； 务 （3）在1000万元（含）至3000万元之间的，每次收取1000元； （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 10.2支付流程 （1）通知推送：中标结果发布后，系统自动道推送缴费通知（含应缴金额及支付链接）； （2）费用查询：供应商登录“中交招采网-服务管理”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网- 服务管理－发票下载”模块获取。 11.监督机构 国 监督机构名称：中交二航局科工（武汉）有限公司纪委监察部 举报电话：中027-82796466 举报邮箱：sneb_kggs@ccccltd.cn 12.其他 投标保证金采用银行转账形式的需转至中交二航局科工（武汉）有限公司账户（账 号：42001186108053006379-0006开户行：建行武汉长江支行，行号：105521000053），并备注二航科工燕尾山机 电照明项目纤维编绕管投标保证金。 13.联系方式 采购 人：中交二航局科工（武汉）有限公司 采购代理机构：中交二航局科工（武汉）有限公司 地 址：武汉市新洲区双柳街星谷大道158号地 址：武汉市新洲区双柳街星谷大道158号 邮政编码：430400 邮政编 码：430400 联系人：李鑫 联系人：毕明 月 电 话：18186145302 电 话：17853118573 电子邮件：18186145302@ccccltd.cn 电子邮件：bimingyue@ccccltd.cn 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076715.html cqdingjiu 2026.08.21 10:06:50 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N10" t="n">
         <v>90</v>
       </c>
@@ -1149,7 +1185,11 @@
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告 重庆巴南天然气有限责任公司 重庆国际生物城配套公寓项目天然气表后管道安装工程 变更公 告 公告编号： RQBGGG202608200006 本公司于2026年08月19日发布的重庆国际生物城配套公寓项目天然气表后管道安装工程公告（编 号：RQCGXY202608170010），现做出如下变更： 网 1、对采购文件第一卷“采购需求“中墙体管道暗埋的具体内容进行明确。墙体管道暗埋应包含墙体开槽，输送 用不锈钢波纹管及钢制槽板的安装，墙体恢复，暗埋管道视频记录。 2、对由响应供应商提供的钢制槽板的规格进行明确。钢制槽板为U型开口槽，采用热镀锌Q235B钢板，钢板厚度 务 不得小于1.2mm，尺寸不得小于U40*30*1.2（宽40mm,高30mm,壁厚1.2mm热镀锌） 3、对由响应供应商提供的F型不锈钢三通，材质可以选用黄铜进行替代。 4、采购文件第二卷“技术规范及要求“中增加T/CECS633-2019 《燃气用户工程不锈钢波纹软管技术规程》。 以上内容在合同中也同步进行调整。 商 除上述变更外，原公告其余内容仍有效。 道 重庆巴南天然气有限责任公司 管 2026-08-20 信息来源:https://www.chinapipe.net/project/d3076704.html cqdingjiu 2026.08.21 10:国06:50 中</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N11" t="n">
         <v>80</v>
       </c>
@@ -1216,7 +1256,11 @@
           <t>合川区中南片区污水管网工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 合川区中南片区污水管网工程（一期） 名称 招标 网 法人 或招 标人 重庆市合川区住房和城乡建设委员会 名称 （盖 务 章） 项目 批准 文件 合川发改投〔2025〕19 号 商 及文 号 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新 主要 建D300排水管道38米；紫外光修复 D300-D道800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 建设 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42 内容 米；完成 D300-D1000管道清障189米、清淤2627米。 拟 招 招标文 合同预 招标 管 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 国 重 庆 市 合川 合 招标 区中 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300- 川 项目 中 南片 D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 公 区 区污 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 开 公 1 2026-09 1708.44 水管 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米， 招 共 网工程 不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清 标 资 （一 淤2627米。 源 期） 交 易 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076543.html cqdingjiu 2026.08.21 10:06:50</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>D800管道：130米；D300排水管道：38米；D800排水管道：755米；D1600管道：73米；D800排水管道：125米；D800排水管道：712米；D1000管道：42米；检查井：11座；管道：189米</t>
+        </is>
+      </c>
       <c r="N12" t="n">
         <v>90</v>
       </c>
@@ -1279,7 +1323,11 @@
           <t>重庆市自来水有限公司球墨铸铁管及管件2026-2027(2年)采购项目(第二次)答疑补遗文件 重庆市自来水有限公司球墨铸铁管及管件2026-2027（2年）采购项目（第二次）答疑 提问1：样品20CM长含承口吗？如果含承口20CM那就太短，标识LOGO无法体现完整建议≥20CM 答1：球墨铸铁管样品含承口，样品长度≥20CM 网 务 招标人：重庆市自来水有限公司 招标代理机构：重庆水务集团公用工程咨询有限公司 商 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d30道76446.html cqdingjiu 2026.08.21 10:06:50 管 国 中</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N13" t="n">
         <v>80</v>
       </c>
@@ -1346,7 +1394,11 @@
           <t>大足区中心城区和龙水镇市政公共排水设施运维(材料)更正一号公告 一、更正项 更正项 更正子项 更正前内容 更正后内容 网上投标 网上投标截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 递交投标响应文件 线下递交投标（响应）文件开始时间 2026-08-20 14:30:00 2026-08-25 14:30:00 递交投标响应文件 线下递交投标（响应）文件截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 网 开标 开标时间 2026-08-20 15:00:00 2026-08-25 15:00:00 招标采购（附件） 附件 务 二、补遗更正说明 清单限价重新做调整，开标时间已更正，详见更正文件内容 商 三、联系方式 采购执行方： 道 单位名称：重庆誉双项目管理有限公司 联系人：陈老师 联系电话：13996336872 采购需求方： 管 单位名称：重庆市大足区茂泰市政工程有限公司 联系人：谢老师 联系电话：18523539371 信息来源:https://www.chinapipe.net/project/d3076319.html 国 cqdingjiu 2026.08.21 10:06:50 中</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N14" t="n">
         <v>80</v>
       </c>
@@ -1413,7 +1465,11 @@
           <t>璧山区2026年大路街道三台村智慧设施农业建设项目招标计划表 重庆市工程建设项目招标计划表 项目 璧山区2026年大路街道三台村智慧设施农业建设项目 名称 招标 法人 或招 网 标人 中农良品（重庆）生态农业有限公司 名称 （盖 章） 项目 批准 务 文件 及文 号 主要 1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流 建设 装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6. 内容 都市农文旅配套建设1000平方米。 商 招 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 道 璧 山 区2026 重 年 庆 大 市 路 公 招标 街 管 共 项目 道 资 三 公 源 台 项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米； 2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、 开 交 1 村 二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套； 3.项目后勤及仓储配套（含装修）5000平方米； 4.土方回填及场地平整53000平 2026-09 9182.25 招 易 智 方米； 5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米； 6.都市农文旅配套建设1000平方米。 标 中 慧 心 设 国 璧 施 山 农 分 业 中 建 心 设 项 目 中 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076777.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>水渠管网：1387米</t>
+        </is>
+      </c>
       <c r="N15" t="n">
         <v>80</v>
       </c>
@@ -1480,7 +1536,11 @@
           <t>长寿区江南街道污水处理厂更新改造工程项目公告 长寿区江南街道污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目长寿区江南街道污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源为企业 自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：长寿区江南街道污水处理厂更新改造工程包括但不限于以下内容新建混凝池-三沉池；还建格栅池； 厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统；原斜管沉淀池改 造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰）。拆除原有污泥池，新增临时污泥储罐 务 并还建污泥池；污泥堆场临时改建及恢复；实施技改期间的临时排放工程；进行基础的自控改造。 2.2 比选范围：长寿区江南街道污水处理厂更新改造工程施工图范围中的所有工作内容，包括但不限于土建工 程、设备及安装工程、工艺管道工程、电气工程、临排工程等内容，具体以比选人提供的图纸、技术规范、设 备需求清单、答疑资料、澄清资料、其他补遗资料等相关商内容为准。 2.3 建设地点：重庆市长寿区江南街道。 2.4 工期：110日历天（实际开工日期以监理工道程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 3. 参选人资格要求 管 3.1 本次比选要求参选人具备以下条件： （1）独立法人资格； （2）建设行政主管部国门颁发的有效的市政公用工程施工总承包二级及以上资质； 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 中 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月 27 日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务 大厦5楼。 5.2 比选截止时间：2026年8月 27 日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 网 联系人：曹老师 电话：023-71618725 务 代理机构：重庆招标采购（集团）有限责任公司 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 商 联系人：高老师 电话：023-67706841 道 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 管 信息来源:https://www.chinapipe.net/project/d3076456.html cqdingjiu 2026.08.21 10:06:51 国 中</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N16" t="n">
         <v>90</v>
       </c>
@@ -1547,7 +1607,11 @@
           <t>潼南区新胜镇、双江镇污水处理厂更新改造工程项目项目公告 潼南区新胜镇、双江镇污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目潼南区新胜镇、双江镇污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源 为企业自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：潼南区新胜镇污水处理厂更新改造工程，主要建设内容为新增200m?/d一体化污水处理设备基础； 更新现有污水处理系统设备，提高现有沉淀池二沉池、三沉池液位；升级处理系统（干化池改建为污泥池，新 增叠螺脱水机，改建污泥堆场及雨棚）；新建风机房－配电室防尘防渗地坪。潼南区双江镇污水处理厂更新改 务 造工程，主要建设内容为将原有斜管沉淀池改建为好氧池，新建3座竖流沉淀池，配套安装相关设备；更新污水 处理系统中老旧及故障设备；新建储药加药区与一体化危废储存间，完善污水处理配套设施。 2.2 比选范围：潼南区新胜镇、双江镇污水处理厂更新改造工程施工图范围中的工作内容（一体化设备采购及 相关安装工作除外），包括但不限于土建工程、附属工程商（包括但不限于绿化工程、工艺管线工程、电气及自 控工程、临排清淤工程等）、一体化污水处理设备基础、标准化建设、配套设备材料采购及安装工程等内容， 其中一体化设备采购及相关安装工作不在本次比选范围内；具体以比选人提供的图纸、技术规范、工程量清单、 答疑资料、澄清资料、其他补遗资料等相关内容为准。 道 2.3 建设地点：潼南区新胜镇、双江镇。 2.4 工期：120日历天（实际开工日期以监理工程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 管 3. 参选人资格要求 3.1 本次比选要求参选人具备以下条件： 国 （1）独立法人资格； （2）建设行政主管部门颁发的有效的市政公用工程施工总承包二级及以上资质； 中 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月27日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务大厦5 楼。 5.2 比选截止时间：2026年8月27日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 网 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 务 联系人：陈老师 电话：023-42756696 商 代理机构：重庆招标采购（集团）有限责任公司 道 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 联系人：高老师 管 电话：023-67706841 重庆水务电子商务平台国咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3076454.html cqdingjiu 2026.08.21 10:06:51 中</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N17" t="n">
         <v>90</v>
       </c>
@@ -1610,7 +1674,11 @@
           <t>重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 采购需求单位(全称) 重庆医科大学附属第二医院总务科 项目名称 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程 项目内容 给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源 采购预算 409674.71元 网 拟采购供应商全称 东部自来水分公司 配套业务用房第二市政水源从重庆水资源产业股份有限公司东部自来水分公司管辖范围 单一来源采购理由 的管网具体接入，属于市政管网施工，具有特殊要求。 务 公示时间 2026年8月19日-2026年8月25日 联系人及联系电话 刘老师 023-63693215 注：1.以上陈述是否真实，欢迎社会各界监督，公示时间商至少5个工作日； 2.公示期内无异议的，采购管理处将进行该项目采购；有异议请将意见反映采购人。 信息来源:https://www.chinapipe.net/project/d30道76334.html cqdingjiu 2026.08.21 10:06:51 管 国 中</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N18" t="n">
         <v>80</v>
       </c>
@@ -1677,7 +1745,11 @@
           <t>中铁二院工程集团有限责任公司G319黔江区正阳至城西段改建工程管线探测工作线上询价采购公告 中铁二院工程集团有限责任公司G319黔江区正阳至城西 段改建工程管线探测工作线上询价采购 ZTEYCQ-XJ-2026-019 网 采购单位: 中铁二院工程集团有限责任公司 发布时间: 2026-08-19 16:10 报价截止时间: 务 2026-08-21 17:00 招标方联系人: 杨先生 招标方联系电话: 商 13883021521 招标方邮箱: 监督方联系人: 李先生 道 监督方联系电话: 15823237919 监督方邮箱: 保证金: 0元 管 结算与发票信息: 详情 交货信息: 详情 国 其他说明事项: 标的明细 流水号：询2026081900304 中 计量单 技术标准及要 序号 标的名称 数量 交货期 送货地址 位 求 G319黔江区正阳至城西段 合同签订后5天内完成 西南区-重庆市-市辖 1 1 项 详见询价文件 改建工程管线探测工作 本项目服务内容。 区-黔江区-项目地点 信息来源:https://www.chinapipe.net/project/d3076309.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N19" t="n">
         <v>80</v>
       </c>
@@ -1744,7 +1816,11 @@
           <t>乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 1.招标条件 本招标项目乌江涪陵榨菜绿色智能化生产基地(一期)已由重庆市涪陵区发展和改革委员会以重庆市企业投资项目 备案证2020-500102-13-03-000003 批准建设，项目业主为重庆市涪陵榨菜集团股份有限公司，建设资金来自企业 自筹，项目出资比例为100% ，招标人为重庆市涪陵榨菜集团股份有限公司。项目已具备招标条件，现对乌江 涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 2.1 建设地点： 重庆市涪陵区马鞍街道人和社区 。 网 2.2 项目概况与建设规模：建筑面积约369384.27㎡。本项目蒸汽管道主要为室外蒸汽管道φ219x6mm，管道材质： 20#地上敷设，由14#锅炉房分汽缸分别接至6#和8#智能化车间分汽缸，蒸汽管道运行压力1.08MPa，管道设计压 力1.2MPa。 务 2.3 本次招标项目合同估算金额：580.643717万元。 2.4 招标范围： 商 （1）蒸汽管道系统本体：从锅炉房分汽缸后（含分气缸阀门）至6#车间、8#车间分气缸处，所有蒸汽管道、管 件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温（含保温层及保 护层）工作。 道 （2）钢结构桁架工程：负责本项目范围内所有钢结构架空桁架（管廊）的采购、运输、制作、安装、防腐工作。 （3）管道附件及控制系统：负责本工程范围内所有阀门、压力表、温度表、流量计、电动/气动执行机构以及配 套仪表电缆、桥架、保护管的采购、运输、安装、接线。负责与DCS/PLC系统接口的接线与联动调试。 管 （4）调试与验收：组织并确保整个蒸汽管道系统（含分气缸后段末端管道、桁架及其安全附件）通过项目所在 地特种设备安全监察管理部门实施的安装监督检验。负责报检、配合现场检验、整改、出具深化图纸并由设计 单位审核盖章、特种设备法定报检取证的全部费用，包括但不限于：施工前办理安装告知，设计院盖章审核， 施工中接受并通过安装国监督检验，最终负责取得《压力管道安装监督检验证书》与《特种设备使用登记证》， 确保蒸汽管道投入使用并备案，提交全套法定检验报告。 （5）土建工作部分 中 1）管架和桁架基础的施工，包括但不限于钢结构桁架的混凝土独立基础的土方开挖、浇筑、养护及回填恢复。 2）管道穿墙/板孔洞的开挖、封堵与修复。 3）室内外地面的开挖（包括但不限于疏水井、沟槽开挖、通行地沟、设备基础开挖）与恢复（包括但不限于土 方回填、渣土弃运、地面硬化）。 4）桁架及设备接地线的施工，包括但不限于接地极制作、接地干线敷设，并与厂区主接地网可靠连接，接地电 阻测试合格。 具体详见施工图、招标文件、工程量清单、答疑补遗等资料。 2.5 工期要求： 60 日历天 缺陷责任期要求： 24 个月 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：投标人应同时具备以下(1)、(2)项资质： （1）具备建设行政主管部门颁发的有效的建筑工程施工总承包二级及以上资质； （2）具备有效的《中华人民共和国特种设备生产许可证》（许可子项目：工业管道安装GC2级及以上）。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 网 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 务 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（涪陵区） （https://www.cqggzy.com/fulingweb/）下载招标文件、工程商量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网（涪陵区道）（https://www.cqggzy.com/fulingweb/）本项目招标公告网页下 方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-23 17:00:00前。 4.3招标人应于2026-08-24 18:00:00前在重庆市公共资源交易网（涪陵区）（https://www.cqggzy.com/fulingweb/）发 布澄清。 5.投标文件递交的内容 管 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-09 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 国 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（涪陵区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 中重庆市涪陵榨菜集团股份有限公司 代理机构: 中招国际招标有限公司 重庆两江新区黄山大道中段53号5-1（双 地 址: 重庆市涪陵区江北街道办事处二渡村一组 地 址: 鱼座A栋5楼） 邮 编: 408000 邮 编: 项目负责人: 徐老师 项目负责人: 寿云凤 电 话: 13212467016 电 话: 023-68881331-9032 传 真: 传 真: 电子邮箱: bsd2me@126.com 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市涪陵区发展和改革委员会 电 话: 023-72203687 2026年08月19日 乌江 涪陵 榨菜 绿色 智能 化生 产基地 (一 期)6#、 8#车 网 间蒸 汽管 道安 装工 务 程 中 中 国 国 重 银 重 商民 重 庆 行 庆 生 庆 涪 股 涪 银 涪 陵 份 陵 行 陵 重 投 公 有 道公 股 公 庆 标 共 限 共 份 共 银 开 保 户 资 公 资 有 资 行 户 证 110292140553VA00154 9902001860445897 430102029007791845-275 名 源 司 源 限 源 涪 行 金 交 重 交 公 交 陵 账 管 易 庆 易 司 易 支 号 有 涪 有 重 有 行 限 陵 限 庆 限 公 马 公 涪 公 国 司 鞍 司 陵 司 支 支 行 行 中 信息来源:https://www.chinapipe.net/project/d3076300.html cqdingjiu 2026.08.21 10:06:51</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>蒸汽管道：1.08M</t>
+        </is>
+      </c>
       <c r="N20" t="n">
         <v>95</v>
       </c>
@@ -1811,7 +1887,11 @@
           <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程询比采购公告 采购公告 公告编号： RQXYGG202608190057 一、采购项目基本情况 采购人：重庆巴南天然气有限责任公司 网 采购项目编号：RQCGXY202608170010 采购项目名称：重庆国际生物城配套公寓项目天然气表后管道安装工程 务 采购内容和范围：完成重庆国际生物城配套公寓项目 （民用1020户）天然气表后管道定制化服务。（含安装燃 气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个， 其它配套管件及辅材，墙体管道暗埋等） 二、供应商资格要求 商 1. 资质要求:资质要求： 1.响应供应商为中华人民共和国境内合法注册的独立法人或其他组织，具有独立承担民事责任能力，具有独立订 立合同的权利。 道 2.响应供应商应具备市政公用工程施工总承包三级及以上资质、具备有效的安全生产许可证。 3.响应供应商应为本项目配备项目负责人一名，持有市政公用工程或机电工程专业二级建造师及以上资质，且为 本单位在职人员并提供社保证明。 4.响应供应商应为本项目配备专职安全员一名，持有安全生产考核合格C证，且为本单位在职人员并提供社保证 管 明。 5.项目负责人及专职安全员社保证明期限须包含2026年5月至2026年7月。提供的社保证明，须体现上述人员的姓 名、身份证号（或社保号）、单位名称、本单位参保时间（或起始参保时间），并带有社保部门公章或社保部 门的有效电子印章。 2. 信用要求:6.信用要求国： （1）响应供应商（含联合体响应的成员单位）未被“国家企业信用信息公示系统” 网站（www.gsxt.gov.cn）列 入严重违法失信企业名单（如：提供网站查询界面截图）； （2）响应供应商（含联合体响应的成员单位）未被 “信用中国”网站（www.creditchina.gov.cn）列入严重失信 主体名单（中如：提供网站查询界面截图）。 三、采购文件的获取 采购文件在 华润守正采购交易平台 发布，不再另行线下提供纸质采购文件，凡有意参与者请自行登录守正平台 查看和下载采购文件。 四、响应文件的提交 响应文件提交 / 报价截止时间： 2026-08-25 08:00:00 （北京时间，若有变化另行通知）。 响应文件提交 / 报价方式：在响应文件提交 / 报价截止时间前，通过 华润守正采购交易平台 提交电子响应文件或 报价，逾期提交将被拒收。 五、采购人联系方式 联系人：何俊 电话：15178855716 邮箱：1460553040@qq.com 六、采购明细 行号 采购内容 需求数量 单位 补充说明 1 重庆国际生物城配套公寓项目天然气表后管道定制化服务 1 元/次 具体内容详见采购文件 七、答疑澄清、通知 答疑澄清、通知等文件一经在 华润守正采购交易平台 发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注 华润守正采购交易平台 发布的相关信息，并及时查阅和处理。 八、服务费交纳 网 本项目向成交人收取服务费,供应商收到预成交通知书和服务费交款通知书10日内,向平台运营方(华润守正招标有 限公司)支付服务费,经确认无误后由采购人发送成交通知书。平台运营方在收到服务费后向成交人开具服务费发 票。 收费标准：项目总成交金额＜50万元的采购项目，免收服务费。项目总成交金额≥50万元的采购项目，按成交金 务 额的0.15%向成交人收取（金额四舍五入，精确到分）。单项目总收费封顶100000元。其他说明：（1）总价采购， 收费基数为成交金额；单价、费率采购，收费基数为预算金额。（2）单项目存在多个成交人情形的，按总成交 金额计算收费总额，各成交人按成交比例分摊；项目总成交金额50万以上，但单个成交人成交金额少于50万仍按 比例收取服务费。 商 退款说明：成交通知书发布后,平台提供相关服务已完成,成交人已交纳服务费不予退还。 多成交人服务费收取示例： 以某项目总成交金额100万为例,A、B、C多成交人情形,总服务费为0.15万, 供应商A成交金额为50万,A服务费为0.075万; 供应商B成交金额为30万,B服务费为0.045万; 道 供应商C成交金额为20万,C服务费为0.03万。 九、其它事项 管 1.本公告在 华润守正采购交易平台 ( https://www.szecp.com.cn/ )上公开发布。 2.本项目采购通过守正平台线上进行，供应商需注册 华润守正采购交易平台 ，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 国 3.如对采购项目有异议，请登录 华润守正采购交易平台 ,通过异议菜单提出。 2026年08月19日 中 信息来源:https://www.chinapipe.net/project/d3076125.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N21" t="n">
         <v>80</v>
       </c>
@@ -1874,7 +1954,11 @@
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)非金属管道管件阀门采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）非金属管道管件阀门采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约 330 万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采 购”包括不限于非金属管道管件阀门所含设计、制造、试验、出厂检验、防腐、运输（含保护、包装及运输、 货到现场车板交货）、保险（交货验收前）、指导安装、调试、备件及专用工具、税费、技术资料和图纸及质 保期内的各种备品、备件的供应及相关的技术服务、产品质量证明书及原材料检测报告等。（详见“第五章货 物需求一览中表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 2.6 交货期： 2.6.1合同签订后3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向买方提交完整的技术资料，以供设计院开展相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）投标人具备有效的《中华人民共和国特种设备生产许可证》压力管道管子-B级及以上资质、压力管道管 件B2级及以上资质； （3）投标人具备塑料管道管子、管件的型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4. 招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年 8 月19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 网 5.投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月10 日上午09时30分，地点在重庆市公共资源交易中心开标厅（地 址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见一、二楼大厅显示屏。 务 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 商 本次招标公告在中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 道 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 管 联 系 人：张先生 电 话：023-40717888 国 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区五里店五简路2号重庆咨询大厦A栋20楼2001室 中 项目负责人：彭文婷 电 话： 023-67703002 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购 户名 开户行 投标保证金账号 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000631258 支行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051303372 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630010400 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000002549 贸易试验区分行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835014652 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146619529 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764260665 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020038958 信息来源:https://www.chinapipe.net/project/d3076119.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N22" t="n">
         <v>85</v>
       </c>
@@ -1937,7 +2021,11 @@
           <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)衬氟管道及管件采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）衬氟管道及管件采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约225万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）衬氟管道及管件采购一批” 包括但不限于制造、涂漆、包装、运输、配合验收工作、检验检测、产品质量证明书等。（详见“第五章货物 （材料）需求一览表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 中 2.6 交货期： 2.6.1合同签订后 3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向招标方提交完整的技术资料，以供设计院开展设备相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）具备有效的《中华人民共和国特种设备生产许可证》-压力管道元件制造-元件组合装置。 （3）具有防腐管道元件特种设备型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4、招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年8 月 19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 5、投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月 10 日上午09时30分，地点在重庆市公共资源交易中心开标厅 （地址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见网一、二楼大厅显示屏。 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 务 本次招标公告在 中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 商 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 道 联 系 人：张先生 电 话：023-40717888 管 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区国五里店五简路2号重庆咨询大厦A栋20楼2001室 项目负责人：彭文婷 电 话： 023-67703002 中 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630011190 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835003139 坝支行 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000000834 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146638621 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051302432 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000620855 支行 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020013554 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764235261 信息来源:https://www.chinapipe.net/project/d3076111.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N23" t="n">
         <v>85</v>
       </c>
@@ -2004,7 +2092,11 @@
           <t>重庆市益康环保工程有限公司永川分公司蒸汽管道改造项目询价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3076108.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N24" t="n">
         <v>60</v>
       </c>
@@ -2071,7 +2163,11 @@
           <t>南岸区融侨大道、江南大道片区2023年排水管网改造项目(三标段)招标计划表 重庆市工程建设项目招标计划表 项目名 南岸区融侨大道、江南大道片区 2023年排水管网改造项目（三标段） 称 网 招标法 人或招 重庆市南岸区城市建设发展（集团）有限公司 标人名称 （盖章） 务 项目批 准文件 南岸发改〔2024〕304《南岸区融侨大道、江南大道片区2023年排水管网改造项目总投资概算的批复》 及文号 主要建 包括改造市政混接点194个，改造管网8582米，商管径d300~d1500;缺陷管网开挖修复1355米，管 设内容 径d300~d600;非开挖修复8679米，管径d300~d1200。 招标文件 拟交 合同预估 招标内 招标 序号 招标项目名称 计划发布 易场 金额(万 备注 道容 方式 时间 所 元) 51处雨 污混错 重庆 招标项 接点位 管 市公 目 改 南岸区融侨大道、江南大道片区 2023年排 公开 共资 1 造，1082 2026-08 6600.00 水管网改造项目（三标段） 招标 源交 个管网 易中 三四级 国 心 缺陷修 复。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 中 信息来源:https://www.chinapipe.net/project/d3076097.html cqdingjiu 2026.08.21 10:06:52</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>管网：8582米；缺陷管网：1355米</t>
+        </is>
+      </c>
       <c r="N25" t="n">
         <v>80</v>
       </c>
@@ -2138,7 +2234,11 @@
           <t>中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购公告 永川三教水厂项目 已具备采购条件，现公开邀请供应商参加询比采购活动。 1.采购项目简介 1.1 采购项目名称：中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购。 1.2 采购方案编号：FA00000663117。 网 1.3 采购人：中交一公局重庆工程有限公司。 1.4 采购代理机构：/。 务 1.5 采购项目资金：已落实 1.6 采购项目概况： 商 永川三教水厂项目：项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建 净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、 综合楼、生产建（构）筑物以及附属建筑物等。项目合同额1.7亿元，工期450天。 道 项目地址：重庆市永川区。 2.采购范围及相关要求 管 2.1 采购范围：钢筋混凝土排水管。 2.2 交货期：2026年9月-2026年12月。 2.3 交货地点：重庆市永国川区项目指定地点。 2.4 物资质量标准：满足《混凝土和钢筋混凝土排水管》（GB/T 11836-2023）的相关要求。 3.供应商资格要求 中 3.1 供应商应依法设立且满足如下要求： （1）资质要求：本次询比采购要求供应商须是在中华人民共和国境内依法注册，具有合法有效的营业执照、税 务登记、组织机构代码等证件，具有独立法人资格、具有采购物资生产经营范围的生产商或代理商（销售商）。 （2）财务要求：供应商必须是经税务部门注册登记核准的纳税人，有依法纳税的良好记录。 （3）业绩要求：无。 （4）信誉要求：无不良履约记录、未列入工程所在地质量监督部门和中国交建、中交一公局集团企业黑名单。 因质量原因被交通部质监站通报，正在进行整改的生产厂家和产品不得参与投标。生产商或代理商（销售商） 具有良好的社会信誉，近3年内没有与骗取合同有关的犯罪或严重违法行为而引起的诉讼和仲裁；近3年不曾在合 同中严重违约或被逐；财产未被接管或冻结，企业未处于禁止或取消投标状态；在最高人民法院、信用中国 （www.creditchina.gov.cn）或各级信用信息共享平台查询拟入库单位无不良行为记录。 （5）其他要求：无。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他：无。 4.供应商报名 4.1 有意参加询比采购活动的单位，请于2026年8月19日15时00分至2026年8月26日17时00分（北京时间，下同，法 定公休日、节假日不休），登录“中交招采网”（网址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 网 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 务 5.供应商报价 5.1 报价结束（递交响应文件截止）时间为2026年8月26日17时00分。 商 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的电 子响应文件，采购人将拒收。 5.3电子采购的供应商响应文件由线上电子报价道表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 子报价表的数据为准。 6.开标 管 6.1 开标时间：与报价结束时间相同。 6.2 开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标。 国 7.发布公告的媒介 本询比采购公告在 “中交招采网” 上发布。 中 8.评审办法 本项目评审办法采用 经评审的最低价法 。 9.合同主要条款 9.1 付款条件：按月结算，上月11日至本月10日为一个结算对账期，乙方必须按照甲方要求开具合规的增值税专 用发票，无发票不予付款。结算完成后1个月内支付已结算金额的70%，剩余30%货款在结算完成后3个月内支付。 付款方式为银行转账，甲方有权采用票据支付或者供应链支付的方式支付货款，因此产生的费用包含在综合单 价中，乙方不得因此调价和索赔。如遇业主支付不及时，乙方应予理解。 9.2 履约保证金的递交： （1）R不要求递交 （2）要求递交，保证金金额：/，保证金形式：/，其他形式：/ 。 10.监督机构 监督机构名称： 中交一公局重庆工程有限公司审计部 11.成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联系400-676-5885，中标服务费请按7咨询。 11.1 收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； （3）在1000万元（含）至3000万元之间的，每次收取1000元； 务 （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 11.2 支付流程 （1）通知推送：中标结果发布后，系统自动推送缴费通知（含应缴金额及支付链接）； 道 （2）费用查询：供应商登录“中交招采网—供应商协同—服务费”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网— 供应商协同—服务费—发票查询”模块获取。 12.其他 国 / 。 13.联系方式 中 采 购 人：中交一公局重庆工程有限公司 地 址：重庆市江北区创富路5号 邮 编：361021 联 系 人：汪仁宽 电 话：13527572392 电子邮件：1176245792@qq.com 项目联系人及电话： 序号 项目名称 联系人 联系电话 1 永川三教水厂项目 高博 17788661005 中交一公局重庆工程有限公司 2026年8月19日 物资信息 序号 设备物资名称 设备物资说明 税率 单位 网 1 钢筋混凝土排水管 2000mm Ⅲ级 承插口 13% 米 信息来源:https://www.chinapipe.net/project/d3076078.html 务 cqdingjiu 2026.08.21 10:06:52 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>厂外管网：4.6km；钢筋混凝土排水管：2000m</t>
+        </is>
+      </c>
       <c r="N26" t="n">
         <v>90</v>
       </c>
@@ -2205,7 +2305,11 @@
           <t>长江流域云阳青龙段污水管网一体化建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 长江流域云阳青龙段污水管网一体化建设项目 招标法人或 招标人名称 云阳县青江环境综合整治有限公司 网 （盖章） 项目批准文 云阳发改资环【2025】55号 件及文号 务 主要建设内 新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。 容 招标方 招标文件计 拟交易场 合同预估金额 序号 招标项目名称 招标内容 备注 式 划发布时间 所 (万元) 商 长江流域云阳 新建污水管网55.5千米， 重庆市公 青龙段污水管 其中DN200管网12千 公开招 共资源交 1 网一体化建设 米、DN300管网24千 2026-08 9100.00 标 易中心云 项目EPC总承 米、DN40道0管网19.5千 招标项目 阳分中心 包 米等。 新建污水管网55.5千米， 长江流域云阳 重庆市公 其中DN200管网12千 青龙段污水管 公开招 共资源交 2 管米、DN300管网24千 2026-08 140.00 网一体化建设 标 易中心云 米、DN400管网19.5千 项目监理 阳分中心 米等监理。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 国 信息来源:https://www.chinapipe.net/project/d3075867.html cqdingjiu 2026.08.21 10:06:53 中</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>DN200管网：12千米；DN300管网：24千米；DN400管网：19.5千米；污水管网：55.5千米</t>
+        </is>
+      </c>
       <c r="N27" t="n">
         <v>80</v>
       </c>
@@ -2268,7 +2372,11 @@
           <t>中国电建水电四局华中公司重庆轨道交通17号线一期5标项目雨污水排水迁改工程施工劳务分包采购项目公开询 比采购公告 询比采购公告 采购编号： PC-0104-26J6-FP0895 一、采购条件 受中国水利水电第四工程局有限公司重庆轨道交通17号线一期5标项目委托，中水电四局华中（武汉）工程有限 公司以公开询比方式采购重庆轨道交通17号线一期5标雨污水排水迁改工程项目网，建设资金来源已落实。目前项 目已具备采购条件，现进行公开询比采购。 二、项目概况、采购范围 务 1、项目概况：重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3 站5 区间的土建）：高龙大道 站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子 站区间、石家院子站～终点区间、7/17号线联络线区间。 2、采购范围： 商 （1）雨污水排水迁改工程 （2）工程招标范围工作内容：17号线一期5标道中高龙大道站、斑竹林站及高斑竖井位于城市既有道路下方，设计 采用明挖法施工。为保证市政排水管网的正常使用，在明挖施工前需对既有管网进行临时迁改，车站结构施工 后进行恢复。施工PE钢带管长度2387米、B型排水管长度2799m、钢筋混凝土管127米，检查井239座劳务部分。 （3）施工内容详见工程量清单，以及为完成此项工程而做的一切工作。 管 3、计划工期:计划开工日期：2026年9月25日（具体时间以采购人通知为准），计划完工日期：2027年 12 月25 日； 合同工期总日历天数为457天。 4、质量要求：符合《国给水排水管道工程施工及验收规范》（GB 50268）、《混凝土结构工程施工质量验收规范》 （GB 50204）、《城镇道路工程施工与质量验收规范》（CJJ 1-2008）以及项目所在地最新的相关法规、标准和 图集。工程质量全面达到设计要求和标准，其中：验收合格率 100%，优良率达 90%以上，工程综合验收质量评 定达优良标准。 中 5、付款方式：采用银行转账/支票支付工程价款，月度结算完成具备付款条件后30天内工程进度款支付比例约定 为扣除各项保证金及费用后应付价款不低于65%；清算完成并签订《退场协议》后30天内工程进度款支付比例约 定为扣除各项保证金及费用后应付价款不低于80%；清算完成并签订《退场协议》后一年内工程进度款支付比例 约定为扣除响应人缺陷责任等相关费用后应付价款不低于90%；清算完成并签订《退场协议》，办理完成保证金 退还手续后两年内，工程进度款支付比例约定为扣除响应人缺陷责任等相关费用后应付价款的100%。 6、其他：无。 三、响应人资格要求 响应人必须满足以下全部资格要求： （1）资质要求：施工劳务不分等级 （2）主要人员要求:授权委托人（如有）及项目经理、专职安全员应提供社保和劳动合同。其中劳动合同至少提 供首、末两页，并且包含有关人员的详细信息;社保证明应提供响应截止时间前三个月的社保缴纳记录。 （3）安全三类人员要求:应提供企业主要负责人安全A证、项目经理B证、专职安全员C证。 （4）响应人具有良好的银行资信和商业信誉，没有处于被责令停业，财产被接管、冻结、破产状态。 （5）响应人应具有 雨污水排水迁改 工程的施工业绩，在近 5年内(2021年7月-2026年7月内签订)的施工合同不少 于 1 个，且签订单项合同金额均在 100 万元以上（应附成交通知书和（或）合同扫描件）。 （6）其它要求:无。 （7）本次采购不接受联合体响应。 四、采购文件的获取 凡满足本公告规定资格要求并有意参加的响应人，请于2026年8月22日10时00分前在中国电建采购招标数智化平台 （https://bid.powerchina.cn/bidweb/#/login，以下简称“数智化平台”）获取采购文件，采购文件免费提供。 五、响应文件的递交 1、响应文件递交的截止时间（响应截止时间，下同）为2026年8月26日10时30分网（北京时间），响应人应在截止 时间前通过数智化平台递交电子响应文件。 2、本次采购将通过数智化平台全程在线开展，电子响应文件的加密、提交等流程须响应人在线进行操作。响应 人须提前办理数字证书用于在线递交响应文件，办理方式详见数智化平台首页，并严格按照要求进行在线操作， 务 因操作流程失误造成的递交失败将由响应人自行承担后果。 3、开启由“数智化平台”在响应截止时间后自动对响应文件进行解密，响应人及时关注开启结果。 4、响应截止时间如有变动，采购人将及时通知已获取采商购文件的响应人。 六、发布公告的媒介 本次询比采购公告同时在中国电建阳光采购网道（https://bid-zb.powerchina.cn）上发布。 七、评审办法 采用综合评估法。 管 八、联系方式 采 购 人： 中水电四局华中（武汉）工程有限公司 国 地 址： 湖北省武汉市江岸区塔子湖东路健美街30号立城中心商务楼13、14层 邮 编： 430014 中 联 系 人： 王飞 电 话： 15827222587 电子邮箱： 107830343@qq.com 九、提出异议的渠道和方式 单位名称： 中水电四局华中（武汉）工程有限公司 电 话： 17708178186 电子邮箱： sjhzgsjw@163.com 十、纪检监督机构 响应人或者其他利害关系人认为本次采购活动存在违规违纪行为的，可以书面形式向中国水利水电第四工程局 有限公司中水电四局华中（武汉）工程有限公司纪委办公室（联系方式：17708178186）提出投诉。 2026年8月 19 日 报价网址:https://bid.powerchina.cn/notice/detail?id=2409510708 信息来源:https://www.chinapipe.net/project/d3075750.html cqdingjiu 2026.08.21 10:06:53 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>型排水管：2799m；钢筋混凝土管：127米；检查井：239座</t>
+        </is>
+      </c>
       <c r="N28" t="n">
         <v>85</v>
       </c>
@@ -2335,7 +2443,11 @@
           <t>万州区2026年超长期特别国债高标准农田建设项目拟进行预制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜的 信息公告 1.采购条件 1.1本项目万州区2026年超长期特别国债高标准农田建设项目工程已由 重庆市万州路桥建设有限公司承建，项目 业主为重庆市万州区农业技术与机械推广中心，代建业主为重庆市万州区农业发展有限公司，建设资金为国债 资金，项目出资比例为 100% ，承包人为重庆市万州路桥建设有限公司。项目已具备施工条件，现对该项目的预 制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜发布信息公告。 网 2.项目概况与采购范围 2.1建设地点：重庆市万州区走马镇、瀼渡镇、罗田镇、余家镇、高梁镇、分水镇、柱山乡等7个镇乡。 务 2.2本项目材料采购拟进行比选情况如下： 罗田镇谷山片区材料采购费暂定金额约： 17.5万元； 余家镇桥亭片区材料采购费暂定金额约： 17.99万元； 商 柱山乡山田片区材料采购费暂定金额约： 26.32 万元； 走马镇凉风片区材料采购费暂定金额约： 15.道66万元； 瀼渡镇高村片区材料采购费暂定金额约： 17.72 万元； 分水镇大冲片区材料采购费暂定金额约： 47.12 万元； 管 高梁镇茨坪片区材料采购费暂定金额约： 10.7万元； （以上片区片区金额为暂定金额，最终比选限价金额以比选文件为准）。 国 2.3计划采购周期： 以合同签订为准 日历天。 2.4采购范围：本项目各片区所包含的预制钢筋砼管、成品混凝土仿木栏杆等材料。 中 3.供应商资格要求 3.1本次材料采购要求供应商具备独立企业法人，具有本次所需材料生产能力的厂家或经销商等，其经营范围和 权限应满足本次所需材料的要求，并依法取得国家行政主管部门颁发的有效工商营业执照(建筑材料销售或水泥 制品制造、水泥制品销售等相关营业资格），所提供产品必须满足各项检测要求，达到国家现行标准规定的合 格标准。具有良好的商业信誉和充分的供应保障能力，具备相应售后服务能力。要求竞选人为一般纳税人，可 开具13%税率增值税专用发票，提供一般纳税人认定证明。 3.2本次供应商单位优先选择万州本地企业。 3.3本次 不接受 联合体竞选。 4. 报名要求 4.1报名时间：2026年8月 19日9:00起至 8月21日17:00止。 4.2报名地点：重庆市万州路桥建设有限公司经营部（重庆市万州区天城东路278号）。 4.3报名时，须提交有效的营业执照(有效工商营业执照((建筑材料销售或水泥制品制造、水泥制品销售等相关营 业资格）)，前述证书均为复印件并加盖单位公章。法定代表人参加报名的不需要授权委托书，只需要提供法定 代表人身份证明；非法定代表人参加报名的除提供法定代表人身份证明外还须提供授权委托书、委托代理人身 份证明。 4.4 本项目材料采购需提前报名。经资格预审合格后，通知资格预审合格的供应商，到承包人单位领取相关文件。 4.5本项目材料采购设七个片区进行比选，为保证比选公平、公正、有效，规定同一参选单位报名片区上限为2个， 且最终仅限中选一个片区。 5.联系方式 承包人：重庆市万州路桥建设有限公司 地 址：重庆市万州区天城东路278号 网 联系人： 张红娟 电 话：15923491915 务 邮 箱： 商 重庆市万州路桥建设有限公司 2026年8月19日 道 信息来源:https://www.chinapipe.net/project/d3075512.html cqdingjiu 2026.08.21 10:06:53 管 国 中</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N29" t="n">
         <v>80</v>
       </c>
@@ -2402,7 +2514,11 @@
           <t>中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水 管道)招标采购流标公告 发布单位：中国铁建/中铁十一局/六公司 发布时间：2026-08-19 10:40:49 投标截至时间：2026-08-18 10:00:00 内容： 各投标人： 网 中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资（污水 管道）公开招标采购（采购编号： CR1106-JC-2026-26-02）评标工作，已于北京时间2026年08月18日10:00整，在 铁建云链（https://www.crccep.com）线上平台公开开标。评审委员会根据招标文件载明的评审办法完成评审工作， 现将评审结果公示如下： 务 一、招标公告发布日期及媒体 招标公告发布日期：2026年07月27日至2026年08月01日 商 招标公告媒体：铁建云链（https://www.crccep.com） 二、拟中标信息 道 公开招标采购编号：CR1106-JC-2026-26-02 包件号：WSGD-01 序号 供应商名称 推荐排序 管 1 无 1 国 以上包件有效投标不足三家，本次招标做流标处理。 三、公示时间 中 自2026年08月19日始，至2026年08月22日止。在公示期间，所有竞标人和其他利害关系人如对公示的评审结果有 异议，可以向相关监督部门举报，逾期将不再受理。举报人必须由其法定代表人或者授权代表签字并盖章，其 他组织或者个人举报的，必须由其主要负责人或者本人签字，并附有效身份证明复印件。举报人如实反映情况 受法律保护。 公示期满，如无异议，即时生效。 监督竞诉受理部门： 中铁十一局集团第六工程有限公司招采中心 联系电话：18671041790 信息来源:https://www.chinapipe.net/project/d3075461.html cqdingjiu 2026.08.21 10:06:53</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N30" t="n">
         <v>80</v>
       </c>
@@ -2465,7 +2581,11 @@
           <t>协同创新区-四期房建三标段镀锌管件物资竞价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3075420.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N31" t="n">
         <v>60</v>
       </c>
@@ -2532,7 +2652,11 @@
           <t>中化重庆涪陵化工搬迁后污水处理厂建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 中化重庆涪陵化工搬迁后污水处理厂建设项目 招标法人或 招标人名称 重庆市涪陵交通旅游建设投资集团有限公司 网 （盖章） 项目批准文 涪发改委发[2019] 505号 件及文号 务 主要建设内 新建一体化提升泵站及管道约5000m，投资约800万元。 容 招标 招标 招标文件计 拟交易 合同预估 序号 招标项目名称 备注 内容 方式 划发布时间 场所 金额(万元) 商 本招标计划与2026年5 月25日发布的招标项目 中化重庆涪陵 重庆市 名称为“中化重庆涪陵 招标项目 化工搬迁后污 涪陵区 公道开 化工搬迁后污水处理厂 1 水处理厂建设 施工 2026-09 公共资 800.00 招标 建设项目（场外连接管 项目（场外干 源交易 网）”的招标计划，除 管部分） 中心 招标项目名称调整外， 其余内容完全一致。 管 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075591.html cqdingjiu 2026.08.21 10:国06:54 中</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>一体化提升泵站及管道：5000m</t>
+        </is>
+      </c>
       <c r="N32" t="n">
         <v>80</v>
       </c>
@@ -2599,7 +2723,11 @@
           <t>綦江区污水处理厂设施设备更新改造工程(二期)招标公告 1.招标条件 本招标项目 綦江区污水处理厂设施设备更新改造工程（二期） 已由 重庆市綦江区发展和改革委员会 以 重庆市企业投资备案证（项目代码：2502-500110-04-01-844057） 批准建设，项目业主为 重庆南州城市管 理服务有限公司 ，建设资金来自 上级补助和业主自筹 ，项目出资比例为 100% ，招标人为 重庆南州 城市管理服务有限公司。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用经评审的最低 投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 綦江区 2.2 项目概况与建设规模：对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造， 务 包括配电柜、风机、污水提升泵、在线监测等设备更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污 水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。 2.3 本项目工程总投资金额： 约1327.40万元 商 2.4 招标范围： 本项目设计施工图和招标文件、答疑、补遗、工程量清单等资料所涉及的全部内容。 2.5 工期要求： 180日历天 道 缺陷责任期要求： 24个月 2.6 标段划分（如有）： / 管 2.7 其他： / 3.政府采购工程 国 3.1 是否属于政府采购工程：否 4.投标人资格要求 中 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（綦江区） （https://www.cqggzy.com/qijiangweb/）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网（綦江区）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间 从本公告发布至2026-08-22 18:00:00前。 5.3招标人应于2026-09-11 18:00:00前在重庆市公共资源交易网（綦江区）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（綦江区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆南州城市管理服务有限公司 代理机构: 永卓国际工程技术有限公司 地 址: 重庆市綦江区红星美凯龙生活广场3幢19-3 地 址: 两江新区网泰山大道东段98号2幢10-12号 邮 编: 邮 编: 项目负责人: 赵老师 项目负责人: 廖淼 电 话: 023-48690537 电 话: 务023-60391733 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 商开户银行: 账 号: 账 号: 监督部门: 道 电 话: 2026年08月18日 綦江区污水处理厂设施设备更新改造工程（二期） 管 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051287453 中国农业银行股份有限公司重庆自由贸 重庆联合产权交易所集国团股份有限公司 312601010400083780000031123 易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146631326 信息来源:https://www.chinapipe.net/project/d3075589.html 中 cqdingjiu 2026.08.21 10:06:54</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N33" t="n">
         <v>90</v>
       </c>
@@ -2666,7 +2794,11 @@
           <t>南岸区峡口、迎龙片区农村供水保障提升工程招标计划表 重庆市工程建设项目招标计划表 项目 南岸区峡口、迎龙片区农村供水保障提升工程 名称 招标 网 法人 或招 标人 重庆市江南城市建设发展（集团）有限公司 名称 务 （盖 章） 项目 批准 商 文件 南岸发改﹝2026﹞156号 及文 号 本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体 主要 化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统， 建设 对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平 内容 台。概算批复工程建安费2975.27万元。 管 拟 招 招标文 合同预 招标 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 国 所 南岸 重 区峡 庆 口、 中 市 迎龙 朱家岩水厂升级改造工程：对全厂老旧设备进行设备更新；对全 公 片区 公 厂进行智慧化改造，增加高级工艺控制系统；对厂区建筑和构筑 共 农村 开 1 物修缮；优化加药系统投加模式，增加精确加药系统；对全厂部 2026-08 资 1600.00 供水 招 分老旧管道进行更换；金属防腐工程，对金属设备和管道的防锈 源 保障 标 刷漆工作。 交 提升 招标 易 工程 项目 中 （一 心 标段） 南岸 重 区峡 庆 口、 市 迎龙 公 片区 管网工程：延伸、改造峡口镇、迎龙镇等4个乡镇 46 公里 公 共 农村 DN40~DN300 配水主支管，36公里 DN20入户管道，新建3座一体 开 2 2026-08 资 1300.00 供水 化智慧加压泵房，入户水表改造 1752 户，并配套建设监测计量 招 源 保障 基础设施。 标 交 提升 易 工程 中 （二 心 标段） 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075572.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>DN300农村供水管网：81km</t>
+        </is>
+      </c>
       <c r="N34" t="n">
         <v>90</v>
       </c>
@@ -2733,7 +2865,11 @@
           <t>北碚区东阳天府片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区东阳天府片区农村供水提升工程 招标法人或招 标人名称（盖 重庆北碚文旅产业发展有限公司 网 章） 项目批准文件 及文号 务 工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水 主要建设内容 管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网 附属设施。 招标项目名 招标内 招标方 招标文件计划 拟交易场 合同预估金 序号 商 备注 称 容 式 发布时间 所 额(万元) 北碚区东阳 招标项目 重庆市公 天府片区农 施工招 公开招 1 2026-08 共资源交 8457.00 村供水提升 标 道标 易中心 工程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075569.html 管 cqdingjiu 2026.08.21 10:06:55 国 中</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>DN150供水管网：82千米；DN100以下供水管网：320千米；主要建设内容包含改造供水管网：437千米；管网：35千米</t>
+        </is>
+      </c>
       <c r="N35" t="n">
         <v>80</v>
       </c>
@@ -2800,7 +2936,11 @@
           <t>北碚区澄江片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区澄江片区农村供水提升工程 招标法人或招标 重庆北碚文旅产业发展有限公司 人名称（盖章） 网 项目批准文件及 文号 改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供 主要建设内容 务 水管网68.5km及其附属设施。 招标项目名 招标文件计划 合同预估金 序号 招标内容 招标方式 拟交易场所 备注 称 发布时间 额(万元) 招标项目 北碚区澄江 商重庆市公共 1 片区农村供 施工招标 公开招标 2026-08 资源交易中 8741.00 水提升工程 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 道 信息来源:https://www.chinapipe.net/project/d3075568.html cqdingjiu 2026.08.21 10:06:55 管 国 中</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>DN600供水管网：2.9km；DN300供水管网：88.863km；水管网：68.5km</t>
+        </is>
+      </c>
       <c r="N36" t="n">
         <v>80</v>
       </c>
@@ -2867,7 +3007,11 @@
           <t>涪陵区江东街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区江东街道农村供水保障能力提升工程（二期） 名称 招标 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 项目 网 批准 文件 涪陵发改〔2026〕471号 及文 号 主要 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 建设 以及配套电气工程。 务 内容 招 标 合 文 同 招 件 预 招标 标 招标方 计 拟交易 备 序号 招标项目名商称 估 项目 内 式 划 场所 注 金额 容 发 (万 布 元) 时 间 重 道 庆 市 涪 陵 公 区 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 开 公 1 涪陵区江东街道农村供水保障能力提升工程（二期） 2026-09 3137.22 管以及配套电气工程。 招 共 标 资 源 交 易 中 心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075558.html cqdingjiu 2026.08.21 10:06:55 中</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>加压泵站：4座</t>
+        </is>
+      </c>
       <c r="N37" t="n">
         <v>80</v>
       </c>
@@ -2934,7 +3078,11 @@
           <t>涪陵区龙桥街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 涪陵区龙桥街道农村供水保障能力 项目名称 提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水 名称（盖 有限公司 章） 网 项目批准 文件及文 涪陵发改〔2026〕466号 号 改造荣桂水厂老化、破损、生锈的 务 输水管道7.36公里。马武水厂增设 废水回收及污泥浓缩系统1套。荣 桂水厂增设废水回收及污泥浓缩系 主要建设 统1套。新建配水管道总长0.74公里； 商 内容 改造配水管道总长139.42公里。新 建1座微型集成泵房及改造1座泵 站(原牌坊泵站)。新增管网监测设 施40套。 道 招标 合同 招 文件 预估 标 招标方 拟交易 备 招标项目 序号 招标项目名称 计划 金 内 式 场所 注 管 发布 额(万 容 时间 元) 改造荣桂水厂老化、 破损、生锈的输水管 国 道7.36公里。马武水厂 增设废水回收及污泥 重庆 浓缩系统1套。荣桂水 市涪 厂增设废水回收及污 公 陵区 中 涪陵区龙桥街道农村供水保障能力 泥浓缩系统1套。新建 开 1 2026-09 公共 3236.36 提升工程 配水管道总长0.74公里； 招 资源 改造配水管道总 标 交易 长139.42公里。新建1 中心 座微型集成泵房及改 造1座泵站(原牌坊泵 站)。新增管网监测设 施40套。 本计划表所列招标项目信息均为暂 备注 定，最终以实际招标时的信 信息来源:https://www.chinapipe.net/project/d3075556.html cqdingjiu 2026.08.21 10:06:55</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>输水管道：7.36公里；配水管道：0.74公里；配水管道：139.42公里</t>
+        </is>
+      </c>
       <c r="N38" t="n">
         <v>90</v>
       </c>
@@ -3001,7 +3149,11 @@
           <t>涪陵区百胜镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区百胜镇农村供水保障能力提升工程 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕465号 及文 号 务 主要 建设整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。 内容 招 拟 标 招招标文 合同预 交 序项 标件计划 估金 备 招标内容 易 号目 方发布时 额(万 注 场 名 商 式间 所 元) 称 涪 陵 区 重 百 庆 胜 市 招标 镇 涪 项目 农 道 陵 村 公 区 供整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1开 公 1 2026-09 1489.90 水套及配套电气工程。 招 共 保 标 资 障 源 能 交 力 易 提 中 管 升 心 工 程 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075553.html 国 cqdingjiu 2026.08.21 10:06:55 中</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>取水泵站水泵：1套；及整治输配水管网：111.47公里；加压泵站：2座</t>
+        </is>
+      </c>
       <c r="N39" t="n">
         <v>80</v>
       </c>
@@ -3068,7 +3220,11 @@
           <t>涪陵区清溪镇农村供水保障能力提升工程招标计划 重庆市工程建设项目招标计划表 项目名称 涪陵区清溪镇农村供水保障能力提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕467号 务 号 对清溪水厂原取水口进行改造。改造清溪水厂输水管道长6.38公里。清溪水厂新建3000m3/d集成水 主要建设 厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04 内容 公里。四合村泵站增加1套备用加压泵。新商增管网监测设施35套。 招标项目 招标方 招标文件计 拟交易场 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 所 (万元) 对清溪水厂原道取水口进行 改造。改造清溪水厂输水 管道长6.38公里。清溪水厂 涪陵区清 新建3000m3/d集成水厂1套， 重庆市涪 招标项目 溪镇农村 增设废水回收及污泥浓缩 公开招 陵区公共 管 1 供水保障 2026-09 2888.89 系统1套。新建配水管道总 标 资源交易 能力提升 长2.46公里。改造配水管道 中心 工程 总长145.04公里。四合村泵 站增加1套备用加压泵。新 国 增管网监测设施35套。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075552.html 中 cqdingjiu 2026.08.21 10:06:55</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>清溪水厂输水管道：6.38公里；配水管道：2.46公里；四合村泵站：1套；新商增管网：35套；管道：6.38公里；增管网：35套</t>
+        </is>
+      </c>
       <c r="N40" t="n">
         <v>80</v>
       </c>
@@ -3135,7 +3291,11 @@
           <t>涪陵区珍溪镇农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区珍溪镇农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕476号 及文号 (一)改造11000m3/d(旺水垭6000m3/d和二水厂5000m3/d)原水处理系统及辅助设施，主要有加氯系统、 加药系统、清水池、絮凝池、重力无阀滤池、商污水处理回收池、二水厂泵房设备等及其他辅助设施。 主要建 (二)更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪 设内容 湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km， 新建应急泵站至百汇大桥配水管9km：百汇至观将泵站4.5km；共计37.3km。 道 招标项目 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 场所 (万元) (一)改造11000m3/d(旺水 垭6000m3/d和二水厂5000m3/d) 管 原水处理系统及辅助设施，主 要有加氯系统、加药系统、清 水池、絮凝池、重力无阀滤池、 污水处理回收池、二水厂泵房 涪陵国区珍 设备等及其他辅助设施。(二) 重庆市 招标项 溪镇农村 更换旺水垭水厂至张家塘配水 涪陵区 目 供水保障 公开招 1 管13.5km，张家塘至滴水配水 2026-09 公共资 3427.27 能力提升 标 管长3.3km，全长16.8km；滴水 源交易 中工程（一 至洪湖配水管长0.3km；更换八 中心 期） 一水库至旺水垭水厂引水 管1.7km，更换珍溪二水厂至珍 溪大桥配水管5km，新建应急 泵站至百汇大桥配水管9km： 百汇至观将泵站4.5km；共 计37.3km。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075551.html cqdingjiu 2026.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>应急泵站：9km；百汇至观将泵站：4.5km；泵站：9km</t>
+        </is>
+      </c>
       <c r="N41" t="n">
         <v>80</v>
       </c>
@@ -3202,7 +3362,11 @@
           <t>涪陵区武陵山镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区武陵山镇农村供水保障能力提升工程 名称 招标 网 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 务 （盖 章） 项目 批准 商 文件 涪陵发改〔2026〕468号 及文 号 主要 道 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高位水箱4座（总容积 354立方米），武 建设 陵山水厂新建废水处理系统1套及配套电气工程等。 内容 招 管 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 国 称 涪 陵 区 中 重 武 庆 陵 市 山 招标 涪 镇 项目 陵 农 公 区 村 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高 开 公 1 供 位水箱4座（总容积 354立方米），武陵山水厂新建废水处理系统1套 2026-09 1861.77 招 共 水 及配套电气工程等。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075549.html cqdingjiu 2026.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>及整治输配水管网：124.26千米；加压泵站：5座</t>
+        </is>
+      </c>
       <c r="N42" t="n">
         <v>80</v>
       </c>
@@ -3269,7 +3433,11 @@
           <t>涪陵区江东街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区江东街道农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕470 号 及文号 主要建 建设配水管网总长 34.80km，新建加压泵站 2 座、改造已成泵站 2 座、新建加氯加药间 1 座、新建高位 设内容 水箱 7 座、新建计量监测设施以及配套电气工程商。 招 招标文件 拟交 合同预估 序 招标项 标 备 招标内容 计划发布 易场 金额(万 号 目名称 方 注 道 时间 所 元) 式 涪陵区 重庆 招标项 江东街 市涪 目 建设配水管网总长 34.80km，新建加压泵站 2 座、 公 道农村 陵区 管 改造已成泵站 2 座、新建加氯加药间 1 座、新建高 开 1 供水保 2026-09 公共 3503.77 位水箱 7 座、新建计量监测设施以及配套电气工 招 障能力 资源 程。 标 提升工程 交易 （一期） 中心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075548.html cqdingjiu 20中26.08.21 10:06:56</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>配水管网：34.80km；加压泵站：2座；已成泵站：2座</t>
+        </is>
+      </c>
       <c r="N43" t="n">
         <v>90</v>
       </c>
@@ -3332,7 +3500,11 @@
           <t>中国电建水电五局二公司重庆轨道交通17号线一期7标内外涂环氧消防复合钢管管件采购项目公开竞价采购(二次 挂网)变更公告(一) 详见附件。 信息来源:https://www.chinapipe.net/project/d3075376.html cqdingjiu 2026.08.21 10:06:56 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N44" t="n">
         <v>60</v>
       </c>
@@ -3399,7 +3571,11 @@
           <t>涪陵区蔺市街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（一期） 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕474号 及文 号 主要 务 建设新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。 内容 拟 招招标文 合同预 招标 交 序 标件计划 估金 备 项目招标内容 易 号 方发布时 额(万 注 名称 场 式间 元) 所 商 重 庆 涪陵 市 区蔺 招标 市街 涪 项目 道农 陵 公 区 村供 新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收 开 公 1 水保 2026-09 3611.91 及污泥浓缩处理系统。 招 共 障能 道 标 资 力提 源 升工程 交 （一 易 期） 中 心 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075278.html 管 cqdingjiu 2026.08.21 10:06:57 国 中</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>配水管网：396.72km</t>
+        </is>
+      </c>
       <c r="N45" t="n">
         <v>80</v>
       </c>
@@ -3466,7 +3642,11 @@
           <t>涪陵区李渡街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区李渡街道农村供水保障能力提升工程 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕469号 及文 号 商 主要 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套 建设 附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建测控井78座。 内容 招 拟 标 道 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 管 涪 陵 区 重 李 庆 渡 市 街 国 招标 涪 道 项目 陵 农 公 区 村 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂 开 公 1 供 塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建 2026-09 2372.74 招 共 水中测控井78座。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075277.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>配水主管网：193.71千米；泵站：1座；集成泵站：4座</t>
+        </is>
+      </c>
       <c r="N46" t="n">
         <v>80</v>
       </c>
@@ -3533,7 +3713,11 @@
           <t>涪陵区珍溪镇农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目名称 涪陵区珍溪镇农村供水保障能力提升工程（二期） 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕477号 务 号 (一)本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管 主要建设 有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵 内容 站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水 箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。 招标项目名 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 称 式 划发布时间 场所 (万元) 道 (一)本项目对珍溪镇23个 村(社区)安装配水管网660km 及配套附属设施，其 中：1.De160~De40的PE管 管 有232km；2.连接各村社 涪陵区珍溪 重庆市 的De32~De20的PE管有381km； 招标项目 镇农村供水 涪陵区 3.219~32的衬塑钢 公开招 1 保障能力提 2026-09 公共资 2182.77 管47km。(二)购置安装泵 标 升工国程（二 源交易 站14座(一用一备共计28台水 期） 中心 泵)，其中新建泵站10座、更 换泵站4座及配套电力设施; 新建不锈钢水箱2座等。(三) 中 购置安装(0~25kg)减压阀61 个;排污阀(25kg）3个。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075275.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>配水管网：660km；的衬塑钢管：47km；泵站：4座；泵站：10座；换泵站：4座</t>
+        </is>
+      </c>
       <c r="N47" t="n">
         <v>90</v>
       </c>
@@ -3600,7 +3784,11 @@
           <t>涪陵区蔺市街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（二期） 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕475号 及文 号 商 主要 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 105.307km（dn20-dn40PE 建设 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座；新建测控井 52座。 内容 拟 招 招标文 合同预 招标 交 序 道 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 重 庆 涪陵 管 市 区蔺 涪 招标 市街 陵 项目 道农 公 区 村供 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 开 公 1 水保 105.307km（dn20-dn40PE 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座； 2026-09 2652.89 国 招 共 障能 新建测控井 52座。 标 资 力提 源 升工程 交 （二 易 期） 中 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075274.html cqdingjiu 2026.08.21 10:06:57</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>管网：105.307km；泵站：1座</t>
+        </is>
+      </c>
       <c r="N48" t="n">
         <v>80</v>
       </c>
@@ -3663,7 +3851,11 @@
           <t>重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目项目公告 重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称）比选公告 1.比选条件 本比选项目重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称），比选人为重庆市排 网 水有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。中标后合同与重庆市豪洋水务 建设管理有限公司签订。现对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 2.项目概况与比选范围 务 2.1 建设地点：重庆市巴南区 2.2 项目概况：本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1,该管道为自流管道， 位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道 为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现 象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水 厂的正常收水及运行，需对该段管道进行改造。 道 2.3 比选范围：拆除现状管道为DN600混凝土管，同时需拆除并新建9座检查井。 2.4 工期要求：30日历天，以甲方通知进场时间为准。 管 2.5缺陷责任期要求：24个月 3.投标人资格要求 国 3.1 本次比选要求投标人须具备以下条件： 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质。 中 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 项内容。 3.2 本次比选接受不联合体投标。 4.比选文件的获取 4.1 投标人于2026年8月 18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子 版，以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都 视为投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的 一切后果由投标人自行负责。各投标单位应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行供应商注册，填写相关信息，审批过后成为 平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价、递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，将被否决投标。 4.4 比选文件每份售价800元，售后不退。投标单位在递交纸质投标文件时扫描支付，否则比选人拒绝接收其投标 文件。 5.投标文件的递交 5.1 电子投标文件递交时间：2026年8月24日14时30分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年8月24日14时00分至14时30分（北京时间），地点：重庆水务招标采购中心 （重庆市两江新区嘉华路36号重庆水务大厦5楼）。 5.3 投标截止时间：2026年 8月24日14时30分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆市排水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝中区长江滨江路126号 地 址：重庆市两江新区嘉华路36号重庆水务大厦 道 联 系 人： 黄老师 联 系 人： 黄晓华 电 话： 023-67767416 电 话： 18523396416 管 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3075272.html 国 cqdingjiu 2026.08.21 10:06:57 中</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N49" t="n">
         <v>90</v>
       </c>
@@ -3730,7 +3922,11 @@
           <t>重庆市潼南城区老旧供水管网改造工程招标计划 重庆市工程建设项目招标计划表 项目名称 重庆市潼南城区老旧供水管网改造工程 招标法人或招 标人名称（盖 重庆市潼南自来水有限公司 网 章） 项目批准文件 及文号 务 主要建设内容 改建潼南城区输水主管网约39.63km及配套相应阀门阀件等 招标方 招标文件计 拟交易场 合同预估 序号 招标项目名称 招标内容 备注 式 划发布时间 所 金额(万元) 对城区供水管网上商 重庆市潼南城 老旧阀门阀件、设 区老旧供水管 重庆市潼 招标项目 施设备进行更换， 网改造工程 公开招 南区公共 1 保障供水管网稳定 2026-09 918.00 （城区配套阀 标 资源交易 运行合道理增设部分 门阀件改造工 中心 计量及压力监控、 程） 水质监控等。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3075266.html cqdingjiu 2026.08.21 10:06:58 国 中</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>输水主管网：39.63km</t>
+        </is>
+      </c>
       <c r="N50" t="n">
         <v>80</v>
       </c>
@@ -3797,7 +3993,11 @@
           <t>关于为【重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购】公开选取【工程设计】 机构的公告 我单位在重庆市网上中介超市公开选取工程设计中介服务机构，现将相关事项公告如下： 该项目为直接选取项目，由采购人从报名的中介服务机构中直接选定一家中介服务机构进行项目服务。 项目 重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购 名称 网 采购 重庆市开州区河堰镇人民政府 人 投资 审批 否 务 项目 是否 破产 商 业务 否 服务 项目 采购 道 所需 中介 其他 服务 事项 管 所需 服务 工程设计 类型 项目实施地点为国河堰镇清泉社区，项目建设内容为：硬化2米宽生产便道5.5千米，100方防旱池1口，50方 服务 蓄水池1口，标准自动化育苗大棚1个，蔬菜小棚20个，水源处理设施1套，水肥一体化配套设施1套，新 内容 建50平方米设备管理房，完善蔬菜基地配套设施等。工程总投资335万元。选取此项目设计单位（含预算 编制服务）。 中 中介 机构 资质（资格）要求 要求 资质 （资 1、报名单位提供有效的营业执照，资质证书（资质丙级或丙级以上），具备从事项目设计服务工作； 2、 格） 具有独立承担民事责任的能力； 3、具有良好的商业信誉和健全的财务会计制度； 4、具有履行合同所必 要求 需的专业技术能力； 5、有依法缴纳税收和社会保障资金的良好记录。 说明 其他 要求 无 说明 服务 时限 无要求，按照合同双方自行约定 说明 服务 3.1%费率 金额 金额 按文件要求执行 说明 选取 直接选取 方式 需规 避机 构 规避 原因 选取 2026-08-20 16:00:00 （选取时间到达后不接受报名，建议中介机构至少在选取开始半小时前完成报名。） 时间 采购 人业 网 务咨 重庆市开州区河堰镇人民政府（18716685679） 询电 话 采购 务 需求 26清泉社区项目设计服务采购说明.pdf 书下 载 商 2026-08-18 信息来源:https://www.chinapipe.net/project/d3075198.html 道 cqdingjiu 2026.08.21 10:06:58 管 国 中</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N51" t="n">
         <v>90</v>
       </c>
@@ -3864,7 +4064,11 @@
           <t>重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目招标公告 1.招标条件 本招标项目重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目已由重庆市开州区发展和改革委员会以开州 发改审〔2026〕357号批准建设，项目业主为重庆市开州区长沙镇人民政府，建设资金来自开州区2026年中央和 市级提前批财政衔接推进乡村振兴补助资金，项目出资比例为 100% ，招标人为重庆市开州区长沙镇人民 政府。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：开州区长沙镇桔香村 2.2 项目概况与建设规模：1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输 线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米， 务 周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。 2.3 本项目工程总投资金额： 500万元 本次招标项目合同估算金额： 446.278921万元 商 2.4 招标范围：招标人发布的由重庆中煜华资工程技术有限公司设计的《重庆市开州区2026年长沙镇桔香村柑橘 基地改造提升项目》施工图及图纸说明、招标文件(含补遗)及工程量清单、答疑资料、澄清资料范围内所涉及的 工作内容，具体以招标人发布的工程量清单及道施工图为准。 2.5 工期要求： 150日历天 缺陷责任期要求： 12个月 管 2.6 标段划分（如有）： / 2.7 其他： / 国 3.政府采购工程 3.1 是否属于政府采购工程：是 中 3.2 是否专门面向中小企业预留：否，按照《政府采购促进中小企业发展管理办法》第六条第(三)“按照本办法 规定预留采购份额 无法确保充分供应、充分竞争，或者存在可能影响政府采购目标实现的情形”的规定，故本 项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的建筑工程施工总承包叁级及以 上资质或市政公用工程施工总承包叁级及以上资质或水利水电工程施工总承包叁级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）下载招 标文件、工程量清单、电子图纸等资料。参与投标的投标人需在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）完成市 场主体信息登记以及CA数字证书办理，办理方式请参见 重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、 重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）导航栏“主体信息”页面中“市场主 体信息登记”、“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完 成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告 发布至2026-08-21 17:00:00前。 5.3招标人应于2026-08-25 23:59:59前在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源 交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）发布澄清。 6.投标文件递交的内容 网 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-21 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 务 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交 易监督网上发布。] 商 8.联系方式 招 标 人: 重庆市开州区长沙镇人民政府 代理机构: 重庆毅仁建设项目管理有限公司 重庆市开州区文峰街道天鹅湖社区富厚街158号附10 地 址: 重庆市开州区长沙镇山花街1号 地 址: 道号 邮 编: 邮 编: 项目负责人: 丁敬余 项目负责人: 谭毅 电 话: 15826368887 管电 话: 13452653126 传 真: 传 真: 电子邮箱: 1415705480@qq.com 电子邮箱: 开户银行: 国 开户银行: 账 号: 账 号: 监督部门:中重庆市开州区公共资源交易管理局 电 话: 023-52218977 2026年08月17日 重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目 户名 开户行 投标保证金账号 重庆市开州区公共资源交易中心 重庆农村商业银行股份有限公司开州支行 3401010120010012772000200 中国农业银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 314401010400104500000006031 业部 中国工商银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 9558853100005824176 业部 重庆市开州区公共资源交易中心 重庆银行股份有限公司开州支行 680101040007547-100984 重庆市开州区公共资源交易中心 中国银行股份有限公司重庆开州支行 108865555576VA00149 信息来源:https://www.chinapipe.net/project/d3075199.html cqdingjiu 2026.08.21 10:06:58</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N52" t="n">
         <v>90</v>
       </c>
@@ -3931,7 +4135,11 @@
           <t>万盛城区老旧供水管网更新改造工程答疑及补遗(一) 万盛城区老旧供水管网更新改造工程 答疑及补遗（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程答疑及补遗（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。? 问题2：本项目是否采用异地评标方式？ 答：是 。 商 问题3：本项目是否有业主代表，如有，请明确业主代表数量。 答：是，本项目评标委员会共7人，其中在重道庆市综合评标专家库随机抽取5人，招标人代表2人 。 问题4：投标函中的缺陷责任期可以填“达到招标文件的要求”吗？ 答：可以。 管 问题5：污水处理厂提标改造及附属管道施工业绩满足吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 国 问题6：投标文件格式中下划线上、空格处、表格中无需要填写或无法填写内容的，是填“/”或“无”还是可以 不填(空白)，对此有无要求？ 答：无要求。? 中 问题7：我公司业绩为epc业绩，我公司与设计单位组成联合体承接，竣工验收报告中施工单位盖章由我公司盖章， 请问需要提供联合体协议书吗？ 。 答： 根据招标文件第二章“投标人须知前附表”1.4.1 第3条业绩要求中：“注：（2）投标人提供的业绩为联 合体业绩的，其在该业绩中的工作分工应与本项目承担的工作一致。”要求，故需要提供联合体协议书。 问题8：投标函附录中，工期、分包和工程质量要求对应的约定内容，可以统一填写“达到招标文件要求”吗？ 答：填写“达到招标文件的要求”或按照招标文件相关条款填写具体内容均可 。 问题9：招标人提供的工程量清单单项最高限价中金额为零的，清单综合单价报价可以为0吗？ 答：投标人的工程量清单单项报价不得为零报价(招标人提供的工程量清单单项最高限价中金额为零的除外)或者 负数报价，否则由评标委员会作否决投标处理。 问题10：招标人应当在法定时间内确定中标人。招标人或者招标投标交易场所运行服务机构应当在中标通知书发 出后 5 日内，向除中标人以外的其他投标人退还纸质投标保函正本，并书面通知相关金融机构本项目准予提前注 销纸质投标保函。具体注销事宜由投标人与金融机构协商。保函原件上需要加盖正本吗？ 答：需要。但不将加盖正本作为评审因素。 问题11：我公司业绩为三个项目合并招标，三个项目合起来满足业绩要求，但分别签了三个合同和分别验收，请 问我公司业绩满足业绩要求吗？ 答：不满足。? 问题12：财务报告可以只提供审计报告、现金流量表、资产负债表、利润表吗？ 答：可以 。 问题13：业绩要求的竣工时间是指竣工验收时间吗？ 答：是的。 网 问题14：重庆市电子招投标系统投标文件-报价部分“己标价工程量清单”-“投标总价”页面招标人名称需要填 写吗？ 务 答：由投标人自行决定是否填写，是否填写不作为评审因素。 问题15：请问招标人是否委派业主专家参与评标吗？ 答：是，本项目评标委员会共7人，其中在重庆市综合评商标专家库随机抽取5人，招标人代表2人。 问题16：自来水厂或者净水厂含管道施工业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需道满足招标文件要求。? 问题17：有没有人行贿专家，有的话我们就不参加了。 答：本项目评标委员会由招标人按法律法规及相关规定依法组建。 管 问题18：招标文件第八章投标文件格式中（二）承诺部分是否包含招标文件要求的所有承诺，投标人是否还需要 提供其他格式之外的其他承诺？ 答：请各潜在投标人仔国细阅读招标文件，并按招标文件要求提供相应承诺。 问题19：财务报告可以不提供财务报表附注吗？ 答：可以。 中 问题20：乡、镇供水厂及供水管道业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题21：在职的已退休的注册人员，其社保局出具的养老证明已无法提供，该类人员是否可以用退休证、注册证 及在本单位注册的证明文件替代？ 答：退休证等材料不能替代养老保险证明，按招标文件执行。? 问题22：本项目是异地评标吗？ 答：是。 问题23：现在除了没有警戒线和技术方案的低价项目评标专家不被围猎，哪个项目不围猎评标专家，请问招标人 如何保证公平？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题24：没有低价警戒线怎么保证中高价呢？ 答：本项目未设置低价警戒线，通过综合评估法对各潜在投标人进行评审。分值由技术、商务、报价组成，综 合实力优良的投标人合理中高价可依靠综合得分优势参与竞争，同时招标文件履约追责条款约束投标人理性报 价，保障合理报价竞争环境。 问题25：现场递交纸质保函原件是否需要本项目投标人须知前附表中要求的委托代理人持授权委托书和养老保险 证明材料复印件递交吗？ 答：现场递交纸质保函原件的人员不作要求 。 问题26：请问投标文件制作系统软件导出的电子投标文件格式与加盖公章的招标文件PDF文件中的投标文件格式 不一致的以哪个为准？ 网 答：电子投标系统中锁定不可修改的格式（如封面、投标函）直接填空即可，其他投标文件格式以加盖公章的 招标文件PDF文件为准。? 问题27：专业分包业绩满足业绩要求吗？ 务 答：不满足。 问题28： 市政道路包含给水管网施工业绩满足业绩要求吗？ 商 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题29：技术负责人在资格审查部分中提供了工程类高级及以上职称证后，在商务部分中再提供工程类高级及以 上职称证可以加分吗？ 道 答：可以。 问题30：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 管 全是万盛的公司中的！业主、专家全是你们自己人吧？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 国 二、补遗 1、本次重新发布本项目的工程量清单，在《重庆市公共资源交易网》(綦江区) （https://www.cqggzy.com/qijiangweb/）网上发布，请投标人自行下载。 中 招 标 人：重庆市万盛经济技术开发区城市管理局 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 信息来源:https://www.chinapipe.net/project/d3074975.html cqdingjiu 2026.08.21 10:06:58</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N53" t="n">
         <v>80</v>
       </c>
@@ -3998,7 +4206,11 @@
           <t>重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 1.招标条件 本招标项目 重庆市巴南区土桥片区内涝积水整治工程已由重庆市巴南区发展和改革委员会以巴南发改审 发[2025]33号文批准建设，项目业主为重庆市巴南区住房和城乡建设委员会，代建业主为重庆市巴南公路建设有 限公司，建设资金来自区级财政资金统筹，项目出资比例为 100%，招标人为重庆市巴南公路建设有限公司。 项目已具备招标条件，现对该工程的勘察设计进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 2.1 建设地点：重庆市巴南区花溪街道、李家沱街道 务 2.2 项目概况与建设规模：为解决片区内涝问题，在李家沱街道、花溪街道改建 d400-d800 雨水管网 9665m，管材 采用高密度聚乙烯(HDPE)缠绕结构壁管 B型管；改建 d1商000-d1400雨水管网 664m，管材采用高密度聚乙 烯(HDPE)缠绕结构壁管 B 型管、III 级钢筋混凝土管；改建 d1500-d2000 雨水管网 426m，管材采用III 级钢筋混凝 土管;改建 d2100-d2600 雨水管网 1000m，管材采用 III 级钢筋混凝土管；修复雨水管网 5345m，增加智能感知设 备6 套。 道 2.3 本项目工程总投资金额：13477.10万元 管 本次招标项目工程费估算金额：11061.83万元 国 本次招标项目勘察设计合同估算金额：334.544万元 中 2.4 招标范围：主要包括勘察、施工图设计（包含高边坡、深基坑）和相应阶段的勘察工作，以及提供施工现场 全过程技术服务，并配合业主办理相关手续等，具体范围为： （1）勘察部分：完成本项目范围内的勘察工作，包括但不限于排水管网排查、1:500地形图测量、地质钻勘、管 线内窥、物探、综合管线测量，市政管网错混接点测量及调查等工作，解决区域地下空间臭气问题，勘察成果 需达到重庆市城市建成区排水管网排查技术导则的要求，并配合业主完成对应的成果审查等事宜。 （2）设计部分：包括不限于完成本项目的施工图设计、施工期间交通组织设计、桥梁（涉轨）安全论证方案及 施工期间至竣工验收阶段，质量保修阶段的设计配合服务，配合办理施工图审查相关手续及竣工验收阶段、质 量保修阶段的设计服务等工作以及协助招标人完成各项审批手续办理等工作。 2.5 勘察设计服务期限：30日历天 2.6 标段划分（如有）：/ 2.7 其他：/ 3.政府采购工程 3.投标人资格要求 3.1 本次招标要求投标人须具备以下条件： 网 3.1.1 本次招标要求投标人具备的资质条件： 务 投标人应同时具有建设行政主管部门颁发的下列勘察和设计两类资质： 商 I、投标人应具备下列勘察资质之一： 道 ①工程勘察综合甲级资质。 管 ②工程勘察专业类（岩土工程）专业甲级资质和工程勘察专业类（工程测量）甲级资质； 国 II、投标人应具备下列设计资质之一： 中 ①工程设计综合甲级资质； ②工程设计市政行业甲级资质； ③工程设计市政行业(燃气工程、轨道交通工程除外)甲级资质； ④工程设计市政行业(排水工程)甲级资质。 3.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的勘察设计能力，详见招标文件第二章投标人须知 前附表第1.4.1项内容。 3.2 本次招标接受联合体投标。联合体投标的，应满足下列要求：联合体组成单位数量不超过2家，由负责设计 任务的单位作为联合体牵头人。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件及其附件、澄 清、修改、补充通知、最高限价通知等资料。参与投标的投标人需在重庆市公共网资源交易网完成市场主体信息 登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息 登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程 电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 务 布至2026-08-23 12:00:00前。 4.3招标人应于2026-08-26 17:00:00前在重庆市公共资源交易网发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-24 09:30，投标人应当在投标截止时间前，通过互 商 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督道网、重庆市公共资源交易网、重庆市公共资源交易网（巴南区） 发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 重庆市巴南公路建设有限公司 代理机构: 重庆云远项目管理有限公司 管 地 址: 重庆市巴南区龙洲大道265号 地 址: 重庆市九龙坡区渝隆大厦28楼 邮 编: 邮 编: 项目负责人: 牟老师 项目负责人: 李强 国 电 话: 023-66238079 电 话: 023-68434996 传 真: 传 真: 电子邮箱: 电子邮箱: 中 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市巴南区发展和改革委员会 电 话: 023-66221670 2026年08月18日 重庆市巴南区土桥片区内涝积水整治工程勘察设计 户名 开户行 投标保证金账号 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000001675 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051304894 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020041267 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764210157 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000682897 支行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835000509 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146639123 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630018252 信息来源:https://www.chinapipe.net/project/d3074953.html cqdingjiu 2026.08.21 10:06:58 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>d800 雨水管网：9665m；d1400雨水管网：664m；d2000 雨水管网：426m；d2600 雨水管网：1000m；雨水管网：5345m</t>
+        </is>
+      </c>
       <c r="N54" t="n">
         <v>95</v>
       </c>
@@ -4065,7 +4277,11 @@
           <t>重庆燃气集团股份有限公司输配分公司大渡口调压站至二郎调压站次高压燃气管线工程(大渡口段)公告 采购 公告 公告编号： RQXYGG202608130064 一、采购项目基本情况 网 采购人：重庆燃气集团股份有限公司输配分公司 采购项目编号：RQCGXY202608130040 务 采购项目名称：大渡口调压站至二郎调压站次高压燃气管线工程（大渡口段） 采购内容或范围：安装部分： ①材料验收（甲供材料：阀门、管材、弯头、标志桩等）、运输及履带式挖掘机及人工布管； ②管道管件安装， 新旧管道的碰口；③安装DN400直埋球阀1座； ④管道和商焊口的除锈及防腐； ⑤管道下沟后15KV电火花检测； ⑥管道的清管，强度及严密性试验；⑦警示带敷设和线路标志桩（砖）安装； ⑧监检手续等。 土建部分： ①清表； ②扫线、平整场地； ③沟槽、基坑、阀井砌筑； ④回填土方； ⑤余方弃置； ⑥人工开挖人行道（花 台），公路及路面恢复； ⑦其他线缆穿跨越工道程施工，交通组织； ⑧水工保护等。 （具体内容详见施工图纸和 工程量清单） 公告发布时间 ：2026-08-18 14:39:10 管 二、采购人联系方式 联系人：王瑶 电话：023-67502265 国 邮箱：wangyao232@crcgas.com 三、采购明细 中 行号 采购内容 需求数量 单位 补充说明 拟邀请单位 大渡口调压站至二郎调压站次高压燃气管线 重庆燃气安装工程有限责任公 1 1 项目 无 工程(大渡口段) 司 四、服务费交纳 本项目不收取服务费。 五、 其他 事项 1.本公告在华润守正 采购交易 平 台（ https://www.szecp.com.cn/ ）上公开 发布。 2. 本项目采购通过守正平台线上进行，供应商需注册华润守正 采购交易 平台，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 3 .答疑澄清、通知等文件一经在华润守正 采购交易 平台发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注华润守正 采购交易 平台发布的相关信息，并及时查阅和处理。 4 .若有参与意向 ， 请于 2026-08-22 00:00:00前联系采购人 （联系方式见公示内容）反馈。 5 .若有异议 ， 请于 2026-08-22 00:00:00前提出异议 。 信息来源:https://www.chinapipe.net/project/d3074793.html cqdingjiu 2026.08.21 10:06:59 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N55" t="n">
         <v>80</v>
       </c>
@@ -4132,7 +4348,11 @@
           <t>石柱公司2026-2027年度用户供水管道安装及管网抢(维)修工程(第二次)项目公告 石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（比选公告 1.比选条件 本比选项目石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（项目名称），比选人 为重庆石柱水利水电实业开发有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。现 对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 网 2.项目概况与比选范围 2.1 建设地点：比选人指定地点 务 2.2 项目概况与建设规模：2026-2027年度用户供水管道安装及管网抢（维）修服务 2.3 本次比选项目合同估算金额：约280万元 商 2.4 比选范围：完成石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程包括公司供水范围内用户 各类管道及管件安装、水表安装及更换、阀门安装等、并完成配套土建工程、零星签证等工程量清单所列项目、 管网抢维修和公司所属生产单元零星项目，具体内容详见第五章 工程量清单。 道 2.5 工期要求：1年 缺陷责任期要求：24个月 管 3.投标人资格要求 3.1 本次比选要求投标人须具备以下条件： 国 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质； 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 中 项内容。 3.2 本次比选不接受联合体投标。 4.比选文件的获取 4.1 投标人于2026年08月18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子版， 以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都视为 投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的一切 后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价，递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，被视为无效。 4.4比选文件每份售价1000 元，售后不退。投标人在递交纸质投标文件时支付，否则比选人拒绝接收其投标文 件。 5.投标文件的递交 5.1电子投标文件递交时间：2026年08月24日10时00分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年08月24日09时30分至10时00分，地点：水务集团招标采购中心（重庆市两江新 区嘉华路36号重庆水务大厦五楼）。 5.3 投标截止时间：2026年08月24日10时00分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆石柱水利水电实业开发有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市石柱土家族自治县都督大道11号 地 址：重庆市两江新区嘉华路36号重庆水务大厦1018 联 系 人：王老师 联 系 人：颜老师 道 电 话：13658292968 电 话：023-67901915 重庆水务电子商务平台咨询电话：管023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3074720.html cqdingjiu 2026.08.21 10:06:59 国 中</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N56" t="n">
         <v>90</v>
       </c>
@@ -4195,7 +4415,11 @@
           <t>万盛城区老旧供水管网更新改造工程(甲供材料)答疑(一) 万盛城区老旧供水管网更新改造工程（甲供材料） 答疑（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程（甲供材料）答疑（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。 问题2：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 全是万盛的公司中的！业主、专家全是你们自己人吧？ 商 答：本项目招标文件严格按照《重庆市工程建设项目货物采购招标文件示范文本（2026年版）》编制，且本项目 评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题3：3PE管道部分壁厚是多少呢？ 道 答：本项目采购的3PE防腐钢管的管道部分壁厚须符合国标标准并达到设计要求。 招 标 人：重庆市万盛经济技术开发区城市管理局 管 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 国 信息来源:https://www.chinapipe.net/project/d3074712.html cqdingjiu 2026.08.21 10:06:59 中</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N57" t="n">
         <v>80</v>
       </c>
@@ -4262,7 +4486,11 @@
           <t>南岸区茶园片区乡镇老旧供水管网更新改造工程更正公告 南岸区茶园片区乡镇老旧供水管网更新改造工程更正公 告 发布日期： 2026年8月18日 网 首次公示日期： 2026年8月14日 更正日期： 2026年8月18日 采购人名称： 重庆市江南城市建设发展（集团）有限公司务 采购人地址： 重庆市南岸区米兰路51号电子信息标准化厂房2号楼 联系人： 赵老师 商 电话： 023-62820331 采购代理机构名称： 重庆多杰数字科技咨询服务有限公司 采购代理机构地址： 重庆市重庆市经开区重庆市经开区长生桥镇江峡路8号13-1幢1楼 道 经办人名称： 李佩奇、戴沛轩、李倩 联系电话： 023-67648437 本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展 更正事项： 水土保持监管测工作。 https://www.gec123.com/notices/detail/1665701682723590144 信息来源:https://www.c国hinapipe.net/project/d3074669.html cqdingjiu 2026.08.21 10:07:01 中</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N58" t="n">
         <v>80</v>
       </c>
@@ -4325,7 +4553,11 @@
           <t>中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部排水钢管询价采购公告 中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 排水钢管询价采购公告 询价编号：ZT1105-XJ-2026-561-1 尊敬的各潜在供应商: 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与中铁十一局集团有限公司宜涪高铁重庆段站 前3标项目经理ZT1105-XJ-2026-561-1，排水钢管材料的报价。 一、项目概况 务 中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治（县）。合同金额28.01亿元，合同工期73个月， 开工日期：2024年12月，竣工日期：2030年12月。主要工程：新方斗山隧道(10660m)、石板坡隧道(4148m)、城北 隧道(3228m)、刘家坪隧道(2077m);刘家店子1号大桥工程(224.096m)、刘家店子2号大桥(232.099m)、城北大 桥(330.241m)、冉家湾大桥(355.245m),采用移动模架和支商架法现浇施工，其中24米移动模架施工6孔；32米支架法 施工5孔，移动模架施工28孔;正线铺无砟道床43.808Km。 二、询价内容 道 本次计划对排水钢管、GG-01材料进行询价，询价内容如下： 询价物资一览表 管 序号 包件号 物资名称 规格型号 计量单位 数量 备注 1 GG-01 排水钢管 Φ200*6m 米 3000 Q235B，壁厚6mm 合计 3000 国 说明：1.表中数量为计划数量，实际采购过程中可能有所调整，最终结算按照实际采购数量结算。 2.收货地点：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 中 三、技术质量及报价要求 1. 此次排水钢管、GG-01各项技术性能：Q235B 碳素结构钢无缝钢管，符合 GB/T8163 标准。质量需满足甲方项 目部正常使用的要求，保证产品的质量合格，满足试验室检测所有要求，详见技术规格书。 2.报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、结算及付款方式 自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发票认证完成之日起第6个月，支付至本次结算 金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内，累计支付总额不超结算总金额的75%，剩 余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理末次结算后第二年，支付金额应大于等于 尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总额的15%；办理末次结算后第四年，全部 付清）。 五、报价人资格要求 1.营业范围要求：在中华人民共和国境内依法注册、符合项目经营范围，具有询价物资生产或供应经验 的生产商或代理商，并且具有合法有效的营业执照。 2.生产能力要求：生产商须具备询价物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定。代 理商需出具制造厂出具签字盖章的授权函。 3.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8 月至今）国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；需满足排水钢管的相关所 有要求。 4.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年12月至今）企业或企业法定代表人有人民法院生效判决、裁 定认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接 受通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合 作方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 5.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★6.下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、报价人需要提供的资料 1.营业执照复印件、法人身份证复印件、开户许可证、授商权委托书、报价表和报价人资格要求中所需的证明资料， 所有资料需加盖公司鲜章。 2.生产厂家资质，产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、询价报名截止时间 管 有意参加本次询价采购的报价人须在铁建云链平台（https://www.crccep.cn）完成供应商注册，并于2026年8月18 日9时00分至2026年8月21日9时00分在网上完成报名工作。 八、询价截止时间 国 凡有意参加本次询价采购的报价人，请于 2026年8月21日14时00分 前提交报价。截止时间前未完成报价文件传 输的，视为放弃报价。 供应商报价必须严格按照《报价表》格式进行报价。 中 九、联系方式 采购组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村71号 采购人名称：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 地址：重庆市石柱土家族自治县金彰工业园区C区中铁十一局项目部 联系人：罗先生 联系电话：18580400001（提供采购服务支持） 中铁十一局集团有限公司 物资设备集中采购管理中心第五分中心 2026年8月18日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3074654.html cqdingjiu 2026.08.21 10:07:01 网 务 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>排水钢管 Φ200*6m：3000米</t>
+        </is>
+      </c>
       <c r="N59" t="n">
         <v>90</v>
       </c>
@@ -4388,7 +4620,11 @@
           <t>中铁建设集团(重庆)建设有限公司重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热 交换机组采购竞价补遗公告二 各 投标单位 ： 根据参加报名的潜在投标单位数量不满足招标方充分竞价要求的情况，此次重庆协同创新区供冷供热能源站及 配套系统工程冷却塔、分集水器、水板式热交换机组采购竞价资格预审报名截止日期将延期至 8月19日（周三） 上午9:00。 特此说明。 网 中铁建设集团（重庆）建设有限公司 2026年8月17日 务 信息来源:https://www.chinapipe.net/project/d3074650.html cqdingjiu 2026.08.21 10:07:01 商 道 管 国 中</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N60" t="n">
         <v>80</v>
       </c>
@@ -4455,7 +4691,11 @@
           <t>城口县东安及河鱼片区污水管网建设项目(一期)招标计划表 重庆市工程建设项目招标计划表 项 名 目 称城口县东安及河鱼片区污水管网建设项目（一期） 招标 法人 或招 标人城口县生态环境局 名称 （盖 网 章） 项目 批准 文件 及文 号 主 建 内 要 设 容 在 污 城 水 口 处 县 理 东 站 安 1座 镇 ， 等 改 片 建 区 后 新 设 建 计 污 规 水 模 管 20 网 0m 29 3 . / 0 d 0 。 km，其中新建dn110污水管5.80km，dn160污水管2.75km，dn200污水管0.57km，DN300污水干管4.36km，D 务 N400污水干管8.12km，DN200压力管7.4km,以及建设配套泵站2座,化粪池56座，隔油池32座。改扩建 序号 招标项目名称 招标内容 招标方式 招标文件计划发布时间 拟交易场所 合同预估金额(万元) 备注 招 项 标 目1 城 建 口 设 县 项 东 目 安 （ 及 一 河 期 鱼 ） 片区污水管网 工程施工 公开招标 2026-09 城 易 口 中 县 心 公共资源交 3400.00 本 暂 为 计 定 准 划 ， 。 表 最 所 终 列 以 招 实 标 际 项 招 目 标 信 时 息 的 均 信 为 息 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3074602.html 商 cqdingjiu 2026.08.21 10:07:01 道 管 国 中</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>dn110污水管：5.80km；dn160污水管：2.75km；dn200污水管：0.57km；DN200压力管：7.4km；泵站：2座</t>
+        </is>
+      </c>
       <c r="N61" t="n">
         <v>90</v>
       </c>
@@ -4518,7 +4758,11 @@
           <t>阀门产业园(管网改造)项目招标公告 阀门产业园（管网改造）项目招标公告 1.招标条件 本招标项目 阀门产业园（管网改造）项目已由垫江县发展和改革委员会以垫江发改委发【2022】459 号（批文 名称及编号）批准建设，项目业主为 垫江县丹香建设有限公司，建设资金来自 自筹资金 （资金来源）， 项目出资比例为 100% ，招标人为 垫江县丹香建设有限公司。项目已具备招标条件，现对该项目的施工进 行公开招标，评标办法采用经评审的最低投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 重庆市垫江县高新区县城组团 2.2 项目概况与建设规模： 场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路 务 长4000米，包括道路、综合管网等基础配套设施等。 2.3 本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元 商 2.4 招标范围： 包括土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等。具体详见施工图和 工程量清单。 道 2.5 工期要求：建设工期180日历天 缺陷责任期要求：24个月 管 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 国 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 中 4.1.1 本次招标要求投标人具备的资质条件： 具备建设行政主管部门颁发的有效的市政公用工程施工总承包叁 级及以上资质 ； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标 不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易监督网、重庆市公共资源交易网 （垫江县）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易监督网、 重庆市公共资源交易网（垫江县）完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资 源交易监督网、重庆市公共资源交易网（垫江县）导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 4.2投标人可在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）本项目招标公告网页下方“我要 提问”栏提出疑问，提问时间从本公告发布至2026-08-24 09:00:00前。 4.3招标人应于2026-08-24 23:59:59前在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-18 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 垫江县丹香建设有限公司 代理机构: 重庆博钰大数据科技有限公司 地 址: 地 址: 重庆市垫江县桂溪街道南内街88号 网 邮 编: 邮 编: 项目负责人: 熊老师 项目负责人: 郭威 电 话: 023-74630098 电 话: 023-74692498 务 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 商 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 道 2026年08月18日 信息来源:https://www.chinapipe.net/project/d3074578.html cqdingjiu 2026.08.21 10:07:02 管 国 中</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
       <c r="N62" t="n">
         <v>90</v>
       </c>

</xml_diff>

<commit_message>
Publish Chongqing and Sichuan tenders
</commit_message>
<xml_diff>
--- a/site/matches-positive.xlsx
+++ b/site/matches-positive.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,7 +496,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>璧山项目钢筋混凝土管询价公告</t>
+          <t>中建四局(四川)建设有限公司总部重庆交通大学双福校区三期建设项目(图情中心组团)工程总承包(EPC)项目雨水管网工程采购公告</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -527,27 +527,27 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>璧山区</t>
+          <t>江津区</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。</t>
+          <t>包括雨水检查井、钢筋砼承插式雨水管道铺设、中粗砂回填等内容</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>项目总投资44亿元，其中建安费28.6亿元，含市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>钢筋混凝土管及管件</t>
+          <t>雨水管网工程</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>璧山项目钢筋混凝土管询价公告 本项目位于璧山区，建设范围为双龙大道以北，璧铜线以东、渝蓉高速以南、玉泉湖（璧南河）以西区域，用 地面积约6平方公里。项目建设遵循循序渐进、分期、分块实施原则，采用“总体开发、分步实施”的方式进行 建设开发，合作期限8年，包含建设期和运营期（缺陷责任期），其中建设期6年，共分三期实施。第一期实施玉 泉湖以西，第二期实施璧南河以西，第三期实施渝蓉高速下道口。项目总投资44亿元，其中建安费28.6亿元，含 市政道路26公里，公共服务设施7.4万方，绿化及广场99万方，河道治理11.9公里。项目开发建设内容包括片区范 围内的基础设施、人才教育基地、水系生态整治、绿化及广场、公共交通场等。本次采购的内容为本项目一期 实施的市政道路所需的钢筋混凝土管及管件，预计供货时间为2026年8月至2027年4月。 网 登录地 mhem&amp;cNh6e0&amp;ce2C2m3s1e71=a64so0d9FAe=0903%e08005206E%6772dm6=%82he29&amp;=cI8p9eeyAs%7t?E%5lB%1iB%a1DetE%c9eweNAi%1iotvB%n/9cE%7.cBe9%ccAiE%p.E%s9%/29址/A%2:：psE%7tAhtD%B8%E%6B%7B%7E%5%78D9%E%5C9%F%9E%7AE%A%1E%9%78%78E%8B%4AD%N&amp;8E%6m657optUa3%6=6290%e3ni51B%5917E%443d6=E%862B%I8eAc%A1iD&amp;88no%tE%4BA%A%4E%7AC%AC%E%4BA%C8%E%8%88AA%E%5A8%A%1E%5B%7A%5E%7A%8B8%E%5B%1%08E%6C9%%98E%9%99%09E%5%58AC%E%5F%8B%8E%8A%5BF%E%9%38A%8EF%BC%%88E%5B9%BD%E%9%99%58EF%BC%%98E%6%59B%0E%5AD%%79E%7BB%F%8E%6B%5E8%E%4BA%A%7E%4B%8A9%E%5B9%AD%E%5C8%BA%E%9%58D8%E%5A%5%79E%9A%1B%9E%7B9%AE%EF%BC%%88E%8A%5BF%E%7%98%78E%5C8%BA%EF%BC%%98E%9A%1B%9E%7B9%AE%E%7=BgB&amp;upC%a=sod&amp;euF%pN=8Flk&amp;cmsusheaE%c7=te%0a9m%6he=8tT&amp;cpS7eeyeE%s9sha%&amp;3c2845d5=pur5A6I&amp;8optUni 信息来源:https://www.chinapipe.net/project/d3077008.html 务 cqdingjiu 2026.08.21 10:06:40 商 道 管 国 中</t>
+          <t>中建四局(四川)建设有限公司总部重庆交通大学双福校区三期建设项目(图情中心组团)工程总承包(EPC)项目雨 水管网工程采购公告 一、采购概况 1.采购名称：【重庆交通大学双福校区三期建设项目（图情中心组团）工程总承包（EPC）项目雨水管网工程】。 2.工程概况：【1.项目概况：本项目规划用地82876.94㎡，总建筑面积约108691.83㎡，其中9#行政楼建筑层 数6F/-2F，建筑高度为31.5m，10#图书馆建筑层数8F/-2F，建筑高度为57.1m，11#研究生楼建筑层数6F/-1F，建筑 高度为31.5m，12#地下车库建筑层数-2F，建筑高度为-8.7m。2.结构类型：所有楼栋主要结构形式为框架结构3.工 网 程地点: 重庆市江津区福星大道1号】。 3.标段划分：【本工程仅一个标段】。 4.采购内容：【重庆交通大学双福校区三期建设项目（图情中心组团务）工程总承包（EPC）项目雨水管网工程， 包括雨水检查井、钢筋砼承插式雨水管道铺设、中粗砂回填等内容，详见工程量清单】。 5.质量要求：【（1）质量标准：（1）工程施工的质量要求：工程质量应符合强制性质量标准，符合国家和重庆 市现行有关施工质量验收规范要求，并达到合格标准。商 （2）质量创优目标：/ 】。 6.工期要求：【暂定开工日期：2026年9月15日，竣工日期：2027年10月30日，总工期410日历天】。 道 7.文明要求：【（1）安全控制目标：杜绝发生重伤及以上生产安全责任事故，安全轻伤事故率小于1‰；不发生 社会影响较大的其他事故或险肇事件。 （2）安全生产、文明施工达到《管建筑施工安全检查标准（JGJ59-2011）》合格要求。 （3）杜绝机械设备事故、火灾事故和公共安全事故、防止职业病发生；贯彻落实《职业病防治法》、《职业健 康监护技术规范》等国家法律法规要求，关爱员工健康，不发生职业健康损誉事件。 国 （4）创优目标：市级建筑施工安全文明工地】。 8.付款条件：【 中 （1）月进度付款，按照甲方累计确认的已完合格工程量工程价款的【75】%，挂账后于60天内支付应付进度款； （2）乙方完成承包范围内全部工作内容并经甲方经验收合格，挂账后于60天内付款至已完成合格工程量工程价 款的【80】%。 （3）乙方完成承包范围内的全部工作内容并经验收合格及有关部门备案，且双方完成最终结算后，于60天内支 付至合格工程结算总价的【97】%，剩余【3】%作为工程质量保修金。养护期2年，扣除已发生的维护费用后， 甲方无息退还剩余保修金。 （4）本工程采用【银行转账、供应链（一年期以内）、票据（一年期以内）、以物抵债】方式向乙方支付货款。 如涉及贴息费用，贴息费由【甲】方承担。如由甲方承担贴息费，乙方须提供银行出具的贴息相关证明材料， 贴息费甲乙双方通过结算方式办理，乙方根据结算金额开具发票，贴息所产生的增值税税金由【乙方】承担， 甲方按合同中约定的工程进度款支付条件进行支付，贴息费不再产生逾期利息。】。 9.拟选定成交单位数：【1家】。 二、响应人资格 1.响应人报名前需通过“云筑网”（网址：https://jicai.yzw.cn/home）认证并进入中建系统合格分供商资源库，经 采购人资格审查合格后方可参与报价。 2.响应人须具备以下基本条件： （1）具有公司制独立法人主体资格，经营范围有效，时间有效（提供营业执照、法人身份证复印件、授权委托 书、被委托人身份证复印件等证明资料，在本公司本级资源库内分供商可不提供）； （2）办公场所、组织架构：具有固定的办公场所，公司组织架构合理，人员配置充足（提供企业简介、固定办 公地点影像资料、公司组织架构证明等证明资料，在本公司本级资源库内分供商可不提供）； （3）纳税人资格：提供纳税人证明或税务事项通知等证明资料（在本公司本级资源库内分供商可不提供）； （4）诚信经营：经核查政府平台近两年内无、质量事故通报，云筑网无不良记录，不得存在挂靠，必须为法人 直营单位（提供政府平台（中国裁判文书网、中国执行信息公开网、国家企业信用信息公示系统）查询记录截 图、法人直营承诺书等资料证明，在本公司本级资源库内分供商可不提供）； 网 （5）合法经营：遵守国家法律、依法经营、合约期间无违法犯罪记录、无因管理不善、履约不力导致的案件； （6）历史业绩：根据采购物提供对应业绩资料（提供相关合同关键页等资料证明，在本公司本级资源库内分供 商可不提供） 务 （7）资质：本工程无专业承包资质要求】。 3.响应资格审核不通过的情形： 商 1)在云筑网被本上级单位列为“不良行为分供商”或“禁用分供商”； 2)涉嫌围采串采的，如:法人身份证号重复、法人手机号重复、联系人重复、联系人手机号重复、IP地址重 复、MAC地址重复、邮箱地址重复、工商关联道的不同单位; 3)在严重失信或被执行企业名单； 4)分供商(法人)处于被限制高消费状态、司法拍卖影响企业正常运行、破产清算影响企业正常运营； 管 5)“换马甲”的中建股份、中建四局原禁用单位； 6）响应人未上传采购公告要求之资料，或上传资料不符合要求； 国 4.本次采购【不接受】联合体响应。 5.如响应单位提供虚假资料的，任何时候一经发现，取消其响应资格。 中 三、报名响应 1.响应时间：【以“云筑网”平台显示时间为准】，逾期不再接受响应。 2.响应方式：通过“云筑网”进行网上报名，不接受其他方式响应。 3.已在“云筑网”完成分供商注册的响应人，可直接在“云筑网”签收采购公告后响应。 4.响应担保：本次响应担保为【/】元，响应人应于报价截止日24小时前缴纳。 四、资格审查资料清单及格式 响应人报名时需按资格审查要求上传至云筑网，具体要求：按照顺序签字盖章扫描成一个PDF文件以附件形式上 传云筑网，统一命名为：响应报名文件-****单位，不得上传多个附件或压缩文件，不按要求上传资料的资格审 查不通过。 （一）资格审查资料清单（本级库内单位可不提供）： 1)《分供商准入资格预审表》（见附件1）； 2)法定代表人身份证明(见附件2)； 3)法定代表人授权书(见附件3)； 4)被委托人身份证明(见附件4)； 5)企业证明资料(见附件5)； 6)纳税证明或税务事项通知(见附件6)； 7)诚信经营证明(见附件7)； 8)现场拟派人员证书扫描件(见附件8)； 9)近3年施工类似业绩资料（见附件9）； 网 10)响应单位可提供的其他证明企业情况的资料。 五、发放采购文件 务 1.采购人通过“云筑网”对资格审查合格的响应人发放采购文件。 2.发放时间：【以“云筑网”平台显示时间为准 】。 商 3.联系人：【王青松】，联系方式：【18323827265】，联系地址：【四川省成都市双流区金为创新中心19楼】。 4.其他未尽事宜详见采购文件。 道 六、投诉通道 响应人如遇账款、合同、结算、廉洁、安全、环保、禁用等相关问题，可通过云筑网分供商投诉平台 （https://ts.yzw.cn/complaint）提交投诉材料，平台将按规定予以受理和处理。 管 采购人： 中国建筑第四工程局有限公司 国 信息来源:https://www.chinapipe.net/project/d3078437.html cqdingjiu 2026.08.24 12:31:34 中</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -560,14 +560,14 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>重庆, 四川, 管材, 招标, 商机</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告</t>
+          <t>五局三西南(重庆)鑫旭达项目室外管材及预制构件采购公告</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>房建</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -596,49 +596,45 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>忠县</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。</t>
+          <t>中建五局第三建设有限公司鑫旭达西南地区生产基地项目室外管材及预制构件采购</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>本项目工程总投资金额：约3140万元；本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。</t>
+          <t>本次采购估价：28万元</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>高标准农田建设工程</t>
+          <t>室外管材及预制构件</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(三标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程已由 忠县发展和改革委员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来自 业 主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具备招标条 件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 务 2.1 建设地点： 忠县花桥镇、新立镇、石宝镇、兴峰乡。 商 2.2 项目概况与建设规模①忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二标段）：田块整治 工程：旱地区域撂荒地整治278.95亩；灌溉与排水工程：新建200m蓄水池6座、PE75管道967m、新建1.2*1.2m箱 涵16m、新建2*2m箱涵8m；田间道路工程：新建2.5m混凝土生产路15114m、改建2.5m混凝土生产路1078m、新 建2.5m泥结碎石生产路910m、改建2.5m泥结碎道石生产路279m、新建3.0m混凝土生产路601m、改建3.5m混凝土机 耕路4587m；地力提升工程：施有机肥278.95亩；其他工程：工号牌124块。 管 ②忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）：田块整治工程：旱地区域撂荒地 整治195.54亩；灌溉与排水工程：新建100m蓄水池4座、新建200m蓄水池6座、PE75管道5258m、PE90管 道1375m、PE110管道2156m、改建0.5*0.6m混凝土排水沟740m、改建0.6*0.8m混凝土排水沟109m、改建0.8*1.0m混 凝土排水沟296m、改建1*1.5m混凝土排水沟262m、新建3*2m盖板涵1座；田间道路工程：新建2.5m混凝土生产 路11359m、改建2.5m混国凝土生产路3430m、新建2.5m泥结碎石生产路1834m、新建3.0m混凝土生产路350m；农田 防护工程：新建1.0m高挡土墙39m；地力提升工程：施有机肥195.54亩；其他工程：工号牌142块。 中 2.3 本项目工程总投资金额：约3140万元； 本次招标项目合同估算金额：二标段 1022万元；三标段 735 万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： 标段划分情况、建设规模及标段合同估算金额等内容如下： 合同估算金额 序号 项目名称 建设地点 （万元） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（二 1 花桥镇、新立镇 1022 标段） 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三 2 石宝镇、兴峰乡 735 标段） 网 本项目共分为2个标段，每家投标单位仅对2个标段中的任意1个标段进行投标，若同时参与2个及以上标段投标的， 其投标文件无效。 务 2.7 其他： / 商 3.政府采购工程 道 3.1 是否属于政府采购工程：是 □否 管 3.2 是否专门面向中小企业预留：是 国 专门面向中小企业预留的实施方式： 中 方式一：本项目整体面向中小企业。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字 证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责 任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要网提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-10-12 09:30，投标人应当在投标截止时间前，通过互 务 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 商 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 道 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 管 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 国 开户银行: 开户银行: 账 号: 账 号: 中 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（三标段） 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005499 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421353 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891814619 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082001038 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00385 信息来源:https://www.chinapipe.net/project/d3076880.html cqdingjiu 2026.08.21 10:06:45</t>
+          <t>五局三西南(重庆)鑫旭达项目室外管材及预制构件采购公告 中建五局第三建设有限公司重庆城市公司 五局三西南（重庆）鑫旭达项目室外管材及预制构件采购 五局三西南（重庆）鑫旭达西南地区生 产基地项目室外管材及预制构件采购公告 网 采购编号:cscecXXX 务 商 道 采购人：中建五局第三建设有限公司 采购日期： 2026 年 08 月 管 鑫旭达西南地区生产基地项目室外管材及预制构件采购公告 国 中建五局第三建设有限公司鑫旭达西南地区生产基地项目室外管材及检查井采购，现面向社会公开采购，诚邀 符合资格条件、能提供优质服务的国内专业公司参加采购合作事宜。 一、基本情况 中 1、采购组织单位：鑫旭达西南地区生产基地项目 2、本次采购内容：室外管材及预制构件 3、工程地点：重庆市涪陵高新区聚业大道北侧 4、合同履约期限：2026年08月-2027年12月 5、本次采购预估数量：管材4802米；预制构件247个 6、本次采购估价：28万元 7、本次采购报价方式：价税分离单价报价 8、计划进场日期：2026年08月28日 9、响应担保：0.28万元（采购完成后若无违规、不诚信操作可立即退还） 10、质量要求：必须符合相应国家标准，若行业标准或地方标准高于国家标准的，执行行业标准或地方标准。材 料尺寸、外管、环刚度、强度以及用料等均国家符合质量验收标准。 11、品牌要求：管材：顾地、中财、利财、联塑、伟星等同等级品牌。 二、付款方式： 1、支付方式：本合同采用【银行转账支票、网银转账、银行承兑汇票、银行保理、商业承兑汇票、国内信用证、 应收账款电子凭证及其他】常规支付方式的付款方式。 2、过程付款方式：甲方在次月的30日支付上月月度结算货款的【70】%，双方办理完毕最终结算后【60】个日 历天内付至总结算货款（且不超含税合同价款）的【97】%，预留质保金【3】%在保修期满且乙方已履行完所 有的保修责任后付清。甲乙双方协商一致同意本合同采用【银行转账支票、网银转账、银行承兑汇票、银行保 理、商业承兑汇票、国内信用证、应收账款电子凭证及其他】常规支付方式的付款方式，付款过程中产生的贴 息费用及手续费由【乙方】承担，每次付款前乙方应提供结算值【100%】的发票，否则甲方可拒绝付款。 网 三、报名条件： 1、报名参与单位必须是独立的法人单位，具备一般纳税人资格供方优先。报名参与单位在近2年内不曾在任何合 同中违约或因报名参与单位的原因而使任何合同被解除、未发生因自身原因造成的诉讼情况。报名参与单位应 务 具备较强的资源组织能力、供货能力、抗风险能力、售后服务能力和资金实力。响应方应随时接受采购方对响 应方设备性能、合格证、保险资料等进行检查。 2、未被列入失信被执行人、重大税收违法案件当事人名单、政府采购严重违法失信行为记录名单； 商 3、未处于被责令停业、响应资格被取消或者财产被接管、冻结和破产状态； 4、不在中建局及公司、分公司不合格名录/黑名单内； 道 5、单位负责人为同一人或者存在直接控股、管理关系的不同响应人，不得同时参加本工程响应； 6、符合《中华人民共和国采购法》、《政府采购法》等法律法规的要求； 管 7、响应单位报名阶段提供与采购标的物规格型号相符的以下证书，可认定为本次采购的绿色建材分供商：绿色 建材产品一星、二星、三星认证证书；中建绿色建材企业认证证书；绿色产品认证证书；中国环境保护标志证 书；中国节能标志证书；中国森林认证证书；入选工信部和省级绿色工厂，享受绿色建材分供商优惠条件。绿 色建材分供商需将认证证书以电子版或扫描件的形式与报名文件一同上传至云筑网。 国 四、响应报名 1、网络报名地点：响应人登录（http://www.yzw.cn），进入平台，填报企业相关资料，进行网络注册认证，通知 我司进行资审通过后，进行网上报名。 中 2、报名所需提交的资料包括： （1）营业执照，建筑业企业资质证书、安全生产标准化证书复印件(正副本均可)、法定代表人授权书证明原件。 （2）参与单位近两年的工作业绩（主要为所招地区业绩）。 （3）参与单位资信等级证书，质量、环境、职业健康安全管理体系认证书原件。 （4）参与单位可提供的其他证明企业情况的资料。 3、采购文件的获取：经资格审查入围的响应人，将对其发放电子版采购文件，登录中建采购网络交易采购平台 （http://www.yzw.cn），网上获取采购文件电子版，并依据文件要求于平台上响应截止日前进行网上响应。 4、严禁报名IP地址重复，IP地址重复者资审均不通过。 五、对本次采购提出询问，请按以下方式联系： 联系人：杨飞 联系电话：16623122372 中建五局第三建设有限公司 2026年08月20日 附件一： 法定代表人授权书 网 致：中建五局第三建设有限公司 务 本授权书声明：位于 （填公司地址） 的 （填公司名称） 的 （填法人 姓名）代表本公司授权 （填被授权人姓名）为本公司的唯一合法代理人，代表本公司参加中建五局第三建设 有限公司 XX项目XX采购采购活动，并在整个采购活动中，以本公司名义全权处理包括递交企业和产品响应资 质材料，确认响应相关信息，响应产品报价、议价，交纳商相关费用，签订采购合同，执行和完成采购周期内的 售后服务等一切与之有关的事务，并保证所提供的资质证明材料真实、合法、完整、有效。 道 本授权书于： 年 月 日签字生效，特此声明。 授权期限为： 年 月 日起至合同终止。授权期限内无特殊情况不变更合法代理人（被授权 人）。 管 法定代表人(签字) 被授权人(签字) 国 授权单位名称（盖章） 联系电话 中 授权人身份证正面 授权人身份证背面 被授权人身份证正面 被授权人身份证背面 点击查看内容 信息来源:https://www.chinapipe.net/project/d3078389.html cqdingjiu 2026.08.24 12:31:34</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>管道：967m；管道：5258m；管道：2156m</t>
+          <t>管材4802米；预制构件247个</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>重庆, 高标准农田建设工程, 资金情况, 产品种类</t>
+          <t>重庆, 管材, 预制构件, 采购</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(一标段)招标公告</t>
+          <t>中建桥梁有限公司西部(重庆)科学城德感片区污水管网修复完善工程项目(白沙部分新增)市政工程采购公告</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -648,7 +644,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>水利</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -667,49 +663,45 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>忠县</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>田块整治工程、灌溉与排水工程、田间道路工程、地力提升工程、其他工程</t>
+          <t>西部（重庆）科学城德感片区污水管网修复完善工程项目所需（白沙部分新增）市政工程专业分包工程，包括非开挖紫外光修复、安装前道内部勘测、清淤、封堵气囊、导排水，钢内衬成环回顶，铺设防划垫膜，主物料的拉入、连接充气设备、安装排水软管、物料的充气/紫外光固化、冷却物料、切除管口扎头多余务、抽出内膜、CCTV检测验收、拆除堵通水修复，管道铺设、管件、检查井、完成建筑垃圾清理，路面恢复等主要工序和辅助工序。</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>项目总投资金额约3140万元，本次招标项目合同估算金额一标段1167万元</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>高标准农田建设工程</t>
+          <t>市政工程专业分包工程</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程(一标段)招标公告 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）招标公告 1.招标条件 本招标项目忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）已由 忠县发展和改革委 员会 以 忠发改审批〔2026］753号批准建设，项目业主为 忠县畅达建设投资有限公司 ，建设资金来 自 业主自筹资金，项目出资比例为 100% ，招标人为 忠县畅达建设投资有限公司 。项目已具 备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 网 务 2.项目概况与招标范围 商 2.1 建设地点： 忠县马灌镇、三汇镇、永丰镇。 道 2.2 项目概况与建设规模：忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）：田块整治 工程：水田整治50.67亩、水田区域撂荒地整治79亩、旱地区域撂荒地整治62.83亩；灌溉与排水工程：新 建200m蓄水池5座、新建500m蓄水池1座、泵站1座；田间道路工程：新建2.5m混凝土生产路12325m、改 建2.5m混凝土生产路8549m、新建2.5m泥结碎石生产路1223m、新建3.0m混凝土生产路576m、改建3.0m混凝土生 管 产路648m、改建3.0m混凝土生产路（拆除原1.5m宽路）266m、改建3.5m混凝土机耕路1662m；地力提升工程：施 有机肥136.48亩；其他工程：公示牌1座、工号牌213块。 国 2.3 本项目工程总投资金额：约3140万元； 中 本次招标项目合同估算金额：一标段1167万元。 2.4 招标范围：以忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段）施工图所示范围的所 有内容为准，详见发布的施工图，工程量清单，招标文件及其补充文件。 2.5 工期要求：工期要求：90日历天 ，缺陷责任期为 24个月。 2.6 标段划分： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 网 方式一：本项目整体面向中小企业。 务 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 商 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质或水利水电工程施工总承包三级及以上资质或公路工程施工总承包三级及以上资质； 道 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 管 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 国 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 中 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（忠县）下载招标文件、工 程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及CA数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 5.2投标人可在重庆市公共资源交易网（忠县）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从 本公告发布至2026-08-24 12:00:00前。 5.3招标人应于2026-08-25 18:00:00前在重庆市公共资源交易网（忠县）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-10 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（忠县）发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 忠县畅达建设投资有限公司 代理机构: 重庆市忠资项目管理有限公司 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 谭超 项目负责人: 张钰枝 电 话: 023-54216300 电 话: 18002358213 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 网 监督部门: 忠县发展和改革委员会 电 话: 023-54456078 务 2026年08月20日 忠县2026年花桥镇大柏村等7个乡镇16个村高标准农田建设工程（一标段） 商 户名 开户行 投标保证金账号 忠县公共资源综合交易中心 重庆农村商业银行股份有限公司忠县支行 3501010120010008082000104 忠县公共资源综合交易中心 中国农业银行股份有限公司重庆忠县支行营业部 314501010400145900000005469 道 忠县公共资源综合交易中心 中国工商银行股份有限公司忠县支行 9558853100005421379 忠县公共资源综合交易中心 中国银行股份有限公司重庆忠县支行 111669494227VA00387 忠县公共资源综合交易中心 中国邮政储蓄银行股份有限公司忠县支行 95000601001203891884496 管 信息来源:https://www.chinapipe.net/project/d3076876.html cqdingjiu 2026.08.21 10:06:46 国 中</t>
+          <t>中建桥梁有限公司西部(重庆)科学城德感片区污水管网修复完善工程项目(白沙部分新增)市政工程采购公告 为满足中建桥梁有限公司对中建桥梁有限公司西部（重庆）科学城德感片区污水管网修复完善工程项目生产需 求，现就西部（重庆）科学城德感片区污水管网修复完善工程项目所需（白沙部分新增）市政工程专业分包工 程进行采购，诚邀符合资格要求、能提供优质服务的供应商参与报名。 一、工程概况 1、采购主体：中建桥梁有限公司 网 2、工程地址：重庆市江津区 3、采购内容：非开挖紫外光修复、安装前道内部勘测、清淤、封堵气囊、导排水，钢内衬成环回顶，铺设防划 垫膜，主物料的拉入、连接充气设备、安装排水软管、物料的充气/紫外光固化、冷却物料、切除管口扎头多余 务 废料，抽出内膜、CCTV检测验收、拆除堵通水修复，管道铺设、管件、检查井、完成建筑垃圾清理，路面恢复 等一切所需要的主要工序和上述未明示但实际完成承包项目内容所需的辅助工序所包括的全部工作内容。 二、报名单位资格要求 商 1、具有中华人民共和国企业独立法人资格，持有工商行政管理部门核发并通过最近年检的法人营业执照。代理 人须得到报名单位的授权。 2、资质要求：具备有效的资质证书、安全生道产许可证及相关认证证书，须具备市政公用工程施工总承包资质叁 级及以上资质或具有相关资质成建制单位；具备法律主体资格，具有独立订立及履行合同的能力，可开具增值 税专用发票。 3、业绩要求：在国内有关部门和行业的监督检查中没有不良记录；与中建桥梁有限公司及下属各单位没有不良 管 合作记录； 4、人员、设备、资金、服务、信誉等方面具有相应的能力。 5、成交分供商同意使国用云筑网（http://www.yzw.cn）筑易签电子签章功能完成采购合同签订；鼓励无纸化办公， 推荐分供商使用云筑网电子公章功能完成采购报名和报价工作。 6、存在以下情形的，原则上不得参与本次采购： 中 （1）严重违法失信企业； （2）失信被执行企业； （3）经营异常企业； （4）采购主体本上级单位禁用分供商的“换马甲”企业。 三、报名 1、报名方式 已在云筑网（http://www.yzw.cn）上注册的供应商，并经中建股份本下级任意单位认证“专业分包类”的分供商， 登录后即可报名。 2、报名时间。 公告发布时间： 2026 年8 月20 日（北京时间）。 报名截止时间为： 2026 年 8 月 24日 09 时 00 分（北京时间），具体以云筑网公示时间为准。 3、采购文件的获取 经资格审查入围的报名单位，登录云筑网下载采购文件，并依据采购文件要求于采购文件响应截止日前在云筑 网上递交响应文件。 4、报名及采购文件响应阶段 IP 地址相同的分供商直接淘汰。报名阶段存在信息重叠、工商关联（同一高管或 董监高，或股权关联（四层及以下））的分供商最多允许一家通过资格审查；报价阶段存在信息重叠、工商关联 （同一高管或董监高，或股权关联（四层及以下））的分供商直接淘汰。 5、报名附件格式参照公告附件要求，内容包括： （1）《分包商资质审查表》； 网 （2） 三证合一的营业执照； （3） 资质证书 务 （4） 安全生产许可证 （5） 法定代表人身份证明，授权委托书，授权委托人身份证复印件（正反面）； （6） 其他证明企业情况的资料（如企业荣誉及相关证书商，业绩等，办公场所、生产车间、仓储照片等）； 上述资料（1）至（5）项为必须项，第（6）项为选择项，报名单位可根据公司实际情况选择填写第6（项），所 有报名资料按照以上顺序盖章后扫描成一个 PDF 版电子文件，报名时将 PDF 版电子文件上传至云筑网。 道 四、保证金 报名成功并通过资审的分供商，在签收采购文件前缴纳1万元的采购响应保证金，报名单位可通过云筑网线上缴 纳保证金或购买保证保险（二选一），保证金在采购成交结果公示后30个工作日内退还，保险不予退还。 管 保证金缴纳操作如有问题，请报名单位联系云筑网客服，联系电话：4006-818-555。 若发生下列情况之一，采购人不予退还响应人所缴纳的保证金： 国 （1）响应人在响应截止日至采购人发布成交通知之日期间撤销其响应文件的； （2）提供虚假的材料谋取成交的； 中 （3）成交分供商收到成交通知后在规定的期限内未按采购文件要求签订采购合同的； （4）违反廉政承诺内容的； （5）采购期间发生其它违法、违规行为的。 五、联系方式 联系人：张继涛 电话：13919184919 联系人：游镇华 电话：13212385162 信息来源:https://www.chinapipe.net/project/d3078567.html cqdingjiu 2026.08.24 12:31:34</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>泵站：1座</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>重庆, 高标准农田建设工程, 投资金额, 产品种类</t>
+          <t>重庆, 市政工程, 污水管网修复</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>永川区农村供水管网巩固提升改造工程(东部片区)答疑补遗文件</t>
+          <t>重庆高速巨能建设集团有限公司城开高速城开隧道泄水洞施工项目第一批物资(排水材料)进行优选采购公告</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -719,7 +711,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>交通</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -738,49 +730,45 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>永川区</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>农村供水管网巩固提升改造工程</t>
+          <t>本项目涉及采购钢带增强聚乙烯螺旋波纹管和钢带波纹管密封胶圈，用于重庆高速巨能建设集团有限公司城开高速城开隧道泄水洞施工项目。</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>供水管网</t>
+          <t>[object Object],[object Object]</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>永川区农村供水管网巩固提升改造工程(东部片区)答疑补遗文件 永川区农村供水管网巩固提升改造工程（东部片区） 补遗文件（01） 各潜在投标人： 现将“永川区农村供水管网巩固提升改造工程（东部片区）”招标文件补遗通知如下，本次发布的补遗文件中 的所有内容与招标文件具有同等法律效力，如与招标文件、答疑补遗文件（01）网不一致时，以本补遗文件为准。 请各潜在投标人自行下载本补遗文件，不管下载与否，都视为全部知晓其全部内容。 一、本招标项目招标文件第二章投标人须知前附表第1.4.1项第1条第（3）款中“具备建设行政主管部门颁发的有 效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由建设行政主管部门颁发的有效的安全生产 务 考核合格证书。”修改为： “（3）具备建设行政主管部门颁发的有效的安全生产许可证，企业主要负责人、拟派项目经理具备相应的由水 行政主管部门颁发的有效的安全生产考核合格证书”。 商 二、本招标项目招标文件第二章投标人须知前附表第1.4.1项中第3条“业绩要求”修改为： “投标人自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成过1个单项合同 输配水管网长度不少于100km的水利工程施工道业绩。 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 管 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 三、本招标项目招标文国件第二章投标人须知前附表第1.4.1项中第5条中的“5.3项目经理业绩要求”修改为： “投标人拟派的项目经理自2023年1月1日起至投标截止日止（以合同工程完工日期或工程竣工日期为准），完成 过1个单项合同输配水管网长度不少于100km的水利工程施工业绩，并在该业绩中担任项目经理。 中 提供：供该业绩的合同协议书和合同工程完工证书（或合同工程验收鉴定书或工程竣工证书副本或竣工验收鉴 定书）的证明材料。若提供的上述业绩证明材料不能体现上述业绩指标的，应补充提供业主证明。 注：（1）当上述业绩证明材料中针对同一指标存在不一致时，以合同工程完工证书（或合同工程验收鉴定书或 工程竣工证书副本或竣工验收鉴定书）的证明材料为准。（2）投标人提供的业绩为联合体业绩的，其在该业绩 中的工作分工应与本项目承担的工作一致。” 四、本招标项目的投标文件递交的截止时间（投标截止时间）调整为2026年9月4日9时30分（北京时间），开标 时间及投标保证金递交截止时间相应顺延。 招标人：重庆市永川区惠永水务有限公司 招标代理机构：重庆永川政鑫综合能源有限公司 2026年8月20日 信息来源:https://www.chinapipe.net/project/d3076870.html cqdingjiu 2026.08.21 10:06:46</t>
+          <t>重庆高速巨能建设集团有限公司城开高速城开隧道泄水洞施工项目第一批物资(排水材料)进行优选采购公告 供应商应当在投标截止时间前，通过注册供应商账号在重庆高速集团物资采购平台 （http://113.250.85.222:8099/merchants/login）上进行报价并将投标文件扫描上传至该平台。 根据《国有企业采购操作规范》、《重庆高速巨能建设集团有限公司采购管理办法》等有关规定，重庆高速巨 能建设集团有限公司城开高速城开隧道泄水洞施工项目第一批物资（排水材料）进行优选采购，现将本次优选 有关事项公告如下： 一、优选项目名称：重庆高速巨能建设集团有限公司城开高速城开隧道泄水洞施网工项目第一批物资（排水材料） 采购项目 二、项目编号：GSJNCK-XSD-WZ-2026-0001 务 三、中选人数： （一）1名 （二）2名 □（供货比例第一名按 / %、第二名 / %） 商 （三）3名 □（供货比例第一名按 / %、第二名 / %、第三名 / %） 四、采购方式：公开优选 道 仅限于重庆高速集团物资采购平台：http://113.250.85.222:8099/merchants/login?redirect=%2F 五、优选范围表 管 序号 材料名称 规格型号 单位 暂定采购量 交货地点 备注 1 钢带增强聚乙烯螺旋波纹管 DN1200(PE)承插式 米 1884 重庆市开州区满月镇 国 2 钢带波纹管密封胶圈 DN1200 个 314 重庆市开州区满月镇 总合计 2198 六、竞选报价 中 （一）竞选报价为物资运送到采购人指定地点的不含税到场价，包括但不限于 材料费、人工费、仓储费、各项 税费、装车费、运输费、下车费、利润等所有一切其他费用。 （二）二次竞选：无。 七、竞选人资格 （一）竞选人必须是在中华人民共和国境内依法注册，具有独立法人资格，具有优选标的物经营范围的生产商 或销售商。 （二）本次优选不接受联合体参选，单位负责人为同一人或者存在控股、管理关系的不同单位，不得同时参加 竞选，否则，相关竞选均被否决。 （三）竞选人必须为巨能集团集采平台内的合格供应商（状态为：可投标，信息维护更新后的缴费年度显示 为2026年），否则视为未参与竞选，（高速集团内部单位除外），供应商注册网 址：http://222.178.219.165:7001/merchants/login。 （四）竞选人已按优选文件要求已缴纳竞选保证金（若有），否则，相关竞选将被否决。 （五）竞选人在国家企业信用信息公示系统中未被列入严重违法失信企业名单，同时必须为三年内与重庆高速 巨能建设集团有限公司无诉讼纠纷的公司，否则，相关竞选将被否决。 八、质量要求 （一）质量技术要求： 1、钢带增强聚乙烯螺旋波纹管：DN1200(PE)承插式，《埋地排水用钢带增强聚乙烯(PE)螺旋波纹管》CJ/T 225-2011。 （二）合同履行过程中中选供应商所供货物被采购人、监理、业主及行业监管部门抽检不合格的，采购人有权 单方面解除合同，并将中选供应商清退出场，所产生的一切损失由中选供应商承担，给采购人造成经济损失费 用采购人可在货款中直接扣除作为经济损失补偿，同时采购人保留诉讼的权利。同时将其列入集团供应商黑名 单，永久不得在集团范围内参与采购竞选。 网 九、付款方式 （一）预付款:无。 务 （二）付款方式：电汇、银行承兑或供应链金融产品（不超过12个月），具体情况根据采购人实际情况确定，中 选供应商不得以任何理由拒绝，若中选供应商接收银行承兑、供应链经融产品后需进行提前兑付时，贴息费用 由中选供应商自行承担； 商 （三）供货周期：以采购人需求时间为准； （四）结算、支付方式：材料进场验收合格后中选供应商与采购方双方每月10日办理结算，中选供应商每 月15-20日前向采购方提供当月结算金额等额的道增值税专用发票，采购方进行线上挂票，达到付款条件后，采购 方60日内支付结算货款的95%，剩余5%货款作为质量保证金，质量保证金在合同履约完成后3个月内无息支付。 （五）在合同履行期间，若因国家税务政策调整导致的税率变更，双方签订补充协议进行变更，合同不含税总 价不变。 管 （六）清单量为暂定数量，最终结算数量以双方共同验收并签字确认的结算验收单为准。 十、优选限价 国 暂定采购 优选限价（不含 序号 材料名称 规格型号 单位 量 税） 单价 总中价（元） （元） 1 钢带增强聚乙烯螺旋波纹管 DN1200(PE)承插式 米 1884 1060.00 1997040.00 2 钢带波纹管密封胶圈 DN1200 个 314 80.00 25120.00 总合计 2198 2022160.00 本次优选采用清单价+总价双限价原则，即竞选人无论清单报价超限价或竞选总价超限价，采购人均作无效竞选 处理 十一、优选文件的获取 由竞选人在重庆高速集团物资采购平台：http://113.250.85.222:8099/merchants/login?redirect=%2F下载优选文件电子 版。 十二、竞选截止时间和地点 （一）电子版竞选文件递交 竞选人须在竞选截止时间 2026年8月27日9时30分前，通过重庆高速集团物资采购平台（网 址：http://113.250.85.222:8099/merchants/login?redirect=%2F）将签章完善的竞选文件扫描件（多页合并成套PDF格 式）进行上传；为方便工作人员统计报价，竞选人须同时上传一份与《竞选报价书》数据一致的Excel电子版报 价清单；竞选人必须在投标页面“投标报价”处填写竞选不含税报价；未上传竞选文件（多页合并成套 PDF 格 式），平台自动拒收，开选现场也不接收。 （二）纸质版竞选文件递交 竞选人须在竞选截止时间2026年8月27日9时30分前将签章完善且装订成册的 贰 份纸质版竞选文件通过现场递 交或邮寄方式提交采购人指定地点（以收到时间为准），逾期拒收。 现场递交地址：重庆市两江新区宝圣东路291号重庆高速巨能建设集团有限公司老办公楼202会议室。 邮寄地址：重庆市两江新区宝圣东路291号重庆高速巨能建设集团有限公司202室； 收件人：王女士，联系电话：15730141615 网 竞选文件须集中装入一个密封袋内，封口处粘贴封条，并在封条的封口处加盖竞选人单位公章（鲜章），“竞 选文件”封袋上写明如下内容： 优选项目名称：重庆高速巨能建设集团有限公司城开高速城开隧道泄水洞施工项目第一批物资（排水材料）采 务 购项目 竞选人名称： 公司 在2026年8月27日9时30分前不得开启（需加盖竞选人单位商公章鲜章）。 （三）竞选人如电子版竞选文件或纸质版竞选文件（缺一项）未提交，则视为未参与竞选。 十三、开选时间及地点 道 本次优选将于2026年8月27日9时30分在重庆市两江新区宝圣东路291号重庆高速巨能建设集团有限公司老办公 楼202会议室开选。 管 十四、竞选保证金：无 重庆高速巨能建设集团有限公司中环分公司 2026年8月19日 国 信息来源:https://www.chinapipe.net/project/d3078467.html cqdingjiu 2026.08.24 12:31:36 中</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>输配水管网：100km</t>
+          <t>排水材料</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>重庆, 农村供水管网, 巩固提升改造, 东部片区, 管材招标</t>
+          <t>重庆, 管材, 招标, 排水材料</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部刺丝滚笼、塑钢模板、泄水管询价采购公告</t>
+          <t>国网重庆电力渝西片区2026年原集体企业和各级产业单位第十四次物资区域联合授权公开谈判采购采购公告</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -790,7 +778,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -809,29 +797,25 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>万州区</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>渝万高铁站前1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~D1K47+550.4，正线长度33.01km，中标造价31.73亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁301孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负责DK0+000~DK57+136段小型构件预制。</t>
+          <t>采购项目名称为物资，具体采购内容包括第十四次物资区域联合授权公开谈判采购。</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>中标造价31.73亿元</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>刺丝滚笼,塑钢模板,泄水管</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部刺丝滚笼、塑钢模板、泄水管询价采购公告 中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 刺丝滚笼、塑钢模板、泄水管询价采购公告 询价编号： ZT1105-XJ-2026-590 尊敬的 各潜 在供应商 : 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与 中铁十一局集团有限公司重庆至万州高铁站 前 1标项目经理部 ZT1105-XJ-2026-590， 刺丝滚笼、塑钢模板、泄水管 的报价。 一、 项目概况 务 渝万高铁站前 1标位于重庆市万州区和忠县境内,起止里程DK14+233.2~ D1K47+550.4，正线长度 33.01km，中标造 价 31.73 亿元。管区内共有隧道8座/22.36km，斜井2座/1.76km;桥梁15座/8.97km，其中，预制及架设梁 301 孔，(40+64+40)m和(45+100+45)m连续梁各1联;区间路基22段/1.68km，土石方约67万方，负 责DK0+000~DK57+136段小型构件预制。合同工期54.7月商，开工日期为2022年11月01日，竣工日期为2027 年04 月30日。 二、 询价内容 道 本次 计划对刺丝滚笼、塑钢模板、泄水管 进行询价，询价内容如下： 询价物资一览表 管 计 序 物资 量 包件号 规格型号 数量 备注 号 名称 单 位 国 刺丝 1 GL-01 2.5mm 6m0.5m 米 6500 半径 ≥225mm，包括刀片刺绳、挂丝、连接卡、支架 滚笼 防护 中 栅栏 2 GL-01 用立 50X30X765X2.5mm 套 500 含抱箍、螺栓等配件 柱支 架 平 塑钢 3 MB-01 350X300mm 方 19.2 400*400,1个挡水沿，配固定手柄 模板 米 平 塑钢 4 MB-01 350X300mm 方 19.2 400*400,2个挡水沿，配固定手柄 模板 米 平 塑钢 5 MB-01 300X300mm 方 75.6 2个挡水沿，配固定手柄 模板 米 平 塑钢 6 MB-01 300X300mm 方 75.6 1个挡水沿，配固定手柄 模板 米 7 SSG-01 管篦 PVC250X200x10mm 个 220 材质硬聚氯乙烯 PVC，详见附图 PVC 8 SSG-01 泄水 135X38mm 块 220 材质硬聚氯乙烯 PVC，详见附图 管盖 U型 9 SSG-01 125mm 个 900 详见附图 管卡 UPV 材质硬聚氯乙烯 PVC，两端接头采用阴阳螺纹连接详见 10 SSG-01 C排 125X8mm螺纹 米 2870 附图 水管 UPV 11 SSG-01 C弯 DN125X8mm90° 个 240 材质硬聚氯乙烯 PVC，详见附图 管 UPV 网 125X125X110mm弹性密 12 SSG-01 C三 个 120 材质硬聚氯乙烯 PVC，详见附图 封圈异径斜三通 通 无压 埋地 务 排污 排水 用硬 13 SSG-01 DN125 个 150 材质硬聚氯乙烯 PVC，详见附图 聚氯 商 乙烯 管 T 型接 头 道 合 计 管 说明： 1. 表中数量为计划数量，实际 采购 过程中可能有所调整，最终结算按照实际 采购 数量结算。 2.收货地点：中铁十一局集团有限公司重庆至万州高铁站前1标项目经理部 三、 技术质量 及报价国 要求 1. 此次 询价物资 各项技术性能要 符合 甲方 的要求，质量满足甲方项目部正常使用的要求，保证 产品 的质量合 格。 具体要求或图纸见询价文件技术规格书。 。 中 2 .报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、 结算及付款方式 每个月 15 日为双方价款结算日期（即上月 16 日至当月 15 日内），结算前双方要在对帐确认单上签字认可，乙 方按双方确认的金额开具增值税专用发票，并自发票开具之日起 7日内传递给甲方。甲乙双方在增值税专用发票 传递过程中必须留取相应的交接签证手续。自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发 票认证完成之日起第6个月，支付至本次结算金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内， 累计支付总额不超结算总金额的75%，剩余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理 末次结算后第二年，支付金额应大于等于尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总 额的15%；办理末次结算后第四年，全部付清）。 五、 报价 人资格要求 1.营业范围要求：在中华人民共和国境内依法注册，具有询价物资生产或供应经验的生产商或代理商，并且具有 合法有效的营业执照。 2.生产能力要求： 生产商须具备 询价 物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定 。 代理商需出具制造厂出具签字盖章的授权函。 3.财务能力要求：报价人为增值税一般纳税人或小规模纳税人，有依法纳税的良好记录。 4.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8月至今） 国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；每种物资全指标技术参数性能满足 国家和行业最新标准的各项规定。 5.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年8月至今）企业或企业法定代表人有人民法院生效判决、裁定 认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接受 通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合作 方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 6.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★7 .下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、 报价人需要提供的资料 1. 营业执照复印件、 法人身份证复印件、 开户许可证、商授权委托书 、 报价表 和报价人资格要求中所需的证明资 料， 所有资料需加盖公司鲜章。 2. 产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、 询价 报名截止 时间 管 有意参加本次询价采购的报价人 须在铁建云链平台 （ https:// www.crccep. cn） 完成供应商注册，并 于 202 6 年 8 月 20 日 9时 00 分 至 202 6 年 8 月 24 日 9时 00 分在网上 完成报名工作。 八、 询价 截止 时间 国 凡有意参加本次询价采购的报价人，请于 202 6 年 8 月 24 日 14 时 00分 前 提交报价。截止时间前未完成 报价 文 件传输的，视为放弃 报价 。 供应商报价必须严格按照《 报价表 》格式进行报价。 中 九、 联系方式 采购 组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村 71号 联系人：胡先生 联系电话： 13983336494 （提供平台服务支持） 采购人名称：中铁十一局集团有限公司重庆至万州高铁站前 1标项目经理部 地址： 重庆市万州区双河口街道檬兴路万州现代综合物流中心信息交易大厅（中铁十一局） 联系人： 唐大伟 联系电话： 18323391938（提供采购服务支持、保证金退还） 中铁十一局集团有限公司物资设备集中采购管理中心 第五分中心 2026 年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076805.html cqdingjiu 2026.08.21 10:06:47 网 务 商 道 管 国 中</t>
+          <t>国网重庆电力渝西片区2026年原集体企业和各级产业单位第十四次物资区域联合授权公开谈判采购采购公告 采购项目编 采购项目状态 正在采购 CY2026S5W4E 号 国网重庆电力渝西片区2026年原集体企业 采购项目名称 和各级产业单位第十四次物资区域联合授 采购类型 物资 权公开谈判采购 采购文件获取截止时 开启应答文 2026-08-25 09:00:00 2026-09-01 09:00:00 间 件时间 网 供应商提出澄清问题 截止时间 国网重庆市电力公司永川供电 开启应答文件地点 ETP 采购人 务分公司 招标代理机 重庆市渝北区青枫北路20号凤 招标代理机构 重庆展泽工程咨询有限公司 构地址 凰D座9楼部分办公用 招标代理机构邮编 401120 商联系人 供应商服务大厅 联系电话 400-1047-177 传真 电子邮箱 JZD_WZ@163.com 信息来源:https://www.chinapipe.net/project/d3078339.html 道 cqdingjiu 2026.08.24 12:31:36 管 国 中</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -840,18 +824,18 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>重庆, 万州, 高铁站前, 刺丝滚笼, 塑钢模板, 泄水管, 询价采购</t>
+          <t>重庆, 物资, 采购</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告</t>
+          <t>国网重庆电力主城一片区2026年原集体企业和各级产业单位第十四次物资区域联合授权公开谈判采购采购公告</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -861,7 +845,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>水利</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -880,49 +864,45 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>垫江县</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目，主要内容包括河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m，化粪池2座；产业基地水肥一体化改造45亩等。</t>
+          <t>采购项目名称为'国网重庆电力主城一片区2026年原集体企业和各级产业单位第十四次物资区域联合授权公开谈判采购'，采购类型为物资。</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>项目总投资金额为642.89万元，本次招标项目合同估算金额约为5014864.52元。</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>水利水电工程施工</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目招标公告 1.招标条件 本招标项目 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 已由 垫江县发展和 改革委员会 以 垫江发改委发〔2026〕20号 文批准建设，项目业主为 垫江县太平镇人民政府，建设资金来 自 大中型后扶资金及自筹资金 ，项目出资比例为 100% ，招标人为垫江县太平镇人民政府。项目已具备招 标条件，现对本项目施工进行公开招标，评标办法采用经评审的最低投标价法。网 务 2.项目概况与招标范围 商 2.1 建设地点：垫江县太平镇桂花村 道 2.2 项目概况与建设规模：主要为河堤护岸岸线整治2100m；产业路扩宽及油化改造775.3m；新建污水管网450m， 化粪池2座；产业基地水肥一体化改造45亩等。 管 2.3 本项目工程总投资金额：642.89万元 国 本次招标项目合同估算金额：约5014864.52元 中 2.4 招标范围：本工程施工图纸所含全部的施工内容，具体以招标人发布的工程量清单为准。 2.5 工期要求：工期为360日历天 ，缺陷责任期为24个月。 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：□是 否，因专门面向中小企业预留无法确保充分供应、充分竞争，根据 《政府采购促进中小企业发展管理办法》第六条第(三)“按本办法规定预留采购份额无法确保充分供应、充分竞 争，或者存在可能影响政府采购目标实现的情形”的规定，本项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 网 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的水利水电工程施工总承包三级 务 及以上资质。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相商应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 道 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 管 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com国/dianjiangweb/)、重庆市公共资源交易监督网下载招标文件、工程量清单、电子图纸等资 料。参与投标的投标人需在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共 资源交易监督网完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督网导航栏“主体信息”页面中“市场主体信息 登记”、“中CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流 程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交易监督 网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-24 17:00:00前。 5.3招标人应于2026-08-28 17:00:00前在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重 庆市公共资源交易监督网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易网(垫江县) (https://www.cqggzy.com/dianjiangweb/)、重庆市公共资源交 易监督网发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 垫江县太平镇人民政府 代理机构: 重庆皓辰建设工程咨询有限公司 重庆市渝北区金开大道1228号大雅金开国际1 地 址: 重庆市垫江县太平镇牡丹路191号 地 址: 栋9-2 邮 编: 邮 编: 项目负责人: 余老师 项目负责人: 雷雨得 电 话: 13996889839 电 话: 023-86018770 18580880860 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 网 2026年08月19日 垫江县2026年度大中型水库移民后期扶持项目—太平镇美丽移民村建设项目 务 户名 开户行 投标保证金账号 垫江县公共资源交易中心 中国农业银行重庆垫江支行 316301010400077950000005966 垫江县公共资源交易中心 中国银行重庆垫江支行 111616885778VA00139 商 垫江县公共资源交易中心 重庆农村商业银行垫江支行 2501010120010009065000128 垫江县公共资源交易中心 工商银行重庆垫江支行营业部 9558853100016843371 垫江县公共资源交易中心 重庆银行垫江支行 820101040000584-101195 道 附件：垫江县2026年度大中型水库移民后期扶持项目-.zip https://www.cqggzy.com/trade/014001/dac54522-3264-4eac-ae47-f434567ce374?categoryNum=014001001007 信息来源:https://www.chinapipe.net管/project/d3076788.html cqdingjiu 2026.08.21 10:06:47 国 中</t>
+          <t>国网重庆电力主城一片区2026年原集体企业和各级产业单位第十四次物资区域联合授权公开谈判采购采购公告 采购项目编 采购项目状态 正在采购 CY2026S1W4E 号 国网重庆电力主城一片区2026年原集体企 采购项目名称 业和各级产业单位第十四次物资区域联合 采购类型 物资 授权公开谈判采购 采购文件获取截止时 开启应答文 2026-08-25 09:00:00 2026-09-01 09:00:00 间 件时间 网 供应商提出澄清问题 截止时间 国网重庆市电力公司市区供电 开启应答文件地点 详见采购公告 采购人 务分公司 招标代理机 重庆市渝北区青枫北路20号凤 招标代理机构 重庆展泽工程咨询有限公司 构地址 凰D座9楼部分办公用 招标代理机构邮编 401120 商联系人 供应商服务大厅 联系电话 400-1047-177 传真 电子邮箱 JZD_WZ@163.com 信息来源:https://www.chinapipe.net/project/d3078338.html 道 cqdingjiu 2026.08.24 12:31:36 管 国 中</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>污水管网：450m</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 水利, 移民, 后期扶持</t>
+          <t>重庆, 物资, 采购公告</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>万州区新田等6个镇乡农村饮水质量提升项目招标计划表</t>
+          <t>忠县忠州和白公街道特色农业节水灌溉保障工程勘察设计招标计划表</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -932,7 +912,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>其他/未识别</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -953,32 +933,32 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>万州区</t>
+          <t>忠县</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>新建水厂1座（新建2000m³茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管径DN20~DN250，管材为涂塑钢管。</t>
+          <t>本工程为9720亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站21座，整治山坪塘44口，建设主要建设水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤墒情系统。</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>合同预估金额：5000万元</t>
+          <t>合同预估金额为137.18万元</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>涂塑钢管</t>
+          <t>节水灌溉设备、智能监控系统、气象监测设备、虫情监测设备、土壤墒情监测设备</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>万州区新田等6个镇乡农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区新田等6个镇乡农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建水厂1座（新建2000m3茨竹水厂），输、配水管道改造与新建，管道总长约226.127km，管 主要建设内容 径DN20~DN250，管材为涂塑钢管。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 备注 称 式 发布时间 所 额(万元) 商 万州区新田 万州区新田 重庆市万 招标项目 等6个镇乡农 等6个镇乡农 公开招 州区公共 1 村饮水质量提 2026-08 5000.00 村饮水质量 标 资源交易 升项目道施工总 提升项目 中心 承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076721.html 管 cqdingjiu 2026.08.21 10:06:48 国 中</t>
+          <t>忠县忠州和白公街道特色农业节水灌溉保障工程勘察设计招标计划表 重庆市工程建设项目招标计划表 项目名称 忠县忠州和白公街道特色农业节水灌溉保障工程勘察设计 招标法人 或招标人 忠县水库运行管理中心 网 名称（盖 章） 项目批准 文件及文 忠发改审批〔2026〕794号 务 号 本工程为9720亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站21座，整治山坪塘44口，建设 主要建设 水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤 内容 墒情系统。 商 招标项目 招标方 招标文件计 拟交易 合同预估 序号 招标内容 备注 名称 式 划发布时间 场所 金额(万元) 本工程为9720道亩柑橘 等特色农业提供抗旱 忠县忠州 供水，新建节水灌溉 本计划表所 和白公街 提灌站21座，整治山 忠县公 列招标项目 招标项目 道特色农 坪塘44口，建设水肥 公开招 共资源 信息均为暂 管 1 业节水灌 2026-08 137.18 一体化系统，完善田 标 综合交 定，最终以 溉保障工 间引水渠堰、排水沟 易中心 实际招标时 程勘察设 及管网，分片区安装 的信息为准 计 智能监控、气象、虫 国 情、土壤墒情系统。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3078219.html 中 cqdingjiu 2026.08.24 12:31:36</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>管道：226.127km</t>
+          <t>抗旱供水；新建节水灌溉提灌站21座；整治山坪塘44口；建设水肥一体化系统；完善田间引水渠堰、排水沟及管网；安装智能监控、气象、虫情、土壤墒情系统</t>
         </is>
       </c>
       <c r="N8" t="n">
@@ -986,14 +966,14 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 商机</t>
+          <t>重庆, 节水灌溉, 柑橘, 抗旱供水, 提灌站, 山坪塘, 水肥一体化, 智能监控, 气象, 虫情, 土壤墒情</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>万州区大周等4个镇乡街道农村饮水质量提升项目招标计划表</t>
+          <t>忠县新生街道特色农业节水灌溉保障工程勘察设计招标计划表</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1024,32 +1004,32 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>万州区</t>
+          <t>忠县</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>新建50m³蓄水池4口、取水池2座；新建50m³/d-100m³/d水厂2座；改造100m³/d-300m³/d水厂5座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设施。</t>
+          <t>本工程为9720亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站21座，整治山坪塘44口，建设主要建设水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤墒情系统。</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>合同预估金额：3000万元</t>
+          <t>合同预估金额为137.18万元</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>DN25-DN250涂塑钢管</t>
+          <t>节水灌溉设备、水肥一体化系统、智能监控系统、气象监测设备、虫情监测设备、土壤墒情监测设备</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>万州区大周等4个镇乡街道农村饮水质量提升项目招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区大周等4个镇乡街道农村饮水质量提升项目 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 及文号 务 新建50m3蓄水池4口、取水池2座；新建50m3/d-100m3/d水厂2座；改造100m3/d-300m3/d水厂5 主要建设内容 座；铺设DN25-DN250涂塑钢管约86km；新建提水泵站8座；配套阀井、电磁流量计等有关设 施。 招标项目名 招标方 招标文件计划 拟交易场 合同预估金 序号 招标内容 商 备注 称 式 发布时间 所 额(万元) 万州区大周 万州区大周 重庆市万 招标项目 等4个镇乡街 等4个镇乡街 公开招 州区公共 1 道农村饮水 道农村饮道水质 2026-08 3000.00 标 资源交易 质量提升项 量提升项目施 中心 目 工总承包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3076720.html cqdingjiu 2026.08.21 10:06:49 国 中</t>
+          <t>忠县新生街道特色农业节水灌溉保障工程勘察设计招标计划表 重庆市工程建设项目招标计划表 项目名称 忠县新生街道特色农业节水灌溉保障工程勘察设计 招标法人 或招标人 忠县水库运行管理中心 网 名称（盖 章） 项目批准 文件及文 忠发改审批〔2026〕794号 务 号 本工程为9720亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站21座，整治山坪塘44口，建设 主要建设 水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤 内容 墒情系统。 商 招标项目 招标方 招标文件计 拟交易 合同预估 序号 招标内容 备注 名称 式 划发布时间 场所 金额(万元) 本工程为9720亩道柑橘等 特色农业提供抗旱供 忠县新生 水，新建节水灌溉提 本计划表所 街道特色 灌站21座，整治山坪 忠县公 列招标项目 招标项目 农业节水 塘44口，建设水肥一 公开招 共资源 信息均为暂 管 1 2026-08 137.18 灌溉保障 体化系统，完善田间 标 综合交 定，最终以 工程勘察 引水渠堰、排水沟及 易中心 实际招标时 设计 管网，分片区安装智 的信息为准 能监控、气象、虫情、 国 土壤墒情系统。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3078218.html 中 cqdingjiu 2026.08.24 12:31:37</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>涂塑钢管：86km；提水泵站：8座</t>
+          <t>抗旱供水；新建节水灌溉提灌站21座；整治山坪塘44口；建设水肥一体化系统；完善田间引水渠堰、排水沟及管网；分片区安装智能监控、气象、虫情、土壤墒情系统</t>
         </is>
       </c>
       <c r="N9" t="n">
@@ -1057,14 +1037,14 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>重庆, 农村饮水质量提升项目, 管材招标, 合同预估金额</t>
+          <t>重庆, 节水灌溉, 柑橘, 抗旱供水, 提灌站, 山坪塘, 水肥一体化, 智能监控</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>二航科工新燕尾山项目纤维编绕拉挤电缆保护套管采购询价通知公告</t>
+          <t>忠县洋渡、任家镇等乡镇特色农业节水灌溉保障工程勘察设计招标计划表</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1074,7 +1054,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1093,45 +1073,49 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>忠县</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。</t>
+          <t>本工程为1.7万亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站18座，整治山坪塘28口，建设水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤墒情系统。</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>采购项目资金为企业自筹。</t>
+          <t>合同预估金额为138.71万元</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>纤维编绕拉挤电缆保护套管(BWFRP100/2.0，79158米)</t>
+          <t>节水灌溉设备、智能监控系统、气象监测设备、虫情监测设备、土壤墒情监测设备</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>二航科工新燕尾山项目纤维编绕拉挤电缆保护套管采购询价通知公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目询比采购 公告 中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程项目已具备采 购条件，现公开邀请供应商参加询比采购活动。 网 1. 采购项目简介 1.1 采购项目名称：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机 电工程项目。 务 1.2采购方案编号：FA00000674478。 1.3 采购人：中交二航局科工（武汉）有限公司西南片区新燕尾山隧道工程施工二标段项目道路照明机电工程 项目经理部。 商 1.4 采购代理机构：中交二航局科工（武汉）有限公司。 1.5 采购项目资金：企业自筹。 道 1.6 采购项目概况：新燕尾山隧道工程位于重庆市内环吉庆隧道北侧，四横线分流道鹿角隧道南侧，西接白居 寺大桥，东接内环快速路，并向东延伸接渝黔复线高速，其所在的道路系统呈东西布置，为主城区南部片区重 要干道。本项目西起太阳岗立交(不含太阳岗立交)，往东穿越铜锣山，止于内环南泉立交(不含南泉立交)。项目 管 全长约6.8km，其中二标段长约3.62公里，采用主干路标准，设计车速60km/h，标准路幅为双向6车道，主要工程 包括长隧道1座(新燕尾山隧道，长2542m)，简易立交1座(花溪立交),互通式立交2座(南温泉立交、苦竹坝立交)。 2.采购范围及相关要求 国 2.1 采购范围：纤维编绕拉挤电缆保护套管（BWFRP100/2.0，79158米）。 2.2 交货期：以甲方实际订单要求为准。 中 2.3 交货地点：重庆市巴南区新燕尾山项目甲方指定位置。 2.4 物资质量标准：满足国家法律法规、标准、规范、设计参数及技术规格书要求。 3.供应商资格要求 3.1 供应商应依法设立且满足如下要求： （1）资质要求：在中华人民共和国境内依法注册，具有独立法人资格、具有采购物资生产或供应经验的企业， 并且具有合法、有效的“三证合一”的营业执照,代理商需提供制造商授权委托书。 （2）财务要求：必须是经税务部门注册登记核准的一般纳税人，有依法纳税的良好记录，提供近三年的财务报 告。 （3）业绩要求：同类产品销售业绩不少于2个，并具备与本招标项目需求相适应的供货能力。 （4）信誉要求：本项目投标截止期前未被“信用中国”、“中国政府采购网”、中国交建物资采购管理信息系 统网站列入失信被执行人、违法案件当事人、违法失信行为记录名单。 （5）其他要求：提供运输方案及生产周期。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他： / 。 4.供应商报名 4.1有意参加询比采购活动的单位，请于2026年 8 月 20 日 11 时 00 分至2026 网 年 8 月 25 日 11 时 00 分（北京时间、下同），登录“中交招采网”（网 址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 务 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 商 5. 供应商报价 5.1 报价结束（递交响应文件截止）时间：2026年 8 月 25 日 11 时 00 分。 道 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的 电子响应文件，采购人将拒收。 5.3电子采购的供应商报价文件由线上电子报价表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 管 子报价表的数据为准。 6. 开标 6.1开标时间：与报价结国束时间相同。 6.2开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标，现场开标地点/。 7. 发布公告的媒介 中 本询比采购公告在中交招采网上发布。 8. 评审办法 本项目评审办法采用 经评审的最低价法 。 9. 合同主要条款 9.1 付款条件：无预付款，到货后办理结算，双方办理完结算手续、卖方提供符合合同要求的正式发票给买方 后60天，买方支付该批材料价值80%的货款，完工结算后支付至97%，剩余3%为质保金，质保期2年，两年后供 应方申请返还3%（无息）；银行转账、承兑、18个月供应链金融混合支付方式。 9.2履约保证金的递交： （1）□不要求递交 （2）要求递交 保证金金额：2万元 ； 保证金形式：银行转账、银行保函等电子保函；其他形式：无 。 10. 成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”（网址：https://zjzcw.iccec.cn）发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联 系4006765885中标服务费请按7咨询。 10.1收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； 务 （3）在1000万元（含）至3000万元之间的，每次收取1000元； （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 10.2支付流程 （1）通知推送：中标结果发布后，系统自动道推送缴费通知（含应缴金额及支付链接）； （2）费用查询：供应商登录“中交招采网-服务管理”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网- 服务管理－发票下载”模块获取。 11.监督机构 国 监督机构名称：中交二航局科工（武汉）有限公司纪委监察部 举报电话：中027-82796466 举报邮箱：sneb_kggs@ccccltd.cn 12.其他 投标保证金采用银行转账形式的需转至中交二航局科工（武汉）有限公司账户（账 号：42001186108053006379-0006开户行：建行武汉长江支行，行号：105521000053），并备注二航科工燕尾山机 电照明项目纤维编绕管投标保证金。 13.联系方式 采购 人：中交二航局科工（武汉）有限公司 采购代理机构：中交二航局科工（武汉）有限公司 地 址：武汉市新洲区双柳街星谷大道158号地 址：武汉市新洲区双柳街星谷大道158号 邮政编码：430400 邮政编 码：430400 联系人：李鑫 联系人：毕明 月 电 话：18186145302 电 话：17853118573 电子邮件：18186145302@ccccltd.cn 电子邮件：bimingyue@ccccltd.cn 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3076715.html cqdingjiu 2026.08.21 10:06:50 网 务 商 道 管 国 中</t>
+          <t>忠县洋渡、任家镇等乡镇特色农业节水灌溉保障工程勘察设计招标计划表 重庆市工程建设项目招标计划表 项目名称 忠县洋渡、任家镇等乡镇特色农业节水灌溉保障工程勘察设计 招标法人 或招标人 忠县水库运行管理中心 网 名称（盖 章） 项目批准 文件及文 忠发改审批[2026]328号 务 号 本工程为1.7万亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站18座，整治山坪塘28口，建 主要建设 设水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土 内容 壤墒情系统。 商 招标项目名 招标 招标文件计 拟交易 合同预估 序号 招标内容 备注 称 方式 划发布时间 场所 金额(万元) 本工程为1.7道万亩柑橘 等特色农业提供抗旱 忠县洋渡、 供水，新建节水灌溉 本计划表所 任家镇等乡 提灌站18座，整治山 忠县公 列招标项目 招标项目 镇特色农业 坪塘28口，建设水肥 公开 共资源 信息均为暂 管 1 2026-08 138.71 节水灌溉保 一体化系统，完善田 招标 综合交 定，最终以 障工程勘察 间引水渠堰、排水沟 易中心 实际招标时 设计 及管网，分片区安装 的信息为准 智能监控、气象、虫 国 情、土壤墒情系统。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3078217.html 中 cqdingjiu 2026.08.24 12:31:37</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>排水钢管 Φ200*6m：3000米</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 光纤电缆保护套管</t>
+          <t>重庆, 节水灌溉, 柑橘, 抗旱供水, 提灌站, 山坪塘, 水肥一体化, 智能监控, 气象, 虫情, 土壤墒情</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告</t>
+          <t>荣昌区2026年古昌镇高标准农田建设项目招标公告</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1141,7 +1125,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1162,47 +1146,47 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>巴南区</t>
+          <t>荣昌区</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告</t>
+          <t>新建高标准农田797.11亩，改造提升高标准农田5710.6亩，其中高效节水灌溉面积3007亩。主要内容包括水田整治、缓坡整治、梯台整治、恢复地类整治、耕地复耕整治、农机进出通道修建、提灌站修建、输水管道铺设、排水沟改建、田间道路改建等。</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>项目总投资金额1592.15万元，本次招标项目合同估算金额1420.76万元，全部来自财政资金。</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>天然气表后管道安装工程</t>
+          <t>高标准农田建设相关材料及设备，如PE输水管道、排水沟、田间道路等。</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程变更公告 重庆巴南天然气有限责任公司 重庆国际生物城配套公寓项目天然气表后管道安装工程 变更公 告 公告编号： RQBGGG202608200006 本公司于2026年08月19日发布的重庆国际生物城配套公寓项目天然气表后管道安装工程公告（编 号：RQCGXY202608170010），现做出如下变更： 网 1、对采购文件第一卷“采购需求“中墙体管道暗埋的具体内容进行明确。墙体管道暗埋应包含墙体开槽，输送 用不锈钢波纹管及钢制槽板的安装，墙体恢复，暗埋管道视频记录。 2、对由响应供应商提供的钢制槽板的规格进行明确。钢制槽板为U型开口槽，采用热镀锌Q235B钢板，钢板厚度 务 不得小于1.2mm，尺寸不得小于U40*30*1.2（宽40mm,高30mm,壁厚1.2mm热镀锌） 3、对由响应供应商提供的F型不锈钢三通，材质可以选用黄铜进行替代。 4、采购文件第二卷“技术规范及要求“中增加T/CECS633-2019 《燃气用户工程不锈钢波纹软管技术规程》。 以上内容在合同中也同步进行调整。 商 除上述变更外，原公告其余内容仍有效。 道 重庆巴南天然气有限责任公司 管 2026-08-20 信息来源:https://www.chinapipe.net/project/d3076704.html cqdingjiu 2026.08.21 10:国06:50 中</t>
+          <t>荣昌区2026年古昌镇高标准农田建设项目招标公告 荣昌区2026年古昌镇高标准农田建设项目招标公告 1.招标条件 1. 招标条件 本招标项目荣昌区2026年古昌镇高标准农田建设项目已由重庆市荣昌区农业农村委员会以荣农发〔2026〕64号批 准建设，项目业主为重庆市荣昌区农田建设中心，建设资金来自财政资金，项目出资比例为100%，招标人为重 庆市荣昌区农田建设中心。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用经评审的最 网 低投标价法。 2.项目概况与招标范围 2. 项目概况与招标范围 务 2.1 建设地点： 古昌镇百合堂村、玉带村 2.2 项目概况与建设规模：新建高标准农田797.11亩，改造提升高标准农田5710.6亩，其中高效节水灌溉面积3007 商 亩。 2.3 本项目工程总投资金额：1592.15万元 本次招标项目合同估算金额：1420.76万元 道 2.4 招标范围：水田整治2622.50亩，缓坡整治21.95亩，梯台整治186.23亩，恢复地类整治44.26亩，耕地复耕整 治283.09亩，农机进出通道8338m；新修提灌站1座，改建提灌站2座，新修Φ250PE输水管道2732m、Φ200PE输水 管道267m、Φ160PE输水管道20928m、Φ110PE输水管道7412m，改建沟带路(1.8×0.8×1.0m)799m，维 管 修2.0×1.5m排水沟1395m、0.8×1.0m排水沟784m；改建3.0m宽田间道6573m、4.0m宽田间道728m。包括所提供的 施工设计图所示范围内的所有内容，具体以招标人提供的图纸、工程量清单、答疑资料、澄清资料、其他补遗 资料等相关内容为准。若施工图与工程量清单不一致时，以工程量清单为准。 2.5 工期要求：工期为1国80日历天 ，缺陷责任期为24个月。 2.6 标段划分（如有）： / 2.7 其他： 中/ 3.政府采购工程 3. 政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式：本项目整体面向中小企业。 4.投标人资格要求 4. 投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的建筑工程施工总承包三级及以 上资质或市政公用工程施工总承包三级及以上资质或水利水电工程施工总承包三级及以上资质 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（荣昌区）下载招标文件、 工程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网（荣昌区）完成市场主体信息登 记以及CA数字证书办理，办理方式请参见重庆市公共资源交易网（荣昌区）导航栏“主体信息”页面中“市场 主体信息登记”、“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法 完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网（荣昌区）本项目招标公告网页下方“我网要提问”栏提出疑问，提问时间 从本公告发布至2026-08-26 17:30:00前。 5.3招标人应于2026-08-28 18:00:00前在重庆市公共资源交易网（荣昌区）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-16 09:30，投标人应当在投标截止时间前，通过互 务 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 商 本次招标公告同时在重庆市公共资源交易网（荣昌区）、重庆市公共资源交易监督网发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆市荣昌区农田建设中心 代理机构: 重庆富毅项目管理有限公司 道 地 址: 地 址: 邮 编: 邮 编: 项目负责人: 李老师 项目负责人: 陈航 管 电 话: 023-85265043 电 话: 16623666557 传 真: 传 真: 电子邮箱: 电子邮箱: 国 开户银行: 开户银行: 账 号: 账 号: 监督部门:中重庆市荣昌区发展和改革委员会 电 话: 023-61471361 2026年08月21日 信息来源:https://www.chinapipe.net/project/d3078214.html cqdingjiu 2026.08.24 12:31:37</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>排水钢管 Φ200*6m：3000米</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>重庆, 天然气表后管道安装工程, 变更公告</t>
+          <t>高标准农田建设, PE输水管道, 排水沟, 田间道路</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>合川区中南片区污水管网工程(一期)招标计划表</t>
+          <t>重庆中法供水2026年金属补偿器及柔性橡胶接头采购项目(第三次)比选公告</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1231,49 +1215,45 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>合川区</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米，螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清淤2627米。</t>
+          <t>重庆中法供水2026年金属补偿器及柔性橡胶接头采购项目(第三次)比选公告</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>合同预估金额为1708.44万元</t>
+          <t>项目资金来自企业自筹，出资比例为100%</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>排水管道、检查井、紫外线修复设备、螺旋缠绕修复材料、树脂修复材料、不锈钢快速锁修复设备</t>
+          <t>柔性橡胶接头,金属补偿器</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>合川区中南片区污水管网工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 合川区中南片区污水管网工程（一期） 名称 招标 网 法人 或招 标人 重庆市合川区住房和城乡建设委员会 名称 （盖 务 章） 项目 批准 文件 合川发改投〔2025〕19 号 商 及文 号 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300-D800管道130米，新增检查井11座，新 主要 建D300排水管道38米；紫外光修复 D300-D道800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 建设 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米，不锈钢快速锁修复 D1000管道42 内容 米；完成 D300-D1000管道清障189米、清淤2627米。 拟 招 招标文 合同预 招标 管 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 国 重 庆 市 合川 合 招标 区中 主要建设内容包含多项管网修复及新建工程，具体为：原位开挖修复 D300- 川 项目 中 南片 D800管道130米，新增检查井11座，新建D300排水管道38米；紫外光修复 公 区 区污 D300-D800排水管道712米，紫外光内衬+钢套筒修复 D300-D800排水管道755米， 开 公 1 2026-09 1708.44 水管 螺旋缠绕修复 D1000-D1600管道73米，局部树脂修复 D300-D800排水管道125米， 招 共 网工程 不锈钢快速锁修复 D1000管道42米；完成 D300-D1000管道清障189米、清 标 资 （一 淤2627米。 源 期） 交 易 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076543.html cqdingjiu 2026.08.21 10:06:50</t>
+          <t>重庆中法供水2026年金属补偿器及柔性橡胶接头采购项目(第三次)比选公告 重庆中法供水2026年金属补偿器及柔性橡胶接头采购项目（第三次） 比选公告 1.比选条件 网 本比选项目重庆中法供水2026年金属补偿器及柔性橡胶接头采购项目（第三次），比选人为重庆中法供水有限公 司，比选项目资金来自企业自筹，出资比例为100%，项目已具备比选条件。现对本项目进行公开比选，诚邀有 兴趣的潜在投标人参与投标。 2.项目概况与比选范围 务 2.1 金属补偿器、柔性橡胶接头采购清单 商 序号 存货编码 材料名称 规格型号 单位 数量 最高单价限价（元） 1 10302603 柔性橡胶接头 DN40（PN10) 个 200 146 1 2 道 10302607 柔性橡胶接头 DN40（PN16) 个 10 146 22 3 10302601 柔性橡胶接头 DN50（PN10） 个 500 186 3 管 4 10302604 柔性橡胶接头 DN50（PN16） 个 10 186 4 5 10302602 柔性橡胶接头 DN80（PN10） 个 200 252 …… 国 6 10202125 柔性橡胶接头 DN80（PN16） 个 10 252 7 10202120 柔性橡胶接头 DN100（PN10） 个 10 300 8 1030中2605 柔性橡胶接头 DN100（PN16） 个 10 300 9 10202121 柔性橡胶接头 DN150（PN10） 个 10 500 10 10202123 柔性橡胶接头 DN150（PN16） 个 10 500 11 10202124 柔性橡胶接头 DN150（PN25) 个 10 660 12 10202122 柔性橡胶接头 DN200（PN10） 个 10 680 13 10302606 柔性橡胶接头 DN200（PN16） 个 10 720 14 10200481 柔性橡胶接头 DN300（PN16） 个 10 1400 15 10302155 金属补偿器 DN40 个 100 230 16 10302157 金属补偿器 DN40 (25KG) 个 10 240 17 10302156 金属补偿器 DN40（16kg） 个 10 230 18 10302140 金属补偿器 DN50 个 100 270 19 10302148 金属补偿器 DN50 （16kg） 个 10 270 20 10302151 金属补偿器 DN50(25KG) 个 10 300 21 10302141 金属补偿器 DN80 个 100 390 22 10302145 金属补偿器 DN80 (16KG) 个 10 390 23 10302146 金属补偿器 DN80 (25KG) 个 10 435 24 10302142 金属补偿器 DN100 个 10 455 25 10302147 金属补偿器 DN100 (16KG) 个 10 455 26 10302152 金属补偿器 DN100(25KG) 个 10 550 27 10302143 金属补偿器 DN150 个 10 630 28 10302149 金属补偿器 DN150 （16kg） 个 10 630 29 10302153 金属补偿器 DN150(25KG) 个 10 840 30 10302144 金属补偿器 DN200 个 10 900 网 31 10302150 金属补偿器 DN200 （16kg） 个 10 950 32 10302154 金属补偿器 DN200(25KG) 个 10 1250 2.2 供货数量、时间和批次：根据工程实际进度与比选人的要求进行务供货，以实际供货量为准，供货时间达到 商务条款的规定。 2.3 交货地点：比选人指定的施工现场。 商 2.4 供货期：两年。 3.投标人资格要求 道 3.1 本次比选允许投标人以投标货物的下列身份参加投标： ?制造商 管 ?代理商、经销商 3.1.1 投标人为制造商应符合以下要求： 投标人必须是依法设立国的，并在中国注册的，具有独立法人地位的企业。 【提供有效的营业执照】 3.1.2 投标人为代理商或经销商应符合以下要求： 中 若投标人为授权代理商或经销商，必须是依法设立的，并在中国注册的，具有独立法人地位的企业,同时应具备 投标产品的制造商对参加本项目投标的授权书。 【提供有效的营业执照、授权书】 注：① 一个制造商仅能委托一个代理商或经销商参加投标，否则均按否决投标处理。 ② 制造商及其授权的代理商或经销商不能同时参加本项目投标，否则均按否决投标处理。 3.2 投标人2025年的年度财务状况不亏损。若投标人为授权代理商或经销商，只能提供本单位的财务状况。 【提供由会计师事务所或审计机构出具的无保留意见的财务审计报告及会计报表，财务报表至少包括现金流量 表、资产负债表、利润表】 3.3 投标产品的制造商须通过质量ISO9001、环境ISO14001、职业健康体系ISO45001认证。 【提供有效的证书】 3.4 投标人须提供2023年1月1日至投标截止日止（以合同签订时间为准）,签订的30万元及以上的同类型产品购 销合同至少1个。 【提供采购合同、不低于前述金额50％的发票，合同与发票的项目名称须一致】 注：①若投标人开具的发票上未能体现具体项目，需附上税务出具的发票清单（清单上需显示采购项目为同类 型产品）。 ②若提供的合同为年度合同未体现具体金额，但实际供货金额达到30万元及以上，应提供与该合同对应的30万元 及以上的同类型产品发票作为佐证。 3.5 根据本次采购清单及技术规范的要求，投标人须承诺具备相关的技术手段和措施、保证产品设计使用寿 命10年以上。 3.6 投标产品的制造商须具备特种设备制造许可证（压力管道）。 网 【提供有效的证书】 3.7 投标人须承诺保证5年内不得停产同型号的投标产品。 务 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 3.8 投标产品须提供卫生疾控中心出具的卫生检测报告和质量监督机构出具的质量检验报告。 【提供有效的检验检测报告】 商 3.9 投标人承诺不得存在下列情形之一： 1）被人民法院列入失信被执行人名单且在被道执行期内； 2）被国家、重庆市（含市或任意区县）有关行政部门行政处罚，且在处罚期限内； 3）投标截止日前两年内（指2024年1月1日至投标截止日止），投标人或其法定代表人被人民法院判定犯行贿罪 管 的； 4）投标截止日前五年内（指2021年1月1日至投标截止日止），投标人与重庆中法供水有限公司有违约情况或终 止合同情况的。 国 【按照第六章 三、资格审查部分“承诺函格式”提供承诺函】 3.10 投标截止日前五年内（指2021年1月1日至投标截止日止），投标人无在我司因产品及服务等对公司生产、 经营、安全造成不良影响的记录；若投标人出现过供水通报事项，因产品质量问题对生产、安全造成影响，存 中 在合同违约等问题，不予参加本次项目投标。 【按照第六章 三、资格审查部分“无不良记录承诺函”提供承诺函，若经验证承诺函不属实，将对中标人作 否决投标处理。】 3.11 投标样品要求： 3.11.1 投标人需提供以下规格型号数量的样品： 【金属补偿器 DN40壹件】，提供的样品应满足第五章技术要求规定。样品为投标人免费提供，不计入采购清 单内。 3.11.2 投标样品同投标文件一并递交。每件样品上分别标明样品的投标人、生产厂家、品牌、名称、规格、型号等 （格式自拟），投标样品必须密封装箱，且在密封包装外贴样品一览表（格式自拟），注明提供样品的投标人、 生产厂家、品牌、名称、规格、型号、数量等。 3.11.3 投标人的样品在开标当日递交至样品区（样品区地点：开标当日咨询比选代理机构），中标人的投标样 品不退还，其余投标人的样品在中标公示期满后5个工作日内退还，如不领取，投标样品按废品处理。 3.11.4 上述对投标样品的密封和标识要求是为便于评标，请投标人积极配合，未按上述要求对投标样品进行密封 和标识的，不作否决投标处理，但由此造成的其他后果由投标人自行承担。 3.12 若投标人违反重庆中法供水有限公司《供应商负面清单管理办法》规定且在处罚期内的，按否决投标处理 （评标委员会根据比选公告后附“供应商负面清单”进行评审）。 3.13 本次比选不接受联合体投标。 特别说明： （1） 本比选文件要求提供的所有检测报告须为近2年内的检测报告（2024年1月1日-投标截止日），此要求不 包括卫生许可批件及其检测报告。 （2） 上述所须提交的相关证明材料复印件均应加盖投标单位法人章并装入投标文件资格审查部分中。上述有 一条不满足则投标文件由评标委员会作否决投标处理。 网 （3） 比选人有权对投标人提供的以上资料进行核实，若发现存在弄虚作假，取消其投标、中标资格，投标人 承担因此造成的相关责任并赔偿相应损失。 务 4.比选文件的获取 4.1 投标人于2026年08月21 日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子 版，以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，采购人和采购代理机构都 商 视为投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的 一切后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 道 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价（须同时递交投标文件）。在投 标截止时间前未按时报名、报价并管上传电子投标文件、递交纸质投标文件，投标文件被视为无效。 4.4 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)上传电子投标文件，电子投标文件应加盖投标人 的单位印章。 国 4.5 投标人在递交投标文件时向招标代理机构支付500 元/份标书费，否则将拒绝接收投标文件。 5.投标文件的递交 中 5.1电子版投标文件递交时间：2026年08月27日10时00分（北京时间）前，投标人自行上传至重庆水务集团电子商 务平台(https://www.cqswjt.cn)； 5.2纸质版投标文件递交时间：2026年08月27日09时30分至10时00分（北京时间），地点：重庆水务集团招标采购 中心（重庆市两江新区嘉华路36号重庆水务大厦五楼。导航：重庆水务大厦东门）。 5.3投标截止时间：2026年08月27 日10时00分（北京时间）。 5.4逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 比 选 人：重庆中法供水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝北区悦来镇悦来水厂 地 址：重庆市两江新区嘉华路36号重庆水务大厦 联 系 人：陈老师 联 系 人： 崔畅 电 话：023-67585971 电 话： 13896264537 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3078192.html cqdingjiu 2026.08.24 12:31:37 网 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>D800管道：130米；D300排水管道：38米；D800排水管道：755米；D1600管道：73米；D800排水管道：125米；D800排水管道：712米；D1000管道：42米；检查井：11座；管道：189米</t>
+          <t>DN40(PN10)个 200; DN40(PN16)个 10; DN50(PN10)个 500; DN50(PN16)个 10; DN80(PN10)个 200; DN80(PN16)个 10; DN100(PN10)个 10; DN100(PN16)个 10; DN150(PN10)个 10; DN150(PN16)个 10; DN150(PN25)个 10; DN200(PN10)个 10; DN200(PN16)个 10; DN300(PN16)个 10; DN40个 100; DN40(25KG)个 10; DN40(16kg)个 10; DN50个 100; DN50(16kg)个 10; DN50(25KG)个 10; DN80个 100; DN80(16KG)个 10; DN80(25KG)个 10; DN100个 10; DN100(16KG)个 10; DN100(25KG)个 10; DN150个 10; DN150(16kg)个 10; DN150(25KG)个 10; DN200个 10; DN200(16kg)个 10; DN200(25KG)个 10</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>重庆, 污水管网工程, 管网修复, 新建工程, 排水管道, 检查井, 紫外线修复, 螺旋缠绕修复, 树脂修复, 不锈钢快速锁修复</t>
+          <t>重庆, 金属补偿器, 柔性橡胶接头, 采购项目, 比选公告</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>重庆市自来水有限公司球墨铸铁管及管件2026-2027(2年)采购项目(第二次)答疑补遗文件</t>
+          <t>川渝高竹新区引调水工程项目招标计划表</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1283,7 +1263,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>其他/未识别</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1305,27 +1285,27 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>本次采购项目涉及球墨铸铁管及管件的供应，具体包括样品的规格和数量要求。</t>
+          <t>新建两岔水库取水浮船1座，设计取水规模为2万m/d；新建两岔水库取水浮船-坛高水厂原输水管道21km。</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>合同预估金额为508万元</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>球墨铸铁管及管件</t>
+          <t>取水浮船、输水管道</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>重庆市自来水有限公司球墨铸铁管及管件2026-2027(2年)采购项目(第二次)答疑补遗文件 重庆市自来水有限公司球墨铸铁管及管件2026-2027（2年）采购项目（第二次）答疑 提问1：样品20CM长含承口吗？如果含承口20CM那就太短，标识LOGO无法体现完整建议≥20CM 答1：球墨铸铁管样品含承口，样品长度≥20CM 网 务 招标人：重庆市自来水有限公司 招标代理机构：重庆水务集团公用工程咨询有限公司 商 2026年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d30道76446.html cqdingjiu 2026.08.21 10:06:50 管 国 中</t>
+          <t>川渝高竹新区引调水工程项目招标计划表 重庆市工程建设项目招标计划表 项目名称 川渝高竹新区引调水工程项目 招标法人或招 标人名称（盖 重庆北碚农业发展有限公司 网 章） 项目批准文件 及文号 务 新建两岔水库取水浮船1座，设计取水规模为2万m/d；新建两岔水库取水浮船-坛高水厂原输 主要建设内容 水管道21km。 招标项目 招标方 招标文件计划 拟交易场 合同预估金额 序号 招标内容 备注 名称 式 发布时间 所 (万元) 商 新建两岔水库取水浮 川渝高竹 船1座，设计取水规 重庆市北 招标项目 新区引调 模为2万m/d；新 公开招 碚区公共 1 2026-08 508.00 水工程项 建两岔水库道取水浮 标 资源综合 目 船-坛高水厂原输水 交易中心 管道21km。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3078130.html cqdingjiu 2026.08.24 12:31:38 国 中</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>排水钢管 Φ200*6m：3000米</t>
         </is>
       </c>
       <c r="N13" t="n">
@@ -1333,14 +1313,14 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>重庆, 球墨铸铁管, 管件, 采购项目</t>
+          <t>重庆, 川渝高竹新区, 引调水工程, 取水浮船, 输水管道</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>大足区中心城区和龙水镇市政公共排水设施运维(材料)更正一号公告</t>
+          <t>石阡县2026年第二批农村供水提质改造项目竞争性磋商公告</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1371,27 +1351,27 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>大足区</t>
+          <t>石阡县</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>大足区中心城区和龙水镇市政公共排水设施的运维(材料)。</t>
+          <t>农村供水提质改造项目</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>预算金额：1950000.00元，最高限价：1911000.00元</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>供水提质改造相关设备和材料</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>大足区中心城区和龙水镇市政公共排水设施运维(材料)更正一号公告 一、更正项 更正项 更正子项 更正前内容 更正后内容 网上投标 网上投标截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 递交投标响应文件 线下递交投标（响应）文件开始时间 2026-08-20 14:30:00 2026-08-25 14:30:00 递交投标响应文件 线下递交投标（响应）文件截止时间 2026-08-20 15:00:00 2026-08-25 15:00:00 网 开标 开标时间 2026-08-20 15:00:00 2026-08-25 15:00:00 招标采购（附件） 附件 务 二、补遗更正说明 清单限价重新做调整，开标时间已更正，详见更正文件内容 商 三、联系方式 采购执行方： 道 单位名称：重庆誉双项目管理有限公司 联系人：陈老师 联系电话：13996336872 采购需求方： 管 单位名称：重庆市大足区茂泰市政工程有限公司 联系人：谢老师 联系电话：18523539371 信息来源:https://www.chinapipe.net/project/d3076319.html 国 cqdingjiu 2026.08.21 10:06:50 中</t>
+          <t>石阡县2026年第二批农村供水提质改造项目竞争性磋商公告 竞争性磋商公告 项目概况 石阡县2026年第二批农村供水提质改造项目 项目的潜在供应商应在铜仁市大力城项目管理有限责任公司（铜 仁市碧江区时代天街1号楼16层16-7室）获取磋商文件，并于2026 年9月 1 日 14 点30分（北京时间）前递 交响应文件。 网 一、项目基本情况 项目编号： TRDLC-2026-022 务 项目名称：石阡县2026年第二批农村供水提质改造项目 采购方式： 竞争性磋商 预算金额： 1950000.00元 商 最高限价： 1911000.00元 采购需求：详见磋商文件 道 合同履行期限： 3个月（90日历天） 本项目（否）接受联合体投标。 管 二、申请人的资格要求： （一）满足《中华人民共和国政府采购法》第二十二条规定； 国 （二）落实政府采购政策需满足的资格要求（根据项目实际情况）： 按财库〔2014〕68号、财库〔2017〕141 号、财库〔2019〕9号、财库〔2020〕46号、财库〔2022〕19号等文件执行。 （三）本项目的特定资格要求：1.本项目是专门面向中小企业采购，若工程的承建企业是中小企业，请供应商按照 中 《政府采购促进中小企业发展管理办法》(财库〔2020〕46号）出具规定的《中小企业声明函》；2.其他特殊资格 要求：本次招标要求投标人须具备水利水电工程施工总承包叁级及以上及以上资质，具备有效的安全生产许可 证；并在人员、设备、资金等方面具有相应的施工能力，其中，投标人拟派项目负责人(项目经理)须具备 水利 水电 专业 贰 级注册建造师，具备有效的安全生产考核合格证书 (B证)，在投标截止日有在其他在 建建设工程(含已经获得中标通知书未开工)担任项目负责人(包括工程总承包中的施工负责人)的，不得以拟派项 目负责人(项目经理) 的身份参加本次投标。 三、获取磋商文件 （一）时间： 2026年 8 月 21 日 17:00 至 2026 年 8 月 28 日 17:00 （北京时间，法定节假 日除外） （二）地点：铜仁市碧江区时代天街1号楼16层16-7室 （三）方式：现场获取，报名时需提交的资料：营业执照复印件，法定代表人身份证明及身份证复印件、授权 委托书原件（法定代表人报名的无需提供此项资料）、被授权人身份证原件及复印件（法定代表人报名的无需 提供此项资料）、上述资料均需加盖单位公章。 网上邮件报名获取：营业执照复印件，法定代表人身份证明及身份证复印件、授权委托书原件（法定代表人报 名的无需提供此项资料）、被授权人身份证原件及复印件（法定代表人报名的无需提供此项资料）、上述资料 均加盖单位公章后将扫描件发送到QQ邮箱1094532301@QQ.com后领取。注：发送后请及时联系18385937396。 注：被授权人需提供本单位2026年任意一个月缴纳社保证明。 （四）售价：人民币300元/套 四、提交响应文件截止时间、开标时间和地点 （一）时间： 2026 年 9 月 1 日 14 点 30 分（北京时间） （二）开标地点：石阡县水务局7楼会议室 五、公告期限 自本公告发布之日起3个工作日。 网 六、其他补充事宜 1.根据《关于印发中小企业划型标准规定的通知》的规定，本项目所属行业分类为 建筑业 。 务 2.采购信息发布网站：在贵州省招标投标公共服务平台上公布。 七、对本次采购提出询问，请按以下方式联系。 商 1.采购人信息： 名 称： 石阡县农村水利水电站 道 地 址： 石阡县泉都街道佛顶山大道水务局办公楼 联系方式： 0856-7931646 管 2.采购代理机构信息： 名 称： 铜仁市大力城项目管理有限责任公司 地 址： 铜仁市碧江区国时代天街1号楼16层16-7室 联系方式： 15286751783 3.项目联系方式： 中 项目联系人： 杨帅 电 话： 15286751783 信息来源:https://www.chinapipe.net/project/d3078119.html cqdingjiu 2026.08.24 12:31:38</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1404,14 +1384,14 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>重庆, 管材招标</t>
+          <t>重庆, 管材招标, 农村供水提质改造</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>璧山区2026年大路街道三台村智慧设施农业建设项目招标计划表</t>
+          <t>万州区后山至弹子农村连片供水保障提升工程招标计划表</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1421,7 +1401,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1442,32 +1422,32 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>璧山区</t>
+          <t>万州区</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6.都市农文旅配套建设1000平方米。</t>
+          <t>新建供水规模10000立方米/天的净水厂1座，厂外配水主干管网长度约40公里，村镇配水支线管网长度约100公里，配套一体化供水泵站共15座，新增原水管约1公里。</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>合同预估金额为9182.25万元</t>
+          <t>合同预估金额6000万元</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>温度调控系统、水肥一体化设备、人工补光系统、二氧化碳补施系统、智能环境控制系统、作业物流装备</t>
+          <t>供水设备、管道</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>璧山区2026年大路街道三台村智慧设施农业建设项目招标计划表 重庆市工程建设项目招标计划表 项目 璧山区2026年大路街道三台村智慧设施农业建设项目 名称 招标 法人 或招 网 标人 中农良品（重庆）生态农业有限公司 名称 （盖 章） 项目 批准 务 文件 及文 号 主要 1.新建茄果类智能种植温室11256平方米；2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、二氧化碳补施系统1套、智能环境控制系统1套、作业物流 建设 装备1套；3.项目后勤及仓储配套（含装修）5000平方米；4.土方回填及场地平整53000平方米；5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米；6. 内容 都市农文旅配套建设1000平方米。 商 招 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 道 璧 山 区2026 重 年 庆 大 市 路 公 招标 街 管 共 项目 道 资 三 公 源 台 项目主要建设内容包括：1.新建茄果类智能种植温室11256平方米； 2.设备采购：购置温度调控系统1套、水肥一体化设备1套、人工补光系统1套、 开 交 1 村 二氧化碳补施系统1套、智能环境控制系统1套、作业物流装备1套； 3.项目后勤及仓储配套（含装修）5000平方米； 4.土方回填及场地平整53000平 2026-09 9182.25 招 易 智 方米； 5.新建道路1584米、水渠管网1387米、停车场6500平方米；配套绿化15000平方米； 6.都市农文旅配套建设1000平方米。 标 中 慧 心 设 国 璧 施 山 农 分 业 中 建 心 设 项 目 中 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3076777.html cqdingjiu 2026.08.21 10:06:51</t>
+          <t>万州区后山至弹子农村连片供水保障提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 万州区后山至弹子农村连片供水保障提升工程 招标法人或招 标人名称（盖 重庆长江水务有限公司 网 章） 项目批准文件 万州发改审投〔2026〕82 号 及文号 务 新建供水规模 10000 立方米/天的净水厂 1 座，厂外配水主干管网长度约 40 公里，村镇配水支线 主要建设内容 管网长度约 100 公里，配套一体化供水泵站共 15 座，新增原水管约 1 公里。 招标项目名 招标方 招标文件计划 合同预估金 序号 招标内容 拟交易场所 备注 称 式 发布时间 额(万元) 商 万州区后山至 万州区后山 招标项目 弹子农村连片 重庆市万州 至弹子农村 公开招 1 供水保障提升 2026-08 区公共资源 6000.00 连片供水保 标 工程施工道总承 交易中心 障提升工程 包 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3078105.html 管 cqdingjiu 2026.08.24 12:31:38 国 中</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>水渠管网：1387米</t>
+          <t>净水厂设备及配件；配水管网及配件；一体化供水泵站设备及配件；原水管</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -1475,14 +1455,14 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>重庆, 智慧设施农业, 招标计划, 项目内容, 资金情况, 产品种类</t>
+          <t>重庆, 供水, 管网, 管材, 招标</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>长寿区江南街道污水处理厂更新改造工程项目公告</t>
+          <t>重庆涪陵电力实业股份有限公司2026年第4批物资公开谈判采购采购公告</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1492,7 +1472,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1513,27 +1493,27 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>长寿区</t>
+          <t>渝北区</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>本项目包括但不限于新建混凝池-三沉池，还建格栅池，厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统，原斜管沉淀池改造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰），拆除原有污泥池，新增临时污泥储罐务并还建污泥池，污泥堆场临时改建及恢复，实施技改期间的临时排放工程，进行基础的自控改造。</t>
+          <t>重庆涪陵电力实业股份有限公司2026年第4批物资公开谈判采购</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>企业自筹，出资比例为100%</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>污水处理设备</t>
+          <t>管道</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>长寿区江南街道污水处理厂更新改造工程项目公告 长寿区江南街道污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目长寿区江南街道污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源为企业 自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：长寿区江南街道污水处理厂更新改造工程包括但不限于以下内容新建混凝池-三沉池；还建格栅池； 厌氧池新增搅拌机，好氧池联通孔短流整改、拆除填料及底部曝气盘，增设可提升曝气系统；原斜管沉淀池改 造为二沉池（新增中心筒、改造成多斗排泥、提高液位，更换三角堰）。拆除原有污泥池，新增临时污泥储罐 务 并还建污泥池；污泥堆场临时改建及恢复；实施技改期间的临时排放工程；进行基础的自控改造。 2.2 比选范围：长寿区江南街道污水处理厂更新改造工程施工图范围中的所有工作内容，包括但不限于土建工 程、设备及安装工程、工艺管道工程、电气工程、临排工程等内容，具体以比选人提供的图纸、技术规范、设 备需求清单、答疑资料、澄清资料、其他补遗资料等相关商内容为准。 2.3 建设地点：重庆市长寿区江南街道。 2.4 工期：110日历天（实际开工日期以监理工道程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 3. 参选人资格要求 管 3.1 本次比选要求参选人具备以下条件： （1）独立法人资格； （2）建设行政主管部国门颁发的有效的市政公用工程施工总承包二级及以上资质； 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 中 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月 27 日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务 大厦5楼。 5.2 比选截止时间：2026年8月 27 日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 网 联系人：曹老师 电话：023-71618725 务 代理机构：重庆招标采购（集团）有限责任公司 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 商 联系人：高老师 电话：023-67706841 道 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 管 信息来源:https://www.chinapipe.net/project/d3076456.html cqdingjiu 2026.08.21 10:06:51 国 中</t>
+          <t>重庆涪陵电力实业股份有限公司2026年第4批物资公开谈判采购采购公告 采购项目编 采购项目状态 正在采购 FLDL-JTWZ-2026D 号 重庆涪陵电力实业股份有限公司2026 采购项目名称 采购类型 物资 年第4批物资公开谈判采购 采购文件获取截止时 开启应答文 2026-08-25 09:00:00 2026-09-01 09:00:00 间 件时间 供应商提出澄清问题 网 截止时间 开启应答文件地点 详见附件 采购人 重庆涪陵电力实业股份有限公司 招标代理机 重庆市渝北区青枫北路20号凤凰D 招标代理机构 重庆展泽工程咨询有限公司 务 构地址 座9楼部分办公用 招标代理机构邮编 401120 联系人 供应商服务大厅 联系电话 400-1047-177 传真 商 电子邮箱 JZD_WZ@163.com 信息来源:https://www.chinapipe.net/project/d3078035.html cqdingjiu 2026.08.24 12:31:38 道 管 国 中</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1542,18 +1522,18 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 污水处理厂</t>
+          <t>重庆, 2026年, 第4批物资公开谈判采购, 管道</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>潼南区新胜镇、双江镇污水处理厂更新改造工程项目项目公告</t>
+          <t>大渡口区2024年居民户内燃气安全设施整改项目(二期)、大渡口区2024年城市燃气管道等老化更新改造项目(二期)招标公告</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1563,7 +1543,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1584,47 +1564,47 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>潼南区</t>
+          <t>大渡口区</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>本项目包括两个子项目：一是潼南区新胜镇污水处理厂的更新改造，主要内容是新增一体化污水处理设备基础，更新现有污水处理系统设备，升级处理系统，新建风机房-配电室防尘防渗地坪；二是潼南区双江镇污水处理厂的更新改造，内容包括将原有斜管沉淀池改建为好氧池，新建竖流沉淀池，更新老旧及故障设备，新建储药加药区和一体化危废储存间，完善污水处理配套设施。</t>
+          <t>大渡口区2024年居民户内燃气安全设施整改项目（二期）更换居民气表约11700只、居民灶前自闭阀约112717只、燃气连接用不锈钢波纹软管约112717根。大渡口区2024年城市燃气管道等老化更新改造项目（二期）更新改造庭院埋地燃气管网约6913m，更新改造燃气立管及表后管道约9419户，更新切断阀约489套等，并配套实施管网开挖回填、路面恢复、绿化恢复等。</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>本项目资金来源为企业自筹，出资比例为100%。</t>
+          <t>本项目工程总投资金额：5800.7万元，大渡口区2024年居民户内燃气安全设施整改项目（二期）总投资3165.12万元，大渡口区2024年城市燃气管道等老化更新改造项目（二期）总投资2635.58万元。</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>污水处理设备、一体化设备、沉淀池、好氧池、竖流沉淀池、储药加药区、一体化危废储存间、污水处理配套设施</t>
+          <t>燃气安全设施、城市燃气管道等老化更新改造</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>潼南区新胜镇、双江镇污水处理厂更新改造工程项目项目公告 潼南区新胜镇、双江镇污水处理厂更新改造工程比选公告 1. 比选条件 本比选项目潼南区新胜镇、双江镇污水处理厂更新改造工程，比选人为重庆环保投资集团有限公司，资金来源 为企业自筹，出资比例为100%。现对该项目进行公开比选，诚邀有兴趣的潜在参选人参与比选。 2. 项目概况与比选范围 网 2.1项目概况：潼南区新胜镇污水处理厂更新改造工程，主要建设内容为新增200m?/d一体化污水处理设备基础； 更新现有污水处理系统设备，提高现有沉淀池二沉池、三沉池液位；升级处理系统（干化池改建为污泥池，新 增叠螺脱水机，改建污泥堆场及雨棚）；新建风机房－配电室防尘防渗地坪。潼南区双江镇污水处理厂更新改 务 造工程，主要建设内容为将原有斜管沉淀池改建为好氧池，新建3座竖流沉淀池，配套安装相关设备；更新污水 处理系统中老旧及故障设备；新建储药加药区与一体化危废储存间，完善污水处理配套设施。 2.2 比选范围：潼南区新胜镇、双江镇污水处理厂更新改造工程施工图范围中的工作内容（一体化设备采购及 相关安装工作除外），包括但不限于土建工程、附属工程商（包括但不限于绿化工程、工艺管线工程、电气及自 控工程、临排清淤工程等）、一体化污水处理设备基础、标准化建设、配套设备材料采购及安装工程等内容， 其中一体化设备采购及相关安装工作不在本次比选范围内；具体以比选人提供的图纸、技术规范、工程量清单、 答疑资料、澄清资料、其他补遗资料等相关内容为准。 道 2.3 建设地点：潼南区新胜镇、双江镇。 2.4 工期：120日历天（实际开工日期以监理工程师签发的工程开工通知明确的开工日期为准），缺陷责任期24 个月。 管 3. 参选人资格要求 3.1 本次比选要求参选人具备以下条件： 国 （1）独立法人资格； （2）建设行政主管部门颁发的有效的市政公用工程施工总承包二级及以上资质； 中 3.2 参选人还应在资质、业绩、资金、人员等方面具有相应的服务能力，详见比选文件第二章参选人须知前附 表第1.4.1项内容。 3.3本次比选不接受联合体参选。 4. 比选文件的获取 4.1 参选人于2026年8月19日起可自行在重庆水务集团电子商务平台（https://www.cqswjt.cn）上下载比选文件电 子版，以及答疑、补遗等比选截止时间前公布的所有相关资料，不管参选人下载与否，比选人和代理机构都视 为参选人收到以上资料并全部知晓有关比选过程和事宜，如因参选人自身原因未能下载相关资料由此产生的一 切后果由参选人自行负责。各参选单位应随时关注网上（https://www.cqswjt.cn）发布的比选文件及相关修改内容。 4.2 参选人须在重庆水务集团电子商务平台（https://www.cqswjt.cn）进行供应商注册，填写相关信息，审批过后 成为平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标（仍须同时提交纸质版参选文件）。参选 人需提前在重庆水务集团电子商务平台（https://www.cqswjt.cn）上注册、报名，下载比选文件，上传参选文件电 子档并报价。在比选截止时间前未按时报名、报价并上传参选文件电子档、递交纸质版参选文件者，将被否决 参选。 5. 比选文件的递交 5.1 参选文件递交时间：2026年8月27日09时00分至09时30分，地点：重庆市两江新区嘉华路36号重庆水务大厦5 楼。 5.2 比选截止时间：2026年8月27日09时30分（北京时间）。 5.3 逾期送达的或者未送达指定地点的参选文件，比选人不予受理。 6. 发布比选公告的媒介 本次比选公告在重庆水务集团电子商务平台（https：//www.cqswjt.cn）上发布。 7. 联系方式 网 比选人：重庆环保投资集团有限公司 地 址：重庆市两江新区礼环南路102号 务 联系人：陈老师 电话：023-42756696 商 代理机构：重庆招标采购（集团）有限责任公司 道 地址：重庆市江北区五简路2号重庆咨询大厦A座2004室 联系人：高老师 管 电话：023-67706841 重庆水务电子商务平台国咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3076454.html cqdingjiu 2026.08.21 10:06:51 中</t>
+          <t>大渡口区2024年居民户内燃气安全设施整改项目(二期)、大渡口区2024年城市燃气管道等老化更新改造项目(二 期)招标公告 大渡口区2024年居民户内燃气安全设施整改项目（二期）、大渡口区2024年城市燃气管道等老化更新改造项目 （二期）招标公告 1.招标条件 本招标项目大渡口区2024年居民户内燃气安全设施整改项目（二期）、大渡口区2024年城市燃气管道等老化更新 改造项目（二期）已由重庆市大渡口区发展和改革委员会以渡发改审发[2026]15号、渡发改审发[2026]16号批准 建设，项目业主为重庆市大渡口区经济和信息化委员会，代建业主为重庆燃气集团股份有限公司大渡口分公司， 建设资金来自争取上级资金、区级财政配套及社会资金，项目出资比例为100%网，招标人为重庆燃气集团股份有 限公司大渡口分公司。项目已具备招标条件，现对该项目的工程总承包进行公开招标，评标办法采用综合评估 法。 2.项目概况与招标范围 务 2.1 建设地点：重庆市大渡口区 2.2 项目概况与建设规模： 商 1.大渡口区2024年居民户内燃气安全设施整改项目（二期）更换居民气表约11700只、居民灶前自闭阀约112717只、 燃气连接用不锈钢波纹软管约112717根。 2.大渡口区2024年城市燃气管道等老化更新改道造项目（二期）更新改造庭院埋地燃气管网约6913m，更新改造燃 气立管及表后管道约9419户，更新切断阀约489套等，并配套实施管网开挖回填、路面恢复、绿化恢复等。 2.3 本项目工程总投资金额：5800.7万元，大渡口区2024年居民户内燃气安全设施整改项目（二期）总投资3165.12 万元，大渡口区2024年城市燃气管道等老化更新改造项目（二期）总投资2635.58万元。 管 本次招标项目合同估算金额：5195.561015万元，其中大渡口区2024年居民户内燃气安全设施整改项目（二期）工 程设计费59.350905万元，工程费2849.79万元；大渡口区2024年城市燃气管道等老化更新改造项目（二期）工程设 计费47.44011万元，工程费2238.98万元。 国 2.4 招标范围：主要包括施工图设计、工程施工等内容，具体范围为： (1)设计部分：本项目范围内的施工图设计、施工及竣工验收阶段、质量保修阶段的设计配合服务，以及协助招 标人完成审中批手续办理等工作。按招标人要求按质按时提交设计成果，并取得国家相关职能部门的批准。 (2)施工部分：包括但不限于设计范围内所涉及的工作内容。 (3)其他部分：项目预算编制、总承包管理（对承包项目的质量、安全、工期、造价等全面管控和负责）。 2.5 工期要求：总工期540日历天，缺陷责任期24个月。其中： 设计周期：施工图设计90日历天； 施工工期：450日历天； 2.6 标段划分（如有）：/ 2.7 其他：/ 3.政府采购工程 3.1 是否属于政府采购工程：是 3.2 是否专门面向中小企业预留：是 本项目以联合体形式面向中小企业，以联合体形式参加本次投标的，联合体中中小企业承担的合同份额需达 到40%以上。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件： 同时具备建设行政主管部门颁发的有效的以下资质： 网 4.1.1.1 设计资质：投标人应同时具备以下(1)、(2)项资质 (1)投标人应具备以下A、B、C项资质之一： 务 A.工程设计综合甲级资质。 B.工程设计市政行业乙级及以上资质。 C.工程设计市政行业(城镇燃气工程)专业乙级及以上资质商。 (2)具备《中华人民共和国特种设备设计许可证》(压力管道)公用管道GB1级或《中华人民共和国特种设备生产许 可证》(压力管道设计)公用管道GB1级。 道 4.1.1.2 施工资质：投标人应同时具备以下(1)、(2)项资质 (1)投标人应具备以下A、B项资质之一： 管 A.具备建设行政主管部门颁发的有效的市政公用工程施工总承包二级及以上资质。 B.具备建设行政主管部门颁发的有效的石油化工工程施工总承包三级及以上资质。 (2)具备有效的《中华人国民共和国特种设备安装改造维修许可证》公用管道GB1级或《中华人民共和国特种设备安 装改造修理许可证》公用管道GB1级或《中华人民共和国特种设备生产许可证》公用管道安装GB1级。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的实施能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 中 4.2 本次招标接受联合体投标。联合体投标的，应满足下列要求：联合体单位成员不得超过2家（含联合体牵头 人），且联合体牵头人须由负责施工的联合体成员予以担任，具体详见投标人须知前附表1.4.2。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件、工程量清单 （如有）、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字 证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责 任自负。 5.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 布至2026-08-26 17:00:00前。 5.3招标人应于2026-08-28 23:59:59前在重庆市公共资源交易网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-14 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网和重庆市公共资源交易网发布。[提示：依法必须招标项目的招 标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆燃气集团股份有限公司大渡口分公司 代理机构: 重庆市义渡工程管理有限公司 重庆市大渡口区春晖路街道翠华园小区11 重庆市大渡口区文体路126号锦天商务中 地 址: 地 址: 栋3层 心东楼535室 邮 编: 400084 邮 编: 400084 项目负责人: 任老师 项目负责人: 唐书霞网 电 话: 023-68551113 电 话: 023-85786930 传 真: 传 真: 电子邮箱: 电子邮箱:务 开户银行: 开户银行: 账 号: 账 号: 商 监督部门: 重庆市大渡口区发展和改革委员会 电 话: 023-68083238 2026年08月21日 信息来源:https://www.chinapipe.net/project/d30道77961.html cqdingjiu 2026.08.24 12:31:38 管 国 中</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>更换居民气表约11700只、居民灶前自闭阀约112717只、燃气连接用不锈钢波纹软管约112717根；更新改造庭院埋地燃气管网约6913m，更新改造燃气立管及表后管道约9419户，更新切断阀约489套等。</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 污水处理厂更新改造</t>
+          <t>重庆, 燃气安全设施, 城市燃气管道, 老化更新改造, 投资金额, 项目总投资</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表</t>
+          <t>荣昌区2026年安富街道高标准农田建设项目招标公告</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1634,7 +1614,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1653,30 +1633,34 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>荣昌区</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源</t>
+          <t>改造提升高标准农田326.59亩，其中高效节水灌溉面积130亩。主要内容包括梯台修筑、梯田修筑、稻虾地块修筑、恢复地类整治、输水管道安装、排水沟修建、机耕道改建等。</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>采购预算 409674.71元</t>
+          <t>项目总投资金额181.43万元，本次招标项目合同估算金额166.35万元，全部由财政资金支持。</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>市政水源</t>
+          <t>建筑工程施工</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程单一来源采购方式公示表 采购需求单位(全称) 重庆医科大学附属第二医院总务科 项目名称 重庆医科大学附属第二医院医疗教学配套业务用房第二市政水源工程 项目内容 给重庆医科大学附属第二医院医疗教学配套业务用房配置第二市政水源 采购预算 409674.71元 网 拟采购供应商全称 东部自来水分公司 配套业务用房第二市政水源从重庆水资源产业股份有限公司东部自来水分公司管辖范围 单一来源采购理由 的管网具体接入，属于市政管网施工，具有特殊要求。 务 公示时间 2026年8月19日-2026年8月25日 联系人及联系电话 刘老师 023-63693215 注：1.以上陈述是否真实，欢迎社会各界监督，公示时间商至少5个工作日； 2.公示期内无异议的，采购管理处将进行该项目采购；有异议请将意见反映采购人。 信息来源:https://www.chinapipe.net/project/d30道76334.html cqdingjiu 2026.08.21 10:06:51 管 国 中</t>
+          <t>荣昌区2026年安富街道高标准农田建设项目招标公告 荣昌区2026年安富街道高标准农田建设项目招标公告 1.招标条件 1. 招标条件 本招标项目荣昌区2026年安富街道高标准农田建设项目已由重庆市荣昌区农业农村委员会以荣农发〔2026〕64号 批准建设，项目业主为重庆市荣昌区农田建设中心，建设资金来自 财政资金，项目出资比例为100%，招标人 为重庆市荣昌区农田建设中心。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用经评审 网 的最低投标价法。 2.项目概况与招标范围 2. 项目概况与招标范围 务 2.1 建设地点：安富街道斑竹村 2.2 项目概况与建设规模：改造提升高标准农田326.59亩，商其中高效节水灌溉面积130亩。 2.3 本项目工程总投资金额：181.43万元 本次招标项目合同估算金额：166.35万元 道 2.4 招标范围：梯台修筑127.5亩，梯田修筑61.56亩，稻虾地块修筑128.83亩，恢复地类整治1.22亩；新建Φ160PE 输水管道1949米，C25混凝土排水沟（0.5m*0.6m）320米；改建3.0m宽C25混凝土机耕道905米。包括所提供的施 工设计图所示范围内的所有内容，具体以招标人提供的图纸、工程量清单、答疑资料、澄清资料、其他补遗资 管 料等相关内容为准。若施工图与工程量清单不一致时，以工程量清单为准。 2.5 工期要求：工期为180日历天 ，缺陷责任期为24个月。 2.6 标段划分（如有）：国 / 2.7 其他： / 3.政府采购工程 中 3. 政府采购工程 3.1 是否属于政府采购工程：是 □否 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式：本项目整体面向中小企业。 4.投标人资格要求 4. 投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的建筑工程施工总承包三级及以 上资质或市政公用工程施工总承包三级及以上资质或水利水电工程施工总承包三级及以上资质。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1条内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（荣昌区）下载招标文件、 工程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网（荣昌区）完成市场主体信息登 记以及CA数字证书办理，办理方式请参见重庆市公共资源交易网（荣昌区）导航栏“主体信息”页面中“市场 主体信息登记”、“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法 完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网（荣昌区）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间 从本公告发布至2026-08-26 17:30:00前。 网 5.3招标人应于2026-08-28 18:00:00前在重庆市公共资源交易网（荣昌区）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-16 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 务 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易网（荣昌区）、重庆市公共资源交易监督网发布。[提示：依法必须招 商 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆市荣昌区农田建设中心 代理机构: 重庆富毅项目管理有限公司 地 址: 地道 址: 邮 编: 邮 编: 项目负责人: 李老师 项目负责人: 陈航 电 话: 023-85265043 管电 话: 16623666557 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 国开户银行: 账 号: 账 号: 监督部门: 重庆市荣昌区发展和改革委员会 中 电 话: 023-61471361 2026年08月21日 信息来源:https://www.chinapipe.net/project/d3077954.html cqdingjiu 2026.08.24 12:31:39</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>梯台修筑127.5亩，梯田修筑61.56亩，稻虾地块修筑128.83亩，恢复地类整治1.22亩；新建Φ160PE输水管道1949米，C25混凝土排水沟（0.5m*0.6m）320米；改建3.0m宽C25混凝土机耕道905米。</t>
         </is>
       </c>
       <c r="N18" t="n">
@@ -1684,14 +1668,14 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>高标准农田, 改造提升, 建筑工程施工, 财政资金, 重庆, 荣昌区</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>中铁二院工程集团有限责任公司G319黔江区正阳至城西段改建工程管线探测工作线上询价采购公告</t>
+          <t>大渡口区2025年老化燃气管道及设施更新改造项目(一期)EPC招标公告</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1701,7 +1685,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>其他/未识别</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1722,32 +1706,32 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>黔江区</t>
+          <t>大渡口区</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>本项目服务内容为G319黔江区正阳至城西段改建工程管线探测工作。</t>
+          <t>大渡口区燃气管线及燃气相关设施设备改造提升，实现燃气管线智能化管理和保障燃气供给安全。</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>项目总投资金额7255.57万元，本次招标项目合同估算金额6408.986万元。</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>管线探测工作</t>
+          <t>燃气管道及相关设施设备</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>中铁二院工程集团有限责任公司G319黔江区正阳至城西段改建工程管线探测工作线上询价采购公告 中铁二院工程集团有限责任公司G319黔江区正阳至城西 段改建工程管线探测工作线上询价采购 ZTEYCQ-XJ-2026-019 网 采购单位: 中铁二院工程集团有限责任公司 发布时间: 2026-08-19 16:10 报价截止时间: 务 2026-08-21 17:00 招标方联系人: 杨先生 招标方联系电话: 商 13883021521 招标方邮箱: 监督方联系人: 李先生 道 监督方联系电话: 15823237919 监督方邮箱: 保证金: 0元 管 结算与发票信息: 详情 交货信息: 详情 国 其他说明事项: 标的明细 流水号：询2026081900304 中 计量单 技术标准及要 序号 标的名称 数量 交货期 送货地址 位 求 G319黔江区正阳至城西段 合同签订后5天内完成 西南区-重庆市-市辖 1 1 项 详见询价文件 改建工程管线探测工作 本项目服务内容。 区-黔江区-项目地点 信息来源:https://www.chinapipe.net/project/d3076309.html cqdingjiu 2026.08.21 10:06:51</t>
+          <t>大渡口区2025年老化燃气管道及设施更新改造项目(一期)EPC招标公告 大渡口区2025年老化燃气管道及设施更新改造项目（一期）EPC招标公告 1.招标条件 本招标项目 大渡口区2025年老化燃气管道及设施更新改造项目（一期） 已由 重庆市大渡口区发展和改革委 员会 以 渡发改审发〔2026〕19号 批准建设，项目业主为 重庆市大渡口区经济和信息化委员会 ，代建业 主为 重庆燃气集团股份有限公司大渡口分公司 ，建设资金来自 争取上级资金、区级财政配套及业主自 筹 ，项目出资比例为 100% ，招标人为 重庆燃气集团股份有限公司大渡口分公司 。项目已具备招标条 件，现对该项目的工程总承包进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：重庆市大渡口区 2.2 项目概况与建设规模：大渡口区燃气管线及燃气相关设施设备改造提升，实现燃气管线智能化管理和保障 燃气供给安全。其中，燃气管线智能化管理包含智能燃气系统设备1018台(套)、保障燃气供给安全包含居民立管 务 更换6443户、户外切断阀1500个、智能家用报警器5000套、户外表箱更换11024个、调压箱更换1025台、标志 桩(砖)10000块。 2.3 本项目工程总投资金额：7255.57万元 商 本次招标项目合同估算金额：6408.986万元，其中工程设计费125.526万元、建筑安装工程费4179.22万元、专业设 备材料类费用2104.24万元。 2.4 招标范围：主要包括施工图设计、工程施道工、设备供货等内容，具体范围为： （1）设计部分：本项目范围内的施工图设计、施工及竣工验收阶段、质量保修阶段的设计配合服务，以及协助 招标人完成审批手续办理等工作。按招标人要求按质按时提交设计成果，并取得国家相关职能部门的批准。 管 （2）施工部分：包括但不限于设计范围内所涉及的工作内容。 （3）设备供货：完成本项目设计范围内的专业设备材料供货、调试及质保。 （4）其他部分：项目国软件智能化工作、预算编制、总承包管理（对承包项目的质量、安全、工期、造价等全面 管控和负责）。 2.5 工期要求：总工期18个月，缺陷责任期24个月。其中： 中 设计周期：施工图设计 90 日历天；其他服务18个月； 专业设备材料到货时间、施工工期：15个月。 2.6 标段划分（如有）： / 2.7 其他：质量保质期：专业设备材料和软件质量保证期5年，国家对于三包产品质保期有规定的从其规定。 3.政府采购工程 3.1 是否属于政府采购工程：是 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式： 本项目以联合体形式面向中小企业，以联合体形式参加本次投标的，联合体中中小企业承担的合同份额需达 到 40 %以上。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件： 同时具备建设行政主管部门颁发的有效的以下资质： 4.1.1.1 设计资质：投标人应同时具备以下(1)、(2)项资质 (1)投标人应具备以下A、B、C项资质之一: A.工程设计综合甲级资质。 B.工程设计市政行业乙级及以上资质。 C.工程设计市政行业(城镇燃气工程)专业乙级及以上资质。 网 (2)具备《中华人民共和国特种设备设计许可证》(压力管道)公用管道GB1级或《中华人民共和国特种设备生产许 可证》(压力管道设计)公用管道GB1级。 务 4.1.1.2 施工资质：投标人应同时具备以下(1)、(2)项资质 (1)投标人应具备以下A、B项资质之一 A.具备建设行政主管部门颁发的有效的市政公用工程施工商总承包二级及以上资质。 B.具备建设行政主管部门颁发的有效的石油化工工程施工总承包三级及以上资质。 (2)具备有效的《中华人民共和国特种设备安装道改造维修许可证》公用管道GB1级或《中华人民共和国特种设备安 装改造修理许可证》公用管道GB1级或《中华人民共和国特种设备生产许可证》公用管道安装GB1级。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的实施能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 管 4.2 本次招标接受联合体投标。联合体投标的，应满足下列要求： 联合体成员单位不得超过3家，具体详见投 标人须知前附表1.4.2。 .技术成果经济补偿 本次招标对未中标人投国标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件、工程量清单 （如有）、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字 中 证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字 证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责 任自负。 5.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 布至2026-08-26 17:00:00前。 5.3招标人应于2026-08-28 23:59:59前在重庆市公共资源交易网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-15 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网发布。[提示：依法必须招标项目的招 标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆燃气集团股份有限公司大渡口分公司 代理机构: 重庆市义渡工程管理有限公司 重庆市大渡口区春晖路街道翠华园小区11 重庆市大渡口区文体路126号锦天商务中 地 址: 地 址: 栋3层 心东楼535室 邮 编: 邮 编: 项目负责人: 任先生 项目负责人: 严力 电 话: 023-68551113 电 话: 023-85786930 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市大渡口区发展和改革委员会 电 话: 023-68083238 2026年08月21日 网 信息来源:https://www.chinapipe.net/project/d3077935.html cqdingjiu 2026.08.24 12:31:39 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>智能燃气系统设备1018台(套)，居民立管务更换6443户，户外切断阀1500个，智能家用报警器5000套，户外表箱更换11024个，调压箱更换1025台，标志桩(砖)10000块。</t>
         </is>
       </c>
       <c r="N19" t="n">
@@ -1755,14 +1739,14 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类, 匹配程度, 匹配关键词</t>
+          <t>重庆, 燃气管道, 老化改造, 智能化管理, 燃气供给安全</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告</t>
+          <t>龙兴新城污水管网工程建设及整治修复项目(二期)招标计划表</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1772,7 +1756,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1791,49 +1775,45 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>涪陵区</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>本项目主要涉及室外蒸汽管道φ219x6mm的安装，管道材质为20#，地上敷设，蒸汽管道运行压力1.08MPa，管道设计压力1.2MPa。蒸汽管道系统包括从锅炉房分汽缸到6#和8#车间分汽缸的所有蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温工作。还包括钢结构桁架工程的采购、运输、制作、安装、防腐工作，以及管道附件及控制系统的采购、运输、安装、接线等工作。此外，还需要进行调试与验收，确保蒸汽管道系统能够正常使用并备案。</t>
+          <t>管网工程、土石方工程等。</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>项目总投资额为580.643717万元，全部为企业自筹资金。</t>
+          <t>合同预估金额为2500万元</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>蒸汽管道、管件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸、钢结构桁架、阀门、压力表、温度表、流量计、电动/气动执行机构、配套仪表电缆、桥架、保护管</t>
+          <t>管网工程、土石方工程</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 乌江涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程招标公告 1.招标条件 本招标项目乌江涪陵榨菜绿色智能化生产基地(一期)已由重庆市涪陵区发展和改革委员会以重庆市企业投资项目 备案证2020-500102-13-03-000003 批准建设，项目业主为重庆市涪陵榨菜集团股份有限公司，建设资金来自企业 自筹，项目出资比例为100% ，招标人为重庆市涪陵榨菜集团股份有限公司。项目已具备招标条件，现对乌江 涪陵榨菜绿色智能化生产基地(一期)6#、8#车间蒸汽管道安装工程施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 2.1 建设地点： 重庆市涪陵区马鞍街道人和社区 。 网 2.2 项目概况与建设规模：建筑面积约369384.27㎡。本项目蒸汽管道主要为室外蒸汽管道φ219x6mm，管道材质： 20#地上敷设，由14#锅炉房分汽缸分别接至6#和8#智能化车间分汽缸，蒸汽管道运行压力1.08MPa，管道设计压 力1.2MPa。 务 2.3 本次招标项目合同估算金额：580.643717万元。 2.4 招标范围： 商 （1）蒸汽管道系统本体：从锅炉房分汽缸后（含分气缸阀门）至6#车间、8#车间分气缸处，所有蒸汽管道、管 件、法兰、螺栓垫片、管道支吊架、补偿器、疏水阀组、分气缸等的采购、运输、安装、保温（含保温层及保 护层）工作。 道 （2）钢结构桁架工程：负责本项目范围内所有钢结构架空桁架（管廊）的采购、运输、制作、安装、防腐工作。 （3）管道附件及控制系统：负责本工程范围内所有阀门、压力表、温度表、流量计、电动/气动执行机构以及配 套仪表电缆、桥架、保护管的采购、运输、安装、接线。负责与DCS/PLC系统接口的接线与联动调试。 管 （4）调试与验收：组织并确保整个蒸汽管道系统（含分气缸后段末端管道、桁架及其安全附件）通过项目所在 地特种设备安全监察管理部门实施的安装监督检验。负责报检、配合现场检验、整改、出具深化图纸并由设计 单位审核盖章、特种设备法定报检取证的全部费用，包括但不限于：施工前办理安装告知，设计院盖章审核， 施工中接受并通过安装国监督检验，最终负责取得《压力管道安装监督检验证书》与《特种设备使用登记证》， 确保蒸汽管道投入使用并备案，提交全套法定检验报告。 （5）土建工作部分 中 1）管架和桁架基础的施工，包括但不限于钢结构桁架的混凝土独立基础的土方开挖、浇筑、养护及回填恢复。 2）管道穿墙/板孔洞的开挖、封堵与修复。 3）室内外地面的开挖（包括但不限于疏水井、沟槽开挖、通行地沟、设备基础开挖）与恢复（包括但不限于土 方回填、渣土弃运、地面硬化）。 4）桁架及设备接地线的施工，包括但不限于接地极制作、接地干线敷设，并与厂区主接地网可靠连接，接地电 阻测试合格。 具体详见施工图、招标文件、工程量清单、答疑补遗等资料。 2.5 工期要求： 60 日历天 缺陷责任期要求： 24 个月 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：投标人应同时具备以下(1)、(2)项资质： （1）具备建设行政主管部门颁发的有效的建筑工程施工总承包二级及以上资质； （2）具备有效的《中华人民共和国特种设备生产许可证》（许可子项目：工业管道安装GC2级及以上）。 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 网 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 务 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（涪陵区） （https://www.cqggzy.com/fulingweb/）下载招标文件、工程商量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网（涪陵区道）（https://www.cqggzy.com/fulingweb/）本项目招标公告网页下 方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-23 17:00:00前。 4.3招标人应于2026-08-24 18:00:00前在重庆市公共资源交易网（涪陵区）（https://www.cqggzy.com/fulingweb/）发 布澄清。 5.投标文件递交的内容 管 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-09 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 国 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（涪陵区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 中重庆市涪陵榨菜集团股份有限公司 代理机构: 中招国际招标有限公司 重庆两江新区黄山大道中段53号5-1（双 地 址: 重庆市涪陵区江北街道办事处二渡村一组 地 址: 鱼座A栋5楼） 邮 编: 408000 邮 编: 项目负责人: 徐老师 项目负责人: 寿云凤 电 话: 13212467016 电 话: 023-68881331-9032 传 真: 传 真: 电子邮箱: bsd2me@126.com 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市涪陵区发展和改革委员会 电 话: 023-72203687 2026年08月19日 乌江 涪陵 榨菜 绿色 智能 化生 产基地 (一 期)6#、 8#车 网 间蒸 汽管 道安 装工 务 程 中 中 国 国 重 银 重 商民 重 庆 行 庆 生 庆 涪 股 涪 银 涪 陵 份 陵 行 陵 重 投 公 有 道公 股 公 庆 标 共 限 共 份 共 银 开 保 户 资 公 资 有 资 行 户 证 110292140553VA00154 9902001860445897 430102029007791845-275 名 源 司 源 限 源 涪 行 金 交 重 交 公 交 陵 账 管 易 庆 易 司 易 支 号 有 涪 有 重 有 行 限 陵 限 庆 限 公 马 公 涪 公 国 司 鞍 司 陵 司 支 支 行 行 中 信息来源:https://www.chinapipe.net/project/d3076300.html cqdingjiu 2026.08.21 10:06:51</t>
+          <t>龙兴新城污水管网工程建设及整治修复项目(二期)招标计划表 重庆市工程建设项目招标计划表 项目名称 龙兴新城污水管网工程建设及整治修复项目（二期） 招标法人或招标 重庆两江新区龙兴新城建设投资有限公司 人名称（盖章） 网 项目批准文件及 文号 主要建设内容 主要建设内容管网工程、土石方工程等。 务 招标方 招标文件计划 拟交易场 合同预估金额 序号 招标项目名称 招标内容 备注 式 发布时间 所 (万元) 龙兴新城污水 招标项目 主要建设内容 重庆市公 管网工程建设 商公开招 1 管网工程、土 2026-09 共资源交 2500.00 及整治修复项目 标 石方工程等。 易中心 （二期） 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 道 信息来源:https://www.chinapipe.net/project/d3077891.html cqdingjiu 2026.08.24 12:31:40 管 国 中</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>蒸汽管道：1.08M</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>重庆, 蒸汽管道, 安装工程, 资金情况, 产品种类</t>
+          <t>重庆, 污水管网工程, 二期, 管网工程, 土石方工程, 2500万元</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程询比采购公告</t>
+          <t>李市镇农村饮水管网改建工程竞争性磋商公告</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1843,7 +1823,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1864,27 +1844,27 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>巴南区</t>
+          <t>江津区</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>完成重庆国际生物城配套公寓项目（民用1020户）天然气表后管道定制化服务。（含安装燃气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个，其它配套管件及辅材，墙体管道暗埋等）</t>
+          <t>李市镇农村饮水管网改建工程</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>预算金额：1,653,882.29元</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>天然气表后管道定制化服务</t>
+          <t>水管</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>重庆巴南天然气有限责任公司重庆国际生物城配套公寓项目天然气表后管道安装工程询比采购公告 采购公告 公告编号： RQXYGG202608190057 一、采购项目基本情况 采购人：重庆巴南天然气有限责任公司 网 采购项目编号：RQCGXY202608170010 采购项目名称：重庆国际生物城配套公寓项目天然气表后管道安装工程 务 采购内容和范围：完成重庆国际生物城配套公寓项目 （民用1020户）天然气表后管道定制化服务。（含安装燃 气输送用不锈钢波纹管RSB-IF-13—12240米（预估）、双外螺纹球阀DN15-1020个、燃气管道自闭阀DN15-1020个， 其它配套管件及辅材，墙体管道暗埋等） 二、供应商资格要求 商 1. 资质要求:资质要求： 1.响应供应商为中华人民共和国境内合法注册的独立法人或其他组织，具有独立承担民事责任能力，具有独立订 立合同的权利。 道 2.响应供应商应具备市政公用工程施工总承包三级及以上资质、具备有效的安全生产许可证。 3.响应供应商应为本项目配备项目负责人一名，持有市政公用工程或机电工程专业二级建造师及以上资质，且为 本单位在职人员并提供社保证明。 4.响应供应商应为本项目配备专职安全员一名，持有安全生产考核合格C证，且为本单位在职人员并提供社保证 管 明。 5.项目负责人及专职安全员社保证明期限须包含2026年5月至2026年7月。提供的社保证明，须体现上述人员的姓 名、身份证号（或社保号）、单位名称、本单位参保时间（或起始参保时间），并带有社保部门公章或社保部 门的有效电子印章。 2. 信用要求:6.信用要求国： （1）响应供应商（含联合体响应的成员单位）未被“国家企业信用信息公示系统” 网站（www.gsxt.gov.cn）列 入严重违法失信企业名单（如：提供网站查询界面截图）； （2）响应供应商（含联合体响应的成员单位）未被 “信用中国”网站（www.creditchina.gov.cn）列入严重失信 主体名单（中如：提供网站查询界面截图）。 三、采购文件的获取 采购文件在 华润守正采购交易平台 发布，不再另行线下提供纸质采购文件，凡有意参与者请自行登录守正平台 查看和下载采购文件。 四、响应文件的提交 响应文件提交 / 报价截止时间： 2026-08-25 08:00:00 （北京时间，若有变化另行通知）。 响应文件提交 / 报价方式：在响应文件提交 / 报价截止时间前，通过 华润守正采购交易平台 提交电子响应文件或 报价，逾期提交将被拒收。 五、采购人联系方式 联系人：何俊 电话：15178855716 邮箱：1460553040@qq.com 六、采购明细 行号 采购内容 需求数量 单位 补充说明 1 重庆国际生物城配套公寓项目天然气表后管道定制化服务 1 元/次 具体内容详见采购文件 七、答疑澄清、通知 答疑澄清、通知等文件一经在 华润守正采购交易平台 发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注 华润守正采购交易平台 发布的相关信息，并及时查阅和处理。 八、服务费交纳 网 本项目向成交人收取服务费,供应商收到预成交通知书和服务费交款通知书10日内,向平台运营方(华润守正招标有 限公司)支付服务费,经确认无误后由采购人发送成交通知书。平台运营方在收到服务费后向成交人开具服务费发 票。 收费标准：项目总成交金额＜50万元的采购项目，免收服务费。项目总成交金额≥50万元的采购项目，按成交金 务 额的0.15%向成交人收取（金额四舍五入，精确到分）。单项目总收费封顶100000元。其他说明：（1）总价采购， 收费基数为成交金额；单价、费率采购，收费基数为预算金额。（2）单项目存在多个成交人情形的，按总成交 金额计算收费总额，各成交人按成交比例分摊；项目总成交金额50万以上，但单个成交人成交金额少于50万仍按 比例收取服务费。 商 退款说明：成交通知书发布后,平台提供相关服务已完成,成交人已交纳服务费不予退还。 多成交人服务费收取示例： 以某项目总成交金额100万为例,A、B、C多成交人情形,总服务费为0.15万, 供应商A成交金额为50万,A服务费为0.075万; 供应商B成交金额为30万,B服务费为0.045万; 道 供应商C成交金额为20万,C服务费为0.03万。 九、其它事项 管 1.本公告在 华润守正采购交易平台 ( https://www.szecp.com.cn/ )上公开发布。 2.本项目采购通过守正平台线上进行，供应商需注册 华润守正采购交易平台 ，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 国 3.如对采购项目有异议，请登录 华润守正采购交易平台 ,通过异议菜单提出。 2026年08月19日 中 信息来源:https://www.chinapipe.net/project/d3076125.html cqdingjiu 2026.08.21 10:06:52</t>
+          <t>李市镇农村饮水管网改建工程竞争性磋商公告 本项目保证金支持电子投标保函形式，如需申请保函请点击右上角“申请投标保函” 项目概况： “李市镇农村饮水管网改建工程”项目的潜在供应商应在“网上获取”获取采购文件，并于 2026年9月1日 10:00 （北京时间）前递交响应文件。 一、项目基本情况 网 项目号：JJQ26B00032 项目名称：李市镇农村饮水管网改建工程 务 采购方式：竞争性磋商 预算金额：1,653,882.29元 商 最高限价：1,653,882.29元 采购需求： 包号：1 道 包内容 最高限价 数量 单位 简要技术要求 李市镇农村饮水管网改建工程 1,653,882.29元 1 项 详见竞争性磋商文件。 最高限价总计：1,653,882.29元 管 合同履行期限：详见竞争性磋商文件。 本项目是否接受联合体：否 国 二、申请人的资格要求 1、满足《中华人民共和国政府采购法》第二十二条规定。 中 2、落实政府采购政策需满足的资格要求： 本项目专门面向中小企业采购，承建企业应为中小微企业（提供中小企业声明函）或监狱企业（提供监狱企业 证明文件）或残疾人福利性单位（提供残疾人福利性单位声明函）。 注： ①“中小企业声明函”应由供应商出具，并加盖供应商公章，声明函格式详见本竞争性磋商文件第七篇“中小 企业声明函”； ②“监狱企业证明文件”应当由供应商（承建企业）提供其属于监狱企业的证明文件，该证明文件由省级以上 监狱管理局、戒毒管理局（含新疆生产建设兵团）出具； ③“残疾人福利性单位声明函”应由供应商（承建企业）提供其出具的“残疾人福利性单位声明函”，并加盖 该残疾人福利性单位公章。 3、本项目的特定资格要求： ①供应商具备建设行政主管部门颁发的有效的水利水电工程施工总承包叁级及以上资质。（响应文件中提供有 效的证书复印件并加盖供应商公章） ②供应商具备建设行政主管部门颁发的有效的安全生产许可证。（响应文件中提供有效的安全生产许可证复印 件并加盖供应商公章） 三、获取竞争性磋商文件的地点、方式、期限及售价 获取文件期限：2026年8月21日 至 2026年8月28日。 每天上午09:00:00至12:00:00，下午12:00:00至17:00:00。（北京时间，法定节假日除外 ） 文件购买费:0.00元/包 获取文件地点：网上获取 方式或事项： 网 （一）供应商应通过重庆市政府采购网（www.ccgp-chongqing.gov.cn）登记加入“重庆市政府采购供应商库”。 务 （二）磋商文件获取方式：凡有意参加磋商的供应商，请到“重庆市政府采购网”→“个人中心”→“在线开 评标”→“电子标书在线获取”处在线下载或获取本项目磋商文件以及图纸、澄清等磋商前公布的所有项目资料 （本次不提供纸质版磋商文件），无论供应商下载或获取与否，均视为已知晓所有磋商内容。磋商文件获取期 限：自公告发布之日起五个工作日。 商 （三）采购公告所附磋商文件仅供阅览使用，供应商只有登录“重庆市政府采购网”→“个人中心”→“在线 开评标”→“电子标书在线获取”处完成网上获取磋商文件才被视为合法获取了采购文件，否则其响应文件将 被拒绝。即：未通过“重庆市政府采购网”→“个人中心”→“在线开评标”→“电子标书在线获取”处下载、 获取磋商文件，将无法上传响应文件。 道 注意事项：本项目为重庆市江津区政府采购电子标项目，首次参与电子标的供应商须申请重庆市政府采购网账 号密码、办理CA证书并下载响应文件制作系统，制作电子响应文件进行互联网线上响应，具体操作流程请下载 采购公告附件进行查看。因未注册重庆市政府采购网账号、未办理CA证书、操作不当等原因造成无法递交响应 管 文件或递交响应文件失败的后果由供应商自行承担。 1.CA证书的办理流程：登录“重庆市政府采购网”→“个人中心”→“在线开评标”→“电子招投标中心” →“相关下载”栏目，下载附件《重庆市全流程电子招投标项目供应商办理正式CA签章流程手册》，并按照要 求操作。 国 2.响应文件制作：登录“重庆市政府采购网”→“个人中心”→“在线开评标”→“电子招投标中心”→“相关 下载”栏目，下载附件《【供应商必看】政府采购（CA版）供应商投标前软件安装手册》、《政府采购全程电 子化采购系统供应商操作手册（CA证书签章版）》和下载响应文件制作工具，并按下载的操作手册引导，完成 中 电子响应文件制作。 四、磋商响应文件递交 磋商响应文件递交开始时间： 2026年8月24日 09:00 磋商响应文件递交截止时间： 2026年9月1日 10:00 磋商响应文件递交地点：本项目采用网上递交方式，投标人于投标截止时间前使用平台提供的客户端投标工具 编制投标文件，然后登录“重庆市政府采购网”，进入“在线开评标”栏目，在“我的投标项目”→“在线投 标”板块提交。 五、评审信息 磋商开始时间： 2026年9月1日 10:00 磋商地点：本项目采用网上开标方式，投标人可在“重庆市政府采购网”→“个人中心”→“在线开评 标”→“开评标大厅”远程参与开标（开标必备设备：CA证书和可以无线上网的笔记本电脑（必须带有摄像头、 麦克风和声卡等功能）、无线网卡等），因投标人自身原因导致未能在规定时间内解密电子投标文件或参与开 标的，其后果由投标人自行承担 六、公告期限 自本公告发布之日起3个工作日 七、其他补充事宜 1.投标人如未在规定时间内（系统默认30分钟，可根据现场响应情况进行延长/变更）解密电子投标文件的情形约 定： （1）因政府采购全程电子化系统客观原因影响解密时间的，采购人/采购代理机构可根据现场实际情况延长解密 时间。投标人在仍不能解密的情况下，投标人可向采购人/采购代理机构申请，网启用上传不加密的电子备份文件 的方法作为补救措施；在规定的时间内，投标人既不解密，也未提供不加密的电子备份文件作为补救措施的， 视为投标人主动放弃对该项目的投标资格。 （2）因投标人主观原因未完成解密工作的，且未在规定时间内提供有效不加密的备份文件的，都视为投标人在 务 提交投标文件截止时间后撤销投标文件，响应无效且投标人不得再参与本项目后续采购活动。如果项目提供了 保证金的，保证金扣除不予退还。 2.本项目采用全流程电子招投标。各投标人需熟悉了解整个政府采购电子化开评标全过程。具体电子化采购规则 以及操作指南请下载项目公告附件《重庆市全流程电子招商投标项目投标人办理正式CA签章流程手册》和《政府 采购全程电子化采购系统供应商操作手册（CA证书签章版）》、《【供应商必看】政府采购（CA版）供应商投 标前软件安装手册》，并按其要求操作。 八、联系方式 道 1、采购人信息 采购人：重庆市江津区李市镇人民政府 管 采购经办人：黄老师 采购人电话：023-47712801 国 采购人地址：重庆市江津区李市镇回龙路57号 2、采购代理机构信息 中 代理机构：重庆爱采招标代理有限公司 代理机构经办人：李老师 代理机构电话：023-62551600 代理机构地址：重庆市巴南区李渡路59号（李家沱大融城B4栋）2-1、2-2 3、项目联系方式 项目联系人：黄老师 项目联系人电话：023-47712801 https://www.cqggzy.com/trade/014005/1666888712375808000?categoryNum=014005001 信息来源:https://www.chinapipe.net/project/d3077886.html cqdingjiu 2026.08.24 12:31:40</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1893,18 +1873,18 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>重庆, 天然气表后管道安装工程, 管材招标</t>
+          <t>重庆, 水管, 农村饮水管网改建工程</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)非金属管道管件阀门采购招标公告</t>
+          <t>长安工业渝北工厂供水管网泄露检测及修复询比采购公告</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1933,45 +1913,49 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>渝北区</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)建设。</t>
+          <t>长安工业渝北工厂供水管网泄露检测及修复询比采购</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>项目资金来自业主自筹，项目出资比例为100%。本次招标项目货物采购估算金额约为330万元。</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>非金属管道管件阀门</t>
+          <t>供水管网泄露检测及修复设备和服务</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)非金属管道管件阀门采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）非金属管道管件阀门采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约 330 万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采 购”包括不限于非金属管道管件阀门所含设计、制造、试验、出厂检验、防腐、运输（含保护、包装及运输、 货到现场车板交货）、保险（交货验收前）、指导安装、调试、备件及专用工具、税费、技术资料和图纸及质 保期内的各种备品、备件的供应及相关的技术服务、产品质量证明书及原材料检测报告等。（详见“第五章货 物需求一览中表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 2.6 交货期： 2.6.1合同签订后3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向买方提交完整的技术资料，以供设计院开展相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）投标人具备有效的《中华人民共和国特种设备生产许可证》压力管道管子-B级及以上资质、压力管道管 件B2级及以上资质； （3）投标人具备塑料管道管子、管件的型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4. 招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年 8 月19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 网 5.投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月10 日上午09时30分，地点在重庆市公共资源交易中心开标厅（地 址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见一、二楼大厅显示屏。 务 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 商 本次招标公告在中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 道 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 管 联 系 人：张先生 电 话：023-40717888 国 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区五里店五简路2号重庆咨询大厦A栋20楼2001室 中 项目负责人：彭文婷 电 话： 023-67703002 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）非金属管道管件阀门采购 户名 开户行 投标保证金账号 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000631258 支行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051303372 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630010400 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000002549 贸易试验区分行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835014652 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146619529 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764260665 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020038958 信息来源:https://www.chinapipe.net/project/d3076119.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
+          <t>长安工业渝北工厂供水管网泄露检测及修复询比采购公告 【长安工业渝北工厂供水管网泄露检测及修复询比采购】采购公告 采购单位 重庆长安智能工业技术服务有限公司 代理机构 标的物 长安工业渝北工厂供水管网泄露检测及修复询比采购 长安工业渝北工厂供水管网泄露检测及修复询比采购公告 网 务 重庆长安智服对长安工业渝北工厂供水管网泄露检测及修复询比采购。现邀具有此采购项供应能力的厂商前来 参与采购活动。请按照本采购文件的要求递交响应文件 1.项目概况与采购范围 商 1.1 采购项目名称：长安工业渝北工厂供水管网泄露检测及修复询比采购 1.2 采购人：长安智服 道 1.3 采购方式：询比采购 1.4采购范围：长安工业渝北工厂供水管网泄露检测及修复询比采购 管 1.5 工期：全面检测总工期：40个工作日。 1.6服务地点：重庆长安工业（集团）有限责任公司机加区 国 2.供应商资格要求 2.1资质要求：供应商须具备法人资格，提供《营业执照》复印件，加盖供应商单位公章。 中 2.2 业绩要求：/。 2.3本项目不接受“三无”供应商投标（“三无”供应商是指：无实缴注册资本、无参保人员、无生产经营场所 的供应商）。供应商须提供不属于“三无”供应商的证明材料： （1）提供有实缴注册资本的证明材料（若供应商属事业单位的不作要求），如：“天眼查”或“企查查”APP 显示实缴资本的页面截图；或国家有关法律法规规定的具有验资资格的机构出具的验资报告等；或其他第三方 机构提供的可以证明供应商有实缴注册资本的证明材料。 （2）提供为员工缴纳社会保险的证明材料，供应商为员工缴纳社会保险汇总表（至少提交近3个月社会保险汇总 表）。 （3）提供有生产经营场所的证明材料，如：不动产权证书复印件，或生产经营场所的租赁合同复印件。 上述材料需加盖供应商单位公章。 2.4人员要求： 委托代理人必须为供应商本单位人员。提供供应商本单位为该委托代理人缴纳养老保险的证明材料（近3个月）， 加盖供应商单位公章。 说明：（1）投标人提交的上述资格审查资料均为扫描件（原件或复印件的扫描件均可），扫描件须清晰可辨； （2）投标人在《投标函》中承诺其提供的上述相关证明材料真实有效，不存在弄虚作假情形。 3.采购文件的获取 3.1 获取时间：2026年8月21日至2026年8月23日17时00分止。 3.2 获取方式：在“南方数字供应链”电子采购平台下载采购文件。 操作：在浏览器中输入平台网址，打开门户页面→点击【供应商/竞买人登录】→在工作台页面点击【询比采购】 菜单→点击【可参与项目】→选择本项目→登记联系人信息→下载采购文件。 说明：参加采购活动的供应商，需在“南方数字供应链”电子采购平台完成注册、办理CA证书（可使用手机下载 “中招互连APP”办理CA证书）。供应商操作指南：打开门户页面→在顶部右网侧点击【帮助中心】→在下拉菜 单中点击【操作手册】→点击【非招标业务-供应商操作手册】。 4.投标文件递交和开标 务 4.1 投标文件递交截止时间：2026年8月 27日北京时间9:30分结束。 4.2递交方式：在“南方数字供应链”电子采购平台上传递交投标文件电子版。 供应商除了在平台递交电子投标文件外，还需递交纸质版商投标文件1份（采购人用于存档）。纸质版投标文件投 递渠道方式为邮寄递交或现场投递。邮寄递交地址：重庆江北区大石坝8村长安公司5号门岗 。联系人：陈敏 13896127511。 4.3 开标时间：2026年8月27日北京时间 9：30道分。开标地点：网上。 说明：本次采购项目为非涉密项目，所投递的响应文件不得涉及国家秘密、工作秘密及其他内部敏感信息。 4.4洽谈时间与地点:采购人电话通知。 管 5、发布采购信息的媒介 本项目采购信息在“南方数字供应链平台”（https://www.cse-ssc.com）-“非招标采购”业务板块上发布。 国 6、联系方式： 采购人：重庆长安智能工业技术服务有限公司 中 地址：重庆市江北区大石坝8村长安公司5号门岗 联系人：陈 敏 联系电话：13896127511 信息来源:https://www.chinapipe.net/project/d3077867.html cqdingjiu 2026.08.24 12:31:41</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>全面检测总工期：40个工作日。</t>
         </is>
       </c>
       <c r="N22" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 资金, 产品</t>
+          <t>重庆, 供水管网泄露检测及修复, 询比采购</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)衬氟管道及管件采购招标公告</t>
+          <t>万州区旧城供水管网改造工程(三期)管材等材料采购(第二次)招标公告</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1981,7 +1965,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2000,45 +1984,49 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>万州区</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>重庆市映天辉氯碱化工有限公司拟开展废盐综合利用联产20万吨/年离子膜烧碱项目(一期12万吨/年)，包括衬氟管道及管件的采购。</t>
+          <t>该项目对百安坝等3个街道老旧市政供水管道及附属设施进行改造，配套智慧水务物联网感知设备建设，共计改造老旧市政供水管道84.2千米。</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>项目资金来自业主自筹，项目出资比例为100%。货物采购估算金额约为225万元。</t>
+          <t>项目资金来自超长期特别国债资金及业主自筹，项目出资比例为100%，本次招标项目货物采购估算金额为2500万元。</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>衬氟管道及管件</t>
+          <t>管材、管件、阀门类、伸缩器、电磁流量计、法兰及其他等材料</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>废盐综合利用联产20万吨／年离子膜烧碱项目(一期12万吨／年)衬氟管道及管件采购招标公告 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购招标公告 1、招标条件 本招标项目废盐综合利用联产20万吨/年离子膜烧碱项目已由重庆市长寿区发展和改革委员会以 重庆市企业投 资项目备案证（2207-500115-04-05-168305）批准建设，项目业主为重庆市映天辉氯碱化工有限公司，建设资金来 自业主自筹，项目出资比例为100%，招标人为重庆市映天辉氯碱化工有限公司。项目已具备招标条件，现对本 项目的（一期12万吨/年）衬氟管道及管件采购进行公开招标。 网 2、项目概况 2.1 建设地点：重庆长寿经济技术开发区化北路2号。 务 2.2、项目概况与建设规模： 重庆市映天辉氯碱化工有限公司（以下简称“映天辉”）位于重庆长寿经济技术开发区化北路2号，始建于2004 年5月，占地430亩，注册资本34800万元。现为国有控股企商业，是一家集氯碱生产经营、新材料研发经营于一体 的专业型、科技型综合企业，系国家级高新技术企业。 映天辉作为长寿经开区氯碱产业基础平台的龙头化工企业，现有一条氯碱生产线，生产规模为20万吨/年烧碱 （折100%NaOH计）。为建设并贯通氯碱化工道循环经济产业链，保障下游产业链装置氯气需求，实现氯碱产品的 升级和高端化发展，增加产品附加值，降低成本，提高竞争力，映天辉公司经过充分调研和反复论证后，拟开 展废盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）建设。装置在正常运行情况下，按照每年 8000 小时操作。具体要求及参数以第五章货物需求一览表及技术规格标准和要求为准。 管 2.3 本次招标项目货物采购估算金额： 约225万元。 2.4招标范围： 本次招标项目为：“废国盐综合利用联产20万吨/年离子膜烧碱项目（一期12万吨/年）衬氟管道及管件采购一批” 包括但不限于制造、涂漆、包装、运输、配合验收工作、检验检测、产品质量证明书等。（详见“第五章货物 （材料）需求一览表及技术规格标准和要求”）。 2.5 交货地点：货物运送至买方指定地点； 中 2.6 交货期： 2.6.1合同签订后 3个月内，所有货物运送招标人现场并具备安装条件。 2.6.2 中标方应于合同签订之日起7天内，向招标方提交完整的技术资料，以供设计院开展设备相关设计工作。 3、投标人资格要求 3.1 投标人应符合以下要求： （1）投标人具备有效的营业执照。 注：不得将投标人营业执照记载的经营范围作为评审因素。 （2）具备有效的《中华人民共和国特种设备生产许可证》-压力管道元件制造-元件组合装置。 （3）具有防腐管道元件特种设备型式试验证书。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3本次招标不接受代理商投标，不接受联合体投标。 4、招标文件的获取 4.1 凡愿意参加的潜在投标人，从2026年8 月 19 日起至投标截止时间前，均可登录重庆市公共资源交易网 （www.cqggzy.com）直接下载获取招标文件、答疑等开标前的有关资料。在公告期间，各投标人应随时关注网上 发布的招标文件答疑、补遗、澄清等文件内容，不管投标人是否下载，均视为已知晓招标文件的全部内容和有 关事宜。本项目不需要报名，直接投标。 5、投标文件的递交 5.1 投标文件递交的截止时间为 2026年 9 月 10 日上午09时30分，地点在重庆市公共资源交易中心开标厅 （地址：重庆市两江新区青枫北路6号渝兴广场B10栋2层），具体开标地点详见网一、二楼大厅显示屏。 5.2逾期送达的或者未送达指定地点的，或者未按照招标文件要求密封的投标文件，招标人将拒收。 6、发布公告的媒介 务 本次招标公告在 中国招标投标公共服务平台、重庆市公共资源交易网上发布。 7、联系方式 商 招 标 人：重庆市映天辉氯碱化工有限公司 地 址：重庆长寿经济技术开发区化北路二号 道 联 系 人：张先生 电 话：023-40717888 管 招标代理机构： 重庆招标采购（集团）有限责任公司 地 址：重庆市两江新区国五里店五简路2号重庆咨询大厦A栋20楼2001室 项目负责人：彭文婷 电 话： 023-67703002 中 废盐综合利用联产20万吨／年离子膜烧碱项目（一期12万吨／年）衬氟管道及管件采购 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630011190 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835003139 坝支行 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000000834 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146638621 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051302432 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000620855 支行 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020013554 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764235261 信息来源:https://www.chinapipe.net/project/d3076111.html cqdingjiu 2026.08.21 10:06:52</t>
+          <t>万州区旧城供水管网改造工程(三期)管材等材料采购(第二次)招标公告 万州区旧城供水管网改造工程（三期）管材等材料采购 （第二次）招标公告 1.招标条件 本招标项目万州区旧城供水管网改造工程（三期）管材等材料采购已由 重庆市万州区发展和改革委员以 万 州发改审投【2025】16号 批准建设，项目业主为 重庆长江水务有限公司，招标项目资金来自 超长期特别国 债资金及业主自筹 ，项目出资比例为 100% ，招标人为 重庆长江水务有限公司 。项目因首次招标失败， 现对该项目的 管材等材料采购进行第二次公开招标，评标办法采用经评审的最低投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 万州区五桥片区 。 2.2 项目概况与建设规模：该项目对百安坝等3个街道老旧市政供水管道及附属设施进行改造，配套智慧水务物联 务 感知设备建设，共计改造老旧市政供水管道84.2千米。其中，改造DN150供水管线8.1千米、DN200供水管线29.3 千米、DN250供水管线23千米、DN300供水管线5.1千米、DN400管线11.9千米、DN500供水管线6.8千米，管道材 质为3PE防腐内热熔防腐钢管。 2.3 本次招标项目货物采购估算金额： 2500万元。 商 2.4 招标范围： 包括完成管材、管件、阀门类、伸缩器、电磁流量计、法兰及其他等材料的供货（设 计、制造，含备品、备件、专用工器具等）、道装配（含出厂前组装、测试和检验、现场整体组装等）、 装卸、运输（含包装、保险）、验收，以及质量保证期内的维修、维护、保养、人员培训和其它相关伴随服务 等工作内容。 管 2.5 交货地点： 业主指定的施工现场。 2.6 交货期： 60日历天，计划开始交货日期：2026年9月30日（具体以实际通知为准）。 3.政府采购工程 国 3.投标人资格要求 3.1 本次招标允许投标人以投标货物的下列身份参加投标： 中 制造商 代理商（包括经销商、制造商下属销售子公司） 3.1.1 投标人为制造商应符合以下要求： （1）具备独立法人资格； 3.1.2 投标人为代理商应符合以下要求： （1）具备独立法人资格； （2）具备3PE防腐内热熔防腐钢管具有制造商授权书； 注：本招标项目中，一个制造商对同一品牌同一型号的货物，仅能委托一个代理商参加投标，否则 各相关投标均无效；同一品牌同一型号货物的制造商和代理商不得在本招标项目中投标，否则各相关投标均无 效。 （3）投标货物制造商应符合上述3.1.1项的规定。 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表第1.4.1 项内容。 3.3 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在本次招标公告同时在 重庆市公共资源交易监督网和 重庆市公共资源交易网（万州区）上发布。下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人 需在本次招标公告同时在 重庆市公共资源交易监督网和重庆市公共资源交易网（万州区）上发布。完成市场主 体信息登记以及CA数字证书办理，办理方式请参见本次招标公告同时在 重庆市公共资源交易监督网和重庆市公 共资源交易网（万州区）上发布。导航栏“主体信息”页面中“市场主体信息登网记”、“CA 数字证书办理”。 若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在本次招标公告同时在 重庆市公共资源交易监督网和重庆市公共资源交易网（万州区）上发布。本 项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发布至2026-08-25 17:00:00前。 4.3招标人应于2026-08-27 17:00:00前在本次招标公告同时在 重庆市公共资源交易监督网和重庆市公共资源交易网 务 （万州区）上发布。发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-11 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 商 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在本次招标公告同时在 重庆市公共资源交易监督网和重庆市公共资源交易网（万州区）上发 布。发布。[提示：依法必须招标项目的招标道公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 重庆长江水务有限公司 代理机构: 重庆大渝庆项目管理有限公司 重庆市万州区南滨大道1999号（财 重庆市渝北区重庆北站南广场汽车站西 地 址: 管地 址: 富广场）1幢B座第四层 投WORK北站大厦906室 邮 编: 404000 邮 编: 404000 项目负责人: 夏雨 项目负责人: 唐晓帆 国 电 话: 13896299659 电 话: 17723636501 传 真: 传 真: 电子邮箱: 电子邮箱: 598381793@qq.com 中 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市万州区发展和改革委员会 电 话: 023-58339255 2026年08月21日 信息来源:https://www.chinapipe.net/project/d3077724.html cqdingjiu 2026.08.24 12:31:42</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>排水钢管 DN150: 8.1千米；DN200: 29.3千米；DN250: 23千米；DN300: 5.1千米；DN400: 11.9千米；DN500: 6.8千米，材质为3PE防腐内热熔防腐钢管</t>
         </is>
       </c>
       <c r="N23" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>重庆, 废盐综合利用, 离子膜烧碱, 衬氟管道, 管件采购</t>
+          <t>重庆, 管材, 招标, 改造工程</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>重庆市益康环保工程有限公司永川分公司蒸汽管道改造项目询价采购公告</t>
+          <t>2026年度重庆分质供水有限公司不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈钢止回阀采购项目(包1、包2)(第二次)招标公告</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2048,7 +2036,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>其他/未识别</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2067,49 +2055,45 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>永川区</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>蒸汽管道改造</t>
+          <t>为重庆分质供水有限公司提供不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈钢止回阀等设备材料。</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>每个包合同暂估金额为110万元。</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>蒸汽管道</t>
+          <t>不锈钢可调式减压阀,不锈钢静音式止回阀,不锈钢微量排气阀,不锈钢闸阀,不锈钢表前阀,不锈钢球阀,Y型过滤器</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>重庆市益康环保工程有限公司永川分公司蒸汽管道改造项目询价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3076108.html cqdingjiu 2026.08.21 10:06:52 网 务 商 道 管 国 中</t>
+          <t>2026年度重庆分质供水有限公司不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈钢止回阀采购 项目(包1、包2)(第二次)招标公告 2026年度重庆分质供水有限公司不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈钢止回阀采购 项目（包1、包2）（第二次）招标公告 1.招标条件 网 本招标项目2026年度重庆分质供水有限公司不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈钢 止回阀采购项目（包1、包2）（第二次）（项目名称），招标人为重庆分质供水有限公司，招标项目资金来自企 业自筹（资金来源），项目已具备招标条件。现对本项目进行公开招标，诚邀有兴趣的潜在投标人参与投标。 务 2.项目概况与招标范围 2.1项目地点：招标人指定地点。 2.2项目概况：为重庆分质供水有限公司提供不锈钢闸阀、商不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈 钢止回阀等设备材料。 不锈钢类阀门按统一下浮比例进行报价（具体规格见招标文件第五章“供货要求”）。 道 注：①投标人可以任意选择1个或2个分包进行投标，但是同一个投标人只能中标一个分包，当同一个投标人同时 在2个分包中被评审确定为第一中标候选人的，则按照包1、包2的顺序，确定其为第一中标候选人，在其他分包 中不再被确定为中标候选人，按评审结果排序依次递补中标候选人。 管 ②投标人根据参投分包分别制作投标文件、分别填写投标文件中的项目名称，如下： 包1项目分包名称：2026年度重庆分质供水有限公司不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、 不锈钢止回阀采购项目（包1）（第二次）； 国 包2项目分包名称：2026年度重庆分质供水有限公司不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、 不锈钢止回阀采购项目（包2）（第二次）。 每个包合同暂估金额为110万（注：超出合同服务期或合同期间结算金额达到合同暂估金额时，合同自动终止)。 中 供货区域分别为： 包1：北区（涉及区域两江新区、沙坪坝区、北碚区及其他区县，区域可根据甲方工程需求调整）及重庆分质供 水有限公司市外所有项目。 包2：.南区（涉及区域渝中区、南岸区、巴南区、九龙坡区、大渡口区及其他区县，区域可根据甲方工程需求调 整）及重庆分质供水有限公司市外所有项目。 2.3招标范围：为重庆分质供水有限公司提供不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈 钢止回阀等设备材料 2.4货物清单 序号 名称 规格型号 压力等级 单位 备注 1 不锈钢可调式减压阀 DN15 1.6MPa 件 带压力表 2 不锈钢可调式减压阀 DN20 1.6MPa 件 带压力表 3 不锈钢可调式减压阀 DN25 1.6MPa 件 带压力表；提供样品一个 4 不锈钢可调式减压阀 DN32 1.6MPa 件 带压力表 5 不锈钢可调式减压阀 DN40 1.6MPa 件 带压力表 6 不锈钢可调式减压阀 DN50 1.6MPa 件 带压力表 7 不锈钢可调式减压阀 DN65 1.6MPa 件 带压力表 8 不锈钢可调式减压阀 DN80 1.6MPa 件 带压力表 9 不锈钢可调式减压阀 DN100 1.6MPa 件 带压力表 10 不锈钢静音式止回阀 DN15 1.6MPa 件 带压力表；含不锈钢螺栓 11 不锈钢静音式止回阀 DN15 2.5MPa 件 带压力表；含不锈钢螺栓 网 12 不锈钢静音式止回阀 DN20 1.6MPa 件 带压力表；含不锈钢螺栓 13 不锈钢静音式止回阀 DN20 2.5MPa 件 带压力表；含不锈钢螺栓 14 不锈钢静音式止回阀 DN25 1.6MPa 件 带压力表；含不锈钢螺栓 务 15 不锈钢静音式止回阀 DN25 2.5MPa 件 带压力表；含不锈钢螺栓 16 不锈钢静音式止回阀 DN32 1.6MPa 件 带压力表；含不锈钢螺栓 17 不锈钢静音式止回阀 DN32 2.5MPa 件 带压力表；含不锈钢螺栓 商 18 不锈钢静音式止回阀 DN40 1.6MPa 件 带压力表；含不锈钢螺栓 19 不锈钢静音式止回阀 DN40 2.5MPa 件 带压力表；含不锈钢螺栓 20 不锈钢静音式止回阀 DN50 1.6MPa 件 带压力表；含不锈钢螺栓 道 21 不锈钢静音式止回阀 DN50 2.5MPa 件 带压力表；含不锈钢螺栓 22 不锈钢静音式止回阀 DN65 1.6MPa 件 带压力表；含不锈钢螺栓 23 不锈钢静音式止回阀 DN65 2.5MPa 件 带压力表；含不锈钢螺栓 管 24 不锈钢静音式止回阀 DN80 1.6MPa 件 带压力表；含不锈钢螺栓 25 不锈钢静音式止回阀 DN80 2.5MPa 件 带压力表；含不锈钢螺栓 26 不锈钢静音式止回阀 DN100 1.6MPa 件 带压力表；含不锈钢螺栓 国 27 不锈钢静音式止回阀 DN100 2.5MPa 件 带压力表；含不锈钢螺栓 28 不锈钢微量排气阀 DN15 1.6MPa 件 29 不锈钢微量排气阀 DN20 1.6MPa 件 中 30 不锈钢微量排气阀 DN25 1.6MPa 件 31 不锈钢微量排气阀 DN32 1.6MPa 件 32 不锈钢微量排气阀 DN40 1.6MPa 件 33 不锈钢微量排气阀 DN50 1.6MPa 件 34 不锈钢闸阀 DN15 1.6MPa 件 35 不锈钢闸阀 DN20 1.6MPa 件 36 不锈钢闸阀 DN25 1.6MPa 件 37 不锈钢闸阀 DN25 2.5MPa 件 38 不锈钢闸阀 DN32 1.6MPa 件 39 不锈钢闸阀 DN32 2.5MPa 件 40 不锈钢闸阀 DN40 1.6MPa 件 41 不锈钢闸阀 DN40 2.5MPa 件 42 不锈钢闸阀 DN50 1.6MPa 件 43 不锈钢闸阀 DN50 2.5MPa 件 44 不锈钢闸阀 DN65 1.6MPa 件 含不锈钢螺栓 45 不锈钢闸阀 DN65 2.5MPa 件 含不锈钢螺栓 46 不锈钢闸阀 DN80 1.6MPa 件 含不锈钢螺栓 47 不锈钢闸阀 DN80 2.5MPa 件 含不锈钢螺栓 48 不锈钢闸阀 DN100 1.6MPa 件 含不锈钢螺栓 49 不锈钢闸阀 DN100 2.5MPa 件 含不锈钢螺栓 50 不锈钢表前阀 DN15 1.6MPa 件 51 不锈钢表前阀 DN20 1.6MPa 件 52 不锈钢表前阀 DN25 1.6MPa 件 网 53 不锈钢表前阀 DN40 1.6MPa 件 54 不锈钢表前阀 DN50 1.6MPa 件 55 不锈钢表前阀 DN65 1.6MPa 件 务 56 不锈钢表前阀 DN80 1.6MPa 件 57 不锈钢表前阀 DN100 1.6MPa 件 58 不锈钢球阀 DN15 1.6MPa 件 商 59 不锈钢球阀 DN20 1.6MPa 件 60 不锈钢球阀 DN25 1.6MPa 件 61 不锈钢球阀 DN32 1.6MPa 件 道 62 不锈钢球阀 DN40 1.6MPa 件 63 不锈钢球阀 DN50 1.6MPa 件 64 不锈钢球阀 DN65 1.6MPa 件 管 65 Y型过滤器 DN15 1.6MPa 件 66 Y型过滤器 DN15 2.5MPa 件 67 Y型过滤器 DN20 1.6MPa 件 国 68 Y型过滤器 DN20 2.5MPa 件 69 Y型过滤器 DN25 1.6MPa 件 70 Y型过滤器 DN25 2.5MPa 件 中 71 Y型过滤器 DN32 1.6MPa 件 72 Y型过滤器 DN32 2.5MPa 件 73 Y型过滤器 DN40 1.6MPa 件 74 Y型过滤器 DN40 2.5MPa 件 75 Y型过滤器 DN50 1.6MPa 件 76 Y型过滤器 DN50 2.5MPa 件 77 Y型过滤器 DN65 1.6MPa 件 78 Y型过滤器 DN65 2.5MPa 件 2.5 交货地点：招标人指定地点。 2.6 交货期：按业主要求进行供货。合同生效之日起2年或达到合同暂估金额时，合同自行终止。 2.7其他： 2.7.1投标人须按照采购清单要求提供相应型号数量的样品，投标样品须密封装箱，且在密封包装外贴样品一览表 （格式自拟），注明提供样品的投标人名称、生产厂家、品牌、名称、型号、数量等； 2.7.2每件样品上必须分别标明样品的投标人、生产厂家、品牌、名称、型号等（格式自拟），开标时同投标文件 一起提交，由评标委员会核验（提交地点见开标当日交易中心大厅展牌）。本项目第一中标候选人的样品不退还 （第二、三名中标候选人样品在中标通知书发出后5个工作日内退还），其余投标人的样品在评标结束后半小时 内当场退还，如不领取，自行负责。 2.7.3上述要求除递交的样品型号数量应相符外，其余不作为废标的条款，但投标人应主动配合按此要求进行递交。 3.投标人资格要求 3.1 投标人必须是按照国家法律法规设立的，并在中国注册的，具有法人地位的企业；投标人为投标货物的制造 商、代理商或经销商。 网 3.2 投标人还应在业绩、资金、人员等方面具有相应的供货能力，详见招标文件第二章投标人须知前附表 第1.4.1项内容。 务 3.3本次招标不接受联合体投标。 4.招标文件的获取 4.1 本项目招标不需报名，凡有意参加投标者，请于2026年8月21日起在重庆市公共资源交易网（www.cqggzy.com） 下载本招标项目的招标文件等投标截止时间前公布的所有商相关资料，不管投标人下载与否，招标人和招标代理 机构都视为投标人收到以上资料并全部知晓有关招标过程和事宜，由此产生的一切后果由投标人自负。 4.2、招标文件每份售价1000元，售后不退。投标单位在递交投标文件时通过扫描二维码方式支付购买招标文件 的费用，否则招标人和招标代理机构拒绝接收道其投标文件。 5.投标文件的递交 5.1、投标文件递交的截止时间（投标截止时间，下同）为2026年9月14日11时00分（北京时间）前，地点为重庆 管 市渝北区青枫北路6号渝兴广场B10栋2层重庆市公共资源交易中心开标厅（具体房间见开标当天大厅展牌）。 5.2、逾期送达的、未送达指定地点的或者不按照招标文件要求密封的投标文件，招标人将予以拒收。 6.发布公告的媒介 国 本次招标公告在重庆市公共资源交易网(www.cqggzy.com)上发布。 7.联系方式 中 招 标 人：重庆分质供水有限公司 地 址：重庆市两江新区水务大厦 联 系 人：张老师 电 话：17783738201 招标代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市两江新区嘉华路36号水务大厦 联 系 人：罗辑 电 话：18223151922（工作时间9:00-12:00；14：00-17:00其余时间请勿致电） 2026年度重庆分质供水有限公司不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈钢止回阀采 购项目（包1）（第二次） 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公 中国民生银行股份有限公司重庆分行 9902001764108013 司 重庆联合产权交易所集团股份有限公 重庆农村商业银行股份有限公司沙坪 0304010120010028835008268 司 坝支行 重庆联合产权交易所集团股份有限公 重庆三峡银行九龙坡支行 9696801051298012 司 重庆联合产权交易所集团股份有限公 中信银行重庆上清寺支行 3111230034020042416 司 网 重庆联合产权交易所集团股份有限公 中国农业银行股份有限公司重庆自由 312601010400083780000005565 司 贸易试验区分行 重庆联合产权交易所集团股份有限公 招商银行股份有限公司重庆分行 123904808710630019269 司 务 重庆联合产权交易所集团股份有限公 中国建设银行股份有限公司重庆渝中 6232813760000632694 司 支行 重庆联合产权交易所集团股份有限公 重庆银行股份有商限公司七星岗支行 15010202900420146618927 司 信息来源:https://www.chinapipe.net/project/d3077649.html 道 cqdingjiu 2026.08.24 12:31:42 管 国 中</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>DN15 1.6MPa 件 带压力表；含不锈钢螺栓</t>
         </is>
       </c>
       <c r="N24" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>重庆, 蒸汽管道, 改造项目, 询价采购</t>
+          <t>重庆, 不锈钢闸阀, 不锈钢表前阀, 不锈钢减压阀, 不锈钢排气阀, 不锈钢止回阀, 管材招标</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>南岸区融侨大道、江南大道片区2023年排水管网改造项目(三标段)招标计划表</t>
+          <t>酉阳县桃花源新城供水工程管网安装工程专业分包采购公告</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2140,32 +2124,32 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>南岸区</t>
+          <t>酉阳土家族苗族自治县</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>包括改造市政混接点194个，改造管网8582米，缺陷管网开挖修复1355米，非开挖修复8679米。</t>
+          <t>酉阳县桃花源新城供水工程管网安装工程专业分包</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>总投资概算未明确具体金额，但合同预估金额为6600万元。</t>
+          <t>暂无明确资金信息</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>排水管网改造</t>
+          <t>管网安装工程</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>南岸区融侨大道、江南大道片区2023年排水管网改造项目(三标段)招标计划表 重庆市工程建设项目招标计划表 项目名 南岸区融侨大道、江南大道片区 2023年排水管网改造项目（三标段） 称 网 招标法 人或招 重庆市南岸区城市建设发展（集团）有限公司 标人名称 （盖章） 务 项目批 准文件 南岸发改〔2024〕304《南岸区融侨大道、江南大道片区2023年排水管网改造项目总投资概算的批复》 及文号 主要建 包括改造市政混接点194个，改造管网8582米，商管径d300~d1500;缺陷管网开挖修复1355米，管 设内容 径d300~d600;非开挖修复8679米，管径d300~d1200。 招标文件 拟交 合同预估 招标内 招标 序号 招标项目名称 计划发布 易场 金额(万 备注 道容 方式 时间 所 元) 51处雨 污混错 重庆 招标项 接点位 管 市公 目 改 南岸区融侨大道、江南大道片区 2023年排 公开 共资 1 造，1082 2026-08 6600.00 水管网改造项目（三标段） 招标 源交 个管网 易中 三四级 国 心 缺陷修 复。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 中 信息来源:https://www.chinapipe.net/project/d3076097.html cqdingjiu 2026.08.21 10:06:52</t>
+          <t>酉阳县桃花源新城供水工程管网安装工程专业分包采购公告 酉阳县桃花源新城供水工程管网安装工程专业分包 采购公告 一、采购概况 1.采购名称：【酉阳县桃花源新城供水工程管网安装工程专业分包】 网 2.工程概况： 工程名称：酉阳县桃花源新城供水工程 务 项目地址：重庆市酉阳县桃花源新城 建筑规模：【新建5万吨m3/d的水厂一座（含水厂进场道路工程、水厂总图工程、水厂常规处理工程、泥沙处理 工程、水厂电气自控安装工程、水厂厂前办公楼建筑工程商）；5万吨m3/d的取水泵站一座（含泵站的土建工程、 设备采购及安装工程、泵站外电源实施工程）；铺设原水输水管网总长度约16.7公里（含管网土建及安装工程、 管材及管件采购工程）；配套建设新城供水主管约77km（含管网土建及安装工程、管材及管件采购工程）】。 3.标段划分：【本工程仅一个标段】。 道 4.采购内容：【酉阳县桃花源新城供水工程管网安装工程】。 5.质量要求：【达到一次性验收合格标准，工程质量符合国家现行相关规范、规定标准】。 管 6.工期要求：【暂定开工日期：2026年9月20日，竣工日期2026年11月20日，总工期61日历天。实际开竣工日期以 发包人要求为准，分包人应无条件配合且不得对此安排提出异议或索赔】。 7.安全文明要求：【工国程质量符合强制性质量标准，符合国家和重庆市现行有关施工质量验收规范要求，并达到 合格标准，一次验收质量达到合格等级满足承包人质量和管理行为的要求,同时满足项目部技术质量交底要求， 通过验收。质量管理目标：创重庆市优质工程“巴渝杯”。具体施工标准满足《中建四局交通公司房屋建筑项 目安全标准化图集（2026版）》。 中 8.付款条件：【1、本工程无预付款；2、按月支付，按每月完成合格实物量的75%支付进度款；3、合同范围内所 有工程完工确认合格后调整支付比例至85%；4、结算完成后付至分公司终审值的97%，剩余3%质量保证金在本 项目工程验收合格满两年后扣除维修费用且完善甲方请款流程后一次性无息返还。】 9.拟选定成交单位数：【 1 】。 二、报价人资格 1.报价人报名前需通过“云筑网”（网址：https://jicai.yzw.cn/home）认证并进入中建系统合格分供方资源库，经 采购人资格审查合格后方可参与报价。 2.报价人需具备以下基本条件：【具备营业执照、市政公用工程施工总承包贰级及以上资质、安全生产许可证、 有类似项目工程业绩（报名时需上传以上相关附件资料）资信良好，有一定资金能力、人员结构完善、管理能 力强等】。 3.本次采购不接受联合体报价。 4.如报价单位提供虚假资料的，任何时候一经发现，取消其报价资格。 三、报价报名 1.报名时间：【截至2026年8月23日9时，以“云筑网”平台显示时间为准】，逾期不再接受报名。 2.报名方式：通过“云筑网”进行网上报名，不接受其他方式报名。 3.已在“云筑网”完成分供方注册的报价人，可直接在“云筑网”签收采购公告后报名。 未在“云筑网”注册的报价人，需先进行注册，提交以下资料【包括企业营业执照、资质证书、安全生产许可 证、银行开户许可证、主要业绩材料及证明、法定代表人身份证明及身份证等】，经采购人审查合格并完成分 供方认证后，方可报名。 4. 报价保证金：本次报价的报价保证金为【1000】元，报价人应于报价截止日24小时前缴纳。 5.首轮响应文件开启后无条淘汰报价最高的前10%且不少于1家单位（小数向上取整）。 四、发放采购文件 网 1.采购人通过“云筑网”对资格审查合格的报价人发放采购文件。 2.发放时间：见云筑网要求时间。 务 3.联系人：现场联系人：苏忠明 联系方式： 18608774750 ，分公司成本管控中心：【赵经理】，联系方式： 【15925129017】，联系地址：【昆明市官渡区新亚洲体育场星都总部基地48栋 】。 4.其他未尽事宜详见采购文件。 商 采购人：中国建筑第四工程局有限公司 道 日 期：2026年8月20日 管 信息来源:https://www.chinapipe.net/project/d3077567.html cqdingjiu 2026.08.24 12:31:43 国 中</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>管网：8582米；缺陷管网：1355米</t>
+          <t>铺设原水输水管网总长度约16.7公里，配套建设新城供水主管约77km</t>
         </is>
       </c>
       <c r="N25" t="n">
@@ -2173,14 +2157,14 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>重庆, 排水管网改造, 资金情况, 产品种类</t>
+          <t>酉阳县桃花源新城供水工程, 管网安装工程专业分包, 重庆, 管网安装工程</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购公告</t>
+          <t>重庆市巴南区龙洲湾片区城市污水管网更新改造工程施工招标公告</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2211,47 +2195,47 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>永川区</t>
+          <t>巴南区</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、综合楼、生产建（构）筑物以及附属建筑物等。</t>
+          <t>本项目改建及修复管网总长度约30.98公里，雨污水错混接改造以及管网缺失改造DN300-DN600排水管网约2.0公里；修复DN300-DN1000管道约28.98公里。</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>项目合同额1.7亿元</t>
+          <t>项目总投资金额：10063.6万元，本次招标项目合同估算金额：6033.535232万元</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>钢筋混凝土排水管</t>
+          <t>排水管网</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购公告 永川三教水厂项目 已具备采购条件，现公开邀请供应商参加询比采购活动。 1.采购项目简介 1.1 采购项目名称：中交一公局重庆工程有限公司2026年8月钢筋混凝土排水管询比采购。 1.2 采购方案编号：FA00000663117。 网 1.3 采购人：中交一公局重庆工程有限公司。 1.4 采购代理机构：/。 务 1.5 采购项目资金：已落实 1.6 采购项目概况： 商 永川三教水厂项目：项目位于永川区三教镇，项目占地面积41673.42㎡（62.51亩），总建筑面积6078.71㎡，新建 净水厂1座，规模5万吨/天，新建厂外管网4.6km（DN200～DN1000），配套建设净水处理系统、排泥水处理系统、 综合楼、生产建（构）筑物以及附属建筑物等。项目合同额1.7亿元，工期450天。 道 项目地址：重庆市永川区。 2.采购范围及相关要求 管 2.1 采购范围：钢筋混凝土排水管。 2.2 交货期：2026年9月-2026年12月。 2.3 交货地点：重庆市永国川区项目指定地点。 2.4 物资质量标准：满足《混凝土和钢筋混凝土排水管》（GB/T 11836-2023）的相关要求。 3.供应商资格要求 中 3.1 供应商应依法设立且满足如下要求： （1）资质要求：本次询比采购要求供应商须是在中华人民共和国境内依法注册，具有合法有效的营业执照、税 务登记、组织机构代码等证件，具有独立法人资格、具有采购物资生产经营范围的生产商或代理商（销售商）。 （2）财务要求：供应商必须是经税务部门注册登记核准的纳税人，有依法纳税的良好记录。 （3）业绩要求：无。 （4）信誉要求：无不良履约记录、未列入工程所在地质量监督部门和中国交建、中交一公局集团企业黑名单。 因质量原因被交通部质监站通报，正在进行整改的生产厂家和产品不得参与投标。生产商或代理商（销售商） 具有良好的社会信誉，近3年内没有与骗取合同有关的犯罪或严重违法行为而引起的诉讼和仲裁；近3年不曾在合 同中严重违约或被逐；财产未被接管或冻结，企业未处于禁止或取消投标状态；在最高人民法院、信用中国 （www.creditchina.gov.cn）或各级信用信息共享平台查询拟入库单位无不良行为记录。 （5）其他要求：无。 3.2 供应商不得存在下列情形之一： （1）处于被责令停产停业、暂扣或者吊销执照、暂扣或者吊销许可证、吊销资质证书状态； （2）进入清算程序，或被宣告破产，或其他丧失履约能力的情形； （3）已列入黑名单，且未解除限制期限； （4）其他：无。 4.供应商报名 4.1 有意参加询比采购活动的单位，请于2026年8月19日15时00分至2026年8月26日17时00分（北京时间，下同，法 定公休日、节假日不休），登录“中交招采网”（网址：https://zjzcw.iccec.cn）进行报名并下载采购文件。 4.2 已在网并且已通过采购人层级供应商或已增加采购人为合作单位的供应商、上级供应商可直接参与询比采 网 购。在网平级单位供应商未增加采购人为合作单位需进行合作意向申请通过后参与询比采购。 未注册“中交招采网”的单位需先进行注册，推荐单位或合作意向单位选择采购人，审核通过后方可参与询比 采购。 务 5.供应商报价 5.1 报价结束（递交响应文件截止）时间为2026年8月26日17时00分。 商 5.2 供应商应在报价结束时间前，登录“中交招采网”进行线上报价并上传电子响应文件。逾期未完成上传的电 子响应文件，采购人将拒收。 5.3电子采购的供应商响应文件由线上电子报价道表及附件共同组成。当电子报价表与附件内容冲突时，以线上电 子报价表的数据为准。 6.开标 管 6.1 开标时间：与报价结束时间相同。 6.2 开标地点：本次采购在“中交招采网”平台线上开标，不举办现场开标。 国 7.发布公告的媒介 本询比采购公告在 “中交招采网” 上发布。 中 8.评审办法 本项目评审办法采用 经评审的最低价法 。 9.合同主要条款 9.1 付款条件：按月结算，上月11日至本月10日为一个结算对账期，乙方必须按照甲方要求开具合规的增值税专 用发票，无发票不予付款。结算完成后1个月内支付已结算金额的70%，剩余30%货款在结算完成后3个月内支付。 付款方式为银行转账，甲方有权采用票据支付或者供应链支付的方式支付货款，因此产生的费用包含在综合单 价中，乙方不得因此调价和索赔。如遇业主支付不及时，乙方应予理解。 9.2 履约保证金的递交： （1）R不要求递交 （2）要求递交，保证金金额：/，保证金形式：/，其他形式：/ 。 10.监督机构 监督机构名称： 中交一公局重庆工程有限公司审计部 11.成交供应商平台服务费缴纳说明 为进一步提升电子采购平台服务质量，优化运营流程，保障双方合作更加顺畅高效，对参与我司采购活动并成 功中标的供应商分档收取服务费。具体费用以中标通知书中同步生成的服务费订单为准，订单将通过“中交招 采网”发送，发送后10天内需完成费用缴纳。缴费过程中如有问题，请联系400-676-5885，中标服务费请按7咨询。 11.1 收费标准 按照包件分档进行收费，收费标准按以下中标金额进行收取： 网 （1）在100万元（含）至200万元之间的，每次收取100元； （2）在200万元（含）至1000万元之间的，每次收取500元； （3）在1000万元（含）至3000万元之间的，每次收取1000元； 务 （4）在3000万元（含）至1亿元之间的，每次收取3000元； （5）在1亿元（含）以上的，每次收取5000元。 商 11.2 支付流程 （1）通知推送：中标结果发布后，系统自动推送缴费通知（含应缴金额及支付链接）； 道 （2）费用查询：供应商登录“中交招采网—供应商协同—服务费”模块查看待支付费用； （3）在线支付：支持对公银行转账或在线支付，支付成功后生成电子凭证； 管 （4）发票开具：支付完成后5个工作日内，系统自动生成“技术服务费”电子发票，供应商可在“中交招采网— 供应商协同—服务费—发票查询”模块获取。 12.其他 国 / 。 13.联系方式 中 采 购 人：中交一公局重庆工程有限公司 地 址：重庆市江北区创富路5号 邮 编：361021 联 系 人：汪仁宽 电 话：13527572392 电子邮件：1176245792@qq.com 项目联系人及电话： 序号 项目名称 联系人 联系电话 1 永川三教水厂项目 高博 17788661005 中交一公局重庆工程有限公司 2026年8月19日 物资信息 序号 设备物资名称 设备物资说明 税率 单位 网 1 钢筋混凝土排水管 2000mm Ⅲ级 承插口 13% 米 信息来源:https://www.chinapipe.net/project/d3076078.html 务 cqdingjiu 2026.08.21 10:06:52 商 道 管 国 中</t>
+          <t>重庆市巴南区龙洲湾片区城市污水管网更新改造工程施工招标公告 重庆市巴南区龙洲湾片区城市污水管网更新改造工程施工招标公告 1.招标条件 本招标项目 重庆市巴南区龙洲湾片区城市污水管网更新改造工程 已由 重庆市巴南区发展和改革委员会 以 巴南发改审发〔2026〕103号 批准建设，项目业主为重庆市城镇排水事务中心，代建业主为重庆水务环境 控股集团管网有限公司，建设资金来自 争取上级补助资金及区级财政资金配套 ，项目出资比例为100%，招 标人为重庆水务环境控股集团管网有限公司。项目已具备招标条件，现对该项目的施工进行公开招标，评标办 法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：重庆市巴南区龙洲湾街道 2.2 项目概况与建设规模：本项目改建及修复管网总长度约30.98公里，雨污水错混接改造以及管网缺失改 造DN300-DN600排水管网约2.0公里；修复DN300-DN1000管道约28.98公里。危大工程主要涉及深基坑及有限空 务 间作业，其中深基坑对应部位与环节为：加井修复、裂管工作井部分；有限空间作业主要为非开挖修复工程。 2.3 本项目工程总投资金额：10063.6万元 商 本次招标项目合同估算金额：6033.535232万元 2.4 招标范围：招标人提供的工程量清单及编制说明、设计图纸、技术文件等包括的所有工作内容，包括但不 限于：施工图所示范围内的土石方工程，管网改扩建，管道缺陷修复，路面破除恢复、相关附属设施破除及恢 复、行道树的移栽等所有工作内容。具体详见道招标人提供的工程量清单。 2.5 工期要求：270日历天 缺陷责任期要求：24个月 管 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 国 3.1 是否属于政府采购工程：是 3.2 是否专门中面向中小企业预留：是 专门面向中小企业预留的实施方式：本项目以合同分包形式面向中小企业，分包给中小企业的合同份额需达 到40%以上。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件、工程量清单、 电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理， 办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。 若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 布至2026-08-26 17:00:00前。 5.3招标人应于2026-08-28 23:59:59前在重庆市公共资源交易网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-20 10:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在“重庆市公共资源交易监督网”和“重庆市公共资源交易网”发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 网 招 标 人: 重庆水务环境控股集团管网有限公司 代理机构: 重庆市工程管理有限公司 地 址: 重庆市渝中区重庆总部城A区11栋 地 址: 重庆市两江新区五简路2号重咨大厦A座 邮 编: 邮 编: 务 项目负责人: 程鹏 项目负责人: 鲜颖 电 话: 023-63995075 电 话: 17323966277 传 真: 传 真商: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 道账 号: 监督部门: 重庆市巴南区发展和改革委员会 电 话: 023-66221670 管 2026年08月21日 重庆市巴南区龙洲湾片区城市污水管网更新改造工程施工 户名 开户行 投标保证金账号 国 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020004772 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000697127 支行 中 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051303175 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000013052 贸易试验区分行 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630016759 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146619084 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835012249 坝支行 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764158547 信息来源:https://www.chinapipe.net/project/d3077506.html cqdingjiu 2026.08.24 12:31:43</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>厂外管网：4.6km；钢筋混凝土排水管：2000m</t>
+          <t>DN300-DN600排水管网约2.0公里；修复DN300-DN1000管道约28.98公里</t>
         </is>
       </c>
       <c r="N26" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 钢筋混泥土排水管, 永川三教水厂项目</t>
+          <t>重庆, 管材, 招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>长江流域云阳青龙段污水管网一体化建设项目招标计划表</t>
+          <t>土桥、宗申、界石排水箱涵清污分流改造项目施工招标公告</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2280,49 +2264,45 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>云阳县</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。</t>
+          <t>本项目改建及修复管网总长度约30.63公里，雨污水错混接改造以及管网缺失改造DN300-DN800排水管网约6.35公里；修复DN300-DN1200管道约24.28公里。</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>合同预估金额：9100.00万元</t>
+          <t>项目总投资金额：9551.19万元，本次招标项目合同估算金额：5383.510617万元</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>污水管网</t>
+          <t>排水管网</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>长江流域云阳青龙段污水管网一体化建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 长江流域云阳青龙段污水管网一体化建设项目 招标法人或 招标人名称 云阳县青江环境综合整治有限公司 网 （盖章） 项目批准文 云阳发改资环【2025】55号 件及文号 务 主要建设内 新建污水管网55.5千米，其中DN200管网12千米、DN300管网24千米、DN400管网19.5千米等。 容 招标方 招标文件计 拟交易场 合同预估金额 序号 招标项目名称 招标内容 备注 式 划发布时间 所 (万元) 商 长江流域云阳 新建污水管网55.5千米， 重庆市公 青龙段污水管 其中DN200管网12千 公开招 共资源交 1 网一体化建设 米、DN300管网24千 2026-08 9100.00 标 易中心云 项目EPC总承 米、DN40道0管网19.5千 招标项目 阳分中心 包 米等。 新建污水管网55.5千米， 长江流域云阳 重庆市公 其中DN200管网12千 青龙段污水管 公开招 共资源交 2 管米、DN300管网24千 2026-08 140.00 网一体化建设 标 易中心云 米、DN400管网19.5千 项目监理 阳分中心 米等监理。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 国 信息来源:https://www.chinapipe.net/project/d3075867.html cqdingjiu 2026.08.21 10:06:53 中</t>
+          <t>土桥、宗申、界石排水箱涵清污分流改造项目施工招标公告 土桥、宗申、界石排水箱涵清污分流改造项目施工招标公告 1.招标条件 本招标项目 土桥、宗申、界石排水箱涵清污分流改造项目 已由 重庆市巴南区发展和改革委员会 以 巴南发 改审发〔2026〕102号 批准建设，项目业主为重庆市城镇排水事务中心，代建业主为重庆水务环境控股集团管网 有限公司，建设资金来自 争取上级补助资金及区级财政资金配套 ，项目出资比例为100%，招标人为重庆水务 环境控股集团管网有限公司。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估 法。 2.项目概况与招标范围 网 2.1 建设地点：重庆市巴南区花溪、李家沱街道及界石镇 务 2.2 项目概况与建设规模：本项目改建及修复管网总长度约30.63公里，雨污水错混接改造以及管网缺失改 造DN300-DN800排水管网约6.35公里；修复DN300-DN1200管道约24.28公里。项目存在危大工程，危大工程主要 涉及深基坑及有限空间作业，其中深基坑对应部位与环节为：加井修复、微顶管井施工，裂管工作井部分；有 限空间作业主要为箱涵内施工管网及非开挖修复工程。 商 2.3 本项目工程总投资金额：9551.19万元 道 本次招标项目合同估算金额：5383.510617万元 管 2.4 招标范围：招标人提供的工程量清单及编制说明、设计图纸、技术文件等包括的所有工作内容，包括但不限 于：施工图所示范围内的土石方工程，管网改扩建，管道缺陷修复，路面破除恢复、相关附属设施破除及恢复、 行道树的移栽等所有工国作内容。具体详见招标人提供的工程量清单。 2.5 工期要求中：270日历天 缺陷责任期要求：24个月 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 3.1 是否属于政府采购工程：是 3.2 是否专门面向中小企业预留：是 专门面向中小企业预留的实施方式：本项目以合同分包形式面向中小企业，分包给中小企业的合同份额需达 到40%以上。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质； 网 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 务 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿商。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人道在投标前可在重庆市公共资源交易网下载招标文件、工程量清单、 电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理， 办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。 若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 管 布至2026-08-26 17:00:00前。 5.3招标人应于2026-08-28 23:59:59前在重庆市公共资源交易网发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-20 10:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登国录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公中告同时在“重庆市公共资源交易监督网”和“重庆市公共资源交易网”发布。[提示：依法必须招标 项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆水务环境控股集团管网有限公司 代理机构: 重庆市工程管理有限公司 地 址: 重庆市渝中区重庆总部城A区11栋 地 址: 重庆市两江新区五简路2号重咨大厦A座 邮 编: 邮 编: 项目负责人: 程鹏 项目负责人: 鲜颖 电 话: 023-63995075 电 话: 17323966277 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市巴南区发展和改革委员会 电 话: 023-66221670 2026年08月21日 土桥、宗申、界石排水箱涵清污分流改造项目施工 户名 开户行 投标保证金账号 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000012057 贸易试验区分行 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020039234 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764235311 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146612313 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 网9696801051301643 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630014874 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835008473 坝支行 务 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000764299 支行 商 水施-02土桥、宗申、界石排水箱涵清污分流改造项目-管网修复子项附件详见链 接：https://www.cqggzy.com/trade/014001/b09ced5a-3672-45a5-94be-2dcdcab6972e?categoryNum=014001001002 水施-01土桥、宗申、界石排水箱涵清污分流道改造项目-管网改造子项附件详见链 接：https://www.cqggzy.com/trade/014001/b09ced5a-3672-45a5-94be-2dcdcab6972e?categoryNum=014001001002 信息来源:https://www.chinapipe.net/project/d3077435.html cqdingjiu 2026.08.24 12:31:44 管 国 中</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>DN200管网：12千米；DN300管网：24千米；DN400管网：19.5千米；污水管网：55.5千米</t>
+          <t>排水管网修复</t>
         </is>
       </c>
       <c r="N27" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 污水管网, 资金情况, 产品种类</t>
+          <t>重庆, 排水管网, 管网修复, 管网改造</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>中国电建水电四局华中公司重庆轨道交通17号线一期5标项目雨污水排水迁改工程施工劳务分包采购项目公开询比采购公告</t>
+          <t>巫溪县花台片区川主、农坡等5个村迁建区特色农业抗旱供水保障工程勘察设计招标计划表</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2332,7 +2312,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2351,45 +2331,49 @@
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>巫溪县</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3站5区间的土建）：高龙大道站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子站区间、石家院子站～终点区间、7/17号线联络线区间。采购范围为雨污水排水迁改工程。</t>
+          <t>主要整治孝子溪大堰水渠约17.5km;新建孝子溪水库引水管道约17.5km,其中需新建引水隧洞内置管道约1.5km;新建柑橘基地管网约3.25km;改建6000m蓄水池1座；新建2000m蓄水池2座；新建1000m蓄水池1座；新建500m³蓄水池2座；新建柑橘基地滴灌系统1套。</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>建设资金来源已落实，但具体资金数额未明确。</t>
+          <t>合同预估金额为340万元（含水土保持施工图设计）。</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>雨污水排水迁改工程</t>
+          <t>勘察设计服务</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>中国电建水电四局华中公司重庆轨道交通17号线一期5标项目雨污水排水迁改工程施工劳务分包采购项目公开询 比采购公告 询比采购公告 采购编号： PC-0104-26J6-FP0895 一、采购条件 受中国水利水电第四工程局有限公司重庆轨道交通17号线一期5标项目委托，中水电四局华中（武汉）工程有限 公司以公开询比方式采购重庆轨道交通17号线一期5标雨污水排水迁改工程项目网，建设资金来源已落实。目前项 目已具备采购条件，现进行公开询比采购。 二、项目概况、采购范围 务 1、项目概况：重庆轨道交通17号线一期5标段包含金凤北站（不含）～终点（3 站5 区间的土建）：高龙大道 站、斑竹林站、石家院子站、金凤北站～高龙大道站区间、高龙大道站～斑竹林站区间、斑竹林站～石家院子 站区间、石家院子站～终点区间、7/17号线联络线区间。 2、采购范围： 商 （1）雨污水排水迁改工程 （2）工程招标范围工作内容：17号线一期5标道中高龙大道站、斑竹林站及高斑竖井位于城市既有道路下方，设计 采用明挖法施工。为保证市政排水管网的正常使用，在明挖施工前需对既有管网进行临时迁改，车站结构施工 后进行恢复。施工PE钢带管长度2387米、B型排水管长度2799m、钢筋混凝土管127米，检查井239座劳务部分。 （3）施工内容详见工程量清单，以及为完成此项工程而做的一切工作。 管 3、计划工期:计划开工日期：2026年9月25日（具体时间以采购人通知为准），计划完工日期：2027年 12 月25 日； 合同工期总日历天数为457天。 4、质量要求：符合《国给水排水管道工程施工及验收规范》（GB 50268）、《混凝土结构工程施工质量验收规范》 （GB 50204）、《城镇道路工程施工与质量验收规范》（CJJ 1-2008）以及项目所在地最新的相关法规、标准和 图集。工程质量全面达到设计要求和标准，其中：验收合格率 100%，优良率达 90%以上，工程综合验收质量评 定达优良标准。 中 5、付款方式：采用银行转账/支票支付工程价款，月度结算完成具备付款条件后30天内工程进度款支付比例约定 为扣除各项保证金及费用后应付价款不低于65%；清算完成并签订《退场协议》后30天内工程进度款支付比例约 定为扣除各项保证金及费用后应付价款不低于80%；清算完成并签订《退场协议》后一年内工程进度款支付比例 约定为扣除响应人缺陷责任等相关费用后应付价款不低于90%；清算完成并签订《退场协议》，办理完成保证金 退还手续后两年内，工程进度款支付比例约定为扣除响应人缺陷责任等相关费用后应付价款的100%。 6、其他：无。 三、响应人资格要求 响应人必须满足以下全部资格要求： （1）资质要求：施工劳务不分等级 （2）主要人员要求:授权委托人（如有）及项目经理、专职安全员应提供社保和劳动合同。其中劳动合同至少提 供首、末两页，并且包含有关人员的详细信息;社保证明应提供响应截止时间前三个月的社保缴纳记录。 （3）安全三类人员要求:应提供企业主要负责人安全A证、项目经理B证、专职安全员C证。 （4）响应人具有良好的银行资信和商业信誉，没有处于被责令停业，财产被接管、冻结、破产状态。 （5）响应人应具有 雨污水排水迁改 工程的施工业绩，在近 5年内(2021年7月-2026年7月内签订)的施工合同不少 于 1 个，且签订单项合同金额均在 100 万元以上（应附成交通知书和（或）合同扫描件）。 （6）其它要求:无。 （7）本次采购不接受联合体响应。 四、采购文件的获取 凡满足本公告规定资格要求并有意参加的响应人，请于2026年8月22日10时00分前在中国电建采购招标数智化平台 （https://bid.powerchina.cn/bidweb/#/login，以下简称“数智化平台”）获取采购文件，采购文件免费提供。 五、响应文件的递交 1、响应文件递交的截止时间（响应截止时间，下同）为2026年8月26日10时30分网（北京时间），响应人应在截止 时间前通过数智化平台递交电子响应文件。 2、本次采购将通过数智化平台全程在线开展，电子响应文件的加密、提交等流程须响应人在线进行操作。响应 人须提前办理数字证书用于在线递交响应文件，办理方式详见数智化平台首页，并严格按照要求进行在线操作， 务 因操作流程失误造成的递交失败将由响应人自行承担后果。 3、开启由“数智化平台”在响应截止时间后自动对响应文件进行解密，响应人及时关注开启结果。 4、响应截止时间如有变动，采购人将及时通知已获取采商购文件的响应人。 六、发布公告的媒介 本次询比采购公告同时在中国电建阳光采购网道（https://bid-zb.powerchina.cn）上发布。 七、评审办法 采用综合评估法。 管 八、联系方式 采 购 人： 中水电四局华中（武汉）工程有限公司 国 地 址： 湖北省武汉市江岸区塔子湖东路健美街30号立城中心商务楼13、14层 邮 编： 430014 中 联 系 人： 王飞 电 话： 15827222587 电子邮箱： 107830343@qq.com 九、提出异议的渠道和方式 单位名称： 中水电四局华中（武汉）工程有限公司 电 话： 17708178186 电子邮箱： sjhzgsjw@163.com 十、纪检监督机构 响应人或者其他利害关系人认为本次采购活动存在违规违纪行为的，可以书面形式向中国水利水电第四工程局 有限公司中水电四局华中（武汉）工程有限公司纪委办公室（联系方式：17708178186）提出投诉。 2026年8月 19 日 报价网址:https://bid.powerchina.cn/notice/detail?id=2409510708 信息来源:https://www.chinapipe.net/project/d3075750.html cqdingjiu 2026.08.21 10:06:53 网 务 商 道 管 国 中</t>
+          <t>巫溪县花台片区川主、农坡等5个村迁建区特色农业抗旱供水保障工程勘察设计招标计划表 重庆市工程建设项目招标计划表 项目 巫溪县花台片区川主、农坡等5个村迁建区特色农业抗旱供水保障工程勘察设计 名称 招标 法人 或招 标人巫溪县宁之源建设开发（集团）有限公司 名称 网 （盖 章） 项目 批准 文件 及文 号 务 主要 整治孝子溪大堰水渠约17.5km;新建孝子溪水库引水管道约17.5km,其中需新建引水隧洞内置管道约1.5km;新建柑橘基地管网约3.25km;改建6000m蓄水池1座；新建2000m蓄水池2座；新建1000m蓄水池1座；新建500m3 建设 蓄水池2座；新建柑橘基地滴灌系统1套 内容 序号 招标项目名称 招标内容 招标方式 招标文件计划发布时间 拟交易场所 合同预估金额(万元) 备注 招标 巫溪县花台片区川主、农坡 初步设计阶段勘察设计、施工 重庆市公共资源 项目1 等5个村迁建区特色农业抗旱 图阶段勘察设计、水土保持方案 公开招标 2026-09 交易中心巫溪分 340.00 （含水土保持施工图设计）、 供水保障工程勘察设计 洪水影响评价、水资源论证 商中心 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3078207.html cqdingjiu 2026.08.24 12:31:44 道 管 国 中</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>型排水管：2799m；钢筋混凝土管：127米；检查井：239座</t>
+          <t>孝子溪水库引水管道：17.5km；其中需新建引水隧洞内置管道：1.5km；柑橘基地管网：3.25km</t>
         </is>
       </c>
       <c r="N28" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>重庆, 轨道交通, 雨污水排水迁改, 施工劳务分包</t>
+          <t>重庆, 管材招标, 勘察设计, 资金情况, 产品种类</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>万州区2026年超长期特别国债高标准农田建设项目拟进行预制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜的信息公告</t>
+          <t>涪陵区李渡新区水厂工程(一期)施工招标公告</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2399,7 +2383,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>房建</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2420,47 +2404,47 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>万州区</t>
+          <t>涪陵区</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>本项目涉及预制钢筋砼管、成品混凝土仿木栏杆等材料的采购。</t>
+          <t>涪陵区李渡新区水厂工程(一期)设计水量目标为10万m/d，二期水量目标为20万m/d，采用混凝、沉淀、过滤、消毒常规水处理工艺。一期工程项目主要建设内容包括取水及原水输送工程、净水厂工程、配水工程三部分。</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>建设资金为国债资金，项目出资比例为100%。具体预算金额未在文本中明确列出。</t>
+          <t>项目业主为重庆水务环境控股集团渝东自来水有限公司，建设资金来自争取三峡后续工作专项资金、银行贷款和业主自筹等，项目出资比例为100%。</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>预制钢筋砼管,成品混凝土仿木栏杆</t>
+          <t>取水及原水输送工程、净水厂工程、配水工程、供配电专项工程等施工，设备采购与安装（不含智慧化自控设备采购及伴随服务部分）、系统调试与试运行、市政设施保护、拆除与恢复、电力和燃气管线迁改；厂区道路、绿化景观、围墙等配套设施；施工临时道路、施工临时用水与施工临时用电（含道路、用水、用电的手续办理）、施工围挡、配合完成不少于一项区级及以上的科技创新项目、“后五通”的接入等。</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>万州区2026年超长期特别国债高标准农田建设项目拟进行预制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜的 信息公告 1.采购条件 1.1本项目万州区2026年超长期特别国债高标准农田建设项目工程已由 重庆市万州路桥建设有限公司承建，项目 业主为重庆市万州区农业技术与机械推广中心，代建业主为重庆市万州区农业发展有限公司，建设资金为国债 资金，项目出资比例为 100% ，承包人为重庆市万州路桥建设有限公司。项目已具备施工条件，现对该项目的预 制钢筋砼管、成品混凝土仿木栏杆等材料采购事宜发布信息公告。 网 2.项目概况与采购范围 2.1建设地点：重庆市万州区走马镇、瀼渡镇、罗田镇、余家镇、高梁镇、分水镇、柱山乡等7个镇乡。 务 2.2本项目材料采购拟进行比选情况如下： 罗田镇谷山片区材料采购费暂定金额约： 17.5万元； 余家镇桥亭片区材料采购费暂定金额约： 17.99万元； 商 柱山乡山田片区材料采购费暂定金额约： 26.32 万元； 走马镇凉风片区材料采购费暂定金额约： 15.道66万元； 瀼渡镇高村片区材料采购费暂定金额约： 17.72 万元； 分水镇大冲片区材料采购费暂定金额约： 47.12 万元； 管 高梁镇茨坪片区材料采购费暂定金额约： 10.7万元； （以上片区片区金额为暂定金额，最终比选限价金额以比选文件为准）。 国 2.3计划采购周期： 以合同签订为准 日历天。 2.4采购范围：本项目各片区所包含的预制钢筋砼管、成品混凝土仿木栏杆等材料。 中 3.供应商资格要求 3.1本次材料采购要求供应商具备独立企业法人，具有本次所需材料生产能力的厂家或经销商等，其经营范围和 权限应满足本次所需材料的要求，并依法取得国家行政主管部门颁发的有效工商营业执照(建筑材料销售或水泥 制品制造、水泥制品销售等相关营业资格），所提供产品必须满足各项检测要求，达到国家现行标准规定的合 格标准。具有良好的商业信誉和充分的供应保障能力，具备相应售后服务能力。要求竞选人为一般纳税人，可 开具13%税率增值税专用发票，提供一般纳税人认定证明。 3.2本次供应商单位优先选择万州本地企业。 3.3本次 不接受 联合体竞选。 4. 报名要求 4.1报名时间：2026年8月 19日9:00起至 8月21日17:00止。 4.2报名地点：重庆市万州路桥建设有限公司经营部（重庆市万州区天城东路278号）。 4.3报名时，须提交有效的营业执照(有效工商营业执照((建筑材料销售或水泥制品制造、水泥制品销售等相关营 业资格）)，前述证书均为复印件并加盖单位公章。法定代表人参加报名的不需要授权委托书，只需要提供法定 代表人身份证明；非法定代表人参加报名的除提供法定代表人身份证明外还须提供授权委托书、委托代理人身 份证明。 4.4 本项目材料采购需提前报名。经资格预审合格后，通知资格预审合格的供应商，到承包人单位领取相关文件。 4.5本项目材料采购设七个片区进行比选，为保证比选公平、公正、有效，规定同一参选单位报名片区上限为2个， 且最终仅限中选一个片区。 5.联系方式 承包人：重庆市万州路桥建设有限公司 地 址：重庆市万州区天城东路278号 网 联系人： 张红娟 电 话：15923491915 务 邮 箱： 商 重庆市万州路桥建设有限公司 2026年8月19日 道 信息来源:https://www.chinapipe.net/project/d3075512.html cqdingjiu 2026.08.21 10:06:53 管 国 中</t>
+          <t>涪陵区李渡新区水厂工程(一期)施工招标公告 涪陵区李渡新区水厂工程（一期）施工招标公告 1.招标条件 本招标项目涪陵区李渡新区水厂工程（一期）已由重庆市发展和改革委员会以渝发改振兴〔2025〕468号文批准 建设，项目业主为重庆水务环境控股集团渝东自来水有限公司，建设资金来自争取三峡后续工作专项资金、银 行贷款和业主自筹等，项目出资比例为100% ，招标人为重庆水务环境控股集团渝东自来水有限公司。项目已具 备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：涪陵区义和街道，马鞍街道。 务 2.2 项目概况与建设规模： 商 涪陵区李渡新区水厂工程（一期）设计水量目标为10万m/d，二期水量目标为20万m/d，采用混凝、沉淀、 过滤、消毒常规水处理工艺。 道 一期工程项目主要建设内容包括取水及原水输送工程、净水厂工程、配水工程三部分。 管 （一）取水及原水输水工程：新建总规模20万m/d取水工程，深井取水泵房一座（土建按20万m/d实施，设 备分期安装），DN1200--DN1400原水输水管道约4.08千米。 国 （二）净水厂工程：新建10万m/d净水厂一座； 中 （三）配水工程：新建5.5万m/d加压泵站一座、高位水池一座，配套建设配水管道约20千米。 2.3 本次招标项目合同估算金额：约36148万元。 2.4 招标范围： 包括但不限于：施工图设计范围内的取水及原水输送工程、净水厂工程、配水工程、供配电专项工程等施工， 设备采购与安装（不含智慧化自控设备采购及伴随服务部分）、系统调试与试运行、市政设施保护、拆除与恢 复、电力和燃气管线迁改；厂区道路、绿化景观、围墙等配套设施；施工临时道路、施工临时用水与施工临时 用电（含道路、用水、用电的手续办理）、施工围挡、配合完成不少于一项区级及以上的科技创新项目、“后 五通”的接入等。 2.5 工期要求：30个月 缺陷责任期要求：24个月 2.6 标段划分： 本次招标为一个标段 2.7 是否属于政府采购工程：否 网 3.政府采购工程 3.投标人资格要求 务 3.1 本次招标要求投标人须具备以下条件： 商 3.1.1 本次招标要求投标人具备的资质条件： 道 （1）投标人具备独立法人资格。 管 （2）具备建设行政主管部门颁发的有效的市政公用工程施工总承包一级及以上资质。 3.1.2 投标人还应在人员国、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 中 3.2 本次招标接受联合体投标。联合体投标的，应满足下列要求： （1）联合体成员单位不能超过 2家，且联合体成员均须具备独立法人资格。 （2）联合体各方应按招标文件提供的格式签订联合体共同投标协议，并在共同投标协议中明确约定各方拟承担 的工作范围和责任。 （3）联合体各成员应按共同投标协议分工内容提供对应建安工程的资质和业绩。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件、工程量清单、 电子图纸等资料。参与投标的投标人需在重庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理， 办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。 若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 布至2026-08-25 17:00:00前。 4.3招标人应于2026-08-31 17:30:00前在重庆市公共资源交易网发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-22 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期网未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn/）、重庆市公共资源交易网 （https://www.cqggzy.com/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上 务 发布。] 7.联系方式 重庆水务环境控股集团渝东自来水有限 招 标 人: 代理机构: 重庆国际投资咨询集团有限公司 公司 商 重庆市两江新区五里店五简路2号重庆咨询 地 址: 重庆市涪陵区兴华中路71号 地 址: 大厦A幢 邮 编: 邮 编: 道 项目负责人: 蔺老师 项目负责人: 谭杨杰 电 话: 023-72220219 电 话: 023-67107374 传 真: 传 真: 管 电子邮箱: 电子邮箱: 开户银行: 开户银行: 账 号: 账 号: 国 监督部门: 重庆市发展和改革委员会 电 话: 023-67575878 中 2026年08月21日 涪陵区李渡新区水厂工程（一期）施工 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051303399 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835014387 坝支行 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000753318 支行 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630015509 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146638778 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000011634 贸易试验区分行 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764324610 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020026676 信息来源:https://www.chinapipe.net/project/d3077140.html cqdingjiu 2026.08.24 12:31:44</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>排水钢管 Φ200*6m：3000米</t>
         </is>
       </c>
       <c r="N29" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>重庆, 预制钢筋砼管, 成品混凝土仿木栏杆, 国债资金, 高标准农田建设</t>
+          <t>重庆, 管材, 招标, 水厂工程</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水管道)招标采购流标公告</t>
+          <t>中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程CQZSG-2标段项目经理部管材询比采购公告</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2470,7 +2454,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>交通</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2491,12 +2475,12 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>酉阳土家族苗族自治县</t>
+          <t>渝中区</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水管道)公开招标采购。</t>
+          <t>新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程CQZSG-2标段项目经理部管材询比采购</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2506,17 +2490,17 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>污水管道</t>
+          <t>管材</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资(污水 管道)招标采购流标公告 发布单位：中国铁建/中铁十一局/六公司 发布时间：2026-08-19 10:40:49 投标截至时间：2026-08-18 10:00:00 内容： 各投标人： 网 中铁十一局集团第六工程有限公司酉阳县钟多、桃花源片区污水管网新建改造工程(二期)项目经理部物资（污水 管道）公开招标采购（采购编号： CR1106-JC-2026-26-02）评标工作，已于北京时间2026年08月18日10:00整，在 铁建云链（https://www.crccep.com）线上平台公开开标。评审委员会根据招标文件载明的评审办法完成评审工作， 现将评审结果公示如下： 务 一、招标公告发布日期及媒体 招标公告发布日期：2026年07月27日至2026年08月01日 商 招标公告媒体：铁建云链（https://www.crccep.com） 二、拟中标信息 道 公开招标采购编号：CR1106-JC-2026-26-02 包件号：WSGD-01 序号 供应商名称 推荐排序 管 1 无 1 国 以上包件有效投标不足三家，本次招标做流标处理。 三、公示时间 中 自2026年08月19日始，至2026年08月22日止。在公示期间，所有竞标人和其他利害关系人如对公示的评审结果有 异议，可以向相关监督部门举报，逾期将不再受理。举报人必须由其法定代表人或者授权代表签字并盖章，其 他组织或者个人举报的，必须由其主要负责人或者本人签字，并附有效身份证明复印件。举报人如实反映情况 受法律保护。 公示期满，如无异议，即时生效。 监督竞诉受理部门： 中铁十一局集团第六工程有限公司招采中心 联系电话：18671041790 信息来源:https://www.chinapipe.net/project/d3075461.html cqdingjiu 2026.08.21 10:06:53</t>
+          <t>中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程CQZSG-2标段项目经理部管 材询比采购公告 中铁十一局集团有限公司建安分公司招标采购中心就中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房 及配套综合交通枢纽工程CQZSG-2标段项目经理部管材组织询比采购，诚邀有意向的合格供应商参与报价。 一、项目概况及询比采购内容 1.1项目概况 网 （1）新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程位于重庆市中心渝中区中部，具体位置为菜园 坝立交桥以西，龙家湾隧道以东，菜袁路以北，王家坡以南。正在建设的地铁18号线贴临站房北侧，地铁26/27 号线从站区地下通过。项目共划分为4个施工标段，CQZSG-1标段：为国铁站房、地铁站台区域；站北路密不可 分的边坡及场坪工程，包含土石方工程和边坡支护工程，不含机电工程，由中铁建设承建。CQZSG-2标段：为 务 枢纽配套工程，地铁区间、西广场、成都局剩余还建，由中铁十一局承建。CQZSG-3标段：地铁区间、CTC、 站场、东广场，由中铁建工承建。CQZSG-4标段：人防车库、铁路自营车场、综合开发生产配套房屋等，由中 铁二局承建。 （2）标段概况：我方负责新建重庆至黔江铁路重庆站站商房及配套综合交通枢纽工程CQZSG-2标段全部施工内容 （简称B区），主要包含：（1）B区投影范围内盖板以下27号线、26号线明挖区间基坑支护、土石方、区间主体 结构及配套防水、综合接地工程（不含砌筑墙体、装饰装修和机电安装工程），以及承轨层以下市政排水 涵DK1+196（196m）和行包通道；（2）轨道交通26号线暗挖隧道预留工程，其中26左线487m，26号右线408m； （3）站北路E、F、H连接匝道工程，其中E匝道道247m、F匝道285.5m、H匝道174m；（4）B区盖板及以上还建房 屋，其中西侧盖板约3.56万㎡，还建房屋等总建筑面积约3.50万㎡。 1.2询比内容 详见拟采购货物一览表 管 二、供应商资格要求 2.1供应商必须是“中国铁建云链平台”注册并通过审核的供应商。 2.2本次询比采购不接受国被列入“《2026年中国铁建合作方警示名录》、《中铁十一局集团有限公司不良行为供 应商名录》、《JD采购网失信名单》（此项核查针对JMRH项目）”中的供应商,不接受近一年内在铁路建设工程 网公布有违法行为记录及物资供应不良记录、被中国铁路总公司限制投标或已清退出铁路市场的供货商（此项 核查针对铁路站房项目），不接受在铁建云链平台被标记的不良行为供应商。 中 2.3供应商在报价时，如是法定代表人签字的需提供法定代表人身份证复印件、如是法人授权代理人签字的需提 供授权委托书及被授权人身份证复印件。 2.4询比响应供应商需提供营业执照复印件。 2.5其它要求：提供样品、每批次货物必须附符合规范要求的出厂质量检验报告、型式检验报告及合格证或吊牌 等质量证明文件，甲方凭此报告检验质量。 2.6袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠像胶带，另配堵头。 三、拟采购物资及相关要求 3.1拟采购物资一览表 交 序 物资 型号 单 项目 货 交货日 数量 备注 号 名称 规格 位 名称 地 期 址 重 直 庆 径6:0mm 市 包含车 PVC 批次交 壁 渝 丝、黑 1 （袖 米 7100 货与零 厚4:-45.mm 中 色胶布、 阀管） 星交货 单节 新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程 区 管筛、 （具体 长4m CQZSG-2 标段项目经理部 菜 管箍、 以项目 园 堵头等 通知为 坝 一切相 准） 直 网 重 关费用 2 PE管 米 7100 径2:5mm 庆 站 合计 14200 务 3.2技术规格书： 按询比文件第二章项目技术规格书执行 商 3.3结算和付款 3.3.1采购物资报价规则： 道 固定价格。 3.3.2付款方式 （1）货款支付方式：支付方式包管括但不限于银行转账、银行汇票、银行本票、支票、银行承兑汇票、商业承兑 汇票、财务公司票据、供应链票据、其他数字化信用凭证，票据贴息费用由 供货单位 承担。 （2）付款周期：本合同无预付款。甲方在收到乙方提交的合规增值税专用发票，并经税务机关认证通过后次月 支付乙方上月供应期所国供合格物资70%货款，全部货物供应完毕后三个月内付至95%，剩余货款暂时扣留作为质 量保证金，供货完毕后，由乙方提交结算确认单，经甲方审核通过后做最终结算，待所有物资验收合格后12个月 内无息付清。 （3）逾期付款约定：如甲方付款逾期，双方秉持“长期合作，友好往来”原则，在逾期付款行为发生后一年内 中 乙方不向甲方收取逾期付款利息。若一年甲方仍未支付款项，需向乙方支付逾期付款利息，逾期付款利息起算 时间为全部款项到期之日一年后至付清之日，逾期利息的利率为合同订立时中国人民银行授权全国银行间同业 拆借中心公布的一年期贷款市场报价利率(LPR)1倍。 3.4拟采购物资相关的要求 3.4.1本次询比为整体采购，询比响应供应商报价时须写明单价、到站价和运距，报价包含货物制造、运输、装卸、 售后服务等交付采购人使用前所有可能发生的费用，收到报价后不再增补任何费用。 3.4.2交货期：按照采购人规定的期限内分批次运抵交付。 3.4.3供货地点：甲方指定的甲方所属 中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通 枢纽工程CQZSG-2标段项目施工现场。 3.4.4询比响应供应商必须保证产品的质量及售后服务。询比响应供应商提供的货物制造标准及技术规范等，必须 符合最新相关国家标准、部颁标准相关标准和规范的要求，进场提供相关检验检测报告。 3.4.5采购方在确定成交供应商后有权对成交产品的结构、规格做适当调整，调整内容将以工作联系函形式提前发 至供应商。 3.4.6售后服务：本批采购货物若在验收阶段出现不符合规格或质量标准，供应商必须接受退货要求，并在采购人 规定期限内等量补运合格产品，若未按时交付影响采购人使用，供应商必须承担由此给采购单位造成的后续经 济损失。 3.4.7报价方不得虚报各项技术指标，所供货物若不能符合技术要求，成交供应商必须接受全额退还货款，并承担 由此给采购单位造成的经济损失。 3.4.8验收方法及标准 （1）验收依据：询比采购文件、厂家货物技术标准说明及国家有关的质量标准规定，均为验收依据。 （2）货物验收：货物运抵采购人指定交货处后由双方对照采购清单及技术要求进行验收。 （3）其它要求：每批次货物必须附符合规范要求的出厂质量检验报告、型式检验报告及合格证或吊牌等质量证 明文件，甲方凭此报告检验质量。 网 （4）2.6袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠像胶带，另配堵头。 四、报价文件递交 务 4.1此次报价供应商需制作电子报价文件，在递交截止时间前线上递交报价文件。 4.2报价文件递交截止时间：2026年08月24日15时00分。 商 4.3报价文件递交地点：中国铁建云链平台（www.crccep.cn），供应商须登录该平台，在报价文件递交截止时间 前完成所有报价文件资料的上传。 五、发布公告的媒介 道 本次询比公告发布媒体:中国招标投标公共服务平台(www.cebpubservice.com)、中国铁建云链平台（www.crccep.cn） 上同时发布。 管 六、联系方式 1.采购组织单位：中铁十一局集团有限公司建安分公司招标采购中心 地 址：湖北省武汉市国武昌区丁字桥路47号 联 系 人：张先生 联系电话：027-87258521 中 电子邮件：2454774350@qq.com 2.采购人：中铁十一局集团有限公司新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程 CQZSG-2 标段项 目经理部 地 址：重庆市渝中区菜袁路59号 联 系 人：金先生 联系电话：16607273445 电子邮件：2285445503@qq.com 2026年08月21日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3077066.html cqdingjiu 2026.08.24 12:31:44</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠橡胶带，另配堵头。</t>
         </is>
       </c>
       <c r="N30" t="n">
@@ -2524,14 +2508,14 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 酉阳县, 污水管网, 新建改造工程</t>
+          <t>重庆, 管材, 询比采购</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>协同创新区-四期房建三标段镀锌管件物资竞价采购公告</t>
+          <t>中铁十一局集团有限公司新建成渝中线铁路(四川段)站前施工CYZXZQ-1标项目经理部过轨管询价采购公告</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2541,7 +2525,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>房建</t>
+          <t>交通</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2556,49 +2540,57 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>详见附件。</t>
+          <t>本次计划对过轨管材料进行询价，询价内容包括DN125米、DN180米、DN125个、DN180个四种过轨管及其接头。</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>本项目中标金额为26.38亿元，总体工期为1826日历天，计划开工日期为2022年11月30日，计划竣工日期为2027年11月29日。</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>镀锌管件</t>
+          <t>过轨管</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>协同创新区-四期房建三标段镀锌管件物资竞价采购公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3075420.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
+          <t>中铁十一局集团有限公司新建成渝中线铁路(四川段)站前施工CYZXZQ-1标项目经理部过轨管询价采购公告 中铁十一局集团有限公司新建成渝中线铁路（四川 段）站前施工CYZXZQ-1标项目经理部 过轨管询价采购公告 询价编号：ZT1105-XJ-2026-457-2 网 尊敬的各潜在供应商: 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与中铁十一局集团有限公司新建成渝中线铁路 （四川段）站前施工CYZXZQ-1标项目经理部ZT1105-XJ-2026-457-2，过轨管的报价。 务 一、项目概况 中铁十一局集团有限公司新建成渝中线铁路四川段CYZXZQ-1标位于四川省成都市金牛区、成华区、 龙泉驿区 以及安岳境内。主线起止里程 DK282+986～DK288+400,全商长5.414公里。中标金额26.38亿元。 主要工程内容：“一隧一路两厂”,其中隧道0.5座/4.854公里，路基0.56 公里/1.21万方，管片厂1处/10380m管片预 制，板厂1处/96.51公里III 型 板 预制。其中蜀安隧道为我标段的重难点工程，盾构段拟采用1台直径14m 的土压 平衡盾构开挖。本标段报价总价26.38亿元。道 总体工期：1826日历天，计划开工日期2022年11月30日，计划竣工日期2027年11月29日。 管 二、询价内容 本次计划对过轨管材料进行询价，询价内容如下： 国 询价物资一览表 序号 包件号 物资名称 规格型号 计量单位 数量 备注 中 1 过轨管 DN125 米 840 2 过轨管 DN180 米 840 GGG-01 3 过轨管接头 DN125 个 140 4 过轨管接头 DN180 个 140 合计 说明：1.表中数量为计划数量，实际采购过程中可能有所调整，最终结算按照实际采购数量结算。 收货地点：四川省成都市成华区成铁路局客机整备所 三、技术质量及报价要求 1.此次过轨管主要技术性能及规格应满足《地下通信管道用塑料管 第 2 部分：实壁管》 （YD/T 841.2-2016），《给水用聚乙烯(PE)管道系统第 2 部分：管材》（GB/T 13663.2-2018），《地下通信管道 用塑料管 第 1 部分：总则》（YD/T 841.1-2016），《电力电缆导管技术条件 第 3 部分：实壁类塑料电缆导管》 （DL/T 802.3-2023）的要求，质量满足甲方项目部正常使用的要求，保证产品的质量合格，详见技术规格书。 2.报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、结算及付款方式 自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发票认证完成之日起第6个月，支付至本次结算 金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内，累计支付总额不超结算总金额的75%，剩 余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理末次结算后第二年，支付金额应大于等于 尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总额的15%；办理末次结算后第四年，全部 付清）。 五、报价人资格要求 1.营业范围要求：在中华人民共和国境内依法注册，具有询价物资生产或供应网经验的生产商或代理商，并 且具有合法有效的营业执照。 2.生产能力要求：生产商须具备询价物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定。代 理商需出具制造厂出具签字盖章的授权函。 务 3.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8月至今） 国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；每种物资全指标技术参数性能满足 国家和行业最新标准的各项规定。 商 4.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年8月至今）企业或企业法定代表人有人民法院生效判决、裁定 认定的行贿犯罪记录的。④ 对纳入国家铁路局道“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接受 通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合作 方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 5.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 管 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 ★6.下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 国 六、报价人需要提供的资料 1.营业执照复印件、法人身份证复印件、开户许可证、授权委托书、报价表和报价人资格要求中所需的证明资料， 所有资料需中加盖公司鲜章。 2.生产厂家资质，产品质量检测报告等质量证明文件。 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、询价报名截止时间 有意参加本次询价采购的报价人须在铁建云链平台（https://www.crccep.cn）完成供应商注册，并于2026年8月22 日9时00分至2026年8月25日9时00分在网上完成报名工作。 八、询价截止时间 凡有意参加本次询价采购的报价人，请于 2026年8月25日14时00分 前提交报价。截止时间前未完成报价文件传 输的，视为放弃报价。 供应商报价必须严格按照《报价表》格式进行报价。 九、联系方式 采购组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村71号 采购人名称：中铁十一局集团有限公司新建成渝中线铁路（四川段）站前施工CYZXZQ-1标项目经理部 地址：四川省成都市成华区华盛路58号19栋 联系人：向渝 联系电话：15178784487（提供采购服务支持） 中铁十一局集团有限公司 物资设备集中采购管理中心第五分中心 网 2026年8月22日 务 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3078608.html cqdingjiu 2026.08.24 12:31:45 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>DN125米：840米；DN180米：840米；DN125个：140个；DN180个：140个</t>
         </is>
       </c>
       <c r="N31" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 商机</t>
+          <t>重庆, 四川, 管材, 招标, 商机</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>中化重庆涪陵化工搬迁后污水处理厂建设项目招标计划表</t>
+          <t>太行项目不锈钢管件采购招标公告</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2608,7 +2600,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2623,38 +2615,42 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>成都市</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>新建一体化提升泵站及管道约5000m，投资约800万元。</t>
+          <t>法兰及其垫片,沟槽管件,铸铁管件,阀门,检查口,铜制管件,管道用材,套管,补偿器及软接头,过滤器,塑料管件,复合管件,不锈钢管件,钢制管件,阻火器,水箱,其它管件及管道用器材,铝合金管件,玻璃钢管件</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>投资约800万元</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>施工</t>
+          <t>不锈钢管件</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>中化重庆涪陵化工搬迁后污水处理厂建设项目招标计划表 重庆市工程建设项目招标计划表 项目名称 中化重庆涪陵化工搬迁后污水处理厂建设项目 招标法人或 招标人名称 重庆市涪陵交通旅游建设投资集团有限公司 网 （盖章） 项目批准文 涪发改委发[2019] 505号 件及文号 务 主要建设内 新建一体化提升泵站及管道约5000m，投资约800万元。 容 招标 招标 招标文件计 拟交易 合同预估 序号 招标项目名称 备注 内容 方式 划发布时间 场所 金额(万元) 商 本招标计划与2026年5 月25日发布的招标项目 中化重庆涪陵 重庆市 名称为“中化重庆涪陵 招标项目 化工搬迁后污 涪陵区 公道开 化工搬迁后污水处理厂 1 水处理厂建设 施工 2026-09 公共资 800.00 招标 建设项目（场外连接管 项目（场外干 源交易 网）”的招标计划，除 管部分） 中心 招标项目名称调整外， 其余内容完全一致。 管 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075591.html cqdingjiu 2026.08.21 10:国06:54 中</t>
+          <t>太行项目不锈钢管件采购招标公告 四川省工业设备安装集团有限公司 压缩空气供应系统、供水系统、燃油供应系统及变配电系统（室外电缆工艺 用） 太行项目不锈钢管件采购 招标公告 四川省工业设备安装集团有限公司 现就 压缩空气供应系统、供水系统、燃油供应系统及变配电系统（室外 电缆工艺用） 的 法兰及其垫片,沟槽管件,铸铁管件,阀门,检查口,铜制管件,管道用材,套管,补偿器及软接头,过 滤器,塑料管件,复合管件,不锈钢管件,钢制管件,阻火器,水箱,其它管件及管道用器材,铝合金管件,玻璃钢管件 采 购事宜进行公开招标，欢迎有意向的供应商参加投标。 一、采购内容 网 法兰及其垫片,沟槽管件,铸铁管件,阀门,检查口,铜制管件,管道用材,套管,补偿器及软接头,过滤器,塑料管件,复合管 件,不锈钢管件,钢制管件,阻火器,水箱,其它管件及管道用器材,铝合金管件,玻璃钢管件 ，预计总用量约为： 见 附件 。 不锈钢管件 务 二、项目概况 项目名称： 压缩空气供应系统、供水系统、燃油供应系统及变配电系统（室外电缆工艺用） 项目地址： 四川成都市东部新区简州新城指定地点 商 建筑规模： 0㎡ 其他详见招标文件。 三、招标方式 本次采购招标采用公开招标的方式进行，并在道善建云采（四川华西集团有限公司及下属分子公司）发布招标公 告，网址为：https://scm.zghxsjy.com/。 四、投标人资格要求 在善建云采（四川华西集团有限公司及下属分子公司）（https://scm.zghxsjy.com/）已注册的合格分供商均可参与 管 投标。 五、招投标时间节点 （一）招标文件发售截止时间： 2026-08-28 09:00:00 ； 国 （二）投标保证金缴纳的截止时间为： 2026-08-28 09:30:00 ； （三）本次招标的投标截止时间为： 2026-08-28 10:10:00 ； （四）本次招标的开标时间为： 2026-08-28 10:10:00 ； （五）电子标书费售价：人民币 40 元/套，售后不退。 中 六、缴费注意事项 为保证招投标的公平公正，善建云采（四川华西集团有限公司及下属分子公司）已与银行实现系统对接，从缴 费账号生成、缴费确认、标书下载和投标功能开放，全部实现自动化、线上化，请投标人务必按照下述要求缴 纳标书费和投标保证金，避免影响投标。 电子标书费缴纳： 1、投标人一旦决定投标，请在善建云采（四川华西集团有限公司及下属分子公司）上点击“交标书费”，银行 系统会随机自动为该次缴费生成一次性的唯一银行账号。 2、请投标人务必把标书费转入上述银行账户。投标人缴费后，银行系统会同步自动将缴费信息推送至善建云采 （四川华西集团有限公司及下属分子公司）和投标人，善建云采（四川华西集团有限公司及下属分子公司）系 统亦同步开放权限，投标人即可在善建云采（四川华西集团有限公司及下属分子公司）浏览和下载标书。 3、投标人务必严格按照上述要求进行投标操作。若投标人缴费到错误账号，善建云采（四川华西集团有限公司 及下属分子公司）无法开放投标功能，由此无法购买标书、无法投标、退回款项延迟等产生的一切损失，均由 投标人自行承担。 投标保证金缴纳： 1、投标人在善建云采（四川华西集团有限公司及下属分子公司）上点击“交投标保证金”后，由银行系统自动 为该次缴费生成唯一银行账号。 2、请投标人务必把投标保证金转入上述银行账户。投标人缴费后，银行系统会同步自动将缴费信息推送至善建 云采（四川华西集团有限公司及下属分子公司）和投标人，善建云采（四川华西集团有限公司及下属分子公司） 系统亦同步开放权限，投标人即可在善建云采（四川华西集团有限公司及下属分子公司）上传投标文件和填报 投标数据。 3、投标人务必严格按照上述要求进行投标操作。若投标人缴费到错误账号，善建云采（四川华西集团有限公司 及下属分子公司）无法开放投标功能，由此无法投标、退回款项延迟等产生的一切损失，均由投标人自行承担。 投标人缴纳投标保证金必须由投标人对公账户转账，不接受个人账户转款、现金缴存、他人代缴。若出现投标 人使用个人账户转款、现金缴存、他人代缴、未按系统自动生成的对应账号转款、超额转款等，平台将无法自 动退款。在中标公示结束后3个工作日内未收到保证金退款，投标人应在10个工作日后向四川华西数产科技集团 有限公司提供完整的书面缴费依据，四川华西数产科技集团有限公司将在收到投标人提供的完整缴费依据后， 在7个工作日内核实并退款。若出现上述情况投标人可编辑含有“招标项目名称”、“招标单位”的短信发送至： 19950205781（本号码只接受短信联系方式），也可到访四川华西数产科技集团有限公司进行沟通。 系统每次生成的账号，均为一次性账号和唯一性账号，标书费账号与投标保证金账号不同，项目与项目间账号 不同。 七、投标文件的递交 招标人仅接受投标人通过善建云采（四川华西集团有限公司及下属分子公司）提交的投标文件，不接受通过其 他方式提交的书面投标文件。线上投标内容具有法律效力且具有唯一性，请投标网人慎重对待。 八、其他描述 九、其他资格要求 务 十、其他事项 若对招标公告有其他不明事项，请致电： 业务咨询联系人： 安虹静 ，联系电话： 15883776766 ； 商 技术支持联系人： 集采技术部 ，联系电话： 02883382846 ； 十一、声明 本招标公告仅为信息发布，不构成任何法律意义上的要约或承诺。 现予公告。 道 四川省工业设备安装集团有限公司 2026年8月24日 信息来源:https://www.chinapipe.net/project/d3078483.html 管 cqdingjiu 2026.08.24 12:31:45 国 中</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>一体化提升泵站及管道：5000m</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N32" t="n">
@@ -2662,14 +2658,14 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 商机</t>
+          <t>不锈钢管件, 四川, 成都, 招标公告</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>綦江区污水处理厂设施设备更新改造工程(二期)招标公告</t>
+          <t>成都市中兴供水有限公司2026-2028年度管网施工劳务比选磋商公告</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2694,33 +2690,37 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>綦江区</t>
+          <t>武侯区</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造，包括配电柜、风机、污水提升泵、在线监测等设备的更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。</t>
+          <t>本项目比选人为成都市中兴供水有限公司，主要从事市政基础设施、城市供水管网的投资、建设与运营。根据公司业务范围及建设需求，现面向社会进行给水管网施工单位的公开比选，邀请有能力的优秀比选申请人参加我公司的项目比选，并选出二至三家优秀企业共同承担2026年及2028年度成都市中兴供水有限公司供水区域内给水管网的施工任务。</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>上级补助和业主自筹，项目出资比例为100%，本项目工程总投资金额约1327.40万元</t>
+          <t>中选的单位，按照工程预估1000万元作为暂定金额签订合同。</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>污水处理设施设备</t>
+          <t>给水管网施工劳务</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>綦江区污水处理厂设施设备更新改造工程(二期)招标公告 1.招标条件 本招标项目 綦江区污水处理厂设施设备更新改造工程（二期） 已由 重庆市綦江区发展和改革委员会 以 重庆市企业投资备案证（项目代码：2502-500110-04-01-844057） 批准建设，项目业主为 重庆南州城市管 理服务有限公司 ，建设资金来自 上级补助和业主自筹 ，项目出资比例为 100% ，招标人为 重庆南州 城市管理服务有限公司。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用经评审的最低 投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 綦江区 2.2 项目概况与建设规模：对三江污水处理站、綦齿园污水处理厂、信家岩污水处理站的设施设备进行更新改造， 务 包括配电柜、风机、污水提升泵、在线监测等设备更新更换，以及对工艺落后的污水厂完成工艺技改；北渡污 水厂、赶水污水处理厂、工业园区污水厂、食品园污水厂零星设施更新等。 2.3 本项目工程总投资金额： 约1327.40万元 商 2.4 招标范围： 本项目设计施工图和招标文件、答疑、补遗、工程量清单等资料所涉及的全部内容。 2.5 工期要求： 180日历天 道 缺陷责任期要求： 24个月 2.6 标段划分（如有）： / 管 2.7 其他： / 3.政府采购工程 国 3.1 是否属于政府采购工程：否 4.投标人资格要求 中 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包三级 及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网（綦江区） （https://www.cqggzy.com/qijiangweb/）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重 庆市公共资源交易网完成市场主体信息登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏 “主体信息”页面中“市场主体信息登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易网（綦江区）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间 从本公告发布至2026-08-22 18:00:00前。 5.3招标人应于2026-09-11 18:00:00前在重庆市公共资源交易网（綦江区）发布澄清。 6.投标文件递交的内容 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-28 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（綦江区）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 8.联系方式 招 标 人: 重庆南州城市管理服务有限公司 代理机构: 永卓国际工程技术有限公司 地 址: 重庆市綦江区红星美凯龙生活广场3幢19-3 地 址: 两江新区网泰山大道东段98号2幢10-12号 邮 编: 邮 编: 项目负责人: 赵老师 项目负责人: 廖淼 电 话: 023-48690537 电 话: 务023-60391733 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 商开户银行: 账 号: 账 号: 监督部门: 道 电 话: 2026年08月18日 綦江区污水处理厂设施设备更新改造工程（二期） 管 户名 开户行 投标保证金账号 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051287453 中国农业银行股份有限公司重庆自由贸 重庆联合产权交易所集国团股份有限公司 312601010400083780000031123 易试验区分行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146631326 信息来源:https://www.chinapipe.net/project/d3075589.html 中 cqdingjiu 2026.08.21 10:06:54</t>
+          <t>成都市中兴供水有限公司2026-2028年度管网施工劳务比选磋商公告 （一）概况 1、本项目比选人为成都市中兴供水有限公司，主要从事市政基础设施、城市供水管网的投资、建设与运营。根 据公司业务范围及建设需求，现面向社会进行给水管网施工单位的公开比选，邀请有能力的优秀比选申请人参 加我公司的项目比选，并选出二至三家优秀企业共同承担2026年及2028年度成都市中兴供水有限公司供水区域内 给水管网的施工任务。 2、本项目比选为企业自主谈判，组织形式为自行谈判。 网 3、中选的单位，按照工程预估1000万元作为暂定金额签订合同。 （二）比选范围 务 1、工作内容涉及:1）管道施工；2）各类管井砌筑、管道保护等；3）PE管、铸铁管、钢管、衬塑复合管等 给水管道安装（包含建筑体内的管道安装）；4）旧管拆除及新接管道的连接；5）特殊施工项目，如顶管（若实 际项目中涉及）、少量构筑物修建及改造等。 商 2、服务期：2年，以任务发放的开始和结束时间为准。 3、服务地点：成都市武侯区金花辖区约12.9平方公里。 道 4、比选申请人根据自身资质、能力、条件等，可选择不同的模式进行报价，详见比选文件 （三）比选申请人资格要求 管 1、具有独立企业法人资格，持有合法有效的营业执照，注册资金50万元以上，财务状况良好，具有税务部门认 可的增值税纳税人认定表（书），可开具国家认可的增值税专用发票。 2、具有：①国家建设行政主管部门颁发的市政工程总承包叁级及以上资质或房屋建筑工程施工总承包叁级及以 上资质；②有效的施工国作业劳务资质、有效的安全生产许可证（①②可任具其一） 3、业绩要求：申请人应于2024年至2025年期间承接并完成施工至少两个以上的类似工程的劳务分包作业（类似 工程是指：市政给水（或供水或输水）管道工程施工业绩或市政给水（或供水或输水）管道工程，申请人须提 供合同及相关的履行证明），并在人员、设备、资金等方面具有相应的施工能力。 中 4、信誉要求：未处于四川省行政区域内有关行政处罚期间，且未处于投标禁入期内；近3年或成立至今（成立不 足3年的）在经营活动中没有重大违法违规记录。在“信用中国”网站（www.creditchina.gov.cn）中未列入失信被 执行人和重大税收违法案件当事人名单 5、主要人员配备要求： ①项目负责人、技术负责人要求：项目负责人或技术负责人具有工程类中级工程师及以上职称。(项目负责人或 技术负责人相关证书在合同签订时需交由比选人，待合同履行完毕退还) ②本项目管理人员中须至少配备施工员、安全员、资料员、材料员、造价员各1名。 ③主要人员（项目负责人、技术负责人、施工员、安全员、资料员、材料员、造价员）应是比选申请人本单位 人员。 6、不接受联合体参选。 （四）比选文件获取 1、比选申请人报名时需提供：法定代表人持加盖机构鲜章的本人身份证复印件，或授权代理人持法定代表人签 发并加盖机构鲜章的授权委托书原件、加盖机构鲜章的本人身份证复印件；企业营业执照副本复印件；资质证 书副本复印件；安全生产许可证副本复印件；纳税人资格证复印件；开户许可证复印件；管道施工合同及相关 的履行证明。 注：以上所有复印件均须加盖比选申请人鲜章，且须携带原件，现场查验。 2、比选人在接受报名后即对比选申请人资格条件进行审查，条件合格者即可领取商务谈判文件。 3、获取时间：2026年8月24日起（工作日上午9：30至12：00，下午14：00 至17：30）。 4、获取地点：成都市武侯区草金路中段999号附9号成都市中兴供水有限公司二楼成控部 （五）参选文件递交 1、参选文件应按以下规定文件格式及附件要求的内容填写并装订。 网 2、递交参选文件时，应同时提供以下资料查验，否则比选人有权拒收：①营业执照副本原件②安全生产许可证 副本原件③项目经理注册证原件④税务部门认可的纳税人认定表（书）⑤项目负责人或技术负责人具备的相关 资质证书。 务 3、投标文件的递交的截止时间（以比选人通知为准），地点为成都市武侯区草金路中段999号附9号成都市中兴 供水有限公司二楼成控部。 4、逾期送达或未送到指定地点的投标文件，比选人不予商受理。 （六）联系人及联系电话 联系人：杜老师 道 联系电话：028-8200 6199转823 17828175202 公司网站：http://www.zxwatersupply.com/ 管 信息来源:https://www.chinapipe.net/project/d3078430.html cqdingjiu 2026.08.24 12:31:45 国 中</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2729,18 +2729,18 @@
         </is>
       </c>
       <c r="N33" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>重庆, 綦江区, 污水处理厂, 设施设备更新改造, 管材招标</t>
+          <t>成都, 供水, 管网施工, 劳务比选</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>南岸区峡口、迎龙片区农村供水保障提升工程招标计划表</t>
+          <t>北部基地平原公司关于FRPP管Φ160及配套弯头项目采购公告</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>其他/未识别</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2765,53 +2765,49 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>重庆市</t>
+          <t>四川省</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>南岸区</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统，对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平台。</t>
+          <t>北部基地平原公司关于FRPP管Φ160及配套弯头项目采购公告</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>概算批复工程建安费2975.27万元。</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>农村供水管网、智慧加压泵站、水厂升级改造、智能控制系统、加药系统、金属防腐工程、入户管道、入户水表、监测计量基础设施。</t>
+          <t>FRPP管Φ160PN1.0*13.3-黑色, FRPP弯头(90°)Φ160PN1.0*13.3-R=1.5D-黑色</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>南岸区峡口、迎龙片区农村供水保障提升工程招标计划表 重庆市工程建设项目招标计划表 项目 南岸区峡口、迎龙片区农村供水保障提升工程 名称 招标 网 法人 或招 标人 重庆市江南城市建设发展（集团）有限公司 名称 务 （盖 章） 项目 批准 商 文件 南岸发改﹝2026﹞156号 及文 号 本工程主要内容包括新（改）建峡口、道迎龙片区4个乡镇DN20～DN300农村供水管网81km，新建3座一体 主要 化智慧加压泵站。对朱家岩水厂进行升级改造：更换陈旧、老化的工艺、电气设备及自控、仪表系统， 建设 对全厂进行智能化、标准化改造，增加高级工艺控制系统，建设智能化、标准化的农村供水区级管理平 内容 台。概算批复工程建安费2975.27万元。 管 拟 招 招标文 合同预 招标 交 序 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 国 所 南岸 重 区峡 庆 口、 中 市 迎龙 朱家岩水厂升级改造工程：对全厂老旧设备进行设备更新；对全 公 片区 公 厂进行智慧化改造，增加高级工艺控制系统；对厂区建筑和构筑 共 农村 开 1 物修缮；优化加药系统投加模式，增加精确加药系统；对全厂部 2026-08 资 1600.00 供水 招 分老旧管道进行更换；金属防腐工程，对金属设备和管道的防锈 源 保障 标 刷漆工作。 交 提升 招标 易 工程 项目 中 （一 心 标段） 南岸 重 区峡 庆 口、 市 迎龙 公 片区 管网工程：延伸、改造峡口镇、迎龙镇等4个乡镇 46 公里 公 共 农村 DN40~DN300 配水主支管，36公里 DN20入户管道，新建3座一体 开 2 2026-08 资 1300.00 供水 化智慧加压泵房，入户水表改造 1752 户，并配套建设监测计量 招 源 保障 基础设施。 标 交 提升 易 工程 中 （二 心 标段） 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075572.html cqdingjiu 2026.08.21 10:06:54 网 务 商 道 管 国 中</t>
+          <t>北部基地平原公司关于FRPP管Φ160及配套弯头项目采购公告 根据成都云图控股股份有限公司采购管理制度，本着“公开、公平、公正、诚信”的原则，诚邀具备投标资格 供应商参加投标。 1 项目概况 1.1 项目名称：北部基地平原公司关于FRPP管Φ160及配套弯头项目 1.2 项目编号：ZB-2608-1047 1.3 交货地点和时间：按实际订单地址及交期要求； 1.4 物资名称及数量： 网 标的编码 标的名称 规格型号 计量单位 数量 TMP91386 FRPP管Φ160PN1.0*13.3-黑色 4米/根 米 80 务 TMP91392 FRPP弯头(90°)Φ160PN1.0*13.3-R=1.5D-黑色 个 8 2 投标人资格要求 2.1 具有独立法人资格； 商 2.2 具有本项目相应履约能力； 2.3 未被纳入成都云图控股股份有限公司供应商“黑名单”。 3 投标方式 道 登录云图控股采购平台（https://srm.wintrueholding.com/），根据注册要求填报公司信息并上传资质文件，获得准 入审核后报名申请参加本项目。本项目所有的招标公告、变更澄清、中标公告均在本网进行公示。具体查阅本 网站首页下载专区的“供应商系统操作手册”。 4 时间安排 管 投标截止时限：2026-08-25 13:00，投标人应于该时限前完成平台注册、报名、标书费缴纳、投标保证金缴纳、平 台报价和标书上传等工作。 5 标书费与保证金 国 5.1 标书费：0人民币/份，售后不退还； 5.2 投标保证金：0人民币/份； 5.3 标书费和投标保证金请分开支付，收款账号详见项目缴费单，转账时需备注平台提供的缴费附言。 5.4 投标保证金退还：未中标单位在中标公告发布后7个工作日内无息退还；中标单位在签订合同后转为履约保证 中 金，按合同约定履约后7个工作日内退还。 5.5 投标人存在下列行为之一的，投标保证金将不予退还： 5.5.1 违反《供应商廉洁诚信承诺书》的； 5.5.2 在投标活动中有弄虚作假、围标串标的； 5.5.3 中标人放弃中标项目的； 5.5.4 中标公告发出后7个工作日内，中标人无正当理由不与招标人签订合同的、提出附加条件、更改合同实质性 内容的； 5.5.5 中标人拒不足额缴纳招标公告文件所要求履约保证金的； 5.5.6 法律法规规定不予退还的其他情形。 6 招标业务联系方式：白焱公 手机：15315813736 邮箱： 。 7 其他咨询与投诉热线400-066-7019，接通后请按语音提示拨号： 拨号1 设备备件类业务和企业微信相关问题咨询。 拨号2 SRM平台注册、缴费、系统操作、大宗原料业务咨询。 拨号3 标书费发票开具。 拨号4 投诉与举报，或将相关投诉举报资料发至邮箱likaijuan@wintrueholding.com，我们将妥善处理。 成都云图控股股份有限公司供应中心 2026-08-22 11:46 网 附件： 务 点击查看内容 信息来源:https://www.chinapipe.net/project/d3078468.html 商 cqdingjiu 2026.08.24 12:31:47 道 管 国 中</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>DN300农村供水管网：81km</t>
+          <t>FRPP管Φ160PN1.0*13.3-黑色: 80米, FRPP弯头(90°)Φ160PN1.0*13.3-R=1.5D-黑色: 8个</t>
         </is>
       </c>
       <c r="N34" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>重庆, 农村供水保障提升工程, 管材招标, 资金情况, 产品种类</t>
+          <t>FRPP管, 弯头, 四川</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>北碚区东阳天府片区农村供水提升工程招标计划表</t>
+          <t>81-西南-大邑西岭文体-水泥制品-询比采购公告</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2821,7 +2817,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>交通</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2836,53 +2832,49 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>重庆市</t>
+          <t>四川省</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>北碚区</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水主要建设内容管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网附属设施。</t>
+          <t>水泥制品</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>合同预估金额为8457万元</t>
+          <t>项目预算金额为290万元</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>供水管网</t>
+          <t>II级钢筋混凝土管、II级钢筋混凝土管、II级钢筋混凝土管、II级钢筋混凝土管、II级钢筋混凝土管、II级中钢筋混凝土管、钢筋混凝土检查井上井室、钢筋混凝土检查井上井室、钢筋混凝土检查井上井室、钢筋混凝土检查井上井室、钢筋混凝土检查井上井室、钢筋混凝土检查井下井室、钢筋混凝土检查井下井室、钢筋混凝土检查井下井室、钢筋混凝土检查井下井室、钢筋混凝土检查井下井室、钢筋混凝土井筒、预制偏心井盖、预制偏心井盖、预制偏心井盖、预制偏心井盖、单算偏沟式雨水口、双算偏沟式雨水口、钢筋混凝土矩形检查井、钢筋混凝土矩形检查井、钢筋混凝土矩形检查井、钢筋混凝土矩形检查井</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>北碚区东阳天府片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区东阳天府片区农村供水提升工程 招标法人或招 标人名称（盖 重庆北碚文旅产业发展有限公司 网 章） 项目批准文件 及文号 务 工程建设区域为东阳及天府片区，主要建设内容包含改造供水管网437千米，其中DN200供水 主要建设内容 管网35千米，DN100~DN150供水管网82千米，DN100以下供水管网320千米，并配套建设管网 附属设施。 招标项目名 招标内 招标方 招标文件计划 拟交易场 合同预估金 序号 商 备注 称 容 式 发布时间 所 额(万元) 北碚区东阳 招标项目 重庆市公 天府片区农 施工招 公开招 1 2026-08 共资源交 8457.00 村供水提升 标 道标 易中心 工程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075569.html 管 cqdingjiu 2026.08.21 10:06:55 国 中</t>
+          <t>81-西南-大邑西岭文体-水泥制品-询比采购公告 物资采购 【招标公告】81-西南-大邑西岭文体-水泥制品-询比采购 招标编号：cscec2026082000002023946 项目：大邑县西岭文体智能装备功能区基础设施建设工程(二标段) 发布时间：2026-08-21 10:43:38 报名截止：2026-08-26 21:59:00 区域：四川省成都市 招标品类：水泥制品 招标（资格预审）公告 网 中建八局第一建设有限公司 物资采购 务 采 购 商 公 告 道 物资名称： 水泥制品 采购编号： cscec2026082000002023946 采购时间： 2026/8/20 管 第一章采购公告 根据中建八局第一建设有限公司（以下简称公司）管理方针，为满足施工生产需要，现就本采购公告所述工程 项目所需物资进行采购，欢迎符合条件的响应人参加，有关事宜公告如下： 国 一、采购基本信息 采 1 购 人 中建八局第一建设有中限公司 采 2 购 内水泥制品 容 采 3 购 范大邑县西岭文体智能装备功能区基础设施建设工程(二标段)水泥制品 围 概 4 算 金290万元 额 采 5 购 方询比采购 □竞价采购 □谈判采购 □直接采购 式 采 6 购 品 无 □ 品 有 牌 品 要 牌 求 要 ； 求：/ 牌 采 7 购 数见：附件1采购清单 量 质 8 量 标22S521《预制装配式混凝土检查井》、 GB/T-11836-2023《混凝土和钢筋混凝土排水管》，16S518《雨水口》若采购进行时标准规范更新，则以更新后的标准执行 准 付 9 款 方 按 个 月 月 后 □ 3 每 0个 两 工 个 作 月 日 □ 内 季 支 度 付 支 至 付 85 货 % 款 ， ： 满 甲 18 方 个 在 月 每 后 支 30 付 个 周 工 期 作 满 日 后 内 的 支 次 付 月 至 3 9 0 5 日 %, 前 满 支 24 付 个 本 月 周 后 期 30个 结 工 算 作 货 日 款 内 的 支 65% 付 。 至 双 10 方 0% 办 ， 理 以 完 上 成 为 物 2年 资 分 总 4 结 次 算 支 后 付 ， ） 甲 等 方 额 自 付 物 至 资 结 总 算 结 值 算 （ 办 且 理 不 之 超 日 本 起 合 2 同 年 含 平 税 均 金 分 额 4 ） 次 的 （ / 以 %。 每半年为期限支付一次，结算办理完毕满6个月后30个工作日内支付至结算值的75%，满12 式 计 11价 方固定单价□浮动单价 式 增 值 12计 税一般计税 □简易计税 方 式 采 13购 限无 □有，随采购文件发布 价 评 审 14基□无 有，根据预设规则系统自动结算 准 价 响 应 15保□无 有，金额： 10000元 证 金 保 证 金 16缴云筑网 □指定账户（二选一） 纳 方 式 产 17地 要国产 □进口 求 二、响应人资格要求 （一）基本资格要求 网 1．具备法律主体资格，具有独立承担民事责任能力、独立订立及履行合同能力的在中华人民共和国境内注册的 法人或其他组织。 务 2．具备：一般纳税人资格 小规模纳税人。 3．具备国家有关部门、行业或公司要求必须取得的质量、计量、安全、环保认证及其他经营许可；近两年在信 用中国无经营异常或严重违法失信记录；与本级或上下级单位没有不良合作记录。 商 4．响应人注册成立1 年以上，响应人的企业注册资本不得低于 100 万元。 5．响应人须具有3年内混凝土或水泥制品的分供业绩。 道 6．具有良好的商业信誉和健全财务会计制度，能提供会计年度报告。 7．法律、行政法规和本采购公告规定的其他条件。 管 8．采购产品必须是符合国家标准的产品。 9．未与我司存在恶意诉讼、恶意讨薪等法律纠纷。 国 10．响应人未处于被责令停业、响应资格被取消或财产被接管、冻结和破产。 11．未与其他报名单位在云筑网显示信息相关联，报名单位ip不可重复，母子单位不可同时报名，mac地址也不 可重复； 中 12．响应人须为独立法人单位或是经法人单位授权的下属单位。凡是以“**分公司”等非独立法人单位名义报名 或者参与公司采购的供应商必须出具由其上级法人单位加盖公章的授权委托书（格式见附件），否则不得通过 资格审核； 13．响应人在云筑网报名后需积极配合我方完成考察，对于考察未通过或不配合考察的分供商，不予通过资审； 14．能贯彻执行采购文件/框架协议规定的该产品的质量验收标准，接受质量投诉处罚等主要规定； 15．同时符合上述条件，且所提供的资质文件和材料必须真实在有效期内，响应主体一致的响应人，经综合审查 合格后，方可参与响应报价。 （二）相关资格要求 1．资质要求：具有经营规模年收入/ 万元以上，响应企业注册资本不低于 100 万元，工商注册时间不低于 1 年。 2．业绩要求：响应人须具有3年内（ 混凝土或水泥制品）的分供业绩 。 3．其他要求：/ 。 （三）其他要求 启信宝显示响应人为三级关联以内的，不得参加同一采购任务的报价。 三、响应报名 （一）报名方式 通过云筑网进行报名（网址https://www.yzw.cn/）。 （二）报名时间 以云筑网公示报名截止时间为准，逾期不再接受延期报名。 （三）资料范围 网 供应商资格预审表、营业执照、企业法人证明书或法人授权委托书、税务登记证、纳税人身份证明、近三年的 业绩和发票、响应保证金纳税承诺函等等，以上资料扫描件在云筑网报名时以附件形式上传。（必传，否则不 予通过资审。格式详见：第二章 响应文件格式） 务 （四）报名截止时间 自发布公告起不少于48小时。 商 （五）费用承担 响应人在为本次采购所进行的现场考察、事实调查和响应资料编制等一切活动中引起的费用开支和法律事务， 由响应人自行承担，采购人概不承担任何费用道和法律责任。 （六）采购清单 序号 材料名称 规格型号 单位 数量 管 1 II级钢筋混凝土管 DN300*50mm，含胶圈 m 1100.00 2 II级钢筋混凝土管 DN500*55mm，含胶圈 m 1500.00 3 II级钢筋混凝土国管 DN600*60mm，含胶圈 m 1000.00 4 II级钢筋混凝土管 DN800*80mm，含胶圈 m 1100.00 5 II级钢筋混凝土管 DN1000*100mm，含胶圈 m 350.00 6 II级中钢筋混凝土管 DN1200*120mm，含胶圈 m 200.00 7 钢筋混凝土检查井上井室 C30,D800*140mm，含爬梯 m 100.00 8 钢筋混凝土检查井上井室 C30,D1000*140mm，含爬梯 m 100.00 9 钢筋混凝土检查井上井室 C30,D1200*140mm，含爬梯 m 100.00 10 钢筋混凝土检查井上井室 C30,D1500*150mm，含爬梯 m 100.00 11 钢筋混凝土检查井上井室 C30,D1800*180mm，含爬梯 m 100.00 12 钢筋混凝土检查井下井室 C30,D800*140mm，含爬梯，含140mm厚底座 m 100.00 13 钢筋混凝土检查井下井室 C30,D1000*140mm，含爬梯，含140mm厚底座 m 100.00 14 钢筋混凝土检查井下井室 C30,D1200*140mm，含爬梯，含140mm厚底座 m 100.00 15 钢筋混凝土检查井下井室 C30,D1500*150mm，含爬梯，含150mm厚底座 m 100.00 16 钢筋混凝土检查井下井室 C30,D1800*180mm，含爬梯，含180mm厚底座 m 100.00 17 钢筋混凝土井筒 C30,D800*120mm，含爬梯 m 400.00 18 预制偏心井盖 φ1280变800，厚度140mm，含吊钩 个 100.00 19 预制偏心井盖 φ1480变800，厚度140mm，含吊钩 个 100.00 20 预制偏心井盖 φ1800变800，厚度160mm，含吊钩 个 100.00 21 预制偏心井盖 φ2160变800，厚度200mm，含吊钩 个 100.00 22 单算偏沟式雨水口 700*400*800mm*70mm厚度 个 180.00 23 双算偏沟式雨水口 1560*400*800mm*70mm厚度 个 100.00 24 钢筋混凝土矩形检查井 1700*1100*160mm m 10.00 25 钢筋混凝土矩形检查井 1700*1700*160mm m 4.00 26 钢筋混凝土矩形检查井 2100*1800*220mm m 6.00 27 钢筋混凝土矩形检查井 2400*2000*220mm m 4.00 四、响应保证金/响应保证金保险 网 （一）响应保证金/响应保证金保险 1．本次采购的响应保证金为10000 元，允许使用保险或保函等非现金交易担保方式，所有响应单位均要在平台 务 缴纳响应保证金，支付成功后点击页面【去响应】按钮，响应人方可正常参与。 2．云筑网方式：响应人应在采购文件签收后、开启响应文件2天前通过云筑网交付响应保证金或购买响应保证金 保险（报名阶段不需要缴纳响应保证金/保险），购买响应保证金保险视同缴纳响应保证金。 商 3．指定账户方式：响应人应在采购文件签收后、开启响应文件2天前通过“指定账户”交付响应保证金（报名阶 段不需缴纳响应保证金）。指定账户信息及保证金缴纳联系人信息详见采购文件。 4．公司上年度分供商评选名单中三星及以上道供应商、二级及以上分包商免除响应保证金缴纳。 （二）保证金退还 1．未成交退还：未成交响应人的响应保证金在公布成交结果后30个工作日内无息退还，成交人的响应保证金 不 管 转为履约保证金。履约保证金在合同履行完毕并办理完毕总结算书后/ 日内无息退还（履约保证金在签订项目执 行合同时另行约定）。 2．响应保证金有效时间：采购有效期内。 国 3．响应保证金风险指示： （1）响应人未按照采购文件足额缴纳响应保证金，响应无效； 中 （2）响应人未将响应保证金缴纳至采购文件中注明的指定账户，响应无效； （3）响应人已缴纳响应保证金，但未在本次响应保证金缴纳的截止时间前到达响应保证金指定账户，响应无效； （4）响应人缴纳响应保证金的汇款或转账信息中的单位名称与报名单位不完全一致，报名无效； （5）因响应人资料手续不全或不及时申请的原因，导致响应保证金滞后退还或无法退还的情况，责任和后果由 报价单位自行承担。 4．有下列情形之一的，响应保证金将不予退还： (1) 提供虚假的材料谋取成交的； (2) 经采购人审定，有围采串采行为的； (3) 成交人在收到成交通知书后，未在规定期限内与采购人签署合同或未按采购文件规定提交履约担保或未按照 采购文件要求条款签订合同的。 (4) 违反廉政承诺内容或发生其它违规行为的。 (5) 其他。 5．本次采购执行过程受评审小组成员集体监控，由评审组长负责采购执行问题反馈及处理，采购执行过程主要 不良情形及处理标准如下： （1）不良情形一：响应过程中若经评审小组评定为徇私舞弊、串通围采、恶意报价扰乱采购秩序的； 处理标准：不予成交，且在云筑网平台添加不良行为记录、没收保证金，并视情节对不良行为分供单位于云筑 网平台限制合作6-12个月或纳入不合格供应商名录，限制合作范围：公司下属所有项目。 （2）不良情形二：成交单位在响应中恶意低价，扰乱响应环境或低价成交后现场履约不良，实际所供物资与要 求质量不符，影响项目正常物资使用需求的； 处理标准：视情况对不良行为分供单位于云筑网平台限制合作12-24个月或纳入网不合格供应商名录，限制合作范 围：公司下属所有项目。 （3）不良情形三：成交单位无故拒供、擅自变更或者终止履约合同，不履行合同义务或供应能力出现重大问题 的； 务 处理标准：视情况对不良行为分供单位于云筑网平台限制合作12-24个月或纳入不合格供应商名录，限制合作范 围：公司下属所有项目。 （4）不良情形四：资审通过分供单位报价阶段，本次报商价与半年内参加我单位同品类同规格同要求的历史报价 无故存在不合理偏差，经采购工作小组共同决议为不良行为情形的； 处理标准：在云筑网平台添加不良行为记录，并视情况对不良行为分供单位于云筑网平台限制合作6-12个月或纳 入不合格供应商名录，限制合作范围:公司下属道所有项目。 五、报名文件要求 报名文件内容及顺序 管 （1）供应商资格预审表；（必填项） （2）营业执照扫描件；（必填项，正副本均可） 国 （3）一般/小规模纳税人税务登记证明；（必填项，若三证合一上传营业执照内即可；网上税务系统资格查询截 图亦可） （4）响应人提供最新的纳税信用评价信息表（必须为2025年度，若不能提供，需提供说明）、税收完税证明 中 （填发时间近3个月内）、无欠税证明（填发时间近3个月内）； （5）法定代表人身份证明（法人签字并加盖公章）；或法定代表人授权委托书（法人及委托人签字并加盖公章） 及被授权委托人在本单位缴纳的6个月的社保证明；法定代表人身份证明或法定代表人授权委托书身份证及签字 两处均需要盖章，仅盖一处章不予通过资审（必填项）。 （6）企业在“信用中国”网站信用报告自查（要求信用信息报告生成日期不早于采购公告发布时间，并保持其 完整性，盖公司公章）；（必填项） （7）近三年的混凝土或水泥制品 业绩证明合同、对应的发票；（必填项） （8）《绿色建材评价- 混凝土或水泥制品》T/CECS 10025-2019认证证书；（选填项） （9）采购人认为其他所需上传的资料，按以下第/（可多选）条进行约定。 ①《实施工业产品生产许可证管理的产品目录》内的物资工业产品生产许可证； ②本次采购品类的检测报告、代理商需提供厂家授权书、分供合同、发票、履约评价、业主表扬信； ③资源管理部门管理底线要求资料：/（详细描述其他资源使用部门发布的以上未体现的所需管理底线要求资 料）； ④样品提交：根据本项采购要求，评审小组决定报名单位不需要送样；（对于需要寄送样品未寄送的不予通过 资审） 样品数量清单 序号 采购物名称 材料规格、材质、性能、品牌等要求 样品要求 备注 1 / 2 提交地点及收件人：/，联系人及电话 /。 网 样品提交截止时间：/ 年/ 月/ 日 /时前（云筑网报名结束后48小时内）。 （一）报名文件要求 务 1.具体格式详见《第二章 响应文件格式》，以上资料均要求每页加盖公章后扫描成一个PDF文件，不接受单张图 片附件多次上传，不接受其他格式资料，扫描件不清晰视为无效资料；报名时将该PDF文件资料作为报名附件上 传至云筑网；提供虚假报名资料的单位，一经发现，取消其报名资格；报名文件应加盖企业公章，复印件应清 晰、完整； 商 2.若未按响应文件格式要求上传资料、资料不全、资料未签字盖章（空白页、无需填报的页面及目录不做要求）、 资料模糊不清晰均视为无效报名，不予通过资格预审。 道 六、资格审核说明及采购文件发放 （一）资格审核不通过的情形 1．信用中国存在不良行为、黑名管单记录及失信联合惩戒记录（本项采购期间）；与中建八局各子公司存在不良 合作记录 2．被识别有涉嫌围采串采行为的； 国 3．未响应采购公告的实质性要求和条件的； 4．主要内容、格式与采购公告规定不符的或关键内容不全、字迹模糊、无法辨认的； 中 5．响应人提供虚假资料、隐瞒误导采购单位的； 6．响应人或其成员不正当地影响资审工作的； 7．响应人以他人名义递交响应文件、串通递交响应文件、报名文件雷同、以行贿手段或者以弄虚作假等方式递 交响应文件的； 8．云筑网平台报名和响应报价为IP地址相同、显示关联交易方的； 9．启信宝等外部平台查询的信息，经审议后，视为关联交易方的； 10．响应人存在因低价成交后中途恶意调价或恶意停工的； 11．发生相关诉讼且未积极配合解决的、发生上访且造成恶劣影响的，围堵项目部或公司的； 12．响应人资质证书、证件过期，且未上传延期文件的； 13．不满足采购公告相关要求的； 14．响应人不得存在的其他情形：/。 （二）采购文件发放时间 1．发放形式：采购文件以电子版形式发布，不发布书面采购文件； 2．发放对象：经资格审查入围的响应人，收到云筑网短信通知后可登录云筑网（网址http://www.yzw.cn)下载采 购文件。 七、无效采购及其他条款 （一）资审对响应人数量要求 1.资格预审合格条件的响应人数量需满足以下要求：拟成交分供商数量(N)≤3时，有效分供商数量不少于2N+2； 拟成交分供商数量(N)&gt;3时，有效分供商数量不少于N+4。 2.因响应人资审通过不递交响应文件造成影响的，将对响应人暂停响应资格或标网记为不良行为。 （二）延长报名时间或重新组织采购 满足资格预审合格条件的响应人数量不满足要求时，可适当延长报名时间或重新组织采购。 务 （三）特别说明 1.参与采购活动的各方应对采购文件和响应文件中的商业和技术等秘密保密，否则应承担相应的法律责任。 商 2.填写附件2“供应商资格预审表”时，请务必填写上响应人正确邮箱、联系人、联系电话。 （四）采购人联系方式 道 1.各响应单位若对： （1）云筑网供应商账号的注册、维护、密码管理、信息变更； 管 （2）云筑网响应流程与操作方法； （3）成交后的合同订立与订单履约操作等存在疑问的，请详细阅读了解附件2《云筑集采供应商操作手册》，必 要时可通过云筑网在线客服或服务热线：4006-818-555沟通解决。 国 2.各响应单位若对本次采购内容、资格审核要求等存在疑问需要咨询的，请联系： 经办人：熊浩吉联系方式：18223201367 中 资审负责人：刘日光 联系方式：15889573755 3.若对资审结果有异议，需要申诉的，请联系： 申诉邮箱：zjbjcaigou@163.com或zj81caigou@163.com 中建八局第一建设有限公司 2026年8月20日 第二章响应文件格式 封面 中建八局第一建设有限公司 水泥制品物资采购 资 质 文 件 响应单位名称（签章）： 响应单位法人（签字）： 网 响应授权代表（签字）： 联 系 电 话 ： 往来函件邮箱： 务 公司网址（如有）： 报名文件提交日期： 装订顺序 资料名称 备商注 1 响应报名文件封面 必填项 2 报名文件目录 - 3 供应商资格预审表 道必填项 4 营业执照扫描件 必填项 5 一般/小规模纳税人税务登记证明 必填项 6 响应人纳税信用评价信管息表 必填项 7 税收完税证明 必填项 8 无欠税证明 必填项 9 法定代表人国身份证明 必填项 10 法定代表人授权委托书与6个月的社保证明 或填项 11 “信用中国”网站信用报告自查 必填项 12 中响应保证金承诺函 必填项 13 资质证明文件 必填项 14 响应品类对应的近3年业绩合同及发票 必填项 15 绿色建材评价证明 选填项 一、 供应商资格预审表（必填项） 企业名称 响应产品 水泥制品 响应品牌 生产地址 有限责任公司 2023年销售额 (万元) □股份有限公司 □中外合资企业 企业类型 2024年销售额 (万元) □全民所有制企业 □集体所有制企业 2025年销售额 (万元) □独资企业 营业执照号 法定代表人 营业执照 员工人数 注册资本 成立日期 营业期限 企业情况 仓库个数 仓库面积 姓 名 身份证号 被授权人 联系电话 电子邮箱 近三年期产品应用情况（不仅限于我司项目） 已完工程名称 发包工程联系人 联系电话 所供应物资名称 合同额（万元） 合同签订时间 网 二、 营业执照扫描件（必填项） 三、 一般/小规模纳税人税务登记证明（必填项） 务 四、 响应人纳税信用评价信息表（必填项） 2025年 商 五、 税收完税证明（必填项） 填发时间近3个月内 道 六、无欠税证明（必填项） 填发时间近3个月内 管 七、法定代表人身份证明（必填项） 响应人名称： 国 单位性质：有限责任公司 地址： 成立时间：中 年 月 日 经营期限： （姓名）系（公司）的法定代表人，职务：电话：。 特此证明。 附：法定代表人身份证复印件(正反面) 响应人：（盖单位章） 法定代表人：（签字） 年 月 日 八、法定代表人授权委托书（或填项） 响应负责人为法人时不填 中建八局第一建设有限公司： 本授权书声明：位于（公司地址） 的（公司名称） 的（法定代表人姓名）代表本公司授权（被授权人姓名）为 本公司的唯一合法代理人，代表本公司参加81-西南-大邑西岭文体-水泥制品-询比采购采购活动，并在整个采购 采购活动中，以本公司名义全权处理确认采购相关信息，采购工程报价、议价，交纳相关费用，签订合同，除 另有授权委托书外，执行和完成合同周期内的服务等一切与之有关的事务，并保证所提供的资质证明材料真实、 合法、完整、有效。 本授权书于2026年月日签字生效，授权期限自签字生效之日起，至合同履行完成之日止。授权期限内无特殊情况 不变更合法代理人（被授权人）。 法定代表人：(签字) 被授权人：(签字) 授权单位名称：（盖章） 联系电话： 网 附：被授权人身份证复印件(正反面) 九、被授权人在本单位近6个月的社保证明（或填项） 务 响应负责人为法人时不填 十、信用中国报告（必填项） 信用中国企业信用信息报告需满足以下两点要求：1、要商求报告生成日期不早于采购公告发布时间；2、“信用中 国”信用信息报告上传需保持其完整性，否则视为无效报告，不予通过资格预审。 信用中国网址：（https://www.creditchina.gov.cn） 道 十一、响应保证金缴纳承诺函（必填项） 管 中建八局第一建设有限公司 ： 我司自愿缴纳响应保证金1.0 万元，并进一步承诺如下： 我司若在响应或履约过国程中违反有关法律法规及响应文件、合同规定，或有下列情形之一的，贵司可将我司响 应保证金作为罚金进行扣除，同时依照相关响应文件条款进行处罚。 1．我司无正当理由拒签合同； 中 2．我司违法行为导致成交结果被确认无效的； 3. 我司在响应有效期内撤销或修改其响应文件； 4. 我司成交签订合同后未按合同要求进行履约的； 5. 我司行为影响采购工作进行的； 6. 我司出现其他违法、违约情况以及采购小组评定为恶意行为的。 响应单位（盖章）： 法定代表人（签字）： 日期： 年 月 日 十二、业绩合同及发票（必填项） 序号 签约单位 施工地点 施工内容 合同金额 签订时间 备注 合同关键页 对应发票 十三、绿色建材评价认证资料（选填项） 网 请查看报价网 址：https://xy.yzw.cn/sj/bid-detail?tenderId=&amp;source=3&amp;tenderCode=cscec2026082000002023946&amp;tenantId=cscec 务 信息来源:https://www.chinapipe.net/project/d3078565.html cqdingjiu 2026.08.24 12:31:48 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>DN150供水管网：82千米；DN100以下供水管网：320千米；主要建设内容包含改造供水管网：437千米；管网：35千米</t>
+          <t>DN300*50mm，含胶圈：1100.00m；DN500*55mm，含胶圈：1500.00m；DN600*60mm，含胶圈：1000.00m；DN800*80mm，含胶圈：1100.00m；DN1000*100mm，含胶圈：350.00m；DN1200*120mm，含胶圈：200.00m；C30,D800*140mm，含爬梯：100.00m；C30,D1000*140mm，含爬梯：100.00m；C30,D1200*140mm，含爬梯：100.00m；C30,D1500*150mm，含爬梯：100.00m；C30,D1800*180mm，含爬梯：100.00m；C30,D800*140mm，含爬梯，含140mm厚底座：100.00m；C30,D1000*140mm，含爬梯，含140mm厚底座：100.00m；C30,D1200*140mm，含爬梯，含140mm厚底座：100.00m；C30,D1500*150mm，含爬梯，含150mm厚底座：100.00m；C30,D1800*180mm，含爬梯，含180mm厚底座：100.00m；C30,D800*120mm，含爬梯：400.00m；φ1280变800，厚度140mm，含吊钩：100.00个；φ1480变800，厚度140mm，含吊钩：100.00个；φ1800变800，厚度160mm，含吊钩：100.00个；φ2160变800，厚度200mm，含吊钩：100.00个；700*400*800mm*70mm厚度：180.00个；1560*400*800mm*70mm厚度：100.00个；1700*1100*160mm：10.00m；1700*1700*160mm：4.00m；2100*1800*220mm：6.00m；2400*2000*220mm：4.00m</t>
         </is>
       </c>
       <c r="N35" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 农村供水提升工程, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>水泥制品, 采购公告</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>北碚区澄江片区农村供水提升工程招标计划表</t>
+          <t>西南油气田分公司致密气项目部金浅26井地面集输工程招标公告</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2892,7 +2884,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2907,53 +2899,49 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>重庆市</t>
+          <t>四川省</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>北碚区</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供水管网68.5km及其附属设施。</t>
+          <t>金浅26井地面集输工程包括井口模块、除砂器橇、三相分离器橇、密闭装油橇、凝析油罐模块、气田水罐模块、放空分液罐模块、放空模块、出站模块等配套工程。</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>合同预估金额：8741.00万元</t>
+          <t>项目估算金额：450万元（含税）</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>供水管网及相关附属设施</t>
+          <t>地面集输工程所需设备和材料</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>北碚区澄江片区农村供水提升工程招标计划表 重庆市工程建设项目招标计划表 项目名称 北碚区澄江片区农村供水提升工程 招标法人或招标 重庆北碚文旅产业发展有限公司 人名称（盖章） 网 项目批准文件及 文号 改造取水泵站一座，改造DN600供水管网2.9km，DN50~DN300供水管网88.863km，DN25供 主要建设内容 务 水管网68.5km及其附属设施。 招标项目名 招标文件计划 合同预估金 序号 招标内容 招标方式 拟交易场所 备注 称 发布时间 额(万元) 招标项目 北碚区澄江 商重庆市公共 1 片区农村供 施工招标 公开招标 2026-08 资源交易中 8741.00 水提升工程 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 道 信息来源:https://www.chinapipe.net/project/d3075568.html cqdingjiu 2026.08.21 10:06:55 管 国 中</t>
+          <t>西南油气田分公司致密气项目部金浅26井地面集输工程招标公告 第一章 招标公告 西南油气田分公司致密气项目部金浅26井地面集输工程 招标公告 招标编号：ZY26-XN301-GC0253-01 网 1．招标条件 本招标项目西南油气田分公司致密气项目部金浅26井地面集输工程己由西南油气田分公司致密油气勘探开发项目 部批准建设，项目业主为西南油气田分公司致密油气勘探开发项目部，建设资金来自自筹，项目出资比例 务 为100%，招标人为西南油气田分公司致密油气勘探开发项目部。项目己具备招标条件，现对该项目进行公开招 标。 2．项目概况与招标范围 商 2.1建设地点 四川省绵阳市。 道 2.2建设规模及主要建设内容 为保障2026年分公司及项目部产量目标的完成，根据已批复的《关于金浅26井地面集输工程初步设计的批复》 （致密油气〔2026〕99号），结合致密油气勘探开发项目部产能及配套建设工程工作安排需要，拟启动施工单位 管 招标工作。招标人为中国石油天然气股份有限公司西南油气田分公司致密油气勘探开发项目部。项目估算金额： 450万元（含税）。 2.3计划工期 国 合同签订之日起至工程竣工验收止，需书面承诺按甲方要求时间完成。 2.4标段划分及各标段具体内容 中 本次招标共1个标段，具体要求： 标段一：金浅26井地面集输工程：新建金浅26井1座分为井口模块、除砂器橇、三相分离器橇、密闭装油橇、凝 析油罐模块、气田水罐模块、放空分液罐模块、放空模块、出站模块共计九部分等配套工程。该项目估算金额 450万元（含税）。 工程量为初步预估工程量，实际工程量以单位工程施工图0版（工程开工前予以下发）为准。站内设备/阀门、管 材、管配件等为甲供，钢结构、土建及自控等常规用料为乙供；线路直管、热弯、热收缩套（带）为甲供，其 他为乙供，最终以甲乙双方实际签订甲乙供料界面划分清单为准。 2.5招标范围 对金浅26井地面集输工程施工部分进行公开招标。其中具体包含但不限于 （1）站场部分：包括包含工艺安装、总图、结构、建筑、给排水及消防、油漆涂装及保温、热工、绝缘接头焊 接、一次仪表安装、电气（不含投建运实施的外供电）、仪器仪表校检、安全阀检定、入场前的标准化布局 （总图布置及门禁系统）、降噪等施工；不含通信、系统组态、数字化交付、无损检测、防爆电气检测和土建 专业检测。 （2）负责甲供材料的领取、存放、转运、使用、回收、退库、记录等；负责乙供材料（场站：钢结构、给排水 材料、总图土建材料、部分螺栓、垫片等 （3）负责施工过程中环境保护，包括废料、废液、建渣等垃圾回收和处理工作以及设备、设施的保护工作； （4）负责焊接工艺评定（含返修）、焊接工艺规程编制及引用工作； （5）负责配合进行单机试运和联合调试，并按照发包人通知负责投产保运工作； （6）负责特种设备（压力容器）安装告知工作，配合接受地方部门监督检验； （7）按设计要求、标准规范及政府相关管理部门要求应进行特殊要求的检验试验及复检项目； （8）负责本工程工程作业过程中涉及到的地方行政单位、企事业单位及当地居民关系协调； （9）负责道路、河流、沟渠、国防光缆等穿越手续办理及穿越费用的缴纳关工网作。 2.6本次招标设最高投标限价 详见《金浅26井试采地面集输工程（主体工程）招标合同价款说明》，详见第五章报价要求，不满足的其投标将 务 被否决。 报价方式为在此最高投标限价标准的基础上，报整体下浮比例（不含安全文明施工费、规费、税金等不可竞争 费用）。下浮百分比须大于或等于7%，最多保留两位小数。（举例说明： 报价方式为在此最高投标限价标准 的基础上，报整体下浮比例（不含安全文明施工费、规费商、税金等不可竞争费用）。下浮百分比须大于或等 于7%，最多保留两位小数。如：8%、8.0%、9.10%，10.12%均符合要求；若下浮费率为负数或者超过两位小数， 如：-1%，2.432%则不符合要求，投标将被否决。（投标人报价需充分考虑两年内市场变化因素，服务期限内单 价价格不作调整）。 道 2.7质量要求 合格。达到设计要求，无质量、安全事故事件发生，符合国家和行业有关施工及验收规范，以及国家和行业有 关管理规定进行施工和验收。 管 2.8 投标人存在待认定失信行为的处理要求：若投标人在中国石油物资有限公司西南分公司组织实施的其他招标 项目中发生失信行为且当前处于待认定处理期间，应当在投标文件中履行告知义务。对于正式认定处理的失信 行为导致暂停投标资格情形的，招标人有权取消其中标人资格。 国 *3. 投标人资格要求 *1.投标人具备合格有效的加载统一社会信用代码的营业执照。 中 *2.本项目： 不接受联合体投标。 允许，允许分包内容：主体工程（工艺焊接、电仪等）以外的部分，部分非主体、非关键性工作。报建设单 位审批同意后可按程序进行分包。 要求：投标人须承诺：投标人须承诺：投标人拟在中标后将中标项目的部分非主体、非关键性工作进行专业工 程分包或劳务分包的，应取得招标人的同意，将分包单位资质、分包合同和HSE合同等报招标人备案，且分包商 须具有满足分包项目性质要求的资质，分包施工负责人（分包项目经理）具有满足分包项目性质要求的注册建 造师执业资格。接受分包的单位不得再次分包。 对于不具备分包条件或者不符合分包规定的，招标人有权在签订合同或者中标人提出分包要求时予以拒绝。发 现中标人转包或违法分包时，可要求其改正；对于拒不改正的，可报请业主有关部门查处，并终止合同。具体 按照招标人及上级单位发布的相关制度要求执行。 *投标人须承诺：如分包商分包项目为中国石油天然气集团有限公司管理专业，分包商须在中国石油工程建设管 理平台承包商资源库内选择，通过的资质类别和等级与分包项目资质要求一致，状态正常。 不允许代理商投标。 *3.资质要求： *3.1有要求，资质要求： 金浅26井地面集输工程中金浅26井站建设规模7万立方米/天，设计压力8.5 兆帕，属于小型石油化工工程，投标 人须具有石油化工工程施工总承三级及以上资质，具有承压类特种设备安装、修理、改造许可项目工业管道安装 （GC1）许可子项目的中华人民共和国特种设备生产许可证（原中华人民共和国特种设备安装改造维修许可证 （压力管道）：GC类GC1级资质）。过渡期应符合《市场监管总局办公厅关于特种设备行政许可有关事项的通 知》（市监特设发〔2022〕17号）。 注：提供证书资料的影印件，同时在全国建筑市场监管公共服务平台（网址：http://jzsc.mohurd.gov.cn）进行查 询，并将带有“企业资质证书号”的查询结果页面进行截图，载入投标文件中。 网 *3.2投标人须具备有效的许可范围为建筑施工的安全生产许可证（许可证应在有效期内且许可范围与本项目主体 工程相关）。 注：提供证书资料的影印件，同时在企业所在省市相关政府网站（或政府相关信息系统）进行查询，并将查询 务 结果页面截图，载入投标文件中。 *3.3投标人须通过中石油统一组织的公开招标资格评审，通过结果在中国石油工程建设管理平台承包商资源库查 询，通过的资质类别和等级与本项目资质要求一致，状态正常（投标人因换领证书发生等级变更的，应及时维 护承包商资源库等级状态，若换领后证书等级高于承包商商资源库显示等级的，以承包商资源库显示的为准）。 *4人员资格和要求： 有人员要求，人员要求： 道 *4.1项目经理：须具有二级注册建造师资格（机电工程专业）并在注册有效期内且具备有效的安全生产考核合格 证书（B证）。且在施工期间不得担任其他在建项目的项目经理（需提供书面承诺）。 管 注：提供证书和相关佐证资料的影印件，同时在全国建筑市场监管公共服务平台（网 址：http://jzsc.mohurd.gov.cn）进行查询，并将载有“执业注册信息”的查询结果页面进行截图，载入投标文件 中。 若提供的一级建造师注国册证书，须符合《住房和城乡建设部办公厅关于全面实行一级建造师电子注册证书的通知 （建办市〔2021〕40号）的要求，否则会因为注册证书无效而被否决投标。（一级建造师打印电子证书后，应在 个人签名处手写本人签名，未手写签名或签名图像笔迹不一致的，该电子证书无效，下载时间需为提交文件截 至之日前180日内） 中 *4.2 技术负责人：具有5年及以上类似本工程工作经验（提供曾经参与工程的业主证明文件，第一个项目至最新 一个项目时间间隔不低于五年），大学本科及以上学历；且在施工期间不得担任其他在建项目的技术负责人 （需提供书面承诺）。 注：提供学历证书的影印件。 *项目经理与技术负责人不允许兼任。 *4.3安全管理人员：具有不少于1名专职安全员，且应具有在有效期范围内专职安全生产管理人员证书C3且在施 工期间不得担任其他在建项目的安全管理人员（需提供书面承诺）。 注：提供证书资料的影印件。 5.机具设备要求： 无要求。 *6.业绩要求: 近年（2024年1月1日至投标截止时间）（已完成 □已完成或新承接或正在实施）不少于1个类似项目。类 似项目:天然气集输工程工艺安装或天然气处理装置工艺安装施工，业绩证明材料：业绩需提供合同复印件及能 够证明项目完工投运的资料。【合同复印件、完工交接或竣工验收）证明无法体现业绩所需要求的，应提供设 计文件或业主证明进行补充佐证】注：业绩时间以完成投运时间为准 。 *7.财务要求： 7.1要求，投标人为资不抵债的，投标将被否决。 需提供经审计的财务证明资料：投标人需提供2024年度或2025年度经会计师事务所或审计机构审计的财务会计 报表财务报表，包括资产负债表、现金流量表、利润表；若为事业单位投标，提供相关财务证明资料。若投标 人成立时间晚于2026年1月1日，提供成立以来的财务状况表。 网 *8.信誉要求 1、投标人没有处于被责令停业,财产被接管、冻结、破产等状态； 务 2、投标人2024年至投标文件递交截止之日无直接影响本项目履约能力的违法、违规不良记录；不良记录包括但 不限于以下情形：因涉嫌犯罪被办案机关立案追查、审查起诉、被法院判决有罪；在和招标人历史合同履约中 存在因商业欺诈、产品质量问题等实质性侵害招标人权益的行为；被国家、招标人及其上级部门明文规定暂停 或取消交易资格； 商 3、2024年1月1日至投标截止时间投标人、法定代表人或者负责人、拟委任的项目经理无行贿犯罪。 4、投标人没有法律、行政法规规定的其他限制参与招投标活动的情形。 道 5、投标人在开标当日不得在存在以下情形： （1）投标人被“国家企业信用信息公示系统”网站（www.gsxt.gov.cn）列入严重违法失信企业名单。 管 （2）投标人被人民法院在“信用中国”网站（www.creditchina.gov.cn）列入严重失信主体名单。法定代表人或者 负责人被人民法院中国执行信息公开网（https://zxgk.court.gov.cn/shixin/）列为失信被执行人。 （3）开标当日被中国石油招标投标网暂停或取消投标资格。 国 （4）投标人、拟委任的项目经理被“全国建筑市场监管公共服务平台”网站 （http://jzsc.mohurd.gov.cn/asite/jsbpp/index）列入黑名单，或虽然被“全国建筑市场监管公共服务平台”网站 （http://jzsc.mohurd.gov.cn/asite/jsbpp/index）列入黑名单但移除黑名单日期在投标截止时间之后的。 中 据《中国石油天然气集团有限公司“三商”黑名单管理办法》，投标人被纳入“三商”黑名单的惩戒相关 内容见下表。投标人应在投标文件中承诺响应该要求（格式见招标文件第六章投标文件格式）。 黑名单 惩戒适 惩戒主体 惩戒范围 惩戒阶段 信息查询 等级 用 正在参与投标、谈判 或其他竞争性方式采 以中国石油 实行“一处受罚， 1、纳入黑名单的“三商”。 集团公 购的，应认定其不具 招标投标网 全集团 处处受限”，不 2、纳入黑名单的“三商”的法定代表人 司级 有相关资格。 公示信息为 区分类型 （或负责人）、实际控制人在惩戒期内 已经完成定商活动的， 准。 在其他法人企业或组织担任法定代表人 不予发放中标或成交 内 （或负责人）、实际控制人的，该其他 通知书。 网：http/:/bdie.nergyaheadc.npc/#/ 法人企业或组织。 已经发出中标或成交 外 企业级 原则上本单位 通知书的，不再继续 网：hptt/s/:wwwc.npcbdidnigc.om/ 签订合同。 以上1-4条款、6条款投标人在投标文件中提供书面承诺，5条款约定要求以开标当日在相应网站的查询结果为准。 招标专业机构协助评标委员会将通过“信用中国”、“国家企业信用信息公示系统”、“全国建筑市场监管公 共服务平台”和资质、资格强制要求的政府发证机关官方网站方式核查投标人信誉及所提供的证书、资料的真 实性、有效性；核查投标人有无直接影响本项目履约能力的异常、有无违法违规记录等情形。 *9.其他要求： 投标人须提供书面承诺满足《金浅26井试采地面集输工程（主体工程）招标合同价款说明》合同结算条款 相关内容。 投标单位必须提交《廉洁自律承诺书》详见附件《廉洁自律承诺书模板》，招标结束后，中标 单位提交的《廉洁自律承诺书》将作为合同附件。 以上“*”号条款，如不满足，其投标将被否决 4．招标文件的获取 4.1凡有意参加投标的潜在投标人，请于2026-08-21至2026-08-26 23:59:59（北京时间，下同）内完成以下步骤后登 录中国石油电子招标投标交易平台下载电子招标文件。 网 ① 投标登记 登录中国石油电子招标投标交易平台，搜索本项目，在拟投标标包处点击“报名”，网 址：http://ebidmanage.cnpcbidding.com/bidder/ebid/base/login.html。 务 （如未在中国石油电子招标投标交易平台上注册过的潜在投标人需要先注册并通过平台审核。具体操作请参考 中国石油招标投标网操作指南中“投标人用户手册”相关章节。） ② 支付标书费 商 登陆中国石油招标中心招标文件购买平台，在可购买的订单列表下支付标书费，网 址：http://www2.cnpcbidding.com/#/wel/index。 道 （登陆账号和中国石油电子招标投标交易平台一致，密码需要重新设置。投标人首次登录需通过手机验证码登 录，登录后设置登录密码，提交成功后可以同时使用户名密码或手机验证码登录。详见附件《中国石油招标中 心投标商用户操作手册》，咨询电话:4008800114。） 管 4.2招标文件按项目售价为200元人民币／标包（标段），请有意参加投标的潜在投标人确认自身资格条件是否满 足要求，售后不退，应自负其责。 4.3本次招标文件采取线上发售的方式。潜在投标人在4.1规定的时间内完成4.1规定的2项工作（投标登记和支付标 书费）后，潜在投标人国可在中国石油电子招标投标交易平台下载招标文件。 4.4潜在投标人在中国石油招标中心招标文件购买平台上付款成功后，在“我的订单”中会生成一条购买记录， 点击订单详情，自行下载招标文件电子发票，不再开具纸质发票。 中 4.5此次采购招标项目为全流程网上操作，需要使用U-key完成投标工作。 ① 所有首次参与中国石油招标项目投标人必须办理U-key。具体办理通知公告及操作手册下载方法如下：登录中 国石油招标投标网首页：https://www.cnpcbidding.com“通知公告栏目”的“操作指南”中“电子招投标平 台Ukey办理通知公告及操作手册”，即可下载“Ukey办理通知公告及操作手册.zip”。 ② 已办理U-key的投标人应复核U-key证书是否处于有效期内，如证书失效，需按上述程序购买新的U-key。 5．投标文件的递交 5.1本次招标采取网上递交电子投标文件的投标方式 投标文件递交的截止时间（投标截止时间及开标时间，下同）为2026-09-11 08:30:00，投标人应在截止时间前通过 中国石油电子招标投标交易平台递交电子投标文件。 注：请投标人注意：为确保投标有效，对于使用“投标客户端”编制的投标文件，在按照操作要求进行信息关 联、签章、加密和上传后，确保上传的文件的附件状态都是验签完成。点击验签确认，当前状态是“已确认”， 并且下方出现“撤标”按键，才视为成功提交投标文件。其它状态都是投标不成功，请投标人密切关注！如在 投标截止时间前未能成功上传投标文件，投标将被拒绝。（为避免投标人在投标文件递交截止时间前未能成功 上传投标文件，建议投标人提前2日递交投标文件）具体操作流程参见“操作指南-投标人操作手册”。 5.2逾期上传的投标文件，中国石油电子招标投标交易平台将予以拒收。 5.3 潜在投标人应在投标截止时间前须按标段提交投标保证金，每标段 5 万元。 6．发布公告的媒介 本次招标公告在中国招标投标公共服务平台（http://www.cebpubservice.com）、中国石油招标投标 网(http://www.cnpcbidding.com)上发布。（适用于依法必须招标项目） 注：本项目中标候选人公示的内容将包含单位资质证书、项目经理等相关信息，以接受社会监督。若有造假， 将按照法律法规及本招标文件相关规定处理，请投标人认真核实投标资料，确保真实无误。（详见投标文件格 式中公示信息表，投标人需填写） 网 7．联系方式 招 标 人：西南油气田分公司致密油气勘探开发项目部 招标机构：中国石油物资有限公司西南分公司 地 务地 址：四川省成都市青羊区小关庙 址： / 街6号 邮 邮 编： 610017 编： / 商联 系 人： 邹女士/张先 联 系 人： 王老师 生 电 电 话： 18728590001 话： 028-68250085/028-68250035 传 传 真： / 真： / 道 电子邮 电子邮件： / 件： / 网 网 址： / 管 址： / 开户银行： / 开户银行： / 账 账 号： / 国 号： / 财务咨询： 许女 士 电 话： 028-68233741 中 网站注册、U-Key办理、招标管理平台（购买招标文件及投标保证金递交）及电子交易平台操作指导： 咨询电话：4008800114 交易平台运营机构：中油物采信息技术有限公司 能源一号网站邮箱：energyahead@cnpc.com.cn 请务必在操作前认真阅读操作手册，如有疑问再在工作时间咨询。 中国石油物资有限公司西南分公司 (中国石油天然气集团有限公司招标中心西南分中心) 2026年8月21日 附件：投标商操作手册V1.1.pdf 附件：投标保证保险理赔服务书-中意财险.doc 附件：投标保证金保险功能操作手册-投标人.docx 信息来源:https://www.chinapipe.net/project/d3078290.html 网 cqdingjiu 2026.08.24 12:31:50 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>DN600供水管网：2.9km；DN300供水管网：88.863km；水管网：68.5km</t>
+          <t>用于地面集输工程的建设</t>
         </is>
       </c>
       <c r="N36" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 商机</t>
+          <t>管材, 地面集输工程, 四川</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>涪陵区江东街道农村供水保障能力提升工程(二期)招标计划表</t>
+          <t>四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005询比采购公告</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2963,7 +2951,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>水利</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2978,53 +2966,57 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>广安市</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>武胜县</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>主要改造及延伸配水管188.2千米，新建加压泵站4座，新建计量监测设施建设以及配套电气工程。</t>
+          <t>四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005询比采购公告 四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005询比采购公告 四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005已具备采购条件，现公开邀请供应商参加询比采购活动。</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>预算金额为3137.22万元</t>
+          <t>项目资金已落实。</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>管道、加压泵站、计量监测设施、电气设备</t>
+          <t>聚乙烯热收缩套,聚乙烯胶粘带,防腐膏,聚丙烯胶粘带,聚乙烯补伤片</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>涪陵区江东街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区江东街道农村供水保障能力提升工程（二期） 名称 招标 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 项目 网 批准 文件 涪陵发改〔2026〕471号 及文 号 主要 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 建设 以及配套电气工程。 务 内容 招 标 合 文 同 招 件 预 招标 标 招标方 计 拟交易 备 序号 招标项目名商称 估 项目 内 式 划 场所 注 金额 容 发 (万 布 元) 时 间 重 道 庆 市 涪 陵 公 区 改造及延伸配水管 188.2千米，新建加压泵站4座，新建计量监测设施 开 公 1 涪陵区江东街道农村供水保障能力提升工程（二期） 2026-09 3137.22 管以及配套电气工程。 招 共 标 资 源 交 易 中 心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075558.html cqdingjiu 2026.08.21 10:06:55 中</t>
+          <t>四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005询比采购公告 四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005询比采购公告 四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005已具备采购条件，现公 开邀请供应商参加询比采购活动。 1.采购项目简介 1.1采购项目名称：四川油建国家石油天然气大流量计量站成都分站高压检定能网力建设工程防腐材料JLZ-005。 1.2采购人：四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程。 1.3采购执行人：四川石油天然气建设工程有限责任公司采购中心（招标中心）。 务 1.4采购项目资金落实情况：已落实。 1.5采购项目概况：四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005。 商 1.6成交供应商数量及成交份额： 1家，成交份额： 道 第一名：；第二名：；第三名：…… 管 2.采购范围及相关要求（B） 2.1采购范围：${招标/采购范围}。 国 含税 单价 序 行项目 数 监造 物料编码 物资名称 规格型号 产品标准（技术要求） 单位 限 号 号 量 要求 价/ 中 元 辐射交联 不监 1 00010 A19040301000691 聚乙烯热 60.3×450 GB/T23257-2017 套 12 18 造 收缩套 辐射交联 不监 2 00020 A19040301000699 聚乙烯热 114×450 GB/T23257-2017 套 6 30 造 收缩套 辐射交联 不监 3 00030 A19040301000700 聚乙烯热 219.1×450 GB/T23257-2017 套 10 55 造 收缩套 辐射交联 不监 4 00040 A19040301000697 聚乙烯热 323.9×450 GB/T23257-2017 套 10 57 造 收缩套 辐射交联 不监 5 00050 A19040301000694 聚乙烯热 406.4×450 GB/T23257-2017 套 10 90 造 收缩套 辐射交联 不监 6 00060 A19040301000693 聚乙烯热 610×520 GB/T23257-2017 套 16 145 造 收缩套 厚胶型聚 宽50mm厚 不监 7 00070 A19040103000195 乙烯胶粘 度≥1.2mm，配套 SY/T0414-2017 米 800 2.2 造 带 底漆6L 粘贴体防 公 不监 8 00080 A19040405000001 SY/T7036-2016 41.5 53 腐膏 斤 造 粘贴体防 宽100mm厚 不监 9 00090 A19040404000001 SY/T7036-2016 米 400 11 腐带 度≥1.8mm 造 聚丙烯胶 不监 10 00100 A19040103000028 宽75mm×1.4mm SY/T7036-2016 米 800 4.5 粘带 网 造 聚乙烯补 不监 11 00110 A19040401000014 250×1.8mm GB/T23257-2017 kg 100 18 伤片 造 务 2.2交货期：下订单后（15 ）天到货。。 2.3交货地点：四川省广安市武胜县胜利镇柿花场村收货人：佘小兵18981930563。 2.4物资质量标准或主要技术性能指标：详见2.1采购范围商的产品标准（技术要求）。 2.5采购物资名称、规格型号、执行标准、单价限价以本表和分项报价单为准，行项目号、物料编码与系统物资 明细相对应。 道 3.供应商资格要求 3.1供应商应依法设立且具备承担本采购项目的资质条件、能力和信誉： 管 供应商资格要求1：供应商在中华人民共和国境内依法注册，具备合格有效的营业执照、税务登记证、组织机 构 代码 (执行“三证合一”改革的投标人，无需单独提供组织机构代码证和税务登记证，只需提供加载统一代码的 营业执照即可)； 供应商资格要求2：本国次采购不接受联合体。只接受制造商 供应商资格要求3：供应商在云梦泽系统中供应商状态必须正常（非临时供应商），同时具有相应产品的准入产 品品类编码状态正常，本次采购准入产品品类编码 为：A19040301，A19040103，A19040405，A19040404，A19040401。 中 备注：“有效的”是指云梦泽系统资源库中供应商状态及产品（以品类编码为准）状态均为“正常”，状态以 评审当日云梦泽系统供应商状态及产品状态为准。潜在投标人应自行确认云梦泽资源库中状态是否符合采购文 件要求。 供应商资格要求4：供应商未被“国家企业信用信息公示系统”网站（www.gsxt.gov.cn）列入严重违法失信 企 业 名 单 ， 授 权 代 表 人 、 法 定 代 表 人 或 者 负 责 人 未 在 中 国 执 行 信 息 公 开 网 （http://zxgk.court.gov.cn/） 中被列入失信被执行人名单。（提供网站查询截图） 供应商资格要求5：供应商被中国石油天然气集团（股份）有限公司、中国石油工程建设有限公司、四川油建公 司列为“三商”黑名单，“三商”预警清单，取消准入资格、禁止准入、暂停交易资格、 年度评价不合格的 （复查合格除外），采购无效。 供应商资格要求6：在《中国石油天然气集团有限公司采购产品质量监督抽查情况通报》中响应产品被处罚的响 应无效（复查合格的除外）。 供应商资格要求7：根据《中国石油天然气集团有限公司投标人失信行为管理办法》的规定，供应商开标当日未 被中国石油招标投标网暂停或取消投标资格。供应商失信分以开标当日中国石油招标投标网查询的失信行为信 息为准。 供应商资格要求8：供应商须提供书面承诺没有被处于被责令停业,暂扣或者吊销认可证、暂扣或者吊销执照，财 产被接管、冻结、破产、资不抵债等状态； 供应商资格要求9：供应商须提供书面承诺，说明2023年1月1日至投标截止日没有发生因未履行合同、延期交货、 产品质量问题原因导致的合同终止或被起诉产生法律纠纷。 4.采购文件的获取 4.1本项目在云梦泽智慧平台发布，凡有意参加投标的潜在供应商，请于北京时间公告发布时间至2026-08-25 14:00:00严格按照下列步骤完成采购文件购买： 登录云梦泽智慧平台(https://www.ymzec.com/bid/web-outportal/)参与并购买电子采购文件。（具体操作详见：云 梦泽智慧平台&gt;通知公告&gt;操作说明中的“投标人用户手册”的相关章节，平台的操作问题咨询电话：956100 转6）。 网 4.2采购文件每套售价为0.00元人民币，请有意参加投标的潜在供应商确认自身资格条件是否满足要求，售后不退， 应自负其责。 务 4.3采购文件下载：潜在供应商在4.1规定的时间内完成参与并购买电子采购文件操作后，即可在“我的项目”中 下载采购文件。 4.4本次招标项目为全流程网上操作。 商 5.响应文件的递交 5.1 响应文件递交的截止时间（投标截止时间及开标时间，下同）：2026-08-28 10:00（北京时间），投标人应在 截止时间前通过云梦泽智慧平台（https://www道.ymzec.com/bid/web-outportal/）递交电子响应文件，具体操作步骤 见下： ① 在递交电子响应文件前，请确保完成响应文件的制作生成（具体可参考操作手册中制作投标文件的相关章 节）。 管 ② 登录云梦泽智慧平台，进入到投标业务系统的【投标人端】。通过点击顶部导航栏的 “招标投标” 按钮，进入 【招标投标系统首页】，再点击 “进入系统” 按钮，进入【投标端业务系统】 ③ 找到递交入口，在投国标人端的相关项目管理 - 投标 - 进入项目 - 网上投标路径下，找到响应文件递交的操作界 面。点击 “递交” 按钮，上传已制作好的响应文件，并确认签名。 特别注意：为避免受网速及网站技术支持时间的影响，建议于投标截止时间24小时之前完成网上电子响应文件的 递交。 中 5.2响应文件递交截止时间未成功递交的电子响应文件将不被系统接受，视为主动撤回响应文件。 5.3开标地点（网上开标）：云梦泽智慧平台(https://www.ymzec.com/bid/web-outportal/)（所有供应商可登录云梦 泽智慧平台在线参加开标仪式）。 5.4如需递交投标保证金，潜在供应商应在投标截止时间前递交投标保证金（CNY）：。投标保证金有效期与投 标有效期一致，投标保证金采用电汇形式递交，具体递交步骤见下： ①企业钱包充值：潜在投标人应先使用基本存款账户绑定企业钱包，且使用该基本存款账户向企业钱包充值， 使用其他账户进行充值，资金将自动原路退回。 企业钱包充值账户信息： 账户名称：中国石油电子招投标保证金 开户行名称：昆仑银行股份有限公司大庆分行 行号：313265010019 银行账号：26902197555010000027 ②投标保证金递交：选择意向参与的招标项目，并在“递交保证金”环节中选择“钱包支付”方式完成递交。 递交前，请务必检查企业钱包可用余额是否充足。如余额不足，请按①及时充值。 潜在投标人对采购文件有疑问请咨询招标机构联系人；对平台操作有疑问请咨询技术支持团队：956100转6，请 在工作时间咨询。 招标公告/采购公告中未尽事宜或与采购文件不符之处，以采购文件为准。 6.响应文件开启时间和地点 响应文件开启在响应文件递交截止时间的同一时间进行，地点为云梦泽平台在线开启，邀请所有供应商的法定 代表人或其委托代理人登录云梦泽平台招标投标专区参加在线开启会议，供应商网未参加开启会议的，视为默认 开启结果。采取视频会议远程开启的，以采购人通知为准。 7.发布公告的媒介 务 本采购公告在云梦泽招标投标专区上发布。 8.联系方式 采购人（或采购执行人）：四川油建国家石油天然气大流商量计量站成都分站高压检定能力建设工程 地址：成都双流区黄甲镇西航港大道中四段2929号工程建设公司四川油建公司生产科研基地采购中心（招标中心） 联 系人：陈羽璨 道 电话：13658018051 电子邮件：chenyc827_sc@cnpc.com.cn 管 2026年8月21日 信息来源:https://www.c国hinapipe.net/project/d3078197.html cqdingjiu 2026.08.24 12:31:51 中</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>加压泵站：4座</t>
+          <t>[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object]</t>
         </is>
       </c>
       <c r="N37" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>重庆, 四川, 管材, 招标, 商机</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>涪陵区龙桥街道农村供水保障能力提升工程招标计划表</t>
+          <t>南江县城污水处理厂水污染治理设施提标改造项目详细勘察服务磋商公告</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3034,7 +3026,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>水利</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3049,53 +3041,57 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>巴中市</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>南江县</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>改造荣桂水厂老化、破损、生锈的输水管道7.36公里。马武水厂增设废水回收及污泥浓缩系统1套。荣桂水厂增设废水回收及污泥浓缩系统1套。新建配水管道总长0.74公里；改造配水管道总长139.42公里。新建1座微型集成泵房及改造1座泵站(原牌坊泵站)。新增管网监测设施40套。</t>
+          <t>详细勘察服务</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>预估合同金额为3236.36万元人民币</t>
+          <t>预算资金：¥389940.00元</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>输水管道、废水回收及污泥浓缩系统、配水管道、微型集成泵房、泵站、管网监测设施</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>涪陵区龙桥街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 涪陵区龙桥街道农村供水保障能力 项目名称 提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水 名称（盖 有限公司 章） 网 项目批准 文件及文 涪陵发改〔2026〕466号 号 改造荣桂水厂老化、破损、生锈的 务 输水管道7.36公里。马武水厂增设 废水回收及污泥浓缩系统1套。荣 桂水厂增设废水回收及污泥浓缩系 主要建设 统1套。新建配水管道总长0.74公里； 商 内容 改造配水管道总长139.42公里。新 建1座微型集成泵房及改造1座泵 站(原牌坊泵站)。新增管网监测设 施40套。 道 招标 合同 招 文件 预估 标 招标方 拟交易 备 招标项目 序号 招标项目名称 计划 金 内 式 场所 注 管 发布 额(万 容 时间 元) 改造荣桂水厂老化、 破损、生锈的输水管 国 道7.36公里。马武水厂 增设废水回收及污泥 重庆 浓缩系统1套。荣桂水 市涪 厂增设废水回收及污 公 陵区 中 涪陵区龙桥街道农村供水保障能力 泥浓缩系统1套。新建 开 1 2026-09 公共 3236.36 提升工程 配水管道总长0.74公里； 招 资源 改造配水管道总 标 交易 长139.42公里。新建1 中心 座微型集成泵房及改 造1座泵站(原牌坊泵 站)。新增管网监测设 施40套。 本计划表所列招标项目信息均为暂 备注 定，最终以实际招标时的信 信息来源:https://www.chinapipe.net/project/d3075556.html cqdingjiu 2026.08.21 10:06:55</t>
+          <t>南江县城污水处理厂水污染治理设施提标改造项目详细勘察服务磋商公告 四川文欣工程项目管理有限公司（采购代理机构）受南江县雾源污水处理有限公司（采购人）的委托，拟对南 江县城污水处理厂水污染治理设施提标改造项目详细勘察服务采用竞争性磋商方式进行采购，特邀请符合本次 采购要求的供应商参加本项目的磋商。 一、采购项目基本情况 1.项目编号：SWUEECG202642431 网 2.项目名称：南江县城污水处理厂水污染治理设施提标改造项目详细勘察服务 3.采购人：南江县雾源污水处理有限公司。 务 4.采购代理机构：四川文欣工程项目管理有限公司。 二、资金情况 预算资金：¥389940.00元（大写：叁拾捌万玖仟玖佰肆拾商元整） 三、采购项目简介： 详细要求详见磋商文件第五章。 道 四、供应商邀请方式 通过在西南联合产权交易所阳光采购平台（https://swueecg.com/#/index）发布公告的方式，邀请符合相应资格条 管 件的供应商参与采购活动。 五、供应商参加本次采购活动应具备下列条件 1.具有独立承担民事责国任的能力； 2.具有良好的商业信誉和健全的财务会计制度； 3.具有履行合同所必需的设备和专业技术能力； 中 4.具有依法缴纳税收和社会保障资金的良好记录； 5.参加本次采购活动前三年内，在经营活动中没有重大违法记录； 6.法律、行政法规规定的其他条件； 7.落实采购政策需满足的资格要求： 本项目属于专门面向中小企业采购的项目,供应商应为中小微企业（监狱企业、残疾人福利性单位视同小微企 业）。 8.采购项目的特殊要求： ①本项目专门面向中小企业采购,供应商应为中小微企业（监狱企业、残疾人福利性单位视同小微企业）； ②供应商须具有建设行政主管部门颁发的工程勘察（岩土工程（勘察））乙级及以上资质； 六、禁止参加本次采购活动的供应商 1.根据《关于在政府采购活动中查询及使用信用记录有关问题的通知》（财库〔2016〕125号）的要求，四川文欣 工程项目管理有限公司将通过“信用中国”网站（www.creditchina.gov.cn）、“中国政府采购网”网站 （www.ccgp.gov.cn）等渠道查询供应商在采购公告发布之日前的信用记录并保存信用记录结果网页截图，拒绝列 入失信被执行人名单、重大税收违法案件当事人名单、政府采购严重违法失信行为记录名单中的供应商报名参 加本项目的采购活动（以联合体形式参加本项目采购活动，联合体成员存在不良信用记录的，视同联合体存在 不良信用记录）。 2.为采购项目提供整体设计、规范编制或者项目管理、监理、检测等服务的供应商，不得参加本采购项目。供应 商为采购人、采购代理机构在确定采购需求、编制磋商文件过程中提供咨询论证，其提供的咨询论证意见成为 磋商文件中规定的供应商资格条件、技术服务商务要求、评审因素和标准、采购合同等实质性内容条款的，视 同为采购项目提供规范编制。 七、磋商文件获取方式、时间、地点： 网 磋商文件自2026年08月21日9:00至2026年08月27日18：00（北京时间，法定节假日除外）在西南联合产权交易所电 子招采平台网站https://www.swueecg.com，按照网上操作流程（资料下载-供应商操作手册）获取。 本项目磋商文件费用¥ 200.00元/份，供应商须通过本单位对公银行账户转账方式交纳磋商文件费用（不接收个 务 人转账），磋商文件售后不退，参加采购活动的资格不能转让。转账前请核实阳光采购平台转账页面的“项目 信息”，认真阅读“注意事项”并按照“支付信息”进行转账，以磋商文件费用到达指定账户为准，在文件获 取截止时间内未到账的不能获取磋商文件，视为报名不成功。 八、递交响应文件截止时间：2026年09月01日9:30（北京商时间）。 九、递交响应文件地点：响应文件必须在递交响应文件截止时间前送达磋商地点（磋商地点：南江县红塔大 道167号红塔锦城3楼）。逾期送达、密封和标注错误的响应文件，四川文欣工程项目管理有限公司恕不接收。本 次采购不接收邮寄的响应文件，但因邮寄导致道投标截止时间以后送达的响应文件，响应文件不予接收。 十、磋商地点：南江县红塔大道167号红塔锦城3楼。 十一、联系方式 管 采 购 人：南江县雾源污水处理有限公司 通讯地址：四川省巴中市南江县集州街道文光社区中院社 国 邮 编：635600 联 系 人：吴先生 中 联系电话：0827-8177739 采购代理机构：四川文欣工程项目管理有限公司 通讯地址：四川省巴中市巴州区体育馆对面龙北街122号三楼 邮 编：635600 联 系 人：秦女士 联系电话：0827-5267676 信息来源:https://www.chinapipe.net/project/d3078163.html cqdingjiu 2026.08.24 12:31:51</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>输水管道：7.36公里；配水管道：0.74公里；配水管道：139.42公里</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N38" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>涪陵区龙桥街道, 农村供水保障能力提升工程, 输水管道, 废水回收及污泥浓缩系统, 配水管道, 微型集成泵房, 泵站, 管网监测设施</t>
+          <t>管材招标, 重庆, 四川, 近三天</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>涪陵区百胜镇农村供水保障能力提升工程招标计划表</t>
+          <t>绵阳市中心医院蒸汽管道改造(第二次)采购公告</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3105,7 +3101,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>水利</t>
+          <t>房建</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3120,38 +3116,42 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>绵阳市</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>绵阳市</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>整治De315原水管长1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。</t>
+          <t>蒸汽管道改造</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>合同金额1489.90万元</t>
+          <t>最高限价：26.7万元</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>管材、水泵、加压泵站、废水处理系统、电气工程</t>
+          <t>蒸汽管道</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>涪陵区百胜镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区百胜镇农村供水保障能力提升工程 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕465号 及文 号 务 主要 建设整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1套及配套电气工程。 内容 招 拟 标 招招标文 合同预 交 序项 标件计划 估金 备 招标内容 易 号目 方发布时 额(万 注 场 名 商 式间 所 元) 称 涪 陵 区 重 百 庆 胜 市 招标 镇 涪 项目 农 道 陵 村 公 区 供整治 De315原水管长 1.66公里及附属设施，更换取水泵站水泵1套，新建及整治输配水管网总长111.47公里及附属设施，管径De25~De200，新建加压泵站2座，百胜水厂新建废水处理系统1开 公 1 2026-09 1489.90 水套及配套电气工程。 招 共 保 标 资 障 源 能 交 力 易 提 中 管 升 心 工 程 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075553.html 国 cqdingjiu 2026.08.21 10:06:55 中</t>
+          <t>绵阳市中心医院蒸汽管道改造(第二次)采购公告 因工作需要，绵阳市中心医院拟对蒸汽管道改造进行竞争性谈判采购，现面向社会公示，诚邀符合条件要求的 供应商参加。 一、项目编号：MYCH竞谈（2026）013号 二、项目名称：蒸汽管道改造 三、最高限价：26.7万元 网 四、采购内容：蒸汽管道改造 五、参加投标的供应商应具备的条件： 务 1. 具有独立承担民事责任的能力。 2. 具有良好的商业信誉和健全的财务会计制度。 商 3. 具有履行合同所必须的设备和专业技术能力。 4. 有依法缴纳税收和社会保障资金的良好记录。 道 5. 供应商参加本次政府采购活动前三年内，在经营活动中没有重大违法记录。 6. 本项目参加政府采购活动的投标人、法定代表人(非法人负责人、自然人本人)在前3年内不得具有行贿犯罪记 录。 管 7. 法律、行政法规规定的其他条件。 8. 特种设备生产许可证--工业管道GC2。 国 9. 安全生产许可证。 六、提交报名文件方式： 中 1、供应商按照附件要求提交响应文件即视为报名成功。（要求详见附件） 2、供应商提交响应文件资料（盖鲜章）要求按顺序扫描成一个PDF文件发送到2242490135@qq.com邮箱，邮件 名为：蒸汽管道改造+公司名称。邮件正文内容为：公司名称、业务员姓名、业务员联系电话，不按照要求发送 邮件将被拒绝报名。 3、提交响应文件截止时间：2026年8月25日17：00 七、开标时间和地点： 1、开标时间和地点电话另行通知。 八、联系人及电话： 项目咨询：唐老师 0816-2229106 报名咨询：刘老师 18081208357 监督电话： 0816-2237353 竞争性谈判文件-蒸汽管道改造.docx 绵阳市中心医院采购科 2026年8月20日 信息来源:https://www.chinapipe.net/project/d3078145.html 网 cqdingjiu 2026.08.24 12:31:51 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>取水泵站水泵：1套；及整治输配水管网：111.47公里；加压泵站：2座</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N39" t="n">
@@ -3159,14 +3159,14 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>涪陵区百胜镇, 农村供水保障能力提升工程, 管材招标, 重庆</t>
+          <t>蒸汽管道改造, 四川</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>涪陵区清溪镇农村供水保障能力提升工程招标计划</t>
+          <t>璞玉源水务2026成都市蒲江县管道直饮水入户项目设计施工总承包招标公告</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>其他/未识别</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3191,38 +3191,42 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>蒲江县</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>对清溪水厂原取水口进行改造。改造清溪厂输水管道长6.38公里。清溪水厂新建3000m³/d集成水厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04公里。四合村泵站增加1套备用加压泵。新增管网监测设施35套。</t>
+          <t>管道直饮水入户项目的建设内容包括设计及施工总承包。</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>合同预估金额：2888.89万元</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>集成水厂、输水管道、配水管道、加压泵、管网监测设施</t>
+          <t>管道直饮水入户设备</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>涪陵区清溪镇农村供水保障能力提升工程招标计划 重庆市工程建设项目招标计划表 项目名称 涪陵区清溪镇农村供水保障能力提升工程 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕467号 务 号 对清溪水厂原取水口进行改造。改造清溪水厂输水管道长6.38公里。清溪水厂新建3000m3/d集成水 主要建设 厂1套，增设废水回收及污泥浓缩系统1套。新建配水管道总长2.46公里。改造配水管道总长145.04 内容 公里。四合村泵站增加1套备用加压泵。新商增管网监测设施35套。 招标项目 招标方 招标文件计 拟交易场 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 所 (万元) 对清溪水厂原道取水口进行 改造。改造清溪水厂输水 管道长6.38公里。清溪水厂 涪陵区清 新建3000m3/d集成水厂1套， 重庆市涪 招标项目 溪镇农村 增设废水回收及污泥浓缩 公开招 陵区公共 管 1 供水保障 2026-09 2888.89 系统1套。新建配水管道总 标 资源交易 能力提升 长2.46公里。改造配水管道 中心 工程 总长145.04公里。四合村泵 站增加1套备用加压泵。新 国 增管网监测设施35套。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075552.html 中 cqdingjiu 2026.08.21 10:06:55</t>
+          <t>璞玉源水务2026成都市蒲江县管道直饮水入户项目设计施工总承包招标公告 详见附件。 信息来源:https://www.chinapipe.net/project/d3077945.html cqdingjiu 2026.08.24 12:31:52 网 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>清溪水厂输水管道：6.38公里；配水管道：2.46公里；四合村泵站：1套；新商增管网：35套；管道：6.38公里；增管网：35套</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N40" t="n">
@@ -3230,14 +3234,14 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>管道直饮水入户项目, 成都市蒲江县, 设计施工总承包</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>涪陵区珍溪镇农村供水保障能力提升工程(一期)招标计划表</t>
+          <t>中国五冶西充县太平水厂、鹤鸣庵水厂及配套管网建设项目劳务分包采购公告</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3247,7 +3251,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>水利</t>
+          <t>其他/未识别</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3262,53 +3266,57 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>南充市</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>西充县</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>改造11000m³/d(旺水垭6000m³/d和二水厂5000m³/d)原水处理系统及辅助设施，主要包括加氯系统、加药系统、清水池、絮凝池、重力无阀滤池、污水处理回收池、二水厂泵房设备等及其他辅助设施。更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km，新建应急泵站至百汇大桥配水管9km；百汇至观将泵站4.5km；共计37.3km。</t>
+          <t>西充县太平水厂、鹤鸣庵水厂及配套管网建设项目劳务分包</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>合同预估金额3427.27万元</t>
+          <t>采购控制价：2761.638256万元（含税）</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>管材</t>
+          <t>劳务分包</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>涪陵区珍溪镇农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区珍溪镇农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕476号 及文号 (一)改造11000m3/d(旺水垭6000m3/d和二水厂5000m3/d)原水处理系统及辅助设施，主要有加氯系统、 加药系统、清水池、絮凝池、重力无阀滤池、商污水处理回收池、二水厂泵房设备等及其他辅助设施。 主要建 (二)更换旺水垭水厂至张家塘配水管13.5km，张家塘至滴水配水管长3.3km，全长16.8km；滴水至洪 设内容 湖配水管长0.3km；更换八一水库至旺水垭水厂引水管1.7km，更换珍溪二水厂至珍溪大桥配水管5km， 新建应急泵站至百汇大桥配水管9km：百汇至观将泵站4.5km；共计37.3km。 道 招标项目 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 名称 式 划发布时间 场所 (万元) (一)改造11000m3/d(旺水 垭6000m3/d和二水厂5000m3/d) 管 原水处理系统及辅助设施，主 要有加氯系统、加药系统、清 水池、絮凝池、重力无阀滤池、 污水处理回收池、二水厂泵房 涪陵国区珍 设备等及其他辅助设施。(二) 重庆市 招标项 溪镇农村 更换旺水垭水厂至张家塘配水 涪陵区 目 供水保障 公开招 1 管13.5km，张家塘至滴水配水 2026-09 公共资 3427.27 能力提升 标 管长3.3km，全长16.8km；滴水 源交易 中工程（一 至洪湖配水管长0.3km；更换八 中心 期） 一水库至旺水垭水厂引水 管1.7km，更换珍溪二水厂至珍 溪大桥配水管5km，新建应急 泵站至百汇大桥配水管9km： 百汇至观将泵站4.5km；共 计37.3km。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075551.html cqdingjiu 2026.08.21 10:06:56</t>
+          <t>中国五冶西充县太平水厂、鹤鸣庵水厂及配套管网建设项目劳务分包采购公告 一、采购人基本信息： 1、采购人名称：中国五冶集团有限公司 2、地址：四川省成都市锦江区五冶路9号 3、联系人：刘工 网 4、电话：028-80803115 二、采购项目概况 务 1、采购名称：西充县太平水厂、鹤鸣庵水厂及配套管网建设项目 劳务分包 2、项目地点：南充市西充县太平镇 商 3、采购范围：西充县太平水厂、鹤鸣庵水厂及配套管网建设项目劳务分包。 4、采购控制价：2761.638256万元（含税） 道 三、投标单位条件 1、资质要求：本次采购要求投标人在中华人民共和国境内注册，具有独立法人资格，具备合法有效的营业执照， 管 具备住建部门颁发的处于有效期内的施工劳务企业资质（不分类别和等级），且具有有效的安全生产许可证； 2、财务要求：提供上一年度经审计的财务报表（带二维码）。 3、业绩要求：能够反国映近年类似工程业绩的合同或竣工验收有效证明。 4、信誉要求：①投标单位没有处于被责令停业、投标资格被取消、财产被接管、冻结或破产状态等；②近三年 内没有发生骗取中标及发生重大质量、安全或诚信等严重违约、失信或违法问题；③投标单位应为“中国五矿 集团有限公司供应链管理平台（http：//ec.minmetals.com.cn/）”已准入供方；不在中国五矿集团供应商“黑名 中 单”中，服务关系未被五冶集团停用或被评为D级，在五冶内无不良记录。④近三年无直接起诉或仲裁采购人的 案件，且无连带采购人被诉并承担责任的诉讼或仲裁。 5、经营状态：无异常； 6、其他要求：须组建完整健全的项目团队，相应岗位须具备匹配岗位的证书，且团队人员必须是投标单位在册 员工。（包括项目经理、技术负责人、安全员、质量员、材料员、劳资员等）； 7、本次招标不接受联合体投标。 四、资格预审文件的获取 凡有意参加本次采购内容的投标单位，请于本公告发布之日起通过中国五矿集团有限公司供应链管理平台（网 址：https://ec.minmetals.com.cn/）按《资格预审申请表》（详见附件）提交申请。 五、资格预审文件提交截止时间 资格预审文件提交截止时间为2026年8月28日19：00(北京时间)，逾期提交的将被系统拒绝。 时间： 2026 年8月 21 日 信息来源:https://www.chinapipe.net/project/d3077864.html cqdingjiu 2026.08.24 12:31:53 网 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>应急泵站：9km；百汇至观将泵站：4.5km；泵站：9km</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N41" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 供水, 改造</t>
+          <t>四川, 劳务分包, 管材</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>涪陵区武陵山镇农村供水保障能力提升工程招标计划表</t>
+          <t>自贡水务投资集团有限公司供水管道及设施防腐招采公告</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3318,7 +3326,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>水利</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3333,53 +3341,57 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>自贡市</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>自贡市</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>新建及整治输配水管网总长124.26千米，新建加压泵站5座，新建高位水箱4座（总容积354立方米），武陵山水厂新建废水处理系统1套及配套电气工程等。</t>
+          <t>钢管及设施防腐</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>合同预估金额1861.77万元</t>
+          <t>最高限价80万元</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>输配水管网、加压泵站、高位水箱、废水处理系统、电气工程</t>
+          <t>钢管及设施防腐</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>涪陵区武陵山镇农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区武陵山镇农村供水保障能力提升工程 名称 招标 网 法人 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 务 （盖 章） 项目 批准 商 文件 涪陵发改〔2026〕468号 及文 号 主要 道 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高位水箱4座（总容积 354立方米），武 建设 陵山水厂新建废水处理系统1套及配套电气工程等。 内容 招 管 拟 标 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 国 称 涪 陵 区 中 重 武 庆 陵 市 山 招标 涪 镇 项目 陵 农 公 区 村 新建及整治输配水管网总长 124.26千米，新建加压泵站 5座，新建高 开 公 1 供 位水箱4座（总容积 354立方米），武陵山水厂新建废水处理系统1套 2026-09 1861.77 招 共 水 及配套电气工程等。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075549.html cqdingjiu 2026.08.21 10:06:56</t>
+          <t>自贡水务投资集团有限公司供水管道及设施防腐招采公告 自贡水务投资集团有限公司现对供水管道及设施防腐招采项目进行公开招采，现以公 告方式邀请符合本次招采要求的承包商参加招采，内容如下： 一、公告网址：自贡水务投资集团有限公司（http://www.zgwater.com） 二、项目名称：自贡水务投资集团有限公司供水管道及设施防腐招采项目 网 三、承包金额：最高限价80万元。 四、合同有效期限：贰年。 务 五、承包内容：钢管及设施防腐（见下表） 序号 项目名称 规格型号 单位 数量 商 三水厂部分 1 西部水厂管廊管道及加压站部分管道防腐 / ㎡ 500 2 钢制设施、 / ㎡ 6100 设备防腐 3 高新区景苑小区管道防腐 / ㎡ 55 道 4 长葫引水管道DN1200钢管防腐 DN1200 ㎡ 1380 5 一桥硬合厂宿舍侧DN400钢管防腐 DN400 ㎡ 16.5 6 一桥硬合厂宿舍侧DN300钢管防腐 DN300 ㎡ 14.15 管 合计 8065.65 六、中选承包商确定方式：采用最低价法，按总价最低原则确定1家为中选承包商。 国 七、承包商参加本次招采活动应具备的条件： 1、承包商营业执照经营范围须包含承包内容； 中 2、具有独立承担民事责任能力； 3、具有良好的商业信誉和健全的财务会计制度； 4、具有履行施工合同所必须的资金实力、施工专业团队和能力； 5、有依法缴纳税收和社会保障资金的良好记录； 6、参加国内招标等活动前三年内，在经营活动中没有重大违法记录； 7、本项目不接受联合体参加，单位负责人为同一人或存在控股、管理或存在其他利益关系的不同单位，不得同 时参加本次招采。 八、禁止参加本次招采活动的承包商 根据相关规定，拒绝列入失信被执行人名单、重大税收违法案件当事人名单、严重违法失信行为记录名单中的 承包商报名参加本次招采活动。 九、报名方式、时间、地点： 1、报名方式：现场报名、网上报名 1）现场报名：承包商将单位营业执照复印件、防水防腐保温工程专业承包贰级及以上资质证书、《授权委托 书》、经办人身份证复印件、《承包商报名登记表》（均加盖单位公章）交到四川省自贡市自流井区华商北 路199号华商.国际城30栋（自贡水务投资集团有限公司907室）。 2）网上报名：承包商将单位营业执照复印件、防水防腐保温工程专业承包贰级及以上资质证书、《授权委托 书》、经办人身份证复印件、《承包商报名登记表》扫描件（均加盖单位公章）发送至308896569@qq.com。 2、报名截止时间为：2026年8月28日。 3、招采承包文件免费获取，报名后招采资格不能转让。 备注：由承包商自行选择报名方式，招采人依据报名提交的资料收取响应文件。 网 十、递交响应文件截止时间：2026年9月9日上午12:00（北京时间）。 十一、递交响应文件地点：四川省自贡市自流井区华商北路199号华商.国际城30栋11-01号（自贡水务投资集团有 限公司907室，联系人：王文祥）。响应件必须在递交响应文件截止时间前送达招采地点。逾期送达、密封和标 务 注错误的响应文件，招采单位恕不接收。本次招采接收邮寄的响应文件。 十二、项目评审时间：由招采方自行确定时间组织评审。 十三、招采结果：招采结果会在响应文件递交截止时间后商的15个工作日之内在本网站公布。 十四、联系方式 1、招采人：自贡水务投资集团有限公司 道 2、地 址：四川省自贡市自流井区华商北路199号华商.国际城30栋11-01号（自贡水务投资集团有限公司907室） 3、联系人及电话：王文祥 0813-2203668 管 信息来源:https://www.chinapipe.net/project/d3077586.html cqdingjiu 2026.08.24 12:31:53 国 中</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>及整治输配水管网：124.26千米；加压泵站：5座</t>
+          <t>西部水厂管廊管道及加压站部分管道防腐 500㎡，钢制设施、设备防腐 6100㎡，高新区景苑小区管道防腐 55㎡，长葫引水管道DN1200钢管防腐 1380㎡，一桥硬合厂宿舍侧DN400钢管防腐 16.5㎡，一桥硬合厂宿舍侧DN300钢管防腐 14.15㎡</t>
         </is>
       </c>
       <c r="N42" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>涪陵区武陵山镇, 农村供水保障能力提升工程, 重庆, 输配水管网, 加压泵站, 高位水箱, 废水处理系统, 电气工程</t>
+          <t>重庆, 四川, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>涪陵区江东街道农村供水保障能力提升工程(一期)招标计划表</t>
+          <t>射洪市2026年高标准农田建设项目(复兴及潼射片区)-施工-1招标公告</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3404,53 +3416,57 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>遂宁市</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>射洪市</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>建设配水管网总长34.80km，新建加压泵站2座、改造已成泵站2座、新建加氯加药间1座、新建高位水箱7座、新建计量监测设施以及配套电气工程。</t>
+          <t>本项目包括新建及改建高标准农田，涉及田块整治工程、灌溉排水工程、田间道路工程、土壤改良、农田输配电工程、农田防护与生态保护工程。</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>合同预估金额3503.77万元</t>
+          <t>项目资金来自中央投资、省级配套资金、县级配套资金，出资比例为100%。</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>配水管网、加压泵站、加氯加药间、高位水箱、计量监测设施、电气工程</t>
+          <t>高标准农田建设相关材料与设备</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>涪陵区江东街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目名 涪陵区江东街道农村供水保障能力提升工程（一期） 称 招标法 网 人或招 重庆水务环境控股集团渝东自来水有限公司 标人名称 （盖章） 项目批 务 准文件 涪陵发改〔2026〕470 号 及文号 主要建 建设配水管网总长 34.80km，新建加压泵站 2 座、改造已成泵站 2 座、新建加氯加药间 1 座、新建高位 设内容 水箱 7 座、新建计量监测设施以及配套电气工程商。 招 招标文件 拟交 合同预估 序 招标项 标 备 招标内容 计划发布 易场 金额(万 号 目名称 方 注 道 时间 所 元) 式 涪陵区 重庆 招标项 江东街 市涪 目 建设配水管网总长 34.80km，新建加压泵站 2 座、 公 道农村 陵区 管 改造已成泵站 2 座、新建加氯加药间 1 座、新建高 开 1 供水保 2026-09 公共 3503.77 位水箱 7 座、新建计量监测设施以及配套电气工 招 障能力 资源 程。 标 提升工程 交易 （一期） 中心 国 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075548.html cqdingjiu 20中26.08.21 10:06:56</t>
+          <t>射洪市2026年高标准农田建设项目(复兴及潼射片区)-施工-1招标公告 1. 招标条件 1.1本招标项目射洪市2026年高标准农田建设项目（复兴及潼射片区）（项目名称）已由射洪市发展和改革局 （项目审批、核准或备案机关名称）以射洪市发展和改革局关于射洪市2026年高标准农田建设项目可行性研究报 告的批复（射发改发〔2025〕421号）（批文名称及编号）批准建设，项目业主为射洪市茂乾实业有限责任公司， 建设资金来自中央投资、省级配套资金、县级配套资金（资金来源），出资比例为100%，招标人为射洪市茂乾 实业有限责任公司。项目已具备招标条件，现对该项目的 / 施工进行公开招标。 网 1.2本招标项目为遂宁市行政区域内的国家投资工程建设项目，射洪市发展和改革局（核准机关名称）核准（招 标事项核准文号为射发改发〔2025〕421号）的招标组织形式为 委托招标。招标人选择的招标代理机构是四川 丰和工程管理有限公司。 务 2. 项目概况与招标范围 2.1 项目概况 2.1建设地点：复兴片区：金凤社区、大龙村、雷堂村、玉商贞村、观花村、金罐村、新桥村、红桂桥村、灵华村、 博古村、喻家沟村、九圣村；潼射片区：板桥沟村。 2.2规模：新建及改建高标准农田（含田块整冶工程、灌溉排水工程、田间道路工程、土壤改良、农田输配电工 程、农田防护与生态保护工程）。 道 2.3工期：270日历天。 2.4标段划分：复兴及潼射片区施工标段。_（简要说明本次招标项目的建设地点、规模、建设内容、计划工期、 管 标段划分等）。 2.2 招标范围 本项目工程量清单及图国纸范围所示的全部内容_（简要说明本次招标标段名称、招标范围与内容、合同计划工期 等）。 3. 投标人资格要求 中 3.1本次招标要求投标人须具备行政主管部门颁发的水利水电工程施工总承包贰级及以上资质，并在人员、设备、 资金等方面具有相应的施工能力。 3.2本次招标 不接受联合体投标。 3.3各投标人均可就上述合同标段中的1个(具体数量)合同标段投标。招标人不允许投标人拟派的同一批项目主要 人员（项目经理、技术负责人）在1个及以上标段任职。 4. 招标文件的获取 4.1 凡有意参加投标者，请于2026年08月22日00时00分至2026年09月13日17时00分开始登陆：全国公共资源交易 平台（四川省· 遂宁市）（网址：https://www.snsggzyjy.cn ）—“登录”—“遂宁市建设工程网上交易后台管理 系统”，通过数字证书免费下载招标资料（招标文件、技术资料等）（报名结束时间为2026年9月13日17时00 分）。 4.2 除上述方式外，招标人不提供其他任何报名和招标文件获取的方式。 5. 投标文件的递交 5.1投标文件递交的截止时间（投标截止时间，下同）为2026年09月14日09时30分，投标人应在投标截止时间前在 线递交经投标人数字证书加密的数据电文形式投标文件。 6. 发布公告的媒介 本次招标公告在全国公共资源交易平台（四川省）上发布。其他发布公告的媒介全国公共资源交易平台（四川 省·遂宁市）（招标人自行选择，也可不填）。 7. 本项目招标投标行政监督部门 行政监督部门：射洪市农业农村局电 话：0825-6681313 传 真：/ 电子邮件：/ 地 址：射洪市广寒路 网 8. 招标人承诺 本招标文件已经招标人（含招标代理机构）审查，不存在违反国家法律、法规、政策的情形。因招标文件设置 违反国家法律、法规、政策造成的相应后果，由招标人（含招标代理机构）负责。 务 9. 联系方式 招 标 人：射洪市茂乾实业有限责任公司招标代理机构：四川丰和工程管理有限公司 商 地 址：射洪市紫云文化公园B-6栋地 址：中国（四川）自由贸易试验区成都高新区益州大道中段722 号3栋1单元21楼2104号 邮 编：629200邮 编：610041 道 联 系 人：谭老师联 系 人：王女士 电 话：0825-6915636电 话：028-85251050 管 传 真：/ 传 真：/ 电子邮件：/电子邮件：/ 国 网 址：/网 址：/ 开户银行：/开户银行：中国银行雅安雨城区支行 中 账 号：/账 号 ：130737176102 信息来源:https://www.chinapipe.net/project/d3077563.html cqdingjiu 2026.08.24 12:31:54</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>配水管网：34.80km；加压泵站：2座；已成泵站：2座</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N43" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>重庆, 农村供水保障能力提升工程, 配水管网, 加压泵站, 加氯加药间, 高位水箱, 计量监测设施, 电气工程</t>
+          <t>高标准农田, 新建及改建, 水利工程, 四川, 遂宁</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>中国电建水电五局二公司重庆轨道交通17号线一期7标内外涂环氧消防复合钢管管件采购项目公开竞价采购(二次挂网)变更公告(一)</t>
+          <t>盐边县城北片区和清源片区老旧街区改造项目施工一标段招标公告</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3460,7 +3476,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>市政</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3475,49 +3491,57 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>攀枝花市</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>盐边县</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>详见附件。</t>
+          <t>对盐边县城北、清源片区老旧街区进行商提升改造，包括改造中环北路、西环北路、清河西路、盐中巷外立面排危改造约12.28万平方米，街区路面整治约12000平方米，街区雨污排水管网改造约10千米，改造适老化、适儿化服务用房约5000平方米，社区综合服务生活市场改造8500平方米，街区屋面防水改造约9900平方米，改造3500平方米街区边角地配套停车场及充电桩等基础设施，增设路灯280盏，公共活动健身区15处，街角口袋公园4处，改造清河西路、盐中巷街区安道全防护栏5公里，街区架空线入地4千米，弱电管网整治5千米，并同步完善消防、安防、垃圾收储、便民生活设施等配套公共服务设施。</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>项目总投资额：14500万元。</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>内外涂环氧消防复合钢管管件</t>
+          <t>市政公用工程施工总承包</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>中国电建水电五局二公司重庆轨道交通17号线一期7标内外涂环氧消防复合钢管管件采购项目公开竞价采购(二次 挂网)变更公告(一) 详见附件。 信息来源:https://www.chinapipe.net/project/d3075376.html cqdingjiu 2026.08.21 10:06:56 网 务 商 道 管 国 中</t>
+          <t>盐边县城北片区和清源片区老旧街区改造项目施工一标段招标公告 1. 招标条件 1.1本招标项目盐边县城北片区和清源片区老旧街区改造项目(项目名称)已由盐边县发展和改革局(项目 审批、核准或备案机关名称)以关于盐边县城北片区和清源片区老旧街区改造项目可行性研究报告的批复、盐边 发改〔2025〕301号（批文名称及编号）批准建设，项目业主为盐边发展（集团）有限责任公司，建设资金来自 争取上级资金及业主自筹（资金来源），项目出资比例为 100% ，招标人为盐边发展（集团）有限责任公司。 项目已具备招标条件，现对该项目的施工进行公开招标。 网 1.2本招标项目由盐边县发展和改革局 （核准机关名称）核准（招标事项核准文号为盐边发改〔2025〕301号） 的招标组织形式为委托招标（□自行招标委托招标）。招标人选择的招标代理机构是四川骏浩达工程项目管 理有限公司。 务 2. 项目概况与招标范围 2.1 建设地点：盐边县城北片区和清源片区。 2.2 项目规模：拟对盐边县城北、清源片区老旧街区进行商提升改造，包括改造中环北路、西环北路、清河西路、 盐中巷外立面排危改造约12.28万平方米，街区路面整治约12000平方米，街区雨污排水管网改造约10千米，改造 适老化、适儿化服务用房约5000平方米，社区综合服务生活市场改造8500平方米，街区屋面防水改造约9900平方 米，改造3500平方米街区边角地配套停车场及充电桩等基础设施，增设路灯280盏，公共活动健身区15处，街角 口袋公园4处，改造清河西路、盐中巷街区安道全防护栏5公里，街区架空线入地4千米，弱电管网整治5千米，并同 步完善消防、安防、垃圾收储、便民生活设施等配套公共服务设施。 本项目一标段建设内容：对盐边县城北片区中环北路周边房屋外立面排危改造，进行污水管网、雨水管网、局 部给水管网、绿化改造，飞线整治、社区综合服务生活市场改造，并同步完善消防、安防、垃圾收储、便民生 管 活设施等配套公共服务设施。 2.3 项目总投资额：14500万元。 2.4 计划工期：180日历国天。 2.5 招标范围：包括但不限于施工图纸（含变更）和相应工程量清单中的全部工程内容及竣工验收合格及整体 移交、工程保修期内的缺陷修复和保修工作等内容。 中 2.6 标段划分：施工1个标段。 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 3.1本次招标要求投标人须具备 3.1.1资质条件：具有独立法人资格；具有建设行政主管部门颁发的市政公用工程施工总承包二级及以上资质；具 有有效的安全生产许可证。 3.1.2业绩要求： 近年（ 2021 年 1 月 1 日至投标截止时间，不少于3年）（□已完成已完成或新承接或正在施工） 不少于 1 （1至3个）个类似项目。类似项目是指:单项合同金额不低于2000万元的市政工程类项目施工业绩。 □无业绩要求。 3.1.3项目经理的资格要求： 项目经理（项目负责人）资格：市政公用工程 (注册专业)二级及以上（级别）建造师，具有省级及以上住房 城乡建设主管部门颁发的安全生产考核合格证（B证）， / （业绩要求），须为本单位人员（若为联合 体投标，须为联合体牵头人人员）。 □园林绿化工程项目经理（项目负责人）资格： / （职称级别）专业技术职称， / （业绩要 求），须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受不接受联合体投标。联合体投标的，应满足下列要求： / 。 3.3各投标人均可就上述 1 (具体数量)标段投标。 3.4本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东网为大企业、与大企业的负责 人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具体 标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的通 知》（工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除技术 复杂、存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在3000万元以下的施工项目(标段)应勾 务 选此项。） 4. 招标文件的获取 4.1凡有意参加投标者，请于 2026 年 8 月 22 日开始登陆商：□全国公共资源交易平台（四川省） （网址：http://ggzyjy.sc.gov.cn）—“登录”——“交易主体”—“建设工程”，通过数字证书免费下载招标资料 （招标文件、技术资料等）。全国公共资源交易平台（四川省· 攀枝花 市（州））（网 址： http://ggzy.panzhihua.gov.cn/ ）—“登录”—“ 建设工程 ”，通过数字证书免费下载招标资料（招标 文件、技术资料等）。 道 4.2 招标人不提供招标文件获取的其他方式。 5. 投标文件的递交 管 投标文件递交的截止时间（投标截止时间，下同）为 2026 年 9 月 14 日 9 时 30分，投标人应在投 标截止时间前在线递交经投标人数字证书加密的数据电文形式投标文件。 6. 发布公告的媒介 国 本次招标公告在《全国公共资源交易平台（四川省）》和全国公共资源交易平台（四川省.攀枝花 市） (公告发布的其它媒介名称）上发布。 中 7. 行政监督部门 单位名称：盐边县住房和城乡建设局 联系电话：0812-8653726 8. 联系方式 招 标 人：盐边发展（集团）有限责任公司 地 址：四川省盐边县新九镇盐边钒钛产业开发区钛兴南路1号 邮 编：617100 联 系 人：任老师 电 话：0812-8655576 传 真： / 电子邮件： / 网 址： / 开户银行： / 账 号： / □ 招标代理机构： / 招标代理机构：四川骏浩达工程项目管理有限公司 网 地 址：四川省攀枝花市盐边县桐子林镇中环南路146号 邮 编：617100 务 联 系 人：袁溢龙 项目负责人：袁溢龙 商 电 话：0812-8655535 传 真： / 道 电子邮件： / 网 址： / 管 开户银行： / 账 号： / 国 中 2026 年 8 月 21 日 注： （1）若划分标段，则填写标段序号；若划分为两个及以上标段，应分别明确各标段的具体内容、划分情况。 （2）招标人对投标人的资质要求，应是国家对投标人资质的强制性规定。不是国家规定必须具备的资质，不得 作为资质要求。 （3）招标人对投标人的类似项目业绩要求，设置的投资额、面积、长度等规模量化指标不得高于本次招标工程 相应指标，类似项目业绩的定义应明确，用语准确无歧义。 （4）招标人要求投标人需具备的资质一个项目（标段）为一个，因特殊情况需要两个以上资质的，应当接受投 标人组成联合体投标，且限定的联合体成员数量不得少于设定的资质个数。 信息来源:https://www.chinapipe.net/project/d3077560.html cqdingjiu 2026.08.24 12:31:54 网 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>雨污排水管网：10千米；弱电管网：5千米</t>
         </is>
       </c>
       <c r="N44" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>重庆, 四川, 管材, 招标</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>涪陵区蔺市街道农村供水保障能力提升工程(一期)招标计划表</t>
+          <t>川东北现代农业融合发展示范园项目设计施工总承包招标公告</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3542,53 +3566,57 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>南充市</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>南充市</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>新建、更换配水管网396.72km（dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。</t>
+          <t>本项目总占地面积为149道225.64平方米，总建筑面积151550.12平方米，其中新建标准化厂房143913平方米、综合管理用房7637.12平方米，配套建设配套厂区道路、停车场、绿化工程、污水管网、给水管网、强弱电工程等配套工程。</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>合同金额：3611.91万元</t>
+          <t>项目总投资36633万元</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>dn20-dn160PE管、DN40-DN250抗菌耐磨涂塑钢管</t>
+          <t>设计施工总承包</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>涪陵区蔺市街道农村供水保障能力提升工程(一期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（一期） 名称 招标 法人 或招 标人重庆水务环境控股集团渝东自来水有限公司 名称 网 （盖 章） 项目 批准 文件涪陵发改〔2026〕474号 及文 号 主要 务 建设新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收及污泥浓缩处理系统。 内容 拟 招招标文 合同预 招标 交 序 标件计划 估金 备 项目招标内容 易 号 方发布时 额(万 注 名称 场 式间 元) 所 商 重 庆 涪陵 市 区蔺 招标 市街 涪 项目 道农 陵 公 区 村供 新建、更换配水管网 396.72km（dn20-dnl60PE管、DN40-DN250抗菌耐磨涂塑钢管）及配套附属设施;新建测控井108座；调蓄水箱1座;泵房设备更换2台；蔺市水厂、龙泉水厂配套废水回收 开 公 1 水保 2026-09 3611.91 及污泥浓缩处理系统。 招 共 障能 道 标 资 力提 源 升工程 交 （一 易 期） 中 心 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075278.html 管 cqdingjiu 2026.08.21 10:06:57 国 中</t>
+          <t>川东北现代农业融合发展示范园项目设计施工总承包招标公告 1. 招标条件 1.1本招标项目川东北现代农业融合发展示范园项目(项目名称)已由西充县发展和改革局(项目审批、核准或备 案机关名称)以川投资备【2605-511325-04-01-291937】FGQB-0492 号（批文名称及编号）批准建设，项目业主为 西充县德恒建设开发有限责任公司， 建设资金来自企业自筹、银行贷款以及东西部协作资金（资金来源），项 目出资比例为100%，招标人为西充县德恒建设开发有限责任公司。项目已具备招标条件，现对该项目的设计施 工总承包进行公开招标。 网 1.2本招标项目由西充县发展和改革局（核准机关名称）核准（招标事项核准文号为川投资备 【2605-511325-04-01-291937】FGQB-0492 号）的招标组织形式为委托招标。 招标人选择的招标代理机构是四川云 霓工程管理咨询有限公司。 务 2. 项目概况与招标范围 2.1 项目名称：川东北现代农业融合发展示范园项目。 商 2.2建设地点：南充市临江新区西充片区。 2.3建设内容及规模：本项目总占地面积为149道225.64平方米，总建筑面积151550.12平方米，其中新建标准化厂 房143913平方米、综合管理用房7637.12平方米，配套建设配套厂区道路、停车场、绿化工程、污水管网、给水管 网、强弱电工程等配套工程。 2.4计划工期：720日历天。 管 2.5招标范围：本项目设计内容包括但不限于:施工图设计及设计经济测算(含总体投资、清单预算编制等)工作以 及后续配合服务。本项目施工内容包括但不限于:本工程的全部施工设计图纸所表达的范围，项目整体交付以及 竣工验收合格后工程缺陷责任期内的缺陷修复和工程保修等相关工作。 国 2.6标段划分：设计施工总承包1个标段。 2.7标段投资额：项目总投资36633万元。 中 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 3.1本次招标要求投标人须具备 3.1.1资质要求：设计资质要求：具备独立法人资格，具备建设行政主管部门颁发的建筑行业（建筑工程）设计 专业乙级及以上资质；施工资质要求：具备独立法人资格，具备建设行政主管部门颁发的建筑工程施工总承包 二级及以上资质，施工单位须具备有效的安全生产许可证。 3.1.2业绩要求：（本项为多选） □ 设计业绩要求：近年（ 年 月 日 至投标截止时间，不少于3年） 不少 于 （1 至3个）个类似项目。类似项目是指: 。 □ 施工业绩要求：近年（ 年 月 日 至投标截止时间，不少于3年） 不少 于 （1 至3个）个类似项目。类似项目是指: 。 无业绩要求。 3.1.3项目经理的资格要求：具有建筑工程专业二级及以上注册建造师证书□ 由设计负责人兼任由施工负 责人兼任，/（业绩要求），须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.1.4设计负责人的资格要求：具有二级及以上注册建筑师证书，须为投标人本单位人员。 3.1.5施工负责人（建造师，下同）的资格要求：具有建筑工程专业二级及以上注册建造师证书(注册专业)（级 别）建造师，具有省级及以上住房城乡建设主管部门颁发的安全生产考核合格证（B证），须为投标人本单位人 员。 3.2本次招标接受联合体投标。联合体投标的，联合体牵头人应为 □ 设计单位施工单位，同时满足下列要求： ①联合体成员须具有独立法人资格或有效的营业执照，②组成联合体的成员不得超过3家；③联合体各方应签订 联合体协议书，明确联合体牵头人和各方权利义务，并由联合体各方向招标人承担连带责任；④组成联合体投 标应符合相关法律法规对联合体投标的有关规定，联合体各方不得再以自己名义单独或参加其他联合体在同一 工程项目中投标；⑤联合体牵头人负责本项目递交投标文件、缴纳投标保证金等网相关事宜。 □ 3.3 本次招标范围中施工部分的工作仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东为大 企业、与大企业的负责人为同一人的情形的企业均不属于中小企业。若为联合体投标的，本项目联合体协议书 中职责分工为承揽施工工作的所有单位均应属于中小企业）。具体标准以《工业和信息化部、国家统计局、国 务 家发展和改革委员会、财政部关于印发中小企业划型标准规定的通知》（工信部联企业〔2011〕300号）中 的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除技术复杂、存在特殊要求外，我市依法必须 招标的国家投资工程，施工部分招标控制价在8000万元以下3000万元以上的，原则上勾选此项。） 商 □ 3.4 本次招标范围中施工部分的工作仅面向小微企业发包（其中属于大、中企业的分支机构、存在控股股东 为大、中企业、与大、中企业的负责人为同一人的情形的企业均不属于小微企业。若为联合体投标的，本项目 联合体协议书中职责分工为承揽施工工作的所有单位均应属于小微企业）。具体标准以《工业和信息化部、国 家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的通知》（工信部联企业 〔2011〕300号）中的“建筑业”划型标准为准道，投标人应提供小微企业声明函。（除技术复杂、存在特殊要求 外，我市依法必须招标的国家投资工程，施工部分招标控制价在3000万元及以下的，原则上勾选此项。） 4. 招标文件的获取 管 4.1 凡有意参加投标者，请于 2026年08月22日 00时00分 开始，登录全国公共资源交易平台（四川省）（网 址：http://ggzyjy.sc.gov.cn）-&gt;交易平台入口-&gt;南充市-&gt;南充交易系统-建设网、或登录《四川建设网》 （http://www.sccin.com）-&gt;电子招标-&gt;南充市公共资源交易平台登录入口，投标人凭单位CA数字证书（包括但 不限于CFCA、四川CA、重庆CA、天威诚信等）登录，免费获取招标文件（联系电话：028-85569858）。 国 4.2 除上述方式外，招标人不提供其他任何报名和招标文件获取的方式。 5. 投标文件的递交 中 5.1 投标文件递交的截止时间（投标截止时间，下同）为 2026年09月11日 09时10分 ，投标人应在投标截止时间 前，登录全国公共资源交易平台（四川省）（网址：http://ggzyjy.sc.gov.cn）-&gt;交易平台入口-&gt;南充市-&gt;南充交易 系统-建设网、或登录《四川建设网》（http://www.sccin.com）-&gt;电子招标-&gt;南充市公共资源交易平台登录入口， 凭单位CA数字证书登录，在线递交经投标人数字证书签名制作的数据加密电子投标文件。开标地点为：南充市 公共资源交易服务中心（南充市涪江路19号五楼）本项目开标室。 5.2 逾期送达的或者未送达指定地点的投标文件，招标人不予受理。 6. 发布公告的媒介 本次招标公告在《全国公共资源交易平台（四川省）》和四川建设网(公告发布的其它媒介名称）上发布。 7. 行政监督部门 单位名称：西充县住房和城乡建设局 联系电话：0817-4222761 8. 联系方式 □ 招标代理机构： / 招标代理机构：四川云霓工程管理咨询有 招 标 人：西充县德恒建设开发有限责任公司 限公司 地 址：四川省南充市西充县南台街道城南新区数字西充城市超 地 址：成都市武侯区西部智谷D区4 脑三楼303室 栋1单元502号 邮 编：637200 邮 编：610000 联 系 人：张先生 联 系 人：周女士 电 话：0817-8050003 项目负责人：潘云霄 传 真：/ 电 话：028-87776867 电子邮件：/ 传 真：/ 网 址：/ 电子邮件：网/ 开户银行：/ 网 址：/ 账 号：/ 开户银行：/ 账 号：/ 务 商 注： （1）若划分标段，则填写标段序号；若划分为两个及以上标段，应分别明确各标段的具体内容、划分情况。 （2）招标人对投标人的资质要求，应是国家道对投标人资质的强制性规定。不是国家规定必须具备的资质，不 得作为资质要求。 （3）招标人对投标人的类似项目业绩要求，设置的投资额、面积、长度等规模量化指标不得高于本次招标工 程相应指标，类似项目业绩的定义应明确，用语准确无歧义。 管 （4）招标人限定的联合体成员数量不得少于设定的资质个数。 信息来源:https://www.chinapipe.net/project/d3077557.html 国 cqdingjiu 2026.08.24 12:31:54 中</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>配水管网：396.72km</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N45" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 商机</t>
+          <t>现代农业融合发展示范园项目, 设计施工总承包, 四川, 南充市, 西充片区, 36633万元</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>涪陵区李渡街道农村供水保障能力提升工程招标计划表</t>
+          <t>广元市朝天区污水管网提升改造项目(六标段)施工招标公告</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3613,38 +3641,42 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>广元市</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>朝天区</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>改造李渡街道15个村（社区）配水主支管道，更换配水主管网193.71千米（DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治3座，新建测控井78座。</t>
+          <t>中子镇转斗（含何家坝）、校场坝生活污商水处理站覆盖范围内的排水管网更新改造以及检查井等附属设施建设。</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>项目批准文件：涪陵发改[2026]469号</t>
+          <t>项目估算总投资10498.09万元，资金来源为争取上级资金及地方政府配套资金。</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>DN250-DN40抗菌耐磨涂塑钢管、dn40-dn25PE管</t>
+          <t>排水管网更新改造及附属设施建设</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>涪陵区李渡街道农村供水保障能力提升工程招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区李渡街道农村供水保障能力提升工程 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕469号 及文 号 商 主要 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂塑钢管、dn40-dn25PE管）及配套 建设 附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建测控井78座。 内容 招 拟 标 道 招 招标文 合同预 交 序 项 标 件计划 估金 备 招标内容 易 号 目 方 发布时 额(万 注 场 名 式 间 元) 所 称 管 涪 陵 区 重 李 庆 渡 市 街 国 招标 涪 道 项目 陵 农 公 区 村 改造李渡街道 15个村（社区）配水主支管道，更换配水主管网 193.71 千米（DN250-DN40 抗菌耐磨涂 开 公 1 供 塑钢管、dn40-dn25PE管）及配套附属设施，泵站改造1座，新建集成泵站4座，蓄水池整治 3座，新建 2026-09 2372.74 招 共 水中测控井78座。 标 资 保 源 障 交 能 易 力 中 提 心 升 工 程 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075277.html cqdingjiu 2026.08.21 10:06:57</t>
+          <t>广元市朝天区污水管网提升改造项目(六标段)施工招标公告 1. 招标条件 1.1本招标项目广元市朝天区污水管网提升改造项目(项目名称)已由 广元市朝天区发展和改革局(项目审批、核 准或备案机关名称)以 广朝发改项目[2024]108号 （批文名称及编号）批准建设，项目业主为 广元市朝天区 城市建设开发有限责任公司 ，建设资金来自争取上级资金及地方政府配套资金（资金来源），项目出资比例 为 100% ，招标人为广元市朝天区城市建设开发有限责任公司 。项目已具备招标条件，现对该项目的施 工进行公开招标。 网 1.2本招标项目由 广元市朝天区发展和改革局 （核准机关名称）核准（招标事项核准文号为 广朝发改项 目[2024]108号 ）的招标组织形式为 委托招标（□自行招标 委托招标）。招标人选择的招标代理机构 是 中科标禾工程项目管理有限公司 。 务 2. 项目概况与招标范围 2.1 建设地点：朝天区中子镇（转斗、校场坝） 。 2.2 建设规模： 中子镇转斗（含何家坝）、校场坝生活污商水处理站覆盖范围内的排水管网更新改造以及检查 井等附属设施建设 。 2.3 计划投资及资金来源：项目估算总投资 10498.09万元。资金来源为争取上级资金及地方政府配套资金 。 道 2.4 计划工期： 240日历天 。 2.5 招标范围：本项目施工图纸及清单范围内所包含的全部工作内容的施工。 管 2.6 标段划分：施工1个标段。 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 国 3. 投标人资格要求 3.1 本次招标要求投标人须具备： 中 3.1.1 资质条件：具备独立企业法人资格，具备建设行政主管部门颁发的 市政公用工程施工总承包三级及以上资质（须具备有效的安全生产许可证）。 3.1.2 业绩要求： □近年（ 年 月 日至投标截止时间，不少于 3 年）（多项选择： □已完成□已完成或 新承接或正在施工）不少于 （ 1 至 3 个）个类似项目。类似项目是 指: 。 无业绩要求。 3.1.3 项目经理的资格要求： 项目经理（项目负责人）资格： 市政公用工程(注册专业)二级及以上(级别)建造师，具有省级及以上住房城 乡建设主管部门颁发的安全生产考核合格证（B 证），/ （业绩要求） ，须为本单位人员（若为联合体投 标，须为联合体牵头人人员）。 □园林绿化工程项目经理（项目负责人）资格： （职称级别）专业技术职称， （业绩要求） ，须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。3.3 各投标人均可就上 述 1个 (具体数量)标段投标 。 3.4 本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东为大企业、与大企业的负 责人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具 体标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的 通知》（工信部联企业〔2011〕300 号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除 技术复杂、存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在 3000万元以下的施工项目 (标 段) 应勾选此项。） 4. 招标文件的获取 网 4.1 凡有意参加投标者，请于 2026年08月22日开始登录：全国公共资源交易平台（四川省 · 广元市）（网 址： http://www.gyggzyjy.cn/）—“电子交易平台”，通过数字证书免费下载招标资料（招标文件、技术资料 等）。 务 4.2 招标人不提供招标文件获取的其他方式。 商 5.投标文件的递交 道 投标文件递交的截止时间（投标截止时间，下同）为 2026 年09月11日 09时00 分，投标人应在投 标截止时间前在线递交经投标人数字证书加密的数据电文形式投标文件。 6. 发布公告的媒介 管 本次招标公告在《全国公共资源交易平台（四川省）》和全国公共资源交易平台（四川省广元市）上发布。 7.行政监督部门 国 单位名称： 广元市朝天区住房和城乡建设局 联系电话：0839-8622102 中 8. 联系方式 招 标 人：广元市朝天区城市建设开发有限责任公司 地 址：广元市朝天区朝天镇潜溪路一段 邮 编：628012 联 系 人： 刘先生（异议联系人） 电 话： 18398751706 传 真： / 电子邮件： / 网 址： / 开户银行： / 账 号： / 招标代理机构：中科标禾工程项目管理有限公司 地 址： 成都市锦江区锦东路668号国嘉新视界14楼 邮 编： 610065 联 系 人： 吴老师 项目负责人： 王旭波 电 话： 028-86618391 传 真： / 网 电子邮件： / 网 址： / 务 开户银行： / 账 号： / 商 信息来源:https://www.chinapipe.net/project/d3077552.html 道 cqdingjiu 2026.08.24 12:31:54 管 国 中</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>配水主管网：193.71千米；泵站：1座；集成泵站：4座</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N46" t="n">
@@ -3652,14 +3684,14 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 改造, 配水主支管道, 更换配水主管网, 抗菌耐磨涂塑钢管, 泵站改造, 集成泵站, 蓄水池整治, 测控井</t>
+          <t>污水管网, 提升改造, 排水管网, 更新改造, 检查井, 市政公用工程</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>涪陵区珍溪镇农村供水保障能力提升工程(二期)招标计划表</t>
+          <t>苍溪县嘉陵江南北侧中心城区污水管网改造和延伸覆盖项目(一期)施工招标公告</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3684,53 +3716,57 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>广元市</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>苍溪县</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管主要建设有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。</t>
+          <t>新改建管道:DN300污水管道162m、DN500 污水管道1884m、DN600 污水管道112m、DN300 雨水管道466.50m、DN600 雨水管道609m、 DN800 雨水管商道 390m、 DN1000 雨水管道1029m。并对涉及破损路面及配套设施等进行恢复。</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>合同预估金额为2182.77万元</t>
+          <t>项目业主为苍溪县城市管网事务中心，建设资金来自争取上级财政资金和地方自筹（资金来源），项目出资比例为100%。</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>PE管、衬塑钢管、水泵、不锈钢水箱、减压阀、排污阀</t>
+          <t>DN300、DN500、DN600、DN800、DN1000 污水管道和雨水管道</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>涪陵区珍溪镇农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目名称 涪陵区珍溪镇农村供水保障能力提升工程（二期） 招标法人 或招标人 重庆水务环境控股集团渝东自来水有限公司 网 名称（盖 章） 项目批准 文件及文 涪陵发改〔2026〕477号 务 号 (一)本项目对珍溪镇23个村(社区)安装配水管网660km及配套附属设施，其中：1.De160~De40的PE管 主要建设 有232km；2.连接各村社的De32~De20的PE管有381km；3.219~32的衬塑钢管47km。(二)购置安装泵 内容 站14座(一用一备共计28台水泵)，其中新建泵商站10座、更换泵站4座及配套电力设施;新建不锈钢水 箱2座等。(三)购置安装(0~25kg)减压阀61个;排污阀(25kg）3个。 招标项目名 招标方 招标文件计 拟交易 合同预估金额 序号 招标内容 备注 称 式 划发布时间 场所 (万元) 道 (一)本项目对珍溪镇23个 村(社区)安装配水管网660km 及配套附属设施，其 中：1.De160~De40的PE管 管 有232km；2.连接各村社 涪陵区珍溪 重庆市 的De32~De20的PE管有381km； 招标项目 镇农村供水 涪陵区 3.219~32的衬塑钢 公开招 1 保障能力提 2026-09 公共资 2182.77 管47km。(二)购置安装泵 标 升工国程（二 源交易 站14座(一用一备共计28台水 期） 中心 泵)，其中新建泵站10座、更 换泵站4座及配套电力设施; 新建不锈钢水箱2座等。(三) 中 购置安装(0~25kg)减压阀61 个;排污阀(25kg）3个。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075275.html cqdingjiu 2026.08.21 10:06:57</t>
+          <t>苍溪县嘉陵江南北侧中心城区污水管网改造和延伸覆盖项目(一期)施工招标公告 1. 招标条件 1.1本招标项目苍溪县嘉陵江南北侧中心城区污水管网改造和延伸覆盖项目（一期）(项目名称)已由苍溪 县发展和改革局(项目审批、核准或备案机关名称)以苍发改投资[2025]135号（批文名称及编号）批准建设，项目 业主为苍溪县城市管网事务中心，建设资金来自争取上级财政资金和地方自筹（资金来源），项目出资比例 为100%，招标人为苍溪县城市管网事务中心。项目已具备招标条件，现对该项目的施工进行公开招标。 1.2本招标项目由苍溪县发展和改革局（核准机关名称）核准（招标事项核准文网号为苍发改投资[2025]135号）的 招标组织形式为委托招标（□自行招标 委托招标）。招标人选择的招标代理机构是四川伟瑞项目管理有限公 司。 2. 项目概况与招标范围 务 2.1建设地点：陵江镇、百利镇。 2.2建设内容及规模：新改建管道:DN300污水管道162m、DN500 污水管道1884m、DN600 污水管道112m、DN300 雨水管道466.50m、DN600 雨水管道609m、 DN800 雨水管商道 390m、 DN1000 雨水管道1029m。并对涉及破损路面 及配套设施等进行恢复。 2.3工期：300日历天。 道 2.4招标范围： 工程量清单及图纸所示全部内容。 2.5标段划分： 一个标段。 管 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 3.1本次招标要求投标人国须具备 3.1.1资质条件：具备独立法人资格，具备国家行政主管部门颁发的市政公用工程施工总承包三级及以上资质（须 具备有效的安全生产许可证）。 中 3.1.2业绩要求： □近年（ 年 月 日至投标截止时间，不少于3年）（多项选择：□已完成 □已完成或新承接或正在 施工）不少于 （1 至3个）个类似项目。类似项目是指: 。 无业绩要求。 3.1.3项目经理的资格要求： 项目经理（项目负责人）资格：市政公用工程(注册专业)贰级及以上（级别）建造师，具有省级及以上住房城 乡建设主管部门颁发的安全生产考核合格证（B证）， （业绩要求） ，须为本单位人员（若为联合 体投标，须为联合体牵头人人员）。 □园林绿化工程项目经理（项目负责人）资格： （职称级别）专业技术职称， （业绩 要求） ，须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： 。 3.3各投标人均可就上述 1个 (具体数量)标段投标 。 □ 3.4本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东为大企业、与大企业的负责 人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具体 标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的通 知》（工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除技术 复杂、存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在3000万元以下的施工项目(标段) 应勾 选此项。） 4. 招标文件的获取 4.1 凡有意参加投标者，请于2026年8月22日0时0分开始登录：全国公共资源交易平台（四川省·广元市） （网址：http://www.gyggzyjy.cn/）—“电子交易平台”，通过数字证书免费下载招标资料（招标文件、技术资料 等）。 4.2 招标人不提供招标文件获取的其他方式。 网 5. 投标文件的递交 投标文件递交的截止时间（投标截止时间，下同）为2026年9月18日09时30分，投标人应在投标截止时间前在线 务 递交经投标人数字证书加密的数据电文形式投标文件。 6. 发布公告的媒介 本次招标公告在《全国公共资源交易平台（四川省）》商和《全国公共资源交易平台（四川省.广元 市）》(公告发布的其它媒介名称）上发布。 7. 行政监督部门 道 行政监督部门:苍溪县住房和城乡建设局 联系电话0839-5222082 管 8. 联系方式 招 标 人：苍溪县城市国管网事务中心 地 址：苍溪县陵江镇嘉陵路西段72号 邮 编：/ 中 联 系 人：马先生（异议受理） 电 话：0839-2320019 传 真： / 电子邮件： / 网 址： / 开户银行： / 账 号： / 招标代理机构：四川伟瑞项目管理有限公司 地 址：四川省成都市金牛区金府路593号7栋12层9号 邮 编：610036 联 系 人：谢先生 电 话：028-62812735 传 真： / 电子邮件： / 网 址： / 开户银行： / 账 号： / 网 信息来源:https://www.chinapipe.net/project/d3077551.html 务 cqdingjiu 2026.08.24 12:31:54 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>配水管网：660km；的衬塑钢管：47km；泵站：4座；泵站：10座；换泵站：4座</t>
+          <t>排水和雨水排放</t>
         </is>
       </c>
       <c r="N47" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>涪陵区, 珍溪镇, 农村供水, 提升工程, 衬塑钢管, 水泵, 不锈钢水箱, 减压阀, 排污阀</t>
+          <t>苍溪县, 污水管网改造, 延伸覆盖, DN300, DN500, DN600, DN800, DN1000, 雨水管道, 污水管道</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>涪陵区蔺市街道农村供水保障能力提升工程(二期)招标计划表</t>
+          <t>广元市朝天区污水管网提升改造项目(五标段)施工招标公告</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3755,38 +3791,42 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>广元市</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>涪陵区</t>
+          <t>朝天区</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长105.307km（dn20-dn40PE管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建1座改造3座；新建测控井52座。</t>
+          <t>本项目管网部分为新建排水主管网长度约2.08km（雨水管网约0.88km，污水管网约1.2km），管径DN300～DN800；现状管道清淤疏通长度约为1.23km；配套建设检查井等附属构筑物以及路面恢复提升；道路部分为埋地排水管道施工路面破除与恢复，同时对设计范围内其他道路进行路面黑化提升，项目共涉及7条道路的路面改造，其中车行道改造面积约9188平方米，人行道改造约3295平方米。</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>合同预估金额：2652.89万元</t>
+          <t>项目估算总投资10498.09万元，资金来源为争取上级资金及地方政府配套资金。</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>净水设备、PE管、抗菌耐磨涂塑钢管</t>
+          <t>排水主管网、雨水管网、污水管网、检查井、路面恢复提升材料</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>涪陵区蔺市街道农村供水保障能力提升工程(二期)招标计划表 重庆市工程建设项目招标计划表 项目 涪陵区蔺市街道农村供水保障能力提升工程（二期） 名称 招标 法人 网 或招 标人 重庆水务环境控股集团渝东自来水有限公司 名称 （盖 章） 务 项目 批准 文件 涪陵发改〔2026〕475号 及文 号 商 主要 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 105.307km（dn20-dn40PE 建设 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座；新建测控井 52座。 内容 拟 招 招标文 合同预 招标 交 序 道 标 件计划 估金 备 项目 招标内容 易 号 方 发布时 额(万 注 名称 场 式 间 元) 所 重 庆 涪陵 管 市 区蔺 涪 招标 市街 陵 项目 道农 公 区 村供 八方碑水厂扩容购置3000m/d净水设备1套；堡子水厂购置3000m/d净水设备1套；新建、更换管网总长 开 公 1 水保 105.307km（dn20-dn40PE 管、DN32-DN300抗菌耐磨涂塑钢管）及配套附属设施；泵站新建 1座改造3座； 2026-09 2652.89 国 招 共 障能 新建测控井 52座。 标 资 力提 源 升工程 交 （二 易 期） 中 中 心 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3075274.html cqdingjiu 2026.08.21 10:06:57</t>
+          <t>广元市朝天区污水管网提升改造项目(五标段)施工招标公告 1. 招标条件 1.1本招标项目广元市朝天区污水管网提升改造项目(项目名称)已由 广元市朝天区发展和改革局(项目审批、核 准或备案机关名称)以 广朝发改项目[2024]108号 （批文名称及编号）批准建设，项目业主为 广元市朝天区 城市建设开发有限责任公司 ，建设资金来自争取上级资金及地方政府配套资金（资金来源），项目出资比例 为 100% ，招标人为广元市朝天区城市建设开发有限责任公司 。项目已具备招标条件，现对该项目的施 工进行公开招标。 网 1.2本招标项目由 广元市朝天区发展和改革局 （核准机关名称）核准（招标事项核准文号为 广朝发改项 目[2024]108号 ）的招标组织形式为 委托招标（□自行招标 委托招标）。招标人选择的招标代理机构 是 中科标禾工程项目管理有限公司 。 务 2. 项目概况与招标范围 2.1 建设地点：朝天区水磨沟镇 。 2.2 建设规模：本项目管网部分为新建排水主管网长度约商为2.08km （雨水管网约0.88km，污水管网约1.2km），管 径DN300～DN800；现状管道清淤疏通长度约为1.23km；配套建设检查井等附属构筑物以及路面恢复提升；道路 部分为埋地排水管道施工路面破除与恢复，同时对设计范围内其他道路进行路面黑化提升，项目共涉及7条道路 的路面改造，其中车行道改造面积约9188平方米，人行道改造约3295平方米。 道 2.3 计划投资及资金来源：项目估算总投资 10498.09万元。资金来源为争取上级资金及地方政府配套资金 。 2.4 计划工期： 240日历天 。 管 2.5 招标范围：本项目施工图纸及清单范围内所包含的全部工作内容的施工。 2.6 标段划分：施工1个标段。 （说明本次招标项目的国建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 中 3.1 本次招标要求投标人须具备： 3.1.1 资质条件：具备独立企业法人资格，具备建设行政主管部门颁发的 市政公用工程施工总承包三级及以上资质（须具备有效的安全生产许可证）。3.1.2 业绩要求： □近年（ 年 月 日至投标截止时间，不少于 3 年）（多项选择： □已完成□已完成或 新承接或正在施工）不少于 （ 1 至 3 个）个类似项目。类似项目是 指: 。 无业绩要求。 3.1.3 项目经理的资格要求： 项目经理（项目负责人）资格： 市政公用工程(注册专业)二级及以上(级别)建造师，具有省级及以上住房城 乡建设主管部门颁发的安全生产考核合格证（B 证），/ （业绩要求） ，须为本单位人员（若为联合体投 标，须为联合体牵头人人员）。 □园林绿化工程项目经理（项目负责人）资格： （职称级别）专业技术职称， （业绩要求） ，须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。3.3 各投标人均可就上 述 1个 (具体数量)标段投标 。 3.4 本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东为大企业、与大企业的负 责人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具 体标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的 通知》（工信部联企业〔2011〕300 号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除 技术复杂、存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在 3000万元以下的施工项目 (标 段) 应勾选此项。） 4. 招标文件的获取 网 4.1 凡有意参加投标者，请于 2026年08月22日开始登录：全国公共资源交易平台（四川省 · 广元市）（网 址： http://www.gyggzyjy.cn/）—“电子交易平台”，通过数字证书免费下载招标资料（招标文件、技术资料 等）。 务 4.2 招标人不提供招标文件获取的其他方式。 1. 投标文件的递交 商 投标文件递交的截止时间（投标截止时间，下同）为 2026年09月11日 09时00 分，投标人应在投标 截止时间前在线递交经投标人数字证书加密的数据电文形式投标文件。 6. 发布公告的媒介 道 本次招标公告在《全国公共资源交易平台（四川省）》和全国公共资源交易平台（四川省广元市）上发 布。 管 7.行政监督部门 单位名称： 广元市朝天区住房和城乡建设局 联系电话：0839国-8622102 8. 联系方式 中 招 标 人：广元市朝天区城市建设开发有限责任公司 地 址：广元市朝天区朝天镇潜溪路一段 邮 编：628012 联 系 人： 刘先生（异议联系人） 电 话： 18398751706 传 真： / 电子邮件： / 网 址： / 开户银行： / 账 号： / 招标代理机构：中科标禾工程项目管理有限公司 地 址： 成都市锦江区锦东路668号国嘉新视界14楼 邮 编： 610065 联 系 人： 吴老师 项目负责人： 王旭波 电 话： 028-86618391 传 真： / 电子邮件： / 网 网 址： / 开户银行： / 务 账 号： / 信息来源:https://www.chinapipe.net/project/d3077550.html 商 cqdingjiu 2026.08.24 12:31:54 道 管 国 中</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>管网：105.307km；泵站：1座</t>
+          <t>排水主管网 Φ300~Φ800mm 约2.08km；雨水管网 Φ300~Φ800mm 约0.88km；污水管网 Φ300~Φ800mm 约1.2km；现状管道清淤疏通长度约1.23km；配套建设检查井等附属构筑物；路面恢复提升材料，车行道改造面积约9188平方米，人行道改造约3295平方米。</t>
         </is>
       </c>
       <c r="N48" t="n">
@@ -3794,14 +3834,14 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>排水管网, 提升改造, 市政工程, 污水处理, 路面修复</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目项目公告</t>
+          <t>四川省犍为第一中学扩建项目施工招标计划</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3811,7 +3851,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>房建</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3826,29 +3866,37 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>乐山市</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>犍为县</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1，该管道为自流管道，位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水厂的正常收水及运行，需对该段管道进行改造。</t>
+          <t>新建教学综合楼14500㎡、学生宿舍8500㎡、食堂3000㎡，以及附属用房、排水管网等配套基础设施。</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>项目资金来自企业自筹</t>
+          <t>估算总投资100000000.00元</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>DN600混凝土管，检查井</t>
+          <t>房屋建筑</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目项目公告 重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称）比选公告 1.比选条件 本比选项目重庆市排水有限公司鱼洞污水处理厂2026年专件厂线管网改造项目（项目名称），比选人为重庆市排 网 水有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。中标后合同与重庆市豪洋水务 建设管理有限公司签订。现对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 2.项目概况与比选范围 务 2.1 建设地点：重庆市巴南区 2.2 项目概况：本项目涉及管道为鱼洞污水处理厂专件厂线管网，管道编号为WD4-WD8+1,该管道为自流管道， 位于鱼轻桥至河嘴倒虹井段，主要用于收集输送鱼洞大江商至华熙片区的生活污水。该段管道管径为DN600，管道 为混凝土管，主要采用架空明敷的方式沿河敷设。该管道自建成投运以来已有20余年，管道及污水井老化严重现 象十分明显，容易出现破损从而造成污水溢流，造成环保风险。为规避环保风险且保障该段管道以及鱼洞污水 厂的正常收水及运行，需对该段管道进行改造。 道 2.3 比选范围：拆除现状管道为DN600混凝土管，同时需拆除并新建9座检查井。 2.4 工期要求：30日历天，以甲方通知进场时间为准。 管 2.5缺陷责任期要求：24个月 3.投标人资格要求 国 3.1 本次比选要求投标人须具备以下条件： 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质。 中 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 项内容。 3.2 本次比选接受不联合体投标。 4.比选文件的获取 4.1 投标人于2026年8月 18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子 版，以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都 视为投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的 一切后果由投标人自行负责。各投标单位应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行供应商注册，填写相关信息，审批过后成为 平台供应商。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价、递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，将被否决投标。 4.4 比选文件每份售价800元，售后不退。投标单位在递交纸质投标文件时扫描支付，否则比选人拒绝接收其投标 文件。 5.投标文件的递交 5.1 电子投标文件递交时间：2026年8月24日14时30分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年8月24日14时00分至14时30分（北京时间），地点：重庆水务招标采购中心 （重庆市两江新区嘉华路36号重庆水务大厦5楼）。 5.3 投标截止时间：2026年 8月24日14时30分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆市排水有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市渝中区长江滨江路126号 地 址：重庆市两江新区嘉华路36号重庆水务大厦 道 联 系 人： 黄老师 联 系 人： 黄晓华 电 话： 023-67767416 电 话： 18523396416 管 重庆水务电子商务平台咨询电话：023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3075272.html 国 cqdingjiu 2026.08.21 10:06:57 中</t>
+          <t>四川省犍为第一中学扩建项目施工招标计划 犍为县发展和改革局关于《四川省犍 为第一中学扩建项目可行性研究报告 项目批准文件及文号 招标项目名称 四川省犍为第一中学扩建项目施工 （代项目建议书）》的批复(犍发改项 （如有） 目审〔2025〕248号)(犍发改项目审 〔2025〕248号) 招标人 四川省犍为第一中学 联系人及联系方式 杨先生:0833-4266336 估算总投资 100000000.00 项目分类 房屋建网筑工程 （元） 项目占地约42.7亩。新建教学综合楼14500㎡、学生宿舍8500㎡、食堂3000㎡，以及附属用房、排 招标项目概况 水管网等配套基础设施。 务 序号 招标内容 投标人主要资格条件要求 预计招标时间 拟招标内容 1 施工 / 2026-09-21 00:00:00 备注：提前发布的招标计划内容仅供各方主体提前获知项目基本信息和拟招标内容，招标项目的实际信息以招 标人最终发布的招标公告和招标文件为准。 商 信息来源:https://www.chinapipe.net/project/d3077548.html cqdingjiu 2026.08.24 12:31:55 道 管 国 中</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3857,18 +3905,18 @@
         </is>
       </c>
       <c r="N49" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>重庆, 排水公司, 污水处理厂, 管网改造, DN600混凝土管, 检查井</t>
+          <t>扩建项目, 施工招标</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>重庆市潼南城区老旧供水管网改造工程招标计划</t>
+          <t>四川卓勤新材料科技有限公司基膜涂覆一体化项目(二期三标段)预应力高强混凝土管桩采购任务</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3878,7 +3926,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3893,53 +3941,57 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>潼南区</t>
+          <t>邛崃市</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>改建潼南城区输水主管网约39.63km及配套相应阀门阀件等，对城区供水管网上商老旧阀门阀件、设施设备进行更换，合理增设部分计量及压力监控、水质监控等。</t>
+          <t>预应力高强混凝土管桩</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>合同预估金额：918.00万元</t>
+          <t>自筹资金</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>城区配套阀门阀件改造工程</t>
+          <t>预应力高强混凝土管桩</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>重庆市潼南城区老旧供水管网改造工程招标计划 重庆市工程建设项目招标计划表 项目名称 重庆市潼南城区老旧供水管网改造工程 招标法人或招 标人名称（盖 重庆市潼南自来水有限公司 网 章） 项目批准文件 及文号 务 主要建设内容 改建潼南城区输水主管网约39.63km及配套相应阀门阀件等 招标方 招标文件计 拟交易场 合同预估 序号 招标项目名称 招标内容 备注 式 划发布时间 所 金额(万元) 对城区供水管网上商 重庆市潼南城 老旧阀门阀件、设 区老旧供水管 重庆市潼 招标项目 施设备进行更换， 网改造工程 公开招 南区公共 1 保障供水管网稳定 2026-09 918.00 （城区配套阀 标 资源交易 运行合道理增设部分 门阀件改造工 中心 计量及压力监控、 程） 水质监控等。 备注 本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 管 信息来源:https://www.chinapipe.net/project/d3075266.html cqdingjiu 2026.08.21 10:06:58 国 中</t>
+          <t>四川卓勤新材料科技有限公司基膜涂覆一体化项目(二期三标段)预应力高强混凝土管桩采购任务 一、项目基本情况： 1. 采购项目名称： 四川卓勤新材料科技有限公司基膜涂覆一体化项目（二期三标段） 2. 采购人 ： 中国机械工业建设集团有限公司 四川分公司 3. 采购内容 ： 预应力高强混凝土管桩 （详见响应文件材料清单） 网 4. 采购方式 ： 公开竞争性谈判 。 5. 资金来源 ： 自筹 资金 务 6.项目地点： 四川省成都市邛崃市天府新区半导体材料产业功能区崃岭大道 888号 。 7.货物质量标准或主要技术性能指标：质量达到国家及行业现行相关法律法规规定的生产、制造、验收规范合格 标准，且符合后续合同设计图纸要求。 商 二、分供商资格要求 1.本项目的特定资格要求： 道 （ 1）具有独立承担民事责任能力的法人、其他组织，并出具合法有效的营业执照或事业单位法人证书等国家 规定的相关证明；； （ 2 ）供应商应授权合法的人员参加谈判全过程，法定代表人直接参加的须提交其身份证原件及法定代表人 管 证明书，法定代表人授权代表参加谈判的，须出具法定代表人授权书及被授权人身份证原件； （ 3 ）财务状况报告：提供经审计的财务报告（至少包含资产负债表和利润表，成立时间至提交响应文件截 止时间不足一年的可提供成立后任意时段的资产负债表）或报价前六个月内其基本账户银行出具的资信证明 （附开户许可证或基本国账户信息）； （ 4 ）不得为 “信用中国”网站（www.creditchina.gov.cn）中列入“失信被执行人”和“重大税收违法案 件”当事人名单的供应商，不得为中国政府采购（www.ccgp.gov.cn）政府采购“严重违法失信行为记录名单”中 被财政部门禁止参加政府采购活动的供应商； 中 （ 5 ）无重大违法记录声明：供应商须出具参加采购活动前三年内，在经营活动中没有重大违法记录声明； 注： I.不同性质的法人或其他组织可按照国家法律规定提供合法资质；特殊行业 供应商 的分支机构 参与 谈判的 ，还须出具其主管单位或总公司为其参与本项目 报价 及履约行为承担民事责任的承诺书；特殊行 业 供应商 的分支机构 参与谈判 的，财务状况、税收缴纳、社会保障资金缴纳等由主管单位或总公司代缴 （代管）的，提供其主管单位或总公司相应证明材料及情况说明。 Ⅱ. 供应商 负责人为同一人或者存在直接控股、管理关系的不同供应商，不得同时参加本项目采购活动，否 则按 无效 处理。 Ⅲ.根据《关于在政府采购活动中查询及使用信用记录有关问题的通知》（财库〔2016〕125号）的规定，对列入 失信被执行人、重大税收违法案件当事人 名单、政府采购严重违法失信行为记录名单的供应商，拒绝参与本 项目采购活动； （ 6 ）本次采购不接受联合体。 三、采购文件的获取方式 时间： 2026 年 8 月 22 日 12:00 至 2026 年 8 月 25 日 12:00 地点 ：中机建设电子采购平台， http://eps.sinoconst.com.cn/ 方式：网上获取 四、响应文件的递交 截止时间： 2026年8 月 27 日 17 时 00 分 00 秒 ， 供应商 应在截止时间前将编制完成的 响应 文件进行盖章扫描后，上传至 “ 中机建设电子采购平台 ”的提交 响应 报价文件模块，逾期未 完成上传的，系统将拒绝接收 响应 文件并自动对其关闭。 五、谈判时间和地点 网 递交响应文件的分供商应委派代表准时参加谈判活动，谈判开始时间 2026年8 月 28 日 10 时 00 分 00 秒 。谈判方式是通过腾讯视频会议系统。 务 六、发布谈判公告的媒介 本次采购公告在中机建设电子采购平台（ eps.sinoconst.com.cn）发布 七、对本次采购提出询问，请按以下方式联系。 商 采购人信息：中国机械工业建设集团有限公司 四川分公司 地 址：四川省成都市天府新区华府大道 1段蓝道润置地2 707 联 系 人： 丁保平 电话： 13213128433 八、监督 管 本项目的 谈判采购 活动及其相关当事人应当接受有管辖权的 公司合规 监督部门依法实施的监督（公司 纪检部门）。 监督 人 ：邹 忠 国 联系电话： 13778280342 邮 箱： legal@sinoconst.com.cn 中 信息来源:https://www.chinapipe.net/project/d3077502.html cqdingjiu 2026.08.24 12:31:55</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>输水主管网：39.63km</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N50" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>四川, 预应力高强混凝土管桩, 公开竞争性谈判, 自筹资金</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>关于为【重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购】公开选取【工程设计】机构的公告</t>
+          <t>宜宾高新区高场片区老旧小区改造项目等两个工程管网探测及测绘(第二次)询价邀请函公告</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3949,7 +4001,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>其他/未识别</t>
+          <t>房建</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3964,53 +4016,57 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>宜宾市</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>开州区</t>
+          <t>宜宾市</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>该项目涉及硬化生产便道、建设防旱池和蓄水池、建造育苗大棚和小棚、安装水源处理和水肥一体化设施、新建设备管理房以及完善蔬菜基地配套设施等内容。</t>
+          <t>本项目包括宜宾高新区高场片区老旧小区改造项目和宜宾高新区高场片区城中村配套基础设施项目的管网探测及测绘工作。</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>工程总投资335万元。</t>
+          <t>宜宾高新区高场片区老旧小区改造项目建安费用约8349.39万元，宜宾高新区高场片区城中村配套基础设施项目建安费用约12000万元。</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>工程设计服务</t>
+          <t>管网探测设备及服务，建筑单体测绘设备及服务，原始地形地貌测绘设备及服务</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>关于为【重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购】公开选取【工程设计】 机构的公告 我单位在重庆市网上中介超市公开选取工程设计中介服务机构，现将相关事项公告如下： 该项目为直接选取项目，由采购人从报名的中介服务机构中直接选定一家中介服务机构进行项目服务。 项目 重庆市开州区2026年河堰镇清泉社区高山蔬菜基地配套设施项目设计服务采购 名称 网 采购 重庆市开州区河堰镇人民政府 人 投资 审批 否 务 项目 是否 破产 商 业务 否 服务 项目 采购 道 所需 中介 其他 服务 事项 管 所需 服务 工程设计 类型 项目实施地点为国河堰镇清泉社区，项目建设内容为：硬化2米宽生产便道5.5千米，100方防旱池1口，50方 服务 蓄水池1口，标准自动化育苗大棚1个，蔬菜小棚20个，水源处理设施1套，水肥一体化配套设施1套，新 内容 建50平方米设备管理房，完善蔬菜基地配套设施等。工程总投资335万元。选取此项目设计单位（含预算 编制服务）。 中 中介 机构 资质（资格）要求 要求 资质 （资 1、报名单位提供有效的营业执照，资质证书（资质丙级或丙级以上），具备从事项目设计服务工作； 2、 格） 具有独立承担民事责任的能力； 3、具有良好的商业信誉和健全的财务会计制度； 4、具有履行合同所必 要求 需的专业技术能力； 5、有依法缴纳税收和社会保障资金的良好记录。 说明 其他 要求 无 说明 服务 时限 无要求，按照合同双方自行约定 说明 服务 3.1%费率 金额 金额 按文件要求执行 说明 选取 直接选取 方式 需规 避机 构 规避 原因 选取 2026-08-20 16:00:00 （选取时间到达后不接受报名，建议中介机构至少在选取开始半小时前完成报名。） 时间 采购 人业 网 务咨 重庆市开州区河堰镇人民政府（18716685679） 询电 话 采购 务 需求 26清泉社区项目设计服务采购说明.pdf 书下 载 商 2026-08-18 信息来源:https://www.chinapipe.net/project/d3075198.html 道 cqdingjiu 2026.08.21 10:06:58 管 国 中</t>
+          <t>宜宾高新区高场片区老旧小区改造项目等两个工程管网探测及测绘(第二次)询价邀请函公告 询价邀请函 各报价单位： 根据公司安排，将宜宾高新区高场片区老旧小区改造项目等两个工程管网探测及测绘（第二次）进行市场询价， 现诚邀贵公司就根据项目情况参与报价。 一、 项目名称 网 宜宾高新区高场片区老旧小区改造项目等两个工程管网探测及测绘（第二次） 二、项目概况 务 （一）项目地点：宜宾市高新区 （二）项目规模： 商 1.宜宾高新区高场片区老旧小区改造项目（子工程一）：本项目涉及高场片区11个老旧小区，房屋58栋，1956户 居民。改造小区燃气管道17160m，给排水管道18935m，电力和通信线路13320m，改造停车位685个；新增充电 桩137个，小区消防设施58套，户内燃气安全设施1956套，分类垃圾回收站点10个；改造闲置社区用房为日间照 料中心4430m、便民中心5420m，改造小区内道道路10192m及配套基础设施；建安费用约8349.39万元。 2.宜宾高新区高场片区城中村配套基础设施项目（一标段）（子工程二）：本项目实施范围约460亩，涉及户 数690户，共计2277人。具体建设内容包括新建公共配套用房总建筑面积21000m，其中养老托幼等服务设 施15000m、其他公服用房6000m；新建公共停车位1600个及配置400个充电桩；新改建城中村配套道路 管 约4.5km及其他基础设施建设。本标段建设内容包含对高场镇碧水街、通江街、河边街、中学街等进行道路整治、 电力通讯线路下地、人行道改造、街面外立面整治、街道绿化及亮化提升等；新建公共配套用房、公共停车位、 口袋公园等配套公共基础设施；建安费用约12000万元。 （三）工作内容： 国 1.管线探测：收集已有管线资料，现场踏勘；对井盖等明设管线实地调查，采用物探设备探明各类地下隐蔽管线 的规格参数、位置、埋深及走向；实测管线点坐标高程；整理核查数据，编制管线图纸、数据库及技术报告， 并开展相关质量检查验收工作。 中 2.建筑单体测绘：实测建筑平面轮廓、层高、标高、外立面、附属设施及角点坐标，核查建筑现状；绘制平 立剖面图纸，核算建筑面积、编制测绘图纸、计算书及正式测绘报告等相关内容。 3.原始地形地貌测绘：实测场地内建筑物、道路、水系、植被等地物要素及地面高程点，绘制带等高线原始地形 图纸，行程测绘成果。 三、报价人资格要求 （一）具有中国境内注册的独立法人资格。 （二）资质要求：具备国家建设行政主管部门颁发的测绘相关资质。 四、其他说明 （一）本次询价仅为市场调查行为，不作为定标依据。 （二）本次工期为30日历天。 五、递交资料内容 详见附件询价表，营业执照及资质证书。 六、其他要求 （一）报价文件递交截止日期为2026年8月24日17:00 （二）报价方式：网上递交。报价文件采用PDF文件并加盖鲜章，通过宜宾企业阳光采购服务平台线上递交。 （联系人：谢先生 ，电话：0831-8755160） 宜宾市高新投资集团有限公司 网 2026年8月21日 信息来源:https://www.chinapipe.net/project/d3077494.html 务 cqdingjiu 2026.08.24 12:31:55 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>宜宾高新区高场片区老旧小区改造项目：改造小区燃气管道17160m，给排水管道18935m，电力和通信线路13320m，改造停车位685个；新增充电桩137个，小区消防设施58套，户内燃气安全设施1956套，分类垃圾回收站点10个；改造闲置社区用房为日间照料中心4430m、便民中心5420m，改造小区内道路10192m及配套基础设施。宜宾高新区高场片区城中村配套基础设施项目：新建公共配套用房总建筑面积21000m，其中养老托幼等服务设施15000m、其他公服用房6000m；新建公共停车位1600个及配置400个充电桩；新改建城中村配套道路约4.5km及其他基础设施建设。</t>
         </is>
       </c>
       <c r="N51" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>宜宾, 高新区, 老旧小区改造, 管网探测, 测绘</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目招标公告</t>
+          <t>中煤广元煤炭储备项目设备安装工程钢管及型钢采购询价通知</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4020,7 +4076,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>房建</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4035,53 +4091,57 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>广元市</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>开州区</t>
+          <t>广元市</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米，务周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。</t>
+          <t>钢管及型钢采购</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>项目总投资金额：500万元，本次招标项目合同估算金额：446.278921万元</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>柑橘基地改造提升项目</t>
+          <t>热浸锌镀锌无缝钢管,热浸锌镀锌钢管,热浸锌扁铁,热浸锌角钢,热浸锌槽钢,水煤气管热浸锌,无缝钢管</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目招标公告 1.招标条件 本招标项目重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目已由重庆市开州区发展和改革委员会以开州 发改审〔2026〕357号批准建设，项目业主为重庆市开州区长沙镇人民政府，建设资金来自开州区2026年中央和 市级提前批财政衔接推进乡村振兴补助资金，项目出资比例为 100% ，招标人为重庆市开州区长沙镇人民 政府。项目已具备招标条件，现对该项目的施工进行公开招标，评标办法采用综合评估法。 2.项目概况与招标范围 网 2.1 建设地点：开州区长沙镇桔香村 2.2 项目概况与建设规模：1.建设果园水肥一体化系统1套，对示范柑桔果园建设水肥一体智能化系统;2.果园运输 线4000米(含轨道主机、叉车、周转箱、三轮车等配套设施设备);3.建设排灌站一处;4.建设1.8米宽生产便道2000米， 务 周转场300平方米;5.配备载重无人机1台、小型挖机1台、电子控制屏1个;6.建设智慧平台与监测系统软硬件系统等。 2.3 本项目工程总投资金额： 500万元 本次招标项目合同估算金额： 446.278921万元 商 2.4 招标范围：招标人发布的由重庆中煜华资工程技术有限公司设计的《重庆市开州区2026年长沙镇桔香村柑橘 基地改造提升项目》施工图及图纸说明、招标文件(含补遗)及工程量清单、答疑资料、澄清资料范围内所涉及的 工作内容，具体以招标人发布的工程量清单及道施工图为准。 2.5 工期要求： 150日历天 缺陷责任期要求： 12个月 管 2.6 标段划分（如有）： / 2.7 其他： / 国 3.政府采购工程 3.1 是否属于政府采购工程：是 中 3.2 是否专门面向中小企业预留：否，按照《政府采购促进中小企业发展管理办法》第六条第(三)“按照本办法 规定预留采购份额 无法确保充分供应、充分竞争，或者存在可能影响政府采购目标实现的情形”的规定，故本 项目不专门面向中小企业预留。 4.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 4.1.1 本次招标要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的建筑工程施工总承包叁级及以 上资质或市政公用工程施工总承包叁级及以上资质或水利水电工程施工总承包叁级及以上资质； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 5.招标文件的获取 5.1本招标项目采用全流程电子招投标，投标人在投标前可在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）下载招 标文件、工程量清单、电子图纸等资料。参与投标的投标人需在 重庆市公共资源交易监督网 （http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）完成市 场主体信息登记以及CA数字证书办理，办理方式请参见 重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、 重庆市公共资源交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）导航栏“主体信息”页面中“市场主 体信息登记”、“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完 成全流程电子招投标的，责任自负。 5.2投标人可在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告 发布至2026-08-21 17:00:00前。 5.3招标人应于2026-08-25 23:59:59前在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源 交易网（开州区）（https://www.cqggzy.com/kaizhouweb/）发布澄清。 6.投标文件递交的内容 网 6.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-21 09:30，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 6.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 务 7.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网（http://ggzyjyjgj.cq.gov.cn ）、重庆市公共资源交易网（开州区） （https://www.cqggzy.com/kaizhouweb/）发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交 易监督网上发布。] 商 8.联系方式 招 标 人: 重庆市开州区长沙镇人民政府 代理机构: 重庆毅仁建设项目管理有限公司 重庆市开州区文峰街道天鹅湖社区富厚街158号附10 地 址: 重庆市开州区长沙镇山花街1号 地 址: 道号 邮 编: 邮 编: 项目负责人: 丁敬余 项目负责人: 谭毅 电 话: 15826368887 管电 话: 13452653126 传 真: 传 真: 电子邮箱: 1415705480@qq.com 电子邮箱: 开户银行: 国 开户银行: 账 号: 账 号: 监督部门:中重庆市开州区公共资源交易管理局 电 话: 023-52218977 2026年08月17日 重庆市开州区2026年长沙镇桔香村柑橘基地改造提升项目 户名 开户行 投标保证金账号 重庆市开州区公共资源交易中心 重庆农村商业银行股份有限公司开州支行 3401010120010012772000200 中国农业银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 314401010400104500000006031 业部 中国工商银行股份有限公司重庆开州支行营 重庆市开州区公共资源交易中心 9558853100005824176 业部 重庆市开州区公共资源交易中心 重庆银行股份有限公司开州支行 680101040007547-100984 重庆市开州区公共资源交易中心 中国银行股份有限公司重庆开州支行 108865555576VA00149 信息来源:https://www.chinapipe.net/project/d3075199.html cqdingjiu 2026.08.21 10:06:58</t>
+          <t>中煤广元煤炭储备项目设备安装工程钢管及型钢采购询价通知 中煤广元煤炭储备项目设备安装工程钢管及型钢采购 询价通知 中煤第九十二工程有限公司根据采购管理办法，现对“中煤广元煤炭储备项目设备安装工程”所需钢管及型钢 组织公开采购，现邀请符合资质要求的供应商报名参与。 一、采购范围 网 序号 物资名称 规格型号 单位 数量 备注 务 1 热浸锌镀锌无缝钢管 D219X6 米 3600 20# 2 热浸锌镀锌无缝钢管 D159X6 米 200 20# 3 热浸锌镀锌无缝钢管 D133X4 米 100 20#商 4 热浸锌镀锌无缝钢管 D108X4 米 200 20# 5 热浸锌镀锌无缝钢管 D89X4 米 60 20# 6 热浸锌镀锌无缝钢管 D76X3.5 米 道42 20# 7 热浸锌镀锌无缝钢管 D57X3.5 米 120 20# 8 热浸锌镀锌无缝钢管 D45X3 米 18 20# 9 热浸锌镀锌无缝钢管 D38X管3 米 90 20# 10 热浸锌镀锌无缝钢管 D32X3 米 400 20# 11 热浸锌镀锌钢管 DN100 米 900 Q235B 12 热浸锌镀锌钢管国DN65 米 300 Q235B 13 热浸锌镀锌钢管 DN50 米 1000 Q235B 14 热浸锌扁铁 80*8 m 1438 Q235B 15 热浸中锌扁铁 40*6 m 6675 Q235B 16 热浸锌角钢 50*50*5 m 2672 Q235B 17 热浸锌角钢 75*5 m 170 Q235B 18 热浸锌槽钢 10# m 790 Q235B 19 水煤气管热浸锌 DN25 m 1133 Q235B 20 水煤气管热浸锌 DN40 m 87 Q235B 21 水煤气管热浸锌 DN50 m 1083 Q235B 22 水煤气管热浸锌 DN100 m 130 Q235B 23 无缝钢管 D159*6 m 100 20# 1．项目名称：中煤广元煤炭储备项目设备安装工程 2．询价书编码：XJ20260805003 3．采购方式：公开询比 二、供应商资格要求 （一）具备纳税人资格的法人企业； （二）具备生产或经营资质，完成标的物供货能力的生产商或经销商； （三）企业经营、资信状况良好，无不良经营业绩，没有处于被责令停业、财产被接管、冻结、破产状态； （四）未列入中煤集团范围内供应商停用名单； （五）不属于被国家相关部门认定有严重失信行为且处于失信处置期内的供应商； （六）本次采购不接受联合体参与，法定代表人为同一人或者存在控股、管理关系的不同单位，不得同时参加 报价。 网 三、供应商报名、报价及采购文件获取 （一）供应商登录中煤供应链平台（http://ego.chinacoal.com），已注册用户的供应商直接登录通过系统网上报名 报价；未注册的供应商登录系统后先按要求填报企业相关资料，进行网上注册，待我公司进行准入评审后，按 务 照注册申请的账户登录系统网上报名报价。 （二）报名成功的供应商登陆中煤供应链平台下载采购文件。 （三）根据报价揭示情况进行资格后审 商 四、报价揭示时间、地点 （一）报价文件递交截止时间： 2026年8月25道日下午15: 00时(北京时间)。迟到的采购文件将被拒绝。 （二）报价揭示时间：2026年8月25日下午15: 00时(北京时间)。 （三）报价揭示地点：线上报价揭示 管 五、联系方式 采购单位：中煤第九十二工程有限公司 国 地址：河北邯郸市丛台路56号 采购联系人：王鑫：0310-7206473 中 现场联系人：张海鹏：13451436662 2026年8月21日 信息来源:https://www.chinapipe.net/project/d3077488.html cqdingjiu 2026.08.24 12:31:56</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>D219X6 米 3600; D159X6 米 200; D133X4 米 100; D108X4 米 200; D89X4 米 60; D76X3.5 米 120; D57X3.5 米 120; D45X3 米 18; D38X管3 米 90; D32X3 米 400; DN100 米 900; DN65 米 300; DN50 米 1000; 80*8 m 1438; 40*6 m 6675; 50*50*5 m 2672; 75*5 m 170; 10# m 790; DN25 m 1133; DN40 m 87; DN50 m 1083; DN100 m 130; D159*6 m 100</t>
         </is>
       </c>
       <c r="N52" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>重庆, 柑橘基地改造, 水肥一体化系统, 运输线, 排灌站, 生产便道, 无人机, 小型挖机, 智慧平台</t>
+          <t>重庆, 四川, 近三天, 管材招标, 商机</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程答疑及补遗(一)</t>
+          <t>四川省华蓥市重点采煤沉陷区华蓥市高兴镇城镇危旧房改造项目(三期)施工一标段招标公告</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4106,33 +4166,37 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>广安市</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>万盛区</t>
+          <t>华蓥市</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程答疑及补遗。</t>
+          <t>改造城镇危旧房约4.5万平方米，户数共220户，3栋共9个单元。配套小区内道路、供水、供电、供气主管网、消防、路灯等基础设施。新建道四通路与兴政路连接道路64米，铺设安置房一期商业街人行道5766平方米，配套完善排水、路灯、绿化等附属设施。</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>项目业主为华蓥市交通投资开发有限责任公司，建设资金来自上级补助和业主自筹（资金来源），项目出资比例为100%。</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>供水管网</t>
+          <t>市政公用工程施工</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程答疑及补遗(一) 万盛城区老旧供水管网更新改造工程 答疑及补遗（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程答疑及补遗（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。? 问题2：本项目是否采用异地评标方式？ 答：是 。 商 问题3：本项目是否有业主代表，如有，请明确业主代表数量。 答：是，本项目评标委员会共7人，其中在重道庆市综合评标专家库随机抽取5人，招标人代表2人 。 问题4：投标函中的缺陷责任期可以填“达到招标文件的要求”吗？ 答：可以。 管 问题5：污水处理厂提标改造及附属管道施工业绩满足吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 国 问题6：投标文件格式中下划线上、空格处、表格中无需要填写或无法填写内容的，是填“/”或“无”还是可以 不填(空白)，对此有无要求？ 答：无要求。? 中 问题7：我公司业绩为epc业绩，我公司与设计单位组成联合体承接，竣工验收报告中施工单位盖章由我公司盖章， 请问需要提供联合体协议书吗？ 。 答： 根据招标文件第二章“投标人须知前附表”1.4.1 第3条业绩要求中：“注：（2）投标人提供的业绩为联 合体业绩的，其在该业绩中的工作分工应与本项目承担的工作一致。”要求，故需要提供联合体协议书。 问题8：投标函附录中，工期、分包和工程质量要求对应的约定内容，可以统一填写“达到招标文件要求”吗？ 答：填写“达到招标文件的要求”或按照招标文件相关条款填写具体内容均可 。 问题9：招标人提供的工程量清单单项最高限价中金额为零的，清单综合单价报价可以为0吗？ 答：投标人的工程量清单单项报价不得为零报价(招标人提供的工程量清单单项最高限价中金额为零的除外)或者 负数报价，否则由评标委员会作否决投标处理。 问题10：招标人应当在法定时间内确定中标人。招标人或者招标投标交易场所运行服务机构应当在中标通知书发 出后 5 日内，向除中标人以外的其他投标人退还纸质投标保函正本，并书面通知相关金融机构本项目准予提前注 销纸质投标保函。具体注销事宜由投标人与金融机构协商。保函原件上需要加盖正本吗？ 答：需要。但不将加盖正本作为评审因素。 问题11：我公司业绩为三个项目合并招标，三个项目合起来满足业绩要求，但分别签了三个合同和分别验收，请 问我公司业绩满足业绩要求吗？ 答：不满足。? 问题12：财务报告可以只提供审计报告、现金流量表、资产负债表、利润表吗？ 答：可以 。 问题13：业绩要求的竣工时间是指竣工验收时间吗？ 答：是的。 网 问题14：重庆市电子招投标系统投标文件-报价部分“己标价工程量清单”-“投标总价”页面招标人名称需要填 写吗？ 务 答：由投标人自行决定是否填写，是否填写不作为评审因素。 问题15：请问招标人是否委派业主专家参与评标吗？ 答：是，本项目评标委员会共7人，其中在重庆市综合评商标专家库随机抽取5人，招标人代表2人。 问题16：自来水厂或者净水厂含管道施工业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需道满足招标文件要求。? 问题17：有没有人行贿专家，有的话我们就不参加了。 答：本项目评标委员会由招标人按法律法规及相关规定依法组建。 管 问题18：招标文件第八章投标文件格式中（二）承诺部分是否包含招标文件要求的所有承诺，投标人是否还需要 提供其他格式之外的其他承诺？ 答：请各潜在投标人仔国细阅读招标文件，并按招标文件要求提供相应承诺。 问题19：财务报告可以不提供财务报表附注吗？ 答：可以。 中 问题20：乡、镇供水厂及供水管道业绩满足业绩要求吗？ 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题21：在职的已退休的注册人员，其社保局出具的养老证明已无法提供，该类人员是否可以用退休证、注册证 及在本单位注册的证明文件替代？ 答：退休证等材料不能替代养老保险证明，按招标文件执行。? 问题22：本项目是异地评标吗？ 答：是。 问题23：现在除了没有警戒线和技术方案的低价项目评标专家不被围猎，哪个项目不围猎评标专家，请问招标人 如何保证公平？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题24：没有低价警戒线怎么保证中高价呢？ 答：本项目未设置低价警戒线，通过综合评估法对各潜在投标人进行评审。分值由技术、商务、报价组成，综 合实力优良的投标人合理中高价可依靠综合得分优势参与竞争，同时招标文件履约追责条款约束投标人理性报 价，保障合理报价竞争环境。 问题25：现场递交纸质保函原件是否需要本项目投标人须知前附表中要求的委托代理人持授权委托书和养老保险 证明材料复印件递交吗？ 答：现场递交纸质保函原件的人员不作要求 。 问题26：请问投标文件制作系统软件导出的电子投标文件格式与加盖公章的招标文件PDF文件中的投标文件格式 不一致的以哪个为准？ 网 答：电子投标系统中锁定不可修改的格式（如封面、投标函）直接填空即可，其他投标文件格式以加盖公章的 招标文件PDF文件为准。? 问题27：专业分包业绩满足业绩要求吗？ 务 答：不满足。 问题28： 市政道路包含给水管网施工业绩满足业绩要求吗？ 商 答：投标人提供的业绩合同规模和工程类别需满足招标文件要求。 问题29：技术负责人在资格审查部分中提供了工程类高级及以上职称证后，在商务部分中再提供工程类高级及以 上职称证可以加分吗？ 道 答：可以。 问题30：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 管 全是万盛的公司中的！业主、专家全是你们自己人吧？ 答：本项目招标文件严格按照《重庆市房屋建筑和市政基础设施工程施工招标文件示范文本（2026年版）》编制， 且本项目评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 国 二、补遗 1、本次重新发布本项目的工程量清单，在《重庆市公共资源交易网》(綦江区) （https://www.cqggzy.com/qijiangweb/）网上发布，请投标人自行下载。 中 招 标 人：重庆市万盛经济技术开发区城市管理局 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 信息来源:https://www.chinapipe.net/project/d3074975.html cqdingjiu 2026.08.21 10:06:58</t>
+          <t>四川省华蓥市重点采煤沉陷区华蓥市高兴镇城镇危旧房改造项目(三期)施工一标段招标公告 1. 招标条件 1.1本招标项目四川省华蓥市重点采煤沉陷区华蓥市高兴镇城镇危旧房改造项目（三期）(项目名称)已由 华蓥市发展和改革局(项目审批、核准或备案机关名称)以华蓥市发展和改革局关于四川省华蓥市重点采煤沉陷区 华蓥市高兴镇城镇危旧房改造项目（三期）可行性研究报告的批复、华发改投〔2023〕191号（批文名称及编号） 批准建设，项目业主为华蓥市交通投资开发有限责任公司，建设资金来自上级补助和业主自筹（资金来源）， 项目出资比例为100%，招标人为华蓥市交通投资开发有限责任公司。项目已具备招标条件，现对该项目的施工 进行公开招标。 网 1.2本招标项目由华蓥市发展和改革局（核准机关名称）核准（招标事项核准文号为华发改投〔2023〕191号）的 招标组织形式为委托招标（□自行招标 委托招标）。招标人选择的招标代理机构是华蓥市国晟工程项目管理 咨询有限公司。 务 2. 项目概况与招标范围 2.1建设地点：华蓥市高兴镇。 商 2.2建设内容及规模：改造城镇危旧房约4.5万平方米，户数共220户，3栋共9个单元。配套小区内道路、供水、供 电、供气主管网、消防、路灯等基础设施。 本次实施该项目一标段：其实施内容为：新建道四通路与兴政路连接道路64米，铺设安置房一期商业街人行道5766 平方米，配套完善排水、路灯、绿化等附属设施。 2.3计划工期：90日历天。 管 2.4招标范围：本项目施工一标段施工图纸及工程量清单范围内的所有工作。 2.5标段划分：施工一标段。 （说明本次招标项目的国建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 3.1本次招标要求投标人须具备 中 3.1.1资质条件：具有国家建设行政主管部门颁发的市政公用工程施工总承包三级及以上资质。 3.1.2业绩要求： □近年（至投标截止时间，不少于3年）（多项选择：□已完成 □已完成或新承接或正在施工）不少于（1至3个） 个类似项目。类似项目是指:。 无业绩要求。 3.1.3项目经理的资格要求： 项目经理（项目负责人）资格：市政公用工程(注册专业)二级及以上（级别）建造师，具有省级及以上住房城 乡建设主管部门颁发的安全生产考核合格证（B证），/（业绩要求），须为本单位人员（若为联合体投标，须为 联合体牵头人人员）。 □园林绿化工程项目经理（项目负责人）资格：（职称级别）专业技术职称，（业绩要求），须为本单位人员 （若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受不接受联合体投标。联合体投标的，应满足下列要求： /。 3.3各投标人均可就上述1(具体数量)标段投标。 3.4本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东为大企业、与大企业的负责人 为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具体标 准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的通知》 （工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除技术复杂、 存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在3000万元以下的施工项目(标段) 应勾选此项。 ） 4. 招标文件的获取 网 4.1 凡有意参加投标者，请于2026-08-22 开始登录：全国公共资源交易平台（四川省·广安市）（网 址：https://gasggzy.cn）—“电子交易平台登录”—“投标登录”，通过数字证书免费下载招标资料（招标文件、 技术资料等）。 务 4.2 招标人不提供招标文件获取的其他方式。 5. 投标文件的递交 5.1投标文件递交的截止时间（投标截止时间，下同）为2商026-09-11 09:30，投标人应在投标截止时间前在线递交经 投标人数字证书加密的数据电文形式投标文件。 5.2 本项目开标实行（□见面开标使用不见面开标系统）开标方式，关于“不见面开标系统”的流程和注意事 项，请各交易主体在广安市公共资源交易网上道下载查看不见面开标系统操作指南。 6. 发布公告的媒介 本次招标公告在《全国公共资源交易平台（四川省）》和全国公共资源交易服务平台（四川省·四川 管 省）、全国公共资源交易平台（四川省· 广安市）(公告发布的其它媒介名称）上发布。 7.行政监督部门 单位名称：华蓥市发展国和改革局、华蓥市住房和城乡建设局 联系电话：0826-4895386、0826-4830288 8. 联系方式 中 招标人： 华蓥市交通投资开发有限责任公司 地 址： 四川省广安市华蓥市高兴火车站站前片区火车站北侧A幢1层商业4 邮 编： 638600 联系人： 王老师 电 话： 15196525437 传 真： / 电子邮件： / 网 址： / 开户银行： / 账 号： / 招标代理机构： 华蓥市国晟工程项目管理咨询有限公司 地 址： 四川省广安市华蓥市汪杜路397号附38号 邮 编： 638600 联系人： 唐老师 项目负责人： 唐玉琴 电 话： 13541983385 传 真： / 电子邮件： / 网 址： / 开户银行： / 网 账 号： / 日期：2026-08-21 务 注： （1）若划分标段，则填写标段序号；若划分为两个及以上标段，应分别明确各标段的具体内容、划分情况。 （2）招标人对投标人的资质要求，应是国家对投标人资商质的强制性规定。不是国家规定必须具备的资质，不得 作为资质要求。 （3）招标人对投标人的类似项目业绩要求，设置的投资额、面积、长度等规模量化指标不得高于本次招标工程 相应指标，类似项目业绩的定义应明确，用语准确无歧义。 道 （4）招标人要求投标人需具备的资质一个项目（标段）为一个，因特殊情况需要两个以上资质的，应当接受投 标人组成联合体投标，且限定的联合体成员数量不得少于设定的资质个数。 管 信息来源:https://www.chinapipe.net/project/d3077474.html cqdingjiu 2026.08.24 12:31:57 国 中</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -4145,14 +4209,14 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>重庆, 供水管网, 更新改造</t>
+          <t>四川, 华蓥市, 城镇危旧房改造, 市政公用工程, 施工一标段</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告</t>
+          <t>2026年绵阳市安州区高标准农田建设项目施工招标公告</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4162,7 +4226,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>房建</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4177,53 +4241,57 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>绵阳市</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>巴南区</t>
+          <t>安州区</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>为解决片区内涝问题，在李家沱街道、花溪街道改建d400-d800雨水管网9665m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管；改建d1000-d1400雨水管网664m，管材采用高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管；改建d1500-d2000雨水管网426m，管材采用III级钢筋混凝土管；改建d2100-d2600雨水管网1000m，管材采用III级钢筋混凝土管；修复雨水管网5345m，增加智能感知设备6套。</t>
+          <t>本项目包括河清镇高标准改造提升高标准农田3万亩，秀水镇改造提升高标准农田0.6万亩，花荄镇改造提升高标准农田0.3万亩。</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>本次招标项目工程费估算金额：11061.83万元，勘察设计合同估算金额：334.544万元。</t>
+          <t>项目资金来自中央财政资金、地方财政配套资金，出资比例为100%。</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>雨水管网、高密度聚乙烯(HDPE)缠绕结构壁管B型管、III级钢筋混凝土管、智能感知设备</t>
+          <t>高标准农田改造提升</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 重庆市巴南区土桥片区内涝积水整治工程勘察设计招标公告 1.招标条件 本招标项目 重庆市巴南区土桥片区内涝积水整治工程已由重庆市巴南区发展和改革委员会以巴南发改审 发[2025]33号文批准建设，项目业主为重庆市巴南区住房和城乡建设委员会，代建业主为重庆市巴南公路建设有 限公司，建设资金来自区级财政资金统筹，项目出资比例为 100%，招标人为重庆市巴南公路建设有限公司。 项目已具备招标条件，现对该工程的勘察设计进行公开招标，评标办法采用综合评估法。 网 2.项目概况与招标范围 2.1 建设地点：重庆市巴南区花溪街道、李家沱街道 务 2.2 项目概况与建设规模：为解决片区内涝问题，在李家沱街道、花溪街道改建 d400-d800 雨水管网 9665m，管材 采用高密度聚乙烯(HDPE)缠绕结构壁管 B型管；改建 d1商000-d1400雨水管网 664m，管材采用高密度聚乙 烯(HDPE)缠绕结构壁管 B 型管、III 级钢筋混凝土管；改建 d1500-d2000 雨水管网 426m，管材采用III 级钢筋混凝 土管;改建 d2100-d2600 雨水管网 1000m，管材采用 III 级钢筋混凝土管；修复雨水管网 5345m，增加智能感知设 备6 套。 道 2.3 本项目工程总投资金额：13477.10万元 管 本次招标项目工程费估算金额：11061.83万元 国 本次招标项目勘察设计合同估算金额：334.544万元 中 2.4 招标范围：主要包括勘察、施工图设计（包含高边坡、深基坑）和相应阶段的勘察工作，以及提供施工现场 全过程技术服务，并配合业主办理相关手续等，具体范围为： （1）勘察部分：完成本项目范围内的勘察工作，包括但不限于排水管网排查、1:500地形图测量、地质钻勘、管 线内窥、物探、综合管线测量，市政管网错混接点测量及调查等工作，解决区域地下空间臭气问题，勘察成果 需达到重庆市城市建成区排水管网排查技术导则的要求，并配合业主完成对应的成果审查等事宜。 （2）设计部分：包括不限于完成本项目的施工图设计、施工期间交通组织设计、桥梁（涉轨）安全论证方案及 施工期间至竣工验收阶段，质量保修阶段的设计配合服务，配合办理施工图审查相关手续及竣工验收阶段、质 量保修阶段的设计服务等工作以及协助招标人完成各项审批手续办理等工作。 2.5 勘察设计服务期限：30日历天 2.6 标段划分（如有）：/ 2.7 其他：/ 3.政府采购工程 3.投标人资格要求 3.1 本次招标要求投标人须具备以下条件： 网 3.1.1 本次招标要求投标人具备的资质条件： 务 投标人应同时具有建设行政主管部门颁发的下列勘察和设计两类资质： 商 I、投标人应具备下列勘察资质之一： 道 ①工程勘察综合甲级资质。 管 ②工程勘察专业类（岩土工程）专业甲级资质和工程勘察专业类（工程测量）甲级资质； 国 II、投标人应具备下列设计资质之一： 中 ①工程设计综合甲级资质； ②工程设计市政行业甲级资质； ③工程设计市政行业(燃气工程、轨道交通工程除外)甲级资质； ④工程设计市政行业(排水工程)甲级资质。 3.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的勘察设计能力，详见招标文件第二章投标人须知 前附表第1.4.1项内容。 3.2 本次招标接受联合体投标。联合体投标的，应满足下列要求：联合体组成单位数量不超过2家，由负责设计 任务的单位作为联合体牵头人。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易网下载招标文件及其附件、澄 清、修改、补充通知、最高限价通知等资料。参与投标的投标人需在重庆市公共网资源交易网完成市场主体信息 登记以及 CA 数字证书办理，办理方式请参见重庆市公共资源交易网导航栏“主体信息”页面中“市场主体信息 登记”“CA 数字证书办理”。若投标人未及时完成市场主体信息登记和 CA 数字证书办理导致无法完成全流程 电子招投标的，责任自负。 4.2投标人可在重庆市公共资源交易网本项目招标公告网页下方“我要提问”栏提出疑问，提问时间从本公告发 务 布至2026-08-23 12:00:00前。 4.3招标人应于2026-08-26 17:00:00前在重庆市公共资源交易网发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-24 09:30，投标人应当在投标截止时间前，通过互 商 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督道网、重庆市公共资源交易网、重庆市公共资源交易网（巴南区） 发布。[提示：依法必须招标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 重庆市巴南公路建设有限公司 代理机构: 重庆云远项目管理有限公司 管 地 址: 重庆市巴南区龙洲大道265号 地 址: 重庆市九龙坡区渝隆大厦28楼 邮 编: 邮 编: 项目负责人: 牟老师 项目负责人: 李强 国 电 话: 023-66238079 电 话: 023-68434996 传 真: 传 真: 电子邮箱: 电子邮箱: 中 开户银行: 开户银行: 账 号: 账 号: 监督部门: 重庆市巴南区发展和改革委员会 电 话: 023-66221670 2026年08月18日 重庆市巴南区土桥片区内涝积水整治工程勘察设计 户名 开户行 投标保证金账号 中国农业银行股份有限公司重庆自由 重庆联合产权交易所集团股份有限公司 312601010400083780000001675 贸易试验区分行 重庆联合产权交易所集团股份有限公司 重庆三峡银行九龙坡支行 9696801051304894 重庆联合产权交易所集团股份有限公司 中信银行重庆上清寺支行 3111230034020041267 重庆联合产权交易所集团股份有限公司 中国民生银行股份有限公司重庆分行 9902001764210157 中国建设银行股份有限公司重庆渝中 重庆联合产权交易所集团股份有限公司 6232813760000682897 支行 重庆农村商业银行股份有限公司沙坪 重庆联合产权交易所集团股份有限公司 0304010120010028835000509 坝支行 重庆联合产权交易所集团股份有限公司 重庆银行股份有限公司七星岗支行 15010202900420146639123 重庆联合产权交易所集团股份有限公司 招商银行股份有限公司重庆分行 123904808710630018252 信息来源:https://www.chinapipe.net/project/d3074953.html cqdingjiu 2026.08.21 10:06:58 网 务 商 道 管 国 中</t>
+          <t>2026年绵阳市安州区高标准农田建设项目施工招标公告 1. 招标条件 1.1本招标项目2026年绵阳市安州区高标准农田建设项目（项目名称）已由绵阳市农业农村局（项目审批、核准 或备案机关名称）以绵农发【2026】16号（批文名称及编号）批准建设，项目业主为绵阳市安州区土壤肥料站， 建设资金来自中央财政资金、地方财政配套资金（资金来源），出资比例为100%，招标人为绵阳市安州区土壤 肥料站。项目已具备招标条件，现对该项目的2026年绵阳市安州区高标准农田建设项目施工进行公开招标。 网 1.2本招标项目为绵阳市行政区域内的国家投资工程建设项目，绵阳市农业农村局（核准机关名称）核准（招标 事项核准文号为绵农发【2026】16号）的招标组织形式为□自行招标委托招标。招标人选择的招标代理机构是四 川中汇信成工程管理咨询有限公司。 2. 项目概况与招标范围 务 2.1 项目概况 建设地点：河清镇安罗村、白溪村、宝华村、广红村、桂商丰村、皇龙村、金华村、七一村、同盛村、同心村、 月溪村；秀水镇大泉村、农联村、蟠龙村、桥楼村和双泉村；花荄镇龙游村、狮回村。 建设内容及规模：①河清镇高标准改造提升高标准农田3万亩。②秀水镇改造提升高标准农田0.6万亩。③花荄镇 改造提升高标准农田0.3万亩。 道 标段划分：施工一个标段。 计划工期：360 日历天。 管 2.2 招标范围 本项目施工图纸及工程量清单所示的全部内容及发包人根据需要交由承包人实施的三通一平等建设内容（应具 备资质，须为可不执行国招标或政府采购程序的建设内容,应纳入工程变更审批）。 3. 投标人资格要求 中 3.1本次招标要求投标人须具备具备国家行政主管部门颁发的水利水电工程施工总承包二级或以上资质，近3年 （□已完工的□已完工的或正在施工的已完工的或正在施工的或新承接的）1个类似项目（类似项目指：单项合 同金额5000万元以上的水利或农业工程施工总承包（或工程总承包）），并在人员、设备、资金等方面具有相应 的施工能力。 3.2本次招标□接受不接受联合体投标。 联合体投标的，应满足下列要求：/。 3.3各投标人均可就上述合同标段中的1个(具体数量)合同标段投标。招标人□允许不允许投标人拟派的同一批项 目主要人员（项目经理、技术负责人）在1个及以上标段任职。 □3.4本次招标仅面向中小企业发包（其中属于大型企业的分支机构、存在控股股东为大型企业、与大型企业的 负责人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。 具体标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定 的通知》（工信部联企业〔2011〕300 号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除 技术复杂、存在特殊要求外，我市依法必须招标的国家投资工程，投标最高限价在5000万元以下的施工项目（标 段）应勾选此项。） 4. 招标文件的获取 4.1凡有意参加投标者： 请于2026-08-21起登陆全国公共资源交易平台（四川省·绵阳市）（网址：http://ggzy.my.gov.cn），通过数字证 书免费下载招标资料（招标文件、技术资料等）。 4.2 除上述方式外，招标人不提供其他任何报名和招标文件获取的方式。 5. 投标文件的递交 5.1 投标文件递交的截止时间（投标截止时间，下同）为2026-09-10 09:20，投标人应在截止时间前通过全国公 共资源交易平台（四川省·绵阳市）（电子招标投标交易平台）在线递交经投标人数字证书签名制作的数据加 密电子投标文件。 网 5.2逾期送达的投标文件，电子招标投标交易系统将予以拒收。 6. 发布公告的媒介 务 本次招标公告在全国公共资源交易平台（四川省）上发布。其他发布公告的媒介：全国公共资源交易平台（四 川省·绵阳市）（招标人自行选择，也可不填）。 商 7. 本项目招标投标行政监督部门 行政监督部门：绵阳市农业农村局电 话：0816-2268914 道 传 真：/电子邮件：/ 地 址：/ 8. 招标人承诺 管 本招标文件已经招标人（含招标代理机构）审查，不存在违反国家法律、法规、政策的情形。因招标文件设置 违反国家法律、法规、政策造成的相应后果，由招标人（含招标代理机构）负责。 国 9. 联系方式 招标人： 绵阳市安州区土壤肥料站 招标代理机构： 四川中汇信成工程管理咨询有限公司 中 四川省成都市武侯区二环路南三段5号人南大 地 址： 绵阳市安州区花荄镇白鹤路3号 地 址： 厦B座9楼10号 邮 编： 622651 邮 编： 610000 联系人： 董先生 联系人： 秦先生 电 话： 0816-6155882 电 话： 028-87549149 信息来源:https://www.chinapipe.net/project/d3077437.html cqdingjiu 2026.08.24 12:31:57</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>d800 雨水管网：9665m；d1400雨水管网：664m；d2000 雨水管网：426m；d2600 雨水管网：1000m；雨水管网：5345m</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N54" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 雨水管网, 高密度聚乙烯, 钢筋混凝土管</t>
+          <t>高标准农田, 改造提升, 施工招标</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>重庆燃气集团股份有限公司输配分公司大渡口调压站至二郎调压站次高压燃气管线工程(大渡口段)公告</t>
+          <t>金堂县2026年大豆单产提升工程施工招标公告</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4233,7 +4301,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>交通</t>
+          <t>水利</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4248,38 +4316,42 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>大渡口区</t>
+          <t>金堂县</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>安装部分包括材料验收、运输及履带式挖掘机及人工布管、管道管件安装、新旧管道的碰口、安装DN400直埋球阀1座、管道和商焊口的除锈及防腐、管道下沟后15KV电火花检测、管道的清管、强度及严密性试验、警示带敷设和线路标志桩（砖）安装、监检手续等。土建部分包括清表、扫线、平整场地、沟槽、基坑、阀井砌筑、回填土方、余方弃置、人工开挖人行道（花台）、公路及路面恢复、其他线缆穿跨越工道程施工、交通组织、水工保护等。</t>
+          <t>新建滴灌(喷灌)灌区16处，面积2070亩，配套机井5处、提灌站10处，利用现有供水泵站延伸管道灌溉700亩；新建提灌站5座；新建200m3圆形蓄水池10口，整治原有蓄水池4口；整治原有渠道10公里；购置智能灌溉机器人（车）2台。</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>政府资网金</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>燃气管线工程</t>
+          <t>水利设施</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>重庆燃气集团股份有限公司输配分公司大渡口调压站至二郎调压站次高压燃气管线工程(大渡口段)公告 采购 公告 公告编号： RQXYGG202608130064 一、采购项目基本情况 网 采购人：重庆燃气集团股份有限公司输配分公司 采购项目编号：RQCGXY202608130040 务 采购项目名称：大渡口调压站至二郎调压站次高压燃气管线工程（大渡口段） 采购内容或范围：安装部分： ①材料验收（甲供材料：阀门、管材、弯头、标志桩等）、运输及履带式挖掘机及人工布管； ②管道管件安装， 新旧管道的碰口；③安装DN400直埋球阀1座； ④管道和商焊口的除锈及防腐； ⑤管道下沟后15KV电火花检测； ⑥管道的清管，强度及严密性试验；⑦警示带敷设和线路标志桩（砖）安装； ⑧监检手续等。 土建部分： ①清表； ②扫线、平整场地； ③沟槽、基坑、阀井砌筑； ④回填土方； ⑤余方弃置； ⑥人工开挖人行道（花 台），公路及路面恢复； ⑦其他线缆穿跨越工道程施工，交通组织； ⑧水工保护等。 （具体内容详见施工图纸和 工程量清单） 公告发布时间 ：2026-08-18 14:39:10 管 二、采购人联系方式 联系人：王瑶 电话：023-67502265 国 邮箱：wangyao232@crcgas.com 三、采购明细 中 行号 采购内容 需求数量 单位 补充说明 拟邀请单位 大渡口调压站至二郎调压站次高压燃气管线 重庆燃气安装工程有限责任公 1 1 项目 无 工程(大渡口段) 司 四、服务费交纳 本项目不收取服务费。 五、 其他 事项 1.本公告在华润守正 采购交易 平 台（ https://www.szecp.com.cn/ ）上公开 发布。 2. 本项目采购通过守正平台线上进行，供应商需注册华润守正 采购交易 平台，通过平台进行响应文件的递交或 报价，具体操作步骤可查阅网站首页帮助中心的操作手册，也可以联系守正客服。 3 .答疑澄清、通知等文件一经在华润守正 采购交易 平台发布，视为已发放给相应供应商（发放时间即为发出时 间），请随时关注华润守正 采购交易 平台发布的相关信息，并及时查阅和处理。 4 .若有参与意向 ， 请于 2026-08-22 00:00:00前联系采购人 （联系方式见公示内容）反馈。 5 .若有异议 ， 请于 2026-08-22 00:00:00前提出异议 。 信息来源:https://www.chinapipe.net/project/d3074793.html cqdingjiu 2026.08.21 10:06:59 网 务 商 道 管 国 中</t>
+          <t>金堂县2026年大豆单产提升工程施工招标公告 1. 招标条件 1.1本招标项目 金堂县2026年大豆单产提升工程 (项目名称)已由 成都市农业农村局 (项目审批、核 准或备案机关名称)以 成都市农业农村局关于金堂县2026年大豆单产提升工程初步设计方案的批 复、[2026]2-33，成都市农业农村局关于金堂县2026年大豆单产提升工程初步设计方案变更的批复、[2026]8-18 （批文名称及编号）批准建设，项目业主为 金堂县农业农村局 ，建设资金来自 政府资 网 金 （资金来源），项目出资比例为 100% ，招标人为 成都金农兴投资管理有限公司。项目已具 备招标条件，现对该项目的施工进行公开招标。 1.2本招标项目由 成都市农业农村局 （核准机关名称）核准（招标事项核准文号 为 [2026]2-33、[2026]8-18 ）的招标组织形式为 委托招标 （□自行招务标 委托招标）。招标人选择 的招标代理机构是 四川朋顺工程项目管理有限公司 。 2. 项目概况与招标范围 商 2.1建设地点：官仓街道、栖贤街道。 2.2建设规模及内容：新建滴灌(喷灌)灌区16处，面积2070亩，配套机井5处、提灌站10处，利用现有供水泵站延 伸管道灌溉700亩；新建提灌站5座；新建200m3圆形蓄水池10口，整治原有蓄水池4口；整治原有渠道10公里；购 道 置智能灌溉机器人（车）2台。 2.3计划工期：180日历天。 2.4招标范围：本项目施工图及工程管量清单所示全部工程内容。 2.5质量标准：达到国家、行业现行验收合格标准。 2.6标段划分：本项目施工一个标段。 国 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 中 3.1本次招标要求投标人须具备 3.1.1资质要求： 具有国家行政主管部门颁发的水利水电工程施工总承包贰级及以上（含有效期内的叁级）资 质的单位 。 3.1.2业绩要求：（本项为多选） 近年（2023 年 01 月 01 日至投标截止时间，不少于3年）（多项选择：□已完成 已完成或新承接 或正在施工）不少于 1 （1 至3个）个类似项目。类似项目是指: 单项合同金额不低于500万 元水利工程相关施工业绩 。 □无业绩要求。 3.1.3项目负责人的资格要求：具有 水利水电工程专业二级及以上注册建造师 证 书， / （业绩要求） ，须为投标人本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 3.3本次招标仅面向中小企业发包（其中属于大型企业的分支机构、存在控股股东为大型企业、与大型企业的 负责人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。 具体标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定 的通知》（工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除 技术复杂、存在特殊要求外，我省依法必须招标的国家投资工程，投标最高限价在3000万元以下的施工项目（标 段）应勾选此项。） 3.4各投标人均可就上述 1 (具体数量)标段投标，可中标的标段数量为 1 个。 4. 招标文件的获取 4.1凡有意参加投标者，请于 2026 年 08 月 22日起，使用CA数字证书在成都市公共资源电子交易云平 台(www.cdggzy.com）（以下简称“电子交易云平台”）免费下载招标资料（招标文件及相关资料），获得“拟 投标项目回执”。 网 4.2 招标人不提供邮购招标文件服务。 5. 投标文件的递交 务 ●（不见面开标）5.1 投标文件递交的截止时间（投标截止时间，下同）为2026年09月11日09时30分，招标人或其 委托代理机构，以及已在投标截止时间前按规定上传投标文件的投标人，均应在开标当日投标截止时间前登录 不见面开标系统（网址：www.cdggzy.com），录入相关人员姓名、电话等基本信息。投标人未按时登录不见面开 标系统，错过开标解密时间的，由投标人自行承担不利后商果。 ●（不见面开标）5.2 投标人应在解密开始后30分钟内在线完成投标文件解密。投标文件未能在规定时间内成功 解密的，视为投标人未在规定时间内提交投标文件，由投标人自行承担责任。不见面开标项目不接受投标人现 场递交光盘等形式的投标文件，不接受投标人道现场解密投标文件。 6. 发布公告的媒介 本次招标公告在全国公共资源交易平台（四川省）、成都市公共资源交易服务中心（网址：http://ggzyjy.sc.gov.cn、 管 www.cdggzy.com）上发布。 7. 行政监督 单位名称： 金堂县农业国农村局 联系电话： 028-84982519 8.联系方式 中 招 标 人： 成都金农兴投资管理有限公司 地 址：四川省成都市金堂县竹篙镇竹富路466号1栋2楼（食用菌产业园区） 邮 编： 610400 联 系 人： 邓老师 电 话： 028-84905666 招标代理机构： 四川朋顺工程项目管理有限公司 地 址： 成都市青羊区顺城大街269号富力中心A座2103 邮 编： 610000 联 系 人： 朱老师 电 话： 028-86925238 2026 年 08 月 21日 注： （1）若划分标段，则填写标段序号；若划分为两个及以上标段，应分别明确各标段的具体内容、划分情况。 （2）招标人对投标人的资质要求，应是国家对投标人资质的强制性规定。不是国家规定必须具备的资质，不得 作为资质要求。 网 （3）招标人对投标人的类似项目业绩要求，设置的投资额、面积、长度等规模量化指标不得高于本次招标工程 相应指标，类似项目业绩的定义应明确，用语准确无歧义。 务 （4）招标人要求投标人需具备的资质一个项目（标段）为一个，因特殊情况需要两个以上资质的，应当接受投 标人组成联合体投标，且限定的联合体成员数量不得少于设定的资质个数。 信息来源:https://www.chinapipe.net/project/d3077434.html 商 cqdingjiu 2026.08.24 12:31:58 道 管 国 中</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>滴灌(喷灌)灌区设备、机井、提灌站、蓄水池、渠道整治设备、智能灌溉机器人（车）</t>
         </is>
       </c>
       <c r="N55" t="n">
@@ -4287,14 +4359,14 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>金堂县, 大豆单产提升工程, 水利设施, 滴灌, 喷灌, 机井, 提灌站, 蓄水池, 渠道整治, 智能灌溉机器人</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>石柱公司2026-2027年度用户供水管道安装及管网抢(维)修工程(第二次)项目公告</t>
+          <t>金堂县2026年玉米单产提升工程施工招标公告</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4304,7 +4376,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>房建</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4319,53 +4391,57 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>石柱土家族自治县</t>
+          <t>金堂县</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-2027年度用户供水管道安装及管网抢（维）修服务</t>
+          <t>新建输配水管道147.5km，新建首部枢纽21座，田间自动化控制闸阀1474套，中等流量喷枪1349道套、快速取水阀188套，300m3蓄水池2座，移动式喷灌设备10套。</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>项目资金来自企业自筹，合同估算金额约280万元</t>
+          <t>政府资金，网项目出资比例为100%</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>供水管道安装及管网抢（维）修服务</t>
+          <t>输配水管道，首部枢纽，自动化控制闸阀，中等流量喷枪，快速取水阀，蓄水池，移动式喷灌设备</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>石柱公司2026-2027年度用户供水管道安装及管网抢(维)修工程(第二次)项目公告 石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（比选公告 1.比选条件 本比选项目石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程（第二次）（项目名称），比选人 为重庆石柱水利水电实业开发有限公司，比选项目资金来自企业自筹（资金来源），项目已具备比选条件。现 对本项目进行公开比选，诚邀有兴趣的潜在投标人参与投标。 网 2.项目概况与比选范围 2.1 建设地点：比选人指定地点 务 2.2 项目概况与建设规模：2026-2027年度用户供水管道安装及管网抢（维）修服务 2.3 本次比选项目合同估算金额：约280万元 商 2.4 比选范围：完成石柱公司2026-2027年度用户供水管道安装及管网抢（维）修工程包括公司供水范围内用户 各类管道及管件安装、水表安装及更换、阀门安装等、并完成配套土建工程、零星签证等工程量清单所列项目、 管网抢维修和公司所属生产单元零星项目，具体内容详见第五章 工程量清单。 道 2.5 工期要求：1年 缺陷责任期要求：24个月 管 3.投标人资格要求 3.1 本次比选要求投标人须具备以下条件： 国 3.1.1 本次比选要求投标人具备的资质条件：具备建设行政主管部门颁发的有效的市政公用工程施工总承包贰级 及以上资质； 3.1.2 投标人还应在人员、设备、资金等方面具有相应的施工能力，详见比选文件第二章投标人须知前附表第1.4.1 中 项内容。 3.2 本次比选不接受联合体投标。 4.比选文件的获取 4.1 投标人于2026年08月18日起可自行在重庆水务集团电子商务平台(https://www.cqswjt.cn)上下载比选文件电子版， 以及答疑、补遗等投标截止时间前公布的所有相关资料，不管投标人下载与否，比选人和比选代理机构都视为 投标人收到以上资料并全部知晓有关比选过程和事宜，如因投标人自身原因未能下载相关资料由此产生的一切 后果由投标人自行负责。各投标人应随时关注网上(https://www.cqswjt.cn)发布的比选文件及相关修改内容。 4.2 投标人须在重庆水务集团电子商务平台(https://www.cqswjt.cn)进行投标人注册，填写相关信息，审批过后成为 平台投标人。 4.3 此项目将在重庆水务集团电子商务平台系统上进行电子开、评标。投标人需提前在重庆水务集团电子商务平台 (https://www.cqswjt.cn)上注册、报名，下载比选文件，上传电子投标文件并报价，递交纸质投标文件。在投标截 止时间前未按时报名、报价并上传电子投标文件、递交纸质投标文件者，被视为无效。 4.4比选文件每份售价1000 元，售后不退。投标人在递交纸质投标文件时支付，否则比选人拒绝接收其投标文 件。 5.投标文件的递交 5.1电子投标文件递交时间：2026年08月24日10时00分（北京时间）前，投标人自行上传至重庆水务集团电子商务 平台(https://www.cqswjt.cn)； 5.2 纸质投标文件递交时间：2026年08月24日09时30分至10时00分，地点：水务集团招标采购中心（重庆市两江新 区嘉华路36号重庆水务大厦五楼）。 5.3 投标截止时间：2026年08月24日10时00分（北京时间）。 网 5.4 逾期送达的或者未送达指定地点的投标文件，比选人不予受理。 6.发布公告的媒介 务 本次比选公告在重庆水务集团电子商务平台(https://www.cqswjt.cn)上发布。 7.联系方式 商 比 选 人：重庆石柱水利水电实业开发有限公司 比选代理机构：重庆水务集团公用工程咨询有限公司 地 址：重庆市石柱土家族自治县都督大道11号 地 址：重庆市两江新区嘉华路36号重庆水务大厦1018 联 系 人：王老师 联 系 人：颜老师 道 电 话：13658292968 电 话：023-67901915 重庆水务电子商务平台咨询电话：管023-67453670（工作时间：9：00-12：30；14：00-17：00） 信息来源:https://www.chinapipe.net/project/d3074720.html cqdingjiu 2026.08.21 10:06:59 国 中</t>
+          <t>金堂县2026年玉米单产提升工程施工招标公告 1. 招标条件 1.1本招标项目 金堂县2026年玉米单产提升工程 (项目名称)已由 成都市农业农村局 (项目审批、核 准或备案机关名称)以 成都市农业农村局关于金堂县2026年玉米单产提升工程初步设计方案的批复、[2026] 2-32， 成都市农业农村局关于金堂县2026年玉米单产提升工程初步设计方案变更的批复、[2026] 8-17 （批文名称及编 号）批准建设，项目业主为 金堂县农业农村局 ，建设资金来自 政府资金 （资金来源）， 网 项目出资比例为 100% ，招标人为 成都金农兴投资管理有限公司 。项目已具备招标条件，现对该 项目的施工进行公开招标。 1.2本招标项目由 成都市农业农村局 （核准机关名称）核准（招标事项核准文号为 ）的招标组织形式 为 委托招标 （□自行招标 委托招标）。招标人选择的招标代理机构务是 四川方裕工程项目管理有限 公司 。 2. 项目概况与招标范围 商 2.1建设地点：金堂县。 2.2建设规模及内容：新建输配水管道147.5km，新建首部枢纽21座（其中包括自动反冲洗砂石过滤器、自动反冲 洗叠片式过滤器，增压水泵，施肥设施及相应的电气设施等），田间自动化控制闸阀1474套，中等流量喷枪1349 道 套、快速取水阀188套，300m3蓄水池2座，移动式喷灌设备10套。 2.3计划工期：180日历天。 2.4招标范围：本项目施工图及工程管量清单所示全部工程内容。 2.5质量标准：达到国家、行业现行验收合格标准。 2.6标段划分：本项目施工一个标段。 国 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 中 3.1本次招标要求投标人须具备 3.1.1资质要求： 具有国家行政主管部门颁发的水利水电工程施工总承包贰级及以上（含有效期内的叁级）资 质的单位 。 3.1.2业绩要求：（本项为多选） 近年（2023 年 01 月 01 日至投标截止时间，不少于3年）（多项选择：□已完成 已完成或新承接 或正在施工）不少于 1 （1 至3个）个类似项目。类似项目是指: 单项合同金额不低于500万 元水利工程相关施工业绩 。 □无业绩要求。 3.1.3项目负责人的资格要求：具有 水利水电工程专业二级及以上注册建造师 证 书， / （业绩要求） ，须为投标人本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： / 。 3.3本次招标仅面向中小企业发包（其中属于大型企业的分支机构、存在控股股东为大型企业、与大型企业的 负责人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。 具体标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定 的通知》（工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除 技术复杂、存在特殊要求外，我省依法必须招标的国家投资工程，投标最高限价在3000万元以下的施工项目（标 段）应勾选此项。） 3.4各投标人均可就上述 1 (具体数量)标段投标，可中标的标段数量为 1 个。 4. 招标文件的获取 4.1凡有意参加投标者，请于2026 年 08 月 22日起，使用CA数字证书在成都市公共资源电子交易云平 台(www.cdggzy.com）（以下简称“电子交易云平台”）免费下载招标资料（招标文件及相关资料），获得“拟 投标项目回执”。 网 4.2 招标人不提供邮购招标文件服务。 5. 投标文件的递交 务 ●（不见面开标）5.1 投标文件递交的截止时间（投标截止时间，下同）为2026年09月14日09时30分，招标人或其 委托代理机构，以及已在投标截止时间前按规定上传投标文件的投标人，均应在开标当日投标截止时间前登录 不见面开标系统（网址：www.cdggzy.com），录入相关人员姓名、电话等基本信息。投标人未按时登录不见面开 标系统，错过开标解密时间的，由投标人自行承担不利后商果。 ●（不见面开标）5.2 投标人应在解密开始后30分钟内在线完成投标文件解密。投标文件未能在规定时间内成功 解密的，视为投标人未在规定时间内提交投标文件，由投标人自行承担责任。不见面开标项目不接受投标人现 场递交光盘等形式的投标文件，不接受投标人道现场解密投标文件。 6. 发布公告的媒介 本次招标公告在全国公共资源交易平台（四川省）、成都市公共资源交易服务中心（网址：http://ggzyjy.sc.gov.cn、 管 www.cdggzy.com）上发布。 7. 行政监督 单位名称： 金堂县农业国农村局 联系电话： 028-84982519 8.联系方式 中 招 标 人： 成都金农兴投资管理有限公司 地 址：四川省成都市金堂县竹篙镇竹富路466号1栋2楼（食用菌产业园区） 邮 编： 610400 联 系 人： 邓老师 电 话： 028-84905666 招标代理机构： 四川方裕工程项目管理有限公司 地 址： 成都市郫都区福粮路锦巷兰台十一栋2106 邮 编： 610000 联 系 人： 刘老师 电 话： 028-63947572 2026 年 08 月 21日 注： （1）若划分标段，则填写标段序号；若划分为两个及以上标段，应分别明确各标段的具体内容、划分情况。 （2）招标人对投标人的资质要求，应是国家对投标人资质的强制性规定。不是国家规定必须具备的资质，不得 作为资质要求。 网 （3）招标人对投标人的类似项目业绩要求，设置的投资额、面积、长度等规模量化指标不得高于本次招标工程 相应指标，类似项目业绩的定义应明确，用语准确无歧义。 务 （4）招标人要求投标人需具备的资质一个项目（标段）为一个，因特殊情况需要两个以上资质的，应当接受投 标人组成联合体投标，且限定的联合体成员数量不得少于设定的资质个数。 商 信息来源:https://www.chinapipe.net/project/d3077433.html cqdingjiu 2026.08.24 12:31:58 道 管 国 中</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>排水钢管 Φ200*6m：3000米</t>
         </is>
       </c>
       <c r="N56" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>重庆, 供水管道安装, 管网抢修, 企业自筹, 280万元</t>
+          <t>金堂县, 2026年玉米单产提升工程, 输配水管道, 自动化控制闸阀, 蓄水池, 移动式喷灌设备</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程(甲供材料)答疑(一)</t>
+          <t>攀枝花市钒钛高新区金江片区排水防涝能力提升工程施工招标公告</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4390,34 +4466,42 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>攀枝花市</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>攀枝花市</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程涉及3PE防腐钢管的采购，其管道部分壁厚需符合国标标准并达到设计要求。</t>
+          <t>项目改造金江片区排水防涝管网及设施，主要包含以下内容:（1）改造B*H=600*800排水边沟2238m;（2）改造B*H=1500*2000排洪沟1306道m，B*H=2000*1500排洪沟120m,B*H=2500*3000排洪沟450m，B*H=3500*4000排洪沟2800m，B*H=5000*4000 排洪沟2845mB*H=6000*4000排洪沟545m;（3）排洪沟清淤18484m;排洪涵清淤2500m;（4）改造两座雨水调蓄池，规模为8000t/d和1000t/d;（5）同步布设智能物联感知设备。</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>项目详情中未提及具体资金情况。</t>
+          <t>总投资6920万元</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>3PE防腐钢管</t>
+          <t>排水边沟、排洪沟、雨水调蓄池、智能物联感知设备</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>万盛城区老旧供水管网更新改造工程(甲供材料)答疑(一) 万盛城区老旧供水管网更新改造工程（甲供材料） 答疑（一） 各潜在投标人： 现将万盛城区老旧供水管网更新改造工程（甲供材料）答疑（一）相关条款通知如下： 网 一、答疑 问题1：请问招标人是否委派业主专家参与评标吗？ 务 答：是，本项目评标委员会共7人，其中在重庆市综合评标专家库随机抽取5人，招标人代表2人。 问题2：万盛的项目挂綦江来投这样都还控制不了还全是你们万盛公司中的？是有啥猫腻是吧？参考之前的项目 全是万盛的公司中的！业主、专家全是你们自己人吧？ 商 答：本项目招标文件严格按照《重庆市工程建设项目货物采购招标文件示范文本（2026年版）》编制，且本项目 评标委员会由招标人按法律法规及相关规定依法组建，欢迎各潜在投标人积极参与投标。 问题3：3PE管道部分壁厚是多少呢？ 道 答：本项目采购的3PE防腐钢管的管道部分壁厚须符合国标标准并达到设计要求。 招 标 人：重庆市万盛经济技术开发区城市管理局 管 招标代理机构：重庆力圣建设工程咨询有限公司 2026年8月18日 国 信息来源:https://www.chinapipe.net/project/d3074712.html cqdingjiu 2026.08.21 10:06:59 中</t>
+          <t>攀枝花市钒钛高新区金江片区排水防涝能力提升工程施工招标公告 1. 招标条件 1.1本招标项目攀枝花市钒钛高新区金江片区排水防涝能力提升工程(项目名称)已由攀枝花钒钛高新技术 产业开发区科技创新和经济发展局(项目审批、核准或备案机关名称)以关于批复攀枝花市钒钛高新区金江片区排 水防涝能力提升工程可行性研究报告的函、攀钒钛科经函[2025]56号（批文名称及编号）批准建设，项目业主为 攀枝花钒钛高新技术产业开发区投资和政务服务中心，建设资金来自上级补助资金及地方配套资金（资金来 源），项目出资比例为100%，招标人为攀枝花钒钛高新技术产业开发区投资和政务服务中心。项目已具备招标 条件，现对该项目的施工进行公开招标。 网 1.2本招标项目由攀枝花钒钛高新技术产业开发区科技创新和经济发展局（核准机关名称）核准（招标事项核准 文号为攀钒钛科经函[2025]56号）的招标组织形式为委托招标（□自行招标 委托招标）。招标人选择的招标代 理机构是四川省中城泰达工程咨询集团有限公司。 务 2. 项目概况与招标范围 2.1项目名称：攀枝花市钒钛高新区金江片区排水防涝能力提升工程。 商 2.2建设地点：攀枝花市钒钛高新区金江片金江片区。 2.3建设内容及投资：项目改造金江片区排水防涝管网及设施，主要包含以下内容:（1）改造B*H=600*800排水边 沟2238m;（2）改造B*H=1500*2000排洪沟1306道m，B*H=2000*1500排洪沟120m,B*H=2500*3000排洪 沟450m，B*H=3500*4000排洪沟2800m，B*H=5000*4000 排洪沟2845mB*H=6000*4000排洪沟545m;（3）排洪沟清 淤18484m;排洪涵清淤2500m;（4）改造两座雨水调蓄池，规模为8000t/d和1000t/d;（5）同步布设智能物联感知设 备；总投资6920万元。 管 2.4招标范围：本项目施工图设计范围内的全部内容，施工直至竣工验收合格及整体移交、工程保修期内的缺陷 修复和保修工作等全部工作，具体范围详见招标工程量清单。 2.5标段划分：1个标段。 国 2.6计划工期：540日历天。 2.7质量要求：达到国家现行施工质量验收规范的合格标准 。 中 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 3.1本次招标要求投标人须具备 3.1.1资质条件： （1）具有独立法人资格；（2）具有建设行政主管部门颁发的市政公用工程施工总承包二级及 以上资质 。 3.1.2业绩要求： 近年（ 2023 年 1 月 1 日至投标截止时间，不少于3年）（□已完成 已完成或新承接或正在施工）不少于 1 （1至3个）个类似项目。类似项目是指: 市政公用工程施工业绩(业绩需提供省级及以上公共资源交易网中标公示 查询截图，在建或新承接还需提供中标通知书及施工合同，已完成的还需提供中标通知书、施工合同及竣工验 收报告 。 □无业绩要求。 3.1.3项目经理的资格要求： 项目经理（项目负责人）资格： 市政公用工程 (注册专业)二级及以上（级别）建造师，具有省级及以上住房 城乡建设主管部门颁发的安全生产考核合格证（B证），/（业绩要求），须为本单位人员（若为联合体投标，须 为联合体牵头人人员）。 □园林绿化工程项目经理（项目负责人）资格： （职称级别）专业技术职称， （业绩 要求），须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： 。 3.3各投标人均可就上述 1 (具体数量)标段投标。 □ 3.4本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股网东为大企业、与大企业的负责人 为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具体标 准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的通知》 （工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除技术复杂、 存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在3000万元以下的施工项目(标段)应勾选此项。 务 ） 4. 招标文件的获取 4.1 凡有意参加投标者，请于 2026 年 08 月 22 日开始登陆商：□全国公共资源交易平台（四川省）（网 址：http://ggzyjy.sc.gov.cn）—“登录”——“交易主体”—“建设工程”，通过数字证书免费下载招标资料（招 标文件、技术资料等）。全国公共资源交易平台（四川省· 攀枝花 市（州））（网址： http://www. pzhggzy.cn ）—“登录”—“ 攀枝花市工程建设交易系统 ”，通过数字证书免费下载招标资料（招标文件、技术资料等）。 道 4.2 招标人不提供招标文件获取的其他方式。 5. 投标文件的递交 管 投标文件递交的截止时间（投标截止时间，下同）为2026年09月14日9时30分，投标人应在投标截止时间前在线 递交经投标人数字证书加密的数据电文形式投标文件。 6. 发布公告的媒介 国 本次招标公告在《全国公共资源交易平台（四川省）》和全国公共资源交易平台（四川省·攀枝花 市）(公告发布的其它媒介名称）上发布。 7.行政监督部门 中 单位名称： 攀枝花钒钛高新技术产业开发区自然资源和建设交通局 联系电话： / 8. 联系方式 招 标 人：攀枝花钒钛高新技术产业开发区投资和政务服务中心 地 址：攀枝花市仁和区科创路8号 邮 编：617000 联 系 人：彭老师 电 话：0812-3982759 传 真：/ 电子邮件：/ 网 址：/ 开户银行：/ 账 号：/ 招标代理机构：四川省中城泰达工程咨询集团有限公司 地 址：成都市金牛区金科中路32号迪舒美领4栋12号 网 邮 编：610000 联 系 人：饶先生 务 项目负责人：饶寨东 电 话：028-87776626 商 信息来源:https://www.chinapipe.net/project/d3077430.html cqdingjiu 2026.08.24 12:31:58 道 管 国 中</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>排水边沟 B*H=600*800 2238m; 排洪沟 B*H=1500*2000 1306道m, B*H=2000*1500 120m, B*H=2500*3000 450m, B*H=3500*4000 2800m, B*H=5000*4000 2845m, B*H=6000*4000 545m; 排洪沟清淤 18484m; 排洪涵清淤 2500m; 雨水调蓄池 8000t/d 和 1000t/d</t>
         </is>
       </c>
       <c r="N57" t="n">
@@ -4425,14 +4509,14 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 3PE防腐钢管, 资金情况, 产品种类</t>
+          <t>排水防涝, 排水边沟, 排洪沟, 雨水调蓄池</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>南岸区茶园片区乡镇老旧供水管网更新改造工程更正公告</t>
+          <t>中二十四局集团上海电务电化有限公司天眉乐高速公路项目JD3标、JA3标隔离栅、防落物网、防眩板、电缆、光缆及硅芯管询价补遗公告</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4442,7 +4526,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>交通</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4457,38 +4541,42 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>乐山市</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>南岸区</t>
+          <t>乐山市</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展水土保持监管测工作。</t>
+          <t>本次询价采购JD-03包件硅芯管的底色、色谱如下：商序号规格底色添加色标颜色1Φ40/33黑色黑色道2Φ40/33黑色白色1x43Φ40/33黑色黄色1x44Φ40/33黑色蓝色管1x45Φ40/33黑色绿色1x46Φ40/33黑色红色1x47Φ40/33黑色国紫色1x48Φ40/33黑色白色2x39Φ40/33黑色黄色2x310Φ40/33黑色蓝色2x311Φ40/33黑色绿色2x312Φ40/33黑色红色2x313Φ40/33黑色紫色2x314Φ40/33黑色白色3x215Φ40/33黑色黄色3x216Φ40/33黑色蓝色3x217Φ40/33黑色绿色3x218Φ40/33黑色红色3x2</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>项目详细内容无法识别</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>供水管网</t>
+          <t>硅芯管</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>南岸区茶园片区乡镇老旧供水管网更新改造工程更正公告 南岸区茶园片区乡镇老旧供水管网更新改造工程更正公 告 发布日期： 2026年8月18日 网 首次公示日期： 2026年8月14日 更正日期： 2026年8月18日 采购人名称： 重庆市江南城市建设发展（集团）有限公司务 采购人地址： 重庆市南岸区米兰路51号电子信息标准化厂房2号楼 联系人： 赵老师 商 电话： 023-62820331 采购代理机构名称： 重庆多杰数字科技咨询服务有限公司 采购代理机构地址： 重庆市重庆市经开区重庆市经开区长生桥镇江峡路8号13-1幢1楼 道 经办人名称： 李佩奇、戴沛轩、李倩 联系电话： 023-67648437 本项目比选范围修改为：在项目动工前完成水土保持方案审批程序，项目建设过程开展 更正事项： 水土保持监管测工作。 https://www.gec123.com/notices/detail/1665701682723590144 信息来源:https://www.c国hinapipe.net/project/d3074669.html cqdingjiu 2026.08.21 10:07:01 中</t>
+          <t>中二十四局集团上海电务电化有限公司天眉乐高速公路项目JD3标、JA3标隔离栅、防落物网、防眩板、电缆、 光缆及硅芯管询价补遗公告 各潜在报价单位： 为保障本次询价采购工作公平、公正、公开开展，确保各报价单位准确、完整理解本次询价项目相关要求，针 对本次 【 中铁二十四局集团上海电务电化有限公司天眉乐高速公路项目 JD3标、JA3标隔离栅、防落物网、防眩 板、电缆、光缆及硅芯管询价 】 （询价编号： CR24(2026)-DWDH-XJ-TML-JDJA-01）询价文件，经采购单位核 查确认，现对文件相关内容作如下 补遗 、补充及更正，本 补遗 与原询价文件具有同等法律效力。 网 一、 补遗如下 1.原文件内容：【 第二章 供应商报价 ， 报价函附件 3付款方的承诺 】 ； 务 更正后内容：【第二章 供应商报价，报价函附件 3付款 方式 的承诺】 ， 报价单位 应说明响应询价文件中的付款 方式。 2. 本次询价采购 JD-03包件硅芯管的底色、色谱如下： 商 序号 规格 底色 添加色标 颜 色 1 Φ40/33 黑色 黑色 道 2 Φ40/33 黑色 白色 1×4 3 Φ40/33 黑色 黄色 1×4 4 Φ40/33 黑色 兰色 管1×4 5 Φ40/33 黑色 绿色 1×4 6 Φ40/33 黑色 红色 1×4 7 Φ40/33 黑色 国紫色 1×4 8 Φ40/33 黑色 白色 2×3 9 Φ40/33 黑色 黄色 2×3 中 10 Φ40/33 黑色 兰色 2×3 11 Φ40/33 黑色 绿色 2×3 12 Φ40/33 黑色 红色 2×3 13 Φ40/33 黑色 紫色 2×3 14 Φ40/33 黑色 白色 3×2 15 Φ40/33 黑色 黄色 3×2 16 Φ40/33 黑色 兰色 3×2 17 Φ40/33 黑色 绿色 3×2 18 Φ40/33 黑色 红色 3×2 3.本次询价采购采用经评审的最低投标价报价法：质量、服务满足询价文件全部实质性条款，经资格及符合性审 查合格后，按有效报价由低至高排序，推荐合理最低价为成交供应商。 二、补充说明事项 1.本 补遗 为本次询价文件的组成部分，与原询价文件内容不一致之处，以本 补遗 为准；本 补遗 未提及的内容， 仍按原询价文件规定执行。 2.各报价单位须充分研读本 补遗 全部内容，严格按照 补遗 后的完整文件要求编制、提交报价文件，未结合本 补 遗 制作的报价文件，视为无效报价。 3 .各潜在报价单位收到本 补遗 后，无需单独回复确认，自行落实文件解读及报价编制工作即可。 三、联系方式 1.采购 组织 单位 ： 中铁二十四局集团有限公司设备物资集采中心电务分中心 联 系 人： 陈先生 联系 电话： 021-51226136 2.采购人 ： 中铁二十四局集团上海电务电化有限公司天眉乐高速公路项目 JD3标网、JA3标项目经理部 地 址： 四川省乐山市市中区佛光路 525号 技术 联系人： 左先生 务 联系 电话： 19136188150 中铁二十四局集团有限公司设备物资集采中心电务分中心 商 2026 年 8 月 20 日 信息来源:https://www.chinapipe.net/project/d3077384.html 道 cqdingjiu 2026.08.24 12:31:58 管 国 中</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>Φ40/33黑色白色1x4；Φ40/33黑色黄色1x4；Φ40/33黑色蓝色1x4；Φ40/33黑色绿色1x4；Φ40/33黑色红色1x4；Φ40/33黑色国紫色1x4；Φ40/33黑色白色2x3；Φ40/33黑色黄色2x3；Φ40/33黑色蓝色2x3；Φ40/33黑色绿色2x3；Φ40/33黑色红色2x3；Φ40/33黑色紫色2x3；Φ40/33黑色白色3x2；Φ40/33黑色黄色3x2；Φ40/33黑色蓝色3x2；Φ40/33黑色绿色3x2；Φ40/33黑色红色3x2</t>
         </is>
       </c>
       <c r="N58" t="n">
@@ -4496,14 +4584,14 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>重庆, 管材招标, 商机</t>
+          <t>重庆, 四川, 近三天, 管材, 招标商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部排水钢管询价采购公告</t>
+          <t>贡井区2026年大豆单产提升工程招标计划</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4528,49 +4616,57 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>自贡市</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>贡井区</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治县。合同金额28.01亿元，合同工期73个月，主要工程包括新方斗山隧道、石板坡隧道、城北隧道、刘家坪隧道、刘家店子1号大桥工程、刘家店子2号大桥、城北大桥、冉家湾大桥，采用移动模架和支商架法现浇施工，正线铺无砟道床43.808Km。</t>
+          <t>实施建设大豆种植智能滴灌系统2处，共计300亩智能滴灌示范区网，新建蓄水池23座；开展大豆单产提升技术推广。</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>合同金额28.01亿元</t>
+          <t>估算总投资14455000.00元</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>排水钢管Φ200*6m</t>
+          <t>智能滴灌系统、蓄水池</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部排水钢管询价采购公告 中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 排水钢管询价采购公告 询价编号：ZT1105-XJ-2026-561-1 尊敬的各潜在供应商: 网 本着公平、公正、公开、诚实信用的原则，诚挚的邀请贵公司参与中铁十一局集团有限公司宜涪高铁重庆段站 前3标项目经理ZT1105-XJ-2026-561-1，排水钢管材料的报价。 一、项目概况 务 中铁十一局集团宜涪高铁3标项目，位于重庆市石柱土家族自治（县）。合同金额28.01亿元，合同工期73个月， 开工日期：2024年12月，竣工日期：2030年12月。主要工程：新方斗山隧道(10660m)、石板坡隧道(4148m)、城北 隧道(3228m)、刘家坪隧道(2077m);刘家店子1号大桥工程(224.096m)、刘家店子2号大桥(232.099m)、城北大 桥(330.241m)、冉家湾大桥(355.245m),采用移动模架和支商架法现浇施工，其中24米移动模架施工6孔；32米支架法 施工5孔，移动模架施工28孔;正线铺无砟道床43.808Km。 二、询价内容 道 本次计划对排水钢管、GG-01材料进行询价，询价内容如下： 询价物资一览表 管 序号 包件号 物资名称 规格型号 计量单位 数量 备注 1 GG-01 排水钢管 Φ200*6m 米 3000 Q235B，壁厚6mm 合计 3000 国 说明：1.表中数量为计划数量，实际采购过程中可能有所调整，最终结算按照实际采购数量结算。 2.收货地点：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 中 三、技术质量及报价要求 1. 此次排水钢管、GG-01各项技术性能：Q235B 碳素结构钢无缝钢管，符合 GB/T8163 标准。质量需满足甲方项 目部正常使用的要求，保证产品的质量合格，满足试验室检测所有要求，详见技术规格书。 2.报价按要求综合报价，包含但不限于材料费、搬运、储存、装车、运杂、售后服务费、利润、税费等除到场所 需的一切费用。在报价税率不同时，以不含税总价作为评审依据。 四、结算及付款方式 自发票认证完成之日起第3个月，支付至本次结算金额的30%；自发票认证完成之日起第6个月，支付至本次结算 金额的累计70%（即在本阶段支付40%）；在办理末次结算后1年内，累计支付总额不超结算总金额的75%，剩 余25%的尾款在3年内付清，且甲方每年付款比例不低于15%（如：办理末次结算后第二年，支付金额应大于等于 尾款总额的15%；办理末次结算后第三年，支付金额应大于等于尾款总额的15%；办理末次结算后第四年，全部 付清）。 五、报价人资格要求 1.营业范围要求：在中华人民共和国境内依法注册、符合项目经营范围，具有询价物资生产或供应经验 的生产商或代理商，并且具有合法有效的营业执照。 2.生产能力要求：生产商须具备询价物资生产能力，生产工艺、装备必须符合国家产业发展政策的相关规定。代 理商需出具制造厂出具签字盖章的授权函。 3.质量保证能力要求：产品质量符合最新国家或行业质量标准并满足设计要求，具有近两年（2024年8 月至今）国家认可的第三方检测机构出具的报价物资达到国家标准的合格检测报告；需满足排水钢管的相关所 有要求。 4.履约信用要求：1.报价单位财产未被接管或冻结；2.报价单位不得存在的其他情形：①因存在不良行为被中国 国家铁路集团有限公司限制参与物资采购活动的；②报价物资被中国国家铁路集团有限公司禁止或暂停在铁路 上使用的；③自报价文件递交之日起前3年（2023年12月至今）企业或企业法定代表人有人民法院生效判决、裁 定认定的行贿犯罪记录的。④ 对纳入国家铁路局“黑名单”管理的单位，在公布期限内，不接受其报价；3.不接 受通过“信用中国”网站查询相关主体为失信被执行人的报价单位；4.本次询价不接受在最新一期《中国铁建合 作方警示名录》范围内，以及被采购人或其上级单位列入限制交易供应商名单的报价单位。 网 5.经评审通过的报价相同的报价人，由报价文件内企业注册资本金较多的报价人排序在前;若企业注册资本金也相 同，则由铁建云链平台询价报名响应时间在前的报价人排序在前。若报名时间也相同，则由评审小组商议并出 具一致意见以确定排序。 务 ★6.下列情形拒绝报价：铁建云链网站查询供应商关联关系，且经评审委员会评定认为属于相互串通报价的行为。 六、报价人需要提供的资料 1.营业执照复印件、法人身份证复印件、开户许可证、授商权委托书、报价表和报价人资格要求中所需的证明资料， 所有资料需加盖公司鲜章。 2.生产厂家资质，产品质量检测报告等质量证明文件。 道 ★以上资料报价单位必须对应提供，资料缺失将导致报价被拒绝。 七、询价报名截止时间 管 有意参加本次询价采购的报价人须在铁建云链平台（https://www.crccep.cn）完成供应商注册，并于2026年8月18 日9时00分至2026年8月21日9时00分在网上完成报名工作。 八、询价截止时间 国 凡有意参加本次询价采购的报价人，请于 2026年8月21日14时00分 前提交报价。截止时间前未完成报价文件传 输的，视为放弃报价。 供应商报价必须严格按照《报价表》格式进行报价。 中 九、联系方式 采购组织单位：中铁十一局集团有限公司物资设备集中采购管理中心第五分中心 地址：重庆市沙坪坝区新桥新村71号 采购人名称：中铁十一局集团有限公司宜涪高铁重庆段站前3标项目经理部 地址：重庆市石柱土家族自治县金彰工业园区C区中铁十一局项目部 联系人：罗先生 联系电话：18580400001（提供采购服务支持） 中铁十一局集团有限公司 物资设备集中采购管理中心第五分中心 2026年8月18日 报价网址：https://www.crccep.com 信息来源:https://www.chinapipe.net/project/d3074654.html cqdingjiu 2026.08.21 10:07:01 网 务 商 道 管 国 中</t>
+          <t>贡井区2026年大豆单产提升工程招标计划 项目批准文件及文号 贡发改批[2026]18号(贡发 招标项目名称 贡井区2026年大豆单产提升工程 （如有） 改批[2026]18号) 招标人 自贡市贡井区农业农村局 联系人及联系方式 陈老师:0813-3307310 估算总投资 14455000.00 项目分类 市政基础设施工程 （元） 新建、改造6处农村机电提灌站及农村机电提灌站相关设施建设，提升改善大豆灌面约30000亩; 招标项目概况 实施建设大豆种植智能滴灌系统2处，共计300亩智能滴灌示范区网，新建蓄水池23座;开展大豆单 产提升技术推广。 序号 招标内容 投标人主要资格条件要求 预计招标时间 拟招标内容 1 施工 详见招标文件 2026-09-21 00:00:00 务 备注：提前发布的招标计划内容仅供各方主体提前获知项目基本信息和拟招标内容，招标项目的实际信息以招 标人最终发布的招标公告和招标文件为准。 信息来源:https://www.chinapipe.net/project/d3077426.html 商 cqdingjiu 2026.08.24 12:31:58 道 管 国 中</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米</t>
+          <t>新建蓄水池23座；实施建设大豆种植智能滴灌系统2处，共计300亩智能滴灌示范区网。</t>
         </is>
       </c>
       <c r="N59" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>重庆, 排水钢管, 询价采购</t>
+          <t>贡井区, 2026年, 大豆单产提升工程, 智能滴灌系统, 蓄水池, 投资金额</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>中铁建设集团(重庆)建设有限公司重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热交换机组采购竞价补遗公告二</t>
+          <t>隆昌市住房和城乡建设局隆昌市城市核心区南部片区燃气配套管网改造项目焊缝探伤检测采购废标公告</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4595,29 +4691,37 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>内江市</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>隆昌市</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热交换机组采购。</t>
+          <t>隆昌市城市核心区南部片区燃气配套管网改造项目焊缝探伤检测采购</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>项目详细内容无法识别</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>冷却塔、分集水器、水板式热交换机组</t>
+          <t>焊缝探伤检测服务</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>中铁建设集团(重庆)建设有限公司重庆协同创新区供冷供热能源站及配套系统工程冷却塔、分集水器、水板式热 交换机组采购竞价补遗公告二 各 投标单位 ： 根据参加报名的潜在投标单位数量不满足招标方充分竞价要求的情况，此次重庆协同创新区供冷供热能源站及 配套系统工程冷却塔、分集水器、水板式热交换机组采购竞价资格预审报名截止日期将延期至 8月19日（周三） 上午9:00。 特此说明。 网 中铁建设集团（重庆）建设有限公司 2026年8月17日 务 信息来源:https://www.chinapipe.net/project/d3074650.html cqdingjiu 2026.08.21 10:07:01 商 道 管 国 中</t>
+          <t>隆昌市住房和城乡建设局隆昌市城市核心区南部片区燃气配套管网改造项目焊缝探伤检测采购废标公告 一、项目基本情况 采购项目编号：N5110832026000184 采购项目名称：隆昌市城市核心区南部片区燃气配套管网改造项目焊缝探伤检测采购 二、项目终止的原因 网 终止合同包：合同包1 终止原因： 务 合同包一的废标原因为：符合专业条件的供应商或者对招标文件作实质响应的供应商不足三家的；。 三、项目后续执行情况 商 合同包1:重新开展采购活动 道 四、其他补充事宜 投诉受理单位：本项目同级财政部门，即内江市隆昌市财政局 管 联系电话：0832-3911628 联系人：钟老师 国 地址：隆昌市滨江路3段64号 五、凡对本次公告内容提出询问，请按以下方式联系。 中 1.采购人信息 名称：隆昌市住房和城乡建设局 地址：四川省隆昌市金鹅街道康复东路62号 联系方式：18581037348 2.采购代理机构信息 名称：四川梦意招标代理有限公司 地址：四川省内江市隆昌市金鹅镇环城北路二段81号 联系方式：18283278039 3.项目联系方式 项目联系人：袁女士 电话：18283278039 四川梦意招标代理有限公司 2026年08月21日 信息来源:https://www.chinapipe.net/project/d3077360.html cqdingjiu 2026.08.24 12:31:59 网 务 商 道 管 国 中</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4626,18 +4730,18 @@
         </is>
       </c>
       <c r="N60" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>重庆协同创新区, 供冷供热能源站, 冷却塔, 分集水器, 水板式热交换机组, 采购竞价</t>
+          <t>隆昌市, 燃气配套管网改造, 焊缝探伤检测</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>城口县东安及河鱼片区污水管网建设项目(一期)招标计划表</t>
+          <t>华蓥市全域乡村振兴建设项目(一期)21号公路和美乡村建设项目二标段招标公告</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4647,7 +4751,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>市政</t>
+          <t>交通</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4662,53 +4766,57 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>广安市</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>城口县</t>
+          <t>华蓥市</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>在城口县东安镇新建一座污水处理站，铺设不同直径的污水管道共计29.3公里，包括dn110、dn160、dn200、DN300、DN400等规格的污水管道，以及DN200压力管道7.4公里，建设配套泵站2座和化粪池56座、隔油池32座。</t>
+          <t>对全市5万亩高标准农田进行提档升级，建设粮油园区3万亩，全域开展农村人居环境整治，打造乡村旅游聚居村落80个，配套建设乡村振兴道路、停车场和标识导视系统等旅游服务设施等。</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>合同预估金额为3400万元人民币。</t>
+          <t>项目业主为华蓥市农业农村局，建设资金来自财政资金及地方专项债券资金，项目出资比例为100%。</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>污水管网、泵站、化粪池、隔油池</t>
+          <t>市政公用工程施工</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>城口县东安及河鱼片区污水管网建设项目(一期)招标计划表 重庆市工程建设项目招标计划表 项 名 目 称城口县东安及河鱼片区污水管网建设项目（一期） 招标 法人 或招 标人城口县生态环境局 名称 （盖 网 章） 项目 批准 文件 及文 号 主 建 内 要 设 容 在 污 城 水 口 处 县 理 东 站 安 1座 镇 ， 等 改 片 建 区 后 新 设 建 计 污 规 水 模 管 20 网 0m 29 3 . / 0 d 0 。 km，其中新建dn110污水管5.80km，dn160污水管2.75km，dn200污水管0.57km，DN300污水干管4.36km，D 务 N400污水干管8.12km，DN200压力管7.4km,以及建设配套泵站2座,化粪池56座，隔油池32座。改扩建 序号 招标项目名称 招标内容 招标方式 招标文件计划发布时间 拟交易场所 合同预估金额(万元) 备注 招 项 标 目1 城 建 口 设 县 项 东 目 安 （ 及 一 河 期 鱼 ） 片区污水管网 工程施工 公开招标 2026-09 城 易 口 中 县 心 公共资源交 3400.00 本 暂 为 计 定 准 划 ， 。 表 最 所 终 列 以 招 实 标 际 项 招 目 标 信 时 息 的 均 信 为 息 备注本计划表所列招标项目信息均为暂定，最终以实际招标时的信息为准 信息来源:https://www.chinapipe.net/project/d3074602.html 商 cqdingjiu 2026.08.21 10:07:01 道 管 国 中</t>
+          <t>华蓥市全域乡村振兴建设项目(一期)21号公路和美乡村建设项目二标段招标公告 1. 招标条件 1.1本招标项目华蓥市全域乡村振兴建设项目(一期)(项目名称)已由华蓥市发展和改革局(项目审批、核 准或备案机关名称)以《华蓥市发展和改革局关于华蓥市全域乡村振兴建设项目(一期)可行性研究报告的批复》 （华发改投〔2022〕37号）（批文名称及编号）批准建设，项目业主为华蓥市农业农村局，建设资金来自财政资 金及地方专项债券资金（资金来源），项目出资比例为100%，招标人为华蓥市农业农村局。项目已具备招标条 件，现对该项目的施工进行公开招标。 网 1.2本招标项目由华蓥市发展和改革局（核准机关名称）核准（招标事项核准文号为华发改投〔2022〕37号）的招 标组织形式为委托招标（□自行招标 委托招标）。招标人选择的招标代理机构是华蓥市国晟工程项目管理咨 询有限公司。 务 2. 项目概况与招标范围 2.1标段划分：21号公路和美乡村建设项目二标段。 2.2建设地点：华蓥市古桥街道、阳和镇、红岩乡。 商 2.3建设内容及规模：对全市5万亩高标准农田进行提档升级，建设粮油园区3 万亩，全域开展农村人居环境整治， 打造乡村旅游聚居村落80个，配套建设乡村振兴道路、停车场和标识导视系统等旅游服务设施等。 道 本次实施该项目21号公路和美乡村建设项目二标段，其实施内容为：21号公路沿线人居环境整治、新建厕所（含 给排水安装工程）、新建一体化净水厂三座，配套建设供水管网，在公路沿线设置标识导视及其他配套附属设 施工程等。 管 2.4计划工期：90日历天。 2.5招标范围：本项目21号公路和美乡村建设项目二标段施工图纸及工程量清单范围内的所有工作。 （说明本次招标项目的国建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 3.1本次招标要求投标人须具备 中 3.1.1资质条件：具备国家建设行政主管部门颁发的市政公用工程施工总承包三级及以上资质。 3.1.2业绩要求： □近年（ 年 月 日至投标截止时间，不少于3年）（□已完成 □已完成或新承接或正在施工）不少 于 （1 至3个）个类似项目。类似项目是指: 。 无业绩要求。 3.1.3项目经理的资格要求： 项目经理（项目负责人）资格：市政公用工程(注册专业)二级及以上（级别）建造师，具有省级及以上住房城 乡建设主管部门颁发的安全生产考核合格证（B证）， / （业绩要求） ，须为本单位人员（若为联合体投 标，须为联合体牵头人人员）。 □园林绿化工程项目经理（项目负责人）资格： （职称级别）专业技术职称， （业绩 要求） ，须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2本次招标□接受 不接受联合体投标。联合体投标的，应满足下列要求： /。 3.3各投标人均可就上述 1 (具体数量)标段投标 。 3.4本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东为大企业、与大企业的负责 人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具体 标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的通 知》（工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除技术 复杂、存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在3000万元以下的施工项目(标段) 应勾 选此项。） 4. 招标文件的获取 4.1 凡有意参加投标者，请于2026年08月22日开始登陆：全国公共资源交易平台（四川省·广安市（州）） （网址：https://zhjy.gazhcs.com/）—“登录”—“投标登录”，通过数字证书免网费下载招标资料（招标文件、技 术资料等）。 4.2 招标人不提供招标文件获取的其他方式。 务 5. 投标文件的递交 5.1投标文件递交的截止时间（投标截止时间，下同）为2026年09月11日09时30分，投标人应在投标截止时间前在 线递交经投标人数字证书加密的数据电文形式投标文件。 商 5.2本项目开标实行（□见面开标；使用不见面开标系统）开标方式，关于“不见面开标系统”的流程和注意 事项，请各交易主体在广安市公共资源交易网上下载查看不见面开标系统操作指南。 6. 发布公告的媒介 道 本次招标公告在《全国公共资源交易平台（四川省）》和全国公共资源交易平台（四川省· 广安市）(公 告发布的其它媒介名称）上发布。 管 7.行政监督部门 单位名称：华蓥市发展和改革局 联系电话：0826-48215国39 8.联系方式 招 标 人：华蓥市农业农村局 中 地 址：四川省广安市华蓥市华翠路9号 邮 编：638600 联 系 人：赵先生 电 话：18160128811 传 真： / 电子邮件： / 网 址： / 开户银行： / 账 号： / □ 招标代理机构： / 招标代理机构：华蓥市国晟工程项目管理咨询有限公司 地 址：四川省广安市华蓥市汪杜路397号附38号 邮 编：638600 联 系 人：谭先生 项目负责人：唐玉琴 网 电 话：0826-4666655 传 真： / 务 电子邮件： / 网 址： / 商 开户银行： / 账 号： / 道 2026年08月21日 管 注： （1）若划分标段，则国填写标段序号；若划分为两个及以上标段，应分别明确各标段的具体内容、划分情况。 （2）招标人对投标人的资质要求，应是国家对投标人资质的强制性规定。不是国家规定必须具备的资质，不得 作为资质要求。 中 （3）招标人对投标人的类似项目业绩要求，设置的投资额、面积、长度等规模量化指标不得高于本次招标工程 相应指标，类似项目业绩的定义应明确，用语准确无歧义。 （4）招标人要求投标人需具备的资质一个项目（标段）为一个，因特殊情况需要两个以上资质的，应当接受投 标人组成联合体投标，且限定的联合体成员数量不得少于设定的资质个数。 信息来源:https://www.chinapipe.net/project/d3077250.html cqdingjiu 2026.08.24 12:32:02</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>dn110污水管：5.80km；dn160污水管：2.75km；dn200污水管：0.57km；DN200压力管：7.4km；泵站：2座</t>
+          <t>原文未提及</t>
         </is>
       </c>
       <c r="N61" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>重庆, 管材, 招标, 商机, 项目地区, 项目内容, 资金情况, 产品种类</t>
+          <t>乡村振兴, 公路, 农村人居环境整治, 乡村旅游</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>阀门产业园(管网改造)项目招标公告</t>
+          <t>中铁七局三公司供应链分公司金属波纹管框架询价公告</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4718,57 +4826,515 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
+          <t>其他/未识别</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>公海</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>成都市</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>温江区</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>预应力混凝土用金属波纹管</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>金属波纹管</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>中铁七局三公司供应链分公司金属波纹管框架询价公告 GYLKJ2026-050 采购单位:中铁七局集团第三工程有限公司 发布时间:2026-08-21 08:56 报价截止时间:2026-08-25 18:00 招标方联系人:杨浩 网 招标方联系电话:18829048334 招标方邮箱: 务 监督方联系人:物资部 监督方联系电话:86367038 商 监督方邮箱: 保证金:0.0元 道 结算与发票信息: 结算方式： 管 支付条件： 发票种类： 发票抬头： 国 税号： 其他要求：中 交货信息: 交货方式: 收货人: 收货人联系方式: 其他说明事项: 流水号：询2026082100043 交 计量 技术标准及 标的编号 标的名称 规格型号 数量 货 送货地址 单位 要求 期 预应力混凝土用 西南区-四川省-成都市-温江区-中 0409001000042 JBG-100Z 13365.0 米 Φ80 金属波纹管 铁七局成温邛高速项目工地 预应力混凝土用 西南区-四川省-成都市-温江区-中 0409001000042 JBG-100Z 36027.0 米 Φ90 金属波纹管 铁七局成温邛高速项目工地 预应力混凝土用 西南区-四川省-成都市-温江区-中 0409001000042 JBG-100Z 920.0 米 Φ100 金属波纹管 铁七局成温邛高速项目工地 报价网址:http://www.crecgec.com 信息来源:https://www.chinapipe.net/project/d3077249.html cqdingjiu 2026.08.24 12:32:02 网 务 商 道 管 国 中</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>13365.0米 Φ80；36027.0米 Φ90；920.0米 Φ100</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>85</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>金属波纹管, 成都</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>布拖县2026年农村生活污水治理项目施工招标公告</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>管材网线索</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
           <t>市政</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>进行中</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>公海</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>重庆市</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路长4000米，包括道路、综合管网等基础配套设施等。</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>阀门产业园(管网改造)项目招标公告 阀门产业园（管网改造）项目招标公告 1.招标条件 本招标项目 阀门产业园（管网改造）项目已由垫江县发展和改革委员会以垫江发改委发【2022】459 号（批文 名称及编号）批准建设，项目业主为 垫江县丹香建设有限公司，建设资金来自 自筹资金 （资金来源）， 项目出资比例为 100% ，招标人为 垫江县丹香建设有限公司。项目已具备招标条件，现对该项目的施工进 行公开招标，评标办法采用经评审的最低投标价法。 2.项目概况与招标范围 网 2.1 建设地点： 重庆市垫江县高新区县城组团 2.2 项目概况与建设规模： 场平面积800亩；新建厂房10000平方米，并完善相关基础配套设施等；新建道路 务 长4000米，包括道路、综合管网等基础配套设施等。 2.3 本项目工程总投资金额：55000万元 本次招标项目合同估算金额：184.669075万元 商 2.4 招标范围： 包括土石方开挖回填、砼支墩、污水管道安装、检查井砌筑、河堤修复等。具体详见施工图和 工程量清单。 道 2.5 工期要求：建设工期180日历天 缺陷责任期要求：24个月 管 2.6 标段划分（如有）： / 2.7 其他： / 3.政府采购工程 国 3.投标人资格要求 4.1 本次招标要求投标人须具备以下条件： 中 4.1.1 本次招标要求投标人具备的资质条件： 具备建设行政主管部门颁发的有效的市政公用工程施工总承包叁 级及以上资质 ； 4.1.2 投标人还应在人员、业绩、设备、资金等方面具有相应的施工能力，详见招标文件第二章投标人须知前附 表第1.4.1项内容。 4.2 本次招标 不接受联合体投标。 .技术成果经济补偿 本次招标对未中标人投标文件中的技术成果给予经济补偿。 给予经济补偿的，招标人将按如下标准支付经济补 偿费： 4.招标文件的获取 4.1本招标项目采用全流程电子招投标，投标人在投标前可在重庆市公共资源交易监督网、重庆市公共资源交易网 （垫江县）下载招标文件、工程量清单、电子图纸等资料。参与投标的投标人需在重庆市公共资源交易监督网、 重庆市公共资源交易网（垫江县）完成市场主体信息登记以及CA数字证书办理，办理方式请参见重庆市公共资 源交易监督网、重庆市公共资源交易网（垫江县）导航栏“主体信息”页面中“市场主体信息登记”、“CA 数 字证书办理”。若投标人未及时完成市场主体信息登记和CA数字证书办理导致无法完成全流程电子招投标的， 责任自负。 4.2投标人可在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）本项目招标公告网页下方“我要 提问”栏提出疑问，提问时间从本公告发布至2026-08-24 09:00:00前。 4.3招标人应于2026-08-24 23:59:59前在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布澄清。 5.投标文件递交的内容 5.1投标文件递交的截止时间（投标截止时间，下同）为2026-09-18 10:00，投标人应当在投标截止时间前，通过互 联网使用CA数字证书登录重庆市电子招投标系统，将加密的电子投标文件上传。 5.2未按要求加密的电子投标文件，将无法上传至重庆市电子招投标系统，逾期未完成投标文件上传的，视为撤 回投标文件。 6.发布公告的媒介 本次招标公告同时在重庆市公共资源交易监督网、重庆市公共资源交易网（垫江县）发布。[提示：依法必须招 标项目的招标公告，必须在重庆市公共资源交易监督网上发布。] 7.联系方式 招 标 人: 垫江县丹香建设有限公司 代理机构: 重庆博钰大数据科技有限公司 地 址: 地 址: 重庆市垫江县桂溪街道南内街88号 网 邮 编: 邮 编: 项目负责人: 熊老师 项目负责人: 郭威 电 话: 023-74630098 电 话: 023-74692498 务 传 真: 传 真: 电子邮箱: 电子邮箱: 开户银行: 开户银行: 商 账 号: 账 号: 监督部门: 垫江县发展和改革委员会 电 话: 023-74517161 道 2026年08月18日 信息来源:https://www.chinapipe.net/project/d3074578.html cqdingjiu 2026.08.21 10:07:02 管 国 中</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>公海</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>凉山彝族自治州</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>布拖县</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>新建2m³三道格化粪池584座、3m³三格化粪池1022座、20m³三格化粪池2座、30m³三格化粪池2座，配套建设入户管、支管、干管、检查井、过滤池等。</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>项目资金来自除布拖县2026年中央和省级财政常态化帮扶资金外的其他渠道，不足部分由业主多渠道筹集。</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>化粪池、管线</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>布拖县2026年农村生活污水治理项目施工招标公告 1. 招标条件 1.1 本招标项目 布拖县2026年农村生活污水治理项目 (项目名称)已由 布拖县发展和改革局 (项目审 批、核准或备案机关名称)以 布发改经信函〔2026〕24号 （批文名称及编号）批准建设 ，项目业主为 凉 山彝族自治州布拖生态环境局 ，建设资金来自 除布拖县2026年中央和省级财政常态化帮扶资金外，不足部 分由业主多渠道筹集。 （资金来源），项目出资比例为 100% ，招标人为 凉山彝族自治州布拖生态环境 局 。项目已具备招标条件，现对该项目的施工进行公开招标。 网 1.2 本招标项目由 布拖县发展和改革局 （核准机关名称）核准（招标事项核准文号为 布发改经信函 〔2026〕24号 ）的招标组织形式为 委托招标 。 招标人选择的招标代理机构是四川兴泉工程项目管理有限 公司。 务 2. 项目概况与招标范围 2.1 建设地点：布拖县俄里坪镇延务村，乐安镇若普村，商 龙潭 镇沿江村、 合井村、 四菲戈洛村 。 2.2 建设规模：主要建设标准内容为新建2m3三道格化粪池 584座、 3m3三格化粪池 1022座、 20m3三格化粪池 2座、 30m3三格化 粪池 2座。配套建设入户管、 支管、 干管、 检查井、 过滤 管 池等。 项目所有新建化粪池、 管线统一采用地理式设计方式 建设。 国 中 （说明本次招标项目的建设地点、规模及投资额、计划工期、招标范围、标段划分及标段投资额等）。 3. 投标人资格要求 3.1 本次招标要求投标人须具备 3.1.1资质条件：具备独立法人资格，具有行政主管部门颁发的市政公用工程施 工总承包三级及以上资质。 3.1.2业绩要求： 近年（ 2023年01月01日 至投标截止时间，不少于3年）已完成 不少于1（1 至3个）个类似项目。类似项目 是指:市政公用工程类施工业绩1000万元及以上。 □ 无业绩要求。 3.1.3项目经理的资格要求 项目经理（项目负责人）资格：市政公用工程二级及以上(注册专业)（级别）建造师，具有省级及以上住房 城乡建设主管部门颁发的安全生产考核合格证（B证），/（业绩要求） ，须为本单位人员（若为联合体投标， 须为联合体牵头人人员）。 □ 园林绿化工程项目经理（项目负责人）资格： （职称级别）专业技术职 称， （业绩要求） ，须为本单位人员（若为联合体投标，须为联合体牵头人人员）。 3.2 本次招标不接受 联合体投标。 3.3 各投标人均可就上述1(具体数量)标段投标 。 3.4 本次招标仅面向中小企业发包（其中属于大企业的分支机构、存在控股股东为大企业、与大企业的负责 人为同一人的情形的企业均不属于中小企业。若为联合体投标的，联合体所有单位均应属于中小企业）。具体 标准以《工业和信息化部、国家统计局、国家发展和改革委员会、财政部关于印发中小企业划型标准规定的通 知》（工信部联企业〔2011〕300号）中的“建筑业”划型标准为准，投标人应提供中小企业声明函。（除技术 复杂、存在特殊要求外，我省依法必须招标的国家投资工程，招标控制价在3000万元以下的施工项目(标段) 应勾 选此项。） 网 4. 招标文件的获取 4.1 凡有意参加投标者，请于 2026年08月20日 登录四川建设网（http://www.sccin.com/）进入“电子招标”栏目， 通过“凉山州公共资源交易平台登录入口”凭单位CFCA数字证书登录，登录并下载招标资料（招标文件、技术 务 资料等）（联系电话：028-85569858）。 4.2 招标人不提供招标文件获取的其他方式。 5. 投标文件的递交 商 投标文件递交的截止时间（投标截止时间，下同）为 2026年09月18日 09时00分 ，投标人应在投标截止时间前 在线递交经投标人数字证书加密的数据电文形式投标文件。 道 6. 发布公告的媒介 本次招标公告在《全国公共资源交易平台（四川省）》和四川建设网(公告发布的其它媒介名称）上发布。 管 7. 行政监督部门 单位名称：布拖县住房和城乡建设局 联系电话：/ 国 8. 联系方式 招 标 人：凉山彝族自治州布拖生态环境局 中 地 址：四川省布拖县平圳路15号 邮 编：615400 联 系 人：刘老师 电 话：0834-8533776 传 真：/ 电子邮件：/ 网 址：/ 开户银行：/ 账 号：/ □ 招标代理机构： / 招标代理机构：四川兴泉工程项目管理有限公司 地 址：四川省成都市天府新区华阳街道中兴上街199号 邮 编：610000 联 系 人：张旭宇 项目负责人：陈程 网 电 话：18308205888 传 真：/ 务 电子邮件：/ 网 址：/ 商 开户银行：/ 账 号：/ 道 2026年08月19日 管 注： （1）若划分标段，则填写标段序号；若划分为两个及以上标段，应分别明确各标段的具体内容、划分情况。 （2）招标人对投标人国的资质要求，应是国家对投标人资质的强制性规定。不是国家规定必须具备的资质，不得 作为资质要求。 （3）招标人对投标人的类似项目业绩要求，设置的投资额、面积、长度等规模量化指标不得高于本次招标工程 相应指标，类似项目业绩的定义应明确，用语准确无歧义。 中 （4）招标人要求投标人需具备的资质一个项目（标段）为一个，因特殊情况需要两个以上资质的，应当接受投 标人组成联合体投标，且限定的联合体成员数量不得少于设定的资质个数。 信息来源:https://www.chinapipe.net/project/d3077246.html cqdingjiu 2026.08.24 12:32:02</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2m³三道格化粪池584座、3m³三格化粪池1022座、20m³三格化粪池2座、30m³三格化粪池2座，配套建设入户管、支管、干管、检查井、过滤池等。</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>80</v>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>农村生活污水治理, 化粪池, 管线</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>凉山州·西昌市特殊教育学校学前教育教学楼改扩建项目招标计划</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>管材网线索</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>市政</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>公海</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>凉山彝族自治州</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>西昌市</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>本项目总规划用地面积为6665.90平方米，总建筑面积约10823.11平方米（其中已建建筑面积4519.92平方米，本次项目建筑面积6303.19平方米），项目总体包含新建1座地下车库及1栋学前教育教学楼和1栋大门，其中地上建筑面积4601.97平方米（学前教育教学楼和大门）；地下建筑面积1701.22平方米（包括地下车库、人防地下室、设备用房等）；改造教学楼及宿舍面积约4519.92平方米（含建筑外墙改造及消防管网改造）；绿化面积约2473.01平方米；道路及广场用地约1814.05平方米；400米室外消防给水管网、200米生活给水管网、400米室外污水管网、400米室外雨水管网、220米室外强电管网、220米室外弱电管网、1个混凝土格栅池等。</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>估算总投资35177600.00元</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>网房屋建筑工程</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>凉山州·西昌市特殊教育学校学前教育教学楼改扩建项目招标计划 西昌市发展和改革局关于凉山 州·西昌市特殊教育学校学前教 招标项目 凉山州·西昌市特殊教育学校学前教育教 项目批准文件及文号 育教学楼改扩建项目可行性研究 名称 学楼改扩建项目 （如有） 报告（代项目建议书）批复(西 发改审批〔2026〕49号) 招标人 西昌市特殊教育学校 联系人及联系方式 赵先生:0834-3223595 估算总投资 35177600.00 项目分类 网房屋建筑工程 （元） 本项目总规划用地面积为6665.90平方米，总建筑面积约10823.11平方米（其中已建建筑面积4519.92平 方米，本次项目建筑面积6303.19平方米），项目总体包含新建1座地下车库及1栋学前教育教学楼和1 栋大门，其中地上建筑面积4601.97平方米（学前教育教学楼和大门）；地下建筑面积1701.22平方米 务 招标项目 （包括地下车库、人防地下室、设备用房等）；改造教学楼及宿舍面积约4519.92平方米（含建筑外 概况 墙改造及消防管网改造）；绿化面积约2473.01平方米；道路及广场地用地约1814.05平方米；400米室 外消防给水管网、200米生活给水管网、400米室外污水管网、400米室外雨水管网、220米室外强电管 网、220米室外弱电管网、1个混凝土格栅池等。 商 拟招标内 序号 招标内容 投标人主要资格条件要求 预计招标时间 容 1 施工 详见招标文件 2026-09-21 00:00:00 备注：提前发布的招标计划内容仅供各方主体道提前获知项目基本信息和拟招标内容，招标项目的实际信息以招 标人最终发布的招标公告和招标文件为准。 信息来源:https://www.chinapipe.net/project/d3077244.html cqdingjiu 2026.08.24 12:32:02 管 国 中</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>外消防给水管网：200米；生活给水管网：400米；室外污水管网：400米；室外雨水管网：220米；米室外弱电管网：1个</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>80</v>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>凉山州, 西昌市, 特殊教育学校, 学前教育教学楼, 改扩建项目, 施工, 管材招标</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>东河(苍溪段)流域水污染治理工程招标计划</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>管材网线索</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>市政</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>公海</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>广元市</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>苍溪县</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>新建污水收集主支管网34.48km、污水入户管64.87km；对现有1座300m³/d污水处理站进行改扩建，将污水处理能力提升至500m³/d；新建污水资源化利用设施3套、视频监控系统9套、水质监测网络1套、水环境风险预警网络1套、监控平台1套；新建150m³/d污水处理站2座、200m³/d污水处理站1座、700m³/d污水处理站1座、化粪池1座、污水提升泵站11座、标志牌9块。</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>估算总投资69670300元</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>市政基础设施工程</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>东河(苍溪段)流域水污染治理工程招标计划 招标项目 东河（苍溪段）流域水污染治理工 项目批准文件及文 苍发改投资〔2026〕 号 名称 程 号 招标人 广元市苍溪生态环境局 联系人及联系方式 王老师;08395587000 估算总投资 69670300 项目分类 市政基础设施工程 （元） 新建污水收集主支管网34.48km、污水入户管64.87km；对现有1座300m3/d污水处理站进行改扩建， 招标项目 将污水处理能力提升至500m3/d；新建污水资源化利用设施3套、视网频监控系统9套、水质监测网络1 概况 套、水环境风险预警网络1套、监控平台1套；新建150m3/d污水处理站2座、200m3/d污水处理站1座、 700m3/d污水处理站1座、化粪池1座、污水提升泵站11座、标志牌9块。 序号 招标内容 预计招标时间 拟交易场所 拟招标内 务 完成本项目施工及 容 1 2026-08 苍溪县 监理等 商 备注：提前发布的招标计划内容仅供各方主体提前获知项目基本信息和拟招标内容，招标项目的实际信息以招 标人最终发布的招标公告和招标文件为准。 道 信息来源:https://www.chinapipe.net/project/d3077243.html cqdingjiu 2026.08.24 12:32:03 管 国 中</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>排水钢管 Φ200*6m：3000米；排水入户管；污水处理站；资源化利用设施；视频监控系统；水质监测网络；水环境风险预警网络；监控平台；污水处理站；化粪池；污水提升泵站；标志牌</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>80</v>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>东河(苍溪段)流域水污染治理工程, 四川, 市政基础设施工程, 污水处理站, 资源化利用设施, 视频监控系统, 水质监测网络, 水环境风险预警网络, 监控平台</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>苍溪县构溪河流域水生态保护修复工程项目招标计划</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>管材网线索</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>市政</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>公海</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>广元市</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>苍溪县</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>新建生态缓冲带23597.6m2；新建底质改良及微地形改造面积约112287m2、新建挺水植物面 招标项目概积22457.4m2、沉水植物面积56143.5m2、浮叶植物面积11228.7m2、网鱼蚌螺修复区面积44914.8m2； 新建生态沟渠1858m，新建污水收集主支管1.6km、入户管1.2km。</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>估算总投资 27726700 元</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>市政基础设施工程</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>苍溪县构溪河流域水生态保护修复工程项目招标计划 招标项目名 苍溪县构溪河流域水生态保护修复 项目批准文件及文 苍发改投资〔2026〕 64号 称 工程 号 招标人 广元市苍溪生态环境局 联系人及联系方式 王老师;08395587000 估算总投资 27726700 项目分类 市政基础设施工程 （元） 新建生态缓冲带23597.6m2；新建底质改良及微地形改造面积约112287m2、新建挺水植物面 招标项目概 积22457.4m2、沉水植物面积56143.5m2、浮叶植物面积11228.7m2、网鱼蚌螺修复区面积44914.8m2； 况 新建生态沟渠1858m，新建污水收集主支管1.6km、入户管1.2km。 序号 招标内容 预计招标时间 拟交易场所 完成本项目施工及 1 2026-08 务市辖区 拟招标内容 监理等 本项目施工及监理 2 2026-08 市辖区 等 商 备注：提前发布的招标计划内容仅供各方主体提前获知项目基本信息和拟招标内容，招标项目的实际信息以招 标人最终发布的招标公告和招标文件为准。 道 信息来源:https://www.chinapipe.net/project/d3077240.html cqdingjiu 2026.08.24 12:32:03 管 国 中</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>排水钢管 Φ200*6m：3000米</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>80</v>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>苍溪县, 构溪河流域, 水生态保护修复, 市政基础设施工程</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>开江县2026年大豆单产提升工程项目招标计划</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>管材网线索</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>其他/未识别</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>公海</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>达州市</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>开江县</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>建设大豆单产提升工程示范区3万亩，其中核心区-水肥一体化滴网灌工程1750亩、辐射区-水源工程28250亩。</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>估算总投资14500000元</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>大豆单产提升工程</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>开江县2026年大豆单产提升工程项目招标计划 招标项目名 项目批准文件及 开江县2026年大豆单产提升工程项目 达市农[2026]25号 称 文号（如有） 联系人及联系方 招标人 开江县农业农村局 唐老师；17748170115 式 估算总投资 14500000 项目分类 农业综合 （元） 建设大豆单产提升工程示范区3万亩，其中核心区-水肥一体化滴网灌工程1750亩、辐射区-水源工 招标项目概 程28250亩。项目规划建设大豆3万亩单产提升工程。涵盖“基础设施+智慧农业+技术集成”三大 况 板块。具体招标内容以招标文件为主。 序号 招标内容 投标人主要资格条件要求 预计招标时间 拟招标内容 务 1 施工、设备等 以最终发布的招标文件为准 2026-09-21 备注：提前发布的招标计划内容仅供各方主体提前获知项目基本信息和拟招标内容，招标项目的实际信息以招 标人最终发布的招标公告和招标文件为准。 信息来源:https://www.chinapipe.net/project/d3077175.html 商 cqdingjiu 2026.08.24 12:32:03 道 管 国 中</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
         <is>
           <t>原文未提及</t>
         </is>
       </c>
-      <c r="N62" t="n">
-        <v>90</v>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>重庆, 管网改造, 投资金额, 产品种类</t>
+      <c r="N67" t="n">
+        <v>80</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>开江县, 2026年, 大豆单产提升工程, 招标计划, 四川, 管材</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>中国铁路成都局集团有限公司成铁总承包公司隆昌市石盘滩大型灌区提升改造项目管道下穿成渝铁路、成渝高铁项目钢筋混凝土管采购流标公告</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>管材网线索</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>公海</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>四川省</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>内江市</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>隆昌市</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>钢筋混凝土管采购</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>钢筋混凝土管</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>中国铁路成都局集团有限公司成铁总承包公司隆昌市石盘滩大型灌区提升改造项目管道下穿成渝铁路、成渝高 铁项目钢筋混凝土管采购流标公告 一、项目名称：隆昌市石盘滩大型灌区提升改造项目管道下穿成渝铁路、成渝高铁工程钢筋混凝土管采购（编 号：WZ 2026-057） 二、公告发布日期：2026年8月18日 三、报名截止时间：2026年8月20日 网 四、拟开标时间：2026年8月27日9：30 五、流标原因：报名采购申请人数少于3家，采购流标。 务 六、联系人：刘老师，联系电话：18349359223。 特此公告！ 商 道 采购人名称：成都铁路工程总承包有限责任公司 日期：2026年8月21日 管 信息来源:https://www.chinapipe.net/project/d3077107.html cqdingjiu 2026.08.24 12:32:03 国 中</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>原文未提及</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>80</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>重庆, 四川, 管材招标, 商机</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish detail URLs in product usage column
</commit_message>
<xml_diff>
--- a/site/matches-positive.xlsx
+++ b/site/matches-positive.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078437.html</t>
         </is>
       </c>
       <c r="N2" t="n">
@@ -619,7 +619,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>管材4802米；预制构件247个</t>
+          <t>https://www.chinapipe.net/project/d3078389.html</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078567.html</t>
         </is>
       </c>
       <c r="N4" t="n">
@@ -753,7 +753,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>排水材料</t>
+          <t>https://www.chinapipe.net/project/d3078467.html</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078339.html</t>
         </is>
       </c>
       <c r="N6" t="n">
@@ -887,7 +887,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078338.html</t>
         </is>
       </c>
       <c r="N7" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>抗旱供水；新建节水灌溉提灌站21座；整治山坪塘44口；建设水肥一体化系统；完善田间引水渠堰、排水沟及管网；安装智能监控、气象、虫情、土壤墒情系统</t>
+          <t>https://www.chinapipe.net/project/d3078219.html</t>
         </is>
       </c>
       <c r="N8" t="n">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>抗旱供水；新建节水灌溉提灌站21座；整治山坪塘44口；建设水肥一体化系统；完善田间引水渠堰、排水沟及管网；分片区安装智能监控、气象、虫情、土壤墒情系统</t>
+          <t>https://www.chinapipe.net/project/d3078218.html</t>
         </is>
       </c>
       <c r="N9" t="n">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米</t>
+          <t>https://www.chinapipe.net/project/d3078217.html</t>
         </is>
       </c>
       <c r="N10" t="n">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米</t>
+          <t>https://www.chinapipe.net/project/d3078214.html</t>
         </is>
       </c>
       <c r="N11" t="n">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>DN40(PN10)个 200; DN40(PN16)个 10; DN50(PN10)个 500; DN50(PN16)个 10; DN80(PN10)个 200; DN80(PN16)个 10; DN100(PN10)个 10; DN100(PN16)个 10; DN150(PN10)个 10; DN150(PN16)个 10; DN150(PN25)个 10; DN200(PN10)个 10; DN200(PN16)个 10; DN300(PN16)个 10; DN40个 100; DN40(25KG)个 10; DN40(16kg)个 10; DN50个 100; DN50(16kg)个 10; DN50(25KG)个 10; DN80个 100; DN80(16KG)个 10; DN80(25KG)个 10; DN100个 10; DN100(16KG)个 10; DN100(25KG)个 10; DN150个 10; DN150(16kg)个 10; DN150(25KG)个 10; DN200个 10; DN200(16kg)个 10; DN200(25KG)个 10</t>
+          <t>https://www.chinapipe.net/project/d3078192.html</t>
         </is>
       </c>
       <c r="N12" t="n">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米</t>
+          <t>https://www.chinapipe.net/project/d3078130.html</t>
         </is>
       </c>
       <c r="N13" t="n">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078119.html</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>净水厂设备及配件；配水管网及配件；一体化供水泵站设备及配件；原水管</t>
+          <t>https://www.chinapipe.net/project/d3078105.html</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078035.html</t>
         </is>
       </c>
       <c r="N16" t="n">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>更换居民气表约11700只、居民灶前自闭阀约112717只、燃气连接用不锈钢波纹软管约112717根；更新改造庭院埋地燃气管网约6913m，更新改造燃气立管及表后管道约9419户，更新切断阀约489套等。</t>
+          <t>https://www.chinapipe.net/project/d3077961.html</t>
         </is>
       </c>
       <c r="N17" t="n">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>梯台修筑127.5亩，梯田修筑61.56亩，稻虾地块修筑128.83亩，恢复地类整治1.22亩；新建Φ160PE输水管道1949米，C25混凝土排水沟（0.5m*0.6m）320米；改建3.0m宽C25混凝土机耕道905米。</t>
+          <t>https://www.chinapipe.net/project/d3077954.html</t>
         </is>
       </c>
       <c r="N18" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>智能燃气系统设备1018台(套)，居民立管务更换6443户，户外切断阀1500个，智能家用报警器5000套，户外表箱更换11024个，调压箱更换1025台，标志桩(砖)10000块。</t>
+          <t>https://www.chinapipe.net/project/d3077935.html</t>
         </is>
       </c>
       <c r="N19" t="n">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077891.html</t>
         </is>
       </c>
       <c r="N20" t="n">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077886.html</t>
         </is>
       </c>
       <c r="N21" t="n">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>全面检测总工期：40个工作日。</t>
+          <t>https://www.chinapipe.net/project/d3077867.html</t>
         </is>
       </c>
       <c r="N22" t="n">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>排水钢管 DN150: 8.1千米；DN200: 29.3千米；DN250: 23千米；DN300: 5.1千米；DN400: 11.9千米；DN500: 6.8千米，材质为3PE防腐内热熔防腐钢管</t>
+          <t>https://www.chinapipe.net/project/d3077724.html</t>
         </is>
       </c>
       <c r="N23" t="n">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>DN15 1.6MPa 件 带压力表；含不锈钢螺栓</t>
+          <t>https://www.chinapipe.net/project/d3077649.html</t>
         </is>
       </c>
       <c r="N24" t="n">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>铺设原水输水管网总长度约16.7公里，配套建设新城供水主管约77km</t>
+          <t>https://www.chinapipe.net/project/d3077567.html</t>
         </is>
       </c>
       <c r="N25" t="n">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>DN300-DN600排水管网约2.0公里；修复DN300-DN1000管道约28.98公里</t>
+          <t>https://www.chinapipe.net/project/d3077506.html</t>
         </is>
       </c>
       <c r="N26" t="n">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>排水管网修复</t>
+          <t>https://www.chinapipe.net/project/d3077435.html</t>
         </is>
       </c>
       <c r="N27" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>孝子溪水库引水管道：17.5km；其中需新建引水隧洞内置管道：1.5km；柑橘基地管网：3.25km</t>
+          <t>https://www.chinapipe.net/project/d3078207.html</t>
         </is>
       </c>
       <c r="N28" t="n">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米</t>
+          <t>https://www.chinapipe.net/project/d3077140.html</t>
         </is>
       </c>
       <c r="N29" t="n">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>袖阀管承压不小于5MPa，单节接头处带连接丝扣(配相应连接头)，间距50cm打孔缠橡胶带，另配堵头。</t>
+          <t>https://www.chinapipe.net/project/d3077066.html</t>
         </is>
       </c>
       <c r="N30" t="n">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>DN125米：840米；DN180米：840米；DN125个：140个；DN180个：140个</t>
+          <t>https://www.chinapipe.net/project/d3078608.html</t>
         </is>
       </c>
       <c r="N31" t="n">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078483.html</t>
         </is>
       </c>
       <c r="N32" t="n">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078430.html</t>
         </is>
       </c>
       <c r="N33" t="n">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>FRPP管Φ160PN1.0*13.3-黑色: 80米, FRPP弯头(90°)Φ160PN1.0*13.3-R=1.5D-黑色: 8个</t>
+          <t>https://www.chinapipe.net/project/d3078468.html</t>
         </is>
       </c>
       <c r="N34" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>DN300*50mm，含胶圈：1100.00m；DN500*55mm，含胶圈：1500.00m；DN600*60mm，含胶圈：1000.00m；DN800*80mm，含胶圈：1100.00m；DN1000*100mm，含胶圈：350.00m；DN1200*120mm，含胶圈：200.00m；C30,D800*140mm，含爬梯：100.00m；C30,D1000*140mm，含爬梯：100.00m；C30,D1200*140mm，含爬梯：100.00m；C30,D1500*150mm，含爬梯：100.00m；C30,D1800*180mm，含爬梯：100.00m；C30,D800*140mm，含爬梯，含140mm厚底座：100.00m；C30,D1000*140mm，含爬梯，含140mm厚底座：100.00m；C30,D1200*140mm，含爬梯，含140mm厚底座：100.00m；C30,D1500*150mm，含爬梯，含150mm厚底座：100.00m；C30,D1800*180mm，含爬梯，含180mm厚底座：100.00m；C30,D800*120mm，含爬梯：400.00m；φ1280变800，厚度140mm，含吊钩：100.00个；φ1480变800，厚度140mm，含吊钩：100.00个；φ1800变800，厚度160mm，含吊钩：100.00个；φ2160变800，厚度200mm，含吊钩：100.00个；700*400*800mm*70mm厚度：180.00个；1560*400*800mm*70mm厚度：100.00个；1700*1100*160mm：10.00m；1700*1700*160mm：4.00m；2100*1800*220mm：6.00m；2400*2000*220mm：4.00m</t>
+          <t>https://www.chinapipe.net/project/d3078565.html</t>
         </is>
       </c>
       <c r="N35" t="n">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>用于地面集输工程的建设</t>
+          <t>https://www.chinapipe.net/project/d3078290.html</t>
         </is>
       </c>
       <c r="N36" t="n">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object],[object Object]</t>
+          <t>https://www.chinapipe.net/project/d3078197.html</t>
         </is>
       </c>
       <c r="N37" t="n">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078163.html</t>
         </is>
       </c>
       <c r="N38" t="n">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3078145.html</t>
         </is>
       </c>
       <c r="N39" t="n">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077945.html</t>
         </is>
       </c>
       <c r="N40" t="n">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077864.html</t>
         </is>
       </c>
       <c r="N41" t="n">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>西部水厂管廊管道及加压站部分管道防腐 500㎡，钢制设施、设备防腐 6100㎡，高新区景苑小区管道防腐 55㎡，长葫引水管道DN1200钢管防腐 1380㎡，一桥硬合厂宿舍侧DN400钢管防腐 16.5㎡，一桥硬合厂宿舍侧DN300钢管防腐 14.15㎡</t>
+          <t>https://www.chinapipe.net/project/d3077586.html</t>
         </is>
       </c>
       <c r="N42" t="n">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077563.html</t>
         </is>
       </c>
       <c r="N43" t="n">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>雨污排水管网：10千米；弱电管网：5千米</t>
+          <t>https://www.chinapipe.net/project/d3077560.html</t>
         </is>
       </c>
       <c r="N44" t="n">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077557.html</t>
         </is>
       </c>
       <c r="N45" t="n">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077552.html</t>
         </is>
       </c>
       <c r="N46" t="n">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>排水和雨水排放</t>
+          <t>https://www.chinapipe.net/project/d3077551.html</t>
         </is>
       </c>
       <c r="N47" t="n">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>排水主管网 Φ300~Φ800mm 约2.08km；雨水管网 Φ300~Φ800mm 约0.88km；污水管网 Φ300~Φ800mm 约1.2km；现状管道清淤疏通长度约1.23km；配套建设检查井等附属构筑物；路面恢复提升材料，车行道改造面积约9188平方米，人行道改造约3295平方米。</t>
+          <t>https://www.chinapipe.net/project/d3077550.html</t>
         </is>
       </c>
       <c r="N48" t="n">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077548.html</t>
         </is>
       </c>
       <c r="N49" t="n">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077502.html</t>
         </is>
       </c>
       <c r="N50" t="n">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>宜宾高新区高场片区老旧小区改造项目：改造小区燃气管道17160m，给排水管道18935m，电力和通信线路13320m，改造停车位685个；新增充电桩137个，小区消防设施58套，户内燃气安全设施1956套，分类垃圾回收站点10个；改造闲置社区用房为日间照料中心4430m、便民中心5420m，改造小区内道路10192m及配套基础设施。宜宾高新区高场片区城中村配套基础设施项目：新建公共配套用房总建筑面积21000m，其中养老托幼等服务设施15000m、其他公服用房6000m；新建公共停车位1600个及配置400个充电桩；新改建城中村配套道路约4.5km及其他基础设施建设。</t>
+          <t>https://www.chinapipe.net/project/d3077494.html</t>
         </is>
       </c>
       <c r="N51" t="n">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>D219X6 米 3600; D159X6 米 200; D133X4 米 100; D108X4 米 200; D89X4 米 60; D76X3.5 米 120; D57X3.5 米 120; D45X3 米 18; D38X管3 米 90; D32X3 米 400; DN100 米 900; DN65 米 300; DN50 米 1000; 80*8 m 1438; 40*6 m 6675; 50*50*5 m 2672; 75*5 m 170; 10# m 790; DN25 m 1133; DN40 m 87; DN50 m 1083; DN100 m 130; D159*6 m 100</t>
+          <t>https://www.chinapipe.net/project/d3077488.html</t>
         </is>
       </c>
       <c r="N52" t="n">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077474.html</t>
         </is>
       </c>
       <c r="N53" t="n">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077437.html</t>
         </is>
       </c>
       <c r="N54" t="n">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>滴灌(喷灌)灌区设备、机井、提灌站、蓄水池、渠道整治设备、智能灌溉机器人（车）</t>
+          <t>https://www.chinapipe.net/project/d3077434.html</t>
         </is>
       </c>
       <c r="N55" t="n">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米</t>
+          <t>https://www.chinapipe.net/project/d3077433.html</t>
         </is>
       </c>
       <c r="N56" t="n">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>排水边沟 B*H=600*800 2238m; 排洪沟 B*H=1500*2000 1306道m, B*H=2000*1500 120m, B*H=2500*3000 450m, B*H=3500*4000 2800m, B*H=5000*4000 2845m, B*H=6000*4000 545m; 排洪沟清淤 18484m; 排洪涵清淤 2500m; 雨水调蓄池 8000t/d 和 1000t/d</t>
+          <t>https://www.chinapipe.net/project/d3077430.html</t>
         </is>
       </c>
       <c r="N57" t="n">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Φ40/33黑色白色1x4；Φ40/33黑色黄色1x4；Φ40/33黑色蓝色1x4；Φ40/33黑色绿色1x4；Φ40/33黑色红色1x4；Φ40/33黑色国紫色1x4；Φ40/33黑色白色2x3；Φ40/33黑色黄色2x3；Φ40/33黑色蓝色2x3；Φ40/33黑色绿色2x3；Φ40/33黑色红色2x3；Φ40/33黑色紫色2x3；Φ40/33黑色白色3x2；Φ40/33黑色黄色3x2；Φ40/33黑色蓝色3x2；Φ40/33黑色绿色3x2；Φ40/33黑色红色3x2</t>
+          <t>https://www.chinapipe.net/project/d3077384.html</t>
         </is>
       </c>
       <c r="N58" t="n">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>新建蓄水池23座；实施建设大豆种植智能滴灌系统2处，共计300亩智能滴灌示范区网。</t>
+          <t>https://www.chinapipe.net/project/d3077426.html</t>
         </is>
       </c>
       <c r="N59" t="n">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077360.html</t>
         </is>
       </c>
       <c r="N60" t="n">
@@ -4801,7 +4801,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077250.html</t>
         </is>
       </c>
       <c r="N61" t="n">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>13365.0米 Φ80；36027.0米 Φ90；920.0米 Φ100</t>
+          <t>https://www.chinapipe.net/project/d3077249.html</t>
         </is>
       </c>
       <c r="N62" t="n">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>2m³三道格化粪池584座、3m³三格化粪池1022座、20m³三格化粪池2座、30m³三格化粪池2座，配套建设入户管、支管、干管、检查井、过滤池等。</t>
+          <t>https://www.chinapipe.net/project/d3077246.html</t>
         </is>
       </c>
       <c r="N63" t="n">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>外消防给水管网：200米；生活给水管网：400米；室外污水管网：400米；室外雨水管网：220米；米室外弱电管网：1个</t>
+          <t>https://www.chinapipe.net/project/d3077244.html</t>
         </is>
       </c>
       <c r="N64" t="n">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米；排水入户管；污水处理站；资源化利用设施；视频监控系统；水质监测网络；水环境风险预警网络；监控平台；污水处理站；化粪池；污水提升泵站；标志牌</t>
+          <t>https://www.chinapipe.net/project/d3077243.html</t>
         </is>
       </c>
       <c r="N65" t="n">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>排水钢管 Φ200*6m：3000米</t>
+          <t>https://www.chinapipe.net/project/d3077240.html</t>
         </is>
       </c>
       <c r="N66" t="n">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077175.html</t>
         </is>
       </c>
       <c r="N67" t="n">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>原文未提及</t>
+          <t>https://www.chinapipe.net/project/d3077107.html</t>
         </is>
       </c>
       <c r="N68" t="n">

</xml_diff>

<commit_message>
Publish project content and detail URLs in product usage
</commit_message>
<xml_diff>
--- a/site/matches-positive.xlsx
+++ b/site/matches-positive.xlsx
@@ -552,7 +552,8 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078437.html</t>
+          <t>包括雨水检查井、钢筋砼承插式雨水管道铺设、中粗砂回填等内容
+https://www.chinapipe.net/project/d3078437.html</t>
         </is>
       </c>
       <c r="N2" t="n">
@@ -619,7 +620,8 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078389.html</t>
+          <t>中建五局第三建设有限公司鑫旭达西南地区生产基地项目室外管材及预制构件采购
+https://www.chinapipe.net/project/d3078389.html</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -686,7 +688,8 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078567.html</t>
+          <t>西部（重庆）科学城德感片区污水管网修复完善工程项目所需（白沙部分新增）市政工程专业分包工程，包括非开挖紫外光修复、安装前道内部勘测、清淤、封堵气囊、导排水，钢内衬成环回顶，铺设防划垫膜，主物料的拉入、连接充气设备、安装排水软管、物料的充气/紫外光固化、冷却物料、切除管口扎头多余务、抽出内膜、CCTV检测验收、拆除堵通水修复，管道铺设、管件、检查井、完成建筑垃圾清理，路面恢复等主要工序和辅助工序。
+https://www.chinapipe.net/project/d3078567.html</t>
         </is>
       </c>
       <c r="N4" t="n">
@@ -753,7 +756,8 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078467.html</t>
+          <t>本项目涉及采购钢带增强聚乙烯螺旋波纹管和钢带波纹管密封胶圈，用于重庆高速巨能建设集团有限公司城开高速城开隧道泄水洞施工项目。
+https://www.chinapipe.net/project/d3078467.html</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -820,7 +824,8 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078339.html</t>
+          <t>采购项目名称为物资，具体采购内容包括第十四次物资区域联合授权公开谈判采购。
+https://www.chinapipe.net/project/d3078339.html</t>
         </is>
       </c>
       <c r="N6" t="n">
@@ -887,7 +892,8 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078338.html</t>
+          <t>采购项目名称为'国网重庆电力主城一片区2026年原集体企业和各级产业单位第十四次物资区域联合授权公开谈判采购'，采购类型为物资。
+https://www.chinapipe.net/project/d3078338.html</t>
         </is>
       </c>
       <c r="N7" t="n">
@@ -958,7 +964,8 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078219.html</t>
+          <t>本工程为9720亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站21座，整治山坪塘44口，建设主要建设水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤墒情系统。
+https://www.chinapipe.net/project/d3078219.html</t>
         </is>
       </c>
       <c r="N8" t="n">
@@ -1029,7 +1036,8 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078218.html</t>
+          <t>本工程为9720亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站21座，整治山坪塘44口，建设主要建设水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤墒情系统。
+https://www.chinapipe.net/project/d3078218.html</t>
         </is>
       </c>
       <c r="N9" t="n">
@@ -1100,7 +1108,8 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078217.html</t>
+          <t>本工程为1.7万亩柑橘等特色农业提供抗旱供水，新建节水灌溉提灌站18座，整治山坪塘28口，建设水肥一体化系统，完善田间引水渠堰、排水沟及管网，分片区安装智能监控、气象、虫情、土壤墒情系统。
+https://www.chinapipe.net/project/d3078217.html</t>
         </is>
       </c>
       <c r="N10" t="n">
@@ -1171,7 +1180,8 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078214.html</t>
+          <t>新建高标准农田797.11亩，改造提升高标准农田5710.6亩，其中高效节水灌溉面积3007亩。主要内容包括水田整治、缓坡整治、梯台整治、恢复地类整治、耕地复耕整治、农机进出通道修建、提灌站修建、输水管道铺设、排水沟改建、田间道路改建等。
+https://www.chinapipe.net/project/d3078214.html</t>
         </is>
       </c>
       <c r="N11" t="n">
@@ -1238,7 +1248,8 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078192.html</t>
+          <t>重庆中法供水2026年金属补偿器及柔性橡胶接头采购项目(第三次)比选公告
+https://www.chinapipe.net/project/d3078192.html</t>
         </is>
       </c>
       <c r="N12" t="n">
@@ -1305,7 +1316,8 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078130.html</t>
+          <t>新建两岔水库取水浮船1座，设计取水规模为2万m/d；新建两岔水库取水浮船-坛高水厂原输水管道21km。
+https://www.chinapipe.net/project/d3078130.html</t>
         </is>
       </c>
       <c r="N13" t="n">
@@ -1376,7 +1388,8 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078119.html</t>
+          <t>农村供水提质改造项目
+https://www.chinapipe.net/project/d3078119.html</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1447,7 +1460,8 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078105.html</t>
+          <t>新建供水规模10000立方米/天的净水厂1座，厂外配水主干管网长度约40公里，村镇配水支线管网长度约100公里，配套一体化供水泵站共15座，新增原水管约1公里。
+https://www.chinapipe.net/project/d3078105.html</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -1518,7 +1532,8 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078035.html</t>
+          <t>重庆涪陵电力实业股份有限公司2026年第4批物资公开谈判采购
+https://www.chinapipe.net/project/d3078035.html</t>
         </is>
       </c>
       <c r="N16" t="n">
@@ -1589,7 +1604,8 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077961.html</t>
+          <t>大渡口区2024年居民户内燃气安全设施整改项目（二期）更换居民气表约11700只、居民灶前自闭阀约112717只、燃气连接用不锈钢波纹软管约112717根。大渡口区2024年城市燃气管道等老化更新改造项目（二期）更新改造庭院埋地燃气管网约6913m，更新改造燃气立管及表后管道约9419户，更新切断阀约489套等，并配套实施管网开挖回填、路面恢复、绿化恢复等。
+https://www.chinapipe.net/project/d3077961.html</t>
         </is>
       </c>
       <c r="N17" t="n">
@@ -1660,7 +1676,8 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077954.html</t>
+          <t>改造提升高标准农田326.59亩，其中高效节水灌溉面积130亩。主要内容包括梯台修筑、梯田修筑、稻虾地块修筑、恢复地类整治、输水管道安装、排水沟修建、机耕道改建等。
+https://www.chinapipe.net/project/d3077954.html</t>
         </is>
       </c>
       <c r="N18" t="n">
@@ -1731,7 +1748,8 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077935.html</t>
+          <t>大渡口区燃气管线及燃气相关设施设备改造提升，实现燃气管线智能化管理和保障燃气供给安全。
+https://www.chinapipe.net/project/d3077935.html</t>
         </is>
       </c>
       <c r="N19" t="n">
@@ -1798,7 +1816,8 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077891.html</t>
+          <t>管网工程、土石方工程等。
+https://www.chinapipe.net/project/d3077891.html</t>
         </is>
       </c>
       <c r="N20" t="n">
@@ -1869,7 +1888,8 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077886.html</t>
+          <t>李市镇农村饮水管网改建工程
+https://www.chinapipe.net/project/d3077886.html</t>
         </is>
       </c>
       <c r="N21" t="n">
@@ -1940,7 +1960,8 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077867.html</t>
+          <t>长安工业渝北工厂供水管网泄露检测及修复询比采购
+https://www.chinapipe.net/project/d3077867.html</t>
         </is>
       </c>
       <c r="N22" t="n">
@@ -2011,7 +2032,8 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077724.html</t>
+          <t>该项目对百安坝等3个街道老旧市政供水管道及附属设施进行改造，配套智慧水务物联网感知设备建设，共计改造老旧市政供水管道84.2千米。
+https://www.chinapipe.net/project/d3077724.html</t>
         </is>
       </c>
       <c r="N23" t="n">
@@ -2078,7 +2100,8 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077649.html</t>
+          <t>为重庆分质供水有限公司提供不锈钢闸阀、不锈钢表前阀、不锈钢减压阀、不锈钢排气阀、不锈钢止回阀等设备材料。
+https://www.chinapipe.net/project/d3077649.html</t>
         </is>
       </c>
       <c r="N24" t="n">
@@ -2149,7 +2172,8 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077567.html</t>
+          <t>酉阳县桃花源新城供水工程管网安装工程专业分包
+https://www.chinapipe.net/project/d3077567.html</t>
         </is>
       </c>
       <c r="N25" t="n">
@@ -2220,7 +2244,8 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077506.html</t>
+          <t>本项目改建及修复管网总长度约30.98公里，雨污水错混接改造以及管网缺失改造DN300-DN600排水管网约2.0公里；修复DN300-DN1000管道约28.98公里。
+https://www.chinapipe.net/project/d3077506.html</t>
         </is>
       </c>
       <c r="N26" t="n">
@@ -2287,7 +2312,8 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077435.html</t>
+          <t>本项目改建及修复管网总长度约30.63公里，雨污水错混接改造以及管网缺失改造DN300-DN800排水管网约6.35公里；修复DN300-DN1200管道约24.28公里。
+https://www.chinapipe.net/project/d3077435.html</t>
         </is>
       </c>
       <c r="N27" t="n">
@@ -2358,7 +2384,8 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078207.html</t>
+          <t>主要整治孝子溪大堰水渠约17.5km;新建孝子溪水库引水管道约17.5km,其中需新建引水隧洞内置管道约1.5km;新建柑橘基地管网约3.25km;改建6000m蓄水池1座；新建2000m蓄水池2座；新建1000m蓄水池1座；新建500m³蓄水池2座；新建柑橘基地滴灌系统1套。
+https://www.chinapipe.net/project/d3078207.html</t>
         </is>
       </c>
       <c r="N28" t="n">
@@ -2429,7 +2456,8 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077140.html</t>
+          <t>涪陵区李渡新区水厂工程(一期)设计水量目标为10万m/d，二期水量目标为20万m/d，采用混凝、沉淀、过滤、消毒常规水处理工艺。一期工程项目主要建设内容包括取水及原水输送工程、净水厂工程、配水工程三部分。
+https://www.chinapipe.net/project/d3077140.html</t>
         </is>
       </c>
       <c r="N29" t="n">
@@ -2500,7 +2528,8 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077066.html</t>
+          <t>新建重庆至黔江铁路重庆站站房及配套综合交通枢纽工程CQZSG-2标段项目经理部管材询比采购
+https://www.chinapipe.net/project/d3077066.html</t>
         </is>
       </c>
       <c r="N30" t="n">
@@ -2575,7 +2604,8 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078608.html</t>
+          <t>本次计划对过轨管材料进行询价，询价内容包括DN125米、DN180米、DN125个、DN180个四种过轨管及其接头。
+https://www.chinapipe.net/project/d3078608.html</t>
         </is>
       </c>
       <c r="N31" t="n">
@@ -2650,7 +2680,8 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078483.html</t>
+          <t>法兰及其垫片,沟槽管件,铸铁管件,阀门,检查口,铜制管件,管道用材,套管,补偿器及软接头,过滤器,塑料管件,复合管件,不锈钢管件,钢制管件,阻火器,水箱,其它管件及管道用器材,铝合金管件,玻璃钢管件
+https://www.chinapipe.net/project/d3078483.html</t>
         </is>
       </c>
       <c r="N32" t="n">
@@ -2725,7 +2756,8 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078430.html</t>
+          <t>本项目比选人为成都市中兴供水有限公司，主要从事市政基础设施、城市供水管网的投资、建设与运营。根据公司业务范围及建设需求，现面向社会进行给水管网施工单位的公开比选，邀请有能力的优秀比选申请人参加我公司的项目比选，并选出二至三家优秀企业共同承担2026年及2028年度成都市中兴供水有限公司供水区域内给水管网的施工任务。
+https://www.chinapipe.net/project/d3078430.html</t>
         </is>
       </c>
       <c r="N33" t="n">
@@ -2792,7 +2824,8 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078468.html</t>
+          <t>北部基地平原公司关于FRPP管Φ160及配套弯头项目采购公告
+https://www.chinapipe.net/project/d3078468.html</t>
         </is>
       </c>
       <c r="N34" t="n">
@@ -2859,7 +2892,8 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078565.html</t>
+          <t>水泥制品
+https://www.chinapipe.net/project/d3078565.html</t>
         </is>
       </c>
       <c r="N35" t="n">
@@ -2926,7 +2960,8 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078290.html</t>
+          <t>金浅26井地面集输工程包括井口模块、除砂器橇、三相分离器橇、密闭装油橇、凝析油罐模块、气田水罐模块、放空分液罐模块、放空模块、出站模块等配套工程。
+https://www.chinapipe.net/project/d3078290.html</t>
         </is>
       </c>
       <c r="N36" t="n">
@@ -3001,7 +3036,8 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078197.html</t>
+          <t>四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005询比采购公告 四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005询比采购公告 四川油建国家石油天然气大流量计量站成都分站高压检定能力建设工程防腐材料JLZ-005已具备采购条件，现公开邀请供应商参加询比采购活动。
+https://www.chinapipe.net/project/d3078197.html</t>
         </is>
       </c>
       <c r="N37" t="n">
@@ -3076,7 +3112,8 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078163.html</t>
+          <t>详细勘察服务
+https://www.chinapipe.net/project/d3078163.html</t>
         </is>
       </c>
       <c r="N38" t="n">
@@ -3151,7 +3188,8 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3078145.html</t>
+          <t>蒸汽管道改造
+https://www.chinapipe.net/project/d3078145.html</t>
         </is>
       </c>
       <c r="N39" t="n">
@@ -3226,7 +3264,8 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077945.html</t>
+          <t>管道直饮水入户项目的建设内容包括设计及施工总承包。
+https://www.chinapipe.net/project/d3077945.html</t>
         </is>
       </c>
       <c r="N40" t="n">
@@ -3301,7 +3340,8 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077864.html</t>
+          <t>西充县太平水厂、鹤鸣庵水厂及配套管网建设项目劳务分包
+https://www.chinapipe.net/project/d3077864.html</t>
         </is>
       </c>
       <c r="N41" t="n">
@@ -3376,7 +3416,8 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077586.html</t>
+          <t>钢管及设施防腐
+https://www.chinapipe.net/project/d3077586.html</t>
         </is>
       </c>
       <c r="N42" t="n">
@@ -3451,7 +3492,8 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077563.html</t>
+          <t>本项目包括新建及改建高标准农田，涉及田块整治工程、灌溉排水工程、田间道路工程、土壤改良、农田输配电工程、农田防护与生态保护工程。
+https://www.chinapipe.net/project/d3077563.html</t>
         </is>
       </c>
       <c r="N43" t="n">
@@ -3526,7 +3568,8 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077560.html</t>
+          <t>对盐边县城北、清源片区老旧街区进行商提升改造，包括改造中环北路、西环北路、清河西路、盐中巷外立面排危改造约12.28万平方米，街区路面整治约12000平方米，街区雨污排水管网改造约10千米，改造适老化、适儿化服务用房约5000平方米，社区综合服务生活市场改造8500平方米，街区屋面防水改造约9900平方米，改造3500平方米街区边角地配套停车场及充电桩等基础设施，增设路灯280盏，公共活动健身区15处，街角口袋公园4处，改造清河西路、盐中巷街区安道全防护栏5公里，街区架空线入地4千米，弱电管网整治5千米，并同步完善消防、安防、垃圾收储、便民生活设施等配套公共服务设施。
+https://www.chinapipe.net/project/d3077560.html</t>
         </is>
       </c>
       <c r="N44" t="n">
@@ -3601,7 +3644,8 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077557.html</t>
+          <t>本项目总占地面积为149道225.64平方米，总建筑面积151550.12平方米，其中新建标准化厂房143913平方米、综合管理用房7637.12平方米，配套建设配套厂区道路、停车场、绿化工程、污水管网、给水管网、强弱电工程等配套工程。
+https://www.chinapipe.net/project/d3077557.html</t>
         </is>
       </c>
       <c r="N45" t="n">
@@ -3676,7 +3720,8 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077552.html</t>
+          <t>中子镇转斗（含何家坝）、校场坝生活污商水处理站覆盖范围内的排水管网更新改造以及检查井等附属设施建设。
+https://www.chinapipe.net/project/d3077552.html</t>
         </is>
       </c>
       <c r="N46" t="n">
@@ -3751,7 +3796,8 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077551.html</t>
+          <t>新改建管道:DN300污水管道162m、DN500 污水管道1884m、DN600 污水管道112m、DN300 雨水管道466.50m、DN600 雨水管道609m、 DN800 雨水管商道 390m、 DN1000 雨水管道1029m。并对涉及破损路面及配套设施等进行恢复。
+https://www.chinapipe.net/project/d3077551.html</t>
         </is>
       </c>
       <c r="N47" t="n">
@@ -3826,7 +3872,8 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077550.html</t>
+          <t>本项目管网部分为新建排水主管网长度约2.08km（雨水管网约0.88km，污水管网约1.2km），管径DN300～DN800；现状管道清淤疏通长度约为1.23km；配套建设检查井等附属构筑物以及路面恢复提升；道路部分为埋地排水管道施工路面破除与恢复，同时对设计范围内其他道路进行路面黑化提升，项目共涉及7条道路的路面改造，其中车行道改造面积约9188平方米，人行道改造约3295平方米。
+https://www.chinapipe.net/project/d3077550.html</t>
         </is>
       </c>
       <c r="N48" t="n">
@@ -3901,7 +3948,8 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077548.html</t>
+          <t>新建教学综合楼14500㎡、学生宿舍8500㎡、食堂3000㎡，以及附属用房、排水管网等配套基础设施。
+https://www.chinapipe.net/project/d3077548.html</t>
         </is>
       </c>
       <c r="N49" t="n">
@@ -3976,7 +4024,8 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077502.html</t>
+          <t>预应力高强混凝土管桩
+https://www.chinapipe.net/project/d3077502.html</t>
         </is>
       </c>
       <c r="N50" t="n">
@@ -4051,7 +4100,8 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077494.html</t>
+          <t>本项目包括宜宾高新区高场片区老旧小区改造项目和宜宾高新区高场片区城中村配套基础设施项目的管网探测及测绘工作。
+https://www.chinapipe.net/project/d3077494.html</t>
         </is>
       </c>
       <c r="N51" t="n">
@@ -4126,7 +4176,8 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077488.html</t>
+          <t>钢管及型钢采购
+https://www.chinapipe.net/project/d3077488.html</t>
         </is>
       </c>
       <c r="N52" t="n">
@@ -4201,7 +4252,8 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077474.html</t>
+          <t>改造城镇危旧房约4.5万平方米，户数共220户，3栋共9个单元。配套小区内道路、供水、供电、供气主管网、消防、路灯等基础设施。新建道四通路与兴政路连接道路64米，铺设安置房一期商业街人行道5766平方米，配套完善排水、路灯、绿化等附属设施。
+https://www.chinapipe.net/project/d3077474.html</t>
         </is>
       </c>
       <c r="N53" t="n">
@@ -4276,7 +4328,8 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077437.html</t>
+          <t>本项目包括河清镇高标准改造提升高标准农田3万亩，秀水镇改造提升高标准农田0.6万亩，花荄镇改造提升高标准农田0.3万亩。
+https://www.chinapipe.net/project/d3077437.html</t>
         </is>
       </c>
       <c r="N54" t="n">
@@ -4351,7 +4404,8 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077434.html</t>
+          <t>新建滴灌(喷灌)灌区16处，面积2070亩，配套机井5处、提灌站10处，利用现有供水泵站延伸管道灌溉700亩；新建提灌站5座；新建200m3圆形蓄水池10口，整治原有蓄水池4口；整治原有渠道10公里；购置智能灌溉机器人（车）2台。
+https://www.chinapipe.net/project/d3077434.html</t>
         </is>
       </c>
       <c r="N55" t="n">
@@ -4426,7 +4480,8 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077433.html</t>
+          <t>新建输配水管道147.5km，新建首部枢纽21座，田间自动化控制闸阀1474套，中等流量喷枪1349道套、快速取水阀188套，300m3蓄水池2座，移动式喷灌设备10套。
+https://www.chinapipe.net/project/d3077433.html</t>
         </is>
       </c>
       <c r="N56" t="n">
@@ -4501,7 +4556,8 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077430.html</t>
+          <t>项目改造金江片区排水防涝管网及设施，主要包含以下内容:（1）改造B*H=600*800排水边沟2238m;（2）改造B*H=1500*2000排洪沟1306道m，B*H=2000*1500排洪沟120m,B*H=2500*3000排洪沟450m，B*H=3500*4000排洪沟2800m，B*H=5000*4000 排洪沟2845mB*H=6000*4000排洪沟545m;（3）排洪沟清淤18484m;排洪涵清淤2500m;（4）改造两座雨水调蓄池，规模为8000t/d和1000t/d;（5）同步布设智能物联感知设备。
+https://www.chinapipe.net/project/d3077430.html</t>
         </is>
       </c>
       <c r="N57" t="n">
@@ -4576,7 +4632,8 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077384.html</t>
+          <t>本次询价采购JD-03包件硅芯管的底色、色谱如下：商序号规格底色添加色标颜色1Φ40/33黑色黑色道2Φ40/33黑色白色1x43Φ40/33黑色黄色1x44Φ40/33黑色蓝色管1x45Φ40/33黑色绿色1x46Φ40/33黑色红色1x47Φ40/33黑色国紫色1x48Φ40/33黑色白色2x39Φ40/33黑色黄色2x310Φ40/33黑色蓝色2x311Φ40/33黑色绿色2x312Φ40/33黑色红色2x313Φ40/33黑色紫色2x314Φ40/33黑色白色3x215Φ40/33黑色黄色3x216Φ40/33黑色蓝色3x217Φ40/33黑色绿色3x218Φ40/33黑色红色3x2
+https://www.chinapipe.net/project/d3077384.html</t>
         </is>
       </c>
       <c r="N58" t="n">
@@ -4651,7 +4708,8 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077426.html</t>
+          <t>实施建设大豆种植智能滴灌系统2处，共计300亩智能滴灌示范区网，新建蓄水池23座；开展大豆单产提升技术推广。
+https://www.chinapipe.net/project/d3077426.html</t>
         </is>
       </c>
       <c r="N59" t="n">
@@ -4726,7 +4784,8 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077360.html</t>
+          <t>隆昌市城市核心区南部片区燃气配套管网改造项目焊缝探伤检测采购
+https://www.chinapipe.net/project/d3077360.html</t>
         </is>
       </c>
       <c r="N60" t="n">
@@ -4801,7 +4860,8 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077250.html</t>
+          <t>对全市5万亩高标准农田进行提档升级，建设粮油园区3万亩，全域开展农村人居环境整治，打造乡村旅游聚居村落80个，配套建设乡村振兴道路、停车场和标识导视系统等旅游服务设施等。
+https://www.chinapipe.net/project/d3077250.html</t>
         </is>
       </c>
       <c r="N61" t="n">
@@ -4876,7 +4936,8 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077249.html</t>
+          <t>预应力混凝土用金属波纹管
+https://www.chinapipe.net/project/d3077249.html</t>
         </is>
       </c>
       <c r="N62" t="n">
@@ -4951,7 +5012,8 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077246.html</t>
+          <t>新建2m³三道格化粪池584座、3m³三格化粪池1022座、20m³三格化粪池2座、30m³三格化粪池2座，配套建设入户管、支管、干管、检查井、过滤池等。
+https://www.chinapipe.net/project/d3077246.html</t>
         </is>
       </c>
       <c r="N63" t="n">
@@ -5026,7 +5088,8 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077244.html</t>
+          <t>本项目总规划用地面积为6665.90平方米，总建筑面积约10823.11平方米（其中已建建筑面积4519.92平方米，本次项目建筑面积6303.19平方米），项目总体包含新建1座地下车库及1栋学前教育教学楼和1栋大门，其中地上建筑面积4601.97平方米（学前教育教学楼和大门）；地下建筑面积1701.22平方米（包括地下车库、人防地下室、设备用房等）；改造教学楼及宿舍面积约4519.92平方米（含建筑外墙改造及消防管网改造）；绿化面积约2473.01平方米；道路及广场用地约1814.05平方米；400米室外消防给水管网、200米生活给水管网、400米室外污水管网、400米室外雨水管网、220米室外强电管网、220米室外弱电管网、1个混凝土格栅池等。
+https://www.chinapipe.net/project/d3077244.html</t>
         </is>
       </c>
       <c r="N64" t="n">
@@ -5101,7 +5164,8 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077243.html</t>
+          <t>新建污水收集主支管网34.48km、污水入户管64.87km；对现有1座300m³/d污水处理站进行改扩建，将污水处理能力提升至500m³/d；新建污水资源化利用设施3套、视频监控系统9套、水质监测网络1套、水环境风险预警网络1套、监控平台1套；新建150m³/d污水处理站2座、200m³/d污水处理站1座、700m³/d污水处理站1座、化粪池1座、污水提升泵站11座、标志牌9块。
+https://www.chinapipe.net/project/d3077243.html</t>
         </is>
       </c>
       <c r="N65" t="n">
@@ -5176,7 +5240,8 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077240.html</t>
+          <t>新建生态缓冲带23597.6m2；新建底质改良及微地形改造面积约112287m2、新建挺水植物面 招标项目概积22457.4m2、沉水植物面积56143.5m2、浮叶植物面积11228.7m2、网鱼蚌螺修复区面积44914.8m2； 新建生态沟渠1858m，新建污水收集主支管1.6km、入户管1.2km。
+https://www.chinapipe.net/project/d3077240.html</t>
         </is>
       </c>
       <c r="N66" t="n">
@@ -5251,7 +5316,8 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077175.html</t>
+          <t>建设大豆单产提升工程示范区3万亩，其中核心区-水肥一体化滴网灌工程1750亩、辐射区-水源工程28250亩。
+https://www.chinapipe.net/project/d3077175.html</t>
         </is>
       </c>
       <c r="N67" t="n">
@@ -5326,7 +5392,8 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>https://www.chinapipe.net/project/d3077107.html</t>
+          <t>钢筋混凝土管采购
+https://www.chinapipe.net/project/d3077107.html</t>
         </is>
       </c>
       <c r="N68" t="n">

</xml_diff>